<commit_message>
data: atualização base chamados 19-06-26 0903
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S574" headerRowCount="1">
-  <autoFilter ref="A1:S574"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S573" headerRowCount="1">
+  <autoFilter ref="A1:S573"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S574"/>
+  <dimension ref="A1:S573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="L25" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M25" s="1" t="inlineStr">
@@ -2388,12 +2388,22 @@
         </is>
       </c>
       <c r="N25" s="1" t="n"/>
-      <c r="O25" s="1" t="n"/>
-      <c r="P25" s="1" t="inlineStr"/>
-      <c r="Q25" s="1" t="inlineStr"/>
+      <c r="O25" s="2" t="n">
+        <v>46192.346565625</v>
+      </c>
+      <c r="P25" s="1" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="Q25" s="1" t="inlineStr">
+        <is>
+          <t>Segue conforme solicitado.</t>
+        </is>
+      </c>
       <c r="R25" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S25" s="1" t="n"/>
@@ -2527,7 +2537,7 @@
       </c>
       <c r="L27" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M27" s="1" t="inlineStr">
@@ -2536,12 +2546,22 @@
         </is>
       </c>
       <c r="N27" s="1" t="n"/>
-      <c r="O27" s="1" t="n"/>
-      <c r="P27" s="1" t="inlineStr"/>
-      <c r="Q27" s="1" t="inlineStr"/>
+      <c r="O27" s="2" t="n">
+        <v>46191.75819690972</v>
+      </c>
+      <c r="P27" s="1" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="Q27" s="1" t="inlineStr">
+        <is>
+          <t>Segue conforme solicitado.</t>
+        </is>
+      </c>
       <c r="R27" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S27" s="1" t="n"/>
@@ -3145,7 +3165,7 @@
       </c>
       <c r="L35" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M35" s="1" t="inlineStr">
@@ -3154,12 +3174,22 @@
         </is>
       </c>
       <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
-      <c r="P35" s="1" t="inlineStr"/>
-      <c r="Q35" s="1" t="inlineStr"/>
+      <c r="O35" s="2" t="n">
+        <v>46191.75739950231</v>
+      </c>
+      <c r="P35" s="1" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="Q35" s="1" t="inlineStr">
+        <is>
+          <t>Segue conforme solicitado.</t>
+        </is>
+      </c>
       <c r="R35" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S35" s="1" t="n"/>
@@ -4770,7 +4800,7 @@
       </c>
       <c r="L56" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M56" s="1" t="inlineStr">
@@ -4779,12 +4809,22 @@
         </is>
       </c>
       <c r="N56" s="1" t="n"/>
-      <c r="O56" s="1" t="n"/>
-      <c r="P56" s="1" t="inlineStr"/>
-      <c r="Q56" s="1" t="inlineStr"/>
+      <c r="O56" s="2" t="n">
+        <v>46191.75782056713</v>
+      </c>
+      <c r="P56" s="1" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="Q56" s="1" t="inlineStr">
+        <is>
+          <t>Segue conforme solicitado.</t>
+        </is>
+      </c>
       <c r="R56" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S56" s="1" t="n"/>
@@ -7738,7 +7778,7 @@
       </c>
       <c r="L95" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M95" s="1" t="inlineStr">
@@ -7746,10 +7786,16 @@
           <t>Ricardo Ferreira</t>
         </is>
       </c>
-      <c r="N95" s="1" t="n"/>
+      <c r="N95" s="2" t="n">
+        <v>46191.7695471875</v>
+      </c>
       <c r="O95" s="1" t="n"/>
       <c r="P95" s="1" t="inlineStr"/>
-      <c r="Q95" s="1" t="inlineStr"/>
+      <c r="Q95" s="1" t="inlineStr">
+        <is>
+          <t>Cliente não enviou o SPED do mês 09/2025, por isso foi entregue em branco e gerou diferença de transporte de saldo. O processo de montagem para retificação está sendo realizado conforme autorização da Claudineia.</t>
+        </is>
+      </c>
       <c r="R95" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -7807,7 +7853,7 @@
       </c>
       <c r="L96" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M96" s="1" t="inlineStr">
@@ -7816,12 +7862,22 @@
         </is>
       </c>
       <c r="N96" s="1" t="n"/>
-      <c r="O96" s="1" t="n"/>
-      <c r="P96" s="1" t="inlineStr"/>
-      <c r="Q96" s="1" t="inlineStr"/>
+      <c r="O96" s="2" t="n">
+        <v>46191.76695482639</v>
+      </c>
+      <c r="P96" s="1" t="inlineStr">
+        <is>
+          <t>ricardof</t>
+        </is>
+      </c>
+      <c r="Q96" s="1" t="inlineStr">
+        <is>
+          <t>Guias recalculadas.</t>
+        </is>
+      </c>
       <c r="R96" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S96" s="1" t="n"/>
@@ -25598,7 +25654,7 @@
       </c>
       <c r="L329" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M329" s="1" t="inlineStr">
@@ -25607,12 +25663,22 @@
         </is>
       </c>
       <c r="N329" s="1" t="n"/>
-      <c r="O329" s="1" t="n"/>
-      <c r="P329" s="1" t="inlineStr"/>
-      <c r="Q329" s="1" t="inlineStr"/>
+      <c r="O329" s="2" t="n">
+        <v>46191.76178888889</v>
+      </c>
+      <c r="P329" s="1" t="inlineStr">
+        <is>
+          <t>mateusm</t>
+        </is>
+      </c>
+      <c r="Q329" s="1" t="inlineStr">
+        <is>
+          <t>Segue documentos solicitados</t>
+        </is>
+      </c>
       <c r="R329" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S329" s="1" t="n"/>
@@ -43018,7 +43084,7 @@
     </row>
     <row r="569">
       <c r="A569" s="1" t="n">
-        <v>80217</v>
+        <v>80225</v>
       </c>
       <c r="B569" s="1" t="inlineStr">
         <is>
@@ -43027,53 +43093,49 @@
       </c>
       <c r="C569" s="1" t="inlineStr">
         <is>
-          <t>Baixa Automática - SPED</t>
+          <t>Chamados</t>
         </is>
       </c>
       <c r="D569" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>B.P.O. - GUARANI CTB</t>
         </is>
       </c>
       <c r="E569" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solicito a baixa do sped fiscal da empresa 5165 - LEGUME S/A na qual o IE dela foi cadastrado no Período 02/10/2025, sendo assim não tem o porque ter tarefas do período de 2023 a 09/2025. segue situação do posto fiscal </t>
+          <t>por gentileza poderia baixar os Das as empresas - 4917 e 4064 em anexo - e observação a guia ICMS da empresa 4059 encontrasse com o responsável e não foi liberado para contabilidade ainda</t>
         </is>
       </c>
       <c r="F569" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G569" s="1" t="n"/>
-      <c r="H569" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H569" s="1" t="n"/>
       <c r="I569" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J569" s="2" t="n">
-        <v>46191.66336269676</v>
+        <v>46191.74847341435</v>
       </c>
       <c r="K569" s="2" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="L569" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M569" s="1" t="inlineStr">
         <is>
-          <t>Jonatan Hayashibara</t>
+          <t>Flavia Dariolli</t>
         </is>
       </c>
       <c r="N569" s="1" t="n"/>
       <c r="O569" s="1" t="n"/>
       <c r="P569" s="1" t="inlineStr"/>
-      <c r="Q569" s="1" t="inlineStr"/>
+      <c r="Q569" s="1" t="n"/>
       <c r="R569" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -43083,7 +43145,7 @@
     </row>
     <row r="570">
       <c r="A570" s="1" t="n">
-        <v>80225</v>
+        <v>76508</v>
       </c>
       <c r="B570" s="1" t="inlineStr">
         <is>
@@ -43092,59 +43154,77 @@
       </c>
       <c r="C570" s="1" t="inlineStr">
         <is>
-          <t>Chamados</t>
+          <t>Verificar Validação Obrigação</t>
         </is>
       </c>
       <c r="D570" s="1" t="inlineStr">
         <is>
-          <t>B.P.O. - GUARANI CTB</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E570" s="1" t="inlineStr">
         <is>
-          <t>por gentileza poderia baixar os Das as empresas - 4917 e 4064 em anexo - e observação a guia ICMS da empresa 4059 encontrasse com o responsável e não foi liberado para contabilidade ainda</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F570" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G570" s="1" t="n"/>
-      <c r="H570" s="1" t="n"/>
+        <v>6605</v>
+      </c>
+      <c r="G570" s="1" t="inlineStr">
+        <is>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
+        </is>
+      </c>
+      <c r="H570" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
       <c r="I570" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J570" s="2" t="n">
-        <v>46191.74847341435</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K570" s="2" t="n">
-        <v>46195</v>
+        <v>46034</v>
       </c>
       <c r="L570" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M570" s="1" t="inlineStr">
         <is>
-          <t>Flavia Dariolli</t>
+          <t>Bianca Castro</t>
         </is>
       </c>
       <c r="N570" s="1" t="n"/>
-      <c r="O570" s="1" t="n"/>
-      <c r="P570" s="1" t="inlineStr"/>
-      <c r="Q570" s="1" t="n"/>
+      <c r="O570" s="2" t="n">
+        <v>46030.75027241898</v>
+      </c>
+      <c r="P570" s="1" t="inlineStr">
+        <is>
+          <t>nicoleo</t>
+        </is>
+      </c>
+      <c r="Q570" s="1" t="inlineStr">
+        <is>
+          <t>Baixadas.</t>
+        </is>
+      </c>
       <c r="R570" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S570" s="1" t="n"/>
     </row>
     <row r="571">
       <c r="A571" s="1" t="n">
-        <v>76508</v>
+        <v>76505</v>
       </c>
       <c r="B571" s="1" t="inlineStr">
         <is>
@@ -43163,15 +43243,15 @@
       </c>
       <c r="E571" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F571" s="1" t="n">
-        <v>6605</v>
+        <v>6640</v>
       </c>
       <c r="G571" s="1" t="inlineStr">
         <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H571" s="1" t="inlineStr">
@@ -43185,7 +43265,7 @@
         </is>
       </c>
       <c r="J571" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K571" s="2" t="n">
         <v>46034</v>
@@ -43202,7 +43282,7 @@
       </c>
       <c r="N571" s="1" t="n"/>
       <c r="O571" s="2" t="n">
-        <v>46030.75027241898</v>
+        <v>46030.63182743055</v>
       </c>
       <c r="P571" s="1" t="inlineStr">
         <is>
@@ -43223,7 +43303,7 @@
     </row>
     <row r="572">
       <c r="A572" s="1" t="n">
-        <v>76505</v>
+        <v>76515</v>
       </c>
       <c r="B572" s="1" t="inlineStr">
         <is>
@@ -43242,15 +43322,15 @@
       </c>
       <c r="E572" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
         </is>
       </c>
       <c r="F572" s="1" t="n">
-        <v>6640</v>
+        <v>6641</v>
       </c>
       <c r="G572" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
         </is>
       </c>
       <c r="H572" s="1" t="inlineStr">
@@ -43264,7 +43344,7 @@
         </is>
       </c>
       <c r="J572" s="2" t="n">
-        <v>46030.60213634259</v>
+        <v>46030.73046079861</v>
       </c>
       <c r="K572" s="2" t="n">
         <v>46034</v>
@@ -43281,7 +43361,7 @@
       </c>
       <c r="N572" s="1" t="n"/>
       <c r="O572" s="2" t="n">
-        <v>46030.63182743055</v>
+        <v>46030.74734336806</v>
       </c>
       <c r="P572" s="1" t="inlineStr">
         <is>
@@ -43290,7 +43370,7 @@
       </c>
       <c r="Q572" s="1" t="inlineStr">
         <is>
-          <t>Baixadas.</t>
+          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
         </is>
       </c>
       <c r="R572" s="1" t="inlineStr">
@@ -43302,7 +43382,7 @@
     </row>
     <row r="573">
       <c r="A573" s="1" t="n">
-        <v>76515</v>
+        <v>76501</v>
       </c>
       <c r="B573" s="1" t="inlineStr">
         <is>
@@ -43321,7 +43401,7 @@
       </c>
       <c r="E573" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
         </is>
       </c>
       <c r="F573" s="1" t="n">
@@ -43343,7 +43423,7 @@
         </is>
       </c>
       <c r="J573" s="2" t="n">
-        <v>46030.73046079861</v>
+        <v>46030.51327708333</v>
       </c>
       <c r="K573" s="2" t="n">
         <v>46034</v>
@@ -43360,7 +43440,7 @@
       </c>
       <c r="N573" s="1" t="n"/>
       <c r="O573" s="2" t="n">
-        <v>46030.74734336806</v>
+        <v>46030.64333047454</v>
       </c>
       <c r="P573" s="1" t="inlineStr">
         <is>
@@ -43369,7 +43449,7 @@
       </c>
       <c r="Q573" s="1" t="inlineStr">
         <is>
-          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
+          <t>Baixadas.</t>
         </is>
       </c>
       <c r="R573" s="1" t="inlineStr">
@@ -43378,85 +43458,6 @@
         </is>
       </c>
       <c r="S573" s="1" t="n"/>
-    </row>
-    <row r="574">
-      <c r="A574" s="1" t="n">
-        <v>76501</v>
-      </c>
-      <c r="B574" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C574" s="1" t="inlineStr">
-        <is>
-          <t>Verificar Validação Obrigação</t>
-        </is>
-      </c>
-      <c r="D574" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E574" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
-        </is>
-      </c>
-      <c r="F574" s="1" t="n">
-        <v>6641</v>
-      </c>
-      <c r="G574" s="1" t="inlineStr">
-        <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
-        </is>
-      </c>
-      <c r="H574" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
-      <c r="I574" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J574" s="2" t="n">
-        <v>46030.51327708333</v>
-      </c>
-      <c r="K574" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="L574" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M574" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N574" s="1" t="n"/>
-      <c r="O574" s="2" t="n">
-        <v>46030.64333047454</v>
-      </c>
-      <c r="P574" s="1" t="inlineStr">
-        <is>
-          <t>nicoleo</t>
-        </is>
-      </c>
-      <c r="Q574" s="1" t="inlineStr">
-        <is>
-          <t>Baixadas.</t>
-        </is>
-      </c>
-      <c r="R574" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S574" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 19-06-26 1330
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -3163,7 +3163,7 @@
       </c>
       <c r="H35" s="1" t="inlineStr">
         <is>
-          <t>Bruno Henrique</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I35" s="1" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="H36" s="1" t="inlineStr">
         <is>
-          <t>Bruno Henrique</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I36" s="1" t="inlineStr">
@@ -5346,7 +5346,11 @@
           <t>Distribuidora J Jotas Ltda.</t>
         </is>
       </c>
-      <c r="H63" s="1" t="n"/>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I63" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -5360,7 +5364,7 @@
       </c>
       <c r="L63" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M63" s="1" t="inlineStr">
@@ -5371,7 +5375,7 @@
       <c r="N63" s="1" t="n"/>
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="inlineStr"/>
-      <c r="Q63" s="1" t="n"/>
+      <c r="Q63" s="1" t="inlineStr"/>
       <c r="R63" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -7697,7 +7701,11 @@
           <t>COMERCIO DE ALIMENTOS VICALI LTDA</t>
         </is>
       </c>
-      <c r="H94" s="1" t="n"/>
+      <c r="H94" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I94" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -7711,7 +7719,7 @@
       </c>
       <c r="L94" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M94" s="1" t="inlineStr">
@@ -7722,7 +7730,7 @@
       <c r="N94" s="1" t="n"/>
       <c r="O94" s="1" t="n"/>
       <c r="P94" s="1" t="inlineStr"/>
-      <c r="Q94" s="1" t="n"/>
+      <c r="Q94" s="1" t="inlineStr"/>
       <c r="R94" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -9496,7 +9504,11 @@
           <t>TERRA BRASIL HORTI FRUTI LTDA</t>
         </is>
       </c>
-      <c r="H117" s="1" t="n"/>
+      <c r="H117" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I117" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -9510,7 +9522,7 @@
       </c>
       <c r="L117" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M117" s="1" t="inlineStr">
@@ -9521,7 +9533,7 @@
       <c r="N117" s="1" t="n"/>
       <c r="O117" s="1" t="n"/>
       <c r="P117" s="1" t="inlineStr"/>
-      <c r="Q117" s="1" t="n"/>
+      <c r="Q117" s="1" t="inlineStr"/>
       <c r="R117" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -10549,7 +10561,11 @@
           <t>SAMPA ATACADO DE GENEROS ALIMENTICIOS E BEBIDAS LTDA</t>
         </is>
       </c>
-      <c r="H131" s="1" t="n"/>
+      <c r="H131" s="1" t="inlineStr">
+        <is>
+          <t>Karina Santos</t>
+        </is>
+      </c>
       <c r="I131" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -10563,7 +10579,7 @@
       </c>
       <c r="L131" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M131" s="1" t="inlineStr">
@@ -10574,7 +10590,7 @@
       <c r="N131" s="1" t="n"/>
       <c r="O131" s="1" t="n"/>
       <c r="P131" s="1" t="inlineStr"/>
-      <c r="Q131" s="1" t="n"/>
+      <c r="Q131" s="1" t="inlineStr"/>
       <c r="R131" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -11604,7 +11620,11 @@
           <t>SAMPATACADO DE GÊNEROS ALIMENTÍCIOS E BEBIDAS LTDA (FILIAL 02)</t>
         </is>
       </c>
-      <c r="H145" s="1" t="n"/>
+      <c r="H145" s="1" t="inlineStr">
+        <is>
+          <t>Karina Santos</t>
+        </is>
+      </c>
       <c r="I145" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -11618,7 +11638,7 @@
       </c>
       <c r="L145" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M145" s="1" t="inlineStr">
@@ -11629,7 +11649,7 @@
       <c r="N145" s="1" t="n"/>
       <c r="O145" s="1" t="n"/>
       <c r="P145" s="1" t="inlineStr"/>
-      <c r="Q145" s="1" t="n"/>
+      <c r="Q145" s="1" t="inlineStr"/>
       <c r="R145" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -16214,7 +16234,11 @@
           <t>DISTRIBUIDOR DE MORANGOS LTDA</t>
         </is>
       </c>
-      <c r="H205" s="1" t="n"/>
+      <c r="H205" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I205" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -16228,7 +16252,7 @@
       </c>
       <c r="L205" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M205" s="1" t="inlineStr">
@@ -16239,7 +16263,7 @@
       <c r="N205" s="1" t="n"/>
       <c r="O205" s="1" t="n"/>
       <c r="P205" s="1" t="inlineStr"/>
-      <c r="Q205" s="1" t="n"/>
+      <c r="Q205" s="1" t="inlineStr"/>
       <c r="R205" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -16348,7 +16372,11 @@
           <t>DISTRIBUIDOR DE MORANGOS LTDA</t>
         </is>
       </c>
-      <c r="H207" s="1" t="n"/>
+      <c r="H207" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I207" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -16362,7 +16390,7 @@
       </c>
       <c r="L207" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M207" s="1" t="inlineStr">
@@ -16373,7 +16401,7 @@
       <c r="N207" s="1" t="n"/>
       <c r="O207" s="1" t="n"/>
       <c r="P207" s="1" t="inlineStr"/>
-      <c r="Q207" s="1" t="n"/>
+      <c r="Q207" s="1" t="inlineStr"/>
       <c r="R207" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -16803,7 +16831,7 @@
       </c>
       <c r="L213" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M213" s="1" t="inlineStr">
@@ -16811,10 +16839,16 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N213" s="1" t="n"/>
+      <c r="N213" s="2" t="n">
+        <v>46192.55170297454</v>
+      </c>
       <c r="O213" s="1" t="n"/>
       <c r="P213" s="1" t="inlineStr"/>
-      <c r="Q213" s="1" t="inlineStr"/>
+      <c r="Q213" s="1" t="inlineStr">
+        <is>
+          <t>Ajustes vão ser reallizados junto ao fechamento</t>
+        </is>
+      </c>
       <c r="R213" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -18090,7 +18124,11 @@
           <t>LITOCOMP INDUSTRIA GRAFICA E EDITORA LTDA</t>
         </is>
       </c>
-      <c r="H230" s="1" t="n"/>
+      <c r="H230" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I230" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -18104,7 +18142,7 @@
       </c>
       <c r="L230" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M230" s="1" t="inlineStr">
@@ -18115,7 +18153,7 @@
       <c r="N230" s="1" t="n"/>
       <c r="O230" s="1" t="n"/>
       <c r="P230" s="1" t="inlineStr"/>
-      <c r="Q230" s="1" t="n"/>
+      <c r="Q230" s="1" t="inlineStr"/>
       <c r="R230" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -19004,7 +19042,11 @@
           <t xml:space="preserve">LINHARES E FONTOURA CONSTRUCAO CIVIL LTDA </t>
         </is>
       </c>
-      <c r="H242" s="1" t="n"/>
+      <c r="H242" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I242" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -19018,7 +19060,7 @@
       </c>
       <c r="L242" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M242" s="1" t="inlineStr">
@@ -19029,7 +19071,7 @@
       <c r="N242" s="1" t="n"/>
       <c r="O242" s="1" t="n"/>
       <c r="P242" s="1" t="inlineStr"/>
-      <c r="Q242" s="1" t="n"/>
+      <c r="Q242" s="1" t="inlineStr"/>
       <c r="R242" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -19486,7 +19528,7 @@
       </c>
       <c r="L248" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M248" s="1" t="inlineStr">
@@ -19494,10 +19536,16 @@
           <t>Rogerio Egidio</t>
         </is>
       </c>
-      <c r="N248" s="1" t="n"/>
+      <c r="N248" s="2" t="n">
+        <v>46192.55194065972</v>
+      </c>
       <c r="O248" s="1" t="n"/>
       <c r="P248" s="1" t="inlineStr"/>
-      <c r="Q248" s="1" t="inlineStr"/>
+      <c r="Q248" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando dpto fiscal retificar a reinf</t>
+        </is>
+      </c>
       <c r="R248" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -19606,7 +19654,11 @@
           <t xml:space="preserve">GM RECICLA SERVICOS LTDA </t>
         </is>
       </c>
-      <c r="H250" s="1" t="n"/>
+      <c r="H250" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I250" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -19620,7 +19672,7 @@
       </c>
       <c r="L250" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M250" s="1" t="inlineStr">
@@ -19631,7 +19683,7 @@
       <c r="N250" s="1" t="n"/>
       <c r="O250" s="1" t="n"/>
       <c r="P250" s="1" t="inlineStr"/>
-      <c r="Q250" s="1" t="n"/>
+      <c r="Q250" s="1" t="inlineStr"/>
       <c r="R250" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23869,7 +23921,11 @@
           <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H306" s="1" t="n"/>
+      <c r="H306" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I306" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -23883,7 +23939,7 @@
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M306" s="1" t="inlineStr">
@@ -23894,7 +23950,7 @@
       <c r="N306" s="1" t="n"/>
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="inlineStr"/>
-      <c r="Q306" s="1" t="n"/>
+      <c r="Q306" s="1" t="inlineStr"/>
       <c r="R306" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25852,7 +25908,11 @@
           <t>L.S.V COMERCIO , LOCACAO ,MONTAGENS E REPRESENTACAO COMERCIAL LTDA</t>
         </is>
       </c>
-      <c r="H332" s="1" t="n"/>
+      <c r="H332" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I332" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -25866,7 +25926,7 @@
       </c>
       <c r="L332" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M332" s="1" t="inlineStr">
@@ -25877,7 +25937,7 @@
       <c r="N332" s="1" t="n"/>
       <c r="O332" s="1" t="n"/>
       <c r="P332" s="1" t="inlineStr"/>
-      <c r="Q332" s="1" t="n"/>
+      <c r="Q332" s="1" t="inlineStr"/>
       <c r="R332" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25917,7 +25977,11 @@
           <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H333" s="1" t="n"/>
+      <c r="H333" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I333" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -25931,7 +25995,7 @@
       </c>
       <c r="L333" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M333" s="1" t="inlineStr">
@@ -25942,7 +26006,7 @@
       <c r="N333" s="1" t="n"/>
       <c r="O333" s="1" t="n"/>
       <c r="P333" s="1" t="inlineStr"/>
-      <c r="Q333" s="1" t="n"/>
+      <c r="Q333" s="1" t="inlineStr"/>
       <c r="R333" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
data: atualização base chamados 22-06-26 0910
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S578" headerRowCount="1">
-  <autoFilter ref="A1:S578"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S575" headerRowCount="1">
+  <autoFilter ref="A1:S575"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S578"/>
+  <dimension ref="A1:S575"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43369,7 +43369,7 @@
     </row>
     <row r="570">
       <c r="A570" s="1" t="n">
-        <v>80255</v>
+        <v>80173</v>
       </c>
       <c r="B570" s="1" t="inlineStr">
         <is>
@@ -43383,12 +43383,12 @@
       </c>
       <c r="D570" s="1" t="inlineStr">
         <is>
-          <t>MG EXPRESS - GC</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E570" s="1" t="inlineStr">
         <is>
-          <t>Boa Tarde Amigos,Podem nos auxiliar na Baixa da Tarefa " Fed - DAS " Colocamos 2 vezes na Baixa Automática mas não está Baixando as tarefas.</t>
+          <t>Bom dia! Por gentileza, poderia realizar a baixa da tarefa DEC 2 quinzena dos clientes abaixo. ISENTO3498	EMPLACA SERVIÇOS LTDA4327	ACCESS EVENTOS E VIAGENS LTDA5780	A Estancia Morro Grande Centro de Reabilitacao Social (Filial 1)5873	FRRD ADMINISTRADORA DE IMOVEIS LTDA5906	A Estancia Morro Grande - Centro de Reabilitacao Social LTDA (Filial 2)5978	HLL LOCADORA DE GUINDASTES LTDA5979	AMATRUDA LOCADORA DE GUINDASTES E ARTICULADOS LTDA6172	MEDICAL DISCOVERY TREINAMENTOS &amp; DESENVOLVIMENTO LTDA.6173	CLINICA TONON DE DERMATOLOGISTA LTDA6266	B. HOVE COMERCIO E INDUSTRIA DE PRODUTOS ABRASIVOS LTDA (FILIAL 1)6267	CEO7 - SERVICOS DE MARKETING E APOIO ADMINISTRATIVO LTDA6415	FABIO PEREIRA DA COSTA6416	SINZATO ENTERTAINMENT LTDA6450	RDF VEICULOS LTDA6501	MD TREINAMENTOS E DESENVOLVIMENTO LTDA6652	RAZEC EMPRESA DE APOIO ADMINISTRATIVO LTDA6766	MASTER IN THREADS CURSOS E EVENTOS SPE LTDA6794	C.M.A EDUCACIONAL LTDA6796	COLÉGIO JOAQUIM MARIA MACHADO DE ASSIS LTDA (FILIAL)6798	LFJ TRANSPORTE LTDA6930	DOMENICO BIEMMI FRANCISCO LEITEERRO ( SEM CERTIFICADO)5084	REPUME REPUXAÇÃO E METALURGICA LTDA (FILIAL 01)5292	EZEKY LTDA</t>
         </is>
       </c>
       <c r="F570" s="1" t="n">
@@ -43406,35 +43406,45 @@
         </is>
       </c>
       <c r="J570" s="2" t="n">
-        <v>46192.67904146991</v>
+        <v>46191.36702172454</v>
       </c>
       <c r="K570" s="2" t="n">
-        <v>46195</v>
+        <v>46192</v>
       </c>
       <c r="L570" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M570" s="1" t="inlineStr">
         <is>
-          <t>Helmer Dantas</t>
+          <t>Ana Santana</t>
         </is>
       </c>
       <c r="N570" s="1" t="n"/>
-      <c r="O570" s="1" t="n"/>
-      <c r="P570" s="1" t="inlineStr"/>
-      <c r="Q570" s="1" t="inlineStr"/>
+      <c r="O570" s="2" t="n">
+        <v>46191.38533472222</v>
+      </c>
+      <c r="P570" s="1" t="inlineStr">
+        <is>
+          <t>gamaral</t>
+        </is>
+      </c>
+      <c r="Q570" s="1" t="inlineStr">
+        <is>
+          <t>Tarefas baixadas</t>
+        </is>
+      </c>
       <c r="R570" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S570" s="1" t="n"/>
     </row>
     <row r="571">
       <c r="A571" s="1" t="n">
-        <v>80173</v>
+        <v>80174</v>
       </c>
       <c r="B571" s="1" t="inlineStr">
         <is>
@@ -43443,7 +43453,7 @@
       </c>
       <c r="C571" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Vencimento de Tarefas</t>
         </is>
       </c>
       <c r="D571" s="1" t="inlineStr">
@@ -43453,7 +43463,7 @@
       </c>
       <c r="E571" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, poderia realizar a baixa da tarefa DEC 2 quinzena dos clientes abaixo. ISENTO3498	EMPLACA SERVIÇOS LTDA4327	ACCESS EVENTOS E VIAGENS LTDA5780	A Estancia Morro Grande Centro de Reabilitacao Social (Filial 1)5873	FRRD ADMINISTRADORA DE IMOVEIS LTDA5906	A Estancia Morro Grande - Centro de Reabilitacao Social LTDA (Filial 2)5978	HLL LOCADORA DE GUINDASTES LTDA5979	AMATRUDA LOCADORA DE GUINDASTES E ARTICULADOS LTDA6172	MEDICAL DISCOVERY TREINAMENTOS &amp; DESENVOLVIMENTO LTDA.6173	CLINICA TONON DE DERMATOLOGISTA LTDA6266	B. HOVE COMERCIO E INDUSTRIA DE PRODUTOS ABRASIVOS LTDA (FILIAL 1)6267	CEO7 - SERVICOS DE MARKETING E APOIO ADMINISTRATIVO LTDA6415	FABIO PEREIRA DA COSTA6416	SINZATO ENTERTAINMENT LTDA6450	RDF VEICULOS LTDA6501	MD TREINAMENTOS E DESENVOLVIMENTO LTDA6652	RAZEC EMPRESA DE APOIO ADMINISTRATIVO LTDA6766	MASTER IN THREADS CURSOS E EVENTOS SPE LTDA6794	C.M.A EDUCACIONAL LTDA6796	COLÉGIO JOAQUIM MARIA MACHADO DE ASSIS LTDA (FILIAL)6798	LFJ TRANSPORTE LTDA6930	DOMENICO BIEMMI FRANCISCO LEITEERRO ( SEM CERTIFICADO)5084	REPUME REPUXAÇÃO E METALURGICA LTDA (FILIAL 01)5292	EZEKY LTDA</t>
+          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
         </is>
       </c>
       <c r="F571" s="1" t="n">
@@ -43471,7 +43481,7 @@
         </is>
       </c>
       <c r="J571" s="2" t="n">
-        <v>46191.36702172454</v>
+        <v>46191.36721832176</v>
       </c>
       <c r="K571" s="2" t="n">
         <v>46192</v>
@@ -43483,12 +43493,12 @@
       </c>
       <c r="M571" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N571" s="1" t="n"/>
       <c r="O571" s="2" t="n">
-        <v>46191.38533472222</v>
+        <v>46191.49335512731</v>
       </c>
       <c r="P571" s="1" t="inlineStr">
         <is>
@@ -43509,7 +43519,7 @@
     </row>
     <row r="572">
       <c r="A572" s="1" t="n">
-        <v>80174</v>
+        <v>76508</v>
       </c>
       <c r="B572" s="1" t="inlineStr">
         <is>
@@ -43518,7 +43528,7 @@
       </c>
       <c r="C572" s="1" t="inlineStr">
         <is>
-          <t>Vencimento de Tarefas</t>
+          <t>Verificar Validação Obrigação</t>
         </is>
       </c>
       <c r="D572" s="1" t="inlineStr">
@@ -43528,16 +43538,20 @@
       </c>
       <c r="E572" s="1" t="inlineStr">
         <is>
-          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F572" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G572" s="1" t="n"/>
+        <v>6605</v>
+      </c>
+      <c r="G572" s="1" t="inlineStr">
+        <is>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
+        </is>
+      </c>
       <c r="H572" s="1" t="inlineStr">
         <is>
-          <t>Gabriel Amaral</t>
+          <t>Nicole Oliveira</t>
         </is>
       </c>
       <c r="I572" s="1" t="inlineStr">
@@ -43546,10 +43560,10 @@
         </is>
       </c>
       <c r="J572" s="2" t="n">
-        <v>46191.36721832176</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K572" s="2" t="n">
-        <v>46192</v>
+        <v>46034</v>
       </c>
       <c r="L572" s="1" t="inlineStr">
         <is>
@@ -43558,21 +43572,21 @@
       </c>
       <c r="M572" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Bianca Castro</t>
         </is>
       </c>
       <c r="N572" s="1" t="n"/>
       <c r="O572" s="2" t="n">
-        <v>46191.49335512731</v>
+        <v>46030.75027241898</v>
       </c>
       <c r="P572" s="1" t="inlineStr">
         <is>
-          <t>gamaral</t>
+          <t>nicoleo</t>
         </is>
       </c>
       <c r="Q572" s="1" t="inlineStr">
         <is>
-          <t>Tarefas baixadas</t>
+          <t>Baixadas.</t>
         </is>
       </c>
       <c r="R572" s="1" t="inlineStr">
@@ -43584,7 +43598,7 @@
     </row>
     <row r="573">
       <c r="A573" s="1" t="n">
-        <v>80260</v>
+        <v>76505</v>
       </c>
       <c r="B573" s="1" t="inlineStr">
         <is>
@@ -43593,30 +43607,30 @@
       </c>
       <c r="C573" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Verificar Validação Obrigação</t>
         </is>
       </c>
       <c r="D573" s="1" t="inlineStr">
         <is>
-          <t>RJ - CTB</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E573" s="1" t="inlineStr">
         <is>
-          <t>Esta com erro honorários na baixa do analise, mas a NF esta ativa e lançada. Em anexo o erro e a NF ativa. Poderia me ajudar?</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F573" s="1" t="n">
-        <v>4944</v>
+        <v>6640</v>
       </c>
       <c r="G573" s="1" t="inlineStr">
         <is>
-          <t>THZ WORK TERCEIRIZADA LTDA</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H573" s="1" t="inlineStr">
         <is>
-          <t>Gabriel Amaral</t>
+          <t>Nicole Oliveira</t>
         </is>
       </c>
       <c r="I573" s="1" t="inlineStr">
@@ -43625,35 +43639,45 @@
         </is>
       </c>
       <c r="J573" s="2" t="n">
-        <v>46192.711678125</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K573" s="2" t="n">
-        <v>46195</v>
+        <v>46034</v>
       </c>
       <c r="L573" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M573" s="1" t="inlineStr">
         <is>
-          <t>Jessica Roque</t>
+          <t>Bianca Castro</t>
         </is>
       </c>
       <c r="N573" s="1" t="n"/>
-      <c r="O573" s="1" t="n"/>
-      <c r="P573" s="1" t="inlineStr"/>
-      <c r="Q573" s="1" t="inlineStr"/>
+      <c r="O573" s="2" t="n">
+        <v>46030.63182743055</v>
+      </c>
+      <c r="P573" s="1" t="inlineStr">
+        <is>
+          <t>nicoleo</t>
+        </is>
+      </c>
+      <c r="Q573" s="1" t="inlineStr">
+        <is>
+          <t>Baixadas.</t>
+        </is>
+      </c>
       <c r="R573" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S573" s="1" t="n"/>
     </row>
     <row r="574">
       <c r="A574" s="1" t="n">
-        <v>80261</v>
+        <v>76515</v>
       </c>
       <c r="B574" s="1" t="inlineStr">
         <is>
@@ -43662,30 +43686,30 @@
       </c>
       <c r="C574" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Verificar Validação Obrigação</t>
         </is>
       </c>
       <c r="D574" s="1" t="inlineStr">
         <is>
-          <t>RJ - CTB</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E574" s="1" t="inlineStr">
         <is>
-          <t>Esta com erro honorários na baixa do analise, mas a NF esta ativa e lançada. Em anexo o erro e a NF ativa. Poderia me ajudar?</t>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
         </is>
       </c>
       <c r="F574" s="1" t="n">
-        <v>4946</v>
+        <v>6641</v>
       </c>
       <c r="G574" s="1" t="inlineStr">
         <is>
-          <t>LEAL PRESTAÇÃO DE SERVIÇOS LTDA</t>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
         </is>
       </c>
       <c r="H574" s="1" t="inlineStr">
         <is>
-          <t>Gabriel Amaral</t>
+          <t>Nicole Oliveira</t>
         </is>
       </c>
       <c r="I574" s="1" t="inlineStr">
@@ -43694,35 +43718,45 @@
         </is>
       </c>
       <c r="J574" s="2" t="n">
-        <v>46192.71273252315</v>
+        <v>46030.73046079861</v>
       </c>
       <c r="K574" s="2" t="n">
-        <v>46195</v>
+        <v>46034</v>
       </c>
       <c r="L574" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M574" s="1" t="inlineStr">
         <is>
-          <t>Jessica Roque</t>
+          <t>Bianca Castro</t>
         </is>
       </c>
       <c r="N574" s="1" t="n"/>
-      <c r="O574" s="1" t="n"/>
-      <c r="P574" s="1" t="inlineStr"/>
-      <c r="Q574" s="1" t="inlineStr"/>
+      <c r="O574" s="2" t="n">
+        <v>46030.74734336806</v>
+      </c>
+      <c r="P574" s="1" t="inlineStr">
+        <is>
+          <t>nicoleo</t>
+        </is>
+      </c>
+      <c r="Q574" s="1" t="inlineStr">
+        <is>
+          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
+        </is>
+      </c>
       <c r="R574" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S574" s="1" t="n"/>
     </row>
     <row r="575">
       <c r="A575" s="1" t="n">
-        <v>76508</v>
+        <v>76501</v>
       </c>
       <c r="B575" s="1" t="inlineStr">
         <is>
@@ -43741,15 +43775,15 @@
       </c>
       <c r="E575" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
         </is>
       </c>
       <c r="F575" s="1" t="n">
-        <v>6605</v>
+        <v>6641</v>
       </c>
       <c r="G575" s="1" t="inlineStr">
         <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
         </is>
       </c>
       <c r="H575" s="1" t="inlineStr">
@@ -43763,7 +43797,7 @@
         </is>
       </c>
       <c r="J575" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46030.51327708333</v>
       </c>
       <c r="K575" s="2" t="n">
         <v>46034</v>
@@ -43780,7 +43814,7 @@
       </c>
       <c r="N575" s="1" t="n"/>
       <c r="O575" s="2" t="n">
-        <v>46030.75027241898</v>
+        <v>46030.64333047454</v>
       </c>
       <c r="P575" s="1" t="inlineStr">
         <is>
@@ -43798,243 +43832,6 @@
         </is>
       </c>
       <c r="S575" s="1" t="n"/>
-    </row>
-    <row r="576">
-      <c r="A576" s="1" t="n">
-        <v>76505</v>
-      </c>
-      <c r="B576" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C576" s="1" t="inlineStr">
-        <is>
-          <t>Verificar Validação Obrigação</t>
-        </is>
-      </c>
-      <c r="D576" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E576" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
-        </is>
-      </c>
-      <c r="F576" s="1" t="n">
-        <v>6640</v>
-      </c>
-      <c r="G576" s="1" t="inlineStr">
-        <is>
-          <t>FORT FRUIT LTDA</t>
-        </is>
-      </c>
-      <c r="H576" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
-      <c r="I576" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J576" s="2" t="n">
-        <v>46030.60213634259</v>
-      </c>
-      <c r="K576" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="L576" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M576" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N576" s="1" t="n"/>
-      <c r="O576" s="2" t="n">
-        <v>46030.63182743055</v>
-      </c>
-      <c r="P576" s="1" t="inlineStr">
-        <is>
-          <t>nicoleo</t>
-        </is>
-      </c>
-      <c r="Q576" s="1" t="inlineStr">
-        <is>
-          <t>Baixadas.</t>
-        </is>
-      </c>
-      <c r="R576" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S576" s="1" t="n"/>
-    </row>
-    <row r="577">
-      <c r="A577" s="1" t="n">
-        <v>76515</v>
-      </c>
-      <c r="B577" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C577" s="1" t="inlineStr">
-        <is>
-          <t>Verificar Validação Obrigação</t>
-        </is>
-      </c>
-      <c r="D577" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E577" s="1" t="inlineStr">
-        <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
-        </is>
-      </c>
-      <c r="F577" s="1" t="n">
-        <v>6641</v>
-      </c>
-      <c r="G577" s="1" t="inlineStr">
-        <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
-        </is>
-      </c>
-      <c r="H577" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
-      <c r="I577" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J577" s="2" t="n">
-        <v>46030.73046079861</v>
-      </c>
-      <c r="K577" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="L577" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M577" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N577" s="1" t="n"/>
-      <c r="O577" s="2" t="n">
-        <v>46030.74734336806</v>
-      </c>
-      <c r="P577" s="1" t="inlineStr">
-        <is>
-          <t>nicoleo</t>
-        </is>
-      </c>
-      <c r="Q577" s="1" t="inlineStr">
-        <is>
-          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
-        </is>
-      </c>
-      <c r="R577" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S577" s="1" t="n"/>
-    </row>
-    <row r="578">
-      <c r="A578" s="1" t="n">
-        <v>76501</v>
-      </c>
-      <c r="B578" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C578" s="1" t="inlineStr">
-        <is>
-          <t>Verificar Validação Obrigação</t>
-        </is>
-      </c>
-      <c r="D578" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E578" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
-        </is>
-      </c>
-      <c r="F578" s="1" t="n">
-        <v>6641</v>
-      </c>
-      <c r="G578" s="1" t="inlineStr">
-        <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
-        </is>
-      </c>
-      <c r="H578" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
-      <c r="I578" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J578" s="2" t="n">
-        <v>46030.51327708333</v>
-      </c>
-      <c r="K578" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="L578" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M578" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N578" s="1" t="n"/>
-      <c r="O578" s="2" t="n">
-        <v>46030.64333047454</v>
-      </c>
-      <c r="P578" s="1" t="inlineStr">
-        <is>
-          <t>nicoleo</t>
-        </is>
-      </c>
-      <c r="Q578" s="1" t="inlineStr">
-        <is>
-          <t>Baixadas.</t>
-        </is>
-      </c>
-      <c r="R578" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S578" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 24-06-26 0903
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1342,7 +1342,11 @@
         <v>0</v>
       </c>
       <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -1356,7 +1360,7 @@
       </c>
       <c r="L12" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M12" s="1" t="inlineStr">
@@ -1367,7 +1371,7 @@
       <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="inlineStr"/>
-      <c r="Q12" s="1" t="n"/>
+      <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -1962,7 +1966,11 @@
           <t>BANDEIRANTES REFRIGERAÇÃO COMERCIAL LTDA</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n"/>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -1976,7 +1984,7 @@
       </c>
       <c r="L20" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M20" s="1" t="inlineStr">
@@ -1987,7 +1995,7 @@
       <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="inlineStr"/>
-      <c r="Q20" s="1" t="n"/>
+      <c r="Q20" s="1" t="inlineStr"/>
       <c r="R20" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -4221,7 +4229,11 @@
           <t>SUPERMERCADO MAGNATA LTDA</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n"/>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Ana Barbosa</t>
+        </is>
+      </c>
       <c r="I49" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -4235,7 +4247,7 @@
       </c>
       <c r="L49" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M49" s="1" t="inlineStr">
@@ -4246,7 +4258,7 @@
       <c r="N49" s="1" t="n"/>
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="inlineStr"/>
-      <c r="Q49" s="1" t="n"/>
+      <c r="Q49" s="1" t="inlineStr"/>
       <c r="R49" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -7290,26 +7302,26 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>80224</v>
+        <v>80235</v>
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>PER/DCOMP - Intimação/Comunicado</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>PER/DCOMP - Intimação/Comunicado</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>3464 - SUPERMERCADO VICALI PARATY LTDA 				(28.466.073/0001-92)Boa tarde, prezados!!Por gentileza, verificar e tomar as devidas providencias, referente a notificação recepcionada no ECAC, sobre: IRREGULARIDADES NA UTILIZAÇÃO DE CRÉDITOS DE PIS/COFINS.Segue notificação em anexo.Qualquer duvida estou a disposição.</t>
+          <t xml:space="preserve">Por gentileza, avaliar debito em aberto na SF inerente a PIS/COFINS. </t>
         </is>
       </c>
       <c r="F89" s="1" t="n">
@@ -7322,63 +7334,74 @@
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="I89" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J89" s="2" t="n">
-        <v>46191.71619447917</v>
+        <v>46192.46505482639</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>46199</v>
+        <v>46195</v>
       </c>
       <c r="L89" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M89" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Diego Lima</t>
         </is>
       </c>
       <c r="N89" s="1" t="n"/>
-      <c r="O89" s="1" t="n"/>
-      <c r="P89" s="1" t="inlineStr"/>
-      <c r="Q89" s="1" t="inlineStr"/>
+      <c r="O89" s="2" t="n">
+        <v>46192.68080598379</v>
+      </c>
+      <c r="P89" s="1" t="inlineStr">
+        <is>
+          <t>fernandaa</t>
+        </is>
+      </c>
+      <c r="Q89" s="1" t="inlineStr">
+        <is>
+          <t>A divergencia é porque o valor pago de PIS e COFINS esta diferente do valor apurado.
+Não identificamos perdcomp para esses tributos.</t>
+        </is>
+      </c>
       <c r="R89" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S89" s="1" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>80235</v>
+        <v>80224</v>
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>PER/DCOMP - Intimação/Comunicado</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>PER/DCOMP - Intimação/Comunicado</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, avaliar debito em aberto na SF inerente a PIS/COFINS. </t>
+          <t>3464 - SUPERMERCADO VICALI PARATY LTDA 				(28.466.073/0001-92)Boa tarde, prezados!!Por gentileza, verificar e tomar as devidas providencias, referente a notificação recepcionada no ECAC, sobre: IRREGULARIDADES NA UTILIZAÇÃO DE CRÉDITOS DE PIS/COFINS.Segue notificação em anexo.Qualquer duvida estou a disposição.</t>
         </is>
       </c>
       <c r="F90" s="1" t="n">
@@ -7391,48 +7414,37 @@
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="I90" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>46192.46505482639</v>
+        <v>46191.71619447917</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>46195</v>
+        <v>46199</v>
       </c>
       <c r="L90" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M90" s="1" t="inlineStr">
         <is>
-          <t>Diego Lima</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N90" s="1" t="n"/>
-      <c r="O90" s="2" t="n">
-        <v>46192.68080598379</v>
-      </c>
-      <c r="P90" s="1" t="inlineStr">
-        <is>
-          <t>fernandaa</t>
-        </is>
-      </c>
-      <c r="Q90" s="1" t="inlineStr">
-        <is>
-          <t>A divergencia é porque o valor pago de PIS e COFINS esta diferente do valor apurado.
-Não identificamos perdcomp para esses tributos.</t>
-        </is>
-      </c>
+      <c r="O90" s="1" t="n"/>
+      <c r="P90" s="1" t="inlineStr"/>
+      <c r="Q90" s="1" t="inlineStr"/>
       <c r="R90" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S90" s="1" t="n"/>
@@ -7787,7 +7799,11 @@
           <t>VTZZ INDUSTRIA E COMÉRCIO LTDA</t>
         </is>
       </c>
-      <c r="H95" s="1" t="n"/>
+      <c r="H95" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I95" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -7801,7 +7817,7 @@
       </c>
       <c r="L95" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M95" s="1" t="inlineStr">
@@ -7812,7 +7828,7 @@
       <c r="N95" s="1" t="n"/>
       <c r="O95" s="1" t="n"/>
       <c r="P95" s="1" t="inlineStr"/>
-      <c r="Q95" s="1" t="n"/>
+      <c r="Q95" s="1" t="inlineStr"/>
       <c r="R95" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -9551,16 +9567,16 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>80158</v>
+        <v>80168</v>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Termos de Intimação</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>Pendência de Débito</t>
+          <t>Receita Federal</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
@@ -9570,29 +9586,29 @@
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>Verificar  a Pendência na conta fiscal  do IPI l 03.2026 saldo 47.157,32 -Darf e comprovante anexo para analise analisar o Mit. Após a análise, caso esteja tudo correto, por gentileza me informe. Solicitarei a correção por meio de processo junto à SEFAZ, com o apoio da Paralegal. Prazo 19.06.2026</t>
+          <t>A D&amp;T recebeu uma carta de cobrança referente aos débitos de IRPJ  e CSLL do 4º trimestre de 2021. A Inara informou que não deveria existir saldo devedor, pois houve compensação desses tributos à época.  Prazo 22.06.2026 (Dna Inara pede urgência na analise)</t>
         </is>
       </c>
       <c r="F118" s="1" t="n">
-        <v>4219</v>
+        <v>4220</v>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>REPUME REPUXAÇÃO E METALÚRGICA LTDA</t>
+          <t>D&amp;T BRASIL INDUSTRIA DE ELETRÔNICOS LTDA</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I118" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J118" s="2" t="n">
-        <v>46190.6549837963</v>
+        <v>46190.77325285879</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>46192</v>
@@ -9607,221 +9623,217 @@
           <t>Simone Marques</t>
         </is>
       </c>
-      <c r="N118" s="1" t="n"/>
+      <c r="N118" s="2" t="n">
+        <v>46192.44483642361</v>
+      </c>
       <c r="O118" s="2" t="n">
-        <v>46191.48537488426</v>
+        <v>46192.4474815625</v>
       </c>
       <c r="P118" s="1" t="inlineStr">
         <is>
-          <t>inascimento</t>
+          <t>pvolpe</t>
         </is>
       </c>
       <c r="Q118" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MIT Retificado- era diferença no codigo </t>
-        </is>
-      </c>
-      <c r="R118" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S118" s="1" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="1" t="n">
-        <v>80168</v>
-      </c>
-      <c r="B119" s="1" t="inlineStr">
-        <is>
-          <t>Termos de Intimação</t>
-        </is>
-      </c>
-      <c r="C119" s="1" t="inlineStr">
-        <is>
-          <t>Receita Federal</t>
-        </is>
-      </c>
-      <c r="D119" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E119" s="1" t="inlineStr">
-        <is>
-          <t>A D&amp;T recebeu uma carta de cobrança referente aos débitos de IRPJ  e CSLL do 4º trimestre de 2021. A Inara informou que não deveria existir saldo devedor, pois houve compensação desses tributos à época.  Prazo 22.06.2026 (Dna Inara pede urgência na analise)</t>
-        </is>
-      </c>
-      <c r="F119" s="1" t="n">
-        <v>4220</v>
-      </c>
-      <c r="G119" s="1" t="inlineStr">
-        <is>
-          <t>D&amp;T BRASIL INDUSTRIA DE ELETRÔNICOS LTDA</t>
-        </is>
-      </c>
-      <c r="H119" s="1" t="inlineStr">
-        <is>
-          <t>Priscila Volpe</t>
-        </is>
-      </c>
-      <c r="I119" s="1" t="inlineStr">
-        <is>
-          <t>EF - INDUSTRIA</t>
-        </is>
-      </c>
-      <c r="J119" s="2" t="n">
-        <v>46190.77325285879</v>
-      </c>
-      <c r="K119" s="2" t="n">
-        <v>46192</v>
-      </c>
-      <c r="L119" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M119" s="1" t="inlineStr">
-        <is>
-          <t>Simone Marques</t>
-        </is>
-      </c>
-      <c r="N119" s="2" t="n">
-        <v>46192.44483642361</v>
-      </c>
-      <c r="O119" s="2" t="n">
-        <v>46192.4474815625</v>
-      </c>
-      <c r="P119" s="1" t="inlineStr">
-        <is>
-          <t>pvolpe</t>
-        </is>
-      </c>
-      <c r="Q119" s="1" t="inlineStr">
         <is>
           <t>Bom Dia, prezados 
 A perdcomp foi indeferida no processo e a perdcomp na época fi realizada pela Marilia do CTB. 
 Por favor, abrir um chamado ao CTBI para a realização  da validação do indeferfimento.</t>
         </is>
       </c>
-      <c r="R119" s="1" t="inlineStr">
+      <c r="R118" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="S119" s="1" t="n"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="S118" s="1" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
         <v>80177</v>
       </c>
-      <c r="B120" s="1" t="inlineStr">
+      <c r="B119" s="1" t="inlineStr">
         <is>
           <t>Termos de Intimação</t>
         </is>
       </c>
-      <c r="C120" s="1" t="inlineStr">
+      <c r="C119" s="1" t="inlineStr">
         <is>
           <t>Receita Federal</t>
         </is>
       </c>
-      <c r="D120" s="1" t="inlineStr">
+      <c r="D119" s="1" t="inlineStr">
         <is>
           <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E120" s="1" t="inlineStr">
+      <c r="E119" s="1" t="inlineStr">
         <is>
           <t>Bom dia! Segue intimação. CARTA - COBRANÇA - COB/ECOB/DEVAT02</t>
         </is>
       </c>
-      <c r="F120" s="1" t="n">
+      <c r="F119" s="1" t="n">
         <v>4220</v>
       </c>
-      <c r="G120" s="1" t="inlineStr">
+      <c r="G119" s="1" t="inlineStr">
         <is>
           <t>D&amp;T BRASIL INDUSTRIA DE ELETRÔNICOS LTDA</t>
         </is>
       </c>
-      <c r="H120" s="1" t="inlineStr">
+      <c r="H119" s="1" t="inlineStr">
         <is>
           <t>Priscila Volpe</t>
         </is>
       </c>
-      <c r="I120" s="1" t="inlineStr">
+      <c r="I119" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n">
+      <c r="J119" s="2" t="n">
         <v>46191.38164320602</v>
       </c>
-      <c r="K120" s="2" t="n">
+      <c r="K119" s="2" t="n">
         <v>46203</v>
       </c>
-      <c r="L120" s="1" t="inlineStr">
+      <c r="L119" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M120" s="1" t="inlineStr">
+      <c r="M119" s="1" t="inlineStr">
         <is>
           <t>Ana Santana</t>
         </is>
       </c>
-      <c r="N120" s="1" t="n"/>
-      <c r="O120" s="2" t="n">
+      <c r="N119" s="1" t="n"/>
+      <c r="O119" s="2" t="n">
         <v>46192.44560752315</v>
       </c>
-      <c r="P120" s="1" t="inlineStr">
+      <c r="P119" s="1" t="inlineStr">
         <is>
           <t>pvolpe</t>
         </is>
       </c>
-      <c r="Q120" s="1" t="inlineStr">
+      <c r="Q119" s="1" t="inlineStr">
         <is>
           <t>Bom Dia, prezados 
 A perdcomp foi indeferida no processo e a perdcomp na época fi realizada pela Marilia do CTB. 
 Por favor, abrir um chamado ao CTBI para a realização  da validação do indeferfimento.</t>
         </is>
       </c>
+      <c r="R119" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S119" s="1" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>80112</v>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>Saldo Credor Incorreto</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>Saldo Credor Incorreto</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E120" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, verificar o transporte de saldo incorreto referente o mes 03/2026 conforme imagem anexa. Qualquer duvida sigo a disposição</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="n">
+        <v>4272</v>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>MERCADINHO J. SILVA - EIRELI</t>
+        </is>
+      </c>
+      <c r="H120" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
+      <c r="I120" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>46189.68182241898</v>
+      </c>
+      <c r="K120" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="L120" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M120" s="1" t="inlineStr">
+        <is>
+          <t>Rogerio Egidio</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>46190.48067052083</v>
+      </c>
+      <c r="O120" s="1" t="n"/>
+      <c r="P120" s="1" t="inlineStr"/>
+      <c r="Q120" s="1" t="inlineStr">
+        <is>
+          <t>verificando.</t>
+        </is>
+      </c>
       <c r="R120" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S120" s="1" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>80112</v>
+        <v>79799</v>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, verificar o transporte de saldo incorreto referente o mes 03/2026 conforme imagem anexa. Qualquer duvida sigo a disposição</t>
+          <t>Segue em anexo mensagem DEC Estadual do cliente: 4319 - SUPERMERCADO SANTA MARIA LTDAComplemento do Assunto: EFD substitutiva pendente de pagamento de taxa</t>
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>4272</v>
+        <v>4319</v>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO J. SILVA - EIRELI</t>
+          <t>SUPERMERCADO SANTA MARIA LTDA</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
@@ -9831,33 +9843,31 @@
       </c>
       <c r="I121" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J121" s="2" t="n">
-        <v>46189.68182241898</v>
+        <v>46182.64187924768</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="L121" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M121" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
-        </is>
-      </c>
-      <c r="N121" s="2" t="n">
-        <v>46190.48067052083</v>
-      </c>
+          <t>Leticia Queiroz</t>
+        </is>
+      </c>
+      <c r="N121" s="1" t="n"/>
       <c r="O121" s="1" t="n"/>
       <c r="P121" s="1" t="inlineStr"/>
       <c r="Q121" s="1" t="inlineStr">
         <is>
-          <t>verificando.</t>
+          <t>Verificando.</t>
         </is>
       </c>
       <c r="R121" s="1" t="inlineStr">
@@ -9865,20 +9875,24 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="S121" s="1" t="n"/>
+      <c r="S121" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>79799</v>
+        <v>79464</v>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Malha Fiscal</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Malha Fiscal</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
@@ -9888,49 +9902,51 @@
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>Segue em anexo mensagem DEC Estadual do cliente: 4319 - SUPERMERCADO SANTA MARIA LTDAComplemento do Assunto: EFD substitutiva pendente de pagamento de taxa</t>
+          <t>Boa tarde! Segue malha fiscal.  Divergências entre os valores a pagar de IRPJ e CSLL apurados na Escrituração Contábil Fiscal (ECF) e os valores informados em Declarações de Débitos e Créditos Tributários Federais (DCTF).QUAL O PRAZO PARA REGULARIZAÇÃO?Até o dia 31/07/2026.</t>
         </is>
       </c>
       <c r="F122" s="1" t="n">
-        <v>4319</v>
+        <v>4327</v>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO SANTA MARIA LTDA</t>
+          <t>ACCESS EVENTOS E VIAGENS LTDA</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="I122" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J122" s="2" t="n">
-        <v>46182.64187924768</v>
+        <v>46168.51368692129</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>46189</v>
+        <v>46170</v>
       </c>
       <c r="L122" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M122" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
-      <c r="N122" s="1" t="n"/>
+          <t>Ana Santana</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="n">
+        <v>46180.42641712963</v>
+      </c>
       <c r="O122" s="1" t="n"/>
       <c r="P122" s="1" t="inlineStr"/>
       <c r="Q122" s="1" t="inlineStr">
         <is>
-          <t>Verificando.</t>
+          <t>RETORNO ATÉ 25/06/2026 - EM ANALISE</t>
         </is>
       </c>
       <c r="R122" s="1" t="inlineStr">
@@ -9938,34 +9954,30 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="S122" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
+      <c r="S122" s="1" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>79464</v>
+        <v>80141</v>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>Malha Fiscal</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>Malha Fiscal</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Segue malha fiscal.  Divergências entre os valores a pagar de IRPJ e CSLL apurados na Escrituração Contábil Fiscal (ECF) e os valores informados em Declarações de Débitos e Créditos Tributários Federais (DCTF).QUAL O PRAZO PARA REGULARIZAÇÃO?Até o dia 31/07/2026.</t>
+          <t xml:space="preserve">Por gentileza encaminhar Balanço e DRE dos últimos 3 anos da ECD. </t>
         </is>
       </c>
       <c r="F123" s="1" t="n">
@@ -9978,50 +9990,54 @@
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Erika Santana</t>
         </is>
       </c>
       <c r="I123" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J123" s="2" t="n">
-        <v>46168.51368692129</v>
+        <v>46190.48975185185</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>46170</v>
+        <v>46191</v>
       </c>
       <c r="L123" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M123" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
-        </is>
-      </c>
-      <c r="N123" s="2" t="n">
-        <v>46180.42641712963</v>
-      </c>
-      <c r="O123" s="1" t="n"/>
-      <c r="P123" s="1" t="inlineStr"/>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N123" s="1" t="n"/>
+      <c r="O123" s="2" t="n">
+        <v>46195.71893035879</v>
+      </c>
+      <c r="P123" s="1" t="inlineStr">
+        <is>
+          <t>erikas</t>
+        </is>
+      </c>
       <c r="Q123" s="1" t="inlineStr">
         <is>
-          <t>RETORNO ATÉ 25/06/2026 - EM ANALISE</t>
+          <t>Segue</t>
         </is>
       </c>
       <c r="R123" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S123" s="1" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>80141</v>
+        <v>80471</v>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
@@ -10040,15 +10056,15 @@
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza encaminhar Balanço e DRE dos últimos 3 anos da ECD. </t>
+          <t>Por gentileza encaminhar balanço e DRE referente 2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="n">
-        <v>4327</v>
+        <v>4359</v>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>ACCESS EVENTOS E VIAGENS LTDA</t>
+          <t>ROBSON DE SOUSA LIMA COMERCIO DE ABRASIVOS</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
@@ -10062,14 +10078,14 @@
         </is>
       </c>
       <c r="J124" s="2" t="n">
-        <v>46190.48975185185</v>
+        <v>46196.41235833333</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>46191</v>
+        <v>46197</v>
       </c>
       <c r="L124" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M124" s="1" t="inlineStr">
@@ -10078,29 +10094,19 @@
         </is>
       </c>
       <c r="N124" s="1" t="n"/>
-      <c r="O124" s="2" t="n">
-        <v>46195.71893035879</v>
-      </c>
-      <c r="P124" s="1" t="inlineStr">
-        <is>
-          <t>erikas</t>
-        </is>
-      </c>
-      <c r="Q124" s="1" t="inlineStr">
-        <is>
-          <t>Segue</t>
-        </is>
-      </c>
+      <c r="O124" s="1" t="n"/>
+      <c r="P124" s="1" t="inlineStr"/>
+      <c r="Q124" s="1" t="inlineStr"/>
       <c r="R124" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S124" s="1" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>80471</v>
+        <v>79608</v>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
@@ -10114,90 +10120,104 @@
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza encaminhar balanço e DRE referente 2025</t>
+          <t>Bom dia!!Por gentileza, gerar BALANÇO E DRE 2025 da empresa 4371.</t>
         </is>
       </c>
       <c r="F125" s="1" t="n">
-        <v>4359</v>
+        <v>4371</v>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>ROBSON DE SOUSA LIMA COMERCIO DE ABRASIVOS</t>
-        </is>
-      </c>
-      <c r="H125" s="1" t="n"/>
+          <t>SUPERMERCADO XODO LTDA</t>
+        </is>
+      </c>
+      <c r="H125" s="1" t="inlineStr">
+        <is>
+          <t>Danielle Silva</t>
+        </is>
+      </c>
       <c r="I125" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J125" s="2" t="n">
-        <v>46196.41235833333</v>
+        <v>46175.47560806713</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>46197</v>
+        <v>46176</v>
       </c>
       <c r="L125" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M125" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N125" s="1" t="n"/>
-      <c r="O125" s="1" t="n"/>
-      <c r="P125" s="1" t="inlineStr"/>
-      <c r="Q125" s="1" t="n"/>
+      <c r="O125" s="2" t="n">
+        <v>46181.60018538195</v>
+      </c>
+      <c r="P125" s="1" t="inlineStr">
+        <is>
+          <t>danielles</t>
+        </is>
+      </c>
+      <c r="Q125" s="1" t="inlineStr">
+        <is>
+          <t>Enviado por e-mail dia 08/06/2026.</t>
+        </is>
+      </c>
       <c r="R125" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S125" s="1" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>79608</v>
+        <v>80213</v>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!!Por gentileza, gerar BALANÇO E DRE 2025 da empresa 4371.</t>
+          <t>Por gentileza enviar:Memoria de Calculo IRPJ/CSLL - 01/2025 a 05/2026Controle Patrimonial com Depreciação Mensal - 06/2021 a 05/2026</t>
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>4371</v>
+        <v>4396</v>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO XODO LTDA</t>
+          <t>SAMPA ATACADO DE GENEROS ALIMENTICIOS E BEBIDAS LTDA</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>Danielle Silva</t>
+          <t>Karina Santos</t>
         </is>
       </c>
       <c r="I126" s="1" t="inlineStr">
@@ -10206,38 +10226,28 @@
         </is>
       </c>
       <c r="J126" s="2" t="n">
-        <v>46175.47560806713</v>
+        <v>46191.64893958333</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>46176</v>
+        <v>46192</v>
       </c>
       <c r="L126" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M126" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N126" s="1" t="n"/>
-      <c r="O126" s="2" t="n">
-        <v>46181.60018538195</v>
-      </c>
-      <c r="P126" s="1" t="inlineStr">
-        <is>
-          <t>danielles</t>
-        </is>
-      </c>
-      <c r="Q126" s="1" t="inlineStr">
-        <is>
-          <t>Enviado por e-mail dia 08/06/2026.</t>
-        </is>
-      </c>
+      <c r="O126" s="1" t="n"/>
+      <c r="P126" s="1" t="inlineStr"/>
+      <c r="Q126" s="1" t="inlineStr"/>
       <c r="R126" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S126" s="1" t="n"/>
@@ -10281,7 +10291,7 @@
       </c>
       <c r="I127" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J127" s="2" t="n">
@@ -10292,7 +10302,7 @@
       </c>
       <c r="L127" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M127" s="1" t="inlineStr">
@@ -10300,9 +10310,7 @@
           <t>Rogerio Egidio</t>
         </is>
       </c>
-      <c r="N127" s="2" t="n">
-        <v>46195.56635929398</v>
-      </c>
+      <c r="N127" s="1" t="n"/>
       <c r="O127" s="1" t="n"/>
       <c r="P127" s="1" t="inlineStr"/>
       <c r="Q127" s="1" t="inlineStr">
@@ -10316,20 +10324,24 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="S127" s="1" t="n"/>
+      <c r="S127" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>80213</v>
+        <v>80228</v>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Documentação</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Solicitação de Documentação</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
@@ -10339,36 +10351,32 @@
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza enviar:Memoria de Calculo IRPJ/CSLL - 01/2025 a 05/2026Controle Patrimonial com Depreciação Mensal - 06/2021 a 05/2026</t>
+          <t>Bom dia!!Por gentileza, enviar MANAD ou resumo de Folha Mensal 06/2021 a 07/2024</t>
         </is>
       </c>
       <c r="F128" s="1" t="n">
-        <v>4396</v>
+        <v>4397</v>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>SAMPA ATACADO DE GENEROS ALIMENTICIOS E BEBIDAS LTDA</t>
-        </is>
-      </c>
-      <c r="H128" s="1" t="inlineStr">
-        <is>
-          <t>Karina Santos</t>
-        </is>
-      </c>
+          <t>SAMPATACADO DE GENEROS ALIMENTÍCIOS E BEBIDAS LTDA (FILIAL 01)</t>
+        </is>
+      </c>
+      <c r="H128" s="1" t="n"/>
       <c r="I128" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J128" s="2" t="n">
-        <v>46191.64893958333</v>
+        <v>46192.39995659722</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="L128" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M128" s="1" t="inlineStr">
@@ -10379,7 +10387,7 @@
       <c r="N128" s="1" t="n"/>
       <c r="O128" s="1" t="n"/>
       <c r="P128" s="1" t="inlineStr"/>
-      <c r="Q128" s="1" t="inlineStr"/>
+      <c r="Q128" s="1" t="n"/>
       <c r="R128" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -10389,72 +10397,86 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>80228</v>
+        <v>76499</v>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentação</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!!Por gentileza, enviar MANAD ou resumo de Folha Mensal 06/2021 a 07/2024</t>
+          <t>ADTO CLIENTES/FORNECEDORES/EMPRÉTIMOS A RECEBER	Avaliar valores constantes nestas contas de : ADTO FORNECEDOR, CLIENTES e EPRÉSTIMOS A RECEBER, se alguns destes valores poderiam ser empréstimos à sócios e que podem distribuidos em 2025, exceto adto de clientes que precisa identificação de qual cliente se refere a baixa considerando que o cliente não recebe se não emitir nota fiscal.PENDÊNCIA FEDERAL: SALDOS	"Cliente precisa apresentar ao cliente CND megativa, ocorre que na última reunião de 2/10/2025 foi apontado: Avaliar Pendência - Débito (SIEF)CNPJ: 14.237.012/0001-49Receita PA/Exerc. Dt. Vcto Vl. Original Sdo. Devedor Multa Juros Sdo. Dev. Cons. Situação0561-07 - IRRF 06/2021 20/07/2021 2.766,99 8,07 1,61 3,77 13,45 DEVEDOR0561-07 - IRRF 07/2021 20/08/2021 341,07 1,12 0,22 0,51 1,85 DEVEDOR1082-21 - CP-SEGUR. 2024 20/12/2024 7.090,18 95,94 19,18 9,30 124,42 DEVEDOR1646-21 - CP-PATRONAL 2024 20/12/2024 1.267,43 19,19 3,83 1,86 24,88 DEVEDORTomar medidas imediatas para regularização."</t>
         </is>
       </c>
       <c r="F129" s="1" t="n">
-        <v>4397</v>
+        <v>4422</v>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>SAMPATACADO DE GENEROS ALIMENTÍCIOS E BEBIDAS LTDA (FILIAL 01)</t>
-        </is>
-      </c>
-      <c r="H129" s="1" t="n"/>
+          <t>ALL SERVICE INSTALAÇÕES E SERVIÇOS LTDA</t>
+        </is>
+      </c>
+      <c r="H129" s="1" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
       <c r="I129" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J129" s="2" t="n">
-        <v>46192.39995659722</v>
+        <v>46030.51013417824</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>46195</v>
+        <v>46037</v>
       </c>
       <c r="L129" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M129" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Ana Santana</t>
         </is>
       </c>
       <c r="N129" s="1" t="n"/>
-      <c r="O129" s="1" t="n"/>
-      <c r="P129" s="1" t="inlineStr"/>
-      <c r="Q129" s="1" t="n"/>
+      <c r="O129" s="2" t="n">
+        <v>46113.60901288194</v>
+      </c>
+      <c r="P129" s="1" t="inlineStr">
+        <is>
+          <t>tatiana</t>
+        </is>
+      </c>
+      <c r="Q129" s="1" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="R129" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S129" s="1" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>76499</v>
+        <v>76368</v>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
@@ -10473,7 +10495,7 @@
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>ADTO CLIENTES/FORNECEDORES/EMPRÉTIMOS A RECEBER	Avaliar valores constantes nestas contas de : ADTO FORNECEDOR, CLIENTES e EPRÉSTIMOS A RECEBER, se alguns destes valores poderiam ser empréstimos à sócios e que podem distribuidos em 2025, exceto adto de clientes que precisa identificação de qual cliente se refere a baixa considerando que o cliente não recebe se não emitir nota fiscal.PENDÊNCIA FEDERAL: SALDOS	"Cliente precisa apresentar ao cliente CND megativa, ocorre que na última reunião de 2/10/2025 foi apontado: Avaliar Pendência - Débito (SIEF)CNPJ: 14.237.012/0001-49Receita PA/Exerc. Dt. Vcto Vl. Original Sdo. Devedor Multa Juros Sdo. Dev. Cons. Situação0561-07 - IRRF 06/2021 20/07/2021 2.766,99 8,07 1,61 3,77 13,45 DEVEDOR0561-07 - IRRF 07/2021 20/08/2021 341,07 1,12 0,22 0,51 1,85 DEVEDOR1082-21 - CP-SEGUR. 2024 20/12/2024 7.090,18 95,94 19,18 9,30 124,42 DEVEDOR1646-21 - CP-PATRONAL 2024 20/12/2024 1.267,43 19,19 3,83 1,86 24,88 DEVEDORTomar medidas imediatas para regularização."</t>
+          <t>PENDÊNCIA FEDERAL: SALDOS	"Cliente precisa apresentar ao cliente CND megativa, ocorre que na última reunião de 2/10/2025 foi apontado: Avaliar Pendência - Débito (SIEF)CNPJ: 14.237.012/0001-49Receita PA/Exerc. Dt. Vcto Vl. Original Sdo. Devedor Multa Juros Sdo. Dev. Cons. Situação0561-07 - IRRF 06/2021 20/07/2021 2.766,99 8,07 1,61 3,77 13,45 DEVEDOR0561-07 - IRRF 07/2021 20/08/2021 341,07 1,12 0,22 0,51 1,85 DEVEDOR1082-21 - CP-SEGUR. 2024 20/12/2024 7.090,18 95,94 19,18 9,30 124,42 DEVEDOR1646-21 - CP-PATRONAL 2024 20/12/2024 1.267,43 19,19 3,83 1,86 24,88 DEVEDORInfelizmente ainda pendente, Tomar medidas imediatas para regularização."</t>
         </is>
       </c>
       <c r="F130" s="1" t="n">
@@ -10495,10 +10517,10 @@
         </is>
       </c>
       <c r="J130" s="2" t="n">
-        <v>46030.51013417824</v>
+        <v>46024.65297202546</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>46037</v>
+        <v>46031</v>
       </c>
       <c r="L130" s="1" t="inlineStr">
         <is>
@@ -10512,7 +10534,7 @@
       </c>
       <c r="N130" s="1" t="n"/>
       <c r="O130" s="2" t="n">
-        <v>46113.60901288194</v>
+        <v>46113.60221331019</v>
       </c>
       <c r="P130" s="1" t="inlineStr">
         <is>
@@ -10533,16 +10555,16 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>76368</v>
+        <v>79643</v>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
@@ -10552,176 +10574,176 @@
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>PENDÊNCIA FEDERAL: SALDOS	"Cliente precisa apresentar ao cliente CND megativa, ocorre que na última reunião de 2/10/2025 foi apontado: Avaliar Pendência - Débito (SIEF)CNPJ: 14.237.012/0001-49Receita PA/Exerc. Dt. Vcto Vl. Original Sdo. Devedor Multa Juros Sdo. Dev. Cons. Situação0561-07 - IRRF 06/2021 20/07/2021 2.766,99 8,07 1,61 3,77 13,45 DEVEDOR0561-07 - IRRF 07/2021 20/08/2021 341,07 1,12 0,22 0,51 1,85 DEVEDOR1082-21 - CP-SEGUR. 2024 20/12/2024 7.090,18 95,94 19,18 9,30 124,42 DEVEDOR1646-21 - CP-PATRONAL 2024 20/12/2024 1.267,43 19,19 3,83 1,86 24,88 DEVEDORInfelizmente ainda pendente, Tomar medidas imediatas para regularização."</t>
+          <t>segue autorregularização do cliente 4457 - yara design e decoração ltda</t>
         </is>
       </c>
       <c r="F131" s="1" t="n">
-        <v>4422</v>
+        <v>4457</v>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>ALL SERVICE INSTALAÇÕES E SERVIÇOS LTDA</t>
+          <t>YARA DESIGN E DECORAÇÃO LTDA</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I131" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J131" s="2" t="n">
-        <v>46024.65297202546</v>
+        <v>46175.70834563657</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>46031</v>
+        <v>46182</v>
       </c>
       <c r="L131" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M131" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N131" s="1" t="n"/>
-      <c r="O131" s="2" t="n">
-        <v>46113.60221331019</v>
-      </c>
-      <c r="P131" s="1" t="inlineStr">
-        <is>
-          <t>tatiana</t>
-        </is>
-      </c>
+      <c r="O131" s="1" t="n"/>
+      <c r="P131" s="1" t="inlineStr"/>
       <c r="Q131" s="1" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t xml:space="preserve">Verificando. </t>
         </is>
       </c>
       <c r="R131" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S131" s="1" t="n"/>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="S131" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>79643</v>
+        <v>80147</v>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Conciliação de Contas</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Conciliação de Contas</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>segue autorregularização do cliente 4457 - yara design e decoração ltda</t>
+          <t>CAP  mês 04 - Necessário verificar esses 6 participantes que estão com divergência entre o arquivo do cliente e nosso Balancete.Necessário desse retorno HOJE para o cliente repassar aos investidores. Grato</t>
         </is>
       </c>
       <c r="F132" s="1" t="n">
-        <v>4457</v>
+        <v>4527</v>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>YARA DESIGN E DECORAÇÃO LTDA</t>
+          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Rachel Lima</t>
         </is>
       </c>
       <c r="I132" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J132" s="2" t="n">
-        <v>46175.70834563657</v>
+        <v>46190.50748202546</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>46182</v>
+        <v>46190</v>
       </c>
       <c r="L132" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M132" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="N132" s="1" t="n"/>
-      <c r="O132" s="1" t="n"/>
-      <c r="P132" s="1" t="inlineStr"/>
+      <c r="O132" s="2" t="n">
+        <v>46190.62353538194</v>
+      </c>
+      <c r="P132" s="1" t="inlineStr">
+        <is>
+          <t>rachell</t>
+        </is>
+      </c>
       <c r="Q132" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificando. </t>
+          <t>posicionado por e-mail, para o Gerente de Contas.</t>
         </is>
       </c>
       <c r="R132" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="S132" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S132" s="1" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>80147</v>
+        <v>77047</v>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Conciliação de Contas</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>Conciliação de Contas</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>CAP  mês 04 - Necessário verificar esses 6 participantes que estão com divergência entre o arquivo do cliente e nosso Balancete.Necessário desse retorno HOJE para o cliente repassar aos investidores. Grato</t>
+          <t>Correção Estoques:Por gentileza, corrigir os estoques no mês 12/2025 para o valor de R$ 401.327,29.</t>
         </is>
       </c>
       <c r="F133" s="1" t="n">
-        <v>4527</v>
+        <v>4545</v>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
+          <t>BF COMERCIO DE ARTIGOS PARA FESTAS, EMBALAGENS E ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>Rachel Lima</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="I133" s="1" t="inlineStr">
@@ -10730,10 +10752,10 @@
         </is>
       </c>
       <c r="J133" s="2" t="n">
-        <v>46190.50748202546</v>
+        <v>46059.65848981481</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>46190</v>
+        <v>46066</v>
       </c>
       <c r="L133" s="1" t="inlineStr">
         <is>
@@ -10742,21 +10764,21 @@
       </c>
       <c r="M133" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
+          <t>mtoledo</t>
         </is>
       </c>
       <c r="N133" s="1" t="n"/>
       <c r="O133" s="2" t="n">
-        <v>46190.62353538194</v>
+        <v>46113.6337659375</v>
       </c>
       <c r="P133" s="1" t="inlineStr">
         <is>
-          <t>rachell</t>
+          <t>tatiana</t>
         </is>
       </c>
       <c r="Q133" s="1" t="inlineStr">
         <is>
-          <t>posicionado por e-mail, para o Gerente de Contas.</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="R133" s="1" t="inlineStr">
@@ -10768,7 +10790,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>77047</v>
+        <v>76375</v>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
@@ -10787,32 +10809,32 @@
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>Correção Estoques:Por gentileza, corrigir os estoques no mês 12/2025 para o valor de R$ 401.327,29.</t>
+          <t>SIMPLES NACIONAL 09/2025	Cliente recebeu duas DARFs de valores diferentes e recolheu os valores d alí constantes, com a referência 09/2025. Levantar recolhimentos e confirmar autenticidade das remessas de duas guias para recolhimento e o que poderá ser feito com o saldo supostamente pago em duplicidade.</t>
         </is>
       </c>
       <c r="F134" s="1" t="n">
-        <v>4545</v>
+        <v>4593</v>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>BF COMERCIO DE ARTIGOS PARA FESTAS, EMBALAGENS E ALIMENTOS LTDA</t>
+          <t>EKIIM RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I134" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J134" s="2" t="n">
-        <v>46059.65848981481</v>
+        <v>46024.6679871875</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>46066</v>
+        <v>46031</v>
       </c>
       <c r="L134" s="1" t="inlineStr">
         <is>
@@ -10821,21 +10843,23 @@
       </c>
       <c r="M134" s="1" t="inlineStr">
         <is>
-          <t>mtoledo</t>
-        </is>
-      </c>
-      <c r="N134" s="1" t="n"/>
+          <t>Ana Santana</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="n">
+        <v>46122.57300196759</v>
+      </c>
       <c r="O134" s="2" t="n">
-        <v>46113.6337659375</v>
+        <v>46182.73449135417</v>
       </c>
       <c r="P134" s="1" t="inlineStr">
         <is>
-          <t>tatiana</t>
+          <t>pvolpe</t>
         </is>
       </c>
       <c r="Q134" s="1" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>resolvido</t>
         </is>
       </c>
       <c r="R134" s="1" t="inlineStr">
@@ -10847,7 +10871,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>76375</v>
+        <v>76806</v>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
@@ -10866,32 +10890,32 @@
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>SIMPLES NACIONAL 09/2025	Cliente recebeu duas DARFs de valores diferentes e recolheu os valores d alí constantes, com a referência 09/2025. Levantar recolhimentos e confirmar autenticidade das remessas de duas guias para recolhimento e o que poderá ser feito com o saldo supostamente pago em duplicidade.</t>
+          <t>Reclassificação AVCB	Reclassificar as despesas atualmente lançadas em "Seguro Incêndio" para a conta de despesas com AVCB (Documentação Predial), conforme solicitado pelo cliente.</t>
         </is>
       </c>
       <c r="F135" s="1" t="n">
-        <v>4593</v>
+        <v>4610</v>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>EKIIM RESTAURANTE LTDA</t>
+          <t>JARDIM ELÉTRICO PRODUÇÕES LTDA</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="I135" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J135" s="2" t="n">
-        <v>46024.6679871875</v>
+        <v>46048.46379232639</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>46031</v>
+        <v>46055</v>
       </c>
       <c r="L135" s="1" t="inlineStr">
         <is>
@@ -10903,20 +10927,18 @@
           <t>Ana Santana</t>
         </is>
       </c>
-      <c r="N135" s="2" t="n">
-        <v>46122.57300196759</v>
-      </c>
+      <c r="N135" s="1" t="n"/>
       <c r="O135" s="2" t="n">
-        <v>46182.73449135417</v>
+        <v>46113.62079417824</v>
       </c>
       <c r="P135" s="1" t="inlineStr">
         <is>
-          <t>pvolpe</t>
+          <t>tatiana</t>
         </is>
       </c>
       <c r="Q135" s="1" t="inlineStr">
         <is>
-          <t>resolvido</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="R135" s="1" t="inlineStr">
@@ -10928,7 +10950,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>76806</v>
+        <v>78342</v>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
@@ -10947,7 +10969,7 @@
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>Reclassificação AVCB	Reclassificar as despesas atualmente lançadas em "Seguro Incêndio" para a conta de despesas com AVCB (Documentação Predial), conforme solicitado pelo cliente.</t>
+          <t>Pendências estaduais	"Em consulta fiscal atualizada, foram identificadas pendências estaduais em aberto, por gentileza verificar"</t>
         </is>
       </c>
       <c r="F136" s="1" t="n">
@@ -10960,19 +10982,19 @@
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I136" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J136" s="2" t="n">
-        <v>46048.46379232639</v>
+        <v>46112.41193811342</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>46055</v>
+        <v>46119</v>
       </c>
       <c r="L136" s="1" t="inlineStr">
         <is>
@@ -10986,16 +11008,16 @@
       </c>
       <c r="N136" s="1" t="n"/>
       <c r="O136" s="2" t="n">
-        <v>46113.62079417824</v>
+        <v>46182.38611759259</v>
       </c>
       <c r="P136" s="1" t="inlineStr">
         <is>
-          <t>tatiana</t>
+          <t>pvolpe</t>
         </is>
       </c>
       <c r="Q136" s="1" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t xml:space="preserve">POR FAVOR, ANEXAR QUAIS AS PENDENCIAS </t>
         </is>
       </c>
       <c r="R136" s="1" t="inlineStr">
@@ -11007,26 +11029,26 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>78342</v>
+        <v>79995</v>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>Pendências estaduais	"Em consulta fiscal atualizada, foram identificadas pendências estaduais em aberto, por gentileza verificar"</t>
+          <t>Bom dia, a Jardim Elétrico entrou em contato conosco e informou que o rendimento de alguel esta incorreto. Peço a gentileza de verificarem o quanto antes.                  Segue os valores que nos foram passados Valor total 12 meses: R$ 347.731,94Retido R$ 84.797,94</t>
         </is>
       </c>
       <c r="F137" s="1" t="n">
@@ -11039,63 +11061,53 @@
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="I137" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J137" s="2" t="n">
-        <v>46112.41193811342</v>
+        <v>46188.37072855324</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>46119</v>
+        <v>46190</v>
       </c>
       <c r="L137" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M137" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N137" s="1" t="n"/>
-      <c r="O137" s="2" t="n">
-        <v>46182.38611759259</v>
-      </c>
-      <c r="P137" s="1" t="inlineStr">
-        <is>
-          <t>pvolpe</t>
-        </is>
-      </c>
-      <c r="Q137" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">POR FAVOR, ANEXAR QUAIS AS PENDENCIAS </t>
-        </is>
-      </c>
+      <c r="O137" s="1" t="n"/>
+      <c r="P137" s="1" t="inlineStr"/>
+      <c r="Q137" s="1" t="inlineStr"/>
       <c r="R137" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S137" s="1" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>79995</v>
+        <v>79894</v>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
@@ -11105,66 +11117,77 @@
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, a Jardim Elétrico entrou em contato conosco e informou que o rendimento de alguel esta incorreto. Peço a gentileza de verificarem o quanto antes.                  Segue os valores que nos foram passados Valor total 12 meses: R$ 347.731,94Retido R$ 84.797,94</t>
+          <t>J:\Importação\AUTO REGULARIZAÇÃO -DIFIS - VINHO NCM 2204\Daniel Oliveira\Memoria Calculo mes 052026Planilha com calculo atualizado para MAIO. Favor incluir na apuração de MAIO</t>
         </is>
       </c>
       <c r="F138" s="1" t="n">
-        <v>4610</v>
+        <v>4685</v>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>JARDIM ELÉTRICO PRODUÇÕES LTDA</t>
+          <t xml:space="preserve">EMPÓRIO SOLERA LTDA </t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I138" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J138" s="2" t="n">
-        <v>46188.37072855324</v>
+        <v>46184.47569001158</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>46190</v>
+        <v>46188</v>
       </c>
       <c r="L138" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M138" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="N138" s="1" t="n"/>
-      <c r="O138" s="1" t="n"/>
-      <c r="P138" s="1" t="inlineStr"/>
-      <c r="Q138" s="1" t="inlineStr"/>
+      <c r="O138" s="2" t="n">
+        <v>46189.53722265046</v>
+      </c>
+      <c r="P138" s="1" t="inlineStr">
+        <is>
+          <t>thaizao</t>
+        </is>
+      </c>
+      <c r="Q138" s="1" t="inlineStr">
+        <is>
+          <t>Valores lançados na apuração 05/2026 conforme planilha disponibilizada pelo GC.
+R$ 7.009.025,06</t>
+        </is>
+      </c>
       <c r="R138" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S138" s="1" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>79894</v>
+        <v>80227</v>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Documentação</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Solicitação de Documentação</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
@@ -11174,64 +11197,62 @@
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>J:\Importação\AUTO REGULARIZAÇÃO -DIFIS - VINHO NCM 2204\Daniel Oliveira\Memoria Calculo mes 052026Planilha com calculo atualizado para MAIO. Favor incluir na apuração de MAIO</t>
+          <t>Bom dia!!Por gentileza, enviar MANAD ou resumo de Folha Mensal 06/2021 a 05/2026.</t>
         </is>
       </c>
       <c r="F139" s="1" t="n">
-        <v>4685</v>
+        <v>4726</v>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPÓRIO SOLERA LTDA </t>
+          <t>SAMPATACADO DE GÊNEROS ALIMENTÍCIOS E BEBIDAS LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Natalia Silva</t>
         </is>
       </c>
       <c r="I139" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J139" s="2" t="n">
-        <v>46184.47569001158</v>
+        <v>46192.39938819445</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="L139" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M139" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N139" s="1" t="n"/>
-      <c r="O139" s="2" t="n">
-        <v>46189.53722265046</v>
-      </c>
-      <c r="P139" s="1" t="inlineStr">
-        <is>
-          <t>thaizao</t>
-        </is>
-      </c>
+      <c r="O139" s="1" t="n"/>
+      <c r="P139" s="1" t="inlineStr"/>
       <c r="Q139" s="1" t="inlineStr">
         <is>
-          <t>Valores lançados na apuração 05/2026 conforme planilha disponibilizada pelo GC.
-R$ 7.009.025,06</t>
+          <t xml:space="preserve">Boa tarde, Rogério !
+Pra quem devemos enviar ? </t>
         </is>
       </c>
       <c r="R139" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S139" s="1" t="n"/>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="S139" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -11304,16 +11325,16 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>80227</v>
+        <v>80517</v>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>Documentação</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentação</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
@@ -11323,54 +11344,43 @@
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!!Por gentileza, enviar MANAD ou resumo de Folha Mensal 06/2021 a 05/2026.</t>
+          <t>Por gentileza, providenciar regularização ocorrência de transporte de saldo credor incorretos nos períodos de 01/2024, 12/2024, 01/2025, 04/2026 conforme situação fiscal anexa.</t>
         </is>
       </c>
       <c r="F141" s="1" t="n">
-        <v>4726</v>
+        <v>4808</v>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>SAMPATACADO DE GÊNEROS ALIMENTÍCIOS E BEBIDAS LTDA (FILIAL 02)</t>
-        </is>
-      </c>
-      <c r="H141" s="1" t="inlineStr">
-        <is>
-          <t>Natalia Silva</t>
-        </is>
-      </c>
+          <t>DAN AGRO COMERCIAL LTDA</t>
+        </is>
+      </c>
+      <c r="H141" s="1" t="n"/>
       <c r="I141" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J141" s="2" t="n">
-        <v>46192.39938819445</v>
+        <v>46196.74807453703</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>46195</v>
+        <v>46213</v>
       </c>
       <c r="L141" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M141" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
-        </is>
-      </c>
-      <c r="N141" s="2" t="n">
-        <v>46195.56649575231</v>
-      </c>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N141" s="1" t="n"/>
       <c r="O141" s="1" t="n"/>
       <c r="P141" s="1" t="inlineStr"/>
-      <c r="Q141" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Boa tarde, Rogério !
-Pra quem devemos enviar ? </t>
-        </is>
-      </c>
+      <c r="Q141" s="1" t="n"/>
       <c r="R141" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -11380,16 +11390,16 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>80517</v>
+        <v>79660</v>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Retificação de Obrigação Acessória</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
@@ -11399,7 +11409,7 @@
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar regularização ocorrência de transporte de saldo credor incorretos nos períodos de 01/2024, 12/2024, 01/2025, 04/2026 conforme situação fiscal anexa.</t>
+          <t>Favor retificar declarações na Sefaz, consta transporte de saldo credor incorreto GIA 01/2024 - 12/2024 E 01/2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="n">
@@ -11410,21 +11420,25 @@
           <t>DAN AGRO COMERCIAL LTDA</t>
         </is>
       </c>
-      <c r="H142" s="1" t="n"/>
+      <c r="H142" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
       <c r="I142" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J142" s="2" t="n">
-        <v>46196.74807453703</v>
+        <v>46176.45003255787</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>46213</v>
+        <v>46183</v>
       </c>
       <c r="L142" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M142" s="1" t="inlineStr">
@@ -11432,10 +11446,16 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N142" s="1" t="n"/>
+      <c r="N142" s="2" t="n">
+        <v>46182.62023232639</v>
+      </c>
       <c r="O142" s="1" t="n"/>
       <c r="P142" s="1" t="inlineStr"/>
-      <c r="Q142" s="1" t="n"/>
+      <c r="Q142" s="1" t="inlineStr">
+        <is>
+          <t>Fazendo levando das ocorrências. Deve ser analisado pois pode influenciar em meses anteriores e posteriores</t>
+        </is>
+      </c>
       <c r="R142" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -11445,16 +11465,16 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>79660</v>
+        <v>80518</v>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Obrigação Acessória</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
@@ -11464,36 +11484,32 @@
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>Favor retificar declarações na Sefaz, consta transporte de saldo credor incorreto GIA 01/2024 - 12/2024 E 01/2025</t>
+          <t>Por gentileza, regularizar transporte de saldo credor incorreto 07/2025, 08/2025, 01/2026 e 02/2026 conforme situação fiscal anexa.</t>
         </is>
       </c>
       <c r="F143" s="1" t="n">
-        <v>4808</v>
+        <v>4810</v>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>DAN AGRO COMERCIAL LTDA</t>
-        </is>
-      </c>
-      <c r="H143" s="1" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>ECOFRUT AGRO COMERCIAL LTDA</t>
+        </is>
+      </c>
+      <c r="H143" s="1" t="n"/>
       <c r="I143" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J143" s="2" t="n">
-        <v>46176.45003255787</v>
+        <v>46196.76729903935</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>46183</v>
+        <v>46213</v>
       </c>
       <c r="L143" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M143" s="1" t="inlineStr">
@@ -11501,16 +11517,10 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N143" s="2" t="n">
-        <v>46182.62023232639</v>
-      </c>
+      <c r="N143" s="1" t="n"/>
       <c r="O143" s="1" t="n"/>
       <c r="P143" s="1" t="inlineStr"/>
-      <c r="Q143" s="1" t="inlineStr">
-        <is>
-          <t>Fazendo levando das ocorrências. Deve ser analisado pois pode influenciar em meses anteriores e posteriores</t>
-        </is>
-      </c>
+      <c r="Q143" s="1" t="n"/>
       <c r="R143" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -12821,16 +12831,16 @@
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
-        <v>79930</v>
+        <v>79948</v>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>Documentação Contábil</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
@@ -12840,7 +12850,7 @@
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderiam providenciar Última declaração do IRPJ entregue do cliente CEREALISTA</t>
+          <t>Por gentileza, poderiam providenciar o BALANÇO E DRE da empresa 5101 - CEREALISTA IDEAL1) Balancete atualizado2) DRE - comprovante de faturamento; Demonstrativo de resultado do exercício 2025informo que tentei gerar o balanço e a DRE porem esta incorreto os resultados apresentados</t>
         </is>
       </c>
       <c r="F161" s="1" t="n">
@@ -12862,10 +12872,10 @@
         </is>
       </c>
       <c r="J161" s="2" t="n">
-        <v>46184.70223510417</v>
+        <v>46185.47699907408</v>
       </c>
       <c r="K161" s="2" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="L161" s="1" t="inlineStr">
         <is>
@@ -12877,9 +12887,11 @@
           <t>Leticia Queiroz</t>
         </is>
       </c>
-      <c r="N161" s="1" t="n"/>
+      <c r="N161" s="2" t="n">
+        <v>46189.73606628472</v>
+      </c>
       <c r="O161" s="2" t="n">
-        <v>46192.46905616898</v>
+        <v>46191.60069417824</v>
       </c>
       <c r="P161" s="1" t="inlineStr">
         <is>
@@ -12888,7 +12900,7 @@
       </c>
       <c r="Q161" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, não entendi, favor ser mais e especifica, seria memoria de cálculo ou alguma obrigação acessória como Sped????? </t>
+          <t>segue balanço e dre 2025</t>
         </is>
       </c>
       <c r="R161" s="1" t="inlineStr">
@@ -12900,16 +12912,16 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>79948</v>
+        <v>79930</v>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>Documentação Contábil</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
@@ -12919,7 +12931,7 @@
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, poderiam providenciar o BALANÇO E DRE da empresa 5101 - CEREALISTA IDEAL1) Balancete atualizado2) DRE - comprovante de faturamento; Demonstrativo de resultado do exercício 2025informo que tentei gerar o balanço e a DRE porem esta incorreto os resultados apresentados</t>
+          <t>Por gentileza, poderiam providenciar Última declaração do IRPJ entregue do cliente CEREALISTA</t>
         </is>
       </c>
       <c r="F162" s="1" t="n">
@@ -12941,10 +12953,10 @@
         </is>
       </c>
       <c r="J162" s="2" t="n">
-        <v>46185.47699907408</v>
+        <v>46184.70223510417</v>
       </c>
       <c r="K162" s="2" t="n">
-        <v>46188</v>
+        <v>46185</v>
       </c>
       <c r="L162" s="1" t="inlineStr">
         <is>
@@ -12956,11 +12968,9 @@
           <t>Leticia Queiroz</t>
         </is>
       </c>
-      <c r="N162" s="2" t="n">
-        <v>46189.73606628472</v>
-      </c>
+      <c r="N162" s="1" t="n"/>
       <c r="O162" s="2" t="n">
-        <v>46191.60069417824</v>
+        <v>46192.46905616898</v>
       </c>
       <c r="P162" s="1" t="inlineStr">
         <is>
@@ -12969,7 +12979,7 @@
       </c>
       <c r="Q162" s="1" t="inlineStr">
         <is>
-          <t>segue balanço e dre 2025</t>
+          <t xml:space="preserve">Bom dia, não entendi, favor ser mais e especifica, seria memoria de cálculo ou alguma obrigação acessória como Sped????? </t>
         </is>
       </c>
       <c r="R162" s="1" t="inlineStr">
@@ -16630,7 +16640,7 @@
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
-        <v>80247</v>
+        <v>80249</v>
       </c>
       <c r="B210" s="1" t="inlineStr">
         <is>
@@ -16649,7 +16659,7 @@
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>Prezadas, periodo ex-contador.cliente com CNPJ inapto URGENTE!com autorização da diretoria (anexo).providenciar a entrega em branco das obrigações abaixo.ECF anual 2023 - DCTF mensal 2023 março, abril, maio, junho, julho - DCTF mensal 2022 fevereiro - DCTF mensal 2021 novembro e dezembro - DCTF mensal 2022 janeiro - DCTF mensal 2021 outubro. .</t>
+          <t xml:space="preserve">Prezadas, periodo ex-contador.cliente com CNPJ inapto URGENTE!com autorização da diretoria (anexo).providenciar a entrega em branco das obrigações abaixo.PGDAS - mensal 2024 fevereiro - EFD Contribuições 2021 outubro, novembro e dezembro. </t>
         </is>
       </c>
       <c r="F210" s="1" t="n">
@@ -16660,21 +16670,25 @@
           <t>APOLO ARTES LTDA</t>
         </is>
       </c>
-      <c r="H210" s="1" t="n"/>
+      <c r="H210" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="I210" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J210" s="2" t="n">
-        <v>46192.65557515046</v>
+        <v>46192.65839660879</v>
       </c>
       <c r="K210" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="L210" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M210" s="1" t="inlineStr">
@@ -16683,93 +16697,89 @@
         </is>
       </c>
       <c r="N210" s="1" t="n"/>
-      <c r="O210" s="1" t="n"/>
-      <c r="P210" s="1" t="inlineStr"/>
-      <c r="Q210" s="1" t="n"/>
-      <c r="R210" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="S210" s="1" t="n"/>
-    </row>
-    <row r="211">
-      <c r="A211" s="1" t="n">
-        <v>80249</v>
-      </c>
-      <c r="B211" s="1" t="inlineStr">
-        <is>
-          <t>Omissão de Obrigações Acessórias</t>
-        </is>
-      </c>
-      <c r="C211" s="1" t="inlineStr">
-        <is>
-          <t>Omissão de Obrigações Acessórias</t>
-        </is>
-      </c>
-      <c r="D211" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E211" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezadas, periodo ex-contador.cliente com CNPJ inapto URGENTE!com autorização da diretoria (anexo).providenciar a entrega em branco das obrigações abaixo.PGDAS - mensal 2024 fevereiro - EFD Contribuições 2021 outubro, novembro e dezembro. </t>
-        </is>
-      </c>
-      <c r="F211" s="1" t="n">
-        <v>5729</v>
-      </c>
-      <c r="G211" s="1" t="inlineStr">
-        <is>
-          <t>APOLO ARTES LTDA</t>
-        </is>
-      </c>
-      <c r="H211" s="1" t="inlineStr">
-        <is>
-          <t>Priscila Volpe</t>
-        </is>
-      </c>
-      <c r="I211" s="1" t="inlineStr">
-        <is>
-          <t>EF - INDUSTRIA</t>
-        </is>
-      </c>
-      <c r="J211" s="2" t="n">
-        <v>46192.65839660879</v>
-      </c>
-      <c r="K211" s="2" t="n">
-        <v>46195</v>
-      </c>
-      <c r="L211" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M211" s="1" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N211" s="1" t="n"/>
-      <c r="O211" s="2" t="n">
+      <c r="O210" s="2" t="n">
         <v>46195.7003940162</v>
       </c>
-      <c r="P211" s="1" t="inlineStr">
+      <c r="P210" s="1" t="inlineStr">
         <is>
           <t>pvolpe</t>
         </is>
       </c>
-      <c r="Q211" s="1" t="inlineStr">
+      <c r="Q210" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">boa tarde, 
 Sped contribuição entregue em 25/05/2022 e DAS 02/2024 entregue dentro do prazo correto. 
 não há pedencias pro parte do fiscal </t>
         </is>
       </c>
+      <c r="R210" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S210" s="1" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="n">
+        <v>80247</v>
+      </c>
+      <c r="B211" s="1" t="inlineStr">
+        <is>
+          <t>Omissão de Obrigações Acessórias</t>
+        </is>
+      </c>
+      <c r="C211" s="1" t="inlineStr">
+        <is>
+          <t>Omissão de Obrigações Acessórias</t>
+        </is>
+      </c>
+      <c r="D211" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E211" s="1" t="inlineStr">
+        <is>
+          <t>Prezadas, periodo ex-contador.cliente com CNPJ inapto URGENTE!com autorização da diretoria (anexo).providenciar a entrega em branco das obrigações abaixo.ECF anual 2023 - DCTF mensal 2023 março, abril, maio, junho, julho - DCTF mensal 2022 fevereiro - DCTF mensal 2021 novembro e dezembro - DCTF mensal 2022 janeiro - DCTF mensal 2021 outubro. .</t>
+        </is>
+      </c>
+      <c r="F211" s="1" t="n">
+        <v>5729</v>
+      </c>
+      <c r="G211" s="1" t="inlineStr">
+        <is>
+          <t>APOLO ARTES LTDA</t>
+        </is>
+      </c>
+      <c r="H211" s="1" t="n"/>
+      <c r="I211" s="1" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="n">
+        <v>46192.65557515046</v>
+      </c>
+      <c r="K211" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="L211" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M211" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N211" s="1" t="n"/>
+      <c r="O211" s="1" t="n"/>
+      <c r="P211" s="1" t="inlineStr"/>
+      <c r="Q211" s="1" t="n"/>
       <c r="R211" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S211" s="1" t="n"/>
@@ -18456,7 +18466,7 @@
       </c>
       <c r="L233" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M233" s="1" t="inlineStr">
@@ -18465,8 +18475,14 @@
         </is>
       </c>
       <c r="N233" s="1" t="n"/>
-      <c r="O233" s="1" t="n"/>
-      <c r="P233" s="1" t="inlineStr"/>
+      <c r="O233" s="2" t="n">
+        <v>46197.37187415509</v>
+      </c>
+      <c r="P233" s="1" t="inlineStr">
+        <is>
+          <t>inascimento</t>
+        </is>
+      </c>
       <c r="Q233" s="1" t="inlineStr">
         <is>
           <t>enviado por email 05/06</t>
@@ -18474,7 +18490,7 @@
       </c>
       <c r="R233" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S233" s="1" t="n"/>
@@ -19266,26 +19282,26 @@
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
-        <v>80136</v>
+        <v>77014</v>
       </c>
       <c r="B244" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C244" s="1" t="inlineStr">
         <is>
-          <t>Saldo Credor Incorreto</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D244" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza verificar saldo credor incorreto. </t>
+          <t>E-cac	Debito em aberto 10/2025 - IRRF e CSRF - enviar para o cliente!Despesas - Assistência Medica	Por favor, Conta 872 - verificar lançamentos (vale refeição lançado errado) e dois laçamento de assist. medica. Foi feito?Comissões	Por favor, Conta 3853 - verificar lançamentos, valor muito abaixo dos meses anteriores. Foi feito?Comissões	Por favor, Conta 948 - Conta igual a 3853 verificar. Foi feito?Pro-LaborePor favor, Conta 1001- sem lançamento na DRE (verificar). Foi feito?</t>
         </is>
       </c>
       <c r="F244" s="1" t="n">
@@ -19298,44 +19314,54 @@
       </c>
       <c r="H244" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Erika Santana</t>
         </is>
       </c>
       <c r="I244" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J244" s="2" t="n">
-        <v>46190.46544413194</v>
+        <v>46057.5935528125</v>
       </c>
       <c r="K244" s="2" t="n">
-        <v>46192</v>
+        <v>46064</v>
       </c>
       <c r="L244" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M244" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Ana Santana</t>
         </is>
       </c>
       <c r="N244" s="1" t="n"/>
-      <c r="O244" s="1" t="n"/>
-      <c r="P244" s="1" t="inlineStr"/>
-      <c r="Q244" s="1" t="inlineStr"/>
+      <c r="O244" s="2" t="n">
+        <v>46113.6484346875</v>
+      </c>
+      <c r="P244" s="1" t="inlineStr">
+        <is>
+          <t>erikas</t>
+        </is>
+      </c>
+      <c r="Q244" s="1" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
       <c r="R244" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S244" s="1" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
-        <v>77014</v>
+        <v>77015</v>
       </c>
       <c r="B245" s="1" t="inlineStr">
         <is>
@@ -19354,7 +19380,7 @@
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>E-cac	Debito em aberto 10/2025 - IRRF e CSRF - enviar para o cliente!Despesas - Assistência Medica	Por favor, Conta 872 - verificar lançamentos (vale refeição lançado errado) e dois laçamento de assist. medica. Foi feito?Comissões	Por favor, Conta 3853 - verificar lançamentos, valor muito abaixo dos meses anteriores. Foi feito?Comissões	Por favor, Conta 948 - Conta igual a 3853 verificar. Foi feito?Pro-LaborePor favor, Conta 1001- sem lançamento na DRE (verificar). Foi feito?</t>
+          <t>Fiscal	EFD 10, 11 e 12/2025 - Transporte de Saldo Credor Incorreto, corrigir por favor!</t>
         </is>
       </c>
       <c r="F245" s="1" t="n">
@@ -19367,23 +19393,23 @@
       </c>
       <c r="H245" s="1" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I245" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J245" s="2" t="n">
-        <v>46057.5935528125</v>
+        <v>46057.59395454861</v>
       </c>
       <c r="K245" s="2" t="n">
         <v>46064</v>
       </c>
       <c r="L245" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M245" s="1" t="inlineStr">
@@ -19391,49 +19417,45 @@
           <t>Ana Santana</t>
         </is>
       </c>
-      <c r="N245" s="1" t="n"/>
-      <c r="O245" s="2" t="n">
-        <v>46113.6484346875</v>
-      </c>
-      <c r="P245" s="1" t="inlineStr">
-        <is>
-          <t>erikas</t>
-        </is>
-      </c>
+      <c r="N245" s="2" t="n">
+        <v>46182.65223278935</v>
+      </c>
+      <c r="O245" s="1" t="n"/>
+      <c r="P245" s="1" t="inlineStr"/>
       <c r="Q245" s="1" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Operação em execução do processo de retificação - prazo 30/06/2026</t>
         </is>
       </c>
       <c r="R245" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S245" s="1" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
-        <v>77015</v>
+        <v>80136</v>
       </c>
       <c r="B246" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="C246" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Saldo Credor Incorreto</t>
         </is>
       </c>
       <c r="D246" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>Fiscal	EFD 10, 11 e 12/2025 - Transporte de Saldo Credor Incorreto, corrigir por favor!</t>
+          <t xml:space="preserve">Por gentileza verificar saldo credor incorreto. </t>
         </is>
       </c>
       <c r="F246" s="1" t="n">
@@ -19446,7 +19468,7 @@
       </c>
       <c r="H246" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I246" s="1" t="inlineStr">
@@ -19455,31 +19477,25 @@
         </is>
       </c>
       <c r="J246" s="2" t="n">
-        <v>46057.59395454861</v>
+        <v>46190.46544413194</v>
       </c>
       <c r="K246" s="2" t="n">
-        <v>46064</v>
+        <v>46192</v>
       </c>
       <c r="L246" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M246" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
-        </is>
-      </c>
-      <c r="N246" s="2" t="n">
-        <v>46182.65223278935</v>
-      </c>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N246" s="1" t="n"/>
       <c r="O246" s="1" t="n"/>
       <c r="P246" s="1" t="inlineStr"/>
-      <c r="Q246" s="1" t="inlineStr">
-        <is>
-          <t>Operação em execução do processo de retificação - prazo 30/06/2026</t>
-        </is>
-      </c>
+      <c r="Q246" s="1" t="inlineStr"/>
       <c r="R246" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21835,7 +21851,11 @@
           <t>RESOLVE MIDIA SOLUTIONS LTDA</t>
         </is>
       </c>
-      <c r="H277" s="1" t="n"/>
+      <c r="H277" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I277" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -21849,7 +21869,7 @@
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
@@ -21860,7 +21880,7 @@
       <c r="N277" s="1" t="n"/>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="inlineStr"/>
-      <c r="Q277" s="1" t="n"/>
+      <c r="Q277" s="1" t="inlineStr"/>
       <c r="R277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22498,7 +22518,11 @@
           <t>CONCEITO LOCADORA LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H286" s="1" t="n"/>
+      <c r="H286" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I286" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -22512,7 +22536,7 @@
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M286" s="1" t="inlineStr">
@@ -22523,7 +22547,7 @@
       <c r="N286" s="1" t="n"/>
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="inlineStr"/>
-      <c r="Q286" s="1" t="n"/>
+      <c r="Q286" s="1" t="inlineStr"/>
       <c r="R286" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24461,154 +24485,140 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
+        <v>80522</v>
+      </c>
+      <c r="B312" s="1" t="inlineStr">
+        <is>
+          <t>Retificação de Obrigação Acessória</t>
+        </is>
+      </c>
+      <c r="C312" s="1" t="inlineStr">
+        <is>
+          <t>Retificação de Obrigação Acessória</t>
+        </is>
+      </c>
+      <c r="D312" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E312" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia, por gentileza verificar mensagem recebida no DEC referente irregularidade na EFD 05/2026.</t>
+        </is>
+      </c>
+      <c r="F312" s="1" t="n">
+        <v>6880</v>
+      </c>
+      <c r="G312" s="1" t="inlineStr">
+        <is>
+          <t>ROBSON DE SOUSA LIMA COMERCIO DE ABRASIVOS (FILIAL)</t>
+        </is>
+      </c>
+      <c r="H312" s="1" t="n"/>
+      <c r="I312" s="1" t="inlineStr">
+        <is>
+          <t>EF - INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="n">
+        <v>46197.36092913194</v>
+      </c>
+      <c r="K312" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="L312" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M312" s="1" t="inlineStr">
+        <is>
+          <t>Beatriz Rangel</t>
+        </is>
+      </c>
+      <c r="N312" s="1" t="n"/>
+      <c r="O312" s="1" t="n"/>
+      <c r="P312" s="1" t="inlineStr"/>
+      <c r="Q312" s="1" t="n"/>
+      <c r="R312" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="S312" s="1" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="1" t="n">
         <v>78847</v>
       </c>
-      <c r="B312" s="1" t="inlineStr">
+      <c r="B313" s="1" t="inlineStr">
         <is>
           <t>Reunião externa</t>
         </is>
       </c>
-      <c r="C312" s="1" t="inlineStr">
+      <c r="C313" s="1" t="inlineStr">
         <is>
           <t>Inclusão de Ata</t>
         </is>
       </c>
-      <c r="D312" s="1" t="inlineStr">
+      <c r="D313" s="1" t="inlineStr">
         <is>
           <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E312" s="1" t="inlineStr">
+      <c r="E313" s="1" t="inlineStr">
         <is>
           <t>Verificar o sindicato Patronal, lembrando que o cliente não abre mais aos domingosCliente tem dificuldade sobre os recebimentos dos atestados demissionaisApresentar ao cliente sobre as obrigações da empresa5350 - AKAFER</t>
         </is>
       </c>
-      <c r="F312" s="1" t="n">
+      <c r="F313" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G312" s="1" t="n"/>
-      <c r="H312" s="1" t="inlineStr">
+      <c r="G313" s="1" t="n"/>
+      <c r="H313" s="1" t="inlineStr">
         <is>
           <t>Mauricio Lermen</t>
         </is>
       </c>
-      <c r="I312" s="1" t="inlineStr">
+      <c r="I313" s="1" t="inlineStr">
         <is>
           <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
-      <c r="J312" s="2" t="n">
+      <c r="J313" s="2" t="n">
         <v>46134.66965193287</v>
       </c>
-      <c r="K312" s="2" t="n">
+      <c r="K313" s="2" t="n">
         <v>46142</v>
       </c>
-      <c r="L312" s="1" t="inlineStr">
+      <c r="L313" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M312" s="1" t="inlineStr">
+      <c r="M313" s="1" t="inlineStr">
         <is>
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N312" s="2" t="n">
+      <c r="N313" s="2" t="n">
         <v>46171.59439259259</v>
       </c>
-      <c r="O312" s="2" t="n">
+      <c r="O313" s="2" t="n">
         <v>46176.76352538195</v>
       </c>
-      <c r="P312" s="1" t="inlineStr">
+      <c r="P313" s="1" t="inlineStr">
         <is>
           <t>mauricio</t>
         </is>
       </c>
-      <c r="Q312" s="1" t="inlineStr">
+      <c r="Q313" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">EM ATENDIMENTO
 </t>
         </is>
       </c>
-      <c r="R312" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="S312" s="1" t="n"/>
-    </row>
-    <row r="313">
-      <c r="A313" s="1" t="n">
-        <v>78425</v>
-      </c>
-      <c r="B313" s="1" t="inlineStr">
-        <is>
-          <t>Ata de Reunião</t>
-        </is>
-      </c>
-      <c r="C313" s="1" t="inlineStr">
-        <is>
-          <t>Inclusão de Ata</t>
-        </is>
-      </c>
-      <c r="D313" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E313" s="1" t="inlineStr">
-        <is>
-          <t>Verificar valores ref. 11/2025 em aberto qual a origem dos débitos e enviar ao cliente para pagamentoverificar SITUAÇÃO FISCAL</t>
-        </is>
-      </c>
-      <c r="F313" s="1" t="n">
-        <v>1180</v>
-      </c>
-      <c r="G313" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO YAMATO LTDA</t>
-        </is>
-      </c>
-      <c r="H313" s="1" t="inlineStr">
-        <is>
-          <t>Renata Cavalheiro</t>
-        </is>
-      </c>
-      <c r="I313" s="1" t="inlineStr">
-        <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
-        </is>
-      </c>
-      <c r="J313" s="2" t="n">
-        <v>46113.68943684028</v>
-      </c>
-      <c r="K313" s="2" t="n">
-        <v>46120</v>
-      </c>
-      <c r="L313" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M313" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N313" s="1" t="n"/>
-      <c r="O313" s="2" t="n">
-        <v>46114.6203158912</v>
-      </c>
-      <c r="P313" s="1" t="inlineStr">
-        <is>
-          <t>renatac</t>
-        </is>
-      </c>
-      <c r="Q313" s="1" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
       <c r="R313" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -24618,137 +24628,220 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>80353</v>
+        <v>78425</v>
       </c>
       <c r="B314" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C314" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D314" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E314" s="1" t="inlineStr">
         <is>
-          <t>Cliente solicitou a atualização da DCTFWeb, pois não conseguiu pagar no vencimento (19/06/2026).</t>
+          <t>Verificar valores ref. 11/2025 em aberto qual a origem dos débitos e enviar ao cliente para pagamentoverificar SITUAÇÃO FISCAL</t>
         </is>
       </c>
       <c r="F314" s="1" t="n">
-        <v>1768</v>
+        <v>1180</v>
       </c>
       <c r="G314" s="1" t="inlineStr">
         <is>
-          <t>FIESTA LTDA</t>
-        </is>
-      </c>
-      <c r="H314" s="1" t="n"/>
+          <t>SUPERMERCADO YAMATO LTDA</t>
+        </is>
+      </c>
+      <c r="H314" s="1" t="inlineStr">
+        <is>
+          <t>Renata Cavalheiro</t>
+        </is>
+      </c>
       <c r="I314" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J314" s="2" t="n">
-        <v>46195.4976246875</v>
+        <v>46113.68943684028</v>
       </c>
       <c r="K314" s="2" t="n">
-        <v>46196</v>
+        <v>46120</v>
       </c>
       <c r="L314" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M314" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N314" s="1" t="n"/>
-      <c r="O314" s="1" t="n"/>
-      <c r="P314" s="1" t="inlineStr"/>
-      <c r="Q314" s="1" t="n"/>
+      <c r="O314" s="2" t="n">
+        <v>46114.6203158912</v>
+      </c>
+      <c r="P314" s="1" t="inlineStr">
+        <is>
+          <t>renatac</t>
+        </is>
+      </c>
+      <c r="Q314" s="1" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
       <c r="R314" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S314" s="1" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
+        <v>80353</v>
+      </c>
+      <c r="B315" s="1" t="inlineStr">
+        <is>
+          <t>DCTFWeb</t>
+        </is>
+      </c>
+      <c r="C315" s="1" t="inlineStr">
+        <is>
+          <t>DCTFWeb</t>
+        </is>
+      </c>
+      <c r="D315" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E315" s="1" t="inlineStr">
+        <is>
+          <t>Cliente solicitou a atualização da DCTFWeb, pois não conseguiu pagar no vencimento (19/06/2026).</t>
+        </is>
+      </c>
+      <c r="F315" s="1" t="n">
+        <v>1768</v>
+      </c>
+      <c r="G315" s="1" t="inlineStr">
+        <is>
+          <t>FIESTA LTDA</t>
+        </is>
+      </c>
+      <c r="H315" s="1" t="inlineStr">
+        <is>
+          <t>Ana Barbosa</t>
+        </is>
+      </c>
+      <c r="I315" s="1" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL VAREJO</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="n">
+        <v>46195.4976246875</v>
+      </c>
+      <c r="K315" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="L315" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M315" s="1" t="inlineStr">
+        <is>
+          <t>Rodrigo Rego</t>
+        </is>
+      </c>
+      <c r="N315" s="1" t="n"/>
+      <c r="O315" s="1" t="n"/>
+      <c r="P315" s="1" t="inlineStr"/>
+      <c r="Q315" s="1" t="inlineStr"/>
+      <c r="R315" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="S315" s="1" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="1" t="n">
         <v>79943</v>
       </c>
-      <c r="B315" s="1" t="inlineStr">
+      <c r="B316" s="1" t="inlineStr">
         <is>
           <t>Ata de Reunião</t>
         </is>
       </c>
-      <c r="C315" s="1" t="inlineStr">
+      <c r="C316" s="1" t="inlineStr">
         <is>
           <t>Inclusão de Ata</t>
         </is>
       </c>
-      <c r="D315" s="1" t="inlineStr">
+      <c r="D316" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
-      <c r="E315" s="1" t="inlineStr">
+      <c r="E316" s="1" t="inlineStr">
         <is>
           <t>* Cliente está realizando a manutenção predial referente ao imóvel aonde localiza-se a Interfrios. Favor verificar e reclassificar tudo com DESPESA E NÃO BENFEITORIA EM IMÓVEIS DE TERCEIROS E ATÉ MESMO IMOBILIZADO - FOI RECLASSIFICADO?* Notas do Ifood, referentes a comissão de outubro, novembro e dezembro não foram enviadas. Em Janeiro eles enviaram NOTAS DE DÉBITO referentes ao ultimo trimestre.* Preciso trazer para o cliente no próximo mês DFC do ano de 2024 para auxiliar o cliente em suas tomadas de decisão - Teremos condições de apresentar?</t>
         </is>
       </c>
-      <c r="F315" s="1" t="n">
+      <c r="F316" s="1" t="n">
         <v>2502</v>
       </c>
-      <c r="G315" s="1" t="inlineStr">
+      <c r="G316" s="1" t="inlineStr">
         <is>
           <t>INTERFRIOS COMÉRCIO DE FRIOS E LATICÍNIOS EIRELI</t>
         </is>
       </c>
-      <c r="H315" s="1" t="inlineStr">
+      <c r="H316" s="1" t="inlineStr">
         <is>
           <t>Edileide Dias</t>
         </is>
       </c>
-      <c r="I315" s="1" t="inlineStr">
+      <c r="I316" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
-      <c r="J315" s="2" t="n">
+      <c r="J316" s="2" t="n">
         <v>46185.4118128125</v>
       </c>
-      <c r="K315" s="2" t="n">
+      <c r="K316" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="L315" s="1" t="inlineStr">
+      <c r="L316" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M315" s="1" t="inlineStr">
+      <c r="M316" s="1" t="inlineStr">
         <is>
           <t>Rodrigo Rego</t>
         </is>
       </c>
-      <c r="N315" s="1" t="n"/>
-      <c r="O315" s="2" t="n">
+      <c r="N316" s="1" t="n"/>
+      <c r="O316" s="2" t="n">
         <v>46185.57578209491</v>
       </c>
-      <c r="P315" s="1" t="inlineStr">
+      <c r="P316" s="1" t="inlineStr">
         <is>
           <t>edileide</t>
         </is>
       </c>
-      <c r="Q315" s="1" t="inlineStr">
+      <c r="Q316" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> Cliente está realizando a manutenção predial referente ao imóvel aonde localiza-se a Interfrios. Favor verificar e reclassificar tudo com DESPESA E NÃO BENFEITORIA EM IMÓVEIS DE TERCEIROS E ATÉ MESMO IMOBILIZADO - FOI RECLASSIFICADO?
 Não foi possivel entender o sua solicitação, pois não identificamos conta com saldo de Bens em Imoveis de terceiros, seria construções em andamento?
@@ -24759,81 +24852,16 @@
 ok,em anexo o dumento solicitado</t>
         </is>
       </c>
-      <c r="R315" s="1" t="inlineStr">
+      <c r="R316" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="S315" s="1" t="n"/>
-    </row>
-    <row r="316">
-      <c r="A316" s="1" t="n">
-        <v>80311</v>
-      </c>
-      <c r="B316" s="1" t="inlineStr">
-        <is>
-          <t>DCTFWeb</t>
-        </is>
-      </c>
-      <c r="C316" s="1" t="inlineStr">
-        <is>
-          <t>DCTFWeb</t>
-        </is>
-      </c>
-      <c r="D316" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E316" s="1" t="inlineStr">
-        <is>
-          <t>Há 3 pendencias de omissão de DCTWeb para o cliente. Dez/2022, Fev/2026 e Mar/2026, por favor verificar e retornar esse chamado, pois está na malha fiscal referente ao mês de dez/2022.</t>
-        </is>
-      </c>
-      <c r="F316" s="1" t="n">
-        <v>2744</v>
-      </c>
-      <c r="G316" s="1" t="inlineStr">
-        <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA  (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H316" s="1" t="n"/>
-      <c r="I316" s="1" t="inlineStr">
-        <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
-        </is>
-      </c>
-      <c r="J316" s="2" t="n">
-        <v>46195.44287422454</v>
-      </c>
-      <c r="K316" s="2" t="n">
-        <v>46198</v>
-      </c>
-      <c r="L316" s="1" t="inlineStr">
-        <is>
-          <t>Sem Responsavel Atribuido</t>
-        </is>
-      </c>
-      <c r="M316" s="1" t="inlineStr">
-        <is>
-          <t>Rodrigo Rego</t>
-        </is>
-      </c>
-      <c r="N316" s="1" t="n"/>
-      <c r="O316" s="1" t="n"/>
-      <c r="P316" s="1" t="inlineStr"/>
-      <c r="Q316" s="1" t="n"/>
-      <c r="R316" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="S316" s="1" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>80317</v>
+        <v>80311</v>
       </c>
       <c r="B317" s="1" t="inlineStr">
         <is>
@@ -24852,7 +24880,7 @@
       </c>
       <c r="E317" s="1" t="inlineStr">
         <is>
-          <t>Verificar os valores informados na DCTFWeb referente ao IRRF, CSRF, CP-SEGUR, CP-PATRONAL, CP-TERCEIROS dos períodos que constam na situação fiscal, pois como o saldo do valor original está diferente do saldo devedor creio que há divergência entre a guia emitida e o que foi informado na DCTFWeb.</t>
+          <t>Há 3 pendencias de omissão de DCTWeb para o cliente. Dez/2022, Fev/2026 e Mar/2026, por favor verificar e retornar esse chamado, pois está na malha fiscal referente ao mês de dez/2022.</t>
         </is>
       </c>
       <c r="F317" s="1" t="n">
@@ -24863,21 +24891,25 @@
           <t>CUCINARE PRO ALIMENTAÇÃO LTDA  (MATRIZ)</t>
         </is>
       </c>
-      <c r="H317" s="1" t="n"/>
+      <c r="H317" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I317" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J317" s="2" t="n">
-        <v>46195.4506077199</v>
+        <v>46195.44287422454</v>
       </c>
       <c r="K317" s="2" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="L317" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M317" s="1" t="inlineStr">
@@ -24888,7 +24920,7 @@
       <c r="N317" s="1" t="n"/>
       <c r="O317" s="1" t="n"/>
       <c r="P317" s="1" t="inlineStr"/>
-      <c r="Q317" s="1" t="n"/>
+      <c r="Q317" s="1" t="inlineStr"/>
       <c r="R317" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24898,62 +24930,66 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>80415</v>
+        <v>80317</v>
       </c>
       <c r="B318" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="C318" s="1" t="inlineStr">
         <is>
-          <t>Balanço e DRE</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="D318" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E318" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!Por gentileza, solicito o envio do Balanço e da DRE referentes ao exercício de 2025Caso não seja possível anexar os documentos neste chamado, peço a gentileza de encaminhá-los para o meu e-mail:apoio.gc11@mgcontecnica.com.brInformo que tentei gerar os documentos por aqui, porém os valores apresentados não estão conciliando com as informações esperadas.Como se trata de uma demanda com certa urgência, peço, se possível, que os documentos sejam encaminhados ainda hoje.Desde já, agradeço pela atenção e fico no aguardo.</t>
+          <t>Verificar os valores informados na DCTFWeb referente ao IRRF, CSRF, CP-SEGUR, CP-PATRONAL, CP-TERCEIROS dos períodos que constam na situação fiscal, pois como o saldo do valor original está diferente do saldo devedor creio que há divergência entre a guia emitida e o que foi informado na DCTFWeb.</t>
         </is>
       </c>
       <c r="F318" s="1" t="n">
-        <v>3638</v>
+        <v>2744</v>
       </c>
       <c r="G318" s="1" t="inlineStr">
         <is>
-          <t>MEE LOCAÇÃO DE EQUIPAMENTOS LTDA</t>
-        </is>
-      </c>
-      <c r="H318" s="1" t="n"/>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA  (MATRIZ)</t>
+        </is>
+      </c>
+      <c r="H318" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I318" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>46195.68175674768</v>
+        <v>46195.4506077199</v>
       </c>
       <c r="K318" s="2" t="n">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="L318" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M318" s="1" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N318" s="1" t="n"/>
       <c r="O318" s="1" t="n"/>
       <c r="P318" s="1" t="inlineStr"/>
-      <c r="Q318" s="1" t="n"/>
+      <c r="Q318" s="1" t="inlineStr"/>
       <c r="R318" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24963,16 +24999,16 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>78854</v>
+        <v>80415</v>
       </c>
       <c r="B319" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="C319" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Balanço e DRE</t>
         </is>
       </c>
       <c r="D319" s="1" t="inlineStr">
@@ -24982,53 +25018,47 @@
       </c>
       <c r="E319" s="1" t="inlineStr">
         <is>
-          <t>IMPORTANTEPor gentileza, necessário realizar a captura de 100% dos arquivos XML referentes a compras realizadas pela empresa de janeiro a novembro/2025, para a contabilização correta de todas as compras realizadas pela empresa no período citado.</t>
+          <t>Prezados, boa tarde!Por gentileza, solicito o envio do Balanço e da DRE referentes ao exercício de 2025Caso não seja possível anexar os documentos neste chamado, peço a gentileza de encaminhá-los para o meu e-mail:apoio.gc11@mgcontecnica.com.brInformo que tentei gerar os documentos por aqui, porém os valores apresentados não estão conciliando com as informações esperadas.Como se trata de uma demanda com certa urgência, peço, se possível, que os documentos sejam encaminhados ainda hoje.Desde já, agradeço pela atenção e fico no aguardo.</t>
         </is>
       </c>
       <c r="F319" s="1" t="n">
-        <v>4811</v>
+        <v>3638</v>
       </c>
       <c r="G319" s="1" t="inlineStr">
         <is>
-          <t>ORIVALDO DAN</t>
+          <t>MEE LOCAÇÃO DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="H319" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="I319" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J319" s="2" t="n">
-        <v>46134.74738626157</v>
+        <v>46195.68175674768</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>46142</v>
+        <v>46196</v>
       </c>
       <c r="L319" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M319" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N319" s="2" t="n">
-        <v>46183.48642873843</v>
-      </c>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
+      <c r="N319" s="1" t="n"/>
       <c r="O319" s="1" t="n"/>
       <c r="P319" s="1" t="inlineStr"/>
-      <c r="Q319" s="1" t="inlineStr">
-        <is>
-          <t>Fazendo levantamento das notas enviadas pelo cliente e o que consta no gax para confirmar com o GC se realmente devem ser lançadas.</t>
-        </is>
-      </c>
+      <c r="Q319" s="1" t="inlineStr"/>
       <c r="R319" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25038,166 +25068,172 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
+        <v>78854</v>
+      </c>
+      <c r="B320" s="1" t="inlineStr">
+        <is>
+          <t>Ata de Reunião</t>
+        </is>
+      </c>
+      <c r="C320" s="1" t="inlineStr">
+        <is>
+          <t>Inclusão de Ata</t>
+        </is>
+      </c>
+      <c r="D320" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E320" s="1" t="inlineStr">
+        <is>
+          <t>IMPORTANTEPor gentileza, necessário realizar a captura de 100% dos arquivos XML referentes a compras realizadas pela empresa de janeiro a novembro/2025, para a contabilização correta de todas as compras realizadas pela empresa no período citado.</t>
+        </is>
+      </c>
+      <c r="F320" s="1" t="n">
+        <v>4811</v>
+      </c>
+      <c r="G320" s="1" t="inlineStr">
+        <is>
+          <t>ORIVALDO DAN</t>
+        </is>
+      </c>
+      <c r="H320" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
+      <c r="I320" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="n">
+        <v>46134.74738626157</v>
+      </c>
+      <c r="K320" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="L320" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M320" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N320" s="2" t="n">
+        <v>46183.48642873843</v>
+      </c>
+      <c r="O320" s="1" t="n"/>
+      <c r="P320" s="1" t="inlineStr"/>
+      <c r="Q320" s="1" t="inlineStr">
+        <is>
+          <t>Fazendo levantamento das notas enviadas pelo cliente e o que consta no gax para confirmar com o GC se realmente devem ser lançadas.</t>
+        </is>
+      </c>
+      <c r="R320" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="S320" s="1" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="1" t="n">
         <v>79765</v>
       </c>
-      <c r="B320" s="1" t="inlineStr">
+      <c r="B321" s="1" t="inlineStr">
         <is>
           <t>Balanço e DRE</t>
         </is>
       </c>
-      <c r="C320" s="1" t="inlineStr">
+      <c r="C321" s="1" t="inlineStr">
         <is>
           <t>Balanço e DRE</t>
         </is>
       </c>
-      <c r="D320" s="1" t="inlineStr">
+      <c r="D321" s="1" t="inlineStr">
         <is>
           <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E320" s="1" t="inlineStr">
+      <c r="E321" s="1" t="inlineStr">
         <is>
           <t>providenciar balanço de e dre da empresa 5044 ano: 2025</t>
         </is>
       </c>
-      <c r="F320" s="1" t="n">
+      <c r="F321" s="1" t="n">
         <v>5044</v>
       </c>
-      <c r="G320" s="1" t="inlineStr">
+      <c r="G321" s="1" t="inlineStr">
         <is>
           <t>BARATÃO SÃO LUCAS LTDA</t>
         </is>
       </c>
-      <c r="H320" s="1" t="inlineStr">
+      <c r="H321" s="1" t="inlineStr">
         <is>
           <t>Edileide Dias</t>
         </is>
       </c>
-      <c r="I320" s="1" t="inlineStr">
+      <c r="I321" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
-      <c r="J320" s="2" t="n">
+      <c r="J321" s="2" t="n">
         <v>46181.69699834491</v>
       </c>
-      <c r="K320" s="2" t="n">
+      <c r="K321" s="2" t="n">
         <v>46182</v>
       </c>
-      <c r="L320" s="1" t="inlineStr">
+      <c r="L321" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M320" s="1" t="inlineStr">
+      <c r="M321" s="1" t="inlineStr">
         <is>
           <t>Daniela Silva</t>
         </is>
       </c>
-      <c r="N320" s="1" t="n"/>
-      <c r="O320" s="2" t="n">
+      <c r="N321" s="1" t="n"/>
+      <c r="O321" s="2" t="n">
         <v>46181.73338240741</v>
       </c>
-      <c r="P320" s="1" t="inlineStr">
+      <c r="P321" s="1" t="inlineStr">
         <is>
           <t>edileide</t>
         </is>
       </c>
-      <c r="Q320" s="1" t="inlineStr">
+      <c r="Q321" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Boa tarde
 Segue conforme solicitado
 </t>
         </is>
       </c>
-      <c r="R320" s="1" t="inlineStr">
+      <c r="R321" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="S320" s="1" t="n"/>
-    </row>
-    <row r="321">
-      <c r="A321" s="1" t="n">
-        <v>78445</v>
-      </c>
-      <c r="B321" s="1" t="inlineStr">
-        <is>
-          <t>Ata de Reunião</t>
-        </is>
-      </c>
-      <c r="C321" s="1" t="inlineStr">
-        <is>
-          <t>Inclusão de Ata</t>
-        </is>
-      </c>
-      <c r="D321" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E321" s="1" t="inlineStr">
-        <is>
-          <t>Verificar EFD Transporte de Saldo Credor Incorreto ref. 08/2025, 11/2025 e 12/2025Verificar se o cliente responde o e-mail com as críticas das NFs de entrada</t>
-        </is>
-      </c>
-      <c r="F321" s="1" t="n">
-        <v>5100</v>
-      </c>
-      <c r="G321" s="1" t="inlineStr">
-        <is>
-          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
-        </is>
-      </c>
-      <c r="H321" s="1" t="inlineStr">
-        <is>
-          <t>Thaiza Oliveira</t>
-        </is>
-      </c>
-      <c r="I321" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J321" s="2" t="n">
-        <v>46114.57570729167</v>
-      </c>
-      <c r="K321" s="2" t="n">
-        <v>46121</v>
-      </c>
-      <c r="L321" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M321" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N321" s="1" t="n"/>
-      <c r="O321" s="1" t="n"/>
-      <c r="P321" s="1" t="inlineStr"/>
-      <c r="Q321" s="1" t="inlineStr"/>
-      <c r="R321" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="S321" s="1" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>78446</v>
+        <v>78445</v>
       </c>
       <c r="B322" s="1" t="inlineStr">
         <is>
-          <t>Reunião externa</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C322" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata de reunião</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D322" s="1" t="inlineStr">
@@ -25207,7 +25243,7 @@
       </c>
       <c r="E322" s="1" t="inlineStr">
         <is>
-          <t>Enviar guia para pagamentoEnviar guia para pagamento</t>
+          <t>Verificar EFD Transporte de Saldo Credor Incorreto ref. 08/2025, 11/2025 e 12/2025Verificar se o cliente responde o e-mail com as críticas das NFs de entrada</t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
@@ -25220,23 +25256,23 @@
       </c>
       <c r="H322" s="1" t="inlineStr">
         <is>
-          <t>Renata Cavalheiro</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="I322" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>46114.57664811343</v>
+        <v>46114.57570729167</v>
       </c>
       <c r="K322" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L322" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M322" s="1" t="inlineStr">
@@ -25245,38 +25281,28 @@
         </is>
       </c>
       <c r="N322" s="1" t="n"/>
-      <c r="O322" s="2" t="n">
-        <v>46114.61985003472</v>
-      </c>
-      <c r="P322" s="1" t="inlineStr">
-        <is>
-          <t>renatac</t>
-        </is>
-      </c>
-      <c r="Q322" s="1" t="inlineStr">
-        <is>
-          <t>De qual imposto se refere?</t>
-        </is>
-      </c>
+      <c r="O322" s="1" t="n"/>
+      <c r="P322" s="1" t="inlineStr"/>
+      <c r="Q322" s="1" t="inlineStr"/>
       <c r="R322" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S322" s="1" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>79641</v>
+        <v>78446</v>
       </c>
       <c r="B323" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Regime Tributário</t>
+          <t>Reunião externa</t>
         </is>
       </c>
       <c r="C323" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Regime Tributário</t>
+          <t>Inclusão de Ata de reunião</t>
         </is>
       </c>
       <c r="D323" s="1" t="inlineStr">
@@ -25286,32 +25312,32 @@
       </c>
       <c r="E323" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!O cliente em assunto deveria ter migrado para o lucro real no iniciío de 2026.Em conversa com o Ronaldo Dias do Paralegal, devemos retificar as obrigações acessórias e as guias de PIS e COFINS que foram recolhidas como lucro presumido, quando concluido devemos comunicá-lo para que faça o pedido da alteração</t>
+          <t>Enviar guia para pagamentoEnviar guia para pagamento</t>
         </is>
       </c>
       <c r="F323" s="1" t="n">
-        <v>5726</v>
+        <v>5100</v>
       </c>
       <c r="G323" s="1" t="inlineStr">
         <is>
-          <t>VIANA &amp; CIA LTDA</t>
+          <t>A P SOARES DA SILVA MERCADO E PADARIA</t>
         </is>
       </c>
       <c r="H323" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Renata Cavalheiro</t>
         </is>
       </c>
       <c r="I323" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J323" s="2" t="n">
-        <v>46175.70509568287</v>
+        <v>46114.57664811343</v>
       </c>
       <c r="K323" s="2" t="n">
-        <v>46178</v>
+        <v>46121</v>
       </c>
       <c r="L323" s="1" t="inlineStr">
         <is>
@@ -25320,21 +25346,21 @@
       </c>
       <c r="M323" s="1" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N323" s="1" t="n"/>
       <c r="O323" s="2" t="n">
-        <v>46181.75103634259</v>
+        <v>46114.61985003472</v>
       </c>
       <c r="P323" s="1" t="inlineStr">
         <is>
-          <t>pvolpe</t>
+          <t>renatac</t>
         </is>
       </c>
       <c r="Q323" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">deverá ser aberto um chamado sinalizando o reprocesso dessa empresa </t>
+          <t>De qual imposto se refere?</t>
         </is>
       </c>
       <c r="R323" s="1" t="inlineStr">
@@ -25346,7 +25372,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>80110</v>
+        <v>79641</v>
       </c>
       <c r="B324" s="1" t="inlineStr">
         <is>
@@ -25365,7 +25391,7 @@
       </c>
       <c r="E324" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, boa tarde!Solicitamos o reprocesso das obrigações acessorias do periodo de 2026 devido a alteração de regime tributario do lucro presumido para o lucro real.obs:Chamado aberto anteriormente 79641O cliente em assunto deveria ter migrado para o lucro real no iniciío de 2026. </t>
+          <t>Prezados, boa tarde!O cliente em assunto deveria ter migrado para o lucro real no iniciío de 2026.Em conversa com o Ronaldo Dias do Paralegal, devemos retificar as obrigações acessórias e as guias de PIS e COFINS que foram recolhidas como lucro presumido, quando concluido devemos comunicá-lo para que faça o pedido da alteração</t>
         </is>
       </c>
       <c r="F324" s="1" t="n">
@@ -25378,7 +25404,7 @@
       </c>
       <c r="H324" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I324" s="1" t="inlineStr">
@@ -25387,14 +25413,14 @@
         </is>
       </c>
       <c r="J324" s="2" t="n">
-        <v>46189.67080621528</v>
+        <v>46175.70509568287</v>
       </c>
       <c r="K324" s="2" t="n">
-        <v>46192</v>
+        <v>46178</v>
       </c>
       <c r="L324" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M324" s="1" t="inlineStr">
@@ -25403,28 +25429,38 @@
         </is>
       </c>
       <c r="N324" s="1" t="n"/>
-      <c r="O324" s="1" t="n"/>
-      <c r="P324" s="1" t="inlineStr"/>
-      <c r="Q324" s="1" t="inlineStr"/>
+      <c r="O324" s="2" t="n">
+        <v>46181.75103634259</v>
+      </c>
+      <c r="P324" s="1" t="inlineStr">
+        <is>
+          <t>pvolpe</t>
+        </is>
+      </c>
+      <c r="Q324" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deverá ser aberto um chamado sinalizando o reprocesso dessa empresa </t>
+        </is>
+      </c>
       <c r="R324" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S324" s="1" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>78447</v>
+        <v>80110</v>
       </c>
       <c r="B325" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Alteração de Regime Tributário</t>
         </is>
       </c>
       <c r="C325" s="1" t="inlineStr">
         <is>
-          <t>Omissão de Obrigações Acessórias</t>
+          <t>Alteração de Regime Tributário</t>
         </is>
       </c>
       <c r="D325" s="1" t="inlineStr">
@@ -25434,111 +25470,101 @@
       </c>
       <c r="E325" s="1" t="inlineStr">
         <is>
-          <t>Ref. 01/2026 GIA/EFD Não apresentou GIA/EFD Cobrança RecorrenteVerificar MAED - PGDAS-D em aberto Cobrança Recorrente</t>
+          <t xml:space="preserve">Prezados, boa tarde!Solicitamos o reprocesso das obrigações acessorias do periodo de 2026 devido a alteração de regime tributario do lucro presumido para o lucro real.obs:Chamado aberto anteriormente 79641O cliente em assunto deveria ter migrado para o lucro real no iniciío de 2026. </t>
         </is>
       </c>
       <c r="F325" s="1" t="n">
-        <v>5740</v>
+        <v>5726</v>
       </c>
       <c r="G325" s="1" t="inlineStr">
         <is>
-          <t>MARIA VALDENE FERREIRA RIBEIRO</t>
+          <t>VIANA &amp; CIA LTDA</t>
         </is>
       </c>
       <c r="H325" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I325" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J325" s="2" t="n">
-        <v>46114.58255327546</v>
+        <v>46189.67080621528</v>
       </c>
       <c r="K325" s="2" t="n">
-        <v>46121</v>
+        <v>46192</v>
       </c>
       <c r="L325" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M325" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="N325" s="1" t="n"/>
-      <c r="O325" s="2" t="n">
-        <v>46182.53676319445</v>
-      </c>
-      <c r="P325" s="1" t="inlineStr">
-        <is>
-          <t>lorrane</t>
-        </is>
-      </c>
-      <c r="Q325" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde! Sobre qual empresa essa solicitação?</t>
-        </is>
-      </c>
+      <c r="O325" s="1" t="n"/>
+      <c r="P325" s="1" t="inlineStr"/>
+      <c r="Q325" s="1" t="inlineStr"/>
       <c r="R325" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S325" s="1" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>80095</v>
+        <v>78447</v>
       </c>
       <c r="B326" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="C326" s="1" t="inlineStr">
         <is>
-          <t>Recálculo de Guia</t>
+          <t>Omissão de Obrigações Acessórias</t>
         </is>
       </c>
       <c r="D326" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E326" s="1" t="inlineStr">
         <is>
-          <t>Cliente solicitou a atualização da guia para pagamento da Dctfweb referente ao mês de março/2026 para regularização da pendencia.</t>
+          <t>Ref. 01/2026 GIA/EFD Não apresentou GIA/EFD Cobrança RecorrenteVerificar MAED - PGDAS-D em aberto Cobrança Recorrente</t>
         </is>
       </c>
       <c r="F326" s="1" t="n">
-        <v>5886</v>
+        <v>5740</v>
       </c>
       <c r="G326" s="1" t="inlineStr">
         <is>
-          <t>ITA - TECNOLOGIA ASSISTIVA LTDA</t>
+          <t>MARIA VALDENE FERREIRA RIBEIRO</t>
         </is>
       </c>
       <c r="H326" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="I326" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J326" s="2" t="n">
-        <v>46189.54521195602</v>
+        <v>46114.58255327546</v>
       </c>
       <c r="K326" s="2" t="n">
-        <v>46190</v>
+        <v>46121</v>
       </c>
       <c r="L326" s="1" t="inlineStr">
         <is>
@@ -25547,21 +25573,21 @@
       </c>
       <c r="M326" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="N326" s="1" t="n"/>
       <c r="O326" s="2" t="n">
-        <v>46191.47922549769</v>
+        <v>46182.53676319445</v>
       </c>
       <c r="P326" s="1" t="inlineStr">
         <is>
-          <t>inascimento</t>
+          <t>lorrane</t>
         </is>
       </c>
       <c r="Q326" s="1" t="inlineStr">
         <is>
-          <t>ENVIADO POR EMAIL</t>
+          <t>Boa tarde! Sobre qual empresa essa solicitação?</t>
         </is>
       </c>
       <c r="R326" s="1" t="inlineStr">
@@ -25573,39 +25599,39 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>80043</v>
+        <v>80095</v>
       </c>
       <c r="B327" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="C327" s="1" t="inlineStr">
         <is>
-          <t>DCTFWeb</t>
+          <t>Recálculo de Guia</t>
         </is>
       </c>
       <c r="D327" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E327" s="1" t="inlineStr">
         <is>
-          <t>Prezados boa tardePendência - Omissão de DCTFWeb* _________________________________________________________________________________(Período de Apuração)2025 - JAN FEV MAR ABR MAI JUN JUL AGO SET OUT NOV DEZ</t>
+          <t>Cliente solicitou a atualização da guia para pagamento da Dctfweb referente ao mês de março/2026 para regularização da pendencia.</t>
         </is>
       </c>
       <c r="F327" s="1" t="n">
-        <v>5995</v>
+        <v>5886</v>
       </c>
       <c r="G327" s="1" t="inlineStr">
         <is>
-          <t>LITOCOMP INDUSTRIA GRAFICA E EDITORA LTDA</t>
+          <t>ITA - TECNOLOGIA ASSISTIVA LTDA</t>
         </is>
       </c>
       <c r="H327" s="1" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="I327" s="1" t="inlineStr">
@@ -25614,10 +25640,10 @@
         </is>
       </c>
       <c r="J327" s="2" t="n">
-        <v>46188.60840798611</v>
+        <v>46189.54521195602</v>
       </c>
       <c r="K327" s="2" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="L327" s="1" t="inlineStr">
         <is>
@@ -25626,21 +25652,21 @@
       </c>
       <c r="M327" s="1" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N327" s="1" t="n"/>
       <c r="O327" s="2" t="n">
-        <v>46189.6038</v>
+        <v>46191.47922549769</v>
       </c>
       <c r="P327" s="1" t="inlineStr">
         <is>
-          <t>erikas</t>
+          <t>inascimento</t>
         </is>
       </c>
       <c r="Q327" s="1" t="inlineStr">
         <is>
-          <t>Declaração retificadas</t>
+          <t>ENVIADO POR EMAIL</t>
         </is>
       </c>
       <c r="R327" s="1" t="inlineStr">
@@ -25652,51 +25678,51 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>79919</v>
+        <v>80043</v>
       </c>
       <c r="B328" s="1" t="inlineStr">
         <is>
-          <t>Antecipação de ECF</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="C328" s="1" t="inlineStr">
         <is>
-          <t>Antecipação de ECF</t>
+          <t>DCTFWeb</t>
         </is>
       </c>
       <c r="D328" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E328" s="1" t="inlineStr">
         <is>
-          <t>Cliente está fazendo um empréstimo junto ao banco e para a liberação desse empréstimo o banco está solicitando o envio da ECF 2026 AB 2025.</t>
+          <t>Prezados boa tardePendência - Omissão de DCTFWeb* _________________________________________________________________________________(Período de Apuração)2025 - JAN FEV MAR ABR MAI JUN JUL AGO SET OUT NOV DEZ</t>
         </is>
       </c>
       <c r="F328" s="1" t="n">
-        <v>6440</v>
+        <v>5995</v>
       </c>
       <c r="G328" s="1" t="inlineStr">
         <is>
-          <t>INFINITY UTILIDADES LTDA</t>
+          <t>LITOCOMP INDUSTRIA GRAFICA E EDITORA LTDA</t>
         </is>
       </c>
       <c r="H328" s="1" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Erika Santana</t>
         </is>
       </c>
       <c r="I328" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J328" s="2" t="n">
-        <v>46184.5967934375</v>
+        <v>46188.60840798611</v>
       </c>
       <c r="K328" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="L328" s="1" t="inlineStr">
         <is>
@@ -25705,21 +25731,21 @@
       </c>
       <c r="M328" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="N328" s="1" t="n"/>
       <c r="O328" s="2" t="n">
-        <v>46195.73638541667</v>
+        <v>46189.6038</v>
       </c>
       <c r="P328" s="1" t="inlineStr">
         <is>
-          <t>karinasantos</t>
+          <t>erikas</t>
         </is>
       </c>
       <c r="Q328" s="1" t="inlineStr">
         <is>
-          <t>Entrega realizada</t>
+          <t>Declaração retificadas</t>
         </is>
       </c>
       <c r="R328" s="1" t="inlineStr">
@@ -25838,7 +25864,11 @@
           <t>LSV GESTAO COMERCIO LOCACAO MANUTENCAO DE EQUIPAMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H330" s="1" t="n"/>
+      <c r="H330" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I330" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -25852,7 +25882,7 @@
       </c>
       <c r="L330" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M330" s="1" t="inlineStr">
@@ -25863,7 +25893,7 @@
       <c r="N330" s="1" t="n"/>
       <c r="O330" s="1" t="n"/>
       <c r="P330" s="1" t="inlineStr"/>
-      <c r="Q330" s="1" t="n"/>
+      <c r="Q330" s="1" t="inlineStr"/>
       <c r="R330" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25903,7 +25933,11 @@
           <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H331" s="1" t="n"/>
+      <c r="H331" s="1" t="inlineStr">
+        <is>
+          <t>Jackson Silva</t>
+        </is>
+      </c>
       <c r="I331" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -25917,7 +25951,7 @@
       </c>
       <c r="L331" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M331" s="1" t="inlineStr">
@@ -25928,7 +25962,7 @@
       <c r="N331" s="1" t="n"/>
       <c r="O331" s="1" t="n"/>
       <c r="P331" s="1" t="inlineStr"/>
-      <c r="Q331" s="1" t="n"/>
+      <c r="Q331" s="1" t="inlineStr"/>
       <c r="R331" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25970,7 +26004,7 @@
       </c>
       <c r="H332" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="I332" s="1" t="inlineStr">

</xml_diff>

<commit_message>
data: atualização base chamados 30-06-26 0902
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S574" headerRowCount="1">
-  <autoFilter ref="A1:S574"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S575" headerRowCount="1">
+  <autoFilter ref="A1:S575"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S574"/>
+  <dimension ref="A1:S575"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43354,7 +43354,7 @@
     </row>
     <row r="571">
       <c r="A571" s="1" t="n">
-        <v>76508</v>
+        <v>80610</v>
       </c>
       <c r="B571" s="1" t="inlineStr">
         <is>
@@ -43363,77 +43363,63 @@
       </c>
       <c r="C571" s="1" t="inlineStr">
         <is>
-          <t>Verificar Validação Obrigação</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D571" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>RJ - CTB</t>
         </is>
       </c>
       <c r="E571" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>Prezados, a tarefa de totalizador do mês 05 da 6547 continua constando como aberta, mesmo já tendo sido validada conforme documentação anexada.</t>
         </is>
       </c>
       <c r="F571" s="1" t="n">
-        <v>6605</v>
+        <v>6547</v>
       </c>
       <c r="G571" s="1" t="inlineStr">
         <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
-        </is>
-      </c>
-      <c r="H571" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
+          <t>PERSONAL FORCE ASSISTANCE &amp; SERVICES LTDA</t>
+        </is>
+      </c>
+      <c r="H571" s="1" t="n"/>
       <c r="I571" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J571" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46203.36833799769</v>
       </c>
       <c r="K571" s="2" t="n">
-        <v>46034</v>
+        <v>46204</v>
       </c>
       <c r="L571" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M571" s="1" t="inlineStr">
         <is>
-          <t>Bianca Castro</t>
+          <t>Luis Junior</t>
         </is>
       </c>
       <c r="N571" s="1" t="n"/>
-      <c r="O571" s="2" t="n">
-        <v>46030.75027241898</v>
-      </c>
-      <c r="P571" s="1" t="inlineStr">
-        <is>
-          <t>nicoleo</t>
-        </is>
-      </c>
-      <c r="Q571" s="1" t="inlineStr">
-        <is>
-          <t>Baixadas.</t>
-        </is>
-      </c>
+      <c r="O571" s="1" t="n"/>
+      <c r="P571" s="1" t="inlineStr"/>
+      <c r="Q571" s="1" t="n"/>
       <c r="R571" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S571" s="1" t="n"/>
     </row>
     <row r="572">
       <c r="A572" s="1" t="n">
-        <v>76505</v>
+        <v>76508</v>
       </c>
       <c r="B572" s="1" t="inlineStr">
         <is>
@@ -43452,15 +43438,15 @@
       </c>
       <c r="E572" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F572" s="1" t="n">
-        <v>6640</v>
+        <v>6605</v>
       </c>
       <c r="G572" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H572" s="1" t="inlineStr">
@@ -43474,7 +43460,7 @@
         </is>
       </c>
       <c r="J572" s="2" t="n">
-        <v>46030.60213634259</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K572" s="2" t="n">
         <v>46034</v>
@@ -43491,7 +43477,7 @@
       </c>
       <c r="N572" s="1" t="n"/>
       <c r="O572" s="2" t="n">
-        <v>46030.63182743055</v>
+        <v>46030.75027241898</v>
       </c>
       <c r="P572" s="1" t="inlineStr">
         <is>
@@ -43512,7 +43498,7 @@
     </row>
     <row r="573">
       <c r="A573" s="1" t="n">
-        <v>76501</v>
+        <v>76505</v>
       </c>
       <c r="B573" s="1" t="inlineStr">
         <is>
@@ -43531,15 +43517,15 @@
       </c>
       <c r="E573" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F573" s="1" t="n">
-        <v>6641</v>
+        <v>6640</v>
       </c>
       <c r="G573" s="1" t="inlineStr">
         <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H573" s="1" t="inlineStr">
@@ -43553,7 +43539,7 @@
         </is>
       </c>
       <c r="J573" s="2" t="n">
-        <v>46030.51327708333</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K573" s="2" t="n">
         <v>46034</v>
@@ -43570,7 +43556,7 @@
       </c>
       <c r="N573" s="1" t="n"/>
       <c r="O573" s="2" t="n">
-        <v>46030.64333047454</v>
+        <v>46030.63182743055</v>
       </c>
       <c r="P573" s="1" t="inlineStr">
         <is>
@@ -43591,7 +43577,7 @@
     </row>
     <row r="574">
       <c r="A574" s="1" t="n">
-        <v>76515</v>
+        <v>76501</v>
       </c>
       <c r="B574" s="1" t="inlineStr">
         <is>
@@ -43610,7 +43596,7 @@
       </c>
       <c r="E574" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
         </is>
       </c>
       <c r="F574" s="1" t="n">
@@ -43632,7 +43618,7 @@
         </is>
       </c>
       <c r="J574" s="2" t="n">
-        <v>46030.73046079861</v>
+        <v>46030.51327708333</v>
       </c>
       <c r="K574" s="2" t="n">
         <v>46034</v>
@@ -43649,24 +43635,103 @@
       </c>
       <c r="N574" s="1" t="n"/>
       <c r="O574" s="2" t="n">
+        <v>46030.64333047454</v>
+      </c>
+      <c r="P574" s="1" t="inlineStr">
+        <is>
+          <t>nicoleo</t>
+        </is>
+      </c>
+      <c r="Q574" s="1" t="inlineStr">
+        <is>
+          <t>Baixadas.</t>
+        </is>
+      </c>
+      <c r="R574" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S574" s="1" t="n"/>
+    </row>
+    <row r="575">
+      <c r="A575" s="1" t="n">
+        <v>76515</v>
+      </c>
+      <c r="B575" s="1" t="inlineStr">
+        <is>
+          <t>MG Controle</t>
+        </is>
+      </c>
+      <c r="C575" s="1" t="inlineStr">
+        <is>
+          <t>Verificar Validação Obrigação</t>
+        </is>
+      </c>
+      <c r="D575" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E575" s="1" t="inlineStr">
+        <is>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+        </is>
+      </c>
+      <c r="F575" s="1" t="n">
+        <v>6641</v>
+      </c>
+      <c r="G575" s="1" t="inlineStr">
+        <is>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+        </is>
+      </c>
+      <c r="H575" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="I575" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLADORIA</t>
+        </is>
+      </c>
+      <c r="J575" s="2" t="n">
+        <v>46030.73046079861</v>
+      </c>
+      <c r="K575" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="L575" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M575" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Castro</t>
+        </is>
+      </c>
+      <c r="N575" s="1" t="n"/>
+      <c r="O575" s="2" t="n">
         <v>46030.74734336806</v>
       </c>
-      <c r="P574" s="1" t="inlineStr">
+      <c r="P575" s="1" t="inlineStr">
         <is>
           <t>nicoleo</t>
         </is>
       </c>
-      <c r="Q574" s="1" t="inlineStr">
+      <c r="Q575" s="1" t="inlineStr">
         <is>
           <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
         </is>
       </c>
-      <c r="R574" s="1" t="inlineStr">
+      <c r="R575" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="S574" s="1" t="n"/>
+      <c r="S575" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 02-07-26 1355
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1526,7 +1526,7 @@
       </c>
       <c r="L14" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M14" s="1" t="inlineStr">
@@ -1535,12 +1535,22 @@
         </is>
       </c>
       <c r="N14" s="1" t="n"/>
-      <c r="O14" s="1" t="n"/>
-      <c r="P14" s="1" t="inlineStr"/>
-      <c r="Q14" s="1" t="inlineStr"/>
+      <c r="O14" s="2" t="n">
+        <v>46205.57891142361</v>
+      </c>
+      <c r="P14" s="1" t="inlineStr">
+        <is>
+          <t>inascimento</t>
+        </is>
+      </c>
+      <c r="Q14" s="1" t="inlineStr">
+        <is>
+          <t>ao verificarmos com o cliente ainda não tivemos resposta</t>
+        </is>
+      </c>
       <c r="R14" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S14" s="1" t="n"/>
@@ -12039,7 +12049,7 @@
       </c>
       <c r="L148" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M148" s="1" t="inlineStr">
@@ -12048,12 +12058,22 @@
         </is>
       </c>
       <c r="N148" s="1" t="n"/>
-      <c r="O148" s="1" t="n"/>
-      <c r="P148" s="1" t="inlineStr"/>
-      <c r="Q148" s="1" t="inlineStr"/>
+      <c r="O148" s="2" t="n">
+        <v>46205.56024097222</v>
+      </c>
+      <c r="P148" s="1" t="inlineStr">
+        <is>
+          <t>ricardof</t>
+        </is>
+      </c>
+      <c r="Q148" s="1" t="inlineStr">
+        <is>
+          <t>Conforme anexos, as declarações não foram entregues pela MG. O responsável pelo preenchimento é: GILDASIO RIBEIRO MACHADO JUNIOR - CPF 216.647.538-85</t>
+        </is>
+      </c>
       <c r="R148" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S148" s="1" t="n"/>
@@ -13610,7 +13630,7 @@
       </c>
       <c r="L168" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M168" s="1" t="inlineStr">
@@ -13621,8 +13641,14 @@
       <c r="N168" s="2" t="n">
         <v>46182.75536666666</v>
       </c>
-      <c r="O168" s="1" t="n"/>
-      <c r="P168" s="1" t="inlineStr"/>
+      <c r="O168" s="2" t="n">
+        <v>46205.55345760417</v>
+      </c>
+      <c r="P168" s="1" t="inlineStr">
+        <is>
+          <t>ricardof</t>
+        </is>
+      </c>
       <c r="Q168" s="1" t="inlineStr">
         <is>
           <t>Aguardando regularização do acesso ao Posto Fiscal com a senha da Alexandra. Sem ela não conseguimos efetuar consultas e retificar GIA.</t>
@@ -13630,7 +13656,7 @@
       </c>
       <c r="R168" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S168" s="1" t="n"/>
@@ -24249,7 +24275,7 @@
       </c>
       <c r="H305" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I305" s="1" t="inlineStr">
@@ -24265,7 +24291,7 @@
       </c>
       <c r="L305" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M305" s="1" t="inlineStr">
@@ -24274,12 +24300,23 @@
         </is>
       </c>
       <c r="N305" s="1" t="n"/>
-      <c r="O305" s="1" t="n"/>
-      <c r="P305" s="1" t="inlineStr"/>
-      <c r="Q305" s="1" t="inlineStr"/>
+      <c r="O305" s="2" t="n">
+        <v>46205.57428920139</v>
+      </c>
+      <c r="P305" s="1" t="inlineStr">
+        <is>
+          <t>pvolpe</t>
+        </is>
+      </c>
+      <c r="Q305" s="1" t="inlineStr">
+        <is>
+          <t>boa tarde
+retificação realizada na data de 02-07</t>
+        </is>
+      </c>
       <c r="R305" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S305" s="1" t="n"/>
@@ -26643,7 +26680,7 @@
       </c>
       <c r="L336" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M336" s="1" t="inlineStr">
@@ -26652,12 +26689,23 @@
         </is>
       </c>
       <c r="N336" s="1" t="n"/>
-      <c r="O336" s="1" t="n"/>
-      <c r="P336" s="1" t="inlineStr"/>
-      <c r="Q336" s="1" t="inlineStr"/>
+      <c r="O336" s="2" t="n">
+        <v>46205.55968140046</v>
+      </c>
+      <c r="P336" s="1" t="inlineStr">
+        <is>
+          <t>fernandaa</t>
+        </is>
+      </c>
+      <c r="Q336" s="1" t="inlineStr">
+        <is>
+          <t>Períodos fechados.
+E-mail enviado ao cliente para que valide junto ao seu Departamento pessoal as divergências dos valores das verbas de folha.</t>
+        </is>
+      </c>
       <c r="R336" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S336" s="1" t="n"/>
@@ -26712,7 +26760,7 @@
       </c>
       <c r="L337" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M337" s="1" t="inlineStr">
@@ -26721,12 +26769,23 @@
         </is>
       </c>
       <c r="N337" s="1" t="n"/>
-      <c r="O337" s="1" t="n"/>
-      <c r="P337" s="1" t="inlineStr"/>
-      <c r="Q337" s="1" t="inlineStr"/>
+      <c r="O337" s="2" t="n">
+        <v>46205.55982739583</v>
+      </c>
+      <c r="P337" s="1" t="inlineStr">
+        <is>
+          <t>fernandaa</t>
+        </is>
+      </c>
+      <c r="Q337" s="1" t="inlineStr">
+        <is>
+          <t>Períodos fechados.
+E-mail enviado ao cliente para que valide junto ao seu Departamento pessoal as divergências dos valores das verbas de folha.</t>
+        </is>
+      </c>
       <c r="R337" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S337" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 06-07-26 1802
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S605" headerRowCount="1">
-  <autoFilter ref="A1:S605"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:S606" headerRowCount="1">
+  <autoFilter ref="A1:S606"/>
   <tableColumns count="19">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S605"/>
+  <dimension ref="A1:S606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -45855,7 +45855,7 @@
     </row>
     <row r="601">
       <c r="A601" s="1" t="n">
-        <v>80743</v>
+        <v>80776</v>
       </c>
       <c r="B601" s="1" t="inlineStr">
         <is>
@@ -45869,22 +45869,18 @@
       </c>
       <c r="D601" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E601" s="1" t="inlineStr">
         <is>
-          <t>5281 - E A P PINGO - NÃO FOI DISPONIBILZAR O PDF PARA BAIXAR TAREFA  DE DESONERAÇÃO DA FOLHA Preciso que baixem minha tarefa, não consigo fazer porque depende de relatório de DCFWEB que não está mais sendo disponibilizado pelo contábil.Att.Vander</t>
+          <t>Boa tarde, referente a tarefa de serviços prestados da empresa 2209, ela não esta aceitando o arquivo em branco (não possui movimento de serviços) poderiam realizar a baixa por favor</t>
         </is>
       </c>
       <c r="F601" s="1" t="n">
-        <v>5281</v>
-      </c>
-      <c r="G601" s="1" t="inlineStr">
-        <is>
-          <t>E A P PINGO REFRIGERAÇÃO</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G601" s="1" t="n"/>
       <c r="H601" s="1" t="inlineStr">
         <is>
           <t>Gabriel Amaral</t>
@@ -45896,45 +45892,35 @@
         </is>
       </c>
       <c r="J601" s="2" t="n">
-        <v>46209.43690501157</v>
+        <v>46209.74850755787</v>
       </c>
       <c r="K601" s="2" t="n">
         <v>46210</v>
       </c>
       <c r="L601" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M601" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Gustavo Tonan</t>
         </is>
       </c>
       <c r="N601" s="1" t="n"/>
-      <c r="O601" s="2" t="n">
-        <v>46209.45948171296</v>
-      </c>
-      <c r="P601" s="1" t="inlineStr">
-        <is>
-          <t>gamaral</t>
-        </is>
-      </c>
-      <c r="Q601" s="1" t="inlineStr">
-        <is>
-          <t>Tarefa baixada</t>
-        </is>
-      </c>
+      <c r="O601" s="1" t="n"/>
+      <c r="P601" s="1" t="inlineStr"/>
+      <c r="Q601" s="1" t="inlineStr"/>
       <c r="R601" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S601" s="1" t="n"/>
     </row>
     <row r="602">
       <c r="A602" s="1" t="n">
-        <v>76508</v>
+        <v>80743</v>
       </c>
       <c r="B602" s="1" t="inlineStr">
         <is>
@@ -45943,30 +45929,30 @@
       </c>
       <c r="C602" s="1" t="inlineStr">
         <is>
-          <t>Verificar Validação Obrigação</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D602" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E602" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>5281 - E A P PINGO - NÃO FOI DISPONIBILZAR O PDF PARA BAIXAR TAREFA  DE DESONERAÇÃO DA FOLHA Preciso que baixem minha tarefa, não consigo fazer porque depende de relatório de DCFWEB que não está mais sendo disponibilizado pelo contábil.Att.Vander</t>
         </is>
       </c>
       <c r="F602" s="1" t="n">
-        <v>6605</v>
+        <v>5281</v>
       </c>
       <c r="G602" s="1" t="inlineStr">
         <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
+          <t>E A P PINGO REFRIGERAÇÃO</t>
         </is>
       </c>
       <c r="H602" s="1" t="inlineStr">
         <is>
-          <t>Nicole Oliveira</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I602" s="1" t="inlineStr">
@@ -45975,10 +45961,10 @@
         </is>
       </c>
       <c r="J602" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46209.43690501157</v>
       </c>
       <c r="K602" s="2" t="n">
-        <v>46034</v>
+        <v>46210</v>
       </c>
       <c r="L602" s="1" t="inlineStr">
         <is>
@@ -45987,21 +45973,21 @@
       </c>
       <c r="M602" s="1" t="inlineStr">
         <is>
-          <t>Bianca Castro</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N602" s="1" t="n"/>
       <c r="O602" s="2" t="n">
-        <v>46030.75027241898</v>
+        <v>46209.45948171296</v>
       </c>
       <c r="P602" s="1" t="inlineStr">
         <is>
-          <t>nicoleo</t>
+          <t>gamaral</t>
         </is>
       </c>
       <c r="Q602" s="1" t="inlineStr">
         <is>
-          <t>Baixadas.</t>
+          <t>Tarefa baixada</t>
         </is>
       </c>
       <c r="R602" s="1" t="inlineStr">
@@ -46013,7 +45999,7 @@
     </row>
     <row r="603">
       <c r="A603" s="1" t="n">
-        <v>76505</v>
+        <v>76508</v>
       </c>
       <c r="B603" s="1" t="inlineStr">
         <is>
@@ -46032,15 +46018,15 @@
       </c>
       <c r="E603" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F603" s="1" t="n">
-        <v>6640</v>
+        <v>6605</v>
       </c>
       <c r="G603" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H603" s="1" t="inlineStr">
@@ -46054,7 +46040,7 @@
         </is>
       </c>
       <c r="J603" s="2" t="n">
-        <v>46030.60213634259</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K603" s="2" t="n">
         <v>46034</v>
@@ -46071,7 +46057,7 @@
       </c>
       <c r="N603" s="1" t="n"/>
       <c r="O603" s="2" t="n">
-        <v>46030.63182743055</v>
+        <v>46030.75027241898</v>
       </c>
       <c r="P603" s="1" t="inlineStr">
         <is>
@@ -46092,7 +46078,7 @@
     </row>
     <row r="604">
       <c r="A604" s="1" t="n">
-        <v>76515</v>
+        <v>76505</v>
       </c>
       <c r="B604" s="1" t="inlineStr">
         <is>
@@ -46111,15 +46097,15 @@
       </c>
       <c r="E604" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F604" s="1" t="n">
-        <v>6641</v>
+        <v>6640</v>
       </c>
       <c r="G604" s="1" t="inlineStr">
         <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H604" s="1" t="inlineStr">
@@ -46133,7 +46119,7 @@
         </is>
       </c>
       <c r="J604" s="2" t="n">
-        <v>46030.73046079861</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K604" s="2" t="n">
         <v>46034</v>
@@ -46150,7 +46136,7 @@
       </c>
       <c r="N604" s="1" t="n"/>
       <c r="O604" s="2" t="n">
-        <v>46030.74734336806</v>
+        <v>46030.63182743055</v>
       </c>
       <c r="P604" s="1" t="inlineStr">
         <is>
@@ -46159,7 +46145,7 @@
       </c>
       <c r="Q604" s="1" t="inlineStr">
         <is>
-          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
+          <t>Baixadas.</t>
         </is>
       </c>
       <c r="R604" s="1" t="inlineStr">
@@ -46171,7 +46157,7 @@
     </row>
     <row r="605">
       <c r="A605" s="1" t="n">
-        <v>76501</v>
+        <v>76515</v>
       </c>
       <c r="B605" s="1" t="inlineStr">
         <is>
@@ -46190,7 +46176,7 @@
       </c>
       <c r="E605" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
         </is>
       </c>
       <c r="F605" s="1" t="n">
@@ -46212,7 +46198,7 @@
         </is>
       </c>
       <c r="J605" s="2" t="n">
-        <v>46030.51327708333</v>
+        <v>46030.73046079861</v>
       </c>
       <c r="K605" s="2" t="n">
         <v>46034</v>
@@ -46229,24 +46215,103 @@
       </c>
       <c r="N605" s="1" t="n"/>
       <c r="O605" s="2" t="n">
+        <v>46030.74734336806</v>
+      </c>
+      <c r="P605" s="1" t="inlineStr">
+        <is>
+          <t>nicoleo</t>
+        </is>
+      </c>
+      <c r="Q605" s="1" t="inlineStr">
+        <is>
+          <t>Tarefas se encontram baixadas conforme solicitado no chamado: 76436.</t>
+        </is>
+      </c>
+      <c r="R605" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S605" s="1" t="n"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="1" t="n">
+        <v>76501</v>
+      </c>
+      <c r="B606" s="1" t="inlineStr">
+        <is>
+          <t>MG Controle</t>
+        </is>
+      </c>
+      <c r="C606" s="1" t="inlineStr">
+        <is>
+          <t>Verificar Validação Obrigação</t>
+        </is>
+      </c>
+      <c r="D606" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E606" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+        </is>
+      </c>
+      <c r="F606" s="1" t="n">
+        <v>6641</v>
+      </c>
+      <c r="G606" s="1" t="inlineStr">
+        <is>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+        </is>
+      </c>
+      <c r="H606" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="I606" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLADORIA</t>
+        </is>
+      </c>
+      <c r="J606" s="2" t="n">
+        <v>46030.51327708333</v>
+      </c>
+      <c r="K606" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="L606" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M606" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Castro</t>
+        </is>
+      </c>
+      <c r="N606" s="1" t="n"/>
+      <c r="O606" s="2" t="n">
         <v>46030.64333047454</v>
       </c>
-      <c r="P605" s="1" t="inlineStr">
+      <c r="P606" s="1" t="inlineStr">
         <is>
           <t>nicoleo</t>
         </is>
       </c>
-      <c r="Q605" s="1" t="inlineStr">
+      <c r="Q606" s="1" t="inlineStr">
         <is>
           <t>Baixadas.</t>
         </is>
       </c>
-      <c r="R605" s="1" t="inlineStr">
+      <c r="R606" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="S605" s="1" t="n"/>
+      <c r="S606" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 08-07-26 1616
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -14219,7 +14219,7 @@
       </c>
       <c r="L169" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M169" s="1" t="inlineStr">
@@ -14227,9 +14227,17 @@
           <t>Bruno Contieri</t>
         </is>
       </c>
-      <c r="N169" s="1" t="n"/>
-      <c r="O169" s="1" t="n"/>
-      <c r="P169" s="1" t="inlineStr"/>
+      <c r="N169" s="2" t="n">
+        <v>46183.62114679398</v>
+      </c>
+      <c r="O169" s="2" t="n">
+        <v>46211.66080744213</v>
+      </c>
+      <c r="P169" s="1" t="inlineStr">
+        <is>
+          <t>thaizao</t>
+        </is>
+      </c>
       <c r="Q169" s="1" t="inlineStr">
         <is>
           <t>Aguardando definição gerencia departamento e gerencia operacional</t>
@@ -14237,7 +14245,7 @@
       </c>
       <c r="R169" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S169" s="1" t="n"/>
@@ -18401,7 +18409,7 @@
       </c>
       <c r="L220" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M220" s="1" t="inlineStr">
@@ -18409,9 +18417,17 @@
           <t>Yasmin Peixoto</t>
         </is>
       </c>
-      <c r="N220" s="1" t="n"/>
-      <c r="O220" s="1" t="n"/>
-      <c r="P220" s="1" t="inlineStr"/>
+      <c r="N220" s="2" t="n">
+        <v>46183.62145471065</v>
+      </c>
+      <c r="O220" s="2" t="n">
+        <v>46211.66036420139</v>
+      </c>
+      <c r="P220" s="1" t="inlineStr">
+        <is>
+          <t>thaizao</t>
+        </is>
+      </c>
       <c r="Q220" s="1" t="inlineStr">
         <is>
           <t>Aguardando definição gerencia departamento e gerencia operacional</t>
@@ -18419,7 +18435,7 @@
       </c>
       <c r="R220" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="S220" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 09-07-26 1302
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -141,8 +141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:T586" headerRowCount="1">
-  <autoFilter ref="A1:T586"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:T587" headerRowCount="1">
+  <autoFilter ref="A1:T587"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T586"/>
+  <dimension ref="A1:T587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43749,7 +43749,7 @@
     </row>
     <row r="582">
       <c r="A582" s="1" t="n">
-        <v>80672</v>
+        <v>80930</v>
       </c>
       <c r="B582" s="1" t="inlineStr">
         <is>
@@ -43758,52 +43758,46 @@
       </c>
       <c r="C582" s="1" t="inlineStr">
         <is>
-          <t>Criação de Tarefas</t>
+          <t>Baixa automática - Arquivos</t>
         </is>
       </c>
       <c r="D582" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>RJ - DP</t>
         </is>
       </c>
       <c r="E582" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!!Solicito a criação da tarefa manual: Regularização eSocial - Intermitente. Esta tarefa deverá exigir o e-mail de retorno ao cliente para executar a baixa.</t>
+          <t>Por favor, baixar a tarefa eSocial - Fechamento mensal da empresa 6684 - Nova Moda Comercio de Roupas Calçados e Acessórios, porque a empresa não possui colaboradores ativos.</t>
         </is>
       </c>
       <c r="F582" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G582" s="1" t="n"/>
-      <c r="H582" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H582" s="1" t="n"/>
       <c r="I582" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J582" s="2" t="n">
-        <v>46204.49980644676</v>
+        <v>46212.41216331018</v>
       </c>
       <c r="K582" s="2" t="n">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="L582" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M582" s="1" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
-        </is>
-      </c>
-      <c r="N582" s="2" t="n">
-        <v>46209.45593140047</v>
-      </c>
+          <t>Rosilene Silva</t>
+        </is>
+      </c>
+      <c r="N582" s="1" t="n"/>
       <c r="O582" s="1" t="n"/>
       <c r="P582" s="1" t="n"/>
       <c r="Q582" s="1" t="inlineStr"/>
@@ -43817,7 +43811,7 @@
     </row>
     <row r="583">
       <c r="A583" s="1" t="n">
-        <v>76508</v>
+        <v>80672</v>
       </c>
       <c r="B583" s="1" t="inlineStr">
         <is>
@@ -43826,30 +43820,26 @@
       </c>
       <c r="C583" s="1" t="inlineStr">
         <is>
-          <t>Verificar Validação Obrigação</t>
+          <t>Criação de Tarefas</t>
         </is>
       </c>
       <c r="D583" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E583" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>Bom dia!!Solicito a criação da tarefa manual: Regularização eSocial - Intermitente. Esta tarefa deverá exigir o e-mail de retorno ao cliente para executar a baixa.</t>
         </is>
       </c>
       <c r="F583" s="1" t="n">
-        <v>6605</v>
-      </c>
-      <c r="G583" s="1" t="inlineStr">
-        <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G583" s="1" t="n"/>
       <c r="H583" s="1" t="inlineStr">
         <is>
-          <t>Nicole Oliveira</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I583" s="1" t="inlineStr">
@@ -43858,34 +43848,30 @@
         </is>
       </c>
       <c r="J583" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46204.49980644676</v>
       </c>
       <c r="K583" s="2" t="n">
-        <v>46034</v>
+        <v>46206</v>
       </c>
       <c r="L583" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M583" s="1" t="inlineStr">
         <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N583" s="1" t="n"/>
+          <t>Sara Cavalheiro</t>
+        </is>
+      </c>
+      <c r="N583" s="2" t="n">
+        <v>46209.45593140047</v>
+      </c>
       <c r="O583" s="1" t="n"/>
-      <c r="P583" s="3" t="n">
-        <v>46030.75027241898</v>
-      </c>
-      <c r="Q583" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
+      <c r="P583" s="1" t="n"/>
+      <c r="Q583" s="1" t="inlineStr"/>
       <c r="R583" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S583" s="1" t="n"/>
@@ -43893,7 +43879,7 @@
     </row>
     <row r="584">
       <c r="A584" s="1" t="n">
-        <v>76505</v>
+        <v>76508</v>
       </c>
       <c r="B584" s="1" t="inlineStr">
         <is>
@@ -43912,15 +43898,15 @@
       </c>
       <c r="E584" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F584" s="1" t="n">
-        <v>6640</v>
+        <v>6605</v>
       </c>
       <c r="G584" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H584" s="1" t="inlineStr">
@@ -43934,7 +43920,7 @@
         </is>
       </c>
       <c r="J584" s="2" t="n">
-        <v>46030.60213634259</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K584" s="2" t="n">
         <v>46034</v>
@@ -43952,7 +43938,7 @@
       <c r="N584" s="1" t="n"/>
       <c r="O584" s="1" t="n"/>
       <c r="P584" s="3" t="n">
-        <v>46030.63182743055</v>
+        <v>46030.75027241898</v>
       </c>
       <c r="Q584" s="1" t="inlineStr">
         <is>
@@ -43969,7 +43955,7 @@
     </row>
     <row r="585">
       <c r="A585" s="1" t="n">
-        <v>76515</v>
+        <v>76505</v>
       </c>
       <c r="B585" s="1" t="inlineStr">
         <is>
@@ -43988,15 +43974,15 @@
       </c>
       <c r="E585" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F585" s="1" t="n">
-        <v>6641</v>
+        <v>6640</v>
       </c>
       <c r="G585" s="1" t="inlineStr">
         <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H585" s="1" t="inlineStr">
@@ -44010,7 +43996,7 @@
         </is>
       </c>
       <c r="J585" s="2" t="n">
-        <v>46030.73046079861</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K585" s="2" t="n">
         <v>46034</v>
@@ -44028,7 +44014,7 @@
       <c r="N585" s="1" t="n"/>
       <c r="O585" s="1" t="n"/>
       <c r="P585" s="3" t="n">
-        <v>46030.74734336806</v>
+        <v>46030.63182743055</v>
       </c>
       <c r="Q585" s="1" t="inlineStr">
         <is>
@@ -44045,7 +44031,7 @@
     </row>
     <row r="586">
       <c r="A586" s="1" t="n">
-        <v>76501</v>
+        <v>76515</v>
       </c>
       <c r="B586" s="1" t="inlineStr">
         <is>
@@ -44064,7 +44050,7 @@
       </c>
       <c r="E586" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
         </is>
       </c>
       <c r="F586" s="1" t="n">
@@ -44086,7 +44072,7 @@
         </is>
       </c>
       <c r="J586" s="2" t="n">
-        <v>46030.51327708333</v>
+        <v>46030.73046079861</v>
       </c>
       <c r="K586" s="2" t="n">
         <v>46034</v>
@@ -44104,7 +44090,7 @@
       <c r="N586" s="1" t="n"/>
       <c r="O586" s="1" t="n"/>
       <c r="P586" s="3" t="n">
-        <v>46030.64333047454</v>
+        <v>46030.74734336806</v>
       </c>
       <c r="Q586" s="1" t="inlineStr">
         <is>
@@ -44118,6 +44104,82 @@
       </c>
       <c r="S586" s="1" t="n"/>
       <c r="T586" s="1" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="1" t="n">
+        <v>76501</v>
+      </c>
+      <c r="B587" s="1" t="inlineStr">
+        <is>
+          <t>MG Controle</t>
+        </is>
+      </c>
+      <c r="C587" s="1" t="inlineStr">
+        <is>
+          <t>Verificar Validação Obrigação</t>
+        </is>
+      </c>
+      <c r="D587" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E587" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+        </is>
+      </c>
+      <c r="F587" s="1" t="n">
+        <v>6641</v>
+      </c>
+      <c r="G587" s="1" t="inlineStr">
+        <is>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+        </is>
+      </c>
+      <c r="H587" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="I587" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLADORIA</t>
+        </is>
+      </c>
+      <c r="J587" s="2" t="n">
+        <v>46030.51327708333</v>
+      </c>
+      <c r="K587" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="L587" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M587" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Castro</t>
+        </is>
+      </c>
+      <c r="N587" s="1" t="n"/>
+      <c r="O587" s="1" t="n"/>
+      <c r="P587" s="3" t="n">
+        <v>46030.64333047454</v>
+      </c>
+      <c r="Q587" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="R587" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S587" s="1" t="n"/>
+      <c r="T587" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 09-07-26 1802
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -141,8 +141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:T587" headerRowCount="1">
-  <autoFilter ref="A1:T587"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:T588" headerRowCount="1">
+  <autoFilter ref="A1:T588"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T587"/>
+  <dimension ref="A1:T588"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43811,7 +43811,7 @@
     </row>
     <row r="583">
       <c r="A583" s="1" t="n">
-        <v>80672</v>
+        <v>80933</v>
       </c>
       <c r="B583" s="1" t="inlineStr">
         <is>
@@ -43820,52 +43820,46 @@
       </c>
       <c r="C583" s="1" t="inlineStr">
         <is>
-          <t>Criação de Tarefas</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D583" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>SANTOS - EF</t>
         </is>
       </c>
       <c r="E583" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!!Solicito a criação da tarefa manual: Regularização eSocial - Intermitente. Esta tarefa deverá exigir o e-mail de retorno ao cliente para executar a baixa.</t>
+          <t>Boa tarde, estou com problema para dar baixa na na empresa 2648 - JC Marketing, na tarefa de Reinf. Ao colocar o recibo fica dando erro, e também já tentei pela baixa automatica mas não funcionou.Se possível pode dar baixa pra mim na tarefa.</t>
         </is>
       </c>
       <c r="F583" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G583" s="1" t="n"/>
-      <c r="H583" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H583" s="1" t="n"/>
       <c r="I583" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J583" s="2" t="n">
-        <v>46204.49980644676</v>
+        <v>46212.72987685185</v>
       </c>
       <c r="K583" s="2" t="n">
-        <v>46206</v>
+        <v>46216</v>
       </c>
       <c r="L583" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M583" s="1" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
-        </is>
-      </c>
-      <c r="N583" s="2" t="n">
-        <v>46209.45593140047</v>
-      </c>
+          <t>Jasmina Melo</t>
+        </is>
+      </c>
+      <c r="N583" s="1" t="n"/>
       <c r="O583" s="1" t="n"/>
       <c r="P583" s="1" t="n"/>
       <c r="Q583" s="1" t="inlineStr"/>
@@ -43879,7 +43873,7 @@
     </row>
     <row r="584">
       <c r="A584" s="1" t="n">
-        <v>76508</v>
+        <v>80672</v>
       </c>
       <c r="B584" s="1" t="inlineStr">
         <is>
@@ -43888,30 +43882,26 @@
       </c>
       <c r="C584" s="1" t="inlineStr">
         <is>
-          <t>Verificar Validação Obrigação</t>
+          <t>Criação de Tarefas</t>
         </is>
       </c>
       <c r="D584" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E584" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
+          <t>Bom dia!!Solicito a criação da tarefa manual: Regularização eSocial - Intermitente. Esta tarefa deverá exigir o e-mail de retorno ao cliente para executar a baixa.</t>
         </is>
       </c>
       <c r="F584" s="1" t="n">
-        <v>6605</v>
-      </c>
-      <c r="G584" s="1" t="inlineStr">
-        <is>
-          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G584" s="1" t="n"/>
       <c r="H584" s="1" t="inlineStr">
         <is>
-          <t>Nicole Oliveira</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I584" s="1" t="inlineStr">
@@ -43920,34 +43910,30 @@
         </is>
       </c>
       <c r="J584" s="2" t="n">
-        <v>46030.67108090278</v>
+        <v>46204.49980644676</v>
       </c>
       <c r="K584" s="2" t="n">
-        <v>46034</v>
+        <v>46206</v>
       </c>
       <c r="L584" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M584" s="1" t="inlineStr">
         <is>
-          <t>Bianca Castro</t>
-        </is>
-      </c>
-      <c r="N584" s="1" t="n"/>
+          <t>Sara Cavalheiro</t>
+        </is>
+      </c>
+      <c r="N584" s="2" t="n">
+        <v>46209.45593140047</v>
+      </c>
       <c r="O584" s="1" t="n"/>
-      <c r="P584" s="3" t="n">
-        <v>46030.75027241898</v>
-      </c>
-      <c r="Q584" s="1" t="inlineStr">
-        <is>
-          <t>Nicole Oliveira</t>
-        </is>
-      </c>
+      <c r="P584" s="1" t="n"/>
+      <c r="Q584" s="1" t="inlineStr"/>
       <c r="R584" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="S584" s="1" t="n"/>
@@ -43955,7 +43941,7 @@
     </row>
     <row r="585">
       <c r="A585" s="1" t="n">
-        <v>76505</v>
+        <v>76508</v>
       </c>
       <c r="B585" s="1" t="inlineStr">
         <is>
@@ -43974,15 +43960,15 @@
       </c>
       <c r="E585" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
+          <t>Por favor, fazer baixa das tarefas de cadastro de e-mail para as filiais abaixo, pois só fazemos cadastro para as matrizes6605 - RESTAURANTE FLV RAIZ LTDA (FILIAL 1) SP6606 - RESTAURANTE FLV RAIZ LTDA (FILIAL 2) SP6607 - RESTAURANTE FLV RAIZ LTDA (FILIAL 3) SP6608 - RESTAURANTE FLV RAIZ LTDA (FILIAL 4) SP</t>
         </is>
       </c>
       <c r="F585" s="1" t="n">
-        <v>6640</v>
+        <v>6605</v>
       </c>
       <c r="G585" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>RESTAURANTE FLV RAIZ LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H585" s="1" t="inlineStr">
@@ -43996,7 +43982,7 @@
         </is>
       </c>
       <c r="J585" s="2" t="n">
-        <v>46030.60213634259</v>
+        <v>46030.67108090278</v>
       </c>
       <c r="K585" s="2" t="n">
         <v>46034</v>
@@ -44014,7 +44000,7 @@
       <c r="N585" s="1" t="n"/>
       <c r="O585" s="1" t="n"/>
       <c r="P585" s="3" t="n">
-        <v>46030.63182743055</v>
+        <v>46030.75027241898</v>
       </c>
       <c r="Q585" s="1" t="inlineStr">
         <is>
@@ -44031,7 +44017,7 @@
     </row>
     <row r="586">
       <c r="A586" s="1" t="n">
-        <v>76515</v>
+        <v>76505</v>
       </c>
       <c r="B586" s="1" t="inlineStr">
         <is>
@@ -44050,15 +44036,15 @@
       </c>
       <c r="E586" s="1" t="inlineStr">
         <is>
-          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
+          <t>Boa tarde.Por gentileza, excluir tarefas de Procurações ref a empresa 6640 - FORT FRUIT LTDA, pois a mesma não faz DP com a MG</t>
         </is>
       </c>
       <c r="F586" s="1" t="n">
-        <v>6641</v>
+        <v>6640</v>
       </c>
       <c r="G586" s="1" t="inlineStr">
         <is>
-          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+          <t>FORT FRUIT LTDA</t>
         </is>
       </c>
       <c r="H586" s="1" t="inlineStr">
@@ -44072,7 +44058,7 @@
         </is>
       </c>
       <c r="J586" s="2" t="n">
-        <v>46030.73046079861</v>
+        <v>46030.60213634259</v>
       </c>
       <c r="K586" s="2" t="n">
         <v>46034</v>
@@ -44090,7 +44076,7 @@
       <c r="N586" s="1" t="n"/>
       <c r="O586" s="1" t="n"/>
       <c r="P586" s="3" t="n">
-        <v>46030.74734336806</v>
+        <v>46030.63182743055</v>
       </c>
       <c r="Q586" s="1" t="inlineStr">
         <is>
@@ -44107,7 +44093,7 @@
     </row>
     <row r="587">
       <c r="A587" s="1" t="n">
-        <v>76501</v>
+        <v>76515</v>
       </c>
       <c r="B587" s="1" t="inlineStr">
         <is>
@@ -44126,7 +44112,7 @@
       </c>
       <c r="E587" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+          <t>Por favor, fazer baixa das tarefas de Procurações (DET, CONECTIVIDADE, FGTS, FAP) da empresa 6641 - FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA, pois não tem DP conosco.</t>
         </is>
       </c>
       <c r="F587" s="1" t="n">
@@ -44148,7 +44134,7 @@
         </is>
       </c>
       <c r="J587" s="2" t="n">
-        <v>46030.51327708333</v>
+        <v>46030.73046079861</v>
       </c>
       <c r="K587" s="2" t="n">
         <v>46034</v>
@@ -44166,7 +44152,7 @@
       <c r="N587" s="1" t="n"/>
       <c r="O587" s="1" t="n"/>
       <c r="P587" s="3" t="n">
-        <v>46030.64333047454</v>
+        <v>46030.74734336806</v>
       </c>
       <c r="Q587" s="1" t="inlineStr">
         <is>
@@ -44180,6 +44166,82 @@
       </c>
       <c r="S587" s="1" t="n"/>
       <c r="T587" s="1" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" s="1" t="n">
+        <v>76501</v>
+      </c>
+      <c r="B588" s="1" t="inlineStr">
+        <is>
+          <t>MG Controle</t>
+        </is>
+      </c>
+      <c r="C588" s="1" t="inlineStr">
+        <is>
+          <t>Verificar Validação Obrigação</t>
+        </is>
+      </c>
+      <c r="D588" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E588" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.Por favor, fazer baixa da tarefa de cadastro de e-mail Dec Municipal da loja 6640 - FORT FRUIT LTDA SP, pois a mesma não faz parte do município de SP</t>
+        </is>
+      </c>
+      <c r="F588" s="1" t="n">
+        <v>6641</v>
+      </c>
+      <c r="G588" s="1" t="inlineStr">
+        <is>
+          <t>FORT-FRUIT COMERCIO E DISTRIBUICAO LTDA</t>
+        </is>
+      </c>
+      <c r="H588" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="I588" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLADORIA</t>
+        </is>
+      </c>
+      <c r="J588" s="2" t="n">
+        <v>46030.51327708333</v>
+      </c>
+      <c r="K588" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="L588" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M588" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Castro</t>
+        </is>
+      </c>
+      <c r="N588" s="1" t="n"/>
+      <c r="O588" s="1" t="n"/>
+      <c r="P588" s="3" t="n">
+        <v>46030.64333047454</v>
+      </c>
+      <c r="Q588" s="1" t="inlineStr">
+        <is>
+          <t>Nicole Oliveira</t>
+        </is>
+      </c>
+      <c r="R588" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="S588" s="1" t="n"/>
+      <c r="T588" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 13-07-26 0903
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U301" headerRowCount="1">
-  <autoFilter ref="A1:U301"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U299" headerRowCount="1">
+  <autoFilter ref="A1:U299"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U301"/>
+  <dimension ref="A1:U299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5597,7 +5597,11 @@
           <t>PRISTELA PIZZARIA LTDA</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n"/>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I62" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -5611,7 +5615,7 @@
       </c>
       <c r="L62" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M62" s="1" t="inlineStr">
@@ -5623,14 +5627,18 @@
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="n"/>
       <c r="Q62" s="1" t="inlineStr"/>
-      <c r="R62" s="1" t="n"/>
+      <c r="R62" s="1" t="inlineStr"/>
       <c r="S62" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T62" s="1" t="n"/>
-      <c r="U62" s="1" t="inlineStr"/>
+      <c r="U62" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -7791,7 +7799,7 @@
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I89" s="1" t="inlineStr">
@@ -7807,7 +7815,7 @@
       </c>
       <c r="L89" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M89" s="1" t="inlineStr">
@@ -7815,11 +7823,18 @@
           <t>Simone Marques</t>
         </is>
       </c>
-      <c r="N89" s="1" t="n"/>
+      <c r="N89" s="2" t="n">
+        <v>46216.36492291667</v>
+      </c>
       <c r="O89" s="1" t="n"/>
       <c r="P89" s="1" t="n"/>
       <c r="Q89" s="1" t="inlineStr"/>
-      <c r="R89" s="1" t="inlineStr"/>
+      <c r="R89" s="1" t="inlineStr">
+        <is>
+          <t>operação em validação 
+25-07</t>
+        </is>
+      </c>
       <c r="S89" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -8772,7 +8787,7 @@
       </c>
       <c r="L101" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M101" s="1" t="inlineStr">
@@ -8782,14 +8797,8 @@
       </c>
       <c r="N101" s="1" t="n"/>
       <c r="O101" s="1" t="n"/>
-      <c r="P101" s="2" t="n">
-        <v>46213.47285034722</v>
-      </c>
-      <c r="Q101" s="1" t="inlineStr">
-        <is>
-          <t>Fernanda Araujo</t>
-        </is>
-      </c>
+      <c r="P101" s="1" t="n"/>
+      <c r="Q101" s="1" t="inlineStr"/>
       <c r="R101" s="1" t="inlineStr">
         <is>
           <t>Bom dia!
@@ -8798,7 +8807,7 @@
       </c>
       <c r="S101" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T101" s="1" t="n"/>
@@ -9924,7 +9933,11 @@
           <t>PERFIL REFRIGERAÇÃO INDUSTRIA ,COMÉRCIO E SERVIÇO LTDA</t>
         </is>
       </c>
-      <c r="H115" s="1" t="n"/>
+      <c r="H115" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I115" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -9938,7 +9951,7 @@
       </c>
       <c r="L115" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M115" s="1" t="inlineStr">
@@ -9950,14 +9963,18 @@
       <c r="O115" s="1" t="n"/>
       <c r="P115" s="1" t="n"/>
       <c r="Q115" s="1" t="inlineStr"/>
-      <c r="R115" s="1" t="n"/>
+      <c r="R115" s="1" t="inlineStr"/>
       <c r="S115" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T115" s="1" t="n"/>
-      <c r="U115" s="1" t="inlineStr"/>
+      <c r="U115" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -11922,7 +11939,11 @@
           <t>MAC FRIO DISTRIBUIDORA LTDA</t>
         </is>
       </c>
-      <c r="H139" s="1" t="n"/>
+      <c r="H139" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="I139" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -11936,7 +11957,7 @@
       </c>
       <c r="L139" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M139" s="1" t="inlineStr">
@@ -11944,18 +11965,29 @@
           <t>Vander Silva</t>
         </is>
       </c>
-      <c r="N139" s="1" t="n"/>
+      <c r="N139" s="2" t="n">
+        <v>46216.373265625</v>
+      </c>
       <c r="O139" s="1" t="n"/>
       <c r="P139" s="1" t="n"/>
       <c r="Q139" s="1" t="inlineStr"/>
-      <c r="R139" s="1" t="n"/>
+      <c r="R139" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPERAÇÃO EM FASE DE EXECUÇÃO 
+</t>
+        </is>
+      </c>
       <c r="S139" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T139" s="1" t="n"/>
-      <c r="U139" s="1" t="inlineStr"/>
+      <c r="U139" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -11989,7 +12021,11 @@
           <t>M &amp; M INDUSTRIA E COMERCIO LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H140" s="1" t="n"/>
+      <c r="H140" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="I140" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -12003,7 +12039,7 @@
       </c>
       <c r="L140" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M140" s="1" t="inlineStr">
@@ -12011,18 +12047,28 @@
           <t>Vander Silva</t>
         </is>
       </c>
-      <c r="N140" s="1" t="n"/>
+      <c r="N140" s="2" t="n">
+        <v>46216.37073711806</v>
+      </c>
       <c r="O140" s="1" t="n"/>
       <c r="P140" s="1" t="n"/>
       <c r="Q140" s="1" t="inlineStr"/>
-      <c r="R140" s="1" t="n"/>
+      <c r="R140" s="1" t="inlineStr">
+        <is>
+          <t>OPERAÇÃO IRÁ REALIZAR A ENTREGA</t>
+        </is>
+      </c>
       <c r="S140" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T140" s="1" t="n"/>
-      <c r="U140" s="1" t="inlineStr"/>
+      <c r="U140" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -13276,7 +13322,11 @@
           <t>AMATRUDA LOCADORA DE GUINDASTES E ARTICULADOS LTDA</t>
         </is>
       </c>
-      <c r="H156" s="1" t="n"/>
+      <c r="H156" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I156" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -13290,7 +13340,7 @@
       </c>
       <c r="L156" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M156" s="1" t="inlineStr">
@@ -13302,14 +13352,18 @@
       <c r="O156" s="1" t="n"/>
       <c r="P156" s="1" t="n"/>
       <c r="Q156" s="1" t="inlineStr"/>
-      <c r="R156" s="1" t="n"/>
+      <c r="R156" s="1" t="inlineStr"/>
       <c r="S156" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T156" s="1" t="n"/>
-      <c r="U156" s="1" t="inlineStr"/>
+      <c r="U156" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -14235,7 +14289,11 @@
           <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
         </is>
       </c>
-      <c r="H168" s="1" t="n"/>
+      <c r="H168" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="I168" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14249,7 +14307,7 @@
       </c>
       <c r="L168" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M168" s="1" t="inlineStr">
@@ -14257,18 +14315,28 @@
           <t>Rogerio Egidio</t>
         </is>
       </c>
-      <c r="N168" s="1" t="n"/>
+      <c r="N168" s="2" t="n">
+        <v>46216.37496550926</v>
+      </c>
       <c r="O168" s="1" t="n"/>
       <c r="P168" s="1" t="n"/>
       <c r="Q168" s="1" t="inlineStr"/>
-      <c r="R168" s="1" t="n"/>
+      <c r="R168" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EM EXECUÇÃO PELA OPERAÇÃO </t>
+        </is>
+      </c>
       <c r="S168" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T168" s="1" t="n"/>
-      <c r="U168" s="1" t="inlineStr"/>
+      <c r="U168" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -14390,7 +14458,7 @@
       </c>
       <c r="H170" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I170" s="1" t="inlineStr">
@@ -14406,7 +14474,7 @@
       </c>
       <c r="L170" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M170" s="1" t="inlineStr">
@@ -14416,12 +14484,22 @@
       </c>
       <c r="N170" s="1" t="n"/>
       <c r="O170" s="1" t="n"/>
-      <c r="P170" s="1" t="n"/>
-      <c r="Q170" s="1" t="inlineStr"/>
-      <c r="R170" s="1" t="inlineStr"/>
+      <c r="P170" s="2" t="n">
+        <v>46216.37008005787</v>
+      </c>
+      <c r="Q170" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R170" s="1" t="inlineStr">
+        <is>
+          <t>PRCOESSO REALIZADO EM 10-07-2026</t>
+        </is>
+      </c>
       <c r="S170" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T170" s="1" t="n"/>
@@ -14463,7 +14541,11 @@
           <t xml:space="preserve">MAGAZINE DAS PANELAS LTDA </t>
         </is>
       </c>
-      <c r="H171" s="1" t="n"/>
+      <c r="H171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I171" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14477,7 +14559,7 @@
       </c>
       <c r="L171" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M171" s="1" t="inlineStr">
@@ -14489,14 +14571,18 @@
       <c r="O171" s="1" t="n"/>
       <c r="P171" s="1" t="n"/>
       <c r="Q171" s="1" t="inlineStr"/>
-      <c r="R171" s="1" t="n"/>
+      <c r="R171" s="1" t="inlineStr"/>
       <c r="S171" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T171" s="1" t="n"/>
-      <c r="U171" s="1" t="inlineStr"/>
+      <c r="U171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -24025,132 +24111,6 @@
       <c r="T299" s="1" t="n"/>
       <c r="U299" s="1" t="inlineStr"/>
     </row>
-    <row r="300">
-      <c r="A300" s="1" t="n">
-        <v>80949</v>
-      </c>
-      <c r="B300" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C300" s="1" t="inlineStr">
-        <is>
-          <t>Erro de Baixa</t>
-        </is>
-      </c>
-      <c r="D300" s="1" t="inlineStr">
-        <is>
-          <t>RJ - EF</t>
-        </is>
-      </c>
-      <c r="E300" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde, poderiam por gentileza baixar a tarefa "confirmação de faturamento"empresas;6957/6965motivo; empresas simples nacional.At.te</t>
-        </is>
-      </c>
-      <c r="F300" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G300" s="1" t="n"/>
-      <c r="H300" s="1" t="n"/>
-      <c r="I300" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J300" s="2" t="n">
-        <v>46213.65257700231</v>
-      </c>
-      <c r="K300" s="2" t="n">
-        <v>46216</v>
-      </c>
-      <c r="L300" s="1" t="inlineStr">
-        <is>
-          <t>Sem Responsavel Atribuido</t>
-        </is>
-      </c>
-      <c r="M300" s="1" t="inlineStr">
-        <is>
-          <t>Beatriz Oliveira</t>
-        </is>
-      </c>
-      <c r="N300" s="1" t="n"/>
-      <c r="O300" s="1" t="n"/>
-      <c r="P300" s="1" t="n"/>
-      <c r="Q300" s="1" t="inlineStr"/>
-      <c r="R300" s="1" t="n"/>
-      <c r="S300" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T300" s="1" t="n"/>
-      <c r="U300" s="1" t="inlineStr"/>
-    </row>
-    <row r="301">
-      <c r="A301" s="1" t="n">
-        <v>80950</v>
-      </c>
-      <c r="B301" s="1" t="inlineStr">
-        <is>
-          <t>MG Controle</t>
-        </is>
-      </c>
-      <c r="C301" s="1" t="inlineStr">
-        <is>
-          <t>Erro de Baixa</t>
-        </is>
-      </c>
-      <c r="D301" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E301" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!Por favor baixar  a tarefa eSocial - Fechamento Mensal da empresa 2791, erro no relatório de base s5012.</t>
-        </is>
-      </c>
-      <c r="F301" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G301" s="1" t="n"/>
-      <c r="H301" s="1" t="n"/>
-      <c r="I301" s="1" t="inlineStr">
-        <is>
-          <t>CONTROLADORIA</t>
-        </is>
-      </c>
-      <c r="J301" s="2" t="n">
-        <v>46213.66592195602</v>
-      </c>
-      <c r="K301" s="2" t="n">
-        <v>46216</v>
-      </c>
-      <c r="L301" s="1" t="inlineStr">
-        <is>
-          <t>Sem Responsavel Atribuido</t>
-        </is>
-      </c>
-      <c r="M301" s="1" t="inlineStr">
-        <is>
-          <t>Edivaldo Veiga</t>
-        </is>
-      </c>
-      <c r="N301" s="1" t="n"/>
-      <c r="O301" s="1" t="n"/>
-      <c r="P301" s="1" t="n"/>
-      <c r="Q301" s="1" t="inlineStr"/>
-      <c r="R301" s="1" t="n"/>
-      <c r="S301" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T301" s="1" t="n"/>
-      <c r="U301" s="1" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
data: atualização base chamados 15-07-26 1524
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U304" headerRowCount="1">
-  <autoFilter ref="A1:U304"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U308" headerRowCount="1">
+  <autoFilter ref="A1:U308"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U304"/>
+  <dimension ref="A1:U308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21556,63 +21556,59 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>76498</v>
+        <v>81075</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C267" s="1" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t>Reabertura de tarefa</t>
         </is>
       </c>
       <c r="D267" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E267" s="1" t="inlineStr">
         <is>
-          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
+          <t>Favor reabrir a tarefa E-SOCIAL e FGTS, EMPRESA KAÇULA, AMBOS tiveram alterações devido correção na folha.</t>
         </is>
       </c>
       <c r="F267" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G267" s="1" t="n"/>
-      <c r="H267" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H267" s="1" t="n"/>
       <c r="I267" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46030.50436203703</v>
+        <v>46218.60342256945</v>
       </c>
       <c r="K267" s="2" t="n">
-        <v>46031</v>
+        <v>46219</v>
       </c>
       <c r="L267" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M267" s="1" t="inlineStr">
         <is>
-          <t>Alaine Neres</t>
+          <t>Camila Oliveira</t>
         </is>
       </c>
       <c r="N267" s="1" t="n"/>
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
       <c r="Q267" s="1" t="inlineStr"/>
-      <c r="R267" s="1" t="inlineStr"/>
+      <c r="R267" s="1" t="n"/>
       <c r="S267" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21623,63 +21619,59 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>76514</v>
+        <v>81076</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
         <is>
-          <t>RJ - EF</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
+          <t>Pessoal, boa tardepor favor baixar a tarefa de REINF da empresa 5835 - CAETE 06/2026esta dando erro de layout pq tivemos que tirar o recibo do ECAC, sci estava com erro.</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G268" s="1" t="n"/>
-      <c r="H268" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H268" s="1" t="n"/>
       <c r="I268" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46030.72255292824</v>
+        <v>46218.61204498843</v>
       </c>
       <c r="K268" s="2" t="n">
-        <v>46031</v>
+        <v>46219</v>
       </c>
       <c r="L268" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M268" s="1" t="inlineStr">
         <is>
-          <t>Glaucia Santos</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="N268" s="1" t="n"/>
       <c r="O268" s="1" t="n"/>
       <c r="P268" s="1" t="n"/>
       <c r="Q268" s="1" t="inlineStr"/>
-      <c r="R268" s="1" t="inlineStr"/>
+      <c r="R268" s="1" t="n"/>
       <c r="S268" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21690,63 +21682,59 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>76892</v>
+        <v>81077</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Baixa automática - Arquivos</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - DP</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
+          <t xml:space="preserve">Boa tarde, pode por favor baixar a tarefa FGTS das empresas 6535 e 6865, uma não possui funcionário e a outra é filial. </t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G269" s="1" t="n"/>
-      <c r="H269" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H269" s="1" t="n"/>
       <c r="I269" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46051.62030378472</v>
+        <v>46218.61339695602</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>46052</v>
+        <v>46219</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Bruna Silva</t>
         </is>
       </c>
       <c r="N269" s="1" t="n"/>
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
       <c r="Q269" s="1" t="inlineStr"/>
-      <c r="R269" s="1" t="inlineStr"/>
+      <c r="R269" s="1" t="n"/>
       <c r="S269" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21757,63 +21745,59 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>77913</v>
+        <v>81078</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C270" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D270" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>Boa tarde!Favor baixar a tarefa Envio de Impostos DCTF Web com os documentos em anexo das lojas 4833, 5020, 5023 e 5197 enviadas por e-mail ao cliente. Em tentativa de baixar, aparece o erro "Não foi possivel efetuar a leitura do arquivo. O mesmo pode estar criptografado ou corrompido."</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G270" s="1" t="n"/>
-      <c r="H270" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H270" s="1" t="n"/>
       <c r="I270" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46218.62635208333</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46097</v>
+        <v>46219</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
+          <t>Aline Petrini</t>
         </is>
       </c>
       <c r="N270" s="1" t="n"/>
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="inlineStr"/>
+      <c r="R270" s="1" t="n"/>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21824,59 +21808,63 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>79609</v>
+        <v>76498</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Endereço</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G271" s="1" t="n"/>
-      <c r="H271" s="1" t="n"/>
+      <c r="H271" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I271" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46030.50436203703</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46205</v>
+        <v>46031</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Alaine Neres</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="Q271" s="1" t="inlineStr"/>
-      <c r="R271" s="1" t="n"/>
+      <c r="R271" s="1" t="inlineStr"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21887,26 +21875,26 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>80515</v>
+        <v>76514</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>RJ - EF</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -21924,10 +21912,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46030.72255292824</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46226</v>
+        <v>46031</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -21936,7 +21924,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Glaucia Santos</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -21954,59 +21942,63 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80697</v>
+        <v>76892</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G273" s="1" t="n"/>
-      <c r="H273" s="1" t="n"/>
+      <c r="H273" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I273" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46051.62030378472</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46237</v>
+        <v>46052</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="n"/>
+      <c r="R273" s="1" t="inlineStr"/>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22017,59 +22009,63 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80714</v>
+        <v>77913</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G274" s="1" t="n"/>
-      <c r="H274" s="1" t="n"/>
+      <c r="H274" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I274" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46241</v>
+        <v>46097</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Larissa Félix</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="Q274" s="1" t="inlineStr"/>
-      <c r="R274" s="1" t="n"/>
+      <c r="R274" s="1" t="inlineStr"/>
       <c r="S274" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22080,16 +22076,16 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>80919</v>
+        <v>79609</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
@@ -22099,7 +22095,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22113,10 +22109,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46239</v>
+        <v>46205</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22125,7 +22121,7 @@
       </c>
       <c r="M275" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="N275" s="1" t="n"/>
@@ -22143,7 +22139,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>80935</v>
+        <v>80515</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22152,7 +22148,7 @@
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
@@ -22162,28 +22158,32 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G276" s="1" t="n"/>
-      <c r="H276" s="1" t="n"/>
+      <c r="H276" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I276" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46241</v>
+        <v>46226</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
@@ -22195,7 +22195,7 @@
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="n"/>
+      <c r="R276" s="1" t="inlineStr"/>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22206,7 +22206,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80936</v>
+        <v>80697</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22215,7 +22215,7 @@
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22225,7 +22225,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22239,10 +22239,10 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
@@ -22269,7 +22269,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80951</v>
+        <v>80714</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22278,7 +22278,7 @@
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22288,7 +22288,7 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22302,7 +22302,7 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K278" s="2" t="n">
         <v>46241</v>
@@ -22332,63 +22332,59 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80989</v>
+        <v>80919</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G279" s="1" t="n"/>
-      <c r="H279" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+      <c r="H279" s="1" t="n"/>
       <c r="I279" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46217</v>
+        <v>46239</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="inlineStr"/>
+      <c r="R279" s="1" t="n"/>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22399,26 +22395,26 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80995</v>
+        <v>80935</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22432,10 +22428,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46217.33131420139</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46219</v>
+        <v>46241</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22444,7 +22440,7 @@
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>Jonatan Hayashibara</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N280" s="1" t="n"/>
@@ -22462,67 +22458,59 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>79793</v>
+        <v>80936</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G281" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
-      <c r="H281" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G281" s="1" t="n"/>
+      <c r="H281" s="1" t="n"/>
       <c r="I281" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46185</v>
+        <v>46241</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="Q281" s="1" t="inlineStr"/>
-      <c r="R281" s="1" t="inlineStr"/>
+      <c r="R281" s="1" t="n"/>
       <c r="S281" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22533,26 +22521,26 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>81068</v>
+        <v>80951</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22566,10 +22554,10 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46218.47815153936</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46220</v>
+        <v>46241</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
@@ -22578,7 +22566,7 @@
       </c>
       <c r="M282" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N282" s="1" t="n"/>
@@ -22596,11 +22584,11 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>81070</v>
+        <v>80989</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
@@ -22615,40 +22603,44 @@
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G283" s="1" t="n"/>
-      <c r="H283" s="1" t="n"/>
+      <c r="H283" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I283" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46218.51467572917</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46220</v>
+        <v>46217</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>João Oliveira</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="n"/>
+      <c r="R283" s="1" t="inlineStr"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22659,7 +22651,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>81071</v>
+        <v>80995</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
@@ -22673,12 +22665,12 @@
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
+          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22692,10 +22684,10 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46218.51533788195</v>
+        <v>46217.33131420139</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
@@ -22704,7 +22696,7 @@
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Jonatan Hayashibara</t>
         </is>
       </c>
       <c r="N284" s="1" t="n"/>
@@ -22722,59 +22714,67 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>81072</v>
+        <v>79793</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G285" s="1" t="n"/>
-      <c r="H285" s="1" t="n"/>
+        <v>5655</v>
+      </c>
+      <c r="G285" s="1" t="inlineStr">
+        <is>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
+      <c r="H285" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I285" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46218.51577677084</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46220</v>
+        <v>46185</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="n"/>
+      <c r="R285" s="1" t="inlineStr"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22785,16 +22785,16 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>81004</v>
+        <v>81068</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
@@ -22804,17 +22804,13 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6869</v>
-      </c>
-      <c r="G286" s="1" t="inlineStr">
-        <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G286" s="1" t="n"/>
       <c r="H286" s="1" t="n"/>
       <c r="I286" s="1" t="inlineStr">
         <is>
@@ -22822,10 +22818,10 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46218.47815153936</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
@@ -22834,7 +22830,7 @@
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N286" s="1" t="n"/>
@@ -22852,16 +22848,16 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81005</v>
+        <v>81070</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
@@ -22871,17 +22867,13 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6870</v>
-      </c>
-      <c r="G287" s="1" t="inlineStr">
-        <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G287" s="1" t="n"/>
       <c r="H287" s="1" t="n"/>
       <c r="I287" s="1" t="inlineStr">
         <is>
@@ -22889,10 +22881,10 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46218.51467572917</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
@@ -22901,7 +22893,7 @@
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N287" s="1" t="n"/>
@@ -22919,7 +22911,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>80961</v>
+        <v>81071</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -22938,17 +22930,13 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>6950</v>
-      </c>
-      <c r="G288" s="1" t="inlineStr">
-        <is>
-          <t>MERCH LTDA (FILIAL 1)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G288" s="1" t="n"/>
       <c r="H288" s="1" t="n"/>
       <c r="I288" s="1" t="inlineStr">
         <is>
@@ -22956,10 +22944,10 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46216.41692731481</v>
+        <v>46218.51533788195</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -22968,7 +22956,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -22986,67 +22974,59 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>79856</v>
+        <v>81072</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C289" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D289" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>4225</v>
-      </c>
-      <c r="G289" s="1" t="inlineStr">
-        <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
-        </is>
-      </c>
-      <c r="H289" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G289" s="1" t="n"/>
+      <c r="H289" s="1" t="n"/>
       <c r="I289" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46218.51577677084</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46184</v>
+        <v>46220</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
       <c r="Q289" s="1" t="inlineStr"/>
-      <c r="R289" s="1" t="inlineStr"/>
+      <c r="R289" s="1" t="n"/>
       <c r="S289" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23057,67 +23037,63 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79855</v>
+        <v>81004</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>4765</v>
+        <v>6869</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
-        </is>
-      </c>
-      <c r="H290" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+        </is>
+      </c>
+      <c r="H290" s="1" t="n"/>
       <c r="I290" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
-      <c r="R290" s="1" t="inlineStr"/>
+      <c r="R290" s="1" t="n"/>
       <c r="S290" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23128,67 +23104,63 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>79833</v>
+        <v>81005</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6125</v>
+        <v>6870</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H291" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>AC HOME PET RAÇÕES LTDA</t>
+        </is>
+      </c>
+      <c r="H291" s="1" t="n"/>
       <c r="I291" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46184</v>
+        <v>46218</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
       <c r="Q291" s="1" t="inlineStr"/>
-      <c r="R291" s="1" t="inlineStr"/>
+      <c r="R291" s="1" t="n"/>
       <c r="S291" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23199,67 +23171,63 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>79834</v>
+        <v>80961</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6162</v>
+        <v>6950</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
-        </is>
-      </c>
-      <c r="H292" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>MERCH LTDA (FILIAL 1)</t>
+        </is>
+      </c>
+      <c r="H292" s="1" t="n"/>
       <c r="I292" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46216.41692731481</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46184</v>
+        <v>46218</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N292" s="1" t="n"/>
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
       <c r="Q292" s="1" t="inlineStr"/>
-      <c r="R292" s="1" t="inlineStr"/>
+      <c r="R292" s="1" t="n"/>
       <c r="S292" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23270,7 +23238,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79865</v>
+        <v>79856</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
@@ -23289,15 +23257,15 @@
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6278</v>
+        <v>4225</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H293" s="1" t="inlineStr">
@@ -23311,10 +23279,10 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
@@ -23323,7 +23291,7 @@
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N293" s="1" t="n"/>
@@ -23341,7 +23309,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79854</v>
+        <v>79855</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
@@ -23360,15 +23328,15 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>6302</v>
+        <v>4765</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
@@ -23382,10 +23350,10 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L294" s="1" t="inlineStr">
         <is>
@@ -23412,16 +23380,16 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79863</v>
+        <v>79833</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
@@ -23431,15 +23399,15 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6404</v>
+        <v>6125</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
@@ -23453,10 +23421,10 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K295" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L295" s="1" t="inlineStr">
         <is>
@@ -23465,7 +23433,7 @@
       </c>
       <c r="M295" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N295" s="1" t="n"/>
@@ -23483,7 +23451,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>79835</v>
+        <v>79834</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23506,11 +23474,11 @@
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>6485</v>
+        <v>6162</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
@@ -23524,7 +23492,7 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K296" s="2" t="n">
         <v>46184</v>
@@ -23554,7 +23522,7 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79866</v>
+        <v>79865</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
@@ -23573,15 +23541,15 @@
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>6539</v>
+        <v>6278</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H297" s="1" t="inlineStr">
@@ -23595,7 +23563,7 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K297" s="2" t="n">
         <v>46185</v>
@@ -23625,7 +23593,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>79859</v>
+        <v>79854</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23644,15 +23612,15 @@
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>6570</v>
+        <v>6302</v>
       </c>
       <c r="G298" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H298" s="1" t="inlineStr">
@@ -23666,10 +23634,10 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
@@ -23678,7 +23646,7 @@
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
@@ -23696,7 +23664,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>79860</v>
+        <v>79863</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
@@ -23715,15 +23683,15 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>6581</v>
+        <v>6404</v>
       </c>
       <c r="G299" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H299" s="1" t="inlineStr">
@@ -23737,7 +23705,7 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K299" s="2" t="n">
         <v>46185</v>
@@ -23767,16 +23735,16 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>79861</v>
+        <v>79835</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C300" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D300" s="1" t="inlineStr">
@@ -23786,15 +23754,15 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>6583</v>
+        <v>6485</v>
       </c>
       <c r="G300" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H300" s="1" t="inlineStr">
@@ -23808,10 +23776,10 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
@@ -23820,7 +23788,7 @@
       </c>
       <c r="M300" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N300" s="1" t="n"/>
@@ -23838,16 +23806,16 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>79867</v>
+        <v>79866</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C301" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D301" s="1" t="inlineStr">
@@ -23857,15 +23825,15 @@
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>6704</v>
+        <v>6539</v>
       </c>
       <c r="G301" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H301" s="1" t="inlineStr">
@@ -23879,7 +23847,7 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K301" s="2" t="n">
         <v>46185</v>
@@ -23909,32 +23877,36 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>81019</v>
+        <v>79859</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C302" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D302" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G302" s="1" t="n"/>
+        <v>6570</v>
+      </c>
+      <c r="G302" s="1" t="inlineStr">
+        <is>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+        </is>
+      </c>
       <c r="H302" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23946,10 +23918,10 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K302" s="2" t="n">
-        <v>46218</v>
+        <v>46185</v>
       </c>
       <c r="L302" s="1" t="inlineStr">
         <is>
@@ -23958,7 +23930,7 @@
       </c>
       <c r="M302" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N302" s="1" t="n"/>
@@ -23976,32 +23948,36 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>81052</v>
+        <v>79860</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C303" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D303" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G303" s="1" t="n"/>
+        <v>6581</v>
+      </c>
+      <c r="G303" s="1" t="inlineStr">
+        <is>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+        </is>
+      </c>
       <c r="H303" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24013,10 +23989,10 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K303" s="2" t="n">
-        <v>46219</v>
+        <v>46185</v>
       </c>
       <c r="L303" s="1" t="inlineStr">
         <is>
@@ -24025,7 +24001,7 @@
       </c>
       <c r="M303" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N303" s="1" t="n"/>
@@ -24043,32 +24019,36 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>81055</v>
+        <v>79861</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C304" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D304" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G304" s="1" t="n"/>
+        <v>6583</v>
+      </c>
+      <c r="G304" s="1" t="inlineStr">
+        <is>
+          <t>DROGA MX LTDA (MATRIZ)</t>
+        </is>
+      </c>
       <c r="H304" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24080,10 +24060,10 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K304" s="2" t="n">
-        <v>46219</v>
+        <v>46185</v>
       </c>
       <c r="L304" s="1" t="inlineStr">
         <is>
@@ -24092,7 +24072,7 @@
       </c>
       <c r="M304" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N304" s="1" t="n"/>
@@ -24107,6 +24087,278 @@
       </c>
       <c r="T304" s="1" t="n"/>
       <c r="U304" s="1" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="1" t="n">
+        <v>79867</v>
+      </c>
+      <c r="B305" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C305" s="1" t="inlineStr">
+        <is>
+          <t>Implantação Contábil</t>
+        </is>
+      </c>
+      <c r="D305" s="1" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL VAREJO</t>
+        </is>
+      </c>
+      <c r="E305" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+        </is>
+      </c>
+      <c r="F305" s="1" t="n">
+        <v>6704</v>
+      </c>
+      <c r="G305" s="1" t="inlineStr">
+        <is>
+          <t>TECNO COM INFORMATICA LTDA</t>
+        </is>
+      </c>
+      <c r="H305" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I305" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="n">
+        <v>46183.62582114583</v>
+      </c>
+      <c r="K305" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="L305" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M305" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N305" s="1" t="n"/>
+      <c r="O305" s="1" t="n"/>
+      <c r="P305" s="1" t="n"/>
+      <c r="Q305" s="1" t="inlineStr"/>
+      <c r="R305" s="1" t="inlineStr"/>
+      <c r="S305" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T305" s="1" t="n"/>
+      <c r="U305" s="1" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="1" t="n">
+        <v>81019</v>
+      </c>
+      <c r="B306" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C306" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D306" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E306" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+        </is>
+      </c>
+      <c r="F306" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" s="1" t="n"/>
+      <c r="H306" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I306" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="n">
+        <v>46217.43210269676</v>
+      </c>
+      <c r="K306" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="L306" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M306" s="1" t="inlineStr">
+        <is>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N306" s="1" t="n"/>
+      <c r="O306" s="1" t="n"/>
+      <c r="P306" s="1" t="n"/>
+      <c r="Q306" s="1" t="inlineStr"/>
+      <c r="R306" s="1" t="inlineStr"/>
+      <c r="S306" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T306" s="1" t="n"/>
+      <c r="U306" s="1" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="1" t="n">
+        <v>81052</v>
+      </c>
+      <c r="B307" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C307" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D307" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E307" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+        </is>
+      </c>
+      <c r="F307" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" s="1" t="n"/>
+      <c r="H307" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I307" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="n">
+        <v>46218.38736744213</v>
+      </c>
+      <c r="K307" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L307" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M307" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N307" s="1" t="n"/>
+      <c r="O307" s="1" t="n"/>
+      <c r="P307" s="1" t="n"/>
+      <c r="Q307" s="1" t="inlineStr"/>
+      <c r="R307" s="1" t="inlineStr"/>
+      <c r="S307" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T307" s="1" t="n"/>
+      <c r="U307" s="1" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="1" t="n">
+        <v>81055</v>
+      </c>
+      <c r="B308" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C308" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D308" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E308" s="1" t="inlineStr">
+        <is>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+        </is>
+      </c>
+      <c r="F308" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" s="1" t="n"/>
+      <c r="H308" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I308" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="n">
+        <v>46218.40379614583</v>
+      </c>
+      <c r="K308" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L308" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M308" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N308" s="1" t="n"/>
+      <c r="O308" s="1" t="n"/>
+      <c r="P308" s="1" t="n"/>
+      <c r="Q308" s="1" t="inlineStr"/>
+      <c r="R308" s="1" t="inlineStr"/>
+      <c r="S308" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T308" s="1" t="n"/>
+      <c r="U308" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 15-07-26 1803
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U309" headerRowCount="1">
-  <autoFilter ref="A1:U309"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U308" headerRowCount="1">
+  <autoFilter ref="A1:U308"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U309"/>
+  <dimension ref="A1:U308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21629,7 +21629,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>81082</v>
+        <v>81083</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
@@ -21638,53 +21638,67 @@
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t>Tarefas baixadas - Ausência de Arquivos</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>Baixar tarefa GFD 3458 funcionarios afastados não tem guia.</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G268" s="1" t="n"/>
-      <c r="H268" s="1" t="n"/>
+      <c r="H268" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I268" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46218.68031246528</v>
+        <v>46218.68119872685</v>
       </c>
       <c r="K268" s="2" t="n">
-        <v>46223</v>
+        <v>46219</v>
       </c>
       <c r="L268" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M268" s="1" t="inlineStr">
         <is>
-          <t>Erica Oliveira</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N268" s="1" t="n"/>
       <c r="O268" s="1" t="n"/>
-      <c r="P268" s="1" t="n"/>
-      <c r="Q268" s="1" t="inlineStr"/>
-      <c r="R268" s="1" t="n"/>
+      <c r="P268" s="2" t="n">
+        <v>46218.7466727662</v>
+      </c>
+      <c r="Q268" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
+      <c r="R268" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+        </is>
+      </c>
       <c r="S268" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T268" s="1" t="n"/>
@@ -21692,7 +21706,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>81083</v>
+        <v>81087</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
@@ -21701,50 +21715,54 @@
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Forçar baixa de tarefas via banco de dados</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde,Por favor baixar a tarefa "retificação FOPAG FOPAG 062026 das empresa 1330 e 2607, está pedindo para anexar arquivo, mas, não tem modelo fixado como exemplo.Obrigado</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G269" s="1" t="n"/>
-      <c r="H269" s="1" t="n"/>
+      <c r="H269" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I269" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46218.68119872685</v>
+        <v>46218.71363287037</v>
       </c>
       <c r="K269" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>David Bragança</t>
         </is>
       </c>
       <c r="N269" s="1" t="n"/>
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
       <c r="Q269" s="1" t="inlineStr"/>
-      <c r="R269" s="1" t="n"/>
+      <c r="R269" s="1" t="inlineStr"/>
       <c r="S269" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21755,7 +21773,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>81085</v>
+        <v>81088</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
@@ -21764,7 +21782,7 @@
       </c>
       <c r="C270" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Criação de Relatórios</t>
         </is>
       </c>
       <c r="D270" s="1" t="inlineStr">
@@ -21774,40 +21792,44 @@
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, baixar a tarefa Envio de ATA de Implantação - DP - SP da empresa 6983, já é cliente da MG não vai ter ata de reunião.</t>
+          <t>Boa tarde!Criar os "problemas", no setor GC - ADMINISTRATIVO - Procurações DPValidar se elas estão orientadas para o uso.</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G270" s="1" t="n"/>
-      <c r="H270" s="1" t="n"/>
+      <c r="H270" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I270" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46218.69246809028</v>
+        <v>46218.72544799768</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Edivaldo Veiga</t>
+          <t>Mauricio Lermen</t>
         </is>
       </c>
       <c r="N270" s="1" t="n"/>
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="n"/>
+      <c r="R270" s="1" t="inlineStr"/>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21818,59 +21840,63 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>81086</v>
+        <v>76498</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Forçar baixa de tarefas via banco de dados</t>
+          <t>Endereço</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, realizar a baixa da tarefa "GFD - FGTS MENSAL" da empresa 1325. Os colaboradores "ativos" na empresa estão afastados por invalidez ou com reclamatória trabalhista em andamento, sendo assim, não há guia de FGTS para emitir.</t>
+          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G271" s="1" t="n"/>
-      <c r="H271" s="1" t="n"/>
+      <c r="H271" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I271" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46218.69883325232</v>
+        <v>46030.50436203703</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46219</v>
+        <v>46031</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Grasiele Santos</t>
+          <t>Alaine Neres</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="Q271" s="1" t="inlineStr"/>
-      <c r="R271" s="1" t="n"/>
+      <c r="R271" s="1" t="inlineStr"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21881,26 +21907,26 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>76498</v>
+        <v>76514</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>RJ - EF</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
+          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -21918,7 +21944,7 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46030.50436203703</v>
+        <v>46030.72255292824</v>
       </c>
       <c r="K272" s="2" t="n">
         <v>46031</v>
@@ -21930,7 +21956,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Alaine Neres</t>
+          <t>Glaucia Santos</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -21948,7 +21974,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>76514</v>
+        <v>76892</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -21962,12 +21988,12 @@
       </c>
       <c r="D273" s="1" t="inlineStr">
         <is>
-          <t>RJ - EF</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
+          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -21985,10 +22011,10 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46030.72255292824</v>
+        <v>46051.62030378472</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46031</v>
+        <v>46052</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
@@ -21997,7 +22023,7 @@
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Glaucia Santos</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
@@ -22015,16 +22041,16 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>76892</v>
+        <v>77913</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -22034,7 +22060,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22052,10 +22078,10 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46051.62030378472</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46052</v>
+        <v>46097</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
@@ -22064,7 +22090,7 @@
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Larissa Félix</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
@@ -22082,63 +22108,59 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>77913</v>
+        <v>79609</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G275" s="1" t="n"/>
-      <c r="H275" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H275" s="1" t="n"/>
       <c r="I275" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46097</v>
+        <v>46205</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M275" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="N275" s="1" t="n"/>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="Q275" s="1" t="inlineStr"/>
-      <c r="R275" s="1" t="inlineStr"/>
+      <c r="R275" s="1" t="n"/>
       <c r="S275" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22149,7 +22171,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>79609</v>
+        <v>80515</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22158,7 +22180,7 @@
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
@@ -22168,40 +22190,44 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G276" s="1" t="n"/>
-      <c r="H276" s="1" t="n"/>
+      <c r="H276" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I276" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46205</v>
+        <v>46226</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N276" s="1" t="n"/>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="n"/>
+      <c r="R276" s="1" t="inlineStr"/>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22212,7 +22238,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80515</v>
+        <v>80697</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22221,7 +22247,7 @@
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22231,32 +22257,28 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G277" s="1" t="n"/>
-      <c r="H277" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H277" s="1" t="n"/>
       <c r="I277" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46226</v>
+        <v>46237</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
@@ -22268,7 +22290,7 @@
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
-      <c r="R277" s="1" t="inlineStr"/>
+      <c r="R277" s="1" t="n"/>
       <c r="S277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22279,7 +22301,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80697</v>
+        <v>80714</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22288,7 +22310,7 @@
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22298,7 +22320,7 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22312,10 +22334,10 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
@@ -22342,16 +22364,16 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80714</v>
+        <v>80919</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
@@ -22361,7 +22383,7 @@
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22375,10 +22397,10 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
@@ -22405,16 +22427,16 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80919</v>
+        <v>80935</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22424,7 +22446,7 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22438,10 +22460,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22468,7 +22490,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>80935</v>
+        <v>80936</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
@@ -22477,7 +22499,7 @@
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22487,7 +22509,7 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22501,7 +22523,7 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K281" s="2" t="n">
         <v>46241</v>
@@ -22531,7 +22553,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>80936</v>
+        <v>80951</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
@@ -22540,7 +22562,7 @@
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
@@ -22550,7 +22572,7 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22564,7 +22586,7 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K282" s="2" t="n">
         <v>46241</v>
@@ -22594,59 +22616,63 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>80951</v>
+        <v>80989</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G283" s="1" t="n"/>
-      <c r="H283" s="1" t="n"/>
+      <c r="H283" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I283" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46241</v>
+        <v>46217</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>João Oliveira</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="n"/>
+      <c r="R283" s="1" t="inlineStr"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22657,11 +22683,11 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>80989</v>
+        <v>80995</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
@@ -22671,49 +22697,45 @@
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G284" s="1" t="n"/>
-      <c r="H284" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+      <c r="H284" s="1" t="n"/>
       <c r="I284" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46217.33131420139</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Jonatan Hayashibara</t>
         </is>
       </c>
       <c r="N284" s="1" t="n"/>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
-      <c r="R284" s="1" t="inlineStr"/>
+      <c r="R284" s="1" t="n"/>
       <c r="S284" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22724,59 +22746,67 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>80995</v>
+        <v>79793</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G285" s="1" t="n"/>
-      <c r="H285" s="1" t="n"/>
+        <v>5655</v>
+      </c>
+      <c r="G285" s="1" t="inlineStr">
+        <is>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
+      <c r="H285" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I285" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46217.33131420139</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46219</v>
+        <v>46185</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Jonatan Hayashibara</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="n"/>
+      <c r="R285" s="1" t="inlineStr"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22787,67 +22817,59 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>79793</v>
+        <v>81068</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G286" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
-      <c r="H286" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G286" s="1" t="n"/>
+      <c r="H286" s="1" t="n"/>
       <c r="I286" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46218.47815153936</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46185</v>
+        <v>46220</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N286" s="1" t="n"/>
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
       <c r="Q286" s="1" t="inlineStr"/>
-      <c r="R286" s="1" t="inlineStr"/>
+      <c r="R286" s="1" t="n"/>
       <c r="S286" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22858,7 +22880,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81068</v>
+        <v>81070</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
@@ -22877,7 +22899,7 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
@@ -22891,7 +22913,7 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46218.47815153936</v>
+        <v>46218.51467572917</v>
       </c>
       <c r="K287" s="2" t="n">
         <v>46220</v>
@@ -22921,7 +22943,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>81070</v>
+        <v>81071</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -22940,7 +22962,7 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
@@ -22954,7 +22976,7 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46218.51467572917</v>
+        <v>46218.51533788195</v>
       </c>
       <c r="K288" s="2" t="n">
         <v>46220</v>
@@ -22984,7 +23006,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81071</v>
+        <v>81072</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -23003,7 +23025,7 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
@@ -23017,7 +23039,7 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46218.51533788195</v>
+        <v>46218.51577677084</v>
       </c>
       <c r="K289" s="2" t="n">
         <v>46220</v>
@@ -23047,16 +23069,16 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>81072</v>
+        <v>81004</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
@@ -23066,13 +23088,17 @@
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G290" s="1" t="n"/>
+        <v>6869</v>
+      </c>
+      <c r="G290" s="1" t="inlineStr">
+        <is>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+        </is>
+      </c>
       <c r="H290" s="1" t="n"/>
       <c r="I290" s="1" t="inlineStr">
         <is>
@@ -23080,10 +23106,10 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46218.51577677084</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46220</v>
+        <v>46218</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
@@ -23092,7 +23118,7 @@
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
@@ -23110,7 +23136,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81004</v>
+        <v>81005</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
@@ -23133,11 +23159,11 @@
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6869</v>
+        <v>6870</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+          <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H291" s="1" t="n"/>
@@ -23147,7 +23173,7 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K291" s="2" t="n">
         <v>46218</v>
@@ -23177,16 +23203,16 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>81005</v>
+        <v>80961</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
@@ -23196,15 +23222,15 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6870</v>
+        <v>6950</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>MERCH LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H292" s="1" t="n"/>
@@ -23214,7 +23240,7 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46216.41692731481</v>
       </c>
       <c r="K292" s="2" t="n">
         <v>46218</v>
@@ -23244,63 +23270,67 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>80961</v>
+        <v>79856</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C293" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D293" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6950</v>
+        <v>4225</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>MERCH LTDA (FILIAL 1)</t>
-        </is>
-      </c>
-      <c r="H293" s="1" t="n"/>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+        </is>
+      </c>
+      <c r="H293" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I293" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46216.41692731481</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46218</v>
+        <v>46184</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N293" s="1" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="n"/>
+      <c r="R293" s="1" t="inlineStr"/>
       <c r="S293" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23311,7 +23341,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79856</v>
+        <v>79855</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
@@ -23330,15 +23360,15 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>4225</v>
+        <v>4765</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
@@ -23352,10 +23382,10 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L294" s="1" t="inlineStr">
         <is>
@@ -23382,16 +23412,16 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79855</v>
+        <v>79833</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
@@ -23401,15 +23431,15 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>4765</v>
+        <v>6125</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
@@ -23423,10 +23453,10 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K295" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L295" s="1" t="inlineStr">
         <is>
@@ -23453,7 +23483,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>79833</v>
+        <v>79834</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23476,11 +23506,11 @@
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>6125</v>
+        <v>6162</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
@@ -23494,7 +23524,7 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K296" s="2" t="n">
         <v>46184</v>
@@ -23524,16 +23554,16 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79834</v>
+        <v>79865</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
@@ -23543,15 +23573,15 @@
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>6162</v>
+        <v>6278</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H297" s="1" t="inlineStr">
@@ -23565,10 +23595,10 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
@@ -23577,7 +23607,7 @@
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
@@ -23595,7 +23625,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>79865</v>
+        <v>79854</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23614,15 +23644,15 @@
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>6278</v>
+        <v>6302</v>
       </c>
       <c r="G298" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H298" s="1" t="inlineStr">
@@ -23636,10 +23666,10 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
@@ -23648,7 +23678,7 @@
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
@@ -23666,7 +23696,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>79854</v>
+        <v>79863</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
@@ -23685,15 +23715,15 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>6302</v>
+        <v>6404</v>
       </c>
       <c r="G299" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H299" s="1" t="inlineStr">
@@ -23707,10 +23737,10 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
@@ -23719,7 +23749,7 @@
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N299" s="1" t="n"/>
@@ -23737,16 +23767,16 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>79863</v>
+        <v>79835</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C300" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D300" s="1" t="inlineStr">
@@ -23756,15 +23786,15 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>6404</v>
+        <v>6485</v>
       </c>
       <c r="G300" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H300" s="1" t="inlineStr">
@@ -23778,10 +23808,10 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
@@ -23790,7 +23820,7 @@
       </c>
       <c r="M300" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N300" s="1" t="n"/>
@@ -23808,16 +23838,16 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>79835</v>
+        <v>79866</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C301" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D301" s="1" t="inlineStr">
@@ -23827,15 +23857,15 @@
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>6485</v>
+        <v>6539</v>
       </c>
       <c r="G301" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H301" s="1" t="inlineStr">
@@ -23849,10 +23879,10 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
@@ -23861,7 +23891,7 @@
       </c>
       <c r="M301" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N301" s="1" t="n"/>
@@ -23879,7 +23909,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>79866</v>
+        <v>79859</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
@@ -23898,15 +23928,15 @@
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>6539</v>
+        <v>6570</v>
       </c>
       <c r="G302" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H302" s="1" t="inlineStr">
@@ -23920,7 +23950,7 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K302" s="2" t="n">
         <v>46185</v>
@@ -23950,7 +23980,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>79859</v>
+        <v>79860</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
@@ -23969,15 +23999,15 @@
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
-        <v>6570</v>
+        <v>6581</v>
       </c>
       <c r="G303" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H303" s="1" t="inlineStr">
@@ -23991,7 +24021,7 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46185</v>
@@ -24021,7 +24051,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>79860</v>
+        <v>79861</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
@@ -24040,15 +24070,15 @@
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
-        <v>6581</v>
+        <v>6583</v>
       </c>
       <c r="G304" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H304" s="1" t="inlineStr">
@@ -24062,7 +24092,7 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K304" s="2" t="n">
         <v>46185</v>
@@ -24092,16 +24122,16 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>79861</v>
+        <v>79867</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C305" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D305" s="1" t="inlineStr">
@@ -24111,15 +24141,15 @@
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
-        <v>6583</v>
+        <v>6704</v>
       </c>
       <c r="G305" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H305" s="1" t="inlineStr">
@@ -24133,7 +24163,7 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K305" s="2" t="n">
         <v>46185</v>
@@ -24163,7 +24193,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>79867</v>
+        <v>81019</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
@@ -24172,27 +24202,23 @@
       </c>
       <c r="C306" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D306" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>6704</v>
-      </c>
-      <c r="G306" s="1" t="inlineStr">
-        <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G306" s="1" t="n"/>
       <c r="H306" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24204,10 +24230,10 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
@@ -24216,7 +24242,7 @@
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N306" s="1" t="n"/>
@@ -24234,7 +24260,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>81019</v>
+        <v>81052</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
@@ -24253,7 +24279,7 @@
       </c>
       <c r="E307" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
@@ -24271,10 +24297,10 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
@@ -24283,7 +24309,7 @@
       </c>
       <c r="M307" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N307" s="1" t="n"/>
@@ -24301,7 +24327,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>81052</v>
+        <v>81055</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
@@ -24320,7 +24346,7 @@
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
@@ -24338,7 +24364,7 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K308" s="2" t="n">
         <v>46219</v>
@@ -24365,73 +24391,6 @@
       </c>
       <c r="T308" s="1" t="n"/>
       <c r="U308" s="1" t="inlineStr"/>
-    </row>
-    <row r="309">
-      <c r="A309" s="1" t="n">
-        <v>81055</v>
-      </c>
-      <c r="B309" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C309" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D309" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E309" s="1" t="inlineStr">
-        <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
-        </is>
-      </c>
-      <c r="F309" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G309" s="1" t="n"/>
-      <c r="H309" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I309" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J309" s="2" t="n">
-        <v>46218.40379614583</v>
-      </c>
-      <c r="K309" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="L309" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M309" s="1" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N309" s="1" t="n"/>
-      <c r="O309" s="1" t="n"/>
-      <c r="P309" s="1" t="n"/>
-      <c r="Q309" s="1" t="inlineStr"/>
-      <c r="R309" s="1" t="inlineStr"/>
-      <c r="S309" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T309" s="1" t="n"/>
-      <c r="U309" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 16-07-26 0902
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U308" headerRowCount="1">
-  <autoFilter ref="A1:U308"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U311" headerRowCount="1">
+  <autoFilter ref="A1:U311"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U308"/>
+  <dimension ref="A1:U311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1178,7 +1178,11 @@
         <v>0</v>
       </c>
       <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Ana Flavia Silva</t>
+        </is>
+      </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL HOLDING</t>
@@ -1192,7 +1196,7 @@
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M9" s="1" t="inlineStr">
@@ -1201,17 +1205,23 @@
         </is>
       </c>
       <c r="N9" s="1" t="n"/>
-      <c r="O9" s="1" t="n"/>
+      <c r="O9" s="2" t="n">
+        <v>46219</v>
+      </c>
       <c r="P9" s="1" t="n"/>
       <c r="Q9" s="1" t="inlineStr"/>
-      <c r="R9" s="1" t="n"/>
+      <c r="R9" s="1" t="inlineStr"/>
       <c r="S9" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T9" s="1" t="n"/>
-      <c r="U9" s="1" t="inlineStr"/>
+      <c r="U9" s="1" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -21495,7 +21505,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>81034</v>
+        <v>81001</v>
       </c>
       <c r="B266" s="1" t="inlineStr">
         <is>
@@ -21509,12 +21519,12 @@
       </c>
       <c r="D266" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E266" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tardecolaborador suede informa colocar comentarios nas tarefas, incluindo previsões e o MGC "apaga" ou "some" parecendo que ela não colocou informação.Por gentileza verificar</t>
+          <t>POR GENTILEZA PODEM BAIXAR A TAREFA "Recebimento de NF ICMS Centr. e Lançamento - 6/2026" DA LOJA 6001 DO MÊS DE JUNHO.</t>
         </is>
       </c>
       <c r="F266" s="1" t="n">
@@ -21532,26 +21542,30 @@
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>46217.58055833333</v>
+        <v>46217.36753545139</v>
       </c>
       <c r="K266" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="L266" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M266" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Diego Pereira</t>
         </is>
       </c>
       <c r="N266" s="1" t="n"/>
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
       <c r="Q266" s="1" t="inlineStr"/>
-      <c r="R266" s="1" t="inlineStr"/>
+      <c r="R266" s="1" t="inlineStr">
+        <is>
+          <t>Tarefa baixada</t>
+        </is>
+      </c>
       <c r="S266" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21562,7 +21576,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>81063</v>
+        <v>81034</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
@@ -21571,17 +21585,17 @@
       </c>
       <c r="C267" s="1" t="inlineStr">
         <is>
-          <t>Abertura de protocolo</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D267" s="1" t="inlineStr">
         <is>
-          <t>MG EXPRESS - GC</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E267" s="1" t="inlineStr">
         <is>
-          <t>Precisamos da baixa da tarefa "Fed - DAS" competência 06/2026 das empresas com arquivos disponíveis no diretório abaixo:\\finlandia\PUBLICA\RomeroBorges\DAS - Documentos chamado</t>
+          <t>Prezados, boa tardecolaborador suede informa colocar comentarios nas tarefas, incluindo previsões e o MGC "apaga" ou "some" parecendo que ela não colocou informação.Por gentileza verificar</t>
         </is>
       </c>
       <c r="F267" s="1" t="n">
@@ -21599,10 +21613,10 @@
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46218.44771315972</v>
+        <v>46217.58055833333</v>
       </c>
       <c r="K267" s="2" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="L267" s="1" t="inlineStr">
         <is>
@@ -21611,7 +21625,7 @@
       </c>
       <c r="M267" s="1" t="inlineStr">
         <is>
-          <t>Romero Borges</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="N267" s="1" t="n"/>
@@ -21629,7 +21643,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>81083</v>
+        <v>81063</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
@@ -21638,17 +21652,17 @@
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Abertura de protocolo</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>MG EXPRESS - GC</t>
         </is>
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Precisamos da baixa da tarefa "Fed - DAS" competência 06/2026 das empresas com arquivos disponíveis no diretório abaixo:\\finlandia\PUBLICA\RomeroBorges\DAS - Documentos chamado</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
@@ -21666,39 +21680,29 @@
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46218.68119872685</v>
+        <v>46218.44771315972</v>
       </c>
       <c r="K268" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L268" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M268" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Romero Borges</t>
         </is>
       </c>
       <c r="N268" s="1" t="n"/>
       <c r="O268" s="1" t="n"/>
-      <c r="P268" s="2" t="n">
-        <v>46218.7466727662</v>
-      </c>
-      <c r="Q268" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
-      <c r="R268" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
-        </is>
-      </c>
+      <c r="P268" s="1" t="n"/>
+      <c r="Q268" s="1" t="inlineStr"/>
+      <c r="R268" s="1" t="inlineStr"/>
       <c r="S268" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T268" s="1" t="n"/>
@@ -21706,7 +21710,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>81087</v>
+        <v>81083</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
@@ -21715,17 +21719,17 @@
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Forçar baixa de tarefas via banco de dados</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,Por favor baixar a tarefa "retificação FOPAG FOPAG 062026 das empresa 1330 e 2607, está pedindo para anexar arquivo, mas, não tem modelo fixado como exemplo.Obrigado</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
@@ -21743,29 +21747,39 @@
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46218.71363287037</v>
+        <v>46218.68119872685</v>
       </c>
       <c r="K269" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N269" s="1" t="n"/>
       <c r="O269" s="1" t="n"/>
-      <c r="P269" s="1" t="n"/>
-      <c r="Q269" s="1" t="inlineStr"/>
-      <c r="R269" s="1" t="inlineStr"/>
+      <c r="P269" s="2" t="n">
+        <v>46218.7466727662</v>
+      </c>
+      <c r="Q269" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
+      <c r="R269" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+        </is>
+      </c>
       <c r="S269" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T269" s="1" t="n"/>
@@ -21840,26 +21854,26 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>76498</v>
+        <v>81090</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t>Chamados</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>B.P.O. - GUARANI CTB</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
+          <t>por gentileza poderia baixar a reeinf da empresas 4059 e a tarefas da caixa postal das empresas 4059, 4064, 4065 ,4066, 4067, 4068, 4602, 4815, 4917 em Anexo</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
@@ -21868,19 +21882,19 @@
       <c r="G271" s="1" t="n"/>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46030.50436203703</v>
+        <v>46218.76292554398</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46031</v>
+        <v>46220</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21889,7 +21903,7 @@
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Alaine Neres</t>
+          <t>Flavia Dariolli</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
@@ -21907,63 +21921,59 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>76514</v>
+        <v>81092</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>RJ - EF</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
+          <t>POR GENTILEZA BAIXAR A TAREFA "CONTA DE ENERGIA" DO MÊS 06/2026 DA EMPRESA 4922 - SUPERMERCADOS CAPPI DUARTE LTDA</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G272" s="1" t="n"/>
-      <c r="H272" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+      <c r="H272" s="1" t="n"/>
       <c r="I272" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46030.72255292824</v>
+        <v>46219.37092832176</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46031</v>
+        <v>46220</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Glaucia Santos</t>
+          <t>Diego Pereira</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
       <c r="Q272" s="1" t="inlineStr"/>
-      <c r="R272" s="1" t="inlineStr"/>
+      <c r="R272" s="1" t="n"/>
       <c r="S272" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21974,16 +21984,16 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>76892</v>
+        <v>76498</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Endereço</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -21993,7 +22003,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
+          <t>2279 - FRUTILAR: de São Paulo para Taboão da Serra, ela mudou de endereço, de São Paulo para Taboão da Serra.E tem notas de serviços prestados para a prefeitura de São Paulo, quando vou converter a nota no site, não deixar por conta do cadastro, consta que não precisar emitir a nota, por ser do mesmo município.</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -22011,10 +22021,10 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46051.62030378472</v>
+        <v>46030.50436203703</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46052</v>
+        <v>46031</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
@@ -22023,7 +22033,7 @@
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Alaine Neres</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
@@ -22041,26 +22051,26 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>77913</v>
+        <v>76514</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>RJ - EF</t>
         </is>
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>Boa tarde !A empresa 6603 esta cadastrada no SCI (BASE VAREJO) com um CNPJ divergente do cadastrado no MG controle.Segue em anexo os cartões CNPJ, para conferencia.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22078,10 +22088,10 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46030.72255292824</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46097</v>
+        <v>46031</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
@@ -22090,7 +22100,7 @@
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
+          <t>Glaucia Santos</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
@@ -22108,59 +22118,63 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>79609</v>
+        <v>76892</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Boa tarde,Identificamos que a loja 5225 – CUCINARE PRO (Filial 71) está com o CNPJ incorreto cadastrado no MG Controle, na aba Clientes.Solicitamos, por gentileza, a correção do CNPJ no sistema.Ficamos no aguardo da confirmação após o ajuste. OBS: ramal para contato: 1341 - Igor bastos</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G275" s="1" t="n"/>
-      <c r="H275" s="1" t="n"/>
+      <c r="H275" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I275" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46051.62030378472</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46205</v>
+        <v>46052</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M275" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N275" s="1" t="n"/>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="Q275" s="1" t="inlineStr"/>
-      <c r="R275" s="1" t="n"/>
+      <c r="R275" s="1" t="inlineStr"/>
       <c r="S275" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22171,26 +22185,26 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>80515</v>
+        <v>77913</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
@@ -22208,10 +22222,10 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46226</v>
+        <v>46097</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
@@ -22220,7 +22234,7 @@
       </c>
       <c r="M276" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Larissa Félix</t>
         </is>
       </c>
       <c r="N276" s="1" t="n"/>
@@ -22238,7 +22252,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80697</v>
+        <v>79609</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22247,7 +22261,7 @@
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22257,7 +22271,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22271,10 +22285,10 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46237</v>
+        <v>46205</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
@@ -22283,7 +22297,7 @@
       </c>
       <c r="M277" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="N277" s="1" t="n"/>
@@ -22301,7 +22315,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80714</v>
+        <v>80515</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22310,7 +22324,7 @@
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22320,28 +22334,32 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G278" s="1" t="n"/>
-      <c r="H278" s="1" t="n"/>
+      <c r="H278" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I278" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46241</v>
+        <v>46226</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M278" s="1" t="inlineStr">
@@ -22353,7 +22371,7 @@
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
-      <c r="R278" s="1" t="n"/>
+      <c r="R278" s="1" t="inlineStr"/>
       <c r="S278" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22364,16 +22382,16 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80919</v>
+        <v>80697</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
@@ -22383,7 +22401,7 @@
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22397,10 +22415,10 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
@@ -22427,7 +22445,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80935</v>
+        <v>80714</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
@@ -22436,7 +22454,7 @@
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22446,7 +22464,7 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22460,7 +22478,7 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K280" s="2" t="n">
         <v>46241</v>
@@ -22490,16 +22508,16 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>80936</v>
+        <v>80919</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22509,7 +22527,7 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22523,10 +22541,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22553,7 +22571,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>80951</v>
+        <v>80935</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
@@ -22572,7 +22590,7 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22586,7 +22604,7 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K282" s="2" t="n">
         <v>46241</v>
@@ -22616,63 +22634,59 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>80989</v>
+        <v>80936</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G283" s="1" t="n"/>
-      <c r="H283" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+      <c r="H283" s="1" t="n"/>
       <c r="I283" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="inlineStr"/>
+      <c r="R283" s="1" t="n"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22683,26 +22697,26 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>80995</v>
+        <v>80951</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22716,10 +22730,10 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46217.33131420139</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46219</v>
+        <v>46241</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
@@ -22728,7 +22742,7 @@
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>Jonatan Hayashibara</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N284" s="1" t="n"/>
@@ -22746,67 +22760,59 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>79793</v>
+        <v>81068</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G285" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
-      <c r="H285" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G285" s="1" t="n"/>
+      <c r="H285" s="1" t="n"/>
       <c r="I285" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46218.47815153936</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46185</v>
+        <v>46220</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="inlineStr"/>
+      <c r="R285" s="1" t="n"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22817,7 +22823,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>81068</v>
+        <v>81070</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
@@ -22836,7 +22842,7 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ3252 Comercio de Alimentos Alves e Farias FILIAL 013257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
@@ -22850,7 +22856,7 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46218.47815153936</v>
+        <v>46218.51467572917</v>
       </c>
       <c r="K286" s="2" t="n">
         <v>46220</v>
@@ -22880,7 +22886,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81070</v>
+        <v>81071</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
@@ -22899,7 +22905,7 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
@@ -22913,7 +22919,7 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46218.51467572917</v>
+        <v>46218.51533788195</v>
       </c>
       <c r="K287" s="2" t="n">
         <v>46220</v>
@@ -22943,7 +22949,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>81071</v>
+        <v>81072</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -22962,7 +22968,7 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
@@ -22976,7 +22982,7 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46218.51533788195</v>
+        <v>46218.51577677084</v>
       </c>
       <c r="K288" s="2" t="n">
         <v>46220</v>
@@ -23006,11 +23012,11 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81072</v>
+        <v>80989</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C289" s="1" t="inlineStr">
@@ -23025,40 +23031,44 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G289" s="1" t="n"/>
-      <c r="H289" s="1" t="n"/>
+      <c r="H289" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I289" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46218.51577677084</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46220</v>
+        <v>46217</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>João Oliveira</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
       <c r="Q289" s="1" t="inlineStr"/>
-      <c r="R289" s="1" t="n"/>
+      <c r="R289" s="1" t="inlineStr"/>
       <c r="S289" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23069,36 +23079,32 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>81004</v>
+        <v>80995</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Bom dia!Solicito acesso a prefeitura de Holambra na qual efetuou uma atualização.Já foi testado o Login e senha com o que está no Intranet quanto também apenas com a inscrição municipalNovo Emissor: https://holambra.citynex.com.br/ords/holambra/f?p=778:70:Antigo: http://179.175.14.22:8080/issweb/paginas/admin/declaracoes/tomador/declaracoesempresas em questão em anexo:com prioridade a B3R</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6869</v>
-      </c>
-      <c r="G290" s="1" t="inlineStr">
-        <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G290" s="1" t="n"/>
       <c r="H290" s="1" t="n"/>
       <c r="I290" s="1" t="inlineStr">
         <is>
@@ -23106,10 +23112,10 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46217.33131420139</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
@@ -23118,7 +23124,7 @@
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Jonatan Hayashibara</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
@@ -23136,63 +23142,67 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81005</v>
+        <v>79793</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6870</v>
+        <v>5655</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
-        </is>
-      </c>
-      <c r="H291" s="1" t="n"/>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
+      <c r="H291" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I291" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46218</v>
+        <v>46185</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
       <c r="Q291" s="1" t="inlineStr"/>
-      <c r="R291" s="1" t="n"/>
+      <c r="R291" s="1" t="inlineStr"/>
       <c r="S291" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23203,16 +23213,16 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>80961</v>
+        <v>81004</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
@@ -23222,15 +23232,15 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6950</v>
+        <v>6869</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>MERCH LTDA (FILIAL 1)</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H292" s="1" t="n"/>
@@ -23240,7 +23250,7 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46216.41692731481</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K292" s="2" t="n">
         <v>46218</v>
@@ -23270,67 +23280,63 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79856</v>
+        <v>81005</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C293" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D293" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>4225</v>
+        <v>6870</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
-        </is>
-      </c>
-      <c r="H293" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>AC HOME PET RAÇÕES LTDA</t>
+        </is>
+      </c>
+      <c r="H293" s="1" t="n"/>
       <c r="I293" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46184</v>
+        <v>46218</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N293" s="1" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="inlineStr"/>
+      <c r="R293" s="1" t="n"/>
       <c r="S293" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23341,67 +23347,63 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79855</v>
+        <v>81091</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>4765</v>
+        <v>6907</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
-        </is>
-      </c>
-      <c r="H294" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+        </is>
+      </c>
+      <c r="H294" s="1" t="n"/>
       <c r="I294" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>46185</v>
+        <v>46223</v>
       </c>
       <c r="L294" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M294" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N294" s="1" t="n"/>
       <c r="O294" s="1" t="n"/>
       <c r="P294" s="1" t="n"/>
       <c r="Q294" s="1" t="inlineStr"/>
-      <c r="R294" s="1" t="inlineStr"/>
+      <c r="R294" s="1" t="n"/>
       <c r="S294" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23412,67 +23414,63 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79833</v>
+        <v>80961</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Bom dia! Por gentileza, solicitado o login e senha da prefeitura da empresa 6950.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6125</v>
+        <v>6950</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H295" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>MERCH LTDA (FILIAL 1)</t>
+        </is>
+      </c>
+      <c r="H295" s="1" t="n"/>
       <c r="I295" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46216.41692731481</v>
       </c>
       <c r="K295" s="2" t="n">
-        <v>46184</v>
+        <v>46218</v>
       </c>
       <c r="L295" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M295" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N295" s="1" t="n"/>
       <c r="O295" s="1" t="n"/>
       <c r="P295" s="1" t="n"/>
       <c r="Q295" s="1" t="inlineStr"/>
-      <c r="R295" s="1" t="inlineStr"/>
+      <c r="R295" s="1" t="n"/>
       <c r="S295" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23483,7 +23481,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>79834</v>
+        <v>79833</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23506,11 +23504,11 @@
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>6162</v>
+        <v>6125</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
@@ -23524,7 +23522,7 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K296" s="2" t="n">
         <v>46184</v>
@@ -23554,16 +23552,16 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79865</v>
+        <v>79834</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
@@ -23573,15 +23571,15 @@
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>6278</v>
+        <v>6162</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H297" s="1" t="inlineStr">
@@ -23595,10 +23593,10 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
@@ -23607,7 +23605,7 @@
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
@@ -23625,7 +23623,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>79854</v>
+        <v>79865</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23644,15 +23642,15 @@
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>6302</v>
+        <v>6278</v>
       </c>
       <c r="G298" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H298" s="1" t="inlineStr">
@@ -23666,10 +23664,10 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
@@ -23678,7 +23676,7 @@
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
@@ -23696,7 +23694,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>79863</v>
+        <v>79854</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
@@ -23715,15 +23713,15 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>6404</v>
+        <v>6302</v>
       </c>
       <c r="G299" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H299" s="1" t="inlineStr">
@@ -23737,10 +23735,10 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
@@ -23749,7 +23747,7 @@
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N299" s="1" t="n"/>
@@ -23767,16 +23765,16 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>79835</v>
+        <v>79863</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C300" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D300" s="1" t="inlineStr">
@@ -23786,15 +23784,15 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>6485</v>
+        <v>6404</v>
       </c>
       <c r="G300" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H300" s="1" t="inlineStr">
@@ -23808,10 +23806,10 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
@@ -23820,7 +23818,7 @@
       </c>
       <c r="M300" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N300" s="1" t="n"/>
@@ -23838,16 +23836,16 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>79866</v>
+        <v>79835</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C301" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D301" s="1" t="inlineStr">
@@ -23857,15 +23855,15 @@
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>6539</v>
+        <v>6485</v>
       </c>
       <c r="G301" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H301" s="1" t="inlineStr">
@@ -23879,10 +23877,10 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
@@ -23891,7 +23889,7 @@
       </c>
       <c r="M301" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N301" s="1" t="n"/>
@@ -23909,7 +23907,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>79859</v>
+        <v>79866</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
@@ -23928,15 +23926,15 @@
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>6570</v>
+        <v>6539</v>
       </c>
       <c r="G302" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H302" s="1" t="inlineStr">
@@ -23950,7 +23948,7 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K302" s="2" t="n">
         <v>46185</v>
@@ -23980,7 +23978,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>79860</v>
+        <v>79859</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
@@ -23999,15 +23997,15 @@
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
-        <v>6581</v>
+        <v>6570</v>
       </c>
       <c r="G303" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H303" s="1" t="inlineStr">
@@ -24021,7 +24019,7 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46185</v>
@@ -24051,7 +24049,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>79861</v>
+        <v>79860</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
@@ -24070,15 +24068,15 @@
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
-        <v>6583</v>
+        <v>6581</v>
       </c>
       <c r="G304" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H304" s="1" t="inlineStr">
@@ -24092,7 +24090,7 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K304" s="2" t="n">
         <v>46185</v>
@@ -24122,16 +24120,16 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>79867</v>
+        <v>79861</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C305" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D305" s="1" t="inlineStr">
@@ -24141,15 +24139,15 @@
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
-        <v>6704</v>
+        <v>6583</v>
       </c>
       <c r="G305" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H305" s="1" t="inlineStr">
@@ -24163,7 +24161,7 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K305" s="2" t="n">
         <v>46185</v>
@@ -24193,7 +24191,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>81019</v>
+        <v>79867</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
@@ -24202,23 +24200,27 @@
       </c>
       <c r="C306" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D306" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G306" s="1" t="n"/>
+        <v>6704</v>
+      </c>
+      <c r="G306" s="1" t="inlineStr">
+        <is>
+          <t>TECNO COM INFORMATICA LTDA</t>
+        </is>
+      </c>
       <c r="H306" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24230,10 +24232,10 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>46218</v>
+        <v>46185</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
@@ -24242,7 +24244,7 @@
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N306" s="1" t="n"/>
@@ -24260,32 +24262,36 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>81052</v>
+        <v>79856</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C307" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D307" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E307" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G307" s="1" t="n"/>
+        <v>4225</v>
+      </c>
+      <c r="G307" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+        </is>
+      </c>
       <c r="H307" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24297,10 +24303,10 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>46219</v>
+        <v>46184</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
@@ -24309,7 +24315,7 @@
       </c>
       <c r="M307" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N307" s="1" t="n"/>
@@ -24327,32 +24333,36 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>81055</v>
+        <v>79855</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C308" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D308" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G308" s="1" t="n"/>
+        <v>4765</v>
+      </c>
+      <c r="G308" s="1" t="inlineStr">
+        <is>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+        </is>
+      </c>
       <c r="H308" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24364,10 +24374,10 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K308" s="2" t="n">
-        <v>46219</v>
+        <v>46185</v>
       </c>
       <c r="L308" s="1" t="inlineStr">
         <is>
@@ -24376,7 +24386,7 @@
       </c>
       <c r="M308" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N308" s="1" t="n"/>
@@ -24391,6 +24401,207 @@
       </c>
       <c r="T308" s="1" t="n"/>
       <c r="U308" s="1" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="1" t="n">
+        <v>81019</v>
+      </c>
+      <c r="B309" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C309" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D309" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E309" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+        </is>
+      </c>
+      <c r="F309" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" s="1" t="n"/>
+      <c r="H309" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I309" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="n">
+        <v>46217.43210269676</v>
+      </c>
+      <c r="K309" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="L309" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M309" s="1" t="inlineStr">
+        <is>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N309" s="1" t="n"/>
+      <c r="O309" s="1" t="n"/>
+      <c r="P309" s="1" t="n"/>
+      <c r="Q309" s="1" t="inlineStr"/>
+      <c r="R309" s="1" t="inlineStr"/>
+      <c r="S309" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T309" s="1" t="n"/>
+      <c r="U309" s="1" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="1" t="n">
+        <v>81052</v>
+      </c>
+      <c r="B310" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C310" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D310" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E310" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+        </is>
+      </c>
+      <c r="F310" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" s="1" t="n"/>
+      <c r="H310" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I310" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="n">
+        <v>46218.38736744213</v>
+      </c>
+      <c r="K310" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L310" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M310" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N310" s="1" t="n"/>
+      <c r="O310" s="1" t="n"/>
+      <c r="P310" s="1" t="n"/>
+      <c r="Q310" s="1" t="inlineStr"/>
+      <c r="R310" s="1" t="inlineStr"/>
+      <c r="S310" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T310" s="1" t="n"/>
+      <c r="U310" s="1" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="1" t="n">
+        <v>81055</v>
+      </c>
+      <c r="B311" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C311" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D311" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E311" s="1" t="inlineStr">
+        <is>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+        </is>
+      </c>
+      <c r="F311" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" s="1" t="n"/>
+      <c r="H311" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I311" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="n">
+        <v>46218.40379614583</v>
+      </c>
+      <c r="K311" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L311" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M311" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N311" s="1" t="n"/>
+      <c r="O311" s="1" t="n"/>
+      <c r="P311" s="1" t="n"/>
+      <c r="Q311" s="1" t="inlineStr"/>
+      <c r="R311" s="1" t="inlineStr"/>
+      <c r="S311" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T311" s="1" t="n"/>
+      <c r="U311" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 16-07-26 1503
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -9173,7 +9173,7 @@
       </c>
       <c r="L106" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M106" s="1" t="inlineStr">
@@ -9185,12 +9185,22 @@
       <c r="O106" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="P106" s="1" t="n"/>
-      <c r="Q106" s="1" t="inlineStr"/>
-      <c r="R106" s="1" t="inlineStr"/>
+      <c r="P106" s="2" t="n">
+        <v>46219.58110721065</v>
+      </c>
+      <c r="Q106" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R106" s="1" t="inlineStr">
+        <is>
+          <t>Segue demonstrativos solicitados</t>
+        </is>
+      </c>
       <c r="S106" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T106" s="1" t="n"/>
@@ -9250,7 +9260,7 @@
       </c>
       <c r="L107" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M107" s="1" t="inlineStr">
@@ -9262,12 +9272,22 @@
       <c r="O107" s="2" t="n">
         <v>46217</v>
       </c>
-      <c r="P107" s="1" t="n"/>
-      <c r="Q107" s="1" t="inlineStr"/>
-      <c r="R107" s="1" t="inlineStr"/>
+      <c r="P107" s="2" t="n">
+        <v>46219.56934945602</v>
+      </c>
+      <c r="Q107" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R107" s="1" t="inlineStr">
+        <is>
+          <t>Vander, como já foi informado algumas vezes, houve uma mudança na baixa da tarefa, e já tinha sido acordado que o TI liberaria um acesso no SCIWEB para a conferencia de vocês.</t>
+        </is>
+      </c>
       <c r="S107" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T107" s="1" t="n"/>
@@ -10998,7 +11018,7 @@
       </c>
       <c r="L128" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M128" s="1" t="inlineStr">
@@ -11010,12 +11030,22 @@
       <c r="O128" s="2" t="n">
         <v>46219</v>
       </c>
-      <c r="P128" s="1" t="n"/>
-      <c r="Q128" s="1" t="inlineStr"/>
-      <c r="R128" s="1" t="inlineStr"/>
+      <c r="P128" s="2" t="n">
+        <v>46219.57306721065</v>
+      </c>
+      <c r="Q128" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R128" s="1" t="inlineStr">
+        <is>
+          <t>Conforme conversado no e-mail os valores do balancete estavam desatualizados, se for necessário fazer outros ajuste por favor orientar via chamado com autorização previa do GM e Diretoria.</t>
+        </is>
+      </c>
       <c r="S128" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T128" s="1" t="n"/>
@@ -11729,7 +11759,7 @@
       </c>
       <c r="L137" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M137" s="1" t="inlineStr">
@@ -11741,12 +11771,22 @@
       <c r="O137" s="2" t="n">
         <v>46219</v>
       </c>
-      <c r="P137" s="1" t="n"/>
-      <c r="Q137" s="1" t="inlineStr"/>
-      <c r="R137" s="1" t="inlineStr"/>
+      <c r="P137" s="2" t="n">
+        <v>46219.5832929051</v>
+      </c>
+      <c r="Q137" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R137" s="1" t="inlineStr">
+        <is>
+          <t>Em anexo</t>
+        </is>
+      </c>
       <c r="S137" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T137" s="1" t="n"/>
@@ -13004,7 +13044,7 @@
       </c>
       <c r="L153" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M153" s="1" t="inlineStr">
@@ -13016,12 +13056,22 @@
       <c r="O153" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="P153" s="1" t="n"/>
-      <c r="Q153" s="1" t="inlineStr"/>
-      <c r="R153" s="1" t="inlineStr"/>
+      <c r="P153" s="2" t="n">
+        <v>46219.59946519676</v>
+      </c>
+      <c r="Q153" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R153" s="1" t="inlineStr">
+        <is>
+          <t>Anexo</t>
+        </is>
+      </c>
       <c r="S153" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T153" s="1" t="n"/>
@@ -13822,7 +13872,7 @@
       </c>
       <c r="L163" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M163" s="1" t="inlineStr">
@@ -13834,12 +13884,22 @@
       <c r="O163" s="2" t="n">
         <v>46217</v>
       </c>
-      <c r="P163" s="1" t="n"/>
-      <c r="Q163" s="1" t="inlineStr"/>
-      <c r="R163" s="1" t="inlineStr"/>
+      <c r="P163" s="2" t="n">
+        <v>46219.57626284722</v>
+      </c>
+      <c r="Q163" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R163" s="1" t="inlineStr">
+        <is>
+          <t>Já foi ajustado conforme solicitado anteriormente na Analise Balanço</t>
+        </is>
+      </c>
       <c r="S163" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T163" s="1" t="n"/>
@@ -16751,7 +16811,11 @@
         <v>0</v>
       </c>
       <c r="G201" s="1" t="n"/>
-      <c r="H201" s="1" t="n"/>
+      <c r="H201" s="1" t="inlineStr">
+        <is>
+          <t>Ana Santana</t>
+        </is>
+      </c>
       <c r="I201" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
@@ -16765,7 +16829,7 @@
       </c>
       <c r="L201" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M201" s="1" t="inlineStr">
@@ -16777,7 +16841,7 @@
       <c r="O201" s="1" t="n"/>
       <c r="P201" s="1" t="n"/>
       <c r="Q201" s="1" t="inlineStr"/>
-      <c r="R201" s="1" t="n"/>
+      <c r="R201" s="1" t="inlineStr"/>
       <c r="S201" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -20167,7 +20231,11 @@
           <t xml:space="preserve">MONTE CARLO LAB SERVICOS ADMINISTRATIVOS E COMERCIO LTDA </t>
         </is>
       </c>
-      <c r="H249" s="1" t="n"/>
+      <c r="H249" s="1" t="inlineStr">
+        <is>
+          <t>Rodrigo Rego</t>
+        </is>
+      </c>
       <c r="I249" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
@@ -20181,7 +20249,7 @@
       </c>
       <c r="L249" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M249" s="1" t="inlineStr">
@@ -20193,7 +20261,7 @@
       <c r="O249" s="1" t="n"/>
       <c r="P249" s="1" t="n"/>
       <c r="Q249" s="1" t="inlineStr"/>
-      <c r="R249" s="1" t="n"/>
+      <c r="R249" s="1" t="inlineStr"/>
       <c r="S249" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -20660,7 +20728,11 @@
           <t>DFG COMERCIO IMPORTACAO, EXPORTACAO E REPRESENTACAO LTDA</t>
         </is>
       </c>
-      <c r="H256" s="1" t="n"/>
+      <c r="H256" s="1" t="inlineStr">
+        <is>
+          <t>Vander Silva</t>
+        </is>
+      </c>
       <c r="I256" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
@@ -20674,7 +20746,7 @@
       </c>
       <c r="L256" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M256" s="1" t="inlineStr">
@@ -20686,7 +20758,7 @@
       <c r="O256" s="1" t="n"/>
       <c r="P256" s="1" t="n"/>
       <c r="Q256" s="1" t="inlineStr"/>
-      <c r="R256" s="1" t="n"/>
+      <c r="R256" s="1" t="inlineStr"/>
       <c r="S256" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21193,7 +21265,7 @@
       </c>
       <c r="L263" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M263" s="1" t="inlineStr">
@@ -21201,11 +21273,17 @@
           <t>Alaine Neres</t>
         </is>
       </c>
-      <c r="N263" s="1" t="n"/>
+      <c r="N263" s="2" t="n">
+        <v>46219.62708564815</v>
+      </c>
       <c r="O263" s="1" t="n"/>
       <c r="P263" s="1" t="n"/>
       <c r="Q263" s="1" t="inlineStr"/>
-      <c r="R263" s="1" t="inlineStr"/>
+      <c r="R263" s="1" t="inlineStr">
+        <is>
+          <t>Empresa possui débitos que impedem a baixa em São Paulo, enviado ao cliente para pagamento e protocolado nomente o processo. Aguardando a baixa definitiva do CCM SP.</t>
+        </is>
+      </c>
       <c r="S263" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21443,7 +21521,11 @@
         <v>0</v>
       </c>
       <c r="G267" s="1" t="n"/>
-      <c r="H267" s="1" t="n"/>
+      <c r="H267" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I267" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21457,7 +21539,7 @@
       </c>
       <c r="L267" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M267" s="1" t="inlineStr">
@@ -21469,7 +21551,7 @@
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
       <c r="Q267" s="1" t="inlineStr"/>
-      <c r="R267" s="1" t="n"/>
+      <c r="R267" s="1" t="inlineStr"/>
       <c r="S267" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21573,7 +21655,11 @@
         <v>0</v>
       </c>
       <c r="G269" s="1" t="n"/>
-      <c r="H269" s="1" t="n"/>
+      <c r="H269" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I269" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21587,7 +21673,7 @@
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M269" s="1" t="inlineStr">
@@ -21599,7 +21685,7 @@
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
       <c r="Q269" s="1" t="inlineStr"/>
-      <c r="R269" s="1" t="n"/>
+      <c r="R269" s="1" t="inlineStr"/>
       <c r="S269" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21636,7 +21722,11 @@
         <v>0</v>
       </c>
       <c r="G270" s="1" t="n"/>
-      <c r="H270" s="1" t="n"/>
+      <c r="H270" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I270" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21650,7 +21740,7 @@
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
@@ -21662,7 +21752,7 @@
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="n"/>
+      <c r="R270" s="1" t="inlineStr"/>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21699,7 +21789,11 @@
         <v>0</v>
       </c>
       <c r="G271" s="1" t="n"/>
-      <c r="H271" s="1" t="n"/>
+      <c r="H271" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I271" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21713,7 +21807,7 @@
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
@@ -21725,7 +21819,7 @@
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="Q271" s="1" t="inlineStr"/>
-      <c r="R271" s="1" t="n"/>
+      <c r="R271" s="1" t="inlineStr"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21762,7 +21856,11 @@
         <v>0</v>
       </c>
       <c r="G272" s="1" t="n"/>
-      <c r="H272" s="1" t="n"/>
+      <c r="H272" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I272" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21776,7 +21874,7 @@
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M272" s="1" t="inlineStr">
@@ -21788,7 +21886,7 @@
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
       <c r="Q272" s="1" t="inlineStr"/>
-      <c r="R272" s="1" t="n"/>
+      <c r="R272" s="1" t="inlineStr"/>
       <c r="S272" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21825,7 +21923,11 @@
         <v>0</v>
       </c>
       <c r="G273" s="1" t="n"/>
-      <c r="H273" s="1" t="n"/>
+      <c r="H273" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I273" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21839,7 +21941,7 @@
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
@@ -21851,7 +21953,7 @@
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="n"/>
+      <c r="R273" s="1" t="inlineStr"/>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21888,7 +21990,11 @@
         <v>0</v>
       </c>
       <c r="G274" s="1" t="n"/>
-      <c r="H274" s="1" t="n"/>
+      <c r="H274" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I274" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21902,7 +22008,7 @@
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M274" s="1" t="inlineStr">
@@ -21914,7 +22020,7 @@
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="Q274" s="1" t="inlineStr"/>
-      <c r="R274" s="1" t="n"/>
+      <c r="R274" s="1" t="inlineStr"/>
       <c r="S274" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21951,7 +22057,11 @@
         <v>0</v>
       </c>
       <c r="G275" s="1" t="n"/>
-      <c r="H275" s="1" t="n"/>
+      <c r="H275" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I275" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -21965,7 +22075,7 @@
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M275" s="1" t="inlineStr">
@@ -21977,7 +22087,7 @@
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="Q275" s="1" t="inlineStr"/>
-      <c r="R275" s="1" t="n"/>
+      <c r="R275" s="1" t="inlineStr"/>
       <c r="S275" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22014,7 +22124,11 @@
         <v>0</v>
       </c>
       <c r="G276" s="1" t="n"/>
-      <c r="H276" s="1" t="n"/>
+      <c r="H276" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I276" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22028,7 +22142,7 @@
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
@@ -22040,7 +22154,7 @@
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="n"/>
+      <c r="R276" s="1" t="inlineStr"/>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22077,7 +22191,11 @@
         <v>0</v>
       </c>
       <c r="G277" s="1" t="n"/>
-      <c r="H277" s="1" t="n"/>
+      <c r="H277" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I277" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22091,7 +22209,7 @@
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
@@ -22103,7 +22221,7 @@
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
-      <c r="R277" s="1" t="n"/>
+      <c r="R277" s="1" t="inlineStr"/>
       <c r="S277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22140,7 +22258,11 @@
         <v>0</v>
       </c>
       <c r="G278" s="1" t="n"/>
-      <c r="H278" s="1" t="n"/>
+      <c r="H278" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I278" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22154,7 +22276,7 @@
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M278" s="1" t="inlineStr">
@@ -22166,7 +22288,7 @@
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
-      <c r="R278" s="1" t="n"/>
+      <c r="R278" s="1" t="inlineStr"/>
       <c r="S278" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22270,7 +22392,11 @@
         <v>0</v>
       </c>
       <c r="G280" s="1" t="n"/>
-      <c r="H280" s="1" t="n"/>
+      <c r="H280" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I280" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22284,7 +22410,7 @@
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M280" s="1" t="inlineStr">
@@ -22296,7 +22422,7 @@
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
-      <c r="R280" s="1" t="n"/>
+      <c r="R280" s="1" t="inlineStr"/>
       <c r="S280" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22408,7 +22534,11 @@
           <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
-      <c r="H282" s="1" t="n"/>
+      <c r="H282" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I282" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22422,7 +22552,7 @@
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M282" s="1" t="inlineStr">
@@ -22434,7 +22564,7 @@
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
-      <c r="R282" s="1" t="n"/>
+      <c r="R282" s="1" t="inlineStr"/>
       <c r="S282" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22475,7 +22605,11 @@
           <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
-      <c r="H283" s="1" t="n"/>
+      <c r="H283" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I283" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22489,7 +22623,7 @@
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
@@ -22501,7 +22635,7 @@
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="n"/>
+      <c r="R283" s="1" t="inlineStr"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22542,7 +22676,11 @@
           <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
-      <c r="H284" s="1" t="n"/>
+      <c r="H284" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I284" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22556,7 +22694,7 @@
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M284" s="1" t="inlineStr">
@@ -22568,7 +22706,7 @@
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
-      <c r="R284" s="1" t="n"/>
+      <c r="R284" s="1" t="inlineStr"/>
       <c r="S284" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22609,7 +22747,11 @@
           <t>MERCH LTDA (FILIAL 1)</t>
         </is>
       </c>
-      <c r="H285" s="1" t="n"/>
+      <c r="H285" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I285" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
@@ -22623,7 +22765,7 @@
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
@@ -22635,7 +22777,7 @@
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="n"/>
+      <c r="R285" s="1" t="inlineStr"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
data: atualização base chamados 16-07-26 1803
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U295" headerRowCount="1">
-  <autoFilter ref="A1:U295"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U292" headerRowCount="1">
+  <autoFilter ref="A1:U292"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U295"/>
+  <dimension ref="A1:U292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21288,7 +21288,7 @@
       </c>
       <c r="L264" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M264" s="1" t="inlineStr">
@@ -21296,11 +21296,17 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N264" s="1" t="n"/>
+      <c r="N264" s="2" t="n">
+        <v>46219.75157017361</v>
+      </c>
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
       <c r="Q264" s="1" t="inlineStr"/>
-      <c r="R264" s="1" t="inlineStr"/>
+      <c r="R264" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviado para registro </t>
+        </is>
+      </c>
       <c r="S264" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21690,7 +21696,7 @@
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
@@ -21698,11 +21704,17 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N270" s="1" t="n"/>
+      <c r="N270" s="2" t="n">
+        <v>46219.74920023148</v>
+      </c>
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="inlineStr"/>
+      <c r="R270" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviada ao cliente</t>
+        </is>
+      </c>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21713,11 +21725,11 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>81070</v>
+        <v>80989</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
@@ -21732,7 +21744,7 @@
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.2681 Comercio de Alimentos Alves e Farias MATRIZ</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
@@ -21741,7 +21753,7 @@
       <c r="G271" s="1" t="n"/>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
@@ -21750,10 +21762,10 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46218.51467572917</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46220</v>
+        <v>46217</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21762,7 +21774,7 @@
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>João Oliveira</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
@@ -21780,35 +21792,39 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>81071</v>
+        <v>79793</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3252 Comercio de Alimentos Alves e Farias FILIAL 01</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G272" s="1" t="n"/>
+        <v>5655</v>
+      </c>
+      <c r="G272" s="1" t="inlineStr">
+        <is>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
       <c r="H272" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I272" s="1" t="inlineStr">
@@ -21817,10 +21833,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46218.51533788195</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46220</v>
+        <v>46185</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -21829,7 +21845,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -21847,16 +21863,16 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>81072</v>
+        <v>81004</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -21866,16 +21882,20 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.3257 Comercio de Alimentos Alves e Farias FILIAL 06</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G273" s="1" t="n"/>
+        <v>6869</v>
+      </c>
+      <c r="G273" s="1" t="inlineStr">
+        <is>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+        </is>
+      </c>
       <c r="H273" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I273" s="1" t="inlineStr">
@@ -21884,10 +21904,10 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46218.51577677084</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46220</v>
+        <v>46218</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
@@ -21896,7 +21916,7 @@
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
@@ -21914,16 +21934,16 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80989</v>
+        <v>81005</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -21933,16 +21953,20 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G274" s="1" t="n"/>
+        <v>6870</v>
+      </c>
+      <c r="G274" s="1" t="inlineStr">
+        <is>
+          <t>AC HOME PET RAÇÕES LTDA</t>
+        </is>
+      </c>
       <c r="H274" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I274" s="1" t="inlineStr">
@@ -21951,10 +21975,10 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
@@ -21963,7 +21987,7 @@
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
@@ -21981,34 +22005,34 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>79793</v>
+        <v>81091</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
-        <v>5655</v>
+        <v>6907</v>
       </c>
       <c r="G275" s="1" t="inlineStr">
         <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H275" s="1" t="inlineStr">
@@ -22022,10 +22046,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46185</v>
+        <v>46223</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22034,7 +22058,7 @@
       </c>
       <c r="M275" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N275" s="1" t="n"/>
@@ -22052,7 +22076,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>81004</v>
+        <v>81161</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22066,25 +22090,25 @@
       </c>
       <c r="D276" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Sarah, boa tarde!Por gentileza incluir no MGC o número da Inscrição Municipal - Prefeitura de Embu das Artes.</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
-        <v>6869</v>
+        <v>6916</v>
       </c>
       <c r="G276" s="1" t="inlineStr">
         <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+          <t>TAITI COMERCIO DE MATERIAIS PARA CONSTRUCAO LTDA (FILIAL 1)</t>
         </is>
       </c>
       <c r="H276" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Sarah Amaro</t>
         </is>
       </c>
       <c r="I276" s="1" t="inlineStr">
@@ -22093,10 +22117,10 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46219.69548784722</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
@@ -22105,7 +22129,7 @@
       </c>
       <c r="M276" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="N276" s="1" t="n"/>
@@ -22123,67 +22147,73 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>81005</v>
+        <v>79833</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
-        <v>6870</v>
+        <v>6125</v>
       </c>
       <c r="G277" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H277" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I277" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46218</v>
+        <v>46184</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
-      <c r="N277" s="1" t="n"/>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="N277" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
-      <c r="R277" s="1" t="inlineStr"/>
+      <c r="R277" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22194,34 +22224,34 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>81091</v>
+        <v>79834</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
-        <v>6907</v>
+        <v>6162</v>
       </c>
       <c r="G278" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H278" s="1" t="inlineStr">
@@ -22231,14 +22261,14 @@
       </c>
       <c r="I278" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46223</v>
+        <v>46184</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
@@ -22247,7 +22277,7 @@
       </c>
       <c r="M278" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N278" s="1" t="n"/>
@@ -22265,63 +22295,67 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>81161</v>
+        <v>79865</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Sarah, boa tarde!Por gentileza incluir no MGC o número da Inscrição Municipal - Prefeitura de Embu das Artes.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
-        <v>6916</v>
+        <v>6278</v>
       </c>
       <c r="G279" s="1" t="inlineStr">
         <is>
-          <t>TAITI COMERCIO DE MATERIAIS PARA CONSTRUCAO LTDA (FILIAL 1)</t>
-        </is>
-      </c>
-      <c r="H279" s="1" t="n"/>
+          <t>EMPORIO DOS FRIOS LTDA</t>
+        </is>
+      </c>
+      <c r="H279" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I279" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46219.69548784722</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46220</v>
+        <v>46185</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="n"/>
+      <c r="R279" s="1" t="inlineStr"/>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22332,16 +22366,16 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>79833</v>
+        <v>79854</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22351,15 +22385,15 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>6125</v>
+        <v>6302</v>
       </c>
       <c r="G280" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H280" s="1" t="inlineStr">
@@ -22373,7 +22407,7 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K280" s="2" t="n">
         <v>46184</v>
@@ -22403,16 +22437,16 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>79834</v>
+        <v>79863</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22422,15 +22456,15 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>6162</v>
+        <v>6404</v>
       </c>
       <c r="G281" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H281" s="1" t="inlineStr">
@@ -22444,10 +22478,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22456,7 +22490,7 @@
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
@@ -22474,16 +22508,16 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>79865</v>
+        <v>79835</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
@@ -22493,15 +22527,15 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
-        <v>6278</v>
+        <v>6485</v>
       </c>
       <c r="G282" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H282" s="1" t="inlineStr">
@@ -22515,10 +22549,10 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
@@ -22527,7 +22561,7 @@
       </c>
       <c r="M282" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N282" s="1" t="n"/>
@@ -22545,7 +22579,7 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>79854</v>
+        <v>79866</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
@@ -22564,15 +22598,15 @@
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
-        <v>6302</v>
+        <v>6539</v>
       </c>
       <c r="G283" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H283" s="1" t="inlineStr">
@@ -22586,10 +22620,10 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
@@ -22598,7 +22632,7 @@
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
@@ -22616,7 +22650,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>79863</v>
+        <v>79859</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
@@ -22635,15 +22669,15 @@
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
-        <v>6404</v>
+        <v>6570</v>
       </c>
       <c r="G284" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H284" s="1" t="inlineStr">
@@ -22657,7 +22691,7 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K284" s="2" t="n">
         <v>46185</v>
@@ -22687,16 +22721,16 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>79835</v>
+        <v>79860</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
@@ -22706,15 +22740,15 @@
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>6485</v>
+        <v>6581</v>
       </c>
       <c r="G285" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H285" s="1" t="inlineStr">
@@ -22728,10 +22762,10 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
@@ -22740,7 +22774,7 @@
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
@@ -22758,7 +22792,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>79866</v>
+        <v>79861</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
@@ -22777,15 +22811,15 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6539</v>
+        <v>6583</v>
       </c>
       <c r="G286" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H286" s="1" t="inlineStr">
@@ -22799,7 +22833,7 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K286" s="2" t="n">
         <v>46185</v>
@@ -22829,16 +22863,16 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>79859</v>
+        <v>79867</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
@@ -22848,15 +22882,15 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6570</v>
+        <v>6704</v>
       </c>
       <c r="G287" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H287" s="1" t="inlineStr">
@@ -22870,7 +22904,7 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K287" s="2" t="n">
         <v>46185</v>
@@ -22900,7 +22934,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>79860</v>
+        <v>79856</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -22919,15 +22953,15 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>6581</v>
+        <v>4225</v>
       </c>
       <c r="G288" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H288" s="1" t="inlineStr">
@@ -22941,10 +22975,10 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -22953,7 +22987,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -22971,7 +23005,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>79861</v>
+        <v>79855</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -22990,15 +23024,15 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>6583</v>
+        <v>4765</v>
       </c>
       <c r="G289" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H289" s="1" t="inlineStr">
@@ -23012,7 +23046,7 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K289" s="2" t="n">
         <v>46185</v>
@@ -23024,7 +23058,7 @@
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
@@ -23042,7 +23076,7 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79867</v>
+        <v>81019</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
@@ -23051,27 +23085,23 @@
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6704</v>
-      </c>
-      <c r="G290" s="1" t="inlineStr">
-        <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G290" s="1" t="n"/>
       <c r="H290" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23079,70 +23109,75 @@
       </c>
       <c r="I290" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
-      <c r="R290" s="1" t="inlineStr"/>
+      <c r="R290" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
+        </is>
+      </c>
       <c r="S290" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T290" s="1" t="n"/>
+      <c r="T290" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
       <c r="U290" s="1" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>79856</v>
+        <v>81052</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>4225</v>
-      </c>
-      <c r="G291" s="1" t="inlineStr">
-        <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G291" s="1" t="n"/>
       <c r="H291" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23154,26 +23189,30 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46184</v>
+        <v>46219</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
       <c r="Q291" s="1" t="inlineStr"/>
-      <c r="R291" s="1" t="inlineStr"/>
+      <c r="R291" s="1" t="inlineStr">
+        <is>
+          <t>cobramos os documentos do antigo contador.</t>
+        </is>
+      </c>
       <c r="S291" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23184,36 +23223,32 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>79855</v>
+        <v>81055</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>4765</v>
-      </c>
-      <c r="G292" s="1" t="inlineStr">
-        <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G292" s="1" t="n"/>
       <c r="H292" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23225,26 +23260,32 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46185</v>
+        <v>46219</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N292" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N292" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
       <c r="Q292" s="1" t="inlineStr"/>
-      <c r="R292" s="1" t="inlineStr"/>
+      <c r="R292" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
       <c r="S292" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23252,226 +23293,6 @@
       </c>
       <c r="T292" s="1" t="n"/>
       <c r="U292" s="1" t="inlineStr"/>
-    </row>
-    <row r="293">
-      <c r="A293" s="1" t="n">
-        <v>81019</v>
-      </c>
-      <c r="B293" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C293" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D293" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E293" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
-        </is>
-      </c>
-      <c r="F293" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G293" s="1" t="n"/>
-      <c r="H293" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I293" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="J293" s="2" t="n">
-        <v>46217.43210269676</v>
-      </c>
-      <c r="K293" s="2" t="n">
-        <v>46218</v>
-      </c>
-      <c r="L293" s="1" t="inlineStr">
-        <is>
-          <t>Devolvido para Solicitante</t>
-        </is>
-      </c>
-      <c r="M293" s="1" t="inlineStr">
-        <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N293" s="1" t="n"/>
-      <c r="O293" s="1" t="n"/>
-      <c r="P293" s="1" t="n"/>
-      <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
-      <c r="S293" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T293" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="U293" s="1" t="inlineStr"/>
-    </row>
-    <row r="294">
-      <c r="A294" s="1" t="n">
-        <v>81052</v>
-      </c>
-      <c r="B294" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C294" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D294" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E294" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
-        </is>
-      </c>
-      <c r="F294" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G294" s="1" t="n"/>
-      <c r="H294" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I294" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J294" s="2" t="n">
-        <v>46218.38736744213</v>
-      </c>
-      <c r="K294" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="L294" s="1" t="inlineStr">
-        <is>
-          <t>Devolvido para Responsável</t>
-        </is>
-      </c>
-      <c r="M294" s="1" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N294" s="1" t="n"/>
-      <c r="O294" s="1" t="n"/>
-      <c r="P294" s="1" t="n"/>
-      <c r="Q294" s="1" t="inlineStr"/>
-      <c r="R294" s="1" t="inlineStr">
-        <is>
-          <t>cobramos os documentos do antigo contador.</t>
-        </is>
-      </c>
-      <c r="S294" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T294" s="1" t="n"/>
-      <c r="U294" s="1" t="inlineStr"/>
-    </row>
-    <row r="295">
-      <c r="A295" s="1" t="n">
-        <v>81055</v>
-      </c>
-      <c r="B295" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C295" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D295" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E295" s="1" t="inlineStr">
-        <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
-        </is>
-      </c>
-      <c r="F295" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G295" s="1" t="n"/>
-      <c r="H295" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I295" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J295" s="2" t="n">
-        <v>46218.40379614583</v>
-      </c>
-      <c r="K295" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="L295" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M295" s="1" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N295" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
-      <c r="O295" s="1" t="n"/>
-      <c r="P295" s="1" t="n"/>
-      <c r="Q295" s="1" t="inlineStr"/>
-      <c r="R295" s="1" t="inlineStr">
-        <is>
-          <t>Aguardando retorno dos dados do contador</t>
-        </is>
-      </c>
-      <c r="S295" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T295" s="1" t="n"/>
-      <c r="U295" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 17-07-26 1619
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -3179,7 +3179,7 @@
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J34" s="2" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="L34" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M34" s="1" t="inlineStr">
@@ -3198,11 +3198,9 @@
           <t>Simone Marques</t>
         </is>
       </c>
-      <c r="N34" s="2" t="n">
-        <v>46190.46143564815</v>
-      </c>
+      <c r="N34" s="1" t="n"/>
       <c r="O34" s="2" t="n">
-        <v>46227</v>
+        <v>46234</v>
       </c>
       <c r="P34" s="1" t="n"/>
       <c r="Q34" s="1" t="inlineStr"/>
@@ -3216,7 +3214,11 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T34" s="1" t="n"/>
+      <c r="T34" s="1" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
+        </is>
+      </c>
       <c r="U34" s="1" t="inlineStr">
         <is>
           <t>Isabella Nascimento</t>
@@ -6703,7 +6705,7 @@
       </c>
       <c r="L77" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M77" s="1" t="inlineStr">
@@ -6715,12 +6717,22 @@
       <c r="O77" s="2" t="n">
         <v>46217</v>
       </c>
-      <c r="P77" s="1" t="n"/>
-      <c r="Q77" s="1" t="inlineStr"/>
-      <c r="R77" s="1" t="inlineStr"/>
+      <c r="P77" s="2" t="n">
+        <v>46220.66134609954</v>
+      </c>
+      <c r="Q77" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R77" s="1" t="inlineStr">
+        <is>
+          <t>Paralegal em atendimento</t>
+        </is>
+      </c>
       <c r="S77" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T77" s="1" t="n"/>
@@ -14220,7 +14232,7 @@
       </c>
       <c r="L169" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M169" s="1" t="inlineStr">
@@ -14234,8 +14246,14 @@
       <c r="O169" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="P169" s="1" t="n"/>
-      <c r="Q169" s="1" t="inlineStr"/>
+      <c r="P169" s="2" t="n">
+        <v>46220.66189042824</v>
+      </c>
+      <c r="Q169" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="R169" s="1" t="inlineStr">
         <is>
           <t>Vai ser conciliado junto ao fechamento 06/2026</t>
@@ -14243,7 +14261,7 @@
       </c>
       <c r="S169" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T169" s="1" t="n"/>
@@ -14504,7 +14522,7 @@
       </c>
       <c r="L173" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M173" s="1" t="inlineStr">
@@ -14518,8 +14536,14 @@
       <c r="O173" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="P173" s="1" t="n"/>
-      <c r="Q173" s="1" t="inlineStr"/>
+      <c r="P173" s="2" t="n">
+        <v>46220.66202916667</v>
+      </c>
+      <c r="Q173" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="R173" s="1" t="inlineStr">
         <is>
           <t>Vai ser feito no fechamento</t>
@@ -14527,7 +14551,7 @@
       </c>
       <c r="S173" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T173" s="1" t="n"/>
@@ -15069,7 +15093,7 @@
       </c>
       <c r="L180" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M180" s="1" t="inlineStr">
@@ -15081,12 +15105,22 @@
       <c r="O180" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="P180" s="1" t="n"/>
-      <c r="Q180" s="1" t="inlineStr"/>
-      <c r="R180" s="1" t="inlineStr"/>
+      <c r="P180" s="2" t="n">
+        <v>46220.66110667824</v>
+      </c>
+      <c r="Q180" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R180" s="1" t="inlineStr">
+        <is>
+          <t>Enviado no email 14/07</t>
+        </is>
+      </c>
       <c r="S180" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T180" s="1" t="n"/>
@@ -15158,7 +15192,7 @@
         <v>46216.74338672453</v>
       </c>
       <c r="O181" s="2" t="n">
-        <v>46217</v>
+        <v>46234</v>
       </c>
       <c r="P181" s="1" t="n"/>
       <c r="Q181" s="1" t="inlineStr"/>
@@ -15314,7 +15348,7 @@
       </c>
       <c r="L183" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M183" s="1" t="inlineStr">
@@ -15326,12 +15360,22 @@
       <c r="O183" s="2" t="n">
         <v>46219</v>
       </c>
-      <c r="P183" s="1" t="n"/>
-      <c r="Q183" s="1" t="inlineStr"/>
-      <c r="R183" s="1" t="inlineStr"/>
+      <c r="P183" s="2" t="n">
+        <v>46220.65923896991</v>
+      </c>
+      <c r="Q183" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R183" s="1" t="inlineStr">
+        <is>
+          <t>Vai ser lançado no fechamento</t>
+        </is>
+      </c>
       <c r="S183" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T183" s="1" t="n"/>
@@ -16043,7 +16087,7 @@
       </c>
       <c r="L192" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M192" s="1" t="inlineStr">
@@ -16055,12 +16099,22 @@
       <c r="O192" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="P192" s="1" t="n"/>
-      <c r="Q192" s="1" t="inlineStr"/>
-      <c r="R192" s="1" t="inlineStr"/>
+      <c r="P192" s="2" t="n">
+        <v>46220.65987260417</v>
+      </c>
+      <c r="Q192" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R192" s="1" t="inlineStr">
+        <is>
+          <t>Estoque ja foi ajustado (solicitação duplicada , recebido via email)</t>
+        </is>
+      </c>
       <c r="S192" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T192" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 20-07-26 0941
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -5376,7 +5376,11 @@
           <t>LUSINDE INVEST EMPREENDIMENTOS S.A.</t>
         </is>
       </c>
-      <c r="H61" s="1" t="n"/>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I61" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -5390,7 +5394,7 @@
       </c>
       <c r="L61" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M61" s="1" t="inlineStr">
@@ -5402,14 +5406,18 @@
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="n"/>
       <c r="Q61" s="1" t="inlineStr"/>
-      <c r="R61" s="1" t="n"/>
+      <c r="R61" s="1" t="inlineStr"/>
       <c r="S61" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T61" s="1" t="n"/>
-      <c r="U61" s="1" t="inlineStr"/>
+      <c r="U61" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -12945,7 +12953,11 @@
           <t xml:space="preserve">PLANET GRAPHICS LTDA </t>
         </is>
       </c>
-      <c r="H153" s="1" t="n"/>
+      <c r="H153" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I153" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -12959,7 +12971,7 @@
       </c>
       <c r="L153" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M153" s="1" t="inlineStr">
@@ -12971,14 +12983,18 @@
       <c r="O153" s="1" t="n"/>
       <c r="P153" s="1" t="n"/>
       <c r="Q153" s="1" t="inlineStr"/>
-      <c r="R153" s="1" t="n"/>
+      <c r="R153" s="1" t="inlineStr"/>
       <c r="S153" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T153" s="1" t="n"/>
-      <c r="U153" s="1" t="inlineStr"/>
+      <c r="U153" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -13087,7 +13103,11 @@
           <t>POWER FINANCIAL DO BRASIL S.A.</t>
         </is>
       </c>
-      <c r="H155" s="1" t="n"/>
+      <c r="H155" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I155" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -13101,7 +13121,7 @@
       </c>
       <c r="L155" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M155" s="1" t="inlineStr">
@@ -13113,14 +13133,18 @@
       <c r="O155" s="1" t="n"/>
       <c r="P155" s="1" t="n"/>
       <c r="Q155" s="1" t="inlineStr"/>
-      <c r="R155" s="1" t="n"/>
+      <c r="R155" s="1" t="inlineStr"/>
       <c r="S155" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T155" s="1" t="n"/>
-      <c r="U155" s="1" t="inlineStr"/>
+      <c r="U155" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -14149,7 +14173,11 @@
           <t>NOVAIS IT SOLUCOES TECNOLOGICAS LTDA</t>
         </is>
       </c>
-      <c r="H168" s="1" t="n"/>
+      <c r="H168" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I168" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14163,7 +14191,7 @@
       </c>
       <c r="L168" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M168" s="1" t="inlineStr">
@@ -14175,14 +14203,18 @@
       <c r="O168" s="1" t="n"/>
       <c r="P168" s="1" t="n"/>
       <c r="Q168" s="1" t="inlineStr"/>
-      <c r="R168" s="1" t="n"/>
+      <c r="R168" s="1" t="inlineStr"/>
       <c r="S168" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T168" s="1" t="n"/>
-      <c r="U168" s="1" t="inlineStr"/>
+      <c r="U168" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -14380,7 +14412,11 @@
           <t>CONCEITO LOCADORA LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n"/>
+      <c r="H171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I171" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14394,7 +14430,7 @@
       </c>
       <c r="L171" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M171" s="1" t="inlineStr">
@@ -14406,14 +14442,18 @@
       <c r="O171" s="1" t="n"/>
       <c r="P171" s="1" t="n"/>
       <c r="Q171" s="1" t="inlineStr"/>
-      <c r="R171" s="1" t="n"/>
+      <c r="R171" s="1" t="inlineStr"/>
       <c r="S171" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T171" s="1" t="n"/>
-      <c r="U171" s="1" t="inlineStr"/>
+      <c r="U171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -14514,7 +14554,11 @@
           <t>CZLOC LOCACAO DE EQUIPAMENTOS PARA CONSTRUCAO CIVIL LTDA</t>
         </is>
       </c>
-      <c r="H173" s="1" t="n"/>
+      <c r="H173" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I173" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14528,7 +14572,7 @@
       </c>
       <c r="L173" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M173" s="1" t="inlineStr">
@@ -14540,14 +14584,18 @@
       <c r="O173" s="1" t="n"/>
       <c r="P173" s="1" t="n"/>
       <c r="Q173" s="1" t="inlineStr"/>
-      <c r="R173" s="1" t="n"/>
+      <c r="R173" s="1" t="inlineStr"/>
       <c r="S173" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T173" s="1" t="n"/>
-      <c r="U173" s="1" t="inlineStr"/>
+      <c r="U173" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -14829,7 +14877,11 @@
           <t>INDUSTRIA E COMERCIO RAIZES DO NORDESTE LTDA</t>
         </is>
       </c>
-      <c r="H177" s="1" t="n"/>
+      <c r="H177" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I177" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14843,7 +14895,7 @@
       </c>
       <c r="L177" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M177" s="1" t="inlineStr">
@@ -14855,14 +14907,18 @@
       <c r="O177" s="1" t="n"/>
       <c r="P177" s="1" t="n"/>
       <c r="Q177" s="1" t="inlineStr"/>
-      <c r="R177" s="1" t="n"/>
+      <c r="R177" s="1" t="inlineStr"/>
       <c r="S177" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T177" s="1" t="n"/>
-      <c r="U177" s="1" t="inlineStr"/>
+      <c r="U177" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -16233,7 +16289,11 @@
           <t>GRIFFY FERRAMENTARIA DE PRECISAO LTDA</t>
         </is>
       </c>
-      <c r="H194" s="1" t="n"/>
+      <c r="H194" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I194" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -16247,7 +16307,7 @@
       </c>
       <c r="L194" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M194" s="1" t="inlineStr">
@@ -16259,14 +16319,18 @@
       <c r="O194" s="1" t="n"/>
       <c r="P194" s="1" t="n"/>
       <c r="Q194" s="1" t="inlineStr"/>
-      <c r="R194" s="1" t="n"/>
+      <c r="R194" s="1" t="inlineStr"/>
       <c r="S194" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T194" s="1" t="n"/>
-      <c r="U194" s="1" t="inlineStr"/>
+      <c r="U194" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -17218,67 +17282,59 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>80792</v>
+        <v>81202</v>
       </c>
       <c r="B208" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C208" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D208" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>1.01.002.0007.00013 - Devoluções de Compra a Receber1.01.002.0007.00014 - Devoluções de Troca a Receber</t>
+          <t>Bom dia, preciso do certificado da empresa 5603 -Carlos Antunes e que seja renovado o certificado da empresa 4793- Costa lima</t>
         </is>
       </c>
       <c r="F208" s="1" t="n">
-        <v>861</v>
-      </c>
-      <c r="G208" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO CASTELO DA SERRA LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H208" s="1" t="inlineStr">
-        <is>
-          <t>Diego Lima</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G208" s="1" t="n"/>
+      <c r="H208" s="1" t="n"/>
       <c r="I208" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J208" s="2" t="n">
-        <v>46210.5704596412</v>
+        <v>46223.39712596065</v>
       </c>
       <c r="K208" s="2" t="n">
-        <v>46213</v>
+        <v>46224</v>
       </c>
       <c r="L208" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M208" s="1" t="inlineStr">
         <is>
-          <t>Rejane Coelho</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="N208" s="1" t="n"/>
       <c r="O208" s="1" t="n"/>
       <c r="P208" s="1" t="n"/>
       <c r="Q208" s="1" t="inlineStr"/>
-      <c r="R208" s="1" t="inlineStr"/>
+      <c r="R208" s="1" t="n"/>
       <c r="S208" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -17289,7 +17345,7 @@
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
-        <v>80732</v>
+        <v>80792</v>
       </c>
       <c r="B209" s="1" t="inlineStr">
         <is>
@@ -17308,7 +17364,7 @@
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>1.01.002.0001.00005 - Acordos Comerciais e Bonificações a Receber</t>
+          <t>1.01.002.0007.00013 - Devoluções de Compra a Receber1.01.002.0007.00014 - Devoluções de Troca a Receber</t>
         </is>
       </c>
       <c r="F209" s="1" t="n">
@@ -17330,10 +17386,10 @@
         </is>
       </c>
       <c r="J209" s="2" t="n">
-        <v>46206.67579409722</v>
+        <v>46210.5704596412</v>
       </c>
       <c r="K209" s="2" t="n">
-        <v>46210</v>
+        <v>46213</v>
       </c>
       <c r="L209" s="1" t="inlineStr">
         <is>
@@ -17360,7 +17416,7 @@
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
-        <v>80733</v>
+        <v>80732</v>
       </c>
       <c r="B210" s="1" t="inlineStr">
         <is>
@@ -17379,7 +17435,7 @@
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>1.01.001.0001.00001 - Caixa</t>
+          <t>1.01.002.0001.00005 - Acordos Comerciais e Bonificações a Receber</t>
         </is>
       </c>
       <c r="F210" s="1" t="n">
@@ -17401,7 +17457,7 @@
         </is>
       </c>
       <c r="J210" s="2" t="n">
-        <v>46206.67633518518</v>
+        <v>46206.67579409722</v>
       </c>
       <c r="K210" s="2" t="n">
         <v>46210</v>
@@ -17431,7 +17487,7 @@
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
-        <v>80734</v>
+        <v>80733</v>
       </c>
       <c r="B211" s="1" t="inlineStr">
         <is>
@@ -17450,7 +17506,7 @@
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>2.01.005.0002.00024 - Faturas Pendentes de Repasse</t>
+          <t>1.01.001.0001.00001 - Caixa</t>
         </is>
       </c>
       <c r="F211" s="1" t="n">
@@ -17472,7 +17528,7 @@
         </is>
       </c>
       <c r="J211" s="2" t="n">
-        <v>46206.6769059375</v>
+        <v>46206.67633518518</v>
       </c>
       <c r="K211" s="2" t="n">
         <v>46210</v>
@@ -17502,16 +17558,16 @@
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
-        <v>80008</v>
+        <v>80734</v>
       </c>
       <c r="B212" s="1" t="inlineStr">
         <is>
-          <t>Certificado</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C212" s="1" t="inlineStr">
         <is>
-          <t>Certificado digital</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D212" s="1" t="inlineStr">
@@ -17521,20 +17577,20 @@
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>Bom diaPor gentileza verificar pois o certificado venceu1065	Martinica Com.	65.486.375/0001-59</t>
+          <t>2.01.005.0002.00024 - Faturas Pendentes de Repasse</t>
         </is>
       </c>
       <c r="F212" s="1" t="n">
-        <v>1065</v>
+        <v>861</v>
       </c>
       <c r="G212" s="1" t="inlineStr">
         <is>
-          <t>MARTINICA COMERCIAL LTDA</t>
+          <t>SUPERMERCADO CASTELO DA SERRA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H212" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Diego Lima</t>
         </is>
       </c>
       <c r="I212" s="1" t="inlineStr">
@@ -17543,10 +17599,10 @@
         </is>
       </c>
       <c r="J212" s="2" t="n">
-        <v>46188.45542777778</v>
+        <v>46206.6769059375</v>
       </c>
       <c r="K212" s="2" t="n">
-        <v>46189</v>
+        <v>46210</v>
       </c>
       <c r="L212" s="1" t="inlineStr">
         <is>
@@ -17555,7 +17611,7 @@
       </c>
       <c r="M212" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Rejane Coelho</t>
         </is>
       </c>
       <c r="N212" s="1" t="n"/>
@@ -17573,16 +17629,16 @@
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
-        <v>79890</v>
+        <v>80008</v>
       </c>
       <c r="B213" s="1" t="inlineStr">
         <is>
-          <t>Solicitação sem retorno</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C213" s="1" t="inlineStr">
         <is>
-          <t>Solicitação sem retorno</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D213" s="1" t="inlineStr">
@@ -17592,20 +17648,20 @@
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,Por gentileza, verificar distribuição de lucros referente 2026, não recebemos nenhum e-mail do grupo Kanashiro.</t>
+          <t>Bom diaPor gentileza verificar pois o certificado venceu1065	Martinica Com.	65.486.375/0001-59</t>
         </is>
       </c>
       <c r="F213" s="1" t="n">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="G213" s="1" t="inlineStr">
         <is>
-          <t>Supermercado Kanashiro Ltda</t>
+          <t>MARTINICA COMERCIAL LTDA</t>
         </is>
       </c>
       <c r="H213" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="I213" s="1" t="inlineStr">
@@ -17614,32 +17670,26 @@
         </is>
       </c>
       <c r="J213" s="2" t="n">
-        <v>46184.46686350695</v>
+        <v>46188.45542777778</v>
       </c>
       <c r="K213" s="2" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="L213" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M213" s="1" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
-        </is>
-      </c>
-      <c r="N213" s="2" t="n">
-        <v>46185.43777230324</v>
-      </c>
+          <t>Edileide Dias</t>
+        </is>
+      </c>
+      <c r="N213" s="1" t="n"/>
       <c r="O213" s="1" t="n"/>
       <c r="P213" s="1" t="n"/>
       <c r="Q213" s="1" t="inlineStr"/>
-      <c r="R213" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, ser mais clara na solicitação, o que deseja ser verificado ?</t>
-        </is>
-      </c>
+      <c r="R213" s="1" t="inlineStr"/>
       <c r="S213" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -17650,39 +17700,39 @@
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
-        <v>78306</v>
+        <v>79890</v>
       </c>
       <c r="B214" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Solicitação sem retorno</t>
         </is>
       </c>
       <c r="C214" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Solicitação sem retorno</t>
         </is>
       </c>
       <c r="D214" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>Bom dia,Por gentileza, verificar distribuição de lucros referente 2026, não recebemos nenhum e-mail do grupo Kanashiro.</t>
         </is>
       </c>
       <c r="F214" s="1" t="n">
-        <v>1286</v>
+        <v>1066</v>
       </c>
       <c r="G214" s="1" t="inlineStr">
         <is>
-          <t>BY ENGENHARIA IMPORTAÇÃO E EXPORTAÇÃO LTDA (MATRIZ)</t>
+          <t>Supermercado Kanashiro Ltda</t>
         </is>
       </c>
       <c r="H214" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="I214" s="1" t="inlineStr">
@@ -17691,26 +17741,32 @@
         </is>
       </c>
       <c r="J214" s="2" t="n">
-        <v>46111.42803700231</v>
+        <v>46184.46686350695</v>
       </c>
       <c r="K214" s="2" t="n">
-        <v>46122</v>
+        <v>46188</v>
       </c>
       <c r="L214" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M214" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
-        </is>
-      </c>
-      <c r="N214" s="1" t="n"/>
+          <t>Karina Santos</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="n">
+        <v>46185.43777230324</v>
+      </c>
       <c r="O214" s="1" t="n"/>
       <c r="P214" s="1" t="n"/>
       <c r="Q214" s="1" t="inlineStr"/>
-      <c r="R214" s="1" t="inlineStr"/>
+      <c r="R214" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, ser mais clara na solicitação, o que deseja ser verificado ?</t>
+        </is>
+      </c>
       <c r="S214" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -17721,16 +17777,16 @@
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
-        <v>79733</v>
+        <v>78306</v>
       </c>
       <c r="B215" s="1" t="inlineStr">
         <is>
-          <t>Malha Fiscal</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C215" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D215" s="1" t="inlineStr">
@@ -17740,20 +17796,20 @@
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>AGUARDANDO RETORNO DESDE 26/06/2026 - ANALISE ENVIADA E-MAIL</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F215" s="1" t="n">
-        <v>1556</v>
+        <v>1286</v>
       </c>
       <c r="G215" s="1" t="inlineStr">
         <is>
-          <t>GENGIBRE ADMINISTRACAO E PARTICIPACOES S.A.</t>
+          <t>BY ENGENHARIA IMPORTAÇÃO E EXPORTAÇÃO LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H215" s="1" t="inlineStr">
         <is>
-          <t>Karine Gusmão</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="I215" s="1" t="inlineStr">
@@ -17762,10 +17818,10 @@
         </is>
       </c>
       <c r="J215" s="2" t="n">
-        <v>46180.49354722222</v>
+        <v>46111.42803700231</v>
       </c>
       <c r="K215" s="2" t="n">
-        <v>46182</v>
+        <v>46122</v>
       </c>
       <c r="L215" s="1" t="inlineStr">
         <is>
@@ -17774,7 +17830,7 @@
       </c>
       <c r="M215" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N215" s="1" t="n"/>
@@ -17792,7 +17848,7 @@
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
-        <v>79731</v>
+        <v>79733</v>
       </c>
       <c r="B216" s="1" t="inlineStr">
         <is>
@@ -17811,20 +17867,20 @@
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>RETIFICAR DCTF ANO BASE 2023 - CONFORME EMAIL ENVIADO AO CLIENTE EM 27/05/2026</t>
+          <t>AGUARDANDO RETORNO DESDE 26/06/2026 - ANALISE ENVIADA E-MAIL</t>
         </is>
       </c>
       <c r="F216" s="1" t="n">
-        <v>1931</v>
+        <v>1556</v>
       </c>
       <c r="G216" s="1" t="inlineStr">
         <is>
-          <t>GRILD - PLASTIC INDÚSTRIA, COMÉRCIO E IMPORTAÇÃO LTDA</t>
+          <t>GENGIBRE ADMINISTRACAO E PARTICIPACOES S.A.</t>
         </is>
       </c>
       <c r="H216" s="1" t="inlineStr">
         <is>
-          <t>Luiz Ferreira</t>
+          <t>Karine Gusmão</t>
         </is>
       </c>
       <c r="I216" s="1" t="inlineStr">
@@ -17833,10 +17889,10 @@
         </is>
       </c>
       <c r="J216" s="2" t="n">
-        <v>46180.44674649306</v>
+        <v>46180.49354722222</v>
       </c>
       <c r="K216" s="2" t="n">
-        <v>46185</v>
+        <v>46182</v>
       </c>
       <c r="L216" s="1" t="inlineStr">
         <is>
@@ -17859,24 +17915,20 @@
         </is>
       </c>
       <c r="T216" s="1" t="n"/>
-      <c r="U216" s="1" t="inlineStr">
-        <is>
-          <t>Erika Santana</t>
-        </is>
-      </c>
+      <c r="U216" s="1" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
-        <v>78322</v>
+        <v>79731</v>
       </c>
       <c r="B217" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Malha Fiscal</t>
         </is>
       </c>
       <c r="C217" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D217" s="1" t="inlineStr">
@@ -17886,20 +17938,20 @@
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>RETIFICAR DCTF ANO BASE 2023 - CONFORME EMAIL ENVIADO AO CLIENTE EM 27/05/2026</t>
         </is>
       </c>
       <c r="F217" s="1" t="n">
-        <v>2209</v>
+        <v>1931</v>
       </c>
       <c r="G217" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">TENDAS PROMOCIONAIS INDUSTRIA E COMÉRCIO LTDA </t>
+          <t>GRILD - PLASTIC INDÚSTRIA, COMÉRCIO E IMPORTAÇÃO LTDA</t>
         </is>
       </c>
       <c r="H217" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Luiz Ferreira</t>
         </is>
       </c>
       <c r="I217" s="1" t="inlineStr">
@@ -17908,10 +17960,10 @@
         </is>
       </c>
       <c r="J217" s="2" t="n">
-        <v>46111.44774475694</v>
+        <v>46180.44674649306</v>
       </c>
       <c r="K217" s="2" t="n">
-        <v>46122</v>
+        <v>46185</v>
       </c>
       <c r="L217" s="1" t="inlineStr">
         <is>
@@ -17920,7 +17972,7 @@
       </c>
       <c r="M217" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="N217" s="1" t="n"/>
@@ -17934,43 +17986,47 @@
         </is>
       </c>
       <c r="T217" s="1" t="n"/>
-      <c r="U217" s="1" t="inlineStr"/>
+      <c r="U217" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
-        <v>80013</v>
+        <v>78322</v>
       </c>
       <c r="B218" s="1" t="inlineStr">
         <is>
-          <t>Certificado</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C218" s="1" t="inlineStr">
         <is>
-          <t>Certificado digital</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D218" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza verificar pois o certificado venceu2480	Marques Distribuidora de Horti Frutti Transportes Ltda	17.515.145/0001-28</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F218" s="1" t="n">
-        <v>2480</v>
+        <v>2209</v>
       </c>
       <c r="G218" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARQUES DISTRIBUIDORA DE HORTI FRUTTI TRANSPORTES LTDA </t>
+          <t xml:space="preserve">TENDAS PROMOCIONAIS INDUSTRIA E COMÉRCIO LTDA </t>
         </is>
       </c>
       <c r="H218" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I218" s="1" t="inlineStr">
@@ -17979,10 +18035,10 @@
         </is>
       </c>
       <c r="J218" s="2" t="n">
-        <v>46188.46272334491</v>
+        <v>46111.44774475694</v>
       </c>
       <c r="K218" s="2" t="n">
-        <v>46189</v>
+        <v>46122</v>
       </c>
       <c r="L218" s="1" t="inlineStr">
         <is>
@@ -17991,7 +18047,7 @@
       </c>
       <c r="M218" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N218" s="1" t="n"/>
@@ -18009,7 +18065,7 @@
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
-        <v>80039</v>
+        <v>80013</v>
       </c>
       <c r="B219" s="1" t="inlineStr">
         <is>
@@ -18028,15 +18084,15 @@
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde por gentileza verificar, pois não temos procuração eletronica para sdd</t>
+          <t>Por gentileza verificar pois o certificado venceu2480	Marques Distribuidora de Horti Frutti Transportes Ltda	17.515.145/0001-28</t>
         </is>
       </c>
       <c r="F219" s="1" t="n">
-        <v>2491</v>
+        <v>2480</v>
       </c>
       <c r="G219" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">HARVEST HORTIFRUTTI LTDA </t>
+          <t xml:space="preserve">MARQUES DISTRIBUIDORA DE HORTI FRUTTI TRANSPORTES LTDA </t>
         </is>
       </c>
       <c r="H219" s="1" t="inlineStr">
@@ -18050,7 +18106,7 @@
         </is>
       </c>
       <c r="J219" s="2" t="n">
-        <v>46188.58172743056</v>
+        <v>46188.46272334491</v>
       </c>
       <c r="K219" s="2" t="n">
         <v>46189</v>
@@ -18062,7 +18118,7 @@
       </c>
       <c r="M219" s="1" t="inlineStr">
         <is>
-          <t>Ana Barbosa</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
       <c r="N219" s="1" t="n"/>
@@ -18080,7 +18136,7 @@
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
-        <v>80014</v>
+        <v>80039</v>
       </c>
       <c r="B220" s="1" t="inlineStr">
         <is>
@@ -18099,15 +18155,15 @@
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza disponibilizar o ecpf do socio2500	CAEFHOLD Participações S.A.	17.655.772/0001-64	ANTONIO VAZ SILVA</t>
+          <t>Boa tarde por gentileza verificar, pois não temos procuração eletronica para sdd</t>
         </is>
       </c>
       <c r="F220" s="1" t="n">
-        <v>2500</v>
+        <v>2491</v>
       </c>
       <c r="G220" s="1" t="inlineStr">
         <is>
-          <t>CAEFHOLD Participações S.A.</t>
+          <t xml:space="preserve">HARVEST HORTIFRUTTI LTDA </t>
         </is>
       </c>
       <c r="H220" s="1" t="inlineStr">
@@ -18121,7 +18177,7 @@
         </is>
       </c>
       <c r="J220" s="2" t="n">
-        <v>46188.46337480324</v>
+        <v>46188.58172743056</v>
       </c>
       <c r="K220" s="2" t="n">
         <v>46189</v>
@@ -18133,7 +18189,7 @@
       </c>
       <c r="M220" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Ana Barbosa</t>
         </is>
       </c>
       <c r="N220" s="1" t="n"/>
@@ -18151,39 +18207,39 @@
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
-        <v>78304</v>
+        <v>80014</v>
       </c>
       <c r="B221" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C221" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D221" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>Por gentileza disponibilizar o ecpf do socio2500	CAEFHOLD Participações S.A.	17.655.772/0001-64	ANTONIO VAZ SILVA</t>
         </is>
       </c>
       <c r="F221" s="1" t="n">
-        <v>2620</v>
+        <v>2500</v>
       </c>
       <c r="G221" s="1" t="inlineStr">
         <is>
-          <t>ANTOCON GALVANOPLASTIA LTDA</t>
+          <t>CAEFHOLD Participações S.A.</t>
         </is>
       </c>
       <c r="H221" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="I221" s="1" t="inlineStr">
@@ -18192,10 +18248,10 @@
         </is>
       </c>
       <c r="J221" s="2" t="n">
-        <v>46111.42458850695</v>
+        <v>46188.46337480324</v>
       </c>
       <c r="K221" s="2" t="n">
-        <v>46122</v>
+        <v>46189</v>
       </c>
       <c r="L221" s="1" t="inlineStr">
         <is>
@@ -18204,7 +18260,7 @@
       </c>
       <c r="M221" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
       <c r="N221" s="1" t="n"/>
@@ -18222,39 +18278,39 @@
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
-        <v>81061</v>
+        <v>78304</v>
       </c>
       <c r="B222" s="1" t="inlineStr">
         <is>
-          <t>Certificado</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C222" s="1" t="inlineStr">
         <is>
-          <t>Certificado digital</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D222" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>Bom diaPor gentileza realizar a assinatura do ecf do cliente 2821-Espite</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F222" s="1" t="n">
-        <v>2821</v>
+        <v>2620</v>
       </c>
       <c r="G222" s="1" t="inlineStr">
         <is>
-          <t>ESPITE PARTICIPAÇÕES S.A.</t>
+          <t>ANTOCON GALVANOPLASTIA LTDA</t>
         </is>
       </c>
       <c r="H222" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I222" s="1" t="inlineStr">
@@ -18263,10 +18319,10 @@
         </is>
       </c>
       <c r="J222" s="2" t="n">
-        <v>46218.42798252315</v>
+        <v>46111.42458850695</v>
       </c>
       <c r="K222" s="2" t="n">
-        <v>46219</v>
+        <v>46122</v>
       </c>
       <c r="L222" s="1" t="inlineStr">
         <is>
@@ -18275,7 +18331,7 @@
       </c>
       <c r="M222" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N222" s="1" t="n"/>
@@ -18293,39 +18349,39 @@
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
-        <v>79738</v>
+        <v>81061</v>
       </c>
       <c r="B223" s="1" t="inlineStr">
         <is>
-          <t>Malha Fiscal</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C223" s="1" t="inlineStr">
         <is>
-          <t>Autorregularização</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D223" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>AGUARDANDO RETORNO DE ANALISE DE MALHA DESDE 25/05/2026 - ANALISE POR E-MAI - SERGIO SUGERIU NA ULTIMA SEMANA QUE PODIAMOS VERIFICAR OS VALORES DE 2022 PARA CREDITO, ANALISEI E VERIFIQUEI QUE A VALOR DE 227.186,29 DE RENDIMENTOS A MAIOR DO QUE ESTA NA DIRF VERIFICAR E LEVANTAR E-MAIL DA EPOCA, NÃO HA PERDCOMP PARA ESTES PERIODOS</t>
+          <t>Bom diaPor gentileza realizar a assinatura do ecf do cliente 2821-Espite</t>
         </is>
       </c>
       <c r="F223" s="1" t="n">
-        <v>2956</v>
+        <v>2821</v>
       </c>
       <c r="G223" s="1" t="inlineStr">
         <is>
-          <t>AGGYO ADMINISTRAÇÃO DE BENS E PARTICIPAÇÕES S.A.</t>
+          <t>ESPITE PARTICIPAÇÕES S.A.</t>
         </is>
       </c>
       <c r="H223" s="1" t="inlineStr">
         <is>
-          <t>Karine Gusmão</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="I223" s="1" t="inlineStr">
@@ -18334,10 +18390,10 @@
         </is>
       </c>
       <c r="J223" s="2" t="n">
-        <v>46180.61864918981</v>
+        <v>46218.42798252315</v>
       </c>
       <c r="K223" s="2" t="n">
-        <v>46182</v>
+        <v>46219</v>
       </c>
       <c r="L223" s="1" t="inlineStr">
         <is>
@@ -18346,7 +18402,7 @@
       </c>
       <c r="M223" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
       <c r="N223" s="1" t="n"/>
@@ -18364,7 +18420,7 @@
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
-        <v>79735</v>
+        <v>79738</v>
       </c>
       <c r="B224" s="1" t="inlineStr">
         <is>
@@ -18383,15 +18439,15 @@
       </c>
       <c r="E224" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">AGUARDANDO RETORNO DA ANALISE DA MALHA DESDE 26/05/2026 - ENVIADO POR E-MAIL </t>
+          <t>AGUARDANDO RETORNO DE ANALISE DE MALHA DESDE 25/05/2026 - ANALISE POR E-MAI - SERGIO SUGERIU NA ULTIMA SEMANA QUE PODIAMOS VERIFICAR OS VALORES DE 2022 PARA CREDITO, ANALISEI E VERIFIQUEI QUE A VALOR DE 227.186,29 DE RENDIMENTOS A MAIOR DO QUE ESTA NA DIRF VERIFICAR E LEVANTAR E-MAIL DA EPOCA, NÃO HA PERDCOMP PARA ESTES PERIODOS</t>
         </is>
       </c>
       <c r="F224" s="1" t="n">
-        <v>2959</v>
+        <v>2956</v>
       </c>
       <c r="G224" s="1" t="inlineStr">
         <is>
-          <t>SAVYS EMPREENDIMENTOS E PARTICIPAÇÕES S.A</t>
+          <t>AGGYO ADMINISTRAÇÃO DE BENS E PARTICIPAÇÕES S.A.</t>
         </is>
       </c>
       <c r="H224" s="1" t="inlineStr">
@@ -18405,7 +18461,7 @@
         </is>
       </c>
       <c r="J224" s="2" t="n">
-        <v>46180.50447491898</v>
+        <v>46180.61864918981</v>
       </c>
       <c r="K224" s="2" t="n">
         <v>46182</v>
@@ -18435,39 +18491,39 @@
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
-        <v>79889</v>
+        <v>79735</v>
       </c>
       <c r="B225" s="1" t="inlineStr">
         <is>
-          <t>Solicitação sem retorno</t>
+          <t>Malha Fiscal</t>
         </is>
       </c>
       <c r="C225" s="1" t="inlineStr">
         <is>
-          <t>Solicitação sem retorno</t>
+          <t>Autorregularização</t>
         </is>
       </c>
       <c r="D225" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E225" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,Por gentileza, verificar distribuição de lucros referente 2026, não recebemos nenhum e-mail do grupo Carvalho, o cliente não possui controle, mas retira todo ano.</t>
+          <t xml:space="preserve">AGUARDANDO RETORNO DA ANALISE DA MALHA DESDE 26/05/2026 - ENVIADO POR E-MAIL </t>
         </is>
       </c>
       <c r="F225" s="1" t="n">
-        <v>3195</v>
+        <v>2959</v>
       </c>
       <c r="G225" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO RT CARVALHO LTDA</t>
+          <t>SAVYS EMPREENDIMENTOS E PARTICIPAÇÕES S.A</t>
         </is>
       </c>
       <c r="H225" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
+          <t>Karine Gusmão</t>
         </is>
       </c>
       <c r="I225" s="1" t="inlineStr">
@@ -18476,10 +18532,10 @@
         </is>
       </c>
       <c r="J225" s="2" t="n">
-        <v>46184.46640107639</v>
+        <v>46180.50447491898</v>
       </c>
       <c r="K225" s="2" t="n">
-        <v>46188</v>
+        <v>46182</v>
       </c>
       <c r="L225" s="1" t="inlineStr">
         <is>
@@ -18488,7 +18544,7 @@
       </c>
       <c r="M225" s="1" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="N225" s="1" t="n"/>
@@ -18506,26 +18562,26 @@
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
-        <v>81194</v>
+        <v>79889</v>
       </c>
       <c r="B226" s="1" t="inlineStr">
         <is>
-          <t>Certificado</t>
+          <t>Solicitação sem retorno</t>
         </is>
       </c>
       <c r="C226" s="1" t="inlineStr">
         <is>
-          <t>Certificado digital</t>
+          <t>Solicitação sem retorno</t>
         </is>
       </c>
       <c r="D226" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E226" s="1" t="inlineStr">
         <is>
-          <t>solicitar que disponibilize o certificado em minha arvore.</t>
+          <t>Bom dia,Por gentileza, verificar distribuição de lucros referente 2026, não recebemos nenhum e-mail do grupo Carvalho, o cliente não possui controle, mas retira todo ano.</t>
         </is>
       </c>
       <c r="F226" s="1" t="n">
@@ -18536,33 +18592,37 @@
           <t>EMPORIO RT CARVALHO LTDA</t>
         </is>
       </c>
-      <c r="H226" s="1" t="n"/>
+      <c r="H226" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
       <c r="I226" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J226" s="2" t="n">
-        <v>46220.61613811342</v>
+        <v>46184.46640107639</v>
       </c>
       <c r="K226" s="2" t="n">
-        <v>46223</v>
+        <v>46188</v>
       </c>
       <c r="L226" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M226" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Karina Santos</t>
         </is>
       </c>
       <c r="N226" s="1" t="n"/>
       <c r="O226" s="1" t="n"/>
       <c r="P226" s="1" t="n"/>
       <c r="Q226" s="1" t="inlineStr"/>
-      <c r="R226" s="1" t="n"/>
+      <c r="R226" s="1" t="inlineStr"/>
       <c r="S226" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -18573,67 +18633,63 @@
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
-        <v>78313</v>
+        <v>81194</v>
       </c>
       <c r="B227" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C227" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D227" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E227" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>solicitar que disponibilize o certificado em minha arvore.</t>
         </is>
       </c>
       <c r="F227" s="1" t="n">
-        <v>3262</v>
+        <v>3195</v>
       </c>
       <c r="G227" s="1" t="inlineStr">
         <is>
-          <t>JCV INDÚSTRIA E COMÉRCIO DE PLÁSTICOS LTDA</t>
-        </is>
-      </c>
-      <c r="H227" s="1" t="inlineStr">
-        <is>
-          <t>Vander Silva</t>
-        </is>
-      </c>
+          <t>EMPORIO RT CARVALHO LTDA</t>
+        </is>
+      </c>
+      <c r="H227" s="1" t="n"/>
       <c r="I227" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J227" s="2" t="n">
-        <v>46111.43707260417</v>
+        <v>46220.61613811342</v>
       </c>
       <c r="K227" s="2" t="n">
-        <v>46122</v>
+        <v>46223</v>
       </c>
       <c r="L227" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M227" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N227" s="1" t="n"/>
       <c r="O227" s="1" t="n"/>
       <c r="P227" s="1" t="n"/>
       <c r="Q227" s="1" t="inlineStr"/>
-      <c r="R227" s="1" t="inlineStr"/>
+      <c r="R227" s="1" t="n"/>
       <c r="S227" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -18644,7 +18700,7 @@
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
-        <v>78309</v>
+        <v>78313</v>
       </c>
       <c r="B228" s="1" t="inlineStr">
         <is>
@@ -18667,11 +18723,11 @@
         </is>
       </c>
       <c r="F228" s="1" t="n">
-        <v>3499</v>
+        <v>3262</v>
       </c>
       <c r="G228" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emplaca Automação e Tecnologia Ltda. </t>
+          <t>JCV INDÚSTRIA E COMÉRCIO DE PLÁSTICOS LTDA</t>
         </is>
       </c>
       <c r="H228" s="1" t="inlineStr">
@@ -18685,7 +18741,7 @@
         </is>
       </c>
       <c r="J228" s="2" t="n">
-        <v>46111.43159019676</v>
+        <v>46111.43707260417</v>
       </c>
       <c r="K228" s="2" t="n">
         <v>46122</v>
@@ -18715,7 +18771,7 @@
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
-        <v>78326</v>
+        <v>78309</v>
       </c>
       <c r="B229" s="1" t="inlineStr">
         <is>
@@ -18738,16 +18794,16 @@
         </is>
       </c>
       <c r="F229" s="1" t="n">
-        <v>3598</v>
+        <v>3499</v>
       </c>
       <c r="G229" s="1" t="inlineStr">
         <is>
-          <t>VTZZ INDUSTRIA E COMÉRCIO LTDA</t>
+          <t xml:space="preserve">Emplaca Automação e Tecnologia Ltda. </t>
         </is>
       </c>
       <c r="H229" s="1" t="inlineStr">
         <is>
-          <t>Simone Marques</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="I229" s="1" t="inlineStr">
@@ -18756,7 +18812,7 @@
         </is>
       </c>
       <c r="J229" s="2" t="n">
-        <v>46111.45085925926</v>
+        <v>46111.43159019676</v>
       </c>
       <c r="K229" s="2" t="n">
         <v>46122</v>
@@ -18786,7 +18842,7 @@
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
-        <v>80038</v>
+        <v>78326</v>
       </c>
       <c r="B230" s="1" t="inlineStr">
         <is>
@@ -18795,30 +18851,30 @@
       </c>
       <c r="C230" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D230" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E230" s="1" t="inlineStr">
         <is>
-          <t>APURAÇÃO IRPJ E CSLL 2025</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F230" s="1" t="n">
-        <v>3661</v>
+        <v>3598</v>
       </c>
       <c r="G230" s="1" t="inlineStr">
         <is>
-          <t>BROGOTÁ INDÚSTRIA GRÁFICA LTDA</t>
+          <t>VTZZ INDUSTRIA E COMÉRCIO LTDA</t>
         </is>
       </c>
       <c r="H230" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Simone Marques</t>
         </is>
       </c>
       <c r="I230" s="1" t="inlineStr">
@@ -18827,10 +18883,10 @@
         </is>
       </c>
       <c r="J230" s="2" t="n">
-        <v>46188.55930297454</v>
+        <v>46111.45085925926</v>
       </c>
       <c r="K230" s="2" t="n">
-        <v>46190</v>
+        <v>46122</v>
       </c>
       <c r="L230" s="1" t="inlineStr">
         <is>
@@ -18839,7 +18895,7 @@
       </c>
       <c r="M230" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N230" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 20-07-26 1031
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U300" headerRowCount="1">
-  <autoFilter ref="A1:U300"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U299" headerRowCount="1">
+  <autoFilter ref="A1:U299"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U300"/>
+  <dimension ref="A1:U299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1993,7 +1993,11 @@
           <t>MQ PRODUSERV COMÉRCIO E EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H19" s="1" t="n"/>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -2007,7 +2011,7 @@
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M19" s="1" t="inlineStr">
@@ -2016,17 +2020,23 @@
         </is>
       </c>
       <c r="N19" s="1" t="n"/>
-      <c r="O19" s="1" t="n"/>
+      <c r="O19" s="2" t="n">
+        <v>46226</v>
+      </c>
       <c r="P19" s="1" t="n"/>
       <c r="Q19" s="1" t="inlineStr"/>
-      <c r="R19" s="1" t="n"/>
+      <c r="R19" s="1" t="inlineStr"/>
       <c r="S19" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T19" s="1" t="n"/>
-      <c r="U19" s="1" t="inlineStr"/>
+      <c r="U19" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -2461,7 +2471,11 @@
           <t xml:space="preserve">A.H.M.H. PARTICIPACOES S.A. </t>
         </is>
       </c>
-      <c r="H25" s="1" t="n"/>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL HOLDING</t>
@@ -2475,7 +2489,7 @@
       </c>
       <c r="L25" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M25" s="1" t="inlineStr">
@@ -2484,10 +2498,12 @@
         </is>
       </c>
       <c r="N25" s="1" t="n"/>
-      <c r="O25" s="1" t="n"/>
+      <c r="O25" s="2" t="n">
+        <v>46225</v>
+      </c>
       <c r="P25" s="1" t="n"/>
       <c r="Q25" s="1" t="inlineStr"/>
-      <c r="R25" s="1" t="n"/>
+      <c r="R25" s="1" t="inlineStr"/>
       <c r="S25" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -2528,7 +2544,11 @@
           <t>Adlpar Investimentos S.A.</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n"/>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL HOLDING</t>
@@ -2542,7 +2562,7 @@
       </c>
       <c r="L26" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M26" s="1" t="inlineStr">
@@ -2551,10 +2571,12 @@
         </is>
       </c>
       <c r="N26" s="1" t="n"/>
-      <c r="O26" s="1" t="n"/>
+      <c r="O26" s="2" t="n">
+        <v>46225</v>
+      </c>
       <c r="P26" s="1" t="n"/>
       <c r="Q26" s="1" t="inlineStr"/>
-      <c r="R26" s="1" t="n"/>
+      <c r="R26" s="1" t="inlineStr"/>
       <c r="S26" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -3507,7 +3529,11 @@
           <t>ESQUADRIAS SIDNEY LTDA</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n"/>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I38" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -3521,7 +3547,7 @@
       </c>
       <c r="L38" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M38" s="1" t="inlineStr">
@@ -3530,17 +3556,23 @@
         </is>
       </c>
       <c r="N38" s="1" t="n"/>
-      <c r="O38" s="1" t="n"/>
+      <c r="O38" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="P38" s="1" t="n"/>
       <c r="Q38" s="1" t="inlineStr"/>
-      <c r="R38" s="1" t="n"/>
+      <c r="R38" s="1" t="inlineStr"/>
       <c r="S38" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T38" s="1" t="n"/>
-      <c r="U38" s="1" t="inlineStr"/>
+      <c r="U38" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -4169,7 +4201,11 @@
           <t>DISTRIBUIDORA DE HORTIFRUTIGRANJEIROS 3 BBB LTDA  (MATRIZ)</t>
         </is>
       </c>
-      <c r="H46" s="1" t="n"/>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>Lucas Fischer</t>
+        </is>
+      </c>
       <c r="I46" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -4183,7 +4219,7 @@
       </c>
       <c r="L46" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M46" s="1" t="inlineStr">
@@ -4192,10 +4228,12 @@
         </is>
       </c>
       <c r="N46" s="1" t="n"/>
-      <c r="O46" s="1" t="n"/>
+      <c r="O46" s="2" t="n">
+        <v>46227</v>
+      </c>
       <c r="P46" s="1" t="n"/>
       <c r="Q46" s="1" t="inlineStr"/>
-      <c r="R46" s="1" t="n"/>
+      <c r="R46" s="1" t="inlineStr"/>
       <c r="S46" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -5309,7 +5347,11 @@
           <t>AF DATALINK CABOS, CONEXOES E SISTEMAS LTDA</t>
         </is>
       </c>
-      <c r="H60" s="1" t="n"/>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I60" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -5323,7 +5365,7 @@
       </c>
       <c r="L60" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M60" s="1" t="inlineStr">
@@ -5332,17 +5374,23 @@
         </is>
       </c>
       <c r="N60" s="1" t="n"/>
-      <c r="O60" s="1" t="n"/>
+      <c r="O60" s="2" t="n">
+        <v>46225</v>
+      </c>
       <c r="P60" s="1" t="n"/>
       <c r="Q60" s="1" t="inlineStr"/>
-      <c r="R60" s="1" t="n"/>
+      <c r="R60" s="1" t="inlineStr"/>
       <c r="S60" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T60" s="1" t="n"/>
-      <c r="U60" s="1" t="inlineStr"/>
+      <c r="U60" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -7501,7 +7549,11 @@
           <t>SAMPA ATACADO DE GENEROS ALIMENTICIOS E BEBIDAS LTDA</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n"/>
+      <c r="H87" s="1" t="inlineStr">
+        <is>
+          <t>Renata Cavalheiro</t>
+        </is>
+      </c>
       <c r="I87" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL VAREJO</t>
@@ -7515,7 +7567,7 @@
       </c>
       <c r="L87" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M87" s="1" t="inlineStr">
@@ -7525,12 +7577,22 @@
       </c>
       <c r="N87" s="1" t="n"/>
       <c r="O87" s="1" t="n"/>
-      <c r="P87" s="1" t="n"/>
-      <c r="Q87" s="1" t="inlineStr"/>
-      <c r="R87" s="1" t="n"/>
+      <c r="P87" s="2" t="n">
+        <v>46223.41618116898</v>
+      </c>
+      <c r="Q87" s="1" t="inlineStr">
+        <is>
+          <t>Renata Cavalheiro</t>
+        </is>
+      </c>
+      <c r="R87" s="1" t="inlineStr">
+        <is>
+          <t>Já foi enviado em 17/07/26.</t>
+        </is>
+      </c>
       <c r="S87" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T87" s="1" t="n"/>
@@ -10069,7 +10131,11 @@
           <t>T C DE CASTRO EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
-      <c r="H118" s="1" t="n"/>
+      <c r="H118" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I118" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -10083,7 +10149,7 @@
       </c>
       <c r="L118" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M118" s="1" t="inlineStr">
@@ -10092,17 +10158,23 @@
         </is>
       </c>
       <c r="N118" s="1" t="n"/>
-      <c r="O118" s="1" t="n"/>
+      <c r="O118" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="P118" s="1" t="n"/>
       <c r="Q118" s="1" t="inlineStr"/>
-      <c r="R118" s="1" t="n"/>
+      <c r="R118" s="1" t="inlineStr"/>
       <c r="S118" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T118" s="1" t="n"/>
-      <c r="U118" s="1" t="inlineStr"/>
+      <c r="U118" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -11232,7 +11304,11 @@
           <t xml:space="preserve">Parafutrecos Comercial LTDA </t>
         </is>
       </c>
-      <c r="H132" s="1" t="n"/>
+      <c r="H132" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I132" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -11246,7 +11322,7 @@
       </c>
       <c r="L132" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M132" s="1" t="inlineStr">
@@ -11255,17 +11331,23 @@
         </is>
       </c>
       <c r="N132" s="1" t="n"/>
-      <c r="O132" s="1" t="n"/>
+      <c r="O132" s="2" t="n">
+        <v>46224</v>
+      </c>
       <c r="P132" s="1" t="n"/>
       <c r="Q132" s="1" t="inlineStr"/>
-      <c r="R132" s="1" t="n"/>
+      <c r="R132" s="1" t="inlineStr"/>
       <c r="S132" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T132" s="1" t="n"/>
-      <c r="U132" s="1" t="inlineStr"/>
+      <c r="U132" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -14487,7 +14569,11 @@
           <t>CONCEITO LOCADORA LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H172" s="1" t="n"/>
+      <c r="H172" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I172" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -14501,7 +14587,7 @@
       </c>
       <c r="L172" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M172" s="1" t="inlineStr">
@@ -14510,17 +14596,23 @@
         </is>
       </c>
       <c r="N172" s="1" t="n"/>
-      <c r="O172" s="1" t="n"/>
+      <c r="O172" s="2" t="n">
+        <v>46225</v>
+      </c>
       <c r="P172" s="1" t="n"/>
       <c r="Q172" s="1" t="inlineStr"/>
-      <c r="R172" s="1" t="n"/>
+      <c r="R172" s="1" t="inlineStr"/>
       <c r="S172" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T172" s="1" t="n"/>
-      <c r="U172" s="1" t="inlineStr"/>
+      <c r="U172" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -21710,26 +21802,26 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>81172</v>
+        <v>77913</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C270" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D270" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Por gentileza, poderia realizar a baixa da terafa DEC 2 quinzena dos clientes abaixo?ISENTO3498	EMPLACA SERVIÇOS LTDA4327	ACCESS EVENTOS E VIAGENS LTDA5780	A Estancia Morro Grande Centro de R5873	FRRD ADMINISTRADORA DE IMOVEIS LTDA5906	A Estancia Morro Grande - Centro de5978	HLL LOCADORA DE GUINDASTES LTDA5979	AMATRUDA LOCADORA DE GUINDASTES E A6172	MEDICAL DISCOVERY TREINAMENTOS &amp; DE6173	CLINICA TONON DE DERMATOLOGISTA LTD6416	SINZATO ENTERTAINMENT LTDA6450	RDF VEICULOS LTDA6501	MD TREINAMENTOS E DESENVOLVIMENTO L6652	RAZEC EMPRESA DE APOIO ADMINISTRATI6766	MASTER IN THREADS CURSOS E EVENTOS6794	C.M.A EDUCACIONAL LTDA6796	COLÉGIO JOAQUIM MARIA MACHADO DE AS6798	LFJ TRANSPORTE LTDA6930	DOMENICO BIEMMI FRANCISCO LEITE6415	FABIO PEREIRA DA COSTAERRO DE BAIXA5084	REPUME REPUXAÇÃO E METALURGICA LTDA5292	EZEKY LTDA</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
@@ -21738,48 +21830,38 @@
       <c r="G270" s="1" t="n"/>
       <c r="H270" s="1" t="inlineStr">
         <is>
-          <t>Gabriel Amaral</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I270" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46220.38165829861</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46223</v>
+        <v>46097</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Larissa Félix</t>
         </is>
       </c>
       <c r="N270" s="1" t="n"/>
       <c r="O270" s="1" t="n"/>
-      <c r="P270" s="2" t="n">
-        <v>46220.46443684028</v>
-      </c>
-      <c r="Q270" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
-      <c r="R270" s="1" t="inlineStr">
-        <is>
-          <t>Tarefas baixadas</t>
-        </is>
-      </c>
+      <c r="P270" s="1" t="n"/>
+      <c r="Q270" s="1" t="inlineStr"/>
+      <c r="R270" s="1" t="inlineStr"/>
       <c r="S270" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T270" s="1" t="n"/>
@@ -21787,26 +21869,26 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>77913</v>
+        <v>79609</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
@@ -21815,7 +21897,7 @@
       <c r="G271" s="1" t="n"/>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
@@ -21824,10 +21906,10 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46097</v>
+        <v>46205</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21836,7 +21918,7 @@
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
@@ -21854,7 +21936,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>79609</v>
+        <v>80515</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
@@ -21863,7 +21945,7 @@
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
@@ -21873,7 +21955,7 @@
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -21882,7 +21964,7 @@
       <c r="G272" s="1" t="n"/>
       <c r="H272" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I272" s="1" t="inlineStr">
@@ -21891,26 +21973,32 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46205</v>
+        <v>46226</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
-        </is>
-      </c>
-      <c r="N272" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N272" s="2" t="n">
+        <v>46219.75157017361</v>
+      </c>
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
       <c r="Q272" s="1" t="inlineStr"/>
-      <c r="R272" s="1" t="inlineStr"/>
+      <c r="R272" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviado para registro </t>
+        </is>
+      </c>
       <c r="S272" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21921,7 +22009,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80515</v>
+        <v>80697</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -21930,7 +22018,7 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -21940,7 +22028,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -21949,7 +22037,7 @@
       <c r="G273" s="1" t="n"/>
       <c r="H273" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I273" s="1" t="inlineStr">
@@ -21958,14 +22046,14 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46226</v>
+        <v>46237</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
@@ -21973,17 +22061,11 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N273" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+      <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R273" s="1" t="inlineStr"/>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21994,7 +22076,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80697</v>
+        <v>80714</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22003,7 +22085,7 @@
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -22013,7 +22095,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22022,7 +22104,7 @@
       <c r="G274" s="1" t="n"/>
       <c r="H274" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I274" s="1" t="inlineStr">
@@ -22031,14 +22113,14 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M274" s="1" t="inlineStr">
@@ -22046,11 +22128,18 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N274" s="1" t="n"/>
+      <c r="N274" s="2" t="n">
+        <v>46223.41822326389</v>
+      </c>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="Q274" s="1" t="inlineStr"/>
-      <c r="R274" s="1" t="inlineStr"/>
+      <c r="R274" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+        </is>
+      </c>
       <c r="S274" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22061,16 +22150,16 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>80714</v>
+        <v>80919</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
@@ -22080,7 +22169,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22089,7 +22178,7 @@
       <c r="G275" s="1" t="n"/>
       <c r="H275" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I275" s="1" t="inlineStr">
@@ -22098,10 +22187,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22128,16 +22217,16 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>80919</v>
+        <v>80935</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
@@ -22147,7 +22236,7 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
@@ -22156,7 +22245,7 @@
       <c r="G276" s="1" t="n"/>
       <c r="H276" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I276" s="1" t="inlineStr">
@@ -22165,14 +22254,14 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
@@ -22180,11 +22269,18 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N276" s="1" t="n"/>
+      <c r="N276" s="2" t="n">
+        <v>46223.41869637732</v>
+      </c>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="inlineStr"/>
+      <c r="R276" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+        </is>
+      </c>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22195,7 +22291,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80935</v>
+        <v>80936</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22204,7 +22300,7 @@
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22214,7 +22310,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22223,7 +22319,7 @@
       <c r="G277" s="1" t="n"/>
       <c r="H277" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I277" s="1" t="inlineStr">
@@ -22232,14 +22328,14 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K277" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
@@ -22247,11 +22343,17 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N277" s="1" t="n"/>
+      <c r="N277" s="2" t="n">
+        <v>46220.45547311343</v>
+      </c>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
-      <c r="R277" s="1" t="inlineStr"/>
+      <c r="R277" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviado ao cliente</t>
+        </is>
+      </c>
       <c r="S277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22262,7 +22364,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80936</v>
+        <v>80951</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22271,7 +22373,7 @@
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22281,7 +22383,7 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22299,7 +22401,7 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K278" s="2" t="n">
         <v>46241</v>
@@ -22315,14 +22417,14 @@
         </is>
       </c>
       <c r="N278" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46219.74920023148</v>
       </c>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
       <c r="R278" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>Minuta enviada ao cliente</t>
         </is>
       </c>
       <c r="S278" s="1" t="inlineStr">
@@ -22335,26 +22437,26 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80951</v>
+        <v>80989</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22363,7 +22465,7 @@
       <c r="G279" s="1" t="n"/>
       <c r="H279" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I279" s="1" t="inlineStr">
@@ -22372,32 +22474,26 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46241</v>
+        <v>46217</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N279" s="2" t="n">
-        <v>46219.74920023148</v>
-      </c>
+          <t>João Oliveira</t>
+        </is>
+      </c>
+      <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="inlineStr">
-        <is>
-          <t>Minuta enviada ao cliente</t>
-        </is>
-      </c>
+      <c r="R279" s="1" t="inlineStr"/>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22408,35 +22504,39 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80989</v>
+        <v>79793</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G280" s="1" t="n"/>
+        <v>5655</v>
+      </c>
+      <c r="G280" s="1" t="inlineStr">
+        <is>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22445,10 +22545,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46217</v>
+        <v>46185</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22457,7 +22557,7 @@
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N280" s="1" t="n"/>
@@ -22475,34 +22575,34 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>79793</v>
+        <v>81004</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>5655</v>
+        <v>6869</v>
       </c>
       <c r="G281" s="1" t="inlineStr">
         <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H281" s="1" t="inlineStr">
@@ -22516,10 +22616,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22528,7 +22628,7 @@
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
@@ -22546,7 +22646,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>81004</v>
+        <v>81005</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
@@ -22569,16 +22669,16 @@
         </is>
       </c>
       <c r="F282" s="1" t="n">
-        <v>6869</v>
+        <v>6870</v>
       </c>
       <c r="G282" s="1" t="inlineStr">
         <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+          <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H282" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I282" s="1" t="inlineStr">
@@ -22587,7 +22687,7 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K282" s="2" t="n">
         <v>46218</v>
@@ -22617,39 +22717,39 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>81005</v>
+        <v>81091</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
-        <v>6870</v>
+        <v>6907</v>
       </c>
       <c r="G283" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H283" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I283" s="1" t="inlineStr">
@@ -22658,10 +22758,10 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46218</v>
+        <v>46223</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
@@ -22670,7 +22770,7 @@
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
@@ -22688,34 +22788,34 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>81091</v>
+        <v>79833</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
-        <v>6907</v>
+        <v>6125</v>
       </c>
       <c r="G284" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H284" s="1" t="inlineStr">
@@ -22725,30 +22825,36 @@
       </c>
       <c r="I284" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46223</v>
+        <v>46184</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
-        </is>
-      </c>
-      <c r="N284" s="1" t="n"/>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="N284" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
-      <c r="R284" s="1" t="inlineStr"/>
+      <c r="R284" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S284" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22759,7 +22865,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>79833</v>
+        <v>79834</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
@@ -22782,11 +22888,11 @@
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>6125</v>
+        <v>6162</v>
       </c>
       <c r="G285" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H285" s="1" t="inlineStr">
@@ -22800,14 +22906,14 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K285" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
@@ -22815,17 +22921,11 @@
           <t>Tatiana Linardi</t>
         </is>
       </c>
-      <c r="N285" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+      <c r="N285" s="1" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R285" s="1" t="inlineStr"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22836,16 +22936,16 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>79834</v>
+        <v>79865</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
@@ -22855,15 +22955,15 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6162</v>
+        <v>6278</v>
       </c>
       <c r="G286" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H286" s="1" t="inlineStr">
@@ -22877,10 +22977,10 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
@@ -22889,7 +22989,7 @@
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N286" s="1" t="n"/>
@@ -22907,7 +23007,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>79865</v>
+        <v>79854</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
@@ -22926,15 +23026,15 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6278</v>
+        <v>6302</v>
       </c>
       <c r="G287" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H287" s="1" t="inlineStr">
@@ -22948,10 +23048,10 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
@@ -22960,7 +23060,7 @@
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N287" s="1" t="n"/>
@@ -22978,7 +23078,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>79854</v>
+        <v>79863</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -22997,15 +23097,15 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>6302</v>
+        <v>6404</v>
       </c>
       <c r="G288" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H288" s="1" t="inlineStr">
@@ -23019,10 +23119,10 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -23031,7 +23131,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -23049,16 +23149,16 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>79863</v>
+        <v>79835</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C289" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D289" s="1" t="inlineStr">
@@ -23068,15 +23168,15 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>6404</v>
+        <v>6485</v>
       </c>
       <c r="G289" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H289" s="1" t="inlineStr">
@@ -23090,10 +23190,10 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
@@ -23102,7 +23202,7 @@
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
@@ -23120,16 +23220,16 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79835</v>
+        <v>79866</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
@@ -23139,15 +23239,15 @@
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6485</v>
+        <v>6539</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H290" s="1" t="inlineStr">
@@ -23161,10 +23261,10 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
@@ -23173,7 +23273,7 @@
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
@@ -23191,7 +23291,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>79866</v>
+        <v>79859</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
@@ -23210,15 +23310,15 @@
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6539</v>
+        <v>6570</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H291" s="1" t="inlineStr">
@@ -23232,7 +23332,7 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K291" s="2" t="n">
         <v>46185</v>
@@ -23262,7 +23362,7 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>79859</v>
+        <v>79860</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
@@ -23281,15 +23381,15 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6570</v>
+        <v>6581</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H292" s="1" t="inlineStr">
@@ -23303,7 +23403,7 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K292" s="2" t="n">
         <v>46185</v>
@@ -23333,7 +23433,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79860</v>
+        <v>79861</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
@@ -23352,15 +23452,15 @@
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6581</v>
+        <v>6583</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H293" s="1" t="inlineStr">
@@ -23374,7 +23474,7 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K293" s="2" t="n">
         <v>46185</v>
@@ -23404,16 +23504,16 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79861</v>
+        <v>79867</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
@@ -23423,15 +23523,15 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>6583</v>
+        <v>6704</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
@@ -23445,7 +23545,7 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>46185</v>
@@ -23475,16 +23575,16 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79867</v>
+        <v>79856</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
@@ -23494,15 +23594,15 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6704</v>
+        <v>4225</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
@@ -23516,10 +23616,10 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K295" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L295" s="1" t="inlineStr">
         <is>
@@ -23528,7 +23628,7 @@
       </c>
       <c r="M295" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N295" s="1" t="n"/>
@@ -23546,7 +23646,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>79856</v>
+        <v>79855</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23565,15 +23665,15 @@
       </c>
       <c r="E296" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>4225</v>
+        <v>4765</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
@@ -23587,10 +23687,10 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K296" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L296" s="1" t="inlineStr">
         <is>
@@ -23617,36 +23717,32 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79855</v>
+        <v>81019</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>4765</v>
-      </c>
-      <c r="G297" s="1" t="inlineStr">
-        <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G297" s="1" t="n"/>
       <c r="H297" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23658,26 +23754,31 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
       <c r="Q297" s="1" t="inlineStr"/>
-      <c r="R297" s="1" t="inlineStr"/>
+      <c r="R297" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
+        </is>
+      </c>
       <c r="S297" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23688,7 +23789,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>81019</v>
+        <v>81052</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23707,7 +23808,7 @@
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
@@ -23725,10 +23826,10 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
@@ -23737,7 +23838,7 @@
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
@@ -23746,8 +23847,7 @@
       <c r="Q298" s="1" t="inlineStr"/>
       <c r="R298" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S298" s="1" t="inlineStr">
@@ -23760,7 +23860,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>81052</v>
+        <v>81055</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
@@ -23779,7 +23879,7 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
@@ -23797,14 +23897,14 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K299" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M299" s="1" t="inlineStr">
@@ -23812,13 +23912,15 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N299" s="1" t="n"/>
+      <c r="N299" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
       <c r="Q299" s="1" t="inlineStr"/>
       <c r="R299" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t>Aguardando retorno dos dados do contador</t>
         </is>
       </c>
       <c r="S299" s="1" t="inlineStr">
@@ -23828,79 +23930,6 @@
       </c>
       <c r="T299" s="1" t="n"/>
       <c r="U299" s="1" t="inlineStr"/>
-    </row>
-    <row r="300">
-      <c r="A300" s="1" t="n">
-        <v>81055</v>
-      </c>
-      <c r="B300" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C300" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D300" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E300" s="1" t="inlineStr">
-        <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
-        </is>
-      </c>
-      <c r="F300" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G300" s="1" t="n"/>
-      <c r="H300" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I300" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J300" s="2" t="n">
-        <v>46218.40379614583</v>
-      </c>
-      <c r="K300" s="2" t="n">
-        <v>46219</v>
-      </c>
-      <c r="L300" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M300" s="1" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N300" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
-      <c r="O300" s="1" t="n"/>
-      <c r="P300" s="1" t="n"/>
-      <c r="Q300" s="1" t="inlineStr"/>
-      <c r="R300" s="1" t="inlineStr">
-        <is>
-          <t>Aguardando retorno dos dados do contador</t>
-        </is>
-      </c>
-      <c r="S300" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T300" s="1" t="n"/>
-      <c r="U300" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 20-07-26 1133
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -2317,7 +2317,7 @@
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="L23" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M23" s="1" t="inlineStr">
@@ -2343,12 +2343,23 @@
       </c>
       <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
-      <c r="P23" s="1" t="n"/>
-      <c r="Q23" s="1" t="inlineStr"/>
-      <c r="R23" s="1" t="inlineStr"/>
+      <c r="P23" s="2" t="n">
+        <v>46223.45704140046</v>
+      </c>
+      <c r="Q23" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R23" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EMPRESA NÃO É OPTANTE PELO SIMPLES NACIONAL, O CODIGO DA EMPRESA ESTÁ CORRETO ?
+</t>
+        </is>
+      </c>
       <c r="S23" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T23" s="1" t="n"/>
@@ -5108,7 +5119,11 @@
           <t>DONA LELLA INDÚSTRIA E COMÉRCIO DE PRODUTOS PARA CONFEITARIA LTDA</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n"/>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
       <c r="I57" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -5122,7 +5137,7 @@
       </c>
       <c r="L57" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M57" s="1" t="inlineStr">
@@ -5134,14 +5149,18 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="n"/>
       <c r="Q57" s="1" t="inlineStr"/>
-      <c r="R57" s="1" t="n"/>
+      <c r="R57" s="1" t="inlineStr"/>
       <c r="S57" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T57" s="1" t="n"/>
-      <c r="U57" s="1" t="inlineStr"/>
+      <c r="U57" s="1" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -5426,7 +5445,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I61" s="1" t="inlineStr">
@@ -5442,7 +5461,7 @@
       </c>
       <c r="L61" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M61" s="1" t="inlineStr">
@@ -5450,11 +5469,17 @@
           <t>Cristiane Simões</t>
         </is>
       </c>
-      <c r="N61" s="1" t="n"/>
+      <c r="N61" s="2" t="n">
+        <v>46223.47151377315</v>
+      </c>
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="n"/>
       <c r="Q61" s="1" t="inlineStr"/>
-      <c r="R61" s="1" t="inlineStr"/>
+      <c r="R61" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPERAÇÃO RECALCULANDO </t>
+        </is>
+      </c>
       <c r="S61" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -6163,7 +6188,11 @@
           <t>MIL ACESSORIOS E PRODUTOS PARA CONFEITARIA LTDA</t>
         </is>
       </c>
-      <c r="H70" s="1" t="n"/>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
       <c r="I70" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -6177,7 +6206,7 @@
       </c>
       <c r="L70" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M70" s="1" t="inlineStr">
@@ -6189,14 +6218,18 @@
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="n"/>
       <c r="Q70" s="1" t="inlineStr"/>
-      <c r="R70" s="1" t="n"/>
+      <c r="R70" s="1" t="inlineStr"/>
       <c r="S70" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T70" s="1" t="n"/>
-      <c r="U70" s="1" t="inlineStr"/>
+      <c r="U70" s="1" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -13037,7 +13070,7 @@
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I153" s="1" t="inlineStr">
@@ -13053,7 +13086,7 @@
       </c>
       <c r="L153" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M153" s="1" t="inlineStr">
@@ -13063,12 +13096,23 @@
       </c>
       <c r="N153" s="1" t="n"/>
       <c r="O153" s="1" t="n"/>
-      <c r="P153" s="1" t="n"/>
-      <c r="Q153" s="1" t="inlineStr"/>
-      <c r="R153" s="1" t="inlineStr"/>
+      <c r="P153" s="2" t="n">
+        <v>46223.46573961806</v>
+      </c>
+      <c r="Q153" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R153" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poderiam averiguar com o cliente para que ele pague a taxa ?
+No aguardo </t>
+        </is>
+      </c>
       <c r="S153" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T153" s="1" t="n"/>
@@ -13112,7 +13156,7 @@
       </c>
       <c r="H154" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I154" s="1" t="inlineStr">
@@ -13128,7 +13172,7 @@
       </c>
       <c r="L154" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M154" s="1" t="inlineStr">
@@ -13136,11 +13180,17 @@
           <t>Ana Santana</t>
         </is>
       </c>
-      <c r="N154" s="1" t="n"/>
+      <c r="N154" s="2" t="n">
+        <v>46223.45527280093</v>
+      </c>
       <c r="O154" s="1" t="n"/>
       <c r="P154" s="1" t="n"/>
       <c r="Q154" s="1" t="inlineStr"/>
-      <c r="R154" s="1" t="inlineStr"/>
+      <c r="R154" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EM ANALISE PELA OPERAÇÃO </t>
+        </is>
+      </c>
       <c r="S154" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -13187,7 +13237,7 @@
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I155" s="1" t="inlineStr">
@@ -13203,7 +13253,7 @@
       </c>
       <c r="L155" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M155" s="1" t="inlineStr">
@@ -13213,12 +13263,22 @@
       </c>
       <c r="N155" s="1" t="n"/>
       <c r="O155" s="1" t="n"/>
-      <c r="P155" s="1" t="n"/>
-      <c r="Q155" s="1" t="inlineStr"/>
-      <c r="R155" s="1" t="inlineStr"/>
+      <c r="P155" s="2" t="n">
+        <v>46223.46976207176</v>
+      </c>
+      <c r="Q155" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R155" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAOR, AVERIGUAR JUNTO AO CLIENTE O PAGAMENTO DA TAXA ANUAL </t>
+        </is>
+      </c>
       <c r="S155" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T155" s="1" t="n"/>
@@ -14332,7 +14392,7 @@
       </c>
       <c r="H169" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I169" s="1" t="inlineStr">
@@ -14348,7 +14408,7 @@
       </c>
       <c r="L169" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M169" s="1" t="inlineStr">
@@ -14358,12 +14418,22 @@
       </c>
       <c r="N169" s="1" t="n"/>
       <c r="O169" s="1" t="n"/>
-      <c r="P169" s="1" t="n"/>
-      <c r="Q169" s="1" t="inlineStr"/>
-      <c r="R169" s="1" t="inlineStr"/>
+      <c r="P169" s="2" t="n">
+        <v>46223.47283167824</v>
+      </c>
+      <c r="Q169" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R169" s="1" t="inlineStr">
+        <is>
+          <t>NÃO ENTENDI O CHAMADO</t>
+        </is>
+      </c>
       <c r="S169" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T169" s="1" t="n"/>
@@ -14496,7 +14566,7 @@
       </c>
       <c r="H171" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I171" s="1" t="inlineStr">
@@ -14512,7 +14582,7 @@
       </c>
       <c r="L171" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M171" s="1" t="inlineStr">
@@ -14522,12 +14592,23 @@
       </c>
       <c r="N171" s="1" t="n"/>
       <c r="O171" s="1" t="n"/>
-      <c r="P171" s="1" t="n"/>
-      <c r="Q171" s="1" t="inlineStr"/>
-      <c r="R171" s="1" t="inlineStr"/>
+      <c r="P171" s="2" t="n">
+        <v>46223.46101160879</v>
+      </c>
+      <c r="Q171" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
+      <c r="R171" s="1" t="inlineStr">
+        <is>
+          <t>BOM DIA, 
+JÁ SOLICITADO</t>
+        </is>
+      </c>
       <c r="S171" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T171" s="1" t="n"/>
@@ -14648,7 +14729,7 @@
       </c>
       <c r="H173" s="1" t="inlineStr">
         <is>
-          <t>Nayara Oliveira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="I173" s="1" t="inlineStr">
@@ -14664,7 +14745,7 @@
       </c>
       <c r="L173" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M173" s="1" t="inlineStr">
@@ -14672,11 +14753,17 @@
           <t>Vander Silva</t>
         </is>
       </c>
-      <c r="N173" s="1" t="n"/>
+      <c r="N173" s="2" t="n">
+        <v>46223.46244545139</v>
+      </c>
       <c r="O173" s="1" t="n"/>
       <c r="P173" s="1" t="n"/>
       <c r="Q173" s="1" t="inlineStr"/>
-      <c r="R173" s="1" t="inlineStr"/>
+      <c r="R173" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EM ATENDIMENTO PELA OPERAÇÃO </t>
+        </is>
+      </c>
       <c r="S173" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
data: atualização base chamados 20-07-26 1343
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U300" headerRowCount="1">
-  <autoFilter ref="A1:U300"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U302" headerRowCount="1">
+  <autoFilter ref="A1:U302"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U300"/>
+  <dimension ref="A1:U302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="L8" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M8" s="1" t="inlineStr">
@@ -1123,8 +1123,14 @@
       </c>
       <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
-      <c r="P8" s="1" t="n"/>
-      <c r="Q8" s="1" t="inlineStr"/>
+      <c r="P8" s="2" t="n">
+        <v>46223.53752623843</v>
+      </c>
+      <c r="Q8" s="1" t="inlineStr">
+        <is>
+          <t>Andrea Medeiros</t>
+        </is>
+      </c>
       <c r="R8" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">AGUARDANDO RETORNO DESDE 26/05/2026 - ANALISE ENVIADA VIA E-MAIL </t>
@@ -1132,7 +1138,7 @@
       </c>
       <c r="S8" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T8" s="1" t="n"/>
@@ -21875,26 +21881,26 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>77913</v>
+        <v>81210</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Forçar baixa de tarefas via banco de dados</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t xml:space="preserve">Boa tarde!Peço a gentileza de realizar a baixa na tarefa "GFD - FGTS Mensal" da empresa 2992 M CAVICHIOLLI, ref. a competencia 06/2026. A empresa em questão não tem guia emitida, apenas a da filial - Empresa 3204.Obrigado. </t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
@@ -21903,19 +21909,19 @@
       <c r="G269" s="1" t="n"/>
       <c r="H269" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I269" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46223.55477642361</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>46097</v>
+        <v>46223</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
@@ -21924,7 +21930,7 @@
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
+          <t>Vitor Guedes</t>
         </is>
       </c>
       <c r="N269" s="1" t="n"/>
@@ -21942,26 +21948,26 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>79609</v>
+        <v>81211</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C270" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Abertura de protocolo</t>
         </is>
       </c>
       <c r="D270" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>MG EXPRESS - GC</t>
         </is>
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Por favor, precisamos da baixa das tarefas pendentes referente tarefa "Fed - DAS" da competência 06/2026 com os arquivos disponíveis na pasta "\\finlandia\PUBLICA\RomeroBorges\Fed - DAS"</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
@@ -21970,19 +21976,19 @@
       <c r="G270" s="1" t="n"/>
       <c r="H270" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I270" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46223.56040540509</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46205</v>
+        <v>46224</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
@@ -21991,7 +21997,7 @@
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Romero Borges</t>
         </is>
       </c>
       <c r="N270" s="1" t="n"/>
@@ -22009,26 +22015,26 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>80515</v>
+        <v>77913</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
@@ -22037,7 +22043,7 @@
       <c r="G271" s="1" t="n"/>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
@@ -22046,32 +22052,26 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46226</v>
+        <v>46097</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N271" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N271" s="1" t="n"/>
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="Q271" s="1" t="inlineStr"/>
-      <c r="R271" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R271" s="1" t="inlineStr"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22082,7 +22082,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>80697</v>
+        <v>79609</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
@@ -22091,7 +22091,7 @@
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
@@ -22101,7 +22101,7 @@
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -22119,10 +22119,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46237</v>
+        <v>46205</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -22131,7 +22131,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -22149,7 +22149,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80714</v>
+        <v>80515</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22158,7 +22158,7 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -22177,7 +22177,7 @@
       <c r="G273" s="1" t="n"/>
       <c r="H273" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I273" s="1" t="inlineStr">
@@ -22186,10 +22186,10 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46241</v>
+        <v>46226</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
@@ -22202,15 +22202,14 @@
         </is>
       </c>
       <c r="N273" s="2" t="n">
-        <v>46223.41822326389</v>
+        <v>46219.75157017361</v>
       </c>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
       <c r="R273" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+          <t xml:space="preserve">Enviado para registro </t>
         </is>
       </c>
       <c r="S273" s="1" t="inlineStr">
@@ -22223,16 +22222,16 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80919</v>
+        <v>80697</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -22242,7 +22241,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22260,10 +22259,10 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
@@ -22290,7 +22289,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>80935</v>
+        <v>80714</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22299,7 +22298,7 @@
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
@@ -22309,7 +22308,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22327,7 +22326,7 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K275" s="2" t="n">
         <v>46241</v>
@@ -22343,15 +22342,15 @@
         </is>
       </c>
       <c r="N275" s="2" t="n">
-        <v>46223.41869637732</v>
+        <v>46223.41822326389</v>
       </c>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="Q275" s="1" t="inlineStr"/>
       <c r="R275" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
         </is>
       </c>
       <c r="S275" s="1" t="inlineStr">
@@ -22364,16 +22363,16 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>80936</v>
+        <v>80919</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
@@ -22383,7 +22382,7 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
@@ -22392,7 +22391,7 @@
       <c r="G276" s="1" t="n"/>
       <c r="H276" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I276" s="1" t="inlineStr">
@@ -22401,14 +22400,14 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
@@ -22416,17 +22415,11 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N276" s="2" t="n">
-        <v>46220.45547311343</v>
-      </c>
+      <c r="N276" s="1" t="n"/>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="inlineStr">
-        <is>
-          <t>Minuta enviado ao cliente</t>
-        </is>
-      </c>
+      <c r="R276" s="1" t="inlineStr"/>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22437,7 +22430,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80951</v>
+        <v>80935</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22456,7 +22449,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22465,7 +22458,7 @@
       <c r="G277" s="1" t="n"/>
       <c r="H277" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I277" s="1" t="inlineStr">
@@ -22474,7 +22467,7 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K277" s="2" t="n">
         <v>46241</v>
@@ -22490,14 +22483,15 @@
         </is>
       </c>
       <c r="N277" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46223.41869637732</v>
       </c>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
       <c r="R277" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
         </is>
       </c>
       <c r="S277" s="1" t="inlineStr">
@@ -22510,26 +22504,26 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80989</v>
+        <v>80936</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22538,7 +22532,7 @@
       <c r="G278" s="1" t="n"/>
       <c r="H278" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I278" s="1" t="inlineStr">
@@ -22547,10 +22541,10 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
@@ -22559,18 +22553,18 @@
       </c>
       <c r="M278" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N278" s="2" t="n">
-        <v>46223.4927846875</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
       <c r="R278" s="1" t="inlineStr">
         <is>
-          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S278" s="1" t="inlineStr">
@@ -22583,63 +22577,69 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>81208</v>
+        <v>80951</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião de Sócios</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Reeleição de Diretoria</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
-        <v>5449</v>
-      </c>
-      <c r="G279" s="1" t="inlineStr">
-        <is>
-          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
-        </is>
-      </c>
-      <c r="H279" s="1" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G279" s="1" t="n"/>
+      <c r="H279" s="1" t="inlineStr">
+        <is>
+          <t>Thifany Leite</t>
+        </is>
+      </c>
       <c r="I279" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46223.51713209491</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46225</v>
+        <v>46241</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
-        </is>
-      </c>
-      <c r="N279" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N279" s="2" t="n">
+        <v>46219.74920023148</v>
+      </c>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="n"/>
+      <c r="R279" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviada ao cliente</t>
+        </is>
+      </c>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22650,39 +22650,35 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>79793</v>
+        <v>80989</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G280" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22691,26 +22687,32 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46185</v>
+        <v>46217</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N280" s="1" t="n"/>
+          <t>João Oliveira</t>
+        </is>
+      </c>
+      <c r="N280" s="2" t="n">
+        <v>46223.4927846875</v>
+      </c>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
-      <c r="R280" s="1" t="inlineStr"/>
+      <c r="R280" s="1" t="inlineStr">
+        <is>
+          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
+        </is>
+      </c>
       <c r="S280" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22721,34 +22723,34 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>81209</v>
+        <v>81208</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Ata de Reunião de Sócios</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Reeleição de Diretoria</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>6094</v>
+        <v>5449</v>
       </c>
       <c r="G281" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
         </is>
       </c>
       <c r="H281" s="1" t="n"/>
@@ -22758,10 +22760,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46223.51713209491</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22770,7 +22772,7 @@
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
@@ -22788,34 +22790,34 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>81004</v>
+        <v>79793</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
-        <v>6869</v>
+        <v>5655</v>
       </c>
       <c r="G282" s="1" t="inlineStr">
         <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
+          <t>VANESSA DUARTE RODRIGUES</t>
         </is>
       </c>
       <c r="H282" s="1" t="inlineStr">
@@ -22829,10 +22831,10 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46218</v>
+        <v>46185</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
@@ -22841,7 +22843,7 @@
       </c>
       <c r="M282" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N282" s="1" t="n"/>
@@ -22859,67 +22861,63 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>81005</v>
+        <v>81209</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
-        <v>6870</v>
+        <v>6094</v>
       </c>
       <c r="G283" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
-        </is>
-      </c>
-      <c r="H283" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+        </is>
+      </c>
+      <c r="H283" s="1" t="n"/>
       <c r="I283" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46218</v>
+        <v>46224</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="inlineStr"/>
+      <c r="R283" s="1" t="n"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22930,34 +22928,34 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>81091</v>
+        <v>81004</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
-        <v>6907</v>
+        <v>6869</v>
       </c>
       <c r="G284" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H284" s="1" t="inlineStr">
@@ -22971,10 +22969,10 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46223</v>
+        <v>46218</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
@@ -22983,7 +22981,7 @@
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N284" s="1" t="n"/>
@@ -23001,73 +22999,67 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>79833</v>
+        <v>81005</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>6125</v>
+        <v>6870</v>
       </c>
       <c r="G285" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H285" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I285" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46184</v>
+        <v>46218</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N285" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+          <t>Lorrane Santos</t>
+        </is>
+      </c>
+      <c r="N285" s="1" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R285" s="1" t="inlineStr"/>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23078,34 +23070,34 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>79834</v>
+        <v>81091</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6162</v>
+        <v>6907</v>
       </c>
       <c r="G286" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H286" s="1" t="inlineStr">
@@ -23115,14 +23107,14 @@
       </c>
       <c r="I286" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46184</v>
+        <v>46223</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
@@ -23131,7 +23123,7 @@
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N286" s="1" t="n"/>
@@ -23149,16 +23141,16 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>79865</v>
+        <v>79833</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
@@ -23168,15 +23160,15 @@
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6278</v>
+        <v>6125</v>
       </c>
       <c r="G287" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H287" s="1" t="inlineStr">
@@ -23190,26 +23182,32 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
-        </is>
-      </c>
-      <c r="N287" s="1" t="n"/>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="N287" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O287" s="1" t="n"/>
       <c r="P287" s="1" t="n"/>
       <c r="Q287" s="1" t="inlineStr"/>
-      <c r="R287" s="1" t="inlineStr"/>
+      <c r="R287" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S287" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23220,16 +23218,16 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>79854</v>
+        <v>79834</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C288" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D288" s="1" t="inlineStr">
@@ -23239,15 +23237,15 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>6302</v>
+        <v>6162</v>
       </c>
       <c r="G288" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H288" s="1" t="inlineStr">
@@ -23261,7 +23259,7 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K288" s="2" t="n">
         <v>46184</v>
@@ -23291,7 +23289,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>79863</v>
+        <v>79865</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -23310,15 +23308,15 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>6404</v>
+        <v>6278</v>
       </c>
       <c r="G289" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H289" s="1" t="inlineStr">
@@ -23332,7 +23330,7 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K289" s="2" t="n">
         <v>46185</v>
@@ -23362,16 +23360,16 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79835</v>
+        <v>79854</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
@@ -23381,15 +23379,15 @@
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6485</v>
+        <v>6302</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H290" s="1" t="inlineStr">
@@ -23403,7 +23401,7 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K290" s="2" t="n">
         <v>46184</v>
@@ -23433,7 +23431,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>79866</v>
+        <v>79863</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
@@ -23452,15 +23450,15 @@
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6539</v>
+        <v>6404</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H291" s="1" t="inlineStr">
@@ -23474,7 +23472,7 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K291" s="2" t="n">
         <v>46185</v>
@@ -23504,16 +23502,16 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>79859</v>
+        <v>79835</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
@@ -23523,15 +23521,15 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6570</v>
+        <v>6485</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H292" s="1" t="inlineStr">
@@ -23545,10 +23543,10 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
@@ -23557,7 +23555,7 @@
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N292" s="1" t="n"/>
@@ -23575,7 +23573,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79860</v>
+        <v>79866</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
@@ -23594,15 +23592,15 @@
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6581</v>
+        <v>6539</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H293" s="1" t="inlineStr">
@@ -23616,7 +23614,7 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K293" s="2" t="n">
         <v>46185</v>
@@ -23646,7 +23644,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79861</v>
+        <v>79859</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
@@ -23665,15 +23663,15 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>6583</v>
+        <v>6570</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
@@ -23687,7 +23685,7 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>46185</v>
@@ -23717,16 +23715,16 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79867</v>
+        <v>79860</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
@@ -23736,15 +23734,15 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6704</v>
+        <v>6581</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
@@ -23758,7 +23756,7 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K295" s="2" t="n">
         <v>46185</v>
@@ -23788,7 +23786,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>79856</v>
+        <v>79861</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23807,15 +23805,15 @@
       </c>
       <c r="E296" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>4225</v>
+        <v>6583</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
@@ -23829,10 +23827,10 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K296" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L296" s="1" t="inlineStr">
         <is>
@@ -23841,7 +23839,7 @@
       </c>
       <c r="M296" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N296" s="1" t="n"/>
@@ -23859,16 +23857,16 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79855</v>
+        <v>79867</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
@@ -23878,15 +23876,15 @@
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>4765</v>
+        <v>6704</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H297" s="1" t="inlineStr">
@@ -23900,7 +23898,7 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K297" s="2" t="n">
         <v>46185</v>
@@ -23912,7 +23910,7 @@
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
@@ -23930,32 +23928,36 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>81019</v>
+        <v>79856</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C298" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D298" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G298" s="1" t="n"/>
+        <v>4225</v>
+      </c>
+      <c r="G298" s="1" t="inlineStr">
+        <is>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+        </is>
+      </c>
       <c r="H298" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23967,31 +23969,26 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46218</v>
+        <v>46184</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
       <c r="O298" s="1" t="n"/>
       <c r="P298" s="1" t="n"/>
       <c r="Q298" s="1" t="inlineStr"/>
-      <c r="R298" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
+      <c r="R298" s="1" t="inlineStr"/>
       <c r="S298" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24002,32 +23999,36 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>81052</v>
+        <v>79855</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C299" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D299" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G299" s="1" t="n"/>
+        <v>4765</v>
+      </c>
+      <c r="G299" s="1" t="inlineStr">
+        <is>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+        </is>
+      </c>
       <c r="H299" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -24039,30 +24040,26 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>46219</v>
+        <v>46185</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N299" s="1" t="n"/>
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
       <c r="Q299" s="1" t="inlineStr"/>
-      <c r="R299" s="1" t="inlineStr">
-        <is>
-          <t>cobramos os documentos do antigo contador.</t>
-        </is>
-      </c>
+      <c r="R299" s="1" t="inlineStr"/>
       <c r="S299" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24073,7 +24070,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>81055</v>
+        <v>81019</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
@@ -24092,7 +24089,7 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
@@ -24110,30 +24107,29 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M300" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N300" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N300" s="1" t="n"/>
       <c r="O300" s="1" t="n"/>
       <c r="P300" s="1" t="n"/>
       <c r="Q300" s="1" t="inlineStr"/>
       <c r="R300" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
         </is>
       </c>
       <c r="S300" s="1" t="inlineStr">
@@ -24143,6 +24139,150 @@
       </c>
       <c r="T300" s="1" t="n"/>
       <c r="U300" s="1" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="1" t="n">
+        <v>81052</v>
+      </c>
+      <c r="B301" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C301" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D301" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E301" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+        </is>
+      </c>
+      <c r="F301" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" s="1" t="n"/>
+      <c r="H301" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I301" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="n">
+        <v>46218.38736744213</v>
+      </c>
+      <c r="K301" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L301" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido para Responsável</t>
+        </is>
+      </c>
+      <c r="M301" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N301" s="1" t="n"/>
+      <c r="O301" s="1" t="n"/>
+      <c r="P301" s="1" t="n"/>
+      <c r="Q301" s="1" t="inlineStr"/>
+      <c r="R301" s="1" t="inlineStr">
+        <is>
+          <t>cobramos os documentos do antigo contador.</t>
+        </is>
+      </c>
+      <c r="S301" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T301" s="1" t="n"/>
+      <c r="U301" s="1" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="1" t="n">
+        <v>81055</v>
+      </c>
+      <c r="B302" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C302" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D302" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E302" s="1" t="inlineStr">
+        <is>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+        </is>
+      </c>
+      <c r="F302" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G302" s="1" t="n"/>
+      <c r="H302" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I302" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="n">
+        <v>46218.40379614583</v>
+      </c>
+      <c r="K302" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L302" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M302" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N302" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
+      <c r="O302" s="1" t="n"/>
+      <c r="P302" s="1" t="n"/>
+      <c r="Q302" s="1" t="inlineStr"/>
+      <c r="R302" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
+      <c r="S302" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T302" s="1" t="n"/>
+      <c r="U302" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 20-07-26 1613
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -22138,7 +22138,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>81211</v>
+        <v>81224</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22147,54 +22147,50 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Abertura de protocolo</t>
+          <t>Baixa automática - Arquivos</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
         <is>
-          <t>MG EXPRESS - GC</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Por favor, precisamos da baixa das tarefas pendentes referente tarefa "Fed - DAS" da competência 06/2026 com os arquivos disponíveis na pasta "\\finlandia\PUBLICA\RomeroBorges\Fed - DAS"</t>
+          <t xml:space="preserve">boa tarde por gentileza, poderia esta baixando os sped icms sem movimento, pois não estou conseguindo da baixa devido a estagio 06 , pois a loja não vem sped icms </t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G273" s="1" t="n"/>
-      <c r="H273" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H273" s="1" t="n"/>
       <c r="I273" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46223.56040540509</v>
+        <v>46223.67153248843</v>
       </c>
       <c r="K273" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Romero Borges</t>
+          <t>Vanessa Tavares</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="inlineStr"/>
+      <c r="R273" s="1" t="n"/>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22205,7 +22201,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>81221</v>
+        <v>81223</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22219,45 +22215,53 @@
       </c>
       <c r="D274" s="1" t="inlineStr">
         <is>
-          <t>RJ - GC ADMINISTRATIVO</t>
+          <t>DALBEN - CTB</t>
         </is>
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezados, boa tarde!Solicito que seja realizada baixa das empresas referente a tarefa de DEC 2 quinzena de julho - 4120 - 4124 - 4183 - 4503 - 4504 - 4505 - 5700 (sem certificado no dinamo e não temos acesso ao fisco.)6958 - 6982 (empresas isentas ) </t>
+          <t>Boa tarde!Na baixa da tarefa do REINF, todo o grupo Dalben está dando erro de layout.Arquivos para baixa estão salvos na pasta publica/Dalben</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G274" s="1" t="n"/>
-      <c r="H274" s="1" t="n"/>
+        <v>3212</v>
+      </c>
+      <c r="G274" s="1" t="inlineStr">
+        <is>
+          <t>SUPERMERCADOS DALBEN LTDA. (MATRIZ)</t>
+        </is>
+      </c>
+      <c r="H274" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I274" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46223.65060582176</v>
+        <v>46223.65859783565</v>
       </c>
       <c r="K274" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>Amanda Mesquita</t>
+          <t>Karen Corazza</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="Q274" s="1" t="inlineStr"/>
-      <c r="R274" s="1" t="n"/>
+      <c r="R274" s="1" t="inlineStr"/>
       <c r="S274" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
data: atualização base chamados 21-07-26 0904
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -20826,67 +20826,63 @@
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
-        <v>78305</v>
+        <v>81235</v>
       </c>
       <c r="B255" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C255" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D255" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="E255" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>Não localizei o certificado do empresa 5725 no meu Dinamo por favor disponibilizar.</t>
         </is>
       </c>
       <c r="F255" s="1" t="n">
-        <v>5744</v>
+        <v>5725</v>
       </c>
       <c r="G255" s="1" t="inlineStr">
         <is>
-          <t>ATC LOCAÇÃO E COMÉRCIO LTDA</t>
-        </is>
-      </c>
-      <c r="H255" s="1" t="inlineStr">
-        <is>
-          <t>Beatriz Rangel</t>
-        </is>
-      </c>
+          <t>ELFUTEC - ESCOLA PARA FORMACAO DE USUARIOS DE TECNOLOGIA E CONHECIMENTO LTDA</t>
+        </is>
+      </c>
+      <c r="H255" s="1" t="n"/>
       <c r="I255" s="1" t="inlineStr">
         <is>
           <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J255" s="2" t="n">
-        <v>46111.42608159722</v>
+        <v>46223.83941327546</v>
       </c>
       <c r="K255" s="2" t="n">
-        <v>46122</v>
+        <v>46225</v>
       </c>
       <c r="L255" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M255" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
+          <t>Erika Santana</t>
         </is>
       </c>
       <c r="N255" s="1" t="n"/>
       <c r="O255" s="1" t="n"/>
       <c r="P255" s="1" t="n"/>
       <c r="Q255" s="1" t="inlineStr"/>
-      <c r="R255" s="1" t="inlineStr"/>
+      <c r="R255" s="1" t="n"/>
       <c r="S255" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -20897,7 +20893,7 @@
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
-        <v>78318</v>
+        <v>78305</v>
       </c>
       <c r="B256" s="1" t="inlineStr">
         <is>
@@ -20920,11 +20916,11 @@
         </is>
       </c>
       <c r="F256" s="1" t="n">
-        <v>5801</v>
+        <v>5744</v>
       </c>
       <c r="G256" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nilcap Renovadora de Pneus LTDA </t>
+          <t>ATC LOCAÇÃO E COMÉRCIO LTDA</t>
         </is>
       </c>
       <c r="H256" s="1" t="inlineStr">
@@ -20938,7 +20934,7 @@
         </is>
       </c>
       <c r="J256" s="2" t="n">
-        <v>46111.44276319444</v>
+        <v>46111.42608159722</v>
       </c>
       <c r="K256" s="2" t="n">
         <v>46122</v>
@@ -20968,7 +20964,7 @@
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
-        <v>78311</v>
+        <v>78318</v>
       </c>
       <c r="B257" s="1" t="inlineStr">
         <is>
@@ -20991,11 +20987,11 @@
         </is>
       </c>
       <c r="F257" s="1" t="n">
-        <v>5803</v>
+        <v>5801</v>
       </c>
       <c r="G257" s="1" t="inlineStr">
         <is>
-          <t>Ink Flex Industria Grafica LTDA</t>
+          <t xml:space="preserve">Nilcap Renovadora de Pneus LTDA </t>
         </is>
       </c>
       <c r="H257" s="1" t="inlineStr">
@@ -21009,7 +21005,7 @@
         </is>
       </c>
       <c r="J257" s="2" t="n">
-        <v>46111.43436825232</v>
+        <v>46111.44276319444</v>
       </c>
       <c r="K257" s="2" t="n">
         <v>46122</v>
@@ -21039,7 +21035,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>78301</v>
+        <v>78311</v>
       </c>
       <c r="B258" s="1" t="inlineStr">
         <is>
@@ -21062,16 +21058,16 @@
         </is>
       </c>
       <c r="F258" s="1" t="n">
-        <v>6016</v>
+        <v>5803</v>
       </c>
       <c r="G258" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALUMINIO IMPERIAL LTDA </t>
+          <t>Ink Flex Industria Grafica LTDA</t>
         </is>
       </c>
       <c r="H258" s="1" t="inlineStr">
         <is>
-          <t>Simone Marques</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I258" s="1" t="inlineStr">
@@ -21080,7 +21076,7 @@
         </is>
       </c>
       <c r="J258" s="2" t="n">
-        <v>46111.42218321759</v>
+        <v>46111.43436825232</v>
       </c>
       <c r="K258" s="2" t="n">
         <v>46122</v>
@@ -21110,7 +21106,7 @@
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
-        <v>79830</v>
+        <v>78301</v>
       </c>
       <c r="B259" s="1" t="inlineStr">
         <is>
@@ -21124,25 +21120,25 @@
       </c>
       <c r="D259" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E259" s="1" t="inlineStr">
         <is>
-          <t>O cliente 6068-R.T. CARVALHO Aluguel de Imóveis enviou os recibos anexos correspondentes a receita com aluguéis durante o exercício 2025.No sistema de análise consta movimentação somente nos meses de outubro e novembro 2025, precisamos de um retorno de como tratar.</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F259" s="1" t="n">
-        <v>6068</v>
+        <v>6016</v>
       </c>
       <c r="G259" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">R.T CARVALHO ALUGUEL DE IMOVEIS PROPRIOS LTDA </t>
+          <t xml:space="preserve">ALUMINIO IMPERIAL LTDA </t>
         </is>
       </c>
       <c r="H259" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
+          <t>Simone Marques</t>
         </is>
       </c>
       <c r="I259" s="1" t="inlineStr">
@@ -21151,10 +21147,10 @@
         </is>
       </c>
       <c r="J259" s="2" t="n">
-        <v>46183.45075188657</v>
+        <v>46111.42218321759</v>
       </c>
       <c r="K259" s="2" t="n">
-        <v>46184</v>
+        <v>46122</v>
       </c>
       <c r="L259" s="1" t="inlineStr">
         <is>
@@ -21163,7 +21159,7 @@
       </c>
       <c r="M259" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N259" s="1" t="n"/>
@@ -21181,7 +21177,7 @@
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
-        <v>78321</v>
+        <v>79830</v>
       </c>
       <c r="B260" s="1" t="inlineStr">
         <is>
@@ -21195,25 +21191,25 @@
       </c>
       <c r="D260" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E260" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>O cliente 6068-R.T. CARVALHO Aluguel de Imóveis enviou os recibos anexos correspondentes a receita com aluguéis durante o exercício 2025.No sistema de análise consta movimentação somente nos meses de outubro e novembro 2025, precisamos de um retorno de como tratar.</t>
         </is>
       </c>
       <c r="F260" s="1" t="n">
-        <v>6088</v>
+        <v>6068</v>
       </c>
       <c r="G260" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SINZATO INDUSTRIA E COMERCIO DE CONFECCOES LTDA </t>
+          <t xml:space="preserve">R.T CARVALHO ALUGUEL DE IMOVEIS PROPRIOS LTDA </t>
         </is>
       </c>
       <c r="H260" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="I260" s="1" t="inlineStr">
@@ -21222,17 +21218,21 @@
         </is>
       </c>
       <c r="J260" s="2" t="n">
-        <v>46111.44696084491</v>
+        <v>46183.45075188657</v>
       </c>
       <c r="K260" s="2" t="n">
-        <v>46122</v>
+        <v>46184</v>
       </c>
       <c r="L260" s="1" t="inlineStr">
         <is>
           <t>Esperando Atendimento</t>
         </is>
       </c>
-      <c r="M260" s="1" t="n"/>
+      <c r="M260" s="1" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
       <c r="N260" s="1" t="n"/>
       <c r="O260" s="1" t="n"/>
       <c r="P260" s="1" t="n"/>
@@ -21248,7 +21248,7 @@
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
-        <v>78798</v>
+        <v>78321</v>
       </c>
       <c r="B261" s="1" t="inlineStr">
         <is>
@@ -21267,15 +21267,15 @@
       </c>
       <c r="E261" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">por favor, orientar o cliente sobre a classificação das notas de entrada, por diversas vezes já falamos junto ao cliente sobre essa classificação. exemplo: coroa de flores - classificou como insumo / saco de lixo e copo descartavel - classificou como insumo. No aguardo </t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F261" s="1" t="n">
-        <v>6106</v>
+        <v>6088</v>
       </c>
       <c r="G261" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLANET GRAPHICS LTDA </t>
+          <t xml:space="preserve">SINZATO INDUSTRIA E COMERCIO DE CONFECCOES LTDA </t>
         </is>
       </c>
       <c r="H261" s="1" t="inlineStr">
@@ -21289,21 +21289,17 @@
         </is>
       </c>
       <c r="J261" s="2" t="n">
-        <v>46128.70572581018</v>
+        <v>46111.44696084491</v>
       </c>
       <c r="K261" s="2" t="n">
-        <v>46132</v>
+        <v>46122</v>
       </c>
       <c r="L261" s="1" t="inlineStr">
         <is>
           <t>Esperando Atendimento</t>
         </is>
       </c>
-      <c r="M261" s="1" t="inlineStr">
-        <is>
-          <t>Priscila Volpe</t>
-        </is>
-      </c>
+      <c r="M261" s="1" t="n"/>
       <c r="N261" s="1" t="n"/>
       <c r="O261" s="1" t="n"/>
       <c r="P261" s="1" t="n"/>
@@ -21319,39 +21315,39 @@
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
-        <v>81124</v>
+        <v>78798</v>
       </c>
       <c r="B262" s="1" t="inlineStr">
         <is>
-          <t>Certificado</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C262" s="1" t="inlineStr">
         <is>
-          <t>Certificado digital</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D262" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E262" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia! Por gentileza, atualizar certificado no DINAMO e GAX - colocar na minha árvore. </t>
+          <t xml:space="preserve">por favor, orientar o cliente sobre a classificação das notas de entrada, por diversas vezes já falamos junto ao cliente sobre essa classificação. exemplo: coroa de flores - classificou como insumo / saco de lixo e copo descartavel - classificou como insumo. No aguardo </t>
         </is>
       </c>
       <c r="F262" s="1" t="n">
-        <v>6112</v>
+        <v>6106</v>
       </c>
       <c r="G262" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">MONTE CARLO LAB SERVICOS ADMINISTRATIVOS E COMERCIO LTDA </t>
+          <t xml:space="preserve">PLANET GRAPHICS LTDA </t>
         </is>
       </c>
       <c r="H262" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I262" s="1" t="inlineStr">
@@ -21360,10 +21356,10 @@
         </is>
       </c>
       <c r="J262" s="2" t="n">
-        <v>46219.49444649305</v>
+        <v>46128.70572581018</v>
       </c>
       <c r="K262" s="2" t="n">
-        <v>46220</v>
+        <v>46132</v>
       </c>
       <c r="L262" s="1" t="inlineStr">
         <is>
@@ -21372,7 +21368,7 @@
       </c>
       <c r="M262" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="N262" s="1" t="n"/>
@@ -21390,39 +21386,39 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>79837</v>
+        <v>81124</v>
       </c>
       <c r="B263" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Certificado</t>
         </is>
       </c>
       <c r="C263" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Certificado digital</t>
         </is>
       </c>
       <c r="D263" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E263" s="1" t="inlineStr">
         <is>
-          <t>Segue empresas que não possuem estoque suficiente para bater a lucratividade.6125	Piquini Comercio de Materiais Para Construção LTDA - Matriz 	Casa Glória	02.494.541/0001-49	Bruno	Estoque insuficiente desde 03/2025</t>
+          <t xml:space="preserve">Bom dia! Por gentileza, atualizar certificado no DINAMO e GAX - colocar na minha árvore. </t>
         </is>
       </c>
       <c r="F263" s="1" t="n">
-        <v>6125</v>
+        <v>6112</v>
       </c>
       <c r="G263" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t xml:space="preserve">MONTE CARLO LAB SERVICOS ADMINISTRATIVOS E COMERCIO LTDA </t>
         </is>
       </c>
       <c r="H263" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="I263" s="1" t="inlineStr">
@@ -21431,10 +21427,10 @@
         </is>
       </c>
       <c r="J263" s="2" t="n">
-        <v>46183.47519135417</v>
+        <v>46219.49444649305</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>46184</v>
+        <v>46220</v>
       </c>
       <c r="L263" s="1" t="inlineStr">
         <is>
@@ -21443,7 +21439,7 @@
       </c>
       <c r="M263" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N263" s="1" t="n"/>
@@ -21461,7 +21457,7 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>78325</v>
+        <v>79837</v>
       </c>
       <c r="B264" s="1" t="inlineStr">
         <is>
@@ -21475,25 +21471,25 @@
       </c>
       <c r="D264" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E264" s="1" t="inlineStr">
         <is>
-          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
+          <t>Segue empresas que não possuem estoque suficiente para bater a lucratividade.6125	Piquini Comercio de Materiais Para Construção LTDA - Matriz 	Casa Glória	02.494.541/0001-49	Bruno	Estoque insuficiente desde 03/2025</t>
         </is>
       </c>
       <c r="F264" s="1" t="n">
-        <v>6148</v>
+        <v>6125</v>
       </c>
       <c r="G264" s="1" t="inlineStr">
         <is>
-          <t>VALE CONCRETO LTDA</t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H264" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="I264" s="1" t="inlineStr">
@@ -21502,10 +21498,10 @@
         </is>
       </c>
       <c r="J264" s="2" t="n">
-        <v>46111.45013549768</v>
+        <v>46183.47519135417</v>
       </c>
       <c r="K264" s="2" t="n">
-        <v>46122</v>
+        <v>46184</v>
       </c>
       <c r="L264" s="1" t="inlineStr">
         <is>
@@ -21514,7 +21510,7 @@
       </c>
       <c r="M264" s="1" t="inlineStr">
         <is>
-          <t>Taina Silva</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N264" s="1" t="n"/>
@@ -21532,7 +21528,7 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>78324</v>
+        <v>78325</v>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
@@ -21555,16 +21551,16 @@
         </is>
       </c>
       <c r="F265" s="1" t="n">
-        <v>6261</v>
+        <v>6148</v>
       </c>
       <c r="G265" s="1" t="inlineStr">
         <is>
-          <t>V8 INDUSTRIA E COMERCIO DE PRODUTOS ABRASIVOS LTDA</t>
+          <t>VALE CONCRETO LTDA</t>
         </is>
       </c>
       <c r="H265" s="1" t="inlineStr">
         <is>
-          <t>Simone Marques</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I265" s="1" t="inlineStr">
@@ -21573,7 +21569,7 @@
         </is>
       </c>
       <c r="J265" s="2" t="n">
-        <v>46111.44946597222</v>
+        <v>46111.45013549768</v>
       </c>
       <c r="K265" s="2" t="n">
         <v>46122</v>
@@ -21603,7 +21599,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>78317</v>
+        <v>78324</v>
       </c>
       <c r="B266" s="1" t="inlineStr">
         <is>
@@ -21626,16 +21622,16 @@
         </is>
       </c>
       <c r="F266" s="1" t="n">
-        <v>6288</v>
+        <v>6261</v>
       </c>
       <c r="G266" s="1" t="inlineStr">
         <is>
-          <t>NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (FILIAL 2)</t>
+          <t>V8 INDUSTRIA E COMERCIO DE PRODUTOS ABRASIVOS LTDA</t>
         </is>
       </c>
       <c r="H266" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Simone Marques</t>
         </is>
       </c>
       <c r="I266" s="1" t="inlineStr">
@@ -21644,7 +21640,7 @@
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>46111.44151450232</v>
+        <v>46111.44946597222</v>
       </c>
       <c r="K266" s="2" t="n">
         <v>46122</v>
@@ -21674,7 +21670,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>78289</v>
+        <v>78317</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
@@ -21697,11 +21693,11 @@
         </is>
       </c>
       <c r="F267" s="1" t="n">
-        <v>6289</v>
+        <v>6288</v>
       </c>
       <c r="G267" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (FILIAL 3)</t>
+          <t>NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (FILIAL 2)</t>
         </is>
       </c>
       <c r="H267" s="1" t="inlineStr">
@@ -21715,7 +21711,7 @@
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46111.41423260417</v>
+        <v>46111.44151450232</v>
       </c>
       <c r="K267" s="2" t="n">
         <v>46122</v>
@@ -21745,39 +21741,39 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>81011</v>
+        <v>78289</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de ata de reunião</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>NCM - consultar a tributação do NCM 87116000 - enviar para o cliente!</t>
+          <t>O cliente em questão precisa nos enviar o controle de estoque - bloco K - Sendo assim, precisamos trabalhar juntos nesse quesito para nos respaldarmos em possíveis fiscalização e/ou intimação. Obrigatoriedade de entrega do Bloco K (Livro Registro de Controle da Produção e do Estoque):Obrigados:Empresas industriais ou equiparadas a industrial, enquadradas como:Estabelecimentos industriais dos seguintes CNAEs (de acordo com a Tabela de CNAEs da Receita Federal):Especialmente empresas do Lucro Real ou Lucro Presumido;Principalmente as dos setores de bebidas, alimentos, automotivo, metalurgia, químico, entre outros.Estabelecimentos atacadistas de determinados setores (obrigatoriedade progressiva, dependendo do CNAE e faturamento);Empresas com faturamento anual superior a R$ 300 milhões, conforme escalonamento determinado pelo Ajuste SINIEF 02/2009 e suas alterações.Empresas do Simples Nacional geralmente estão dispensadas, mas é sempre bom verificar legislações estaduais.? Observações importantes: A obrigatoriedade varia conforme o Estado, pois alguns exigem mais informações ou já anteciparam prazos.O Bloco K exige detalhamento mensal de:Insumos consumidos, Produção realizada, Estoque inicial e final,Terceirizações (envio e recebimento de industrialização). Em anexo a planilha modelo que deverá ser preenchida.</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
-        <v>6399</v>
+        <v>6289</v>
       </c>
       <c r="G268" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIQUIM E-BIKE LTDA </t>
+          <t xml:space="preserve"> NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (FILIAL 3)</t>
         </is>
       </c>
       <c r="H268" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="I268" s="1" t="inlineStr">
@@ -21786,10 +21782,10 @@
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46217.3885827199</v>
+        <v>46111.41423260417</v>
       </c>
       <c r="K268" s="2" t="n">
-        <v>46223</v>
+        <v>46122</v>
       </c>
       <c r="L268" s="1" t="inlineStr">
         <is>
@@ -21798,7 +21794,7 @@
       </c>
       <c r="M268" s="1" t="inlineStr">
         <is>
-          <t>Clara Maria</t>
+          <t>Taina Silva</t>
         </is>
       </c>
       <c r="N268" s="1" t="n"/>
@@ -21816,39 +21812,39 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>81112</v>
+        <v>81011</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
-          <t>Apontamentos</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Inclusão de ata de reunião</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!6499 - DFGAssunto: Cobrança do Sindicato ( SECABC) - Assistencial 2025Segue o e-mail encaminhado ao cliente.O sindicato voltou a cobrar as contribuições do período de 2025, eles me ligaram ontem e estou te encaminhando em anexo o e-mail que eles nos enviaram, e estão cobrando uma resposta, segue em anexo também a relação da cobrança.Por telefone eles estão ameaçando entrar com medidas legais e denúncia no MTE.O cliente informou que não vai realizar o pagamento, pois a contabilidade anterior informou que não era necessário realizar o recolhimento da contribuição Assistencial dos colaboradores. Por favor, abordar esse assunto na reunião, aguardo retorno.</t>
+          <t>NCM - consultar a tributação do NCM 87116000 - enviar para o cliente!</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
-        <v>6499</v>
+        <v>6399</v>
       </c>
       <c r="G269" s="1" t="inlineStr">
         <is>
-          <t>DFG COMERCIO IMPORTACAO, EXPORTACAO E REPRESENTACAO LTDA</t>
+          <t xml:space="preserve">LIQUIM E-BIKE LTDA </t>
         </is>
       </c>
       <c r="H269" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="I269" s="1" t="inlineStr">
@@ -21857,10 +21853,10 @@
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46219.48029166667</v>
+        <v>46217.3885827199</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
@@ -21869,7 +21865,7 @@
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>Edivaldo Veiga</t>
+          <t>Clara Maria</t>
         </is>
       </c>
       <c r="N269" s="1" t="n"/>
@@ -21887,7 +21883,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>77557</v>
+        <v>81112</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
@@ -21901,25 +21897,25 @@
       </c>
       <c r="D270" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>A loja 6640 é de São Paulo, porém, a Matriz é de Belém, precisa alinhar quais documentos ele precisam que a gente mande, esse mes solicitaram o SPED, calculo do DIFAL e Calculo do laudo de combustivel (não recebi nenhuma informação). Questionaram também se será considerada a nossa apuação ou a do sistema, porq a nossa deu diferença em "Outras " do ICMS e querem tudo batido igual o deles.Sobre a 6639 é uma transportadora, não recebemos SPED e não encontrei onde extrair no sistema que deram acesso, será sempre montagem aqui? Lançamos tbm o credito outorgado (20%), vimos que foi feito assim no mes anterior com o antigo contador.</t>
+          <t>Bom dia!6499 - DFGAssunto: Cobrança do Sindicato ( SECABC) - Assistencial 2025Segue o e-mail encaminhado ao cliente.O sindicato voltou a cobrar as contribuições do período de 2025, eles me ligaram ontem e estou te encaminhando em anexo o e-mail que eles nos enviaram, e estão cobrando uma resposta, segue em anexo também a relação da cobrança.Por telefone eles estão ameaçando entrar com medidas legais e denúncia no MTE.O cliente informou que não vai realizar o pagamento, pois a contabilidade anterior informou que não era necessário realizar o recolhimento da contribuição Assistencial dos colaboradores. Por favor, abordar esse assunto na reunião, aguardo retorno.</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
-        <v>6640</v>
+        <v>6499</v>
       </c>
       <c r="G270" s="1" t="inlineStr">
         <is>
-          <t>FORT FRUIT LTDA</t>
+          <t>DFG COMERCIO IMPORTACAO, EXPORTACAO E REPRESENTACAO LTDA</t>
         </is>
       </c>
       <c r="H270" s="1" t="inlineStr">
         <is>
-          <t>Bruno Contieri</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="I270" s="1" t="inlineStr">
@@ -21928,10 +21924,10 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46079.72002283565</v>
+        <v>46219.48029166667</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46079</v>
+        <v>46220</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
@@ -21940,7 +21936,7 @@
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Thaiza Oliveira</t>
+          <t>Edivaldo Veiga</t>
         </is>
       </c>
       <c r="N270" s="1" t="n"/>
@@ -21958,76 +21954,70 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>80165</v>
+        <v>77557</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Apontamentos</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>A loja 6640 é de São Paulo, porém, a Matriz é de Belém, precisa alinhar quais documentos ele precisam que a gente mande, esse mes solicitaram o SPED, calculo do DIFAL e Calculo do laudo de combustivel (não recebi nenhuma informação). Questionaram também se será considerada a nossa apuação ou a do sistema, porq a nossa deu diferença em "Outras " do ICMS e querem tudo batido igual o deles.Sobre a 6639 é uma transportadora, não recebemos SPED e não encontrei onde extrair no sistema que deram acesso, será sempre montagem aqui? Lançamos tbm o credito outorgado (20%), vimos que foi feito assim no mes anterior com o antigo contador.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G271" s="1" t="n"/>
+        <v>6640</v>
+      </c>
+      <c r="G271" s="1" t="inlineStr">
+        <is>
+          <t>FORT FRUIT LTDA</t>
+        </is>
+      </c>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Gabriel Amaral</t>
+          <t>Bruno Contieri</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46190.71175925926</v>
+        <v>46079.72002283565</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46191</v>
+        <v>46079</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Thaiza Oliveira</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
       <c r="O271" s="1" t="n"/>
-      <c r="P271" s="2" t="n">
-        <v>46190.7346272338</v>
-      </c>
-      <c r="Q271" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
-      <c r="R271" s="1" t="inlineStr">
-        <is>
-          <t>Tarefas baixadas</t>
-        </is>
-      </c>
+      <c r="P271" s="1" t="n"/>
+      <c r="Q271" s="1" t="inlineStr"/>
+      <c r="R271" s="1" t="inlineStr"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T271" s="1" t="n"/>
@@ -22035,7 +22025,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>80174</v>
+        <v>80165</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
@@ -22044,7 +22034,7 @@
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Vencimento de Tarefas</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
@@ -22054,7 +22044,7 @@
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -22072,10 +22062,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46191.36721832176</v>
+        <v>46190.71175925926</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -22084,13 +22074,13 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="2" t="n">
-        <v>46191.49335512731</v>
+        <v>46190.7346272338</v>
       </c>
       <c r="Q272" s="1" t="inlineStr">
         <is>
@@ -22112,7 +22102,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80250</v>
+        <v>80174</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22121,7 +22111,7 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Vencimento de Tarefas</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -22131,7 +22121,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
+          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -22149,21 +22139,25 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46192.6584477662</v>
+        <v>46191.36721832176</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46195</v>
+        <v>46192</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M273" s="1" t="n"/>
+      <c r="M273" s="1" t="inlineStr">
+        <is>
+          <t>Yasmin Peixoto</t>
+        </is>
+      </c>
       <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="2" t="n">
-        <v>46192.70597966435</v>
+        <v>46191.49335512731</v>
       </c>
       <c r="Q273" s="1" t="inlineStr">
         <is>
@@ -22185,7 +22179,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80709</v>
+        <v>80250</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22204,7 +22198,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22222,25 +22216,21 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46205.72485570602</v>
+        <v>46192.6584477662</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46206</v>
+        <v>46195</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M274" s="1" t="inlineStr">
-        <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
+      <c r="M274" s="1" t="n"/>
       <c r="N274" s="1" t="n"/>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="2" t="n">
-        <v>46205.73248877314</v>
+        <v>46192.70597966435</v>
       </c>
       <c r="Q274" s="1" t="inlineStr">
         <is>
@@ -22262,7 +22252,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>81083</v>
+        <v>80709</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22281,7 +22271,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22299,10 +22289,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46218.68119872685</v>
+        <v>46205.72485570602</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46219</v>
+        <v>46206</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22317,7 +22307,7 @@
       <c r="N275" s="1" t="n"/>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="2" t="n">
-        <v>46218.7466727662</v>
+        <v>46205.73248877314</v>
       </c>
       <c r="Q275" s="1" t="inlineStr">
         <is>
@@ -22326,7 +22316,7 @@
       </c>
       <c r="R275" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+          <t>Tarefas baixadas</t>
         </is>
       </c>
       <c r="S275" s="1" t="inlineStr">
@@ -22339,7 +22329,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>81230</v>
+        <v>81083</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22348,53 +22338,67 @@
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Reabertura de tarefa</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
         <is>
-          <t>RJ - EF</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,solicito a reabertura da tarefa 3659 - Fed - DAS da empresa 4951 - SUPER SERVIÇOS TERCEIRIZADOS DE APOIO LTDA do mês 06.2026, porque houve retificadora com valor.</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G276" s="1" t="n"/>
-      <c r="H276" s="1" t="n"/>
+      <c r="H276" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I276" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46223.71789861111</v>
+        <v>46218.68119872685</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46224</v>
+        <v>46219</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
         <is>
-          <t>Isabela Barbosa</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N276" s="1" t="n"/>
       <c r="O276" s="1" t="n"/>
-      <c r="P276" s="1" t="n"/>
-      <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="n"/>
+      <c r="P276" s="2" t="n">
+        <v>46218.7466727662</v>
+      </c>
+      <c r="Q276" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
+      <c r="R276" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+        </is>
+      </c>
       <c r="S276" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T276" s="1" t="n"/>
@@ -22402,7 +22406,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>81231</v>
+        <v>81236</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22416,45 +22420,49 @@
       </c>
       <c r="D277" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>RJ - EF</t>
         </is>
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tardeSolicito a baixa na tarefa "´Prévia rescisões individuais" da empresa 2109 ICERI E ICERI SUPERMERCADO. Ao tentar realizar a baixa, retornou com uma notificação de erro, informando que o arquivo anexado não é compatível para baixar a tarefa.Segue a mesma em anexo para análise. Obrigado. </t>
+          <t>Bom dia !É enviado ao grupo SERVI um e-mail único de confirmação de faturamento referente a todas as empresas do GRUPO, por favor realizar a baixa da tarefa via banco de dados com o e-mail em anexo.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G277" s="1" t="n"/>
-      <c r="H277" s="1" t="n"/>
+      <c r="H277" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I277" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46223.72315987269</v>
+        <v>46224.35354027778</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M277" s="1" t="inlineStr">
         <is>
-          <t>Vitor Guedes</t>
+          <t>Glaucia Santos</t>
         </is>
       </c>
       <c r="N277" s="1" t="n"/>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
-      <c r="R277" s="1" t="n"/>
+      <c r="R277" s="1" t="inlineStr"/>
       <c r="S277" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22465,59 +22473,70 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>81233</v>
+        <v>77913</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, baixar as tarefas (Prévias rescisões individuais - PREVIA  e Prévias rescisões individuais - 662 -NICOLLY) da empresa 6559. MOTIVO: Cliente solicitou o cancelamento da solicitação.</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G278" s="1" t="n"/>
-      <c r="H278" s="1" t="n"/>
+      <c r="H278" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
       <c r="I278" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46223.74468653935</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46224</v>
+        <v>46097</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M278" s="1" t="inlineStr">
         <is>
-          <t>Edivaldo Veiga</t>
-        </is>
-      </c>
-      <c r="N278" s="1" t="n"/>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N278" s="2" t="n">
+        <v>46223.70421145833</v>
+      </c>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
-      <c r="R278" s="1" t="n"/>
+      <c r="R278" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
+        </is>
+      </c>
       <c r="S278" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22528,26 +22547,26 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>77913</v>
+        <v>79609</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22556,7 +22575,7 @@
       <c r="G279" s="1" t="n"/>
       <c r="H279" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I279" s="1" t="inlineStr">
@@ -22565,33 +22584,26 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46097</v>
+        <v>46205</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
-        </is>
-      </c>
-      <c r="N279" s="2" t="n">
-        <v>46223.70421145833</v>
-      </c>
+          <t>Claudio Correa</t>
+        </is>
+      </c>
+      <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
-        </is>
-      </c>
+      <c r="R279" s="1" t="inlineStr"/>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22602,7 +22614,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>79609</v>
+        <v>80515</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
@@ -22611,7 +22623,7 @@
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22621,7 +22633,7 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22630,7 +22642,7 @@
       <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22639,26 +22651,32 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46205</v>
+        <v>46226</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
-        </is>
-      </c>
-      <c r="N280" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N280" s="2" t="n">
+        <v>46219.75157017361</v>
+      </c>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
-      <c r="R280" s="1" t="inlineStr"/>
+      <c r="R280" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enviado para registro </t>
+        </is>
+      </c>
       <c r="S280" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22669,7 +22687,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>80515</v>
+        <v>80697</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
@@ -22678,7 +22696,7 @@
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22688,7 +22706,7 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22697,7 +22715,7 @@
       <c r="G281" s="1" t="n"/>
       <c r="H281" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I281" s="1" t="inlineStr">
@@ -22706,14 +22724,14 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46226</v>
+        <v>46237</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M281" s="1" t="inlineStr">
@@ -22721,17 +22739,11 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N281" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+      <c r="N281" s="1" t="n"/>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="Q281" s="1" t="inlineStr"/>
-      <c r="R281" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R281" s="1" t="inlineStr"/>
       <c r="S281" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22742,7 +22754,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>80697</v>
+        <v>80714</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
@@ -22751,7 +22763,7 @@
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
@@ -22761,7 +22773,7 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22770,7 +22782,7 @@
       <c r="G282" s="1" t="n"/>
       <c r="H282" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I282" s="1" t="inlineStr">
@@ -22779,14 +22791,14 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M282" s="1" t="inlineStr">
@@ -22794,11 +22806,18 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N282" s="1" t="n"/>
+      <c r="N282" s="2" t="n">
+        <v>46223.41822326389</v>
+      </c>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
-      <c r="R282" s="1" t="inlineStr"/>
+      <c r="R282" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+        </is>
+      </c>
       <c r="S282" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22809,16 +22828,16 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>80714</v>
+        <v>80919</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
@@ -22828,7 +22847,7 @@
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
@@ -22837,7 +22856,7 @@
       <c r="G283" s="1" t="n"/>
       <c r="H283" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I283" s="1" t="inlineStr">
@@ -22846,14 +22865,14 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M283" s="1" t="inlineStr">
@@ -22861,18 +22880,11 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N283" s="2" t="n">
-        <v>46223.41822326389</v>
-      </c>
+      <c r="N283" s="1" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
-      <c r="R283" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
-        </is>
-      </c>
+      <c r="R283" s="1" t="inlineStr"/>
       <c r="S283" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22883,16 +22895,16 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>80919</v>
+        <v>80935</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
@@ -22902,7 +22914,7 @@
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22911,7 +22923,7 @@
       <c r="G284" s="1" t="n"/>
       <c r="H284" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I284" s="1" t="inlineStr">
@@ -22920,14 +22932,14 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M284" s="1" t="inlineStr">
@@ -22935,11 +22947,18 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N284" s="1" t="n"/>
+      <c r="N284" s="2" t="n">
+        <v>46223.41869637732</v>
+      </c>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
-      <c r="R284" s="1" t="inlineStr"/>
+      <c r="R284" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+        </is>
+      </c>
       <c r="S284" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22950,7 +22969,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>80935</v>
+        <v>80936</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
@@ -22959,7 +22978,7 @@
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
@@ -22969,7 +22988,7 @@
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
@@ -22978,7 +22997,7 @@
       <c r="G285" s="1" t="n"/>
       <c r="H285" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I285" s="1" t="inlineStr">
@@ -22987,7 +23006,7 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K285" s="2" t="n">
         <v>46241</v>
@@ -23003,15 +23022,14 @@
         </is>
       </c>
       <c r="N285" s="2" t="n">
-        <v>46223.41869637732</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
       <c r="R285" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S285" s="1" t="inlineStr">
@@ -23024,7 +23042,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>80936</v>
+        <v>80951</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
@@ -23033,7 +23051,7 @@
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
@@ -23043,7 +23061,7 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
@@ -23061,7 +23079,7 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K286" s="2" t="n">
         <v>46241</v>
@@ -23077,14 +23095,14 @@
         </is>
       </c>
       <c r="N286" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46219.74920023148</v>
       </c>
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
       <c r="Q286" s="1" t="inlineStr"/>
       <c r="R286" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>Minuta enviada ao cliente</t>
         </is>
       </c>
       <c r="S286" s="1" t="inlineStr">
@@ -23097,26 +23115,26 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>80951</v>
+        <v>80989</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
@@ -23125,7 +23143,7 @@
       <c r="G287" s="1" t="n"/>
       <c r="H287" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I287" s="1" t="inlineStr">
@@ -23134,10 +23152,10 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46241</v>
+        <v>46217</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
@@ -23146,18 +23164,18 @@
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>João Oliveira</t>
         </is>
       </c>
       <c r="N287" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46223.4927846875</v>
       </c>
       <c r="O287" s="1" t="n"/>
       <c r="P287" s="1" t="n"/>
       <c r="Q287" s="1" t="inlineStr"/>
       <c r="R287" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
         </is>
       </c>
       <c r="S287" s="1" t="inlineStr">
@@ -23170,69 +23188,63 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>80989</v>
+        <v>81208</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Ata de Reunião de Sócios</t>
         </is>
       </c>
       <c r="C288" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Reeleição de Diretoria</t>
         </is>
       </c>
       <c r="D288" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G288" s="1" t="n"/>
-      <c r="H288" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+        <v>5449</v>
+      </c>
+      <c r="G288" s="1" t="inlineStr">
+        <is>
+          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
+        </is>
+      </c>
+      <c r="H288" s="1" t="n"/>
       <c r="I288" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46223.51713209491</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46217</v>
+        <v>46225</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
-        </is>
-      </c>
-      <c r="N288" s="2" t="n">
-        <v>46223.4927846875</v>
-      </c>
+          <t>Rogerio Egidio</t>
+        </is>
+      </c>
+      <c r="N288" s="1" t="n"/>
       <c r="O288" s="1" t="n"/>
       <c r="P288" s="1" t="n"/>
       <c r="Q288" s="1" t="inlineStr"/>
-      <c r="R288" s="1" t="inlineStr">
-        <is>
-          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
-        </is>
-      </c>
+      <c r="R288" s="1" t="n"/>
       <c r="S288" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23243,16 +23255,16 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81208</v>
+        <v>79793</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião de Sócios</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C289" s="1" t="inlineStr">
         <is>
-          <t>Reeleição de Diretoria</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D289" s="1" t="inlineStr">
@@ -23262,44 +23274,48 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>5449</v>
+        <v>5655</v>
       </c>
       <c r="G289" s="1" t="inlineStr">
         <is>
-          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
-        </is>
-      </c>
-      <c r="H289" s="1" t="n"/>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
+      <c r="H289" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
       <c r="I289" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46223.51713209491</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46225</v>
+        <v>46185</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
       <c r="Q289" s="1" t="inlineStr"/>
-      <c r="R289" s="1" t="n"/>
+      <c r="R289" s="1" t="inlineStr"/>
       <c r="S289" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23310,67 +23326,63 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79793</v>
+        <v>81209</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>5655</v>
+        <v>6094</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
-      <c r="H290" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+        </is>
+      </c>
+      <c r="H290" s="1" t="n"/>
       <c r="I290" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46185</v>
+        <v>46224</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
-      <c r="R290" s="1" t="inlineStr"/>
+      <c r="R290" s="1" t="n"/>
       <c r="S290" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23381,36 +23393,32 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81209</v>
+        <v>81225</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t>Boa tarde, Poderiam disponibilizar o login e senha da loja 4545 - FRIOS BRASIL. Municipio de hortolandia e o acesso e link no MGC não entra. Continuo no aguardo.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6094</v>
-      </c>
-      <c r="G291" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G291" s="1" t="n"/>
       <c r="H291" s="1" t="n"/>
       <c r="I291" s="1" t="inlineStr">
         <is>
@@ -23418,10 +23426,10 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46223.67691084491</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
@@ -23430,7 +23438,7 @@
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Beatriz Ferreira</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
@@ -23448,26 +23456,26 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>81225</v>
+        <v>81227</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam disponibilizar o login e senha da loja 4545 - FRIOS BRASIL. Municipio de hortolandia e o acesso e link no MGC não entra. Continuo no aguardo.</t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
@@ -23481,10 +23489,10 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46223.67691084491</v>
+        <v>46223.69836307871</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
@@ -23493,7 +23501,7 @@
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N292" s="1" t="n"/>
@@ -23511,26 +23519,26 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>81227</v>
+        <v>81228</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C293" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D293" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
@@ -23544,10 +23552,10 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46223.70694884259</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
@@ -23556,7 +23564,7 @@
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
+          <t>Beatriz Ferreira</t>
         </is>
       </c>
       <c r="N293" s="1" t="n"/>
@@ -23574,26 +23582,26 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>81228</v>
+        <v>81234</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
+          <t>Atualizar cadastro dos sócios da loja 2681 - COMERCIO ALVES E FARIAS.Tem 99% para a LINDELE no cadastro e a IBUACU que tbm está no quadro societário nem consta no cadastro.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
@@ -23607,10 +23615,10 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46223.70694884259</v>
+        <v>46223.81885586806</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L294" s="1" t="inlineStr">
         <is>
@@ -23619,7 +23627,7 @@
       </c>
       <c r="M294" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
       <c r="N294" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 21-07-26 1732
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U309" headerRowCount="1">
-  <autoFilter ref="A1:U309"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U312" headerRowCount="1">
+  <autoFilter ref="A1:U312"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U309"/>
+  <dimension ref="A1:U312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20911,70 +20911,59 @@
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
-        <v>77913</v>
+        <v>81275</v>
       </c>
       <c r="B260" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C260" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Baixa automática - Arquivos</t>
         </is>
       </c>
       <c r="D260" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E260" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>Boa tarde! Por gentileza, baixar a tarefa PIS/COFINS do cliente 5598 - DISTRIBUIDOR DE MORANGOS, competência 06-2026. Pois não estou conseguindo dar continuidade no processo devido ao seguinte erro: 	"Arquivo não possui informação de competência."</t>
         </is>
       </c>
       <c r="F260" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G260" s="1" t="n"/>
-      <c r="H260" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Ribeiro</t>
-        </is>
-      </c>
+      <c r="H260" s="1" t="n"/>
       <c r="I260" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J260" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46224.72587172453</v>
       </c>
       <c r="K260" s="2" t="n">
-        <v>46097</v>
+        <v>46225</v>
       </c>
       <c r="L260" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M260" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
-        </is>
-      </c>
-      <c r="N260" s="2" t="n">
-        <v>46223.70421145833</v>
-      </c>
+          <t>Thayna Melo</t>
+        </is>
+      </c>
+      <c r="N260" s="1" t="n"/>
       <c r="O260" s="1" t="n"/>
       <c r="P260" s="1" t="n"/>
       <c r="Q260" s="1" t="inlineStr"/>
-      <c r="R260" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
-        </is>
-      </c>
+      <c r="R260" s="1" t="n"/>
       <c r="S260" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -20985,26 +20974,26 @@
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
-        <v>79609</v>
+        <v>77913</v>
       </c>
       <c r="B261" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C261" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D261" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E261" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F261" s="1" t="n">
@@ -21013,7 +21002,7 @@
       <c r="G261" s="1" t="n"/>
       <c r="H261" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I261" s="1" t="inlineStr">
@@ -21022,26 +21011,33 @@
         </is>
       </c>
       <c r="J261" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K261" s="2" t="n">
-        <v>46205</v>
+        <v>46097</v>
       </c>
       <c r="L261" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M261" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
-        </is>
-      </c>
-      <c r="N261" s="1" t="n"/>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N261" s="2" t="n">
+        <v>46223.70421145833</v>
+      </c>
       <c r="O261" s="1" t="n"/>
       <c r="P261" s="1" t="n"/>
       <c r="Q261" s="1" t="inlineStr"/>
-      <c r="R261" s="1" t="inlineStr"/>
+      <c r="R261" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
+        </is>
+      </c>
       <c r="S261" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21052,7 +21048,7 @@
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
-        <v>80515</v>
+        <v>79609</v>
       </c>
       <c r="B262" s="1" t="inlineStr">
         <is>
@@ -21061,7 +21057,7 @@
       </c>
       <c r="C262" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D262" s="1" t="inlineStr">
@@ -21071,7 +21067,7 @@
       </c>
       <c r="E262" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F262" s="1" t="n">
@@ -21080,7 +21076,7 @@
       <c r="G262" s="1" t="n"/>
       <c r="H262" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I262" s="1" t="inlineStr">
@@ -21089,32 +21085,26 @@
         </is>
       </c>
       <c r="J262" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K262" s="2" t="n">
-        <v>46226</v>
+        <v>46205</v>
       </c>
       <c r="L262" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M262" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N262" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+          <t>Claudio Correa</t>
+        </is>
+      </c>
+      <c r="N262" s="1" t="n"/>
       <c r="O262" s="1" t="n"/>
       <c r="P262" s="1" t="n"/>
       <c r="Q262" s="1" t="inlineStr"/>
-      <c r="R262" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R262" s="1" t="inlineStr"/>
       <c r="S262" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21125,7 +21115,7 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>80697</v>
+        <v>80515</v>
       </c>
       <c r="B263" s="1" t="inlineStr">
         <is>
@@ -21134,7 +21124,7 @@
       </c>
       <c r="C263" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D263" s="1" t="inlineStr">
@@ -21144,7 +21134,7 @@
       </c>
       <c r="E263" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F263" s="1" t="n">
@@ -21162,10 +21152,10 @@
         </is>
       </c>
       <c r="J263" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>46237</v>
+        <v>46226</v>
       </c>
       <c r="L263" s="1" t="inlineStr">
         <is>
@@ -21178,14 +21168,14 @@
         </is>
       </c>
       <c r="N263" s="2" t="n">
-        <v>46224.68237751158</v>
+        <v>46219.75157017361</v>
       </c>
       <c r="O263" s="1" t="n"/>
       <c r="P263" s="1" t="n"/>
       <c r="Q263" s="1" t="inlineStr"/>
       <c r="R263" s="1" t="inlineStr">
         <is>
-          <t>Em atendimento</t>
+          <t xml:space="preserve">Enviado para registro </t>
         </is>
       </c>
       <c r="S263" s="1" t="inlineStr">
@@ -21198,7 +21188,7 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>80714</v>
+        <v>80697</v>
       </c>
       <c r="B264" s="1" t="inlineStr">
         <is>
@@ -21207,7 +21197,7 @@
       </c>
       <c r="C264" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D264" s="1" t="inlineStr">
@@ -21217,7 +21207,7 @@
       </c>
       <c r="E264" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F264" s="1" t="n">
@@ -21226,7 +21216,7 @@
       <c r="G264" s="1" t="n"/>
       <c r="H264" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I264" s="1" t="inlineStr">
@@ -21235,10 +21225,10 @@
         </is>
       </c>
       <c r="J264" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K264" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="L264" s="1" t="inlineStr">
         <is>
@@ -21251,15 +21241,14 @@
         </is>
       </c>
       <c r="N264" s="2" t="n">
-        <v>46223.41822326389</v>
+        <v>46224.68237751158</v>
       </c>
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
       <c r="Q264" s="1" t="inlineStr"/>
       <c r="R264" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+          <t>Em atendimento</t>
         </is>
       </c>
       <c r="S264" s="1" t="inlineStr">
@@ -21272,16 +21261,16 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>80919</v>
+        <v>80714</v>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C265" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D265" s="1" t="inlineStr">
@@ -21291,7 +21280,7 @@
       </c>
       <c r="E265" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F265" s="1" t="n">
@@ -21309,14 +21298,14 @@
         </is>
       </c>
       <c r="J265" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K265" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L265" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M265" s="1" t="inlineStr">
@@ -21324,11 +21313,18 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N265" s="1" t="n"/>
+      <c r="N265" s="2" t="n">
+        <v>46223.41822326389</v>
+      </c>
       <c r="O265" s="1" t="n"/>
       <c r="P265" s="1" t="n"/>
       <c r="Q265" s="1" t="inlineStr"/>
-      <c r="R265" s="1" t="inlineStr"/>
+      <c r="R265" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+        </is>
+      </c>
       <c r="S265" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21339,16 +21335,16 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>80935</v>
+        <v>80919</v>
       </c>
       <c r="B266" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C266" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D266" s="1" t="inlineStr">
@@ -21358,7 +21354,7 @@
       </c>
       <c r="E266" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F266" s="1" t="n">
@@ -21376,14 +21372,14 @@
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K266" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L266" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M266" s="1" t="inlineStr">
@@ -21391,18 +21387,11 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N266" s="2" t="n">
-        <v>46223.41869637732</v>
-      </c>
+      <c r="N266" s="1" t="n"/>
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
       <c r="Q266" s="1" t="inlineStr"/>
-      <c r="R266" s="1" t="inlineStr">
-        <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
-        </is>
-      </c>
+      <c r="R266" s="1" t="inlineStr"/>
       <c r="S266" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21413,7 +21402,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>80936</v>
+        <v>80935</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
@@ -21422,7 +21411,7 @@
       </c>
       <c r="C267" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D267" s="1" t="inlineStr">
@@ -21432,7 +21421,7 @@
       </c>
       <c r="E267" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F267" s="1" t="n">
@@ -21441,7 +21430,7 @@
       <c r="G267" s="1" t="n"/>
       <c r="H267" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I267" s="1" t="inlineStr">
@@ -21450,7 +21439,7 @@
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K267" s="2" t="n">
         <v>46241</v>
@@ -21466,14 +21455,15 @@
         </is>
       </c>
       <c r="N267" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46223.41869637732</v>
       </c>
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
       <c r="Q267" s="1" t="inlineStr"/>
       <c r="R267" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
         </is>
       </c>
       <c r="S267" s="1" t="inlineStr">
@@ -21486,7 +21476,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>80951</v>
+        <v>80936</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
@@ -21495,7 +21485,7 @@
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
@@ -21505,7 +21495,7 @@
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
@@ -21523,7 +21513,7 @@
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K268" s="2" t="n">
         <v>46241</v>
@@ -21539,14 +21529,14 @@
         </is>
       </c>
       <c r="N268" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O268" s="1" t="n"/>
       <c r="P268" s="1" t="n"/>
       <c r="Q268" s="1" t="inlineStr"/>
       <c r="R268" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S268" s="1" t="inlineStr">
@@ -21559,26 +21549,26 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>80989</v>
+        <v>80951</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
@@ -21587,7 +21577,7 @@
       <c r="G269" s="1" t="n"/>
       <c r="H269" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I269" s="1" t="inlineStr">
@@ -21596,10 +21586,10 @@
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46216.72016431713</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>46217</v>
+        <v>46241</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
@@ -21608,18 +21598,18 @@
       </c>
       <c r="M269" s="1" t="inlineStr">
         <is>
-          <t>João Oliveira</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N269" s="2" t="n">
-        <v>46223.4927846875</v>
+        <v>46219.74920023148</v>
       </c>
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
       <c r="Q269" s="1" t="inlineStr"/>
       <c r="R269" s="1" t="inlineStr">
         <is>
-          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
+          <t>Minuta enviada ao cliente</t>
         </is>
       </c>
       <c r="S269" s="1" t="inlineStr">
@@ -21632,11 +21622,11 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>81225</v>
+        <v>80989</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C270" s="1" t="inlineStr">
@@ -21651,7 +21641,7 @@
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam disponibilizar o login e senha da loja 4545 - FRIOS BRASIL. Municipio de hortolandia e o acesso e link no MGC não entra. Continuo no aguardo.</t>
+          <t>Por favor, regularizar a Guia ISS gerada em duplicidade da loja 3917 de Itapecerica da Serra. Seguem anexos, guia paga, guia duplicada (para retirar) e comprovante de pagamento.</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
@@ -21660,7 +21650,7 @@
       <c r="G270" s="1" t="n"/>
       <c r="H270" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I270" s="1" t="inlineStr">
@@ -21669,26 +21659,32 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46223.67691084491</v>
+        <v>46216.72016431713</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46226</v>
+        <v>46217</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
-        </is>
-      </c>
-      <c r="N270" s="1" t="n"/>
+          <t>João Oliveira</t>
+        </is>
+      </c>
+      <c r="N270" s="2" t="n">
+        <v>46223.4927846875</v>
+      </c>
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="inlineStr"/>
+      <c r="R270" s="1" t="inlineStr">
+        <is>
+          <t>Solicitação enviada à Prefeitura, aguardando retorno.</t>
+        </is>
+      </c>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21699,26 +21695,26 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>81227</v>
+        <v>81225</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>Boa tarde, Poderiam disponibilizar o login e senha da loja 4545 - FRIOS BRASIL. Municipio de hortolandia e o acesso e link no MGC não entra. Continuo no aguardo.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
@@ -21727,7 +21723,7 @@
       <c r="G271" s="1" t="n"/>
       <c r="H271" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I271" s="1" t="inlineStr">
@@ -21736,10 +21732,10 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46223.67691084491</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21748,7 +21744,7 @@
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
+          <t>Beatriz Ferreira</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
@@ -21766,26 +21762,26 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>81228</v>
+        <v>81227</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -21794,7 +21790,7 @@
       <c r="G272" s="1" t="n"/>
       <c r="H272" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I272" s="1" t="inlineStr">
@@ -21803,10 +21799,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46223.70694884259</v>
+        <v>46223.69836307871</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -21815,7 +21811,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -21833,26 +21829,26 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>81234</v>
+        <v>81228</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Atualizar cadastro dos sócios da loja 2681 - COMERCIO ALVES E FARIAS.Tem 99% para a LINDELE no cadastro e a IBUACU que tbm está no quadro societário nem consta no cadastro.</t>
+          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -21861,7 +21857,7 @@
       <c r="G273" s="1" t="n"/>
       <c r="H273" s="1" t="inlineStr">
         <is>
-          <t>Sarah Amaro</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I273" s="1" t="inlineStr">
@@ -21870,26 +21866,33 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46223.81885586806</v>
+        <v>46223.70694884259</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Lucas Fischer</t>
-        </is>
-      </c>
-      <c r="N273" s="1" t="n"/>
+          <t>Beatriz Ferreira</t>
+        </is>
+      </c>
+      <c r="N273" s="2" t="n">
+        <v>46224.71657758102</v>
+      </c>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="inlineStr"/>
+      <c r="R273" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Estou verificando o acesso  junto a prefeitura.</t>
+        </is>
+      </c>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21900,39 +21903,35 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>81208</v>
+        <v>81234</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião de Sócios</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Reeleição de Diretoria</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
+          <t>Atualizar cadastro dos sócios da loja 2681 - COMERCIO ALVES E FARIAS.Tem 99% para a LINDELE no cadastro e a IBUACU que tbm está no quadro societário nem consta no cadastro.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>5449</v>
-      </c>
-      <c r="G274" s="1" t="inlineStr">
-        <is>
-          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G274" s="1" t="n"/>
       <c r="H274" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Sarah Amaro</t>
         </is>
       </c>
       <c r="I274" s="1" t="inlineStr">
@@ -21941,7 +21940,7 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46223.51713209491</v>
+        <v>46223.81885586806</v>
       </c>
       <c r="K274" s="2" t="n">
         <v>46225</v>
@@ -21953,7 +21952,7 @@
       </c>
       <c r="M274" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
       <c r="N274" s="1" t="n"/>
@@ -21971,16 +21970,16 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>79793</v>
+        <v>81208</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Ata de Reunião de Sócios</t>
         </is>
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Reeleição de Diretoria</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
@@ -21990,20 +21989,20 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
-        <v>5655</v>
+        <v>5449</v>
       </c>
       <c r="G275" s="1" t="inlineStr">
         <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
+          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
         </is>
       </c>
       <c r="H275" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I275" s="1" t="inlineStr">
@@ -22012,10 +22011,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46223.51713209491</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46185</v>
+        <v>46225</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22024,7 +22023,7 @@
       </c>
       <c r="M275" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N275" s="1" t="n"/>
@@ -22042,67 +22041,63 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>81209</v>
+        <v>81270</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
-        <v>6094</v>
+        <v>5604</v>
       </c>
       <c r="G276" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
-        </is>
-      </c>
-      <c r="H276" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+          <t>GRAFICA TABOAO LTDA</t>
+        </is>
+      </c>
+      <c r="H276" s="1" t="n"/>
       <c r="I276" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46224.69047569444</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M276" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N276" s="1" t="n"/>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
-      <c r="R276" s="1" t="inlineStr"/>
+      <c r="R276" s="1" t="n"/>
       <c r="S276" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22113,35 +22108,39 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>81250</v>
+        <v>79793</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G277" s="1" t="n"/>
+        <v>5655</v>
+      </c>
+      <c r="G277" s="1" t="inlineStr">
+        <is>
+          <t>VANESSA DUARTE RODRIGUES</t>
+        </is>
+      </c>
       <c r="H277" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I277" s="1" t="inlineStr">
@@ -22150,10 +22149,10 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46224.44502184028</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46226</v>
+        <v>46185</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
@@ -22162,7 +22161,7 @@
       </c>
       <c r="M277" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N277" s="1" t="n"/>
@@ -22180,32 +22179,36 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>81251</v>
+        <v>81209</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G278" s="1" t="n"/>
+        <v>6094</v>
+      </c>
+      <c r="G278" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+        </is>
+      </c>
       <c r="H278" s="1" t="inlineStr">
         <is>
           <t>Ellen Leite</t>
@@ -22217,10 +22220,10 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46224.44796296296</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
@@ -22229,7 +22232,7 @@
       </c>
       <c r="M278" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N278" s="1" t="n"/>
@@ -22247,26 +22250,26 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>81267</v>
+        <v>81250</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
+          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22284,10 +22287,10 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46224.66958634259</v>
+        <v>46224.44502184028</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
@@ -22296,7 +22299,7 @@
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Rafaella Massuia</t>
         </is>
       </c>
       <c r="N279" s="1" t="n"/>
@@ -22314,39 +22317,35 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>81265</v>
+        <v>81251</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Olá, boa tarde!Recebemos um e-mail do cliente 2992 – M. Cavichiolli informando que houve alteração no quadro societário, com a entrada do sócio Enzo Yuji Iceri Cavichiolli.Ao consultar o sistema Único, verificamos que o referido sócio ainda não consta no cadastro. Solicito, por gentileza, que seja realizada a inclusão para que possamos dar andamento ao processo de retirada de pró-labore a partir da competência 07/2026.Qualquer dúvida, estou à disposição.Obrigado.</t>
+          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>2992</v>
-      </c>
-      <c r="G280" s="1" t="inlineStr">
-        <is>
-          <t>M CAVICHIOLLI COMÉRCIO DE ROUPAS EIRELI</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Sarah Amaro</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22355,10 +22354,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46224.64556646991</v>
+        <v>46224.44796296296</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22367,7 +22366,7 @@
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Rafaella Massuia</t>
         </is>
       </c>
       <c r="N280" s="1" t="n"/>
@@ -22385,39 +22384,35 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>81220</v>
+        <v>81267</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo, 6496 – Arão Pereira – CNPJ nº01.269.926/0001-40 – IE nº13.169.272-0 (suspensa).Solicito uma ajuda com urgencia, teria como verificar o que houve para a IE ser suspensa?</t>
+          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>6496</v>
-      </c>
-      <c r="G281" s="1" t="inlineStr">
-        <is>
-          <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G281" s="1" t="n"/>
       <c r="H281" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I281" s="1" t="inlineStr">
@@ -22426,41 +22421,29 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46223.63413202547</v>
+        <v>46224.66958634259</v>
       </c>
       <c r="K281" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
       <c r="O281" s="1" t="n"/>
-      <c r="P281" s="2" t="n">
-        <v>46223.68206091435</v>
-      </c>
-      <c r="Q281" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R281" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A empresa encontra-se suspensa por não atender notificação enviado no DTE conforme anexo.
-A notificação que ensejou a suspensão, foi lida somente hoje.
-</t>
-        </is>
-      </c>
+      <c r="P281" s="1" t="n"/>
+      <c r="Q281" s="1" t="inlineStr"/>
+      <c r="R281" s="1" t="inlineStr"/>
       <c r="S281" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T281" s="1" t="n"/>
@@ -22468,67 +22451,59 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>81004</v>
+        <v>81274</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
-        <v>6869</v>
-      </c>
-      <c r="G282" s="1" t="inlineStr">
-        <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
-      <c r="H282" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G282" s="1" t="n"/>
+      <c r="H282" s="1" t="n"/>
       <c r="I282" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46224.71483579861</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46218</v>
+        <v>46226</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M282" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N282" s="1" t="n"/>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
-      <c r="R282" s="1" t="inlineStr"/>
+      <c r="R282" s="1" t="n"/>
       <c r="S282" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22539,39 +22514,39 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>81005</v>
+        <v>81265</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Olá, boa tarde!Recebemos um e-mail do cliente 2992 – M. Cavichiolli informando que houve alteração no quadro societário, com a entrada do sócio Enzo Yuji Iceri Cavichiolli.Ao consultar o sistema Único, verificamos que o referido sócio ainda não consta no cadastro. Solicito, por gentileza, que seja realizada a inclusão para que possamos dar andamento ao processo de retirada de pró-labore a partir da competência 07/2026.Qualquer dúvida, estou à disposição.Obrigado.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
-        <v>6870</v>
+        <v>2992</v>
       </c>
       <c r="G283" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>M CAVICHIOLLI COMÉRCIO DE ROUPAS EIRELI</t>
         </is>
       </c>
       <c r="H283" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Sarah Amaro</t>
         </is>
       </c>
       <c r="I283" s="1" t="inlineStr">
@@ -22580,10 +22555,10 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46224.64556646991</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46218</v>
+        <v>46225</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
@@ -22592,7 +22567,7 @@
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>David Bragança</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
@@ -22610,39 +22585,39 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>81091</v>
+        <v>81220</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>Ronaldo, 6496 – Arão Pereira – CNPJ nº01.269.926/0001-40 – IE nº13.169.272-0 (suspensa).Solicito uma ajuda com urgencia, teria como verificar o que houve para a IE ser suspensa?</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
-        <v>6907</v>
+        <v>6496</v>
       </c>
       <c r="G284" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+          <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H284" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I284" s="1" t="inlineStr">
@@ -22651,29 +22626,41 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46223.63413202547</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="L284" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M284" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N284" s="1" t="n"/>
       <c r="O284" s="1" t="n"/>
-      <c r="P284" s="1" t="n"/>
-      <c r="Q284" s="1" t="inlineStr"/>
-      <c r="R284" s="1" t="inlineStr"/>
+      <c r="P284" s="2" t="n">
+        <v>46223.68206091435</v>
+      </c>
+      <c r="Q284" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="R284" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A empresa encontra-se suspensa por não atender notificação enviado no DTE conforme anexo.
+A notificação que ensejou a suspensão, foi lida somente hoje.
+</t>
+        </is>
+      </c>
       <c r="S284" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T284" s="1" t="n"/>
@@ -22681,39 +22668,39 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>81213</v>
+        <v>81004</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Cliente não possuí acesso cadastrado</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>6946</v>
+        <v>6869</v>
       </c>
       <c r="G285" s="1" t="inlineStr">
         <is>
-          <t>FFRA CONCRETOS LTDA</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H285" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I285" s="1" t="inlineStr">
@@ -22722,10 +22709,10 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46223.5798869213</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46225</v>
+        <v>46218</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
@@ -22734,7 +22721,7 @@
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
@@ -22752,51 +22739,51 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>79866</v>
+        <v>81005</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6539</v>
+        <v>6870</v>
       </c>
       <c r="G286" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H286" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I286" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46185</v>
+        <v>46218</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
@@ -22805,7 +22792,7 @@
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N286" s="1" t="n"/>
@@ -22823,34 +22810,34 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>79859</v>
+        <v>81091</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6570</v>
+        <v>6907</v>
       </c>
       <c r="G287" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H287" s="1" t="inlineStr">
@@ -22860,14 +22847,14 @@
       </c>
       <c r="I287" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46185</v>
+        <v>46223</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
@@ -22876,7 +22863,7 @@
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N287" s="1" t="n"/>
@@ -22894,51 +22881,51 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>79860</v>
+        <v>81213</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C288" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D288" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Cliente não possuí acesso cadastrado</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>6581</v>
+        <v>6946</v>
       </c>
       <c r="G288" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>FFRA CONCRETOS LTDA</t>
         </is>
       </c>
       <c r="H288" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I288" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46223.5798869213</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46185</v>
+        <v>46225</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -22947,7 +22934,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -22965,7 +22952,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>79861</v>
+        <v>79866</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -22984,15 +22971,15 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>6583</v>
+        <v>6539</v>
       </c>
       <c r="G289" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H289" s="1" t="inlineStr">
@@ -23006,7 +22993,7 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K289" s="2" t="n">
         <v>46185</v>
@@ -23036,16 +23023,16 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>79867</v>
+        <v>79859</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
@@ -23055,15 +23042,15 @@
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6704</v>
+        <v>6570</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H290" s="1" t="inlineStr">
@@ -23077,7 +23064,7 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K290" s="2" t="n">
         <v>46185</v>
@@ -23107,7 +23094,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>79856</v>
+        <v>79860</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
@@ -23126,15 +23113,15 @@
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>4225</v>
+        <v>6581</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H291" s="1" t="inlineStr">
@@ -23148,10 +23135,10 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
@@ -23160,7 +23147,7 @@
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
@@ -23178,7 +23165,7 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>79855</v>
+        <v>79861</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
@@ -23197,15 +23184,15 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>4765</v>
+        <v>6583</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H292" s="1" t="inlineStr">
@@ -23219,7 +23206,7 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K292" s="2" t="n">
         <v>46185</v>
@@ -23231,7 +23218,7 @@
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N292" s="1" t="n"/>
@@ -23249,7 +23236,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79833</v>
+        <v>79867</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
@@ -23268,15 +23255,15 @@
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6125</v>
+        <v>6704</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H293" s="1" t="inlineStr">
@@ -23290,32 +23277,26 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N293" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N293" s="1" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R293" s="1" t="inlineStr"/>
       <c r="S293" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23326,16 +23307,16 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>79834</v>
+        <v>79856</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
@@ -23345,15 +23326,15 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>6162</v>
+        <v>4225</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
@@ -23367,7 +23348,7 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>46184</v>
@@ -23397,7 +23378,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>79865</v>
+        <v>79855</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
@@ -23416,15 +23397,15 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6278</v>
+        <v>4765</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
@@ -23438,7 +23419,7 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K295" s="2" t="n">
         <v>46185</v>
@@ -23450,7 +23431,7 @@
       </c>
       <c r="M295" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N295" s="1" t="n"/>
@@ -23468,16 +23449,16 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>81243</v>
+        <v>79833</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
-          <t>Auditoria Inversa</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C296" s="1" t="inlineStr">
         <is>
-          <t>Envio de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D296" s="1" t="inlineStr">
@@ -23487,20 +23468,20 @@
       </c>
       <c r="E296" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A antiga contabilidade enviou a ECD do período de responsabilidade tecnica deles (01/01/2025 a 30/06/2025)  sem a inclusão de plano referencial, e para envio da ECF precisamos que essa informação seja inclusa na ECD.Precisamos que seja retificada a ECD com a inclusão do plano referencial da empresa.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>6298</v>
+        <v>6125</v>
       </c>
       <c r="G296" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">T W ALCANTARA ATACAREJO LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H296" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I296" s="1" t="inlineStr">
@@ -23509,26 +23490,32 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46224.42366959491</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K296" s="2" t="n">
-        <v>46225</v>
+        <v>46184</v>
       </c>
       <c r="L296" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M296" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
-        </is>
-      </c>
-      <c r="N296" s="1" t="n"/>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="N296" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O296" s="1" t="n"/>
       <c r="P296" s="1" t="n"/>
       <c r="Q296" s="1" t="inlineStr"/>
-      <c r="R296" s="1" t="inlineStr"/>
+      <c r="R296" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S296" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23539,16 +23526,16 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>79854</v>
+        <v>79834</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
@@ -23558,15 +23545,15 @@
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>6302</v>
+        <v>6162</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H297" s="1" t="inlineStr">
@@ -23580,7 +23567,7 @@
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K297" s="2" t="n">
         <v>46184</v>
@@ -23610,7 +23597,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>79863</v>
+        <v>79865</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23629,15 +23616,15 @@
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>6404</v>
+        <v>6278</v>
       </c>
       <c r="G298" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H298" s="1" t="inlineStr">
@@ -23651,7 +23638,7 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K298" s="2" t="n">
         <v>46185</v>
@@ -23681,16 +23668,16 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>79835</v>
+        <v>81243</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Auditoria Inversa</t>
         </is>
       </c>
       <c r="C299" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Envio de Documentos</t>
         </is>
       </c>
       <c r="D299" s="1" t="inlineStr">
@@ -23700,20 +23687,20 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Bom dia,A antiga contabilidade enviou a ECD do período de responsabilidade tecnica deles (01/01/2025 a 30/06/2025)  sem a inclusão de plano referencial, e para envio da ECF precisamos que essa informação seja inclusa na ECD.Precisamos que seja retificada a ECD com a inclusão do plano referencial da empresa.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>6485</v>
+        <v>6298</v>
       </c>
       <c r="G299" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t xml:space="preserve">T W ALCANTARA ATACAREJO LTDA </t>
         </is>
       </c>
       <c r="H299" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I299" s="1" t="inlineStr">
@@ -23722,10 +23709,10 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46224.42366959491</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>46184</v>
+        <v>46225</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
@@ -23734,7 +23721,7 @@
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N299" s="1" t="n"/>
@@ -23752,35 +23739,39 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>81244</v>
+        <v>79854</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C300" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D300" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G300" s="1" t="n"/>
+        <v>6302</v>
+      </c>
+      <c r="G300" s="1" t="inlineStr">
+        <is>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+        </is>
+      </c>
       <c r="H300" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I300" s="1" t="inlineStr">
@@ -23789,10 +23780,10 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46224.42615887732</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46226</v>
+        <v>46184</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
@@ -23801,7 +23792,7 @@
       </c>
       <c r="M300" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N300" s="1" t="n"/>
@@ -23819,35 +23810,39 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>81245</v>
+        <v>79863</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C301" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D301" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G301" s="1" t="n"/>
+        <v>6404</v>
+      </c>
+      <c r="G301" s="1" t="inlineStr">
+        <is>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
+        </is>
+      </c>
       <c r="H301" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I301" s="1" t="inlineStr">
@@ -23856,10 +23851,10 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46224.42947079861</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>46226</v>
+        <v>46185</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
@@ -23868,7 +23863,7 @@
       </c>
       <c r="M301" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N301" s="1" t="n"/>
@@ -23886,7 +23881,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>81247</v>
+        <v>79835</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
@@ -23895,26 +23890,30 @@
       </c>
       <c r="C302" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D302" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G302" s="1" t="n"/>
+        <v>6485</v>
+      </c>
+      <c r="G302" s="1" t="inlineStr">
+        <is>
+          <t>SMA AGRONEGOCIOS LTDA</t>
+        </is>
+      </c>
       <c r="H302" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I302" s="1" t="inlineStr">
@@ -23923,10 +23922,10 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K302" s="2" t="n">
-        <v>46226</v>
+        <v>46184</v>
       </c>
       <c r="L302" s="1" t="inlineStr">
         <is>
@@ -23935,7 +23934,7 @@
       </c>
       <c r="M302" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N302" s="1" t="n"/>
@@ -23953,7 +23952,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>81248</v>
+        <v>81244</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
@@ -23972,7 +23971,7 @@
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
@@ -23990,7 +23989,7 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46224.43289853009</v>
+        <v>46224.42615887732</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46226</v>
@@ -24020,7 +24019,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>81215</v>
+        <v>81245</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
@@ -24039,7 +24038,7 @@
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
@@ -24057,10 +24056,10 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46223.60068402778</v>
+        <v>46224.42947079861</v>
       </c>
       <c r="K304" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L304" s="1" t="inlineStr">
         <is>
@@ -24069,7 +24068,7 @@
       </c>
       <c r="M304" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N304" s="1" t="n"/>
@@ -24087,7 +24086,7 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>81217</v>
+        <v>81247</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
@@ -24106,7 +24105,7 @@
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
@@ -24124,10 +24123,10 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46223.60780787037</v>
+        <v>46224.43143758102</v>
       </c>
       <c r="K305" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L305" s="1" t="inlineStr">
         <is>
@@ -24136,7 +24135,7 @@
       </c>
       <c r="M305" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N305" s="1" t="n"/>
@@ -24154,7 +24153,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>81218</v>
+        <v>81248</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
@@ -24173,7 +24172,7 @@
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
@@ -24191,10 +24190,10 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46223.6082516551</v>
+        <v>46224.43289853009</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
@@ -24203,7 +24202,7 @@
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N306" s="1" t="n"/>
@@ -24221,7 +24220,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>81019</v>
+        <v>81215</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
@@ -24240,7 +24239,7 @@
       </c>
       <c r="E307" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
@@ -24249,7 +24248,7 @@
       <c r="G307" s="1" t="n"/>
       <c r="H307" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I307" s="1" t="inlineStr">
@@ -24258,14 +24257,14 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46223.60068402778</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>46218</v>
+        <v>46225</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M307" s="1" t="inlineStr">
@@ -24277,12 +24276,7 @@
       <c r="O307" s="1" t="n"/>
       <c r="P307" s="1" t="n"/>
       <c r="Q307" s="1" t="inlineStr"/>
-      <c r="R307" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
+      <c r="R307" s="1" t="inlineStr"/>
       <c r="S307" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24293,7 +24287,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>81052</v>
+        <v>81217</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
@@ -24312,7 +24306,7 @@
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
@@ -24321,7 +24315,7 @@
       <c r="G308" s="1" t="n"/>
       <c r="H308" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I308" s="1" t="inlineStr">
@@ -24330,30 +24324,26 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46223.60780787037</v>
       </c>
       <c r="K308" s="2" t="n">
-        <v>46219</v>
+        <v>46225</v>
       </c>
       <c r="L308" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M308" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N308" s="1" t="n"/>
       <c r="O308" s="1" t="n"/>
       <c r="P308" s="1" t="n"/>
       <c r="Q308" s="1" t="inlineStr"/>
-      <c r="R308" s="1" t="inlineStr">
-        <is>
-          <t>cobramos os documentos do antigo contador.</t>
-        </is>
-      </c>
+      <c r="R308" s="1" t="inlineStr"/>
       <c r="S308" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24364,7 +24354,7 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>81055</v>
+        <v>81218</v>
       </c>
       <c r="B309" s="1" t="inlineStr">
         <is>
@@ -24383,7 +24373,7 @@
       </c>
       <c r="E309" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F309" s="1" t="n">
@@ -24392,7 +24382,7 @@
       <c r="G309" s="1" t="n"/>
       <c r="H309" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I309" s="1" t="inlineStr">
@@ -24401,32 +24391,26 @@
         </is>
       </c>
       <c r="J309" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46223.6082516551</v>
       </c>
       <c r="K309" s="2" t="n">
-        <v>46219</v>
+        <v>46225</v>
       </c>
       <c r="L309" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M309" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N309" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N309" s="1" t="n"/>
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="1" t="n"/>
       <c r="Q309" s="1" t="inlineStr"/>
-      <c r="R309" s="1" t="inlineStr">
-        <is>
-          <t>Aguardando retorno dos dados do contador</t>
-        </is>
-      </c>
+      <c r="R309" s="1" t="inlineStr"/>
       <c r="S309" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24434,6 +24418,222 @@
       </c>
       <c r="T309" s="1" t="n"/>
       <c r="U309" s="1" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="1" t="n">
+        <v>81019</v>
+      </c>
+      <c r="B310" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C310" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D310" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E310" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+        </is>
+      </c>
+      <c r="F310" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" s="1" t="n"/>
+      <c r="H310" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I310" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="n">
+        <v>46217.43210269676</v>
+      </c>
+      <c r="K310" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="L310" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido para Responsável</t>
+        </is>
+      </c>
+      <c r="M310" s="1" t="inlineStr">
+        <is>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N310" s="1" t="n"/>
+      <c r="O310" s="1" t="n"/>
+      <c r="P310" s="1" t="n"/>
+      <c r="Q310" s="1" t="inlineStr"/>
+      <c r="R310" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
+        </is>
+      </c>
+      <c r="S310" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T310" s="1" t="n"/>
+      <c r="U310" s="1" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="1" t="n">
+        <v>81052</v>
+      </c>
+      <c r="B311" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C311" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D311" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E311" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+        </is>
+      </c>
+      <c r="F311" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" s="1" t="n"/>
+      <c r="H311" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I311" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="n">
+        <v>46218.38736744213</v>
+      </c>
+      <c r="K311" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L311" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido para Responsável</t>
+        </is>
+      </c>
+      <c r="M311" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N311" s="1" t="n"/>
+      <c r="O311" s="1" t="n"/>
+      <c r="P311" s="1" t="n"/>
+      <c r="Q311" s="1" t="inlineStr"/>
+      <c r="R311" s="1" t="inlineStr">
+        <is>
+          <t>cobramos os documentos do antigo contador.</t>
+        </is>
+      </c>
+      <c r="S311" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T311" s="1" t="n"/>
+      <c r="U311" s="1" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="1" t="n">
+        <v>81055</v>
+      </c>
+      <c r="B312" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C312" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D312" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E312" s="1" t="inlineStr">
+        <is>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+        </is>
+      </c>
+      <c r="F312" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" s="1" t="n"/>
+      <c r="H312" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I312" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="n">
+        <v>46218.40379614583</v>
+      </c>
+      <c r="K312" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L312" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M312" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N312" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
+      <c r="O312" s="1" t="n"/>
+      <c r="P312" s="1" t="n"/>
+      <c r="Q312" s="1" t="inlineStr"/>
+      <c r="R312" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
+      <c r="S312" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T312" s="1" t="n"/>
+      <c r="U312" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 22-07-26 1325
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U324" headerRowCount="1">
-  <autoFilter ref="A1:U324"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U325" headerRowCount="1">
+  <autoFilter ref="A1:U325"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U324"/>
+  <dimension ref="A1:U325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16628,7 +16628,7 @@
       </c>
       <c r="L199" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M199" s="1" t="inlineStr">
@@ -16640,12 +16640,22 @@
       <c r="O199" s="2" t="n">
         <v>46226</v>
       </c>
-      <c r="P199" s="1" t="n"/>
-      <c r="Q199" s="1" t="inlineStr"/>
-      <c r="R199" s="1" t="inlineStr"/>
+      <c r="P199" s="2" t="n">
+        <v>46225.5485099537</v>
+      </c>
+      <c r="Q199" s="1" t="inlineStr">
+        <is>
+          <t>Emylle Souza</t>
+        </is>
+      </c>
+      <c r="R199" s="1" t="inlineStr">
+        <is>
+          <t>Guia enviada por e-mail.</t>
+        </is>
+      </c>
       <c r="S199" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T199" s="1" t="n"/>
@@ -21712,7 +21722,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>81295</v>
+        <v>81306</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
@@ -21731,28 +21741,32 @@
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Precisamos da baixa da tarefa "Est - ICMS RPA - CÓD. 046-2" referente a competência 06/2026 com arquivos em anexo.</t>
+          <t>Por favor precisamos da baixa tarefa "Fed - PIS/COFINS Cumulativo - 2172" das tarefas com arquivos em anexo.</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G270" s="1" t="n"/>
-      <c r="H270" s="1" t="n"/>
+      <c r="H270" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I270" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46225.47961967593</v>
+        <v>46225.53244189815</v>
       </c>
       <c r="K270" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M270" s="1" t="inlineStr">
@@ -21764,7 +21778,7 @@
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="Q270" s="1" t="inlineStr"/>
-      <c r="R270" s="1" t="n"/>
+      <c r="R270" s="1" t="inlineStr"/>
       <c r="S270" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21775,70 +21789,59 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>77913</v>
+        <v>81307</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C271" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Abertura de protocolo</t>
         </is>
       </c>
       <c r="D271" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>MG EXPRESS - GC</t>
         </is>
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>Precisamos da baixa da tarefa "Fed - PIS/COFINS Não Cumul/Mon - 5856" das empresas com arquivo em anexo.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G271" s="1" t="n"/>
-      <c r="H271" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Ribeiro</t>
-        </is>
-      </c>
+      <c r="H271" s="1" t="n"/>
       <c r="I271" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46225.54769618055</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46097</v>
+        <v>46226</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
-        </is>
-      </c>
-      <c r="N271" s="2" t="n">
-        <v>46223.70421145833</v>
-      </c>
+          <t>Romero Borges</t>
+        </is>
+      </c>
+      <c r="N271" s="1" t="n"/>
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="Q271" s="1" t="inlineStr"/>
-      <c r="R271" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
-        </is>
-      </c>
+      <c r="R271" s="1" t="n"/>
       <c r="S271" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21849,26 +21852,26 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>79609</v>
+        <v>77913</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Comércio</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>TESTE TESTE</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
@@ -21877,7 +21880,7 @@
       <c r="G272" s="1" t="n"/>
       <c r="H272" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I272" s="1" t="inlineStr">
@@ -21886,26 +21889,33 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46175.48423082176</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46205</v>
+        <v>46097</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
-        </is>
-      </c>
-      <c r="N272" s="1" t="n"/>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N272" s="2" t="n">
+        <v>46223.70421145833</v>
+      </c>
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
       <c r="Q272" s="1" t="inlineStr"/>
-      <c r="R272" s="1" t="inlineStr"/>
+      <c r="R272" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
+        </is>
+      </c>
       <c r="S272" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21916,7 +21926,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80515</v>
+        <v>79609</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -21925,7 +21935,7 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Eireli - Comércio</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -21935,7 +21945,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>TESTE TESTE</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -21944,7 +21954,7 @@
       <c r="G273" s="1" t="n"/>
       <c r="H273" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I273" s="1" t="inlineStr">
@@ -21953,32 +21963,26 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46175.48423082176</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46226</v>
+        <v>46205</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N273" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+          <t>Claudio Correa</t>
+        </is>
+      </c>
+      <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="Q273" s="1" t="inlineStr"/>
-      <c r="R273" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R273" s="1" t="inlineStr"/>
       <c r="S273" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21989,7 +21993,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80697</v>
+        <v>80515</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -21998,7 +22002,7 @@
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -22008,7 +22012,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22026,10 +22030,10 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46237</v>
+        <v>46226</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
@@ -22042,14 +22046,14 @@
         </is>
       </c>
       <c r="N274" s="2" t="n">
-        <v>46224.68237751158</v>
+        <v>46219.75157017361</v>
       </c>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="Q274" s="1" t="inlineStr"/>
       <c r="R274" s="1" t="inlineStr">
         <is>
-          <t>Em atendimento</t>
+          <t xml:space="preserve">Enviado para registro </t>
         </is>
       </c>
       <c r="S274" s="1" t="inlineStr">
@@ -22062,7 +22066,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>80714</v>
+        <v>80697</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22071,7 +22075,7 @@
       </c>
       <c r="C275" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D275" s="1" t="inlineStr">
@@ -22081,7 +22085,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22090,7 +22094,7 @@
       <c r="G275" s="1" t="n"/>
       <c r="H275" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I275" s="1" t="inlineStr">
@@ -22099,10 +22103,10 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
@@ -22115,15 +22119,14 @@
         </is>
       </c>
       <c r="N275" s="2" t="n">
-        <v>46223.41822326389</v>
+        <v>46224.68237751158</v>
       </c>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="Q275" s="1" t="inlineStr"/>
       <c r="R275" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+          <t>Em atendimento</t>
         </is>
       </c>
       <c r="S275" s="1" t="inlineStr">
@@ -22136,16 +22139,16 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>80919</v>
+        <v>80714</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C276" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D276" s="1" t="inlineStr">
@@ -22155,7 +22158,7 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
@@ -22173,10 +22176,10 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
@@ -22189,16 +22192,15 @@
         </is>
       </c>
       <c r="N276" s="2" t="n">
-        <v>46225.48500983796</v>
+        <v>46223.41822326389</v>
       </c>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="Q276" s="1" t="inlineStr"/>
       <c r="R276" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezadas(os), bom dia!
-Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
-Atenciosamente, </t>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
         </is>
       </c>
       <c r="S276" s="1" t="inlineStr">
@@ -22211,16 +22213,16 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>80935</v>
+        <v>80919</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22230,7 +22232,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22248,10 +22250,10 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
@@ -22264,15 +22266,16 @@
         </is>
       </c>
       <c r="N277" s="2" t="n">
-        <v>46223.41869637732</v>
+        <v>46225.48500983796</v>
       </c>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="Q277" s="1" t="inlineStr"/>
       <c r="R277" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+          <t xml:space="preserve">Prezadas(os), bom dia!
+Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
+Atenciosamente, </t>
         </is>
       </c>
       <c r="S277" s="1" t="inlineStr">
@@ -22285,7 +22288,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80936</v>
+        <v>80935</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22294,7 +22297,7 @@
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22304,7 +22307,7 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22313,7 +22316,7 @@
       <c r="G278" s="1" t="n"/>
       <c r="H278" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I278" s="1" t="inlineStr">
@@ -22322,7 +22325,7 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K278" s="2" t="n">
         <v>46241</v>
@@ -22338,14 +22341,15 @@
         </is>
       </c>
       <c r="N278" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46223.41869637732</v>
       </c>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
       <c r="R278" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
         </is>
       </c>
       <c r="S278" s="1" t="inlineStr">
@@ -22358,7 +22362,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80951</v>
+        <v>80936</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
@@ -22367,7 +22371,7 @@
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
@@ -22377,7 +22381,7 @@
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22395,7 +22399,7 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K279" s="2" t="n">
         <v>46241</v>
@@ -22411,14 +22415,14 @@
         </is>
       </c>
       <c r="N279" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
       <c r="R279" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S279" s="1" t="inlineStr">
@@ -22431,26 +22435,26 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>81227</v>
+        <v>80951</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22459,7 +22463,7 @@
       <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22468,26 +22472,32 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46224</v>
+        <v>46241</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
-        </is>
-      </c>
-      <c r="N280" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N280" s="2" t="n">
+        <v>46219.74920023148</v>
+      </c>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
-      <c r="R280" s="1" t="inlineStr"/>
+      <c r="R280" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviada ao cliente</t>
+        </is>
+      </c>
       <c r="S280" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22498,26 +22508,26 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>81228</v>
+        <v>81227</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22526,74 +22536,65 @@
       <c r="G281" s="1" t="n"/>
       <c r="H281" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I281" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46223.70694884259</v>
+        <v>46223.69836307871</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="Q281" s="1" t="inlineStr"/>
-      <c r="R281" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Estou verificando o acesso  junto a prefeitura.</t>
-        </is>
-      </c>
+      <c r="R281" s="1" t="inlineStr"/>
       <c r="S281" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T281" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
+      <c r="T281" s="1" t="n"/>
       <c r="U281" s="1" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>81234</v>
+        <v>81228</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>Atualizar cadastro dos sócios da loja 2681 - COMERCIO ALVES E FARIAS.Tem 99% para a LINDELE no cadastro e a IBUACU que tbm está no quadro societário nem consta no cadastro.</t>
+          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22602,65 +22603,74 @@
       <c r="G282" s="1" t="n"/>
       <c r="H282" s="1" t="inlineStr">
         <is>
-          <t>Sarah Amaro</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I282" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46223.81885586806</v>
+        <v>46223.70694884259</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M282" s="1" t="inlineStr">
         <is>
-          <t>Lucas Fischer</t>
+          <t>Beatriz Ferreira</t>
         </is>
       </c>
       <c r="N282" s="1" t="n"/>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
-      <c r="R282" s="1" t="inlineStr"/>
+      <c r="R282" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Estou verificando o acesso  junto a prefeitura.</t>
+        </is>
+      </c>
       <c r="S282" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T282" s="1" t="n"/>
+      <c r="T282" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
       <c r="U282" s="1" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>81250</v>
+        <v>81234</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
+          <t>Atualizar cadastro dos sócios da loja 2681 - COMERCIO ALVES E FARIAS.Tem 99% para a LINDELE no cadastro e a IBUACU que tbm está no quadro societário nem consta no cadastro.</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
@@ -22669,7 +22679,7 @@
       <c r="G283" s="1" t="n"/>
       <c r="H283" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Sarah Amaro</t>
         </is>
       </c>
       <c r="I283" s="1" t="inlineStr">
@@ -22678,10 +22688,10 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46224.44502184028</v>
+        <v>46223.81885586806</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
@@ -22690,7 +22700,7 @@
       </c>
       <c r="M283" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
+          <t>Lucas Fischer</t>
         </is>
       </c>
       <c r="N283" s="1" t="n"/>
@@ -22708,7 +22718,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>81251</v>
+        <v>81250</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
@@ -22727,7 +22737,7 @@
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
+          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22745,7 +22755,7 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46224.44796296296</v>
+        <v>46224.44502184028</v>
       </c>
       <c r="K284" s="2" t="n">
         <v>46226</v>
@@ -22775,26 +22785,26 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>81267</v>
+        <v>81251</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
+          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
@@ -22812,10 +22822,10 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46224.66958634259</v>
+        <v>46224.44796296296</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
@@ -22824,7 +22834,7 @@
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Rafaella Massuia</t>
         </is>
       </c>
       <c r="N285" s="1" t="n"/>
@@ -22842,16 +22852,16 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>81274</v>
+        <v>81267</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
@@ -22861,28 +22871,32 @@
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
+          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G286" s="1" t="n"/>
-      <c r="H286" s="1" t="n"/>
+      <c r="H286" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I286" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46224.71483579861</v>
+        <v>46224.66958634259</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M286" s="1" t="inlineStr">
@@ -22894,7 +22908,7 @@
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
       <c r="Q286" s="1" t="inlineStr"/>
-      <c r="R286" s="1" t="n"/>
+      <c r="R286" s="1" t="inlineStr"/>
       <c r="S286" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22905,7 +22919,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81294</v>
+        <v>81274</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
@@ -22919,12 +22933,12 @@
       </c>
       <c r="D287" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solicito novo acesso da prefeitura de Holambra das empresas 3705 e 4216 </t>
+          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
@@ -22938,10 +22952,10 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46225.47387288194</v>
+        <v>46224.71483579861</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>46230</v>
+        <v>46226</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
@@ -22950,7 +22964,7 @@
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Shofia Gomes</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N287" s="1" t="n"/>
@@ -22968,26 +22982,26 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>81296</v>
+        <v>81294</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C288" s="1" t="inlineStr">
         <is>
-          <t>Outras Cláusulas</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D288" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
+          <t xml:space="preserve">Solicito novo acesso da prefeitura de Holambra das empresas 3705 e 4216 </t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
@@ -23001,10 +23015,10 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46225.4866127662</v>
+        <v>46225.47387288194</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46255</v>
+        <v>46230</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -23013,7 +23027,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Shofia Gomes</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -23031,36 +23045,32 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81304</v>
+        <v>81296</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
-          <t>Retificação de Guia</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C289" s="1" t="inlineStr">
         <is>
-          <t>DARF</t>
+          <t>Outras Cláusulas</t>
         </is>
       </c>
       <c r="D289" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!A Sincoplastic precisa de uma Certidão Federal, mas temos um DARF do 1º Trimestre de 2026 que foi pago com PA e Vencimento errado, sendo correto PA 31/03/2026 e vencimento 30/06/2026, poderiam providenciar o REDARF, segue anexos.</t>
+          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>305</v>
-      </c>
-      <c r="G289" s="1" t="inlineStr">
-        <is>
-          <t>SINCOPLASTIC INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G289" s="1" t="n"/>
       <c r="H289" s="1" t="n"/>
       <c r="I289" s="1" t="inlineStr">
         <is>
@@ -23068,10 +23078,10 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46225.52103645833</v>
+        <v>46225.4866127662</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46226</v>
+        <v>46255</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
@@ -23080,7 +23090,7 @@
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Andrea Medeiros</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
@@ -23098,67 +23108,63 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>81265</v>
+        <v>81304</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Retificação de Guia</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>DARF</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Olá, boa tarde!Recebemos um e-mail do cliente 2992 – M. Cavichiolli informando que houve alteração no quadro societário, com a entrada do sócio Enzo Yuji Iceri Cavichiolli.Ao consultar o sistema Único, verificamos que o referido sócio ainda não consta no cadastro. Solicito, por gentileza, que seja realizada a inclusão para que possamos dar andamento ao processo de retirada de pró-labore a partir da competência 07/2026.Qualquer dúvida, estou à disposição.Obrigado.</t>
+          <t>Boa tarde!A Sincoplastic precisa de uma Certidão Federal, mas temos um DARF do 1º Trimestre de 2026 que foi pago com PA e Vencimento errado, sendo correto PA 31/03/2026 e vencimento 30/06/2026, poderiam providenciar o REDARF, segue anexos.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>2992</v>
+        <v>305</v>
       </c>
       <c r="G290" s="1" t="inlineStr">
         <is>
-          <t>M CAVICHIOLLI COMÉRCIO DE ROUPAS EIRELI</t>
-        </is>
-      </c>
-      <c r="H290" s="1" t="inlineStr">
-        <is>
-          <t>Sarah Amaro</t>
-        </is>
-      </c>
+          <t>SINCOPLASTIC INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+        </is>
+      </c>
+      <c r="H290" s="1" t="n"/>
       <c r="I290" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46224.64556646991</v>
+        <v>46225.52103645833</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Andrea Medeiros</t>
         </is>
       </c>
       <c r="N290" s="1" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
-      <c r="R290" s="1" t="inlineStr"/>
+      <c r="R290" s="1" t="n"/>
       <c r="S290" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23169,39 +23175,39 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81208</v>
+        <v>81265</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião de Sócios</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Reeleição de Diretoria</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
+          <t>Olá, boa tarde!Recebemos um e-mail do cliente 2992 – M. Cavichiolli informando que houve alteração no quadro societário, com a entrada do sócio Enzo Yuji Iceri Cavichiolli.Ao consultar o sistema Único, verificamos que o referido sócio ainda não consta no cadastro. Solicito, por gentileza, que seja realizada a inclusão para que possamos dar andamento ao processo de retirada de pró-labore a partir da competência 07/2026.Qualquer dúvida, estou à disposição.Obrigado.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>5449</v>
+        <v>2992</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
+          <t>M CAVICHIOLLI COMÉRCIO DE ROUPAS EIRELI</t>
         </is>
       </c>
       <c r="H291" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Sarah Amaro</t>
         </is>
       </c>
       <c r="I291" s="1" t="inlineStr">
@@ -23210,7 +23216,7 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46223.51713209491</v>
+        <v>46224.64556646991</v>
       </c>
       <c r="K291" s="2" t="n">
         <v>46225</v>
@@ -23222,7 +23228,7 @@
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>David Bragança</t>
         </is>
       </c>
       <c r="N291" s="1" t="n"/>
@@ -23240,63 +23246,67 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>81270</v>
+        <v>81208</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Ata de Reunião de Sócios</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Reeleição de Diretoria</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
+          <t>Por gentileza, encaminhar a Ata registrada para o cliente.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>5604</v>
+        <v>5449</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>GRAFICA TABOAO LTDA</t>
-        </is>
-      </c>
-      <c r="H292" s="1" t="n"/>
+          <t>RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA</t>
+        </is>
+      </c>
+      <c r="H292" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I292" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46224.69047569444</v>
+        <v>46223.51713209491</v>
       </c>
       <c r="K292" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M292" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N292" s="1" t="n"/>
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
       <c r="Q292" s="1" t="inlineStr"/>
-      <c r="R292" s="1" t="n"/>
+      <c r="R292" s="1" t="inlineStr"/>
       <c r="S292" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23307,7 +23317,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>79793</v>
+        <v>81270</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
@@ -23321,53 +23331,49 @@
       </c>
       <c r="D293" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>5655</v>
+        <v>5604</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
-      <c r="H293" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>GRAFICA TABOAO LTDA</t>
+        </is>
+      </c>
+      <c r="H293" s="1" t="n"/>
       <c r="I293" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46224.69047569444</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46185</v>
+        <v>46225</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N293" s="1" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="inlineStr"/>
+      <c r="R293" s="1" t="n"/>
       <c r="S293" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23378,39 +23384,39 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>81209</v>
+        <v>79793</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>6094</v>
+        <v>5655</v>
       </c>
       <c r="G294" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+          <t>VANESSA DUARTE RODRIGUES</t>
         </is>
       </c>
       <c r="H294" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I294" s="1" t="inlineStr">
@@ -23419,10 +23425,10 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>46224</v>
+        <v>46185</v>
       </c>
       <c r="L294" s="1" t="inlineStr">
         <is>
@@ -23431,7 +23437,7 @@
       </c>
       <c r="M294" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N294" s="1" t="n"/>
@@ -23449,39 +23455,39 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>81220</v>
+        <v>81209</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C295" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D295" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo, 6496 – Arão Pereira – CNPJ nº01.269.926/0001-40 – IE nº13.169.272-0 (suspensa).Solicito uma ajuda com urgencia, teria como verificar o que houve para a IE ser suspensa?</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>6496</v>
+        <v>6094</v>
       </c>
       <c r="G295" s="1" t="inlineStr">
         <is>
-          <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
         </is>
       </c>
       <c r="H295" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I295" s="1" t="inlineStr">
@@ -23490,108 +23496,112 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46223.63413202547</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K295" s="2" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="L295" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M295" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N295" s="1" t="n"/>
       <c r="O295" s="1" t="n"/>
-      <c r="P295" s="2" t="n">
+      <c r="P295" s="1" t="n"/>
+      <c r="Q295" s="1" t="inlineStr"/>
+      <c r="R295" s="1" t="inlineStr"/>
+      <c r="S295" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T295" s="1" t="n"/>
+      <c r="U295" s="1" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="1" t="n">
+        <v>81220</v>
+      </c>
+      <c r="B296" s="1" t="inlineStr">
+        <is>
+          <t>Regularização</t>
+        </is>
+      </c>
+      <c r="C296" s="1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="D296" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E296" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo, 6496 – Arão Pereira – CNPJ nº01.269.926/0001-40 – IE nº13.169.272-0 (suspensa).Solicito uma ajuda com urgencia, teria como verificar o que houve para a IE ser suspensa?</t>
+        </is>
+      </c>
+      <c r="F296" s="1" t="n">
+        <v>6496</v>
+      </c>
+      <c r="G296" s="1" t="inlineStr">
+        <is>
+          <t>ARAO PEREIRA DE SA LTDA (MATRIZ)</t>
+        </is>
+      </c>
+      <c r="H296" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="I296" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="n">
+        <v>46223.63413202547</v>
+      </c>
+      <c r="K296" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="L296" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M296" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N296" s="1" t="n"/>
+      <c r="O296" s="1" t="n"/>
+      <c r="P296" s="2" t="n">
         <v>46223.68206091435</v>
       </c>
-      <c r="Q295" s="1" t="inlineStr">
+      <c r="Q296" s="1" t="inlineStr">
         <is>
           <t>Ronaldo Dias</t>
         </is>
       </c>
-      <c r="R295" s="1" t="inlineStr">
+      <c r="R296" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">A empresa encontra-se suspensa por não atender notificação enviado no DTE conforme anexo.
 A notificação que ensejou a suspensão, foi lida somente hoje.
 </t>
         </is>
       </c>
-      <c r="S295" s="1" t="inlineStr">
+      <c r="S296" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="T295" s="1" t="n"/>
-      <c r="U295" s="1" t="inlineStr"/>
-    </row>
-    <row r="296">
-      <c r="A296" s="1" t="n">
-        <v>81297</v>
-      </c>
-      <c r="B296" s="1" t="inlineStr">
-        <is>
-          <t>Cadastro de Cliente</t>
-        </is>
-      </c>
-      <c r="C296" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Alteração </t>
-        </is>
-      </c>
-      <c r="D296" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E296" s="1" t="inlineStr">
-        <is>
-          <t>Bom dia!Ao acessar o posto fiscal está trazendo uma tela de cadastro, e não permiti acessar sem o preenchimento das informações cadastrais da empresa.</t>
-        </is>
-      </c>
-      <c r="F296" s="1" t="n">
-        <v>6777</v>
-      </c>
-      <c r="G296" s="1" t="inlineStr">
-        <is>
-          <t>A. DE S. JANOCA MERCADO</t>
-        </is>
-      </c>
-      <c r="H296" s="1" t="n"/>
-      <c r="I296" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J296" s="2" t="n">
-        <v>46225.48669829861</v>
-      </c>
-      <c r="K296" s="2" t="n">
-        <v>46226</v>
-      </c>
-      <c r="L296" s="1" t="inlineStr">
-        <is>
-          <t>Sem Responsavel Atribuido</t>
-        </is>
-      </c>
-      <c r="M296" s="1" t="inlineStr">
-        <is>
-          <t>Clara Maria</t>
-        </is>
-      </c>
-      <c r="N296" s="1" t="n"/>
-      <c r="O296" s="1" t="n"/>
-      <c r="P296" s="1" t="n"/>
-      <c r="Q296" s="1" t="inlineStr"/>
-      <c r="R296" s="1" t="n"/>
-      <c r="S296" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="T296" s="1" t="n"/>
@@ -23599,7 +23609,7 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>81004</v>
+        <v>81297</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
@@ -23613,53 +23623,49 @@
       </c>
       <c r="D297" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>Bom dia!Ao acessar o posto fiscal está trazendo uma tela de cadastro, e não permiti acessar sem o preenchimento das informações cadastrais da empresa.</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>6869</v>
+        <v>6777</v>
       </c>
       <c r="G297" s="1" t="inlineStr">
         <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
-      <c r="H297" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>A. DE S. JANOCA MERCADO</t>
+        </is>
+      </c>
+      <c r="H297" s="1" t="n"/>
       <c r="I297" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46225.48669829861</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46218</v>
+        <v>46226</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
+          <t>Clara Maria</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
       <c r="Q297" s="1" t="inlineStr"/>
-      <c r="R297" s="1" t="inlineStr"/>
+      <c r="R297" s="1" t="n"/>
       <c r="S297" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23670,7 +23676,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>81005</v>
+        <v>81004</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
@@ -23693,16 +23699,16 @@
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>6870</v>
+        <v>6869</v>
       </c>
       <c r="G298" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H298" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I298" s="1" t="inlineStr">
@@ -23711,7 +23717,7 @@
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K298" s="2" t="n">
         <v>46218</v>
@@ -23741,39 +23747,39 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>81091</v>
+        <v>81005</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C299" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D299" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>6907</v>
+        <v>6870</v>
       </c>
       <c r="G299" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
+          <t>AC HOME PET RAÇÕES LTDA</t>
         </is>
       </c>
       <c r="H299" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I299" s="1" t="inlineStr">
@@ -23782,10 +23788,10 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K299" s="2" t="n">
-        <v>46223</v>
+        <v>46218</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
@@ -23794,7 +23800,7 @@
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N299" s="1" t="n"/>
@@ -23812,7 +23818,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>81213</v>
+        <v>81091</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
@@ -23821,7 +23827,7 @@
       </c>
       <c r="C300" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D300" s="1" t="inlineStr">
@@ -23831,20 +23837,20 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>Cliente não possuí acesso cadastrado</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>6946</v>
+        <v>6907</v>
       </c>
       <c r="G300" s="1" t="inlineStr">
         <is>
-          <t>FFRA CONCRETOS LTDA</t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H300" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I300" s="1" t="inlineStr">
@@ -23853,10 +23859,10 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46223.5798869213</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>46225</v>
+        <v>46223</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
@@ -23883,51 +23889,51 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>79866</v>
+        <v>81213</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C301" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D301" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Cliente não possuí acesso cadastrado</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>6539</v>
+        <v>6946</v>
       </c>
       <c r="G301" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>FFRA CONCRETOS LTDA</t>
         </is>
       </c>
       <c r="H301" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I301" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46223.5798869213</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>46185</v>
+        <v>46225</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
@@ -23936,7 +23942,7 @@
       </c>
       <c r="M301" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N301" s="1" t="n"/>
@@ -23954,7 +23960,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>79859</v>
+        <v>79866</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
@@ -23973,15 +23979,15 @@
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>6570</v>
+        <v>6539</v>
       </c>
       <c r="G302" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H302" s="1" t="inlineStr">
@@ -23995,7 +24001,7 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K302" s="2" t="n">
         <v>46185</v>
@@ -24025,7 +24031,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>79860</v>
+        <v>79859</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
@@ -24044,15 +24050,15 @@
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
-        <v>6581</v>
+        <v>6570</v>
       </c>
       <c r="G303" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H303" s="1" t="inlineStr">
@@ -24066,7 +24072,7 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46185</v>
@@ -24096,7 +24102,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>79861</v>
+        <v>79860</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
@@ -24115,15 +24121,15 @@
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
-        <v>6583</v>
+        <v>6581</v>
       </c>
       <c r="G304" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H304" s="1" t="inlineStr">
@@ -24137,7 +24143,7 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K304" s="2" t="n">
         <v>46185</v>
@@ -24167,16 +24173,16 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>79867</v>
+        <v>79861</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C305" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D305" s="1" t="inlineStr">
@@ -24186,15 +24192,15 @@
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
-        <v>6704</v>
+        <v>6583</v>
       </c>
       <c r="G305" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H305" s="1" t="inlineStr">
@@ -24208,7 +24214,7 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K305" s="2" t="n">
         <v>46185</v>
@@ -24238,7 +24244,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>79833</v>
+        <v>79867</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
@@ -24257,15 +24263,15 @@
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>6125</v>
+        <v>6704</v>
       </c>
       <c r="G306" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H306" s="1" t="inlineStr">
@@ -24279,32 +24285,26 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N306" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N306" s="1" t="n"/>
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="n"/>
       <c r="Q306" s="1" t="inlineStr"/>
-      <c r="R306" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R306" s="1" t="inlineStr"/>
       <c r="S306" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24315,7 +24315,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>79834</v>
+        <v>79833</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
@@ -24338,11 +24338,11 @@
         </is>
       </c>
       <c r="F307" s="1" t="n">
-        <v>6162</v>
+        <v>6125</v>
       </c>
       <c r="G307" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H307" s="1" t="inlineStr">
@@ -24356,14 +24356,14 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K307" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M307" s="1" t="inlineStr">
@@ -24371,11 +24371,17 @@
           <t>Tatiana Linardi</t>
         </is>
       </c>
-      <c r="N307" s="1" t="n"/>
+      <c r="N307" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O307" s="1" t="n"/>
       <c r="P307" s="1" t="n"/>
       <c r="Q307" s="1" t="inlineStr"/>
-      <c r="R307" s="1" t="inlineStr"/>
+      <c r="R307" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S307" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24386,16 +24392,16 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>79865</v>
+        <v>79834</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C308" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D308" s="1" t="inlineStr">
@@ -24405,15 +24411,15 @@
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
-        <v>6278</v>
+        <v>6162</v>
       </c>
       <c r="G308" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H308" s="1" t="inlineStr">
@@ -24427,10 +24433,10 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K308" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L308" s="1" t="inlineStr">
         <is>
@@ -24439,7 +24445,7 @@
       </c>
       <c r="M308" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N308" s="1" t="n"/>
@@ -24457,16 +24463,16 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>81243</v>
+        <v>79865</v>
       </c>
       <c r="B309" s="1" t="inlineStr">
         <is>
-          <t>Auditoria Inversa</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C309" s="1" t="inlineStr">
         <is>
-          <t>Envio de Documentos</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D309" s="1" t="inlineStr">
@@ -24476,20 +24482,20 @@
       </c>
       <c r="E309" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A antiga contabilidade enviou a ECD do período de responsabilidade tecnica deles (01/01/2025 a 30/06/2025)  sem a inclusão de plano referencial, e para envio da ECF precisamos que essa informação seja inclusa na ECD.Precisamos que seja retificada a ECD com a inclusão do plano referencial da empresa.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F309" s="1" t="n">
-        <v>6298</v>
+        <v>6278</v>
       </c>
       <c r="G309" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">T W ALCANTARA ATACAREJO LTDA </t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H309" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I309" s="1" t="inlineStr">
@@ -24498,14 +24504,14 @@
         </is>
       </c>
       <c r="J309" s="2" t="n">
-        <v>46224.42366959491</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K309" s="2" t="n">
-        <v>46225</v>
+        <v>46185</v>
       </c>
       <c r="L309" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M309" s="1" t="inlineStr">
@@ -24513,18 +24519,11 @@
           <t>Fernanda Araujo</t>
         </is>
       </c>
-      <c r="N309" s="2" t="n">
-        <v>46225.50214903935</v>
-      </c>
+      <c r="N309" s="1" t="n"/>
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="1" t="n"/>
       <c r="Q309" s="1" t="inlineStr"/>
-      <c r="R309" s="1" t="inlineStr">
-        <is>
-          <t>Bom dia!
-Enviado a antiga contabilidade.</t>
-        </is>
-      </c>
+      <c r="R309" s="1" t="inlineStr"/>
       <c r="S309" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24535,16 +24534,16 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>79854</v>
+        <v>81243</v>
       </c>
       <c r="B310" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria Inversa</t>
         </is>
       </c>
       <c r="C310" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Envio de Documentos</t>
         </is>
       </c>
       <c r="D310" s="1" t="inlineStr">
@@ -24554,20 +24553,20 @@
       </c>
       <c r="E310" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Bom dia,A antiga contabilidade enviou a ECD do período de responsabilidade tecnica deles (01/01/2025 a 30/06/2025)  sem a inclusão de plano referencial, e para envio da ECF precisamos que essa informação seja inclusa na ECD.Precisamos que seja retificada a ECD com a inclusão do plano referencial da empresa.</t>
         </is>
       </c>
       <c r="F310" s="1" t="n">
-        <v>6302</v>
+        <v>6298</v>
       </c>
       <c r="G310" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t xml:space="preserve">T W ALCANTARA ATACAREJO LTDA </t>
         </is>
       </c>
       <c r="H310" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I310" s="1" t="inlineStr">
@@ -24576,26 +24575,33 @@
         </is>
       </c>
       <c r="J310" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46224.42366959491</v>
       </c>
       <c r="K310" s="2" t="n">
-        <v>46184</v>
+        <v>46225</v>
       </c>
       <c r="L310" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M310" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N310" s="1" t="n"/>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N310" s="2" t="n">
+        <v>46225.50214903935</v>
+      </c>
       <c r="O310" s="1" t="n"/>
       <c r="P310" s="1" t="n"/>
       <c r="Q310" s="1" t="inlineStr"/>
-      <c r="R310" s="1" t="inlineStr"/>
+      <c r="R310" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia!
+Enviado a antiga contabilidade.</t>
+        </is>
+      </c>
       <c r="S310" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24606,7 +24612,7 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>79863</v>
+        <v>79854</v>
       </c>
       <c r="B311" s="1" t="inlineStr">
         <is>
@@ -24625,15 +24631,15 @@
       </c>
       <c r="E311" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F311" s="1" t="n">
-        <v>6404</v>
+        <v>6302</v>
       </c>
       <c r="G311" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H311" s="1" t="inlineStr">
@@ -24647,10 +24653,10 @@
         </is>
       </c>
       <c r="J311" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K311" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L311" s="1" t="inlineStr">
         <is>
@@ -24659,7 +24665,7 @@
       </c>
       <c r="M311" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N311" s="1" t="n"/>
@@ -24677,16 +24683,16 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>79835</v>
+        <v>79863</v>
       </c>
       <c r="B312" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C312" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D312" s="1" t="inlineStr">
@@ -24696,15 +24702,15 @@
       </c>
       <c r="E312" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F312" s="1" t="n">
-        <v>6485</v>
+        <v>6404</v>
       </c>
       <c r="G312" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H312" s="1" t="inlineStr">
@@ -24718,10 +24724,10 @@
         </is>
       </c>
       <c r="J312" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K312" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L312" s="1" t="inlineStr">
         <is>
@@ -24730,7 +24736,7 @@
       </c>
       <c r="M312" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N312" s="1" t="n"/>
@@ -24748,16 +24754,16 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>79856</v>
+        <v>79835</v>
       </c>
       <c r="B313" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C313" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D313" s="1" t="inlineStr">
@@ -24767,15 +24773,15 @@
       </c>
       <c r="E313" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F313" s="1" t="n">
-        <v>4225</v>
+        <v>6485</v>
       </c>
       <c r="G313" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H313" s="1" t="inlineStr">
@@ -24789,7 +24795,7 @@
         </is>
       </c>
       <c r="J313" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K313" s="2" t="n">
         <v>46184</v>
@@ -24819,7 +24825,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>79855</v>
+        <v>79856</v>
       </c>
       <c r="B314" s="1" t="inlineStr">
         <is>
@@ -24838,15 +24844,15 @@
       </c>
       <c r="E314" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F314" s="1" t="n">
-        <v>4765</v>
+        <v>4225</v>
       </c>
       <c r="G314" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H314" s="1" t="inlineStr">
@@ -24860,10 +24866,10 @@
         </is>
       </c>
       <c r="J314" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K314" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L314" s="1" t="inlineStr">
         <is>
@@ -24890,35 +24896,39 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
-        <v>81244</v>
+        <v>79855</v>
       </c>
       <c r="B315" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C315" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D315" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E315" s="1" t="inlineStr">
         <is>
-          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F315" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G315" s="1" t="n"/>
+        <v>4765</v>
+      </c>
+      <c r="G315" s="1" t="inlineStr">
+        <is>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+        </is>
+      </c>
       <c r="H315" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I315" s="1" t="inlineStr">
@@ -24927,32 +24937,26 @@
         </is>
       </c>
       <c r="J315" s="2" t="n">
-        <v>46224.42615887732</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K315" s="2" t="n">
-        <v>46226</v>
+        <v>46185</v>
       </c>
       <c r="L315" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M315" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N315" s="2" t="n">
-        <v>46225.4986497338</v>
-      </c>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="N315" s="1" t="n"/>
       <c r="O315" s="1" t="n"/>
       <c r="P315" s="1" t="n"/>
       <c r="Q315" s="1" t="inlineStr"/>
-      <c r="R315" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aguardando contato do contador. </t>
-        </is>
-      </c>
+      <c r="R315" s="1" t="inlineStr"/>
       <c r="S315" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24963,7 +24967,7 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="n">
-        <v>81245</v>
+        <v>81244</v>
       </c>
       <c r="B316" s="1" t="inlineStr">
         <is>
@@ -24982,7 +24986,7 @@
       </c>
       <c r="E316" s="1" t="inlineStr">
         <is>
-          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
+          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
         </is>
       </c>
       <c r="F316" s="1" t="n">
@@ -25000,7 +25004,7 @@
         </is>
       </c>
       <c r="J316" s="2" t="n">
-        <v>46224.42947079861</v>
+        <v>46224.42615887732</v>
       </c>
       <c r="K316" s="2" t="n">
         <v>46226</v>
@@ -25016,14 +25020,14 @@
         </is>
       </c>
       <c r="N316" s="2" t="n">
-        <v>46225.4960193287</v>
+        <v>46225.4986497338</v>
       </c>
       <c r="O316" s="1" t="n"/>
       <c r="P316" s="1" t="n"/>
       <c r="Q316" s="1" t="inlineStr"/>
       <c r="R316" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobramos novamente. </t>
+          <t xml:space="preserve">Aguardando contato do contador. </t>
         </is>
       </c>
       <c r="S316" s="1" t="inlineStr">
@@ -25036,7 +25040,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>81247</v>
+        <v>81245</v>
       </c>
       <c r="B317" s="1" t="inlineStr">
         <is>
@@ -25055,7 +25059,7 @@
       </c>
       <c r="E317" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
         </is>
       </c>
       <c r="F317" s="1" t="n">
@@ -25073,7 +25077,7 @@
         </is>
       </c>
       <c r="J317" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46224.42947079861</v>
       </c>
       <c r="K317" s="2" t="n">
         <v>46226</v>
@@ -25089,14 +25093,14 @@
         </is>
       </c>
       <c r="N317" s="2" t="n">
-        <v>46225.49170355324</v>
+        <v>46225.4960193287</v>
       </c>
       <c r="O317" s="1" t="n"/>
       <c r="P317" s="1" t="n"/>
       <c r="Q317" s="1" t="inlineStr"/>
       <c r="R317" s="1" t="inlineStr">
         <is>
-          <t>Aguardando os dados do contador.</t>
+          <t xml:space="preserve">Cobramos novamente. </t>
         </is>
       </c>
       <c r="S317" s="1" t="inlineStr">
@@ -25109,7 +25113,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>81248</v>
+        <v>81247</v>
       </c>
       <c r="B318" s="1" t="inlineStr">
         <is>
@@ -25128,7 +25132,7 @@
       </c>
       <c r="E318" s="1" t="inlineStr">
         <is>
-          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F318" s="1" t="n">
@@ -25146,7 +25150,7 @@
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>46224.43289853009</v>
+        <v>46224.43143758102</v>
       </c>
       <c r="K318" s="2" t="n">
         <v>46226</v>
@@ -25162,14 +25166,14 @@
         </is>
       </c>
       <c r="N318" s="2" t="n">
-        <v>46225.48954270833</v>
+        <v>46225.49170355324</v>
       </c>
       <c r="O318" s="1" t="n"/>
       <c r="P318" s="1" t="n"/>
       <c r="Q318" s="1" t="inlineStr"/>
       <c r="R318" s="1" t="inlineStr">
         <is>
-          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+          <t>Aguardando os dados do contador.</t>
         </is>
       </c>
       <c r="S318" s="1" t="inlineStr">
@@ -25182,7 +25186,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>81215</v>
+        <v>81248</v>
       </c>
       <c r="B319" s="1" t="inlineStr">
         <is>
@@ -25201,7 +25205,7 @@
       </c>
       <c r="E319" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F319" s="1" t="n">
@@ -25219,26 +25223,32 @@
         </is>
       </c>
       <c r="J319" s="2" t="n">
-        <v>46223.60068402778</v>
+        <v>46224.43289853009</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L319" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M319" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N319" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N319" s="2" t="n">
+        <v>46225.48954270833</v>
+      </c>
       <c r="O319" s="1" t="n"/>
       <c r="P319" s="1" t="n"/>
       <c r="Q319" s="1" t="inlineStr"/>
-      <c r="R319" s="1" t="inlineStr"/>
+      <c r="R319" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+        </is>
+      </c>
       <c r="S319" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25249,7 +25259,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>81217</v>
+        <v>81215</v>
       </c>
       <c r="B320" s="1" t="inlineStr">
         <is>
@@ -25268,7 +25278,7 @@
       </c>
       <c r="E320" s="1" t="inlineStr">
         <is>
-          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F320" s="1" t="n">
@@ -25286,7 +25296,7 @@
         </is>
       </c>
       <c r="J320" s="2" t="n">
-        <v>46223.60780787037</v>
+        <v>46223.60068402778</v>
       </c>
       <c r="K320" s="2" t="n">
         <v>46225</v>
@@ -25316,7 +25326,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>81218</v>
+        <v>81217</v>
       </c>
       <c r="B321" s="1" t="inlineStr">
         <is>
@@ -25335,7 +25345,7 @@
       </c>
       <c r="E321" s="1" t="inlineStr">
         <is>
-          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F321" s="1" t="n">
@@ -25353,7 +25363,7 @@
         </is>
       </c>
       <c r="J321" s="2" t="n">
-        <v>46223.6082516551</v>
+        <v>46223.60780787037</v>
       </c>
       <c r="K321" s="2" t="n">
         <v>46225</v>
@@ -25383,7 +25393,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>81019</v>
+        <v>81218</v>
       </c>
       <c r="B322" s="1" t="inlineStr">
         <is>
@@ -25402,7 +25412,7 @@
       </c>
       <c r="E322" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
@@ -25411,7 +25421,7 @@
       <c r="G322" s="1" t="n"/>
       <c r="H322" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I322" s="1" t="inlineStr">
@@ -25420,14 +25430,14 @@
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46223.6082516551</v>
       </c>
       <c r="K322" s="2" t="n">
-        <v>46218</v>
+        <v>46225</v>
       </c>
       <c r="L322" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M322" s="1" t="inlineStr">
@@ -25439,12 +25449,7 @@
       <c r="O322" s="1" t="n"/>
       <c r="P322" s="1" t="n"/>
       <c r="Q322" s="1" t="inlineStr"/>
-      <c r="R322" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
+      <c r="R322" s="1" t="inlineStr"/>
       <c r="S322" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25455,7 +25460,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>81052</v>
+        <v>81019</v>
       </c>
       <c r="B323" s="1" t="inlineStr">
         <is>
@@ -25474,7 +25479,7 @@
       </c>
       <c r="E323" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F323" s="1" t="n">
@@ -25492,10 +25497,10 @@
         </is>
       </c>
       <c r="J323" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K323" s="2" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="L323" s="1" t="inlineStr">
         <is>
@@ -25504,7 +25509,7 @@
       </c>
       <c r="M323" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N323" s="1" t="n"/>
@@ -25513,7 +25518,8 @@
       <c r="Q323" s="1" t="inlineStr"/>
       <c r="R323" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
         </is>
       </c>
       <c r="S323" s="1" t="inlineStr">
@@ -25526,7 +25532,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>81055</v>
+        <v>81052</v>
       </c>
       <c r="B324" s="1" t="inlineStr">
         <is>
@@ -25545,7 +25551,7 @@
       </c>
       <c r="E324" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F324" s="1" t="n">
@@ -25563,14 +25569,14 @@
         </is>
       </c>
       <c r="J324" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K324" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L324" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M324" s="1" t="inlineStr">
@@ -25578,15 +25584,13 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N324" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+      <c r="N324" s="1" t="n"/>
       <c r="O324" s="1" t="n"/>
       <c r="P324" s="1" t="n"/>
       <c r="Q324" s="1" t="inlineStr"/>
       <c r="R324" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S324" s="1" t="inlineStr">
@@ -25596,6 +25600,79 @@
       </c>
       <c r="T324" s="1" t="n"/>
       <c r="U324" s="1" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="1" t="n">
+        <v>81055</v>
+      </c>
+      <c r="B325" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C325" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D325" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E325" s="1" t="inlineStr">
+        <is>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+        </is>
+      </c>
+      <c r="F325" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G325" s="1" t="n"/>
+      <c r="H325" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I325" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="n">
+        <v>46218.40379614583</v>
+      </c>
+      <c r="K325" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L325" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M325" s="1" t="inlineStr">
+        <is>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N325" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
+      <c r="O325" s="1" t="n"/>
+      <c r="P325" s="1" t="n"/>
+      <c r="Q325" s="1" t="inlineStr"/>
+      <c r="R325" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
+      <c r="S325" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T325" s="1" t="n"/>
+      <c r="U325" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 23-07-26 1347
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -9583,7 +9583,7 @@
       </c>
       <c r="L111" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M111" s="1" t="inlineStr">
@@ -9595,12 +9595,22 @@
       <c r="O111" s="2" t="n">
         <v>46226</v>
       </c>
-      <c r="P111" s="1" t="n"/>
-      <c r="Q111" s="1" t="inlineStr"/>
-      <c r="R111" s="1" t="inlineStr"/>
+      <c r="P111" s="2" t="n">
+        <v>46226.56213445602</v>
+      </c>
+      <c r="Q111" s="1" t="inlineStr">
+        <is>
+          <t>Diogo Calazans</t>
+        </is>
+      </c>
+      <c r="R111" s="1" t="inlineStr">
+        <is>
+          <t>Segue em anexo</t>
+        </is>
+      </c>
       <c r="S111" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T111" s="1" t="n"/>

</xml_diff>

<commit_message>
data: atualização base chamados 27-07-26 1002
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U391" headerRowCount="1">
-  <autoFilter ref="A1:U391"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U393" headerRowCount="1">
+  <autoFilter ref="A1:U393"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U391"/>
+  <dimension ref="A1:U393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1261,7 +1261,11 @@
         <v>0</v>
       </c>
       <c r="G10" s="1" t="n"/>
-      <c r="H10" s="1" t="n"/>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -1275,7 +1279,7 @@
       </c>
       <c r="L10" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M10" s="1" t="inlineStr">
@@ -1287,14 +1291,18 @@
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
       <c r="Q10" s="1" t="inlineStr"/>
-      <c r="R10" s="1" t="n"/>
+      <c r="R10" s="1" t="inlineStr"/>
       <c r="S10" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T10" s="1" t="n"/>
-      <c r="U10" s="1" t="inlineStr"/>
+      <c r="U10" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -8536,7 +8544,11 @@
           <t>AERODUTO EQUIPAMENTOS INDUSTRIAIS LTDA</t>
         </is>
       </c>
-      <c r="H99" s="1" t="n"/>
+      <c r="H99" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I99" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -8550,7 +8562,7 @@
       </c>
       <c r="L99" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M99" s="1" t="inlineStr">
@@ -8562,14 +8574,18 @@
       <c r="O99" s="1" t="n"/>
       <c r="P99" s="1" t="n"/>
       <c r="Q99" s="1" t="inlineStr"/>
-      <c r="R99" s="1" t="n"/>
+      <c r="R99" s="1" t="inlineStr"/>
       <c r="S99" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T99" s="1" t="n"/>
-      <c r="U99" s="1" t="inlineStr"/>
+      <c r="U99" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -9877,7 +9893,7 @@
       </c>
       <c r="L115" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M115" s="1" t="inlineStr">
@@ -9889,8 +9905,14 @@
       <c r="O115" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="P115" s="1" t="n"/>
-      <c r="Q115" s="1" t="inlineStr"/>
+      <c r="P115" s="2" t="n">
+        <v>46230.41147511574</v>
+      </c>
+      <c r="Q115" s="1" t="inlineStr">
+        <is>
+          <t>Mariana Pires</t>
+        </is>
+      </c>
       <c r="R115" s="1" t="inlineStr">
         <is>
           <t>Boa tarde, 
@@ -9899,7 +9921,7 @@
       </c>
       <c r="S115" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T115" s="1" t="n"/>
@@ -12774,7 +12796,11 @@
           <t>G13 IMPORTAÇÃO E EXPORTAÇÃO LTDA (FILIAL 3)</t>
         </is>
       </c>
-      <c r="H150" s="1" t="n"/>
+      <c r="H150" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I150" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -12788,7 +12814,7 @@
       </c>
       <c r="L150" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M150" s="1" t="inlineStr">
@@ -12800,14 +12826,18 @@
       <c r="O150" s="1" t="n"/>
       <c r="P150" s="1" t="n"/>
       <c r="Q150" s="1" t="inlineStr"/>
-      <c r="R150" s="1" t="n"/>
+      <c r="R150" s="1" t="inlineStr"/>
       <c r="S150" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T150" s="1" t="n"/>
-      <c r="U150" s="1" t="inlineStr"/>
+      <c r="U150" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -12922,7 +12952,11 @@
           <t>CAF LOG TRANSPORTES RODOVIARIOS E ARMAZENS LTDA</t>
         </is>
       </c>
-      <c r="H152" s="1" t="n"/>
+      <c r="H152" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I152" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -12936,7 +12970,7 @@
       </c>
       <c r="L152" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M152" s="1" t="inlineStr">
@@ -12948,14 +12982,18 @@
       <c r="O152" s="1" t="n"/>
       <c r="P152" s="1" t="n"/>
       <c r="Q152" s="1" t="inlineStr"/>
-      <c r="R152" s="1" t="n"/>
+      <c r="R152" s="1" t="inlineStr"/>
       <c r="S152" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T152" s="1" t="n"/>
-      <c r="U152" s="1" t="inlineStr"/>
+      <c r="U152" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -13818,7 +13856,11 @@
           <t xml:space="preserve">PLANET GRAPHICS LTDA </t>
         </is>
       </c>
-      <c r="H163" s="1" t="n"/>
+      <c r="H163" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I163" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -13832,7 +13874,7 @@
       </c>
       <c r="L163" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M163" s="1" t="inlineStr">
@@ -13844,14 +13886,18 @@
       <c r="O163" s="1" t="n"/>
       <c r="P163" s="1" t="n"/>
       <c r="Q163" s="1" t="inlineStr"/>
-      <c r="R163" s="1" t="n"/>
+      <c r="R163" s="1" t="inlineStr"/>
       <c r="S163" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T163" s="1" t="n"/>
-      <c r="U163" s="1" t="inlineStr"/>
+      <c r="U163" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -13885,7 +13931,11 @@
           <t xml:space="preserve">PLANET GRAPHICS LTDA </t>
         </is>
       </c>
-      <c r="H164" s="1" t="n"/>
+      <c r="H164" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I164" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -13899,7 +13949,7 @@
       </c>
       <c r="L164" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M164" s="1" t="inlineStr">
@@ -13911,14 +13961,18 @@
       <c r="O164" s="1" t="n"/>
       <c r="P164" s="1" t="n"/>
       <c r="Q164" s="1" t="inlineStr"/>
-      <c r="R164" s="1" t="n"/>
+      <c r="R164" s="1" t="inlineStr"/>
       <c r="S164" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T164" s="1" t="n"/>
-      <c r="U164" s="1" t="inlineStr"/>
+      <c r="U164" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -14279,7 +14333,11 @@
           <t>VALE CONCRETO LTDA</t>
         </is>
       </c>
-      <c r="H169" s="1" t="n"/>
+      <c r="H169" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I169" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14293,7 +14351,7 @@
       </c>
       <c r="L169" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M169" s="1" t="inlineStr">
@@ -14305,14 +14363,18 @@
       <c r="O169" s="1" t="n"/>
       <c r="P169" s="1" t="n"/>
       <c r="Q169" s="1" t="inlineStr"/>
-      <c r="R169" s="1" t="n"/>
+      <c r="R169" s="1" t="inlineStr"/>
       <c r="S169" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T169" s="1" t="n"/>
-      <c r="U169" s="1" t="inlineStr"/>
+      <c r="U169" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -14428,7 +14490,11 @@
           <t>PERIMETRAL SERVICOS LTDA</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n"/>
+      <c r="H171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I171" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14442,7 +14508,7 @@
       </c>
       <c r="L171" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M171" s="1" t="inlineStr">
@@ -14454,14 +14520,18 @@
       <c r="O171" s="1" t="n"/>
       <c r="P171" s="1" t="n"/>
       <c r="Q171" s="1" t="inlineStr"/>
-      <c r="R171" s="1" t="n"/>
+      <c r="R171" s="1" t="inlineStr"/>
       <c r="S171" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T171" s="1" t="n"/>
-      <c r="U171" s="1" t="inlineStr"/>
+      <c r="U171" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -14947,7 +15017,11 @@
           <t>NATURAL NUTS INDUSTRIA E COMERCIO DE ALIMENTOS LTDA (MATRIZ)</t>
         </is>
       </c>
-      <c r="H178" s="1" t="n"/>
+      <c r="H178" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I178" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -14961,7 +15035,7 @@
       </c>
       <c r="L178" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M178" s="1" t="inlineStr">
@@ -14973,14 +15047,18 @@
       <c r="O178" s="1" t="n"/>
       <c r="P178" s="1" t="n"/>
       <c r="Q178" s="1" t="inlineStr"/>
-      <c r="R178" s="1" t="n"/>
+      <c r="R178" s="1" t="inlineStr"/>
       <c r="S178" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T178" s="1" t="n"/>
-      <c r="U178" s="1" t="inlineStr"/>
+      <c r="U178" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -17896,7 +17974,11 @@
           <t>ROBSON DE SOUSA LIMA COMERCIO DE ABRASIVOS (FILIAL)</t>
         </is>
       </c>
-      <c r="H214" s="1" t="n"/>
+      <c r="H214" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="I214" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -17910,7 +17992,7 @@
       </c>
       <c r="L214" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M214" s="1" t="inlineStr">
@@ -17922,14 +18004,18 @@
       <c r="O214" s="1" t="n"/>
       <c r="P214" s="1" t="n"/>
       <c r="Q214" s="1" t="inlineStr"/>
-      <c r="R214" s="1" t="n"/>
+      <c r="R214" s="1" t="inlineStr"/>
       <c r="S214" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T214" s="1" t="n"/>
-      <c r="U214" s="1" t="inlineStr"/>
+      <c r="U214" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -22003,76 +22089,62 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>80165</v>
+        <v>81442</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Procurações DP</t>
         </is>
       </c>
       <c r="C272" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Procurações DP</t>
         </is>
       </c>
       <c r="D272" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t xml:space="preserve">6923 - JGTEC Por gentileza, habilitar função no FGTS Digital com urgência, temos uma rescisão para finalizar até 29/07. </t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G272" s="1" t="n"/>
-      <c r="H272" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H272" s="1" t="n"/>
       <c r="I272" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46190.71175925926</v>
+        <v>46230.40592804398</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46191</v>
+        <v>46231</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
       <c r="O272" s="1" t="n"/>
-      <c r="P272" s="2" t="n">
-        <v>46190.7346272338</v>
-      </c>
-      <c r="Q272" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
-      <c r="R272" s="1" t="inlineStr">
-        <is>
-          <t>Tarefas baixadas</t>
-        </is>
-      </c>
+      <c r="P272" s="1" t="n"/>
+      <c r="Q272" s="1" t="inlineStr"/>
+      <c r="R272" s="1" t="n"/>
       <c r="S272" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T272" s="1" t="n"/>
@@ -22080,7 +22152,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>80174</v>
+        <v>80165</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22089,7 +22161,7 @@
       </c>
       <c r="C273" s="1" t="inlineStr">
         <is>
-          <t>Vencimento de Tarefas</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D273" s="1" t="inlineStr">
@@ -22099,7 +22171,7 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
@@ -22117,10 +22189,10 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46191.36721832176</v>
+        <v>46190.71175925926</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="L273" s="1" t="inlineStr">
         <is>
@@ -22129,13 +22201,13 @@
       </c>
       <c r="M273" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N273" s="1" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="2" t="n">
-        <v>46191.49335512731</v>
+        <v>46190.7346272338</v>
       </c>
       <c r="Q273" s="1" t="inlineStr">
         <is>
@@ -22157,7 +22229,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>80250</v>
+        <v>80174</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22166,7 +22238,7 @@
       </c>
       <c r="C274" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Vencimento de Tarefas</t>
         </is>
       </c>
       <c r="D274" s="1" t="inlineStr">
@@ -22176,7 +22248,7 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
+          <t>Bom dia prezados!Por gentileza dar baixa na tarefa DEC 1 Consulta, pois não possui inscrição estadual.6091 - CARTAO DE TODOS ITAPETININGA LTDA6093 - CARTAO DE TODOS ADMINISTRADORA E VENDAS LTDA6094 - CLINICA SAUDE &amp; VIDA LTDA6095 - N S ACADEMIA SOROCABA VILA CARVALHO LTDA6096 - CLINICA SAUDE &amp; VIDA LTDA (FILIAL)6330 - ADM SERVICE ITAPETININGA E BOTUCATU LTDA6391 - ADMINISTRADORA ACADEMIA ALLPFIT LTDA6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA6371 - CLUBE ATLETICO INDIANO6383 - THSAVEG ASSESSORIA EMPRESARIAL LTDA6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6419 - QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA (FILIAL 1)6359 - MACHADO PRESTACAO DE SERVICOS LTDA1861 - S &amp; B MARKETING E COMUNICAÇÃO VISUAL LTDA6579 - DROGARIA MIX I LTDA (FILIAL 9)3293 - SUPERMERCADO NELSINHO3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
@@ -22194,21 +22266,25 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46192.6584477662</v>
+        <v>46191.36721832176</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>46195</v>
+        <v>46192</v>
       </c>
       <c r="L274" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M274" s="1" t="n"/>
+      <c r="M274" s="1" t="inlineStr">
+        <is>
+          <t>Yasmin Peixoto</t>
+        </is>
+      </c>
       <c r="N274" s="1" t="n"/>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="2" t="n">
-        <v>46192.70597966435</v>
+        <v>46191.49335512731</v>
       </c>
       <c r="Q274" s="1" t="inlineStr">
         <is>
@@ -22230,7 +22306,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>80709</v>
+        <v>80250</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22249,7 +22325,7 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
@@ -22267,25 +22343,21 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46205.72485570602</v>
+        <v>46192.6584477662</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>46206</v>
+        <v>46195</v>
       </c>
       <c r="L275" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M275" s="1" t="inlineStr">
-        <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
+      <c r="M275" s="1" t="n"/>
       <c r="N275" s="1" t="n"/>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="2" t="n">
-        <v>46205.73248877314</v>
+        <v>46192.70597966435</v>
       </c>
       <c r="Q275" s="1" t="inlineStr">
         <is>
@@ -22307,7 +22379,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>81083</v>
+        <v>80709</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22326,7 +22398,7 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
@@ -22344,10 +22416,10 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46218.68119872685</v>
+        <v>46205.72485570602</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>46219</v>
+        <v>46206</v>
       </c>
       <c r="L276" s="1" t="inlineStr">
         <is>
@@ -22362,7 +22434,7 @@
       <c r="N276" s="1" t="n"/>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="2" t="n">
-        <v>46218.7466727662</v>
+        <v>46205.73248877314</v>
       </c>
       <c r="Q276" s="1" t="inlineStr">
         <is>
@@ -22371,7 +22443,7 @@
       </c>
       <c r="R276" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+          <t>Tarefas baixadas</t>
         </is>
       </c>
       <c r="S276" s="1" t="inlineStr">
@@ -22384,7 +22456,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>81269</v>
+        <v>81083</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22393,7 +22465,7 @@
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Vencimento de Tarefas</t>
+          <t>Erro de Baixa</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22403,7 +22475,7 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde prezados!!Por gentileza, baixar a tarefa do DEC 2 quinzena 07/2026 das seguintes empresas, pois não possui inscrição estadual.6371 - CLUBE ATLETICO INDIANO6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
@@ -22421,10 +22493,10 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46224.67642369213</v>
+        <v>46218.68119872685</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>46225</v>
+        <v>46219</v>
       </c>
       <c r="L277" s="1" t="inlineStr">
         <is>
@@ -22433,13 +22505,13 @@
       </c>
       <c r="M277" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N277" s="1" t="n"/>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="2" t="n">
-        <v>46224.68052071759</v>
+        <v>46218.7466727662</v>
       </c>
       <c r="Q277" s="1" t="inlineStr">
         <is>
@@ -22448,7 +22520,7 @@
       </c>
       <c r="R277" s="1" t="inlineStr">
         <is>
-          <t>Tarefas baixadas</t>
+          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
         </is>
       </c>
       <c r="S277" s="1" t="inlineStr">
@@ -22461,7 +22533,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>81279</v>
+        <v>81269</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
@@ -22480,7 +22552,7 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde prezados!!Por gentileza, baixar a tarefa do DEC 2 quinzena 07/2026 das seguintes empresas, pois não possui inscrição estadual.6579 - DROGARIA MIX I LTDA (FILIAL 9)3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
+          <t>Boa tarde prezados!!Por gentileza, baixar a tarefa do DEC 2 quinzena 07/2026 das seguintes empresas, pois não possui inscrição estadual.6371 - CLUBE ATLETICO INDIANO6482 - RRW DISTRIBUIDORA E IMPORTADORA DE PECAS LTDA (FILIAL 1)6556 - CLINICA MEDICA E ODONTOLOGICA AMOR SAUDE BOTUCATU LTDA</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
@@ -22498,7 +22570,7 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46224.74851809028</v>
+        <v>46224.67642369213</v>
       </c>
       <c r="K278" s="2" t="n">
         <v>46225</v>
@@ -22516,7 +22588,7 @@
       <c r="N278" s="1" t="n"/>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="2" t="n">
-        <v>46224.75336643519</v>
+        <v>46224.68052071759</v>
       </c>
       <c r="Q278" s="1" t="inlineStr">
         <is>
@@ -22538,7 +22610,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>81287</v>
+        <v>81279</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
@@ -22547,7 +22619,7 @@
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Envio de Impostos</t>
+          <t>Vencimento de Tarefas</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
@@ -22557,7 +22629,7 @@
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Prezados, bom dia!Peço, por gentileza, que removam as tarefas de impostos das empresas abaixo, pois elas são de responsabilidade da secretária Ana Santana:1286 – BY ENGENHARIA IMPORTAÇÃO E EXPORTAÇÃO LTDA (MATRIZ)2023 – Stantuer Participações Ltda.2576 – P.E. Latina Máquinas para Rotulagem Ltda.2888 – Associação Novo Sentido3499 – Emplaca Automação e Tecnologia Ltda.Além disso, peço que sejam removidas todas as tarefas das demais empresas sob responsabilidade da secretária Ana Santana. Para facilitar a identificação, segue em anexo a relação completa de clientes.</t>
+          <t>Boa tarde prezados!!Por gentileza, baixar a tarefa do DEC 2 quinzena 07/2026 das seguintes empresas, pois não possui inscrição estadual.6579 - DROGARIA MIX I LTDA (FILIAL 9)3465 - Vicali Administração, Participações e Investimentos Ltda.</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22575,10 +22647,10 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46225.39240945602</v>
+        <v>46224.74851809028</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
@@ -22587,13 +22659,13 @@
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="2" t="n">
-        <v>46225.63002103009</v>
+        <v>46224.75336643519</v>
       </c>
       <c r="Q279" s="1" t="inlineStr">
         <is>
@@ -22602,7 +22674,7 @@
       </c>
       <c r="R279" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, as tarefas de impostos não devem ser excluidas e sim transferidas entre responsaveis, por gentileza caso tenha alguma duvida procurar o Juan</t>
+          <t>Tarefas baixadas</t>
         </is>
       </c>
       <c r="S279" s="1" t="inlineStr">
@@ -22615,36 +22687,32 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>81406</v>
+        <v>81287</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
-          <t>Sistema de Análise</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Radar</t>
+          <t>Envio de Impostos</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>Por favor, verifiquei com o TI sobre um problema no Sys Analise de junho/2026 referente ao cliente 2271 e eles me orientaram abrir um chamado com vocês para alterar esse cliente/matriz (1331) para que possa usar Sistema de Analise, pois subiu essa empresa no Radar e não consigo finalizar esse fechamento.Podem verificar, por favor?</t>
+          <t>Prezados, bom dia!Peço, por gentileza, que removam as tarefas de impostos das empresas abaixo, pois elas são de responsabilidade da secretária Ana Santana:1286 – BY ENGENHARIA IMPORTAÇÃO E EXPORTAÇÃO LTDA (MATRIZ)2023 – Stantuer Participações Ltda.2576 – P.E. Latina Máquinas para Rotulagem Ltda.2888 – Associação Novo Sentido3499 – Emplaca Automação e Tecnologia Ltda.Além disso, peço que sejam removidas todas as tarefas das demais empresas sob responsabilidade da secretária Ana Santana. Para facilitar a identificação, segue em anexo a relação completa de clientes.</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>2271</v>
-      </c>
-      <c r="G280" s="1" t="inlineStr">
-        <is>
-          <t>Supermercado Alta Rotação Ltda (Filial 3)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
           <t>Gabriel Amaral</t>
@@ -22656,10 +22724,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46226.58671964121</v>
+        <v>46225.39240945602</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22668,13 +22736,13 @@
       </c>
       <c r="M280" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="N280" s="1" t="n"/>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="2" t="n">
-        <v>46230.37486076389</v>
+        <v>46225.63002103009</v>
       </c>
       <c r="Q280" s="1" t="inlineStr">
         <is>
@@ -22683,7 +22751,7 @@
       </c>
       <c r="R280" s="1" t="inlineStr">
         <is>
-          <t>Filial ajustada</t>
+          <t>Bom dia, as tarefas de impostos não devem ser excluidas e sim transferidas entre responsaveis, por gentileza caso tenha alguma duvida procurar o Juan</t>
         </is>
       </c>
       <c r="S280" s="1" t="inlineStr">
@@ -22696,32 +22764,36 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>81438</v>
+        <v>81406</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Sistema de Análise</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Chamados</t>
+          <t>Radar</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
         <is>
-          <t>B.P.O. - GUARANI CTB</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>por gentileza pode baixar a tarefa do MIT das empresas em anexo - 4059 ,4065, 4066, 4067 ,4068, 4602 ,4815</t>
+          <t>Por favor, verifiquei com o TI sobre um problema no Sys Analise de junho/2026 referente ao cliente 2271 e eles me orientaram abrir um chamado com vocês para alterar esse cliente/matriz (1331) para que possa usar Sistema de Analise, pois subiu essa empresa no Radar e não consigo finalizar esse fechamento.Podem verificar, por favor?</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G281" s="1" t="n"/>
+        <v>2271</v>
+      </c>
+      <c r="G281" s="1" t="inlineStr">
+        <is>
+          <t>Supermercado Alta Rotação Ltda (Filial 3)</t>
+        </is>
+      </c>
       <c r="H281" s="1" t="inlineStr">
         <is>
           <t>Gabriel Amaral</t>
@@ -22733,29 +22805,39 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46230.34684741898</v>
+        <v>46226.58671964121</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M281" s="1" t="inlineStr">
         <is>
-          <t>Flavia Dariolli</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N281" s="1" t="n"/>
       <c r="O281" s="1" t="n"/>
-      <c r="P281" s="1" t="n"/>
-      <c r="Q281" s="1" t="inlineStr"/>
-      <c r="R281" s="1" t="inlineStr"/>
+      <c r="P281" s="2" t="n">
+        <v>46230.37486076389</v>
+      </c>
+      <c r="Q281" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
+      <c r="R281" s="1" t="inlineStr">
+        <is>
+          <t>Filial ajustada</t>
+        </is>
+      </c>
       <c r="S281" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T281" s="1" t="n"/>
@@ -25595,7 +25677,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>81247</v>
+        <v>81248</v>
       </c>
       <c r="B321" s="1" t="inlineStr">
         <is>
@@ -25614,7 +25696,7 @@
       </c>
       <c r="E321" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F321" s="1" t="n">
@@ -25632,7 +25714,7 @@
         </is>
       </c>
       <c r="J321" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46224.43289853009</v>
       </c>
       <c r="K321" s="2" t="n">
         <v>46226</v>
@@ -25648,14 +25730,14 @@
         </is>
       </c>
       <c r="N321" s="2" t="n">
-        <v>46225.49170355324</v>
+        <v>46225.48954270833</v>
       </c>
       <c r="O321" s="1" t="n"/>
       <c r="P321" s="1" t="n"/>
       <c r="Q321" s="1" t="inlineStr"/>
       <c r="R321" s="1" t="inlineStr">
         <is>
-          <t>Aguardando os dados do contador.</t>
+          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
         </is>
       </c>
       <c r="S321" s="1" t="inlineStr">
@@ -25668,26 +25750,26 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>81248</v>
+        <v>81250</v>
       </c>
       <c r="B322" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C322" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D322" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E322" s="1" t="inlineStr">
         <is>
-          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
@@ -25696,41 +25778,35 @@
       <c r="G322" s="1" t="n"/>
       <c r="H322" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I322" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>46224.43289853009</v>
+        <v>46224.44502184028</v>
       </c>
       <c r="K322" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L322" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M322" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N322" s="2" t="n">
-        <v>46225.48954270833</v>
-      </c>
+          <t>Rafaella Massuia</t>
+        </is>
+      </c>
+      <c r="N322" s="1" t="n"/>
       <c r="O322" s="1" t="n"/>
       <c r="P322" s="1" t="n"/>
       <c r="Q322" s="1" t="inlineStr"/>
-      <c r="R322" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
-        </is>
-      </c>
+      <c r="R322" s="1" t="inlineStr"/>
       <c r="S322" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25741,7 +25817,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>81250</v>
+        <v>81251</v>
       </c>
       <c r="B323" s="1" t="inlineStr">
         <is>
@@ -25760,7 +25836,7 @@
       </c>
       <c r="E323" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
+          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
         </is>
       </c>
       <c r="F323" s="1" t="n">
@@ -25778,7 +25854,7 @@
         </is>
       </c>
       <c r="J323" s="2" t="n">
-        <v>46224.44502184028</v>
+        <v>46224.44796296296</v>
       </c>
       <c r="K323" s="2" t="n">
         <v>46226</v>
@@ -25808,26 +25884,26 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>81251</v>
+        <v>81267</v>
       </c>
       <c r="B324" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C324" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D324" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E324" s="1" t="inlineStr">
         <is>
-          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
+          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
         </is>
       </c>
       <c r="F324" s="1" t="n">
@@ -25845,10 +25921,10 @@
         </is>
       </c>
       <c r="J324" s="2" t="n">
-        <v>46224.44796296296</v>
+        <v>46224.66958634259</v>
       </c>
       <c r="K324" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L324" s="1" t="inlineStr">
         <is>
@@ -25857,7 +25933,7 @@
       </c>
       <c r="M324" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N324" s="1" t="n"/>
@@ -25875,63 +25951,63 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>81267</v>
+        <v>81270</v>
       </c>
       <c r="B325" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C325" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D325" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E325" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
+          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
         </is>
       </c>
       <c r="F325" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G325" s="1" t="n"/>
-      <c r="H325" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+        <v>5604</v>
+      </c>
+      <c r="G325" s="1" t="inlineStr">
+        <is>
+          <t>GRAFICA TABOAO LTDA</t>
+        </is>
+      </c>
+      <c r="H325" s="1" t="n"/>
       <c r="I325" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J325" s="2" t="n">
-        <v>46224.66958634259</v>
+        <v>46224.69047569444</v>
       </c>
       <c r="K325" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="L325" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M325" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N325" s="1" t="n"/>
       <c r="O325" s="1" t="n"/>
       <c r="P325" s="1" t="n"/>
       <c r="Q325" s="1" t="inlineStr"/>
-      <c r="R325" s="1" t="inlineStr"/>
+      <c r="R325" s="1" t="n"/>
       <c r="S325" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25942,36 +26018,32 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>81270</v>
+        <v>81274</v>
       </c>
       <c r="B326" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C326" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D326" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E326" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
+          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
         </is>
       </c>
       <c r="F326" s="1" t="n">
-        <v>5604</v>
-      </c>
-      <c r="G326" s="1" t="inlineStr">
-        <is>
-          <t>GRAFICA TABOAO LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G326" s="1" t="n"/>
       <c r="H326" s="1" t="n"/>
       <c r="I326" s="1" t="inlineStr">
         <is>
@@ -25979,10 +26051,10 @@
         </is>
       </c>
       <c r="J326" s="2" t="n">
-        <v>46224.69047569444</v>
+        <v>46224.71483579861</v>
       </c>
       <c r="K326" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L326" s="1" t="inlineStr">
         <is>
@@ -25991,7 +26063,7 @@
       </c>
       <c r="M326" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N326" s="1" t="n"/>
@@ -26009,7 +26081,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>81274</v>
+        <v>81294</v>
       </c>
       <c r="B327" s="1" t="inlineStr">
         <is>
@@ -26023,12 +26095,12 @@
       </c>
       <c r="D327" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E327" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
+          <t xml:space="preserve">Solicito novo acesso da prefeitura de Holambra das empresas 3705 e 4216 </t>
         </is>
       </c>
       <c r="F327" s="1" t="n">
@@ -26042,10 +26114,10 @@
         </is>
       </c>
       <c r="J327" s="2" t="n">
-        <v>46224.71483579861</v>
+        <v>46225.47387288194</v>
       </c>
       <c r="K327" s="2" t="n">
-        <v>46226</v>
+        <v>46230</v>
       </c>
       <c r="L327" s="1" t="inlineStr">
         <is>
@@ -26054,7 +26126,7 @@
       </c>
       <c r="M327" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Shofia Gomes</t>
         </is>
       </c>
       <c r="N327" s="1" t="n"/>
@@ -26072,26 +26144,26 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>81294</v>
+        <v>81296</v>
       </c>
       <c r="B328" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C328" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras Cláusulas</t>
         </is>
       </c>
       <c r="D328" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E328" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solicito novo acesso da prefeitura de Holambra das empresas 3705 e 4216 </t>
+          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
         </is>
       </c>
       <c r="F328" s="1" t="n">
@@ -26105,10 +26177,10 @@
         </is>
       </c>
       <c r="J328" s="2" t="n">
-        <v>46225.47387288194</v>
+        <v>46225.4866127662</v>
       </c>
       <c r="K328" s="2" t="n">
-        <v>46230</v>
+        <v>46255</v>
       </c>
       <c r="L328" s="1" t="inlineStr">
         <is>
@@ -26117,7 +26189,7 @@
       </c>
       <c r="M328" s="1" t="inlineStr">
         <is>
-          <t>Shofia Gomes</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N328" s="1" t="n"/>
@@ -26135,32 +26207,36 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>81296</v>
+        <v>81297</v>
       </c>
       <c r="B329" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C329" s="1" t="inlineStr">
         <is>
-          <t>Outras Cláusulas</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D329" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E329" s="1" t="inlineStr">
         <is>
-          <t>Providenciar a inclusão do CNAE descrito abaixo na empresa.8630-5/03 - ATIVIDADE MÉDICA AMBULATORIAL RESTRITA A CONSULTAS.Ela irá prestar serviços médicos como Pessoa Jurídica, para Hospitais, UBS, Clínicas e Eventos, conforme encaminhamento da resposta dela, pelo WhatsApp.Valor será o mesmo da última alteração do grupo.</t>
+          <t>Bom dia!Ao acessar o posto fiscal está trazendo uma tela de cadastro, e não permiti acessar sem o preenchimento das informações cadastrais da empresa.</t>
         </is>
       </c>
       <c r="F329" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G329" s="1" t="n"/>
+        <v>6777</v>
+      </c>
+      <c r="G329" s="1" t="inlineStr">
+        <is>
+          <t>A. DE S. JANOCA MERCADO</t>
+        </is>
+      </c>
       <c r="H329" s="1" t="n"/>
       <c r="I329" s="1" t="inlineStr">
         <is>
@@ -26168,10 +26244,10 @@
         </is>
       </c>
       <c r="J329" s="2" t="n">
-        <v>46225.4866127662</v>
+        <v>46225.48669829861</v>
       </c>
       <c r="K329" s="2" t="n">
-        <v>46255</v>
+        <v>46226</v>
       </c>
       <c r="L329" s="1" t="inlineStr">
         <is>
@@ -26180,7 +26256,7 @@
       </c>
       <c r="M329" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Clara Maria</t>
         </is>
       </c>
       <c r="N329" s="1" t="n"/>
@@ -26198,16 +26274,16 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>81297</v>
+        <v>81316</v>
       </c>
       <c r="B330" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C330" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t xml:space="preserve">Inclusão de Ata </t>
         </is>
       </c>
       <c r="D330" s="1" t="inlineStr">
@@ -26217,15 +26293,15 @@
       </c>
       <c r="E330" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Ao acessar o posto fiscal está trazendo uma tela de cadastro, e não permiti acessar sem o preenchimento das informações cadastrais da empresa.</t>
+          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
         </is>
       </c>
       <c r="F330" s="1" t="n">
-        <v>6777</v>
+        <v>6674</v>
       </c>
       <c r="G330" s="1" t="inlineStr">
         <is>
-          <t>A. DE S. JANOCA MERCADO</t>
+          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
         </is>
       </c>
       <c r="H330" s="1" t="n"/>
@@ -26235,10 +26311,10 @@
         </is>
       </c>
       <c r="J330" s="2" t="n">
-        <v>46225.48669829861</v>
+        <v>46225.61705821759</v>
       </c>
       <c r="K330" s="2" t="n">
-        <v>46226</v>
+        <v>46231</v>
       </c>
       <c r="L330" s="1" t="inlineStr">
         <is>
@@ -26247,7 +26323,7 @@
       </c>
       <c r="M330" s="1" t="inlineStr">
         <is>
-          <t>Clara Maria</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="N330" s="1" t="n"/>
@@ -26265,7 +26341,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>81316</v>
+        <v>81317</v>
       </c>
       <c r="B331" s="1" t="inlineStr">
         <is>
@@ -26284,15 +26360,15 @@
       </c>
       <c r="E331" s="1" t="inlineStr">
         <is>
-          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
+          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
         </is>
       </c>
       <c r="F331" s="1" t="n">
-        <v>6674</v>
+        <v>6673</v>
       </c>
       <c r="G331" s="1" t="inlineStr">
         <is>
-          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
+          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
         </is>
       </c>
       <c r="H331" s="1" t="n"/>
@@ -26302,7 +26378,7 @@
         </is>
       </c>
       <c r="J331" s="2" t="n">
-        <v>46225.61705821759</v>
+        <v>46225.61752997685</v>
       </c>
       <c r="K331" s="2" t="n">
         <v>46231</v>
@@ -26332,16 +26408,16 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>81317</v>
+        <v>81322</v>
       </c>
       <c r="B332" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Levantamento de Débitos</t>
         </is>
       </c>
       <c r="C332" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inclusão de Ata </t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="D332" s="1" t="inlineStr">
@@ -26351,17 +26427,13 @@
       </c>
       <c r="E332" s="1" t="inlineStr">
         <is>
-          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
+          <t>Prezados, boa tarde!Conforme solicitação do cliente, peço a gentileza de verificar os seguintes pontos:Há parcelamentos e impostos com vencimento até o final deste mês. O cliente solicita verificar a possibilidade de emitir as guias com vencimentos para o dia 31.Solicita também a verificação da existência de eventuais débitos inscritos no CADIN.Em relação ao CADIN, foi identificado um débito que já foi quitado. No entanto, o banco informou que a baixa ainda não consta no sistema. Acreditamos que se trate apenas do prazo de atualização das informações.Peço, por gentileza, que o retorno seja encaminhado também para o e-mail do cliente: nanasupermercado@gmail.com.</t>
         </is>
       </c>
       <c r="F332" s="1" t="n">
-        <v>6673</v>
-      </c>
-      <c r="G332" s="1" t="inlineStr">
-        <is>
-          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G332" s="1" t="n"/>
       <c r="H332" s="1" t="n"/>
       <c r="I332" s="1" t="inlineStr">
         <is>
@@ -26369,10 +26441,10 @@
         </is>
       </c>
       <c r="J332" s="2" t="n">
-        <v>46225.61752997685</v>
+        <v>46225.63980702547</v>
       </c>
       <c r="K332" s="2" t="n">
-        <v>46231</v>
+        <v>46226</v>
       </c>
       <c r="L332" s="1" t="inlineStr">
         <is>
@@ -26381,7 +26453,7 @@
       </c>
       <c r="M332" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N332" s="1" t="n"/>
@@ -26399,32 +26471,36 @@
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
-        <v>81322</v>
+        <v>81343</v>
       </c>
       <c r="B333" s="1" t="inlineStr">
         <is>
-          <t>Levantamento de Débitos</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C333" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Protestos</t>
         </is>
       </c>
       <c r="D333" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E333" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!Conforme solicitação do cliente, peço a gentileza de verificar os seguintes pontos:Há parcelamentos e impostos com vencimento até o final deste mês. O cliente solicita verificar a possibilidade de emitir as guias com vencimentos para o dia 31.Solicita também a verificação da existência de eventuais débitos inscritos no CADIN.Em relação ao CADIN, foi identificado um débito que já foi quitado. No entanto, o banco informou que a baixa ainda não consta no sistema. Acreditamos que se trate apenas do prazo de atualização das informações.Peço, por gentileza, que o retorno seja encaminhado também para o e-mail do cliente: nanasupermercado@gmail.com.</t>
+          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
         </is>
       </c>
       <c r="F333" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G333" s="1" t="n"/>
+        <v>6538</v>
+      </c>
+      <c r="G333" s="1" t="inlineStr">
+        <is>
+          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+        </is>
+      </c>
       <c r="H333" s="1" t="n"/>
       <c r="I333" s="1" t="inlineStr">
         <is>
@@ -26432,10 +26508,10 @@
         </is>
       </c>
       <c r="J333" s="2" t="n">
-        <v>46225.63980702547</v>
+        <v>46225.78787369213</v>
       </c>
       <c r="K333" s="2" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="L333" s="1" t="inlineStr">
         <is>
@@ -26444,7 +26520,7 @@
       </c>
       <c r="M333" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N333" s="1" t="n"/>
@@ -26462,16 +26538,16 @@
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
-        <v>81343</v>
+        <v>81347</v>
       </c>
       <c r="B334" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C334" s="1" t="inlineStr">
         <is>
-          <t>Protestos</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D334" s="1" t="inlineStr">
@@ -26481,15 +26557,15 @@
       </c>
       <c r="E334" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
+          <t>Por favor, o cliente está pedindo a verificação do comunicado em anexo, referente a TFE de 2017.</t>
         </is>
       </c>
       <c r="F334" s="1" t="n">
-        <v>6538</v>
+        <v>2264</v>
       </c>
       <c r="G334" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+          <t>Centro de Distribuição Butantã Ltda.</t>
         </is>
       </c>
       <c r="H334" s="1" t="n"/>
@@ -26499,7 +26575,7 @@
         </is>
       </c>
       <c r="J334" s="2" t="n">
-        <v>46225.78787369213</v>
+        <v>46226.40158105324</v>
       </c>
       <c r="K334" s="2" t="n">
         <v>46227</v>
@@ -26511,7 +26587,7 @@
       </c>
       <c r="M334" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N334" s="1" t="n"/>
@@ -26529,44 +26605,40 @@
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
-        <v>81347</v>
+        <v>81348</v>
       </c>
       <c r="B335" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C335" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D335" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E335" s="1" t="inlineStr">
         <is>
-          <t>Por favor, o cliente está pedindo a verificação do comunicado em anexo, referente a TFE de 2017.</t>
+          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
         </is>
       </c>
       <c r="F335" s="1" t="n">
-        <v>2264</v>
-      </c>
-      <c r="G335" s="1" t="inlineStr">
-        <is>
-          <t>Centro de Distribuição Butantã Ltda.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G335" s="1" t="n"/>
       <c r="H335" s="1" t="n"/>
       <c r="I335" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J335" s="2" t="n">
-        <v>46226.40158105324</v>
+        <v>46226.4148858449</v>
       </c>
       <c r="K335" s="2" t="n">
         <v>46227</v>
@@ -26578,7 +26650,7 @@
       </c>
       <c r="M335" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="N335" s="1" t="n"/>
@@ -26596,43 +26668,47 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>81348</v>
+        <v>81351</v>
       </c>
       <c r="B336" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C336" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D336" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E336" s="1" t="inlineStr">
         <is>
-          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F336" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G336" s="1" t="n"/>
+        <v>3587</v>
+      </c>
+      <c r="G336" s="1" t="inlineStr">
+        <is>
+          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
+        </is>
+      </c>
       <c r="H336" s="1" t="n"/>
       <c r="I336" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J336" s="2" t="n">
-        <v>46226.4148858449</v>
+        <v>46226.44303796296</v>
       </c>
       <c r="K336" s="2" t="n">
-        <v>46227</v>
+        <v>46230</v>
       </c>
       <c r="L336" s="1" t="inlineStr">
         <is>
@@ -26641,7 +26717,7 @@
       </c>
       <c r="M336" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N336" s="1" t="n"/>
@@ -26659,7 +26735,7 @@
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
-        <v>81351</v>
+        <v>81352</v>
       </c>
       <c r="B337" s="1" t="inlineStr">
         <is>
@@ -26682,11 +26758,11 @@
         </is>
       </c>
       <c r="F337" s="1" t="n">
-        <v>3587</v>
+        <v>3812</v>
       </c>
       <c r="G337" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
         </is>
       </c>
       <c r="H337" s="1" t="n"/>
@@ -26696,7 +26772,7 @@
         </is>
       </c>
       <c r="J337" s="2" t="n">
-        <v>46226.44303796296</v>
+        <v>46226.4440716088</v>
       </c>
       <c r="K337" s="2" t="n">
         <v>46230</v>
@@ -26726,7 +26802,7 @@
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
-        <v>81352</v>
+        <v>81353</v>
       </c>
       <c r="B338" s="1" t="inlineStr">
         <is>
@@ -26749,11 +26825,11 @@
         </is>
       </c>
       <c r="F338" s="1" t="n">
-        <v>3812</v>
+        <v>3878</v>
       </c>
       <c r="G338" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
+          <t xml:space="preserve">Cucinare Pro Alimentação </t>
         </is>
       </c>
       <c r="H338" s="1" t="n"/>
@@ -26763,7 +26839,7 @@
         </is>
       </c>
       <c r="J338" s="2" t="n">
-        <v>46226.4440716088</v>
+        <v>46226.44431542824</v>
       </c>
       <c r="K338" s="2" t="n">
         <v>46230</v>
@@ -26793,7 +26869,7 @@
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
-        <v>81353</v>
+        <v>81354</v>
       </c>
       <c r="B339" s="1" t="inlineStr">
         <is>
@@ -26812,17 +26888,13 @@
       </c>
       <c r="E339" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.6421 - DISTRIBUIDORA DE FRUTAS, VERDURAS E LEGUMES CHEGUEI BRASIL LTDA</t>
         </is>
       </c>
       <c r="F339" s="1" t="n">
-        <v>3878</v>
-      </c>
-      <c r="G339" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cucinare Pro Alimentação </t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G339" s="1" t="n"/>
       <c r="H339" s="1" t="n"/>
       <c r="I339" s="1" t="inlineStr">
         <is>
@@ -26830,7 +26902,7 @@
         </is>
       </c>
       <c r="J339" s="2" t="n">
-        <v>46226.44431542824</v>
+        <v>46226.44464961805</v>
       </c>
       <c r="K339" s="2" t="n">
         <v>46230</v>
@@ -26842,7 +26914,7 @@
       </c>
       <c r="M339" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Regiane Santos</t>
         </is>
       </c>
       <c r="N339" s="1" t="n"/>
@@ -26860,7 +26932,7 @@
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
-        <v>81354</v>
+        <v>81355</v>
       </c>
       <c r="B340" s="1" t="inlineStr">
         <is>
@@ -26879,13 +26951,17 @@
       </c>
       <c r="E340" s="1" t="inlineStr">
         <is>
-          <t>Bom Dia, Por favorPreciso da nova senha para acesso ao novo portal GissOnline das lojas abaixo.6421 - DISTRIBUIDORA DE FRUTAS, VERDURAS E LEGUMES CHEGUEI BRASIL LTDA</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F340" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G340" s="1" t="n"/>
+        <v>4012</v>
+      </c>
+      <c r="G340" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+        </is>
+      </c>
       <c r="H340" s="1" t="n"/>
       <c r="I340" s="1" t="inlineStr">
         <is>
@@ -26893,7 +26969,7 @@
         </is>
       </c>
       <c r="J340" s="2" t="n">
-        <v>46226.44464961805</v>
+        <v>46226.44472357639</v>
       </c>
       <c r="K340" s="2" t="n">
         <v>46230</v>
@@ -26905,7 +26981,7 @@
       </c>
       <c r="M340" s="1" t="inlineStr">
         <is>
-          <t>Regiane Santos</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N340" s="1" t="n"/>
@@ -26923,7 +26999,7 @@
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
-        <v>81355</v>
+        <v>81356</v>
       </c>
       <c r="B341" s="1" t="inlineStr">
         <is>
@@ -26946,11 +27022,11 @@
         </is>
       </c>
       <c r="F341" s="1" t="n">
-        <v>4012</v>
+        <v>4013</v>
       </c>
       <c r="G341" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
         </is>
       </c>
       <c r="H341" s="1" t="n"/>
@@ -26960,7 +27036,7 @@
         </is>
       </c>
       <c r="J341" s="2" t="n">
-        <v>46226.44472357639</v>
+        <v>46226.445571875</v>
       </c>
       <c r="K341" s="2" t="n">
         <v>46230</v>
@@ -26990,7 +27066,7 @@
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
-        <v>81356</v>
+        <v>81357</v>
       </c>
       <c r="B342" s="1" t="inlineStr">
         <is>
@@ -27013,11 +27089,11 @@
         </is>
       </c>
       <c r="F342" s="1" t="n">
-        <v>4013</v>
+        <v>4015</v>
       </c>
       <c r="G342" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
+          <t>Cucinare Pro Alimentaçao ( FL 53)</t>
         </is>
       </c>
       <c r="H342" s="1" t="n"/>
@@ -27027,7 +27103,7 @@
         </is>
       </c>
       <c r="J342" s="2" t="n">
-        <v>46226.445571875</v>
+        <v>46226.44603434028</v>
       </c>
       <c r="K342" s="2" t="n">
         <v>46230</v>
@@ -27057,7 +27133,7 @@
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
-        <v>81357</v>
+        <v>81358</v>
       </c>
       <c r="B343" s="1" t="inlineStr">
         <is>
@@ -27080,11 +27156,11 @@
         </is>
       </c>
       <c r="F343" s="1" t="n">
-        <v>4015</v>
+        <v>4373</v>
       </c>
       <c r="G343" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentaçao ( FL 53)</t>
+          <t>SUPERMERCADO XODO LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H343" s="1" t="n"/>
@@ -27094,7 +27170,7 @@
         </is>
       </c>
       <c r="J343" s="2" t="n">
-        <v>46226.44603434028</v>
+        <v>46226.44639907408</v>
       </c>
       <c r="K343" s="2" t="n">
         <v>46230</v>
@@ -27124,7 +27200,7 @@
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
-        <v>81358</v>
+        <v>81359</v>
       </c>
       <c r="B344" s="1" t="inlineStr">
         <is>
@@ -27143,15 +27219,15 @@
       </c>
       <c r="E344" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, a senha que está cadastrada no intranet da como inválida, por gentileza incluir a senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F344" s="1" t="n">
-        <v>4373</v>
+        <v>2710</v>
       </c>
       <c r="G344" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO XODO LTDA (FILIAL 02)</t>
+          <t>HORTIFRUTI BOM DO CAMPO LTDA</t>
         </is>
       </c>
       <c r="H344" s="1" t="n"/>
@@ -27161,7 +27237,7 @@
         </is>
       </c>
       <c r="J344" s="2" t="n">
-        <v>46226.44639907408</v>
+        <v>46226.44737951389</v>
       </c>
       <c r="K344" s="2" t="n">
         <v>46230</v>
@@ -27173,7 +27249,7 @@
       </c>
       <c r="M344" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N344" s="1" t="n"/>
@@ -27191,7 +27267,7 @@
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
-        <v>81359</v>
+        <v>81360</v>
       </c>
       <c r="B345" s="1" t="inlineStr">
         <is>
@@ -27210,15 +27286,15 @@
       </c>
       <c r="E345" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, a senha que está cadastrada no intranet da como inválida, por gentileza incluir a senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F345" s="1" t="n">
-        <v>2710</v>
+        <v>4416</v>
       </c>
       <c r="G345" s="1" t="inlineStr">
         <is>
-          <t>HORTIFRUTI BOM DO CAMPO LTDA</t>
+          <t>SUPERMERCADO MATRIZ LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H345" s="1" t="n"/>
@@ -27228,7 +27304,7 @@
         </is>
       </c>
       <c r="J345" s="2" t="n">
-        <v>46226.44737951389</v>
+        <v>46226.4478790162</v>
       </c>
       <c r="K345" s="2" t="n">
         <v>46230</v>
@@ -27240,7 +27316,7 @@
       </c>
       <c r="M345" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N345" s="1" t="n"/>
@@ -27258,7 +27334,7 @@
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
-        <v>81360</v>
+        <v>81361</v>
       </c>
       <c r="B346" s="1" t="inlineStr">
         <is>
@@ -27281,11 +27357,11 @@
         </is>
       </c>
       <c r="F346" s="1" t="n">
-        <v>4416</v>
+        <v>4605</v>
       </c>
       <c r="G346" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO MATRIZ LTDA (FILIAL 01)</t>
+          <t>AFE SERVICOS ADMINISTRATIVOS LTDA</t>
         </is>
       </c>
       <c r="H346" s="1" t="n"/>
@@ -27295,7 +27371,7 @@
         </is>
       </c>
       <c r="J346" s="2" t="n">
-        <v>46226.4478790162</v>
+        <v>46226.44799988426</v>
       </c>
       <c r="K346" s="2" t="n">
         <v>46230</v>
@@ -27325,7 +27401,7 @@
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
-        <v>81361</v>
+        <v>81362</v>
       </c>
       <c r="B347" s="1" t="inlineStr">
         <is>
@@ -27348,11 +27424,11 @@
         </is>
       </c>
       <c r="F347" s="1" t="n">
-        <v>4605</v>
+        <v>4804</v>
       </c>
       <c r="G347" s="1" t="inlineStr">
         <is>
-          <t>AFE SERVICOS ADMINISTRATIVOS LTDA</t>
+          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
         </is>
       </c>
       <c r="H347" s="1" t="n"/>
@@ -27362,7 +27438,7 @@
         </is>
       </c>
       <c r="J347" s="2" t="n">
-        <v>46226.44799988426</v>
+        <v>46226.44931420139</v>
       </c>
       <c r="K347" s="2" t="n">
         <v>46230</v>
@@ -27392,7 +27468,7 @@
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
-        <v>81362</v>
+        <v>81363</v>
       </c>
       <c r="B348" s="1" t="inlineStr">
         <is>
@@ -27415,11 +27491,11 @@
         </is>
       </c>
       <c r="F348" s="1" t="n">
-        <v>4804</v>
+        <v>4841</v>
       </c>
       <c r="G348" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
+          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H348" s="1" t="n"/>
@@ -27429,7 +27505,7 @@
         </is>
       </c>
       <c r="J348" s="2" t="n">
-        <v>46226.44931420139</v>
+        <v>46226.45019482639</v>
       </c>
       <c r="K348" s="2" t="n">
         <v>46230</v>
@@ -27459,7 +27535,7 @@
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
-        <v>81363</v>
+        <v>81364</v>
       </c>
       <c r="B349" s="1" t="inlineStr">
         <is>
@@ -27482,11 +27558,11 @@
         </is>
       </c>
       <c r="F349" s="1" t="n">
-        <v>4841</v>
+        <v>4918</v>
       </c>
       <c r="G349" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
         </is>
       </c>
       <c r="H349" s="1" t="n"/>
@@ -27496,7 +27572,7 @@
         </is>
       </c>
       <c r="J349" s="2" t="n">
-        <v>46226.45019482639</v>
+        <v>46226.45123028935</v>
       </c>
       <c r="K349" s="2" t="n">
         <v>46230</v>
@@ -27526,7 +27602,7 @@
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
-        <v>81364</v>
+        <v>81365</v>
       </c>
       <c r="B350" s="1" t="inlineStr">
         <is>
@@ -27549,11 +27625,11 @@
         </is>
       </c>
       <c r="F350" s="1" t="n">
-        <v>4918</v>
+        <v>5017</v>
       </c>
       <c r="G350" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
         </is>
       </c>
       <c r="H350" s="1" t="n"/>
@@ -27563,7 +27639,7 @@
         </is>
       </c>
       <c r="J350" s="2" t="n">
-        <v>46226.45123028935</v>
+        <v>46226.45200285879</v>
       </c>
       <c r="K350" s="2" t="n">
         <v>46230</v>
@@ -27593,7 +27669,7 @@
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>81365</v>
+        <v>81366</v>
       </c>
       <c r="B351" s="1" t="inlineStr">
         <is>
@@ -27616,11 +27692,11 @@
         </is>
       </c>
       <c r="F351" s="1" t="n">
-        <v>5017</v>
+        <v>5083</v>
       </c>
       <c r="G351" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
+          <t>PAULO S. DA SILVA</t>
         </is>
       </c>
       <c r="H351" s="1" t="n"/>
@@ -27630,7 +27706,7 @@
         </is>
       </c>
       <c r="J351" s="2" t="n">
-        <v>46226.45200285879</v>
+        <v>46226.4529128125</v>
       </c>
       <c r="K351" s="2" t="n">
         <v>46230</v>
@@ -27660,7 +27736,7 @@
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
-        <v>81366</v>
+        <v>81367</v>
       </c>
       <c r="B352" s="1" t="inlineStr">
         <is>
@@ -27683,11 +27759,11 @@
         </is>
       </c>
       <c r="F352" s="1" t="n">
-        <v>5083</v>
+        <v>5153</v>
       </c>
       <c r="G352" s="1" t="inlineStr">
         <is>
-          <t>PAULO S. DA SILVA</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
         </is>
       </c>
       <c r="H352" s="1" t="n"/>
@@ -27697,7 +27773,7 @@
         </is>
       </c>
       <c r="J352" s="2" t="n">
-        <v>46226.4529128125</v>
+        <v>46226.45361840277</v>
       </c>
       <c r="K352" s="2" t="n">
         <v>46230</v>
@@ -27727,7 +27803,7 @@
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>81367</v>
+        <v>81368</v>
       </c>
       <c r="B353" s="1" t="inlineStr">
         <is>
@@ -27750,11 +27826,11 @@
         </is>
       </c>
       <c r="F353" s="1" t="n">
-        <v>5153</v>
+        <v>5154</v>
       </c>
       <c r="G353" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
         </is>
       </c>
       <c r="H353" s="1" t="n"/>
@@ -27764,7 +27840,7 @@
         </is>
       </c>
       <c r="J353" s="2" t="n">
-        <v>46226.45361840277</v>
+        <v>46226.45395802084</v>
       </c>
       <c r="K353" s="2" t="n">
         <v>46230</v>
@@ -27794,7 +27870,7 @@
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
-        <v>81368</v>
+        <v>81369</v>
       </c>
       <c r="B354" s="1" t="inlineStr">
         <is>
@@ -27813,15 +27889,15 @@
       </c>
       <c r="E354" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F354" s="1" t="n">
-        <v>5154</v>
+        <v>3049</v>
       </c>
       <c r="G354" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
         </is>
       </c>
       <c r="H354" s="1" t="n"/>
@@ -27831,7 +27907,7 @@
         </is>
       </c>
       <c r="J354" s="2" t="n">
-        <v>46226.45395802084</v>
+        <v>46226.45434436342</v>
       </c>
       <c r="K354" s="2" t="n">
         <v>46230</v>
@@ -27843,7 +27919,7 @@
       </c>
       <c r="M354" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N354" s="1" t="n"/>
@@ -27861,7 +27937,7 @@
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
-        <v>81369</v>
+        <v>81370</v>
       </c>
       <c r="B355" s="1" t="inlineStr">
         <is>
@@ -27880,15 +27956,15 @@
       </c>
       <c r="E355" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F355" s="1" t="n">
-        <v>3049</v>
+        <v>5222</v>
       </c>
       <c r="G355" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
         </is>
       </c>
       <c r="H355" s="1" t="n"/>
@@ -27898,7 +27974,7 @@
         </is>
       </c>
       <c r="J355" s="2" t="n">
-        <v>46226.45434436342</v>
+        <v>46226.45476809028</v>
       </c>
       <c r="K355" s="2" t="n">
         <v>46230</v>
@@ -27910,7 +27986,7 @@
       </c>
       <c r="M355" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N355" s="1" t="n"/>
@@ -27928,7 +28004,7 @@
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
-        <v>81370</v>
+        <v>81371</v>
       </c>
       <c r="B356" s="1" t="inlineStr">
         <is>
@@ -27951,11 +28027,11 @@
         </is>
       </c>
       <c r="F356" s="1" t="n">
-        <v>5222</v>
+        <v>5224</v>
       </c>
       <c r="G356" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
         </is>
       </c>
       <c r="H356" s="1" t="n"/>
@@ -27965,7 +28041,7 @@
         </is>
       </c>
       <c r="J356" s="2" t="n">
-        <v>46226.45476809028</v>
+        <v>46226.45489934028</v>
       </c>
       <c r="K356" s="2" t="n">
         <v>46230</v>
@@ -27995,7 +28071,7 @@
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
-        <v>81371</v>
+        <v>81372</v>
       </c>
       <c r="B357" s="1" t="inlineStr">
         <is>
@@ -28018,11 +28094,11 @@
         </is>
       </c>
       <c r="F357" s="1" t="n">
-        <v>5224</v>
+        <v>5311</v>
       </c>
       <c r="G357" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
+          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
         </is>
       </c>
       <c r="H357" s="1" t="n"/>
@@ -28032,7 +28108,7 @@
         </is>
       </c>
       <c r="J357" s="2" t="n">
-        <v>46226.45489934028</v>
+        <v>46226.45548961806</v>
       </c>
       <c r="K357" s="2" t="n">
         <v>46230</v>
@@ -28062,7 +28138,7 @@
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
-        <v>81372</v>
+        <v>81373</v>
       </c>
       <c r="B358" s="1" t="inlineStr">
         <is>
@@ -28085,11 +28161,11 @@
         </is>
       </c>
       <c r="F358" s="1" t="n">
-        <v>5311</v>
+        <v>5583</v>
       </c>
       <c r="G358" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H358" s="1" t="n"/>
@@ -28099,7 +28175,7 @@
         </is>
       </c>
       <c r="J358" s="2" t="n">
-        <v>46226.45548961806</v>
+        <v>46226.45648677083</v>
       </c>
       <c r="K358" s="2" t="n">
         <v>46230</v>
@@ -28129,7 +28205,7 @@
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
-        <v>81373</v>
+        <v>81375</v>
       </c>
       <c r="B359" s="1" t="inlineStr">
         <is>
@@ -28152,11 +28228,11 @@
         </is>
       </c>
       <c r="F359" s="1" t="n">
-        <v>5583</v>
+        <v>5584</v>
       </c>
       <c r="G359" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 01)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H359" s="1" t="n"/>
@@ -28166,7 +28242,7 @@
         </is>
       </c>
       <c r="J359" s="2" t="n">
-        <v>46226.45648677083</v>
+        <v>46226.45693457176</v>
       </c>
       <c r="K359" s="2" t="n">
         <v>46230</v>
@@ -28196,7 +28272,7 @@
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
-        <v>81375</v>
+        <v>81376</v>
       </c>
       <c r="B360" s="1" t="inlineStr">
         <is>
@@ -28215,15 +28291,15 @@
       </c>
       <c r="E360" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F360" s="1" t="n">
-        <v>5584</v>
+        <v>2745</v>
       </c>
       <c r="G360" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H360" s="1" t="n"/>
@@ -28233,7 +28309,7 @@
         </is>
       </c>
       <c r="J360" s="2" t="n">
-        <v>46226.45693457176</v>
+        <v>46226.46478128473</v>
       </c>
       <c r="K360" s="2" t="n">
         <v>46230</v>
@@ -28245,7 +28321,7 @@
       </c>
       <c r="M360" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N360" s="1" t="n"/>
@@ -28263,7 +28339,7 @@
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
-        <v>81376</v>
+        <v>81377</v>
       </c>
       <c r="B361" s="1" t="inlineStr">
         <is>
@@ -28286,11 +28362,11 @@
         </is>
       </c>
       <c r="F361" s="1" t="n">
-        <v>2745</v>
+        <v>3601</v>
       </c>
       <c r="G361" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
         </is>
       </c>
       <c r="H361" s="1" t="n"/>
@@ -28300,7 +28376,7 @@
         </is>
       </c>
       <c r="J361" s="2" t="n">
-        <v>46226.46478128473</v>
+        <v>46226.4658295949</v>
       </c>
       <c r="K361" s="2" t="n">
         <v>46230</v>
@@ -28330,7 +28406,7 @@
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
-        <v>81377</v>
+        <v>81378</v>
       </c>
       <c r="B362" s="1" t="inlineStr">
         <is>
@@ -28353,11 +28429,11 @@
         </is>
       </c>
       <c r="F362" s="1" t="n">
-        <v>3601</v>
+        <v>3692</v>
       </c>
       <c r="G362" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
+          <t>MERCADO DOS DOCES VILA FORMOSA COMERCIAL LTDA (FILIAL 06)</t>
         </is>
       </c>
       <c r="H362" s="1" t="n"/>
@@ -28367,7 +28443,7 @@
         </is>
       </c>
       <c r="J362" s="2" t="n">
-        <v>46226.4658295949</v>
+        <v>46226.46878642361</v>
       </c>
       <c r="K362" s="2" t="n">
         <v>46230</v>
@@ -28397,7 +28473,7 @@
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
-        <v>81378</v>
+        <v>81379</v>
       </c>
       <c r="B363" s="1" t="inlineStr">
         <is>
@@ -28416,15 +28492,15 @@
       </c>
       <c r="E363" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F363" s="1" t="n">
-        <v>3692</v>
+        <v>4079</v>
       </c>
       <c r="G363" s="1" t="inlineStr">
         <is>
-          <t>MERCADO DOS DOCES VILA FORMOSA COMERCIAL LTDA (FILIAL 06)</t>
+          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
         </is>
       </c>
       <c r="H363" s="1" t="n"/>
@@ -28434,7 +28510,7 @@
         </is>
       </c>
       <c r="J363" s="2" t="n">
-        <v>46226.46878642361</v>
+        <v>46226.47010887731</v>
       </c>
       <c r="K363" s="2" t="n">
         <v>46230</v>
@@ -28464,7 +28540,7 @@
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
-        <v>81379</v>
+        <v>81380</v>
       </c>
       <c r="B364" s="1" t="inlineStr">
         <is>
@@ -28487,11 +28563,11 @@
         </is>
       </c>
       <c r="F364" s="1" t="n">
-        <v>4079</v>
+        <v>4339</v>
       </c>
       <c r="G364" s="1" t="inlineStr">
         <is>
-          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
         </is>
       </c>
       <c r="H364" s="1" t="n"/>
@@ -28501,7 +28577,7 @@
         </is>
       </c>
       <c r="J364" s="2" t="n">
-        <v>46226.47010887731</v>
+        <v>46226.47113148148</v>
       </c>
       <c r="K364" s="2" t="n">
         <v>46230</v>
@@ -28531,7 +28607,7 @@
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
-        <v>81380</v>
+        <v>81381</v>
       </c>
       <c r="B365" s="1" t="inlineStr">
         <is>
@@ -28554,11 +28630,11 @@
         </is>
       </c>
       <c r="F365" s="1" t="n">
-        <v>4339</v>
+        <v>4625</v>
       </c>
       <c r="G365" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
+          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H365" s="1" t="n"/>
@@ -28568,7 +28644,7 @@
         </is>
       </c>
       <c r="J365" s="2" t="n">
-        <v>46226.47113148148</v>
+        <v>46226.47206631945</v>
       </c>
       <c r="K365" s="2" t="n">
         <v>46230</v>
@@ -28598,7 +28674,7 @@
     </row>
     <row r="366">
       <c r="A366" s="1" t="n">
-        <v>81381</v>
+        <v>81382</v>
       </c>
       <c r="B366" s="1" t="inlineStr">
         <is>
@@ -28621,11 +28697,11 @@
         </is>
       </c>
       <c r="F366" s="1" t="n">
-        <v>4625</v>
+        <v>4842</v>
       </c>
       <c r="G366" s="1" t="inlineStr">
         <is>
-          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
+          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 03)</t>
         </is>
       </c>
       <c r="H366" s="1" t="n"/>
@@ -28635,7 +28711,7 @@
         </is>
       </c>
       <c r="J366" s="2" t="n">
-        <v>46226.47206631945</v>
+        <v>46226.47387114583</v>
       </c>
       <c r="K366" s="2" t="n">
         <v>46230</v>
@@ -28665,7 +28741,7 @@
     </row>
     <row r="367">
       <c r="A367" s="1" t="n">
-        <v>81382</v>
+        <v>81385</v>
       </c>
       <c r="B367" s="1" t="inlineStr">
         <is>
@@ -28688,11 +28764,11 @@
         </is>
       </c>
       <c r="F367" s="1" t="n">
-        <v>4842</v>
+        <v>5143</v>
       </c>
       <c r="G367" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 03)</t>
+          <t>OLIMPIA ADMINISTRADORA DE SERVIÇOS LTDA</t>
         </is>
       </c>
       <c r="H367" s="1" t="n"/>
@@ -28702,7 +28778,7 @@
         </is>
       </c>
       <c r="J367" s="2" t="n">
-        <v>46226.47387114583</v>
+        <v>46226.48074552084</v>
       </c>
       <c r="K367" s="2" t="n">
         <v>46230</v>
@@ -28732,7 +28808,7 @@
     </row>
     <row r="368">
       <c r="A368" s="1" t="n">
-        <v>81385</v>
+        <v>81387</v>
       </c>
       <c r="B368" s="1" t="inlineStr">
         <is>
@@ -28755,11 +28831,11 @@
         </is>
       </c>
       <c r="F368" s="1" t="n">
-        <v>5143</v>
+        <v>5508</v>
       </c>
       <c r="G368" s="1" t="inlineStr">
         <is>
-          <t>OLIMPIA ADMINISTRADORA DE SERVIÇOS LTDA</t>
+          <t>ALEXANDRA LIBRAZI GIUNGI BARRETO</t>
         </is>
       </c>
       <c r="H368" s="1" t="n"/>
@@ -28769,7 +28845,7 @@
         </is>
       </c>
       <c r="J368" s="2" t="n">
-        <v>46226.48074552084</v>
+        <v>46226.4871065162</v>
       </c>
       <c r="K368" s="2" t="n">
         <v>46230</v>
@@ -28799,7 +28875,7 @@
     </row>
     <row r="369">
       <c r="A369" s="1" t="n">
-        <v>81387</v>
+        <v>81388</v>
       </c>
       <c r="B369" s="1" t="inlineStr">
         <is>
@@ -28822,11 +28898,11 @@
         </is>
       </c>
       <c r="F369" s="1" t="n">
-        <v>5508</v>
+        <v>5654</v>
       </c>
       <c r="G369" s="1" t="inlineStr">
         <is>
-          <t>ALEXANDRA LIBRAZI GIUNGI BARRETO</t>
+          <t>DUARTE E SILVA LTDA</t>
         </is>
       </c>
       <c r="H369" s="1" t="n"/>
@@ -28836,7 +28912,7 @@
         </is>
       </c>
       <c r="J369" s="2" t="n">
-        <v>46226.4871065162</v>
+        <v>46226.4878119213</v>
       </c>
       <c r="K369" s="2" t="n">
         <v>46230</v>
@@ -28866,7 +28942,7 @@
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
-        <v>81388</v>
+        <v>81390</v>
       </c>
       <c r="B370" s="1" t="inlineStr">
         <is>
@@ -28889,11 +28965,11 @@
         </is>
       </c>
       <c r="F370" s="1" t="n">
-        <v>5654</v>
+        <v>5876</v>
       </c>
       <c r="G370" s="1" t="inlineStr">
         <is>
-          <t>DUARTE E SILVA LTDA</t>
+          <t>Cucinare Pro Alimentacao (Filial 82)</t>
         </is>
       </c>
       <c r="H370" s="1" t="n"/>
@@ -28903,7 +28979,7 @@
         </is>
       </c>
       <c r="J370" s="2" t="n">
-        <v>46226.4878119213</v>
+        <v>46226.48955505787</v>
       </c>
       <c r="K370" s="2" t="n">
         <v>46230</v>
@@ -28933,7 +29009,7 @@
     </row>
     <row r="371">
       <c r="A371" s="1" t="n">
-        <v>81390</v>
+        <v>81391</v>
       </c>
       <c r="B371" s="1" t="inlineStr">
         <is>
@@ -28956,11 +29032,11 @@
         </is>
       </c>
       <c r="F371" s="1" t="n">
-        <v>5876</v>
+        <v>5877</v>
       </c>
       <c r="G371" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 82)</t>
+          <t>Cucinare Pro Alimentacao (Filial 83)</t>
         </is>
       </c>
       <c r="H371" s="1" t="n"/>
@@ -28970,7 +29046,7 @@
         </is>
       </c>
       <c r="J371" s="2" t="n">
-        <v>46226.48955505787</v>
+        <v>46226.4918327199</v>
       </c>
       <c r="K371" s="2" t="n">
         <v>46230</v>
@@ -29000,7 +29076,7 @@
     </row>
     <row r="372">
       <c r="A372" s="1" t="n">
-        <v>81391</v>
+        <v>81393</v>
       </c>
       <c r="B372" s="1" t="inlineStr">
         <is>
@@ -29023,11 +29099,11 @@
         </is>
       </c>
       <c r="F372" s="1" t="n">
-        <v>5877</v>
+        <v>5878</v>
       </c>
       <c r="G372" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 83)</t>
+          <t>Cucinare Pro Alimentacao (Filial 84)</t>
         </is>
       </c>
       <c r="H372" s="1" t="n"/>
@@ -29037,7 +29113,7 @@
         </is>
       </c>
       <c r="J372" s="2" t="n">
-        <v>46226.4918327199</v>
+        <v>46226.49427164352</v>
       </c>
       <c r="K372" s="2" t="n">
         <v>46230</v>
@@ -29067,7 +29143,7 @@
     </row>
     <row r="373">
       <c r="A373" s="1" t="n">
-        <v>81393</v>
+        <v>81394</v>
       </c>
       <c r="B373" s="1" t="inlineStr">
         <is>
@@ -29090,11 +29166,11 @@
         </is>
       </c>
       <c r="F373" s="1" t="n">
-        <v>5878</v>
+        <v>5038</v>
       </c>
       <c r="G373" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 84)</t>
+          <t xml:space="preserve">CENTRAL DISTRIBUIDORA DE GESSO LTDA (FILIAL 01) </t>
         </is>
       </c>
       <c r="H373" s="1" t="n"/>
@@ -29104,7 +29180,7 @@
         </is>
       </c>
       <c r="J373" s="2" t="n">
-        <v>46226.49427164352</v>
+        <v>46226.49645659722</v>
       </c>
       <c r="K373" s="2" t="n">
         <v>46230</v>
@@ -29134,7 +29210,7 @@
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
-        <v>81394</v>
+        <v>81395</v>
       </c>
       <c r="B374" s="1" t="inlineStr">
         <is>
@@ -29157,11 +29233,11 @@
         </is>
       </c>
       <c r="F374" s="1" t="n">
-        <v>5038</v>
+        <v>5879</v>
       </c>
       <c r="G374" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRAL DISTRIBUIDORA DE GESSO LTDA (FILIAL 01) </t>
+          <t>Cucinare Pro Alimentacao LTDA (Filial 85)</t>
         </is>
       </c>
       <c r="H374" s="1" t="n"/>
@@ -29171,7 +29247,7 @@
         </is>
       </c>
       <c r="J374" s="2" t="n">
-        <v>46226.49645659722</v>
+        <v>46226.49918903935</v>
       </c>
       <c r="K374" s="2" t="n">
         <v>46230</v>
@@ -29201,7 +29277,7 @@
     </row>
     <row r="375">
       <c r="A375" s="1" t="n">
-        <v>81395</v>
+        <v>81396</v>
       </c>
       <c r="B375" s="1" t="inlineStr">
         <is>
@@ -29224,11 +29300,11 @@
         </is>
       </c>
       <c r="F375" s="1" t="n">
-        <v>5879</v>
+        <v>5880</v>
       </c>
       <c r="G375" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao LTDA (Filial 85)</t>
+          <t>Cucinare Pro Alimentacao LTDA (Filial 86)</t>
         </is>
       </c>
       <c r="H375" s="1" t="n"/>
@@ -29238,7 +29314,7 @@
         </is>
       </c>
       <c r="J375" s="2" t="n">
-        <v>46226.49918903935</v>
+        <v>46226.49988873843</v>
       </c>
       <c r="K375" s="2" t="n">
         <v>46230</v>
@@ -29268,7 +29344,7 @@
     </row>
     <row r="376">
       <c r="A376" s="1" t="n">
-        <v>81396</v>
+        <v>81397</v>
       </c>
       <c r="B376" s="1" t="inlineStr">
         <is>
@@ -29287,15 +29363,15 @@
       </c>
       <c r="E376" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F376" s="1" t="n">
-        <v>5880</v>
+        <v>5882</v>
       </c>
       <c r="G376" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao LTDA (Filial 86)</t>
+          <t>Cucinare Pro Alimentacao LTDA (Filial 88)</t>
         </is>
       </c>
       <c r="H376" s="1" t="n"/>
@@ -29305,7 +29381,7 @@
         </is>
       </c>
       <c r="J376" s="2" t="n">
-        <v>46226.49988873843</v>
+        <v>46226.50144737268</v>
       </c>
       <c r="K376" s="2" t="n">
         <v>46230</v>
@@ -29335,7 +29411,7 @@
     </row>
     <row r="377">
       <c r="A377" s="1" t="n">
-        <v>81397</v>
+        <v>81399</v>
       </c>
       <c r="B377" s="1" t="inlineStr">
         <is>
@@ -29358,11 +29434,11 @@
         </is>
       </c>
       <c r="F377" s="1" t="n">
-        <v>5882</v>
+        <v>5883</v>
       </c>
       <c r="G377" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao LTDA (Filial 88)</t>
+          <t>Cucinare Pro Alimentacao LTDA (Filial 89)</t>
         </is>
       </c>
       <c r="H377" s="1" t="n"/>
@@ -29372,7 +29448,7 @@
         </is>
       </c>
       <c r="J377" s="2" t="n">
-        <v>46226.50144737268</v>
+        <v>46226.50319591435</v>
       </c>
       <c r="K377" s="2" t="n">
         <v>46230</v>
@@ -29402,7 +29478,7 @@
     </row>
     <row r="378">
       <c r="A378" s="1" t="n">
-        <v>81399</v>
+        <v>81400</v>
       </c>
       <c r="B378" s="1" t="inlineStr">
         <is>
@@ -29421,15 +29497,15 @@
       </c>
       <c r="E378" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F378" s="1" t="n">
-        <v>5883</v>
+        <v>5884</v>
       </c>
       <c r="G378" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao LTDA (Filial 89)</t>
+          <t>Cucinare Pro Alimentacao LTDA (Filial 90)</t>
         </is>
       </c>
       <c r="H378" s="1" t="n"/>
@@ -29439,7 +29515,7 @@
         </is>
       </c>
       <c r="J378" s="2" t="n">
-        <v>46226.50319591435</v>
+        <v>46226.50373815972</v>
       </c>
       <c r="K378" s="2" t="n">
         <v>46230</v>
@@ -29469,7 +29545,7 @@
     </row>
     <row r="379">
       <c r="A379" s="1" t="n">
-        <v>81400</v>
+        <v>81401</v>
       </c>
       <c r="B379" s="1" t="inlineStr">
         <is>
@@ -29488,7 +29564,7 @@
       </c>
       <c r="E379" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F379" s="1" t="n">
@@ -29506,7 +29582,7 @@
         </is>
       </c>
       <c r="J379" s="2" t="n">
-        <v>46226.50373815972</v>
+        <v>46226.50527931713</v>
       </c>
       <c r="K379" s="2" t="n">
         <v>46230</v>
@@ -29536,34 +29612,34 @@
     </row>
     <row r="380">
       <c r="A380" s="1" t="n">
-        <v>81401</v>
+        <v>81402</v>
       </c>
       <c r="B380" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração de Contabilista</t>
         </is>
       </c>
       <c r="C380" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Vincular </t>
         </is>
       </c>
       <c r="D380" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E380" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Boa tarde.Ao tentar realizar o DEC da empresa 6944 - MERCADO VIOLETA LTDA (FILIAL 11), informa esta mensagem de "estabelecimento negado" podem verificar se está vinculado para tirar a consulta DEC, por gentileza</t>
         </is>
       </c>
       <c r="F380" s="1" t="n">
-        <v>5884</v>
+        <v>6944</v>
       </c>
       <c r="G380" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao LTDA (Filial 90)</t>
+          <t>MERCADO VIOLETA LTDA (FILIAL 11)</t>
         </is>
       </c>
       <c r="H380" s="1" t="n"/>
@@ -29573,7 +29649,7 @@
         </is>
       </c>
       <c r="J380" s="2" t="n">
-        <v>46226.50527931713</v>
+        <v>46226.50528148148</v>
       </c>
       <c r="K380" s="2" t="n">
         <v>46230</v>
@@ -29585,7 +29661,7 @@
       </c>
       <c r="M380" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="N380" s="1" t="n"/>
@@ -29603,7 +29679,7 @@
     </row>
     <row r="381">
       <c r="A381" s="1" t="n">
-        <v>81402</v>
+        <v>81403</v>
       </c>
       <c r="B381" s="1" t="inlineStr">
         <is>
@@ -29612,7 +29688,7 @@
       </c>
       <c r="C381" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vincular </t>
+          <t>Desvincular</t>
         </is>
       </c>
       <c r="D381" s="1" t="inlineStr">
@@ -29622,15 +29698,15 @@
       </c>
       <c r="E381" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Ao tentar realizar o DEC da empresa 6944 - MERCADO VIOLETA LTDA (FILIAL 11), informa esta mensagem de "estabelecimento negado" podem verificar se está vinculado para tirar a consulta DEC, por gentileza</t>
+          <t>Boa tarde.Ao tentar realizar o DEC da empresa 6983- MEU MORETE SUPERMERCADOS LTDA, informa esta mensagem de "estabelecimento negado" podem verificar se está vinculado para tirar a consulta DEC, por gentileza</t>
         </is>
       </c>
       <c r="F381" s="1" t="n">
-        <v>6944</v>
+        <v>4527</v>
       </c>
       <c r="G381" s="1" t="inlineStr">
         <is>
-          <t>MERCADO VIOLETA LTDA (FILIAL 11)</t>
+          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
         </is>
       </c>
       <c r="H381" s="1" t="n"/>
@@ -29640,7 +29716,7 @@
         </is>
       </c>
       <c r="J381" s="2" t="n">
-        <v>46226.50528148148</v>
+        <v>46226.50946547453</v>
       </c>
       <c r="K381" s="2" t="n">
         <v>46230</v>
@@ -29670,34 +29746,34 @@
     </row>
     <row r="382">
       <c r="A382" s="1" t="n">
-        <v>81403</v>
+        <v>81404</v>
       </c>
       <c r="B382" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Contabilista</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C382" s="1" t="inlineStr">
         <is>
-          <t>Desvincular</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D382" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E382" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde.Ao tentar realizar o DEC da empresa 6983- MEU MORETE SUPERMERCADOS LTDA, informa esta mensagem de "estabelecimento negado" podem verificar se está vinculado para tirar a consulta DEC, por gentileza</t>
+          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F382" s="1" t="n">
-        <v>4527</v>
+        <v>6207</v>
       </c>
       <c r="G382" s="1" t="inlineStr">
         <is>
-          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 92)</t>
         </is>
       </c>
       <c r="H382" s="1" t="n"/>
@@ -29707,7 +29783,7 @@
         </is>
       </c>
       <c r="J382" s="2" t="n">
-        <v>46226.50946547453</v>
+        <v>46226.50961396991</v>
       </c>
       <c r="K382" s="2" t="n">
         <v>46230</v>
@@ -29719,7 +29795,7 @@
       </c>
       <c r="M382" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N382" s="1" t="n"/>
@@ -29737,34 +29813,34 @@
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
-        <v>81404</v>
+        <v>81418</v>
       </c>
       <c r="B383" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Parcelamento Estadual</t>
         </is>
       </c>
       <c r="C383" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>ICMS</t>
         </is>
       </c>
       <c r="D383" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E383" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Boa tarde EllenAssim como conversamos nosso cliente Smart Break possui um débito de ICMS no mês 05 e 06.Precisa fazer um parcelamento em 60 meses e enviar a guia da primeira para ele fazer o pagamento hoje.Caso mês 06 ainda não esteja disponível pode ser feito apenas com o mês 05Jairo já conversou com o cliente e aprovou a proposta.Grato</t>
         </is>
       </c>
       <c r="F383" s="1" t="n">
-        <v>6207</v>
+        <v>4527</v>
       </c>
       <c r="G383" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 92)</t>
+          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
         </is>
       </c>
       <c r="H383" s="1" t="n"/>
@@ -29774,7 +29850,7 @@
         </is>
       </c>
       <c r="J383" s="2" t="n">
-        <v>46226.50961396991</v>
+        <v>46226.66471385417</v>
       </c>
       <c r="K383" s="2" t="n">
         <v>46230</v>
@@ -29786,7 +29862,7 @@
       </c>
       <c r="M383" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="N383" s="1" t="n"/>
@@ -29804,26 +29880,26 @@
     </row>
     <row r="384">
       <c r="A384" s="1" t="n">
-        <v>81418</v>
+        <v>81421</v>
       </c>
       <c r="B384" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Estadual</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C384" s="1" t="inlineStr">
         <is>
-          <t>ICMS</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="D384" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E384" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde EllenAssim como conversamos nosso cliente Smart Break possui um débito de ICMS no mês 05 e 06.Precisa fazer um parcelamento em 60 meses e enviar a guia da primeira para ele fazer o pagamento hoje.Caso mês 06 ainda não esteja disponível pode ser feito apenas com o mês 05Jairo já conversou com o cliente e aprovou a proposta.Grato</t>
+          <t>Assim como conversado com a Ellen. No mês 04 foi apurado o ICMS e o cliente não efetuou o pagamento. No mês 06 foi feito o recalculo e o cliente pagou a guia enviada pela MG.Está constando pendência na conta fiscal. Conforme anexos.</t>
         </is>
       </c>
       <c r="F384" s="1" t="n">
@@ -29841,7 +29917,7 @@
         </is>
       </c>
       <c r="J384" s="2" t="n">
-        <v>46226.66471385417</v>
+        <v>46226.69917303241</v>
       </c>
       <c r="K384" s="2" t="n">
         <v>46230</v>
@@ -29871,63 +29947,71 @@
     </row>
     <row r="385">
       <c r="A385" s="1" t="n">
-        <v>81421</v>
+        <v>81422</v>
       </c>
       <c r="B385" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C385" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D385" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E385" s="1" t="inlineStr">
         <is>
-          <t>Assim como conversado com a Ellen. No mês 04 foi apurado o ICMS e o cliente não efetuou o pagamento. No mês 06 foi feito o recalculo e o cliente pagou a guia enviada pela MG.Está constando pendência na conta fiscal. Conforme anexos.</t>
+          <t>6990 - AMANCIO S ELETRICA (MATRIZ) - por gentileza providencias os documentos do Checklist.</t>
         </is>
       </c>
       <c r="F385" s="1" t="n">
-        <v>4527</v>
-      </c>
-      <c r="G385" s="1" t="inlineStr">
-        <is>
-          <t>SMART BREAK COMERCIO LANCHES S.A.</t>
-        </is>
-      </c>
-      <c r="H385" s="1" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G385" s="1" t="n"/>
+      <c r="H385" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
       <c r="I385" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J385" s="2" t="n">
-        <v>46226.69917303241</v>
+        <v>46226.70303271991</v>
       </c>
       <c r="K385" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L385" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M385" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
-        </is>
-      </c>
-      <c r="N385" s="1" t="n"/>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N385" s="2" t="n">
+        <v>46230.39939193287</v>
+      </c>
       <c r="O385" s="1" t="n"/>
       <c r="P385" s="1" t="n"/>
       <c r="Q385" s="1" t="inlineStr"/>
-      <c r="R385" s="1" t="n"/>
+      <c r="R385" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia!
+Estou aguardando o contato do contador.
+</t>
+        </is>
+      </c>
       <c r="S385" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -29938,7 +30022,7 @@
     </row>
     <row r="386">
       <c r="A386" s="1" t="n">
-        <v>81422</v>
+        <v>81423</v>
       </c>
       <c r="B386" s="1" t="inlineStr">
         <is>
@@ -29957,28 +30041,32 @@
       </c>
       <c r="E386" s="1" t="inlineStr">
         <is>
-          <t>6990 - AMANCIO S ELETRICA (MATRIZ) - por gentileza providencias os documentos do Checklist.</t>
+          <t>6991 - AMANCIO S ELETRICA (FILIAL 1) - por gentileza providencias os documentos do Checklist.</t>
         </is>
       </c>
       <c r="F386" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G386" s="1" t="n"/>
-      <c r="H386" s="1" t="n"/>
+      <c r="H386" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
       <c r="I386" s="1" t="inlineStr">
         <is>
           <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J386" s="2" t="n">
-        <v>46226.70303271991</v>
+        <v>46226.70371354167</v>
       </c>
       <c r="K386" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L386" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M386" s="1" t="inlineStr">
@@ -29986,11 +30074,18 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N386" s="1" t="n"/>
+      <c r="N386" s="2" t="n">
+        <v>46230.39952141204</v>
+      </c>
       <c r="O386" s="1" t="n"/>
       <c r="P386" s="1" t="n"/>
       <c r="Q386" s="1" t="inlineStr"/>
-      <c r="R386" s="1" t="n"/>
+      <c r="R386" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia!
+Estou aguardando o contato do contador.</t>
+        </is>
+      </c>
       <c r="S386" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -30001,40 +30096,44 @@
     </row>
     <row r="387">
       <c r="A387" s="1" t="n">
-        <v>81423</v>
+        <v>81426</v>
       </c>
       <c r="B387" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C387" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Ordinário</t>
         </is>
       </c>
       <c r="D387" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E387" s="1" t="inlineStr">
         <is>
-          <t>6991 - AMANCIO S ELETRICA (FILIAL 1) - por gentileza providencias os documentos do Checklist.</t>
+          <t>ACERT - SIMULAÇÃO DE PARCELAMENTOCliente solicita simulação de parcelamento FEDERAL</t>
         </is>
       </c>
       <c r="F387" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G387" s="1" t="n"/>
+        <v>6559</v>
+      </c>
+      <c r="G387" s="1" t="inlineStr">
+        <is>
+          <t>ACERTONLINE ASSESSORIA EMPRESARIAL LTDA</t>
+        </is>
+      </c>
       <c r="H387" s="1" t="n"/>
       <c r="I387" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J387" s="2" t="n">
-        <v>46226.70371354167</v>
+        <v>46226.7238943287</v>
       </c>
       <c r="K387" s="2" t="n">
         <v>46230</v>
@@ -30046,7 +30145,7 @@
       </c>
       <c r="M387" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N387" s="1" t="n"/>
@@ -30064,34 +30163,34 @@
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
-        <v>81426</v>
+        <v>81429</v>
       </c>
       <c r="B388" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento RFB</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C388" s="1" t="inlineStr">
         <is>
-          <t>Ordinário</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D388" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E388" s="1" t="inlineStr">
         <is>
-          <t>ACERT - SIMULAÇÃO DE PARCELAMENTOCliente solicita simulação de parcelamento FEDERAL</t>
+          <t>Prezados, boa tarde! Por gentileza fazer inscrição municipal do cliente SKEPAR</t>
         </is>
       </c>
       <c r="F388" s="1" t="n">
-        <v>6559</v>
+        <v>1905</v>
       </c>
       <c r="G388" s="1" t="inlineStr">
         <is>
-          <t>ACERTONLINE ASSESSORIA EMPRESARIAL LTDA</t>
+          <t>SKEPAR ADMINISTRAÇÃO E PARTICIPAÇÃO S.A.</t>
         </is>
       </c>
       <c r="H388" s="1" t="n"/>
@@ -30101,7 +30200,7 @@
         </is>
       </c>
       <c r="J388" s="2" t="n">
-        <v>46226.7238943287</v>
+        <v>46226.75350100695</v>
       </c>
       <c r="K388" s="2" t="n">
         <v>46230</v>
@@ -30113,7 +30212,7 @@
       </c>
       <c r="M388" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Karine Gusmão</t>
         </is>
       </c>
       <c r="N388" s="1" t="n"/>
@@ -30131,34 +30230,34 @@
     </row>
     <row r="389">
       <c r="A389" s="1" t="n">
-        <v>81429</v>
+        <v>81431</v>
       </c>
       <c r="B389" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C389" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Sociedade - Comércio</t>
         </is>
       </c>
       <c r="D389" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E389" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde! Por gentileza fazer inscrição municipal do cliente SKEPAR</t>
+          <t>6945 - BRASIL DISTRIBUIDORA - ABERTURA DE CNPJCliente solicita abertura de CNPJ, pretensão colocar no Simples Nacional e transferir os CLT. Usar todos os CNAE da empresa já existente (anexo).Att.Vander</t>
         </is>
       </c>
       <c r="F389" s="1" t="n">
-        <v>1905</v>
+        <v>6945</v>
       </c>
       <c r="G389" s="1" t="inlineStr">
         <is>
-          <t>SKEPAR ADMINISTRAÇÃO E PARTICIPAÇÃO S.A.</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="H389" s="1" t="n"/>
@@ -30168,7 +30267,7 @@
         </is>
       </c>
       <c r="J389" s="2" t="n">
-        <v>46226.75350100695</v>
+        <v>46226.77195251158</v>
       </c>
       <c r="K389" s="2" t="n">
         <v>46230</v>
@@ -30180,7 +30279,7 @@
       </c>
       <c r="M389" s="1" t="inlineStr">
         <is>
-          <t>Karine Gusmão</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N389" s="1" t="n"/>
@@ -30198,16 +30297,16 @@
     </row>
     <row r="390">
       <c r="A390" s="1" t="n">
-        <v>81431</v>
+        <v>81432</v>
       </c>
       <c r="B390" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Processo de Caixa</t>
         </is>
       </c>
       <c r="C390" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Comércio</t>
+          <t>Objeto Social</t>
         </is>
       </c>
       <c r="D390" s="1" t="inlineStr">
@@ -30217,7 +30316,7 @@
       </c>
       <c r="E390" s="1" t="inlineStr">
         <is>
-          <t>6945 - BRASIL DISTRIBUIDORA - ABERTURA DE CNPJCliente solicita abertura de CNPJ, pretensão colocar no Simples Nacional e transferir os CLT. Usar todos os CNAE da empresa já existente (anexo).Att.Vander</t>
+          <t>6945 - BRASIL DISTRIBUIDORA - INCLUSÃO DE ATIVIDADE PARA EXCLUIR EMPRESA DO SIMPLESReynaldo em conversa com cliente decidiram incluir atividade proibida no SIMPLES NACIONAL, para força uma exclusão fora do período normal. Por favor seguir com inclusão de CNAE para viabilizar o plano do MASTER. Att.Vander</t>
         </is>
       </c>
       <c r="F390" s="1" t="n">
@@ -30235,7 +30334,7 @@
         </is>
       </c>
       <c r="J390" s="2" t="n">
-        <v>46226.77195251158</v>
+        <v>46226.78004016203</v>
       </c>
       <c r="K390" s="2" t="n">
         <v>46230</v>
@@ -30265,34 +30364,34 @@
     </row>
     <row r="391">
       <c r="A391" s="1" t="n">
-        <v>81432</v>
+        <v>81440</v>
       </c>
       <c r="B391" s="1" t="inlineStr">
         <is>
-          <t>Processo de Caixa</t>
+          <t>Alteração de Contabilista</t>
         </is>
       </c>
       <c r="C391" s="1" t="inlineStr">
         <is>
-          <t>Objeto Social</t>
+          <t xml:space="preserve">Vincular </t>
         </is>
       </c>
       <c r="D391" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E391" s="1" t="inlineStr">
         <is>
-          <t>6945 - BRASIL DISTRIBUIDORA - INCLUSÃO DE ATIVIDADE PARA EXCLUIR EMPRESA DO SIMPLESReynaldo em conversa com cliente decidiram incluir atividade proibida no SIMPLES NACIONAL, para força uma exclusão fora do período normal. Por favor seguir com inclusão de CNAE para viabilizar o plano do MASTER. Att.Vander</t>
+          <t>Ao consultar os dados do cliente no CADESP continua vinculado as informações do antigo contador.</t>
         </is>
       </c>
       <c r="F391" s="1" t="n">
-        <v>6945</v>
+        <v>6795</v>
       </c>
       <c r="G391" s="1" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t>COLÉGIO JOAQUIM MARIA MACHADO DE ASSIS LTDA</t>
         </is>
       </c>
       <c r="H391" s="1" t="n"/>
@@ -30302,10 +30401,10 @@
         </is>
       </c>
       <c r="J391" s="2" t="n">
-        <v>46226.78004016203</v>
+        <v>46230.38834112269</v>
       </c>
       <c r="K391" s="2" t="n">
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="L391" s="1" t="inlineStr">
         <is>
@@ -30314,7 +30413,7 @@
       </c>
       <c r="M391" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N391" s="1" t="n"/>
@@ -30329,6 +30428,136 @@
       </c>
       <c r="T391" s="1" t="n"/>
       <c r="U391" s="1" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="1" t="n">
+        <v>81443</v>
+      </c>
+      <c r="B392" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C392" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D392" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E392" s="1" t="inlineStr">
+        <is>
+          <t>Por favor, providenciar senha de acesso para prefeitura.</t>
+        </is>
+      </c>
+      <c r="F392" s="1" t="n">
+        <v>2710</v>
+      </c>
+      <c r="G392" s="1" t="inlineStr">
+        <is>
+          <t>HORTIFRUTI BOM DO CAMPO LTDA</t>
+        </is>
+      </c>
+      <c r="H392" s="1" t="n"/>
+      <c r="I392" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="n">
+        <v>46230.4132091088</v>
+      </c>
+      <c r="K392" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="L392" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M392" s="1" t="inlineStr">
+        <is>
+          <t>Francisco Pimenta</t>
+        </is>
+      </c>
+      <c r="N392" s="1" t="n"/>
+      <c r="O392" s="1" t="n"/>
+      <c r="P392" s="1" t="n"/>
+      <c r="Q392" s="1" t="inlineStr"/>
+      <c r="R392" s="1" t="n"/>
+      <c r="S392" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T392" s="1" t="n"/>
+      <c r="U392" s="1" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="1" t="n">
+        <v>81444</v>
+      </c>
+      <c r="B393" s="1" t="inlineStr">
+        <is>
+          <t>Levantamento de Débitos</t>
+        </is>
+      </c>
+      <c r="C393" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D393" s="1" t="inlineStr">
+        <is>
+          <t>EF - INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="E393" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia! Prezados,Por gentileza, poderia nos orientar como devemos prosseguir com a emissão de guia de ISS de débitos que estão constando no sistema de conformidade. No caso, não houve destaque do ISS devido pelo prestador, em algumas notas fiscais de serviços prestados. Porém, o recolhimento é devido. Devo gerar a guia avulsa para o cliente efetuar os pagamentos, e posteriormente ser aberto um processo administrativo? Aguardo a orientação correta. </t>
+        </is>
+      </c>
+      <c r="F393" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G393" s="1" t="n"/>
+      <c r="H393" s="1" t="n"/>
+      <c r="I393" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="n">
+        <v>46230.4154966088</v>
+      </c>
+      <c r="K393" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="L393" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M393" s="1" t="inlineStr">
+        <is>
+          <t>Thayna Melo</t>
+        </is>
+      </c>
+      <c r="N393" s="1" t="n"/>
+      <c r="O393" s="1" t="n"/>
+      <c r="P393" s="1" t="n"/>
+      <c r="Q393" s="1" t="inlineStr"/>
+      <c r="R393" s="1" t="n"/>
+      <c r="S393" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T393" s="1" t="n"/>
+      <c r="U393" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: atualização base chamados 27-07-26 1255
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U396" headerRowCount="1">
-  <autoFilter ref="A1:U396"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U397" headerRowCount="1">
+  <autoFilter ref="A1:U397"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U396"/>
+  <dimension ref="A1:U397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30710,6 +30710,69 @@
       <c r="T396" s="1" t="n"/>
       <c r="U396" s="1" t="inlineStr"/>
     </row>
+    <row r="397">
+      <c r="A397" s="1" t="n">
+        <v>81463</v>
+      </c>
+      <c r="B397" s="1" t="inlineStr">
+        <is>
+          <t>Regularização</t>
+        </is>
+      </c>
+      <c r="C397" s="1" t="inlineStr">
+        <is>
+          <t>Outro</t>
+        </is>
+      </c>
+      <c r="D397" s="1" t="inlineStr">
+        <is>
+          <t>SANTOS - GC</t>
+        </is>
+      </c>
+      <c r="E397" s="1" t="inlineStr">
+        <is>
+          <t>Poderiam por gentileza providenciar o CLI do cliente 2058 - SUPERMERCADO ONDAS DE PRAIA GRANDE LTDA</t>
+        </is>
+      </c>
+      <c r="F397" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G397" s="1" t="n"/>
+      <c r="H397" s="1" t="n"/>
+      <c r="I397" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J397" s="2" t="n">
+        <v>46230.51642866898</v>
+      </c>
+      <c r="K397" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="L397" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M397" s="1" t="inlineStr">
+        <is>
+          <t>Rafaella Massuia</t>
+        </is>
+      </c>
+      <c r="N397" s="1" t="n"/>
+      <c r="O397" s="1" t="n"/>
+      <c r="P397" s="1" t="n"/>
+      <c r="Q397" s="1" t="inlineStr"/>
+      <c r="R397" s="1" t="n"/>
+      <c r="S397" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T397" s="1" t="n"/>
+      <c r="U397" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
data: atualização base chamados 28-07-26 1304
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1978,7 +1978,7 @@
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M19" s="1" t="inlineStr">
@@ -1986,10 +1986,18 @@
           <t>Isabelli Afonso</t>
         </is>
       </c>
-      <c r="N19" s="1" t="n"/>
+      <c r="N19" s="2" t="n">
+        <v>46203.40876751157</v>
+      </c>
       <c r="O19" s="1" t="n"/>
-      <c r="P19" s="1" t="n"/>
-      <c r="Q19" s="1" t="inlineStr"/>
+      <c r="P19" s="2" t="n">
+        <v>46231.50784575231</v>
+      </c>
+      <c r="Q19" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R19" s="1" t="inlineStr">
         <is>
           <t>OPERAÇÃO VALIDANDO O QUESTIONAMENTO DA PREFEITURA</t>
@@ -1997,7 +2005,7 @@
       </c>
       <c r="S19" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T19" s="1" t="n"/>
@@ -7031,7 +7039,9 @@
         </is>
       </c>
       <c r="N81" s="1" t="n"/>
-      <c r="O81" s="1" t="n"/>
+      <c r="O81" s="2" t="n">
+        <v>46244</v>
+      </c>
       <c r="P81" s="1" t="n"/>
       <c r="Q81" s="1" t="inlineStr"/>
       <c r="R81" s="1" t="inlineStr"/>
@@ -7097,7 +7107,7 @@
       </c>
       <c r="L82" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M82" s="1" t="inlineStr">
@@ -7111,8 +7121,14 @@
       <c r="O82" s="2" t="n">
         <v>46233</v>
       </c>
-      <c r="P82" s="1" t="n"/>
-      <c r="Q82" s="1" t="inlineStr"/>
+      <c r="P82" s="2" t="n">
+        <v>46231.50410795139</v>
+      </c>
+      <c r="Q82" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R82" s="1" t="inlineStr">
         <is>
           <t>operação em validação 
@@ -7121,7 +7137,7 @@
       </c>
       <c r="S82" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T82" s="1" t="n"/>
@@ -12368,7 +12384,7 @@
       </c>
       <c r="L146" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M146" s="1" t="inlineStr">
@@ -12380,8 +12396,14 @@
       <c r="O146" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="P146" s="1" t="n"/>
-      <c r="Q146" s="1" t="inlineStr"/>
+      <c r="P146" s="2" t="n">
+        <v>46231.50914070602</v>
+      </c>
+      <c r="Q146" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R146" s="1" t="inlineStr">
         <is>
           <t>PRCOESSO REALIZADO EM 10-07-2026</t>
@@ -12389,7 +12411,7 @@
       </c>
       <c r="S146" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T146" s="1" t="n"/>
@@ -12449,7 +12471,7 @@
       </c>
       <c r="L147" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M147" s="1" t="inlineStr">
@@ -12461,8 +12483,14 @@
       <c r="O147" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="P147" s="1" t="n"/>
-      <c r="Q147" s="1" t="inlineStr"/>
+      <c r="P147" s="2" t="n">
+        <v>46231.50889270833</v>
+      </c>
+      <c r="Q147" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="R147" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">poderiam averiguar com o cliente para que ele pague a taxa ?
@@ -12471,7 +12499,7 @@
       </c>
       <c r="S147" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T147" s="1" t="n"/>
@@ -13297,7 +13325,9 @@
         </is>
       </c>
       <c r="N157" s="1" t="n"/>
-      <c r="O157" s="1" t="n"/>
+      <c r="O157" s="2" t="n">
+        <v>46244</v>
+      </c>
       <c r="P157" s="1" t="n"/>
       <c r="Q157" s="1" t="inlineStr"/>
       <c r="R157" s="1" t="inlineStr"/>
@@ -13372,7 +13402,9 @@
         </is>
       </c>
       <c r="N158" s="1" t="n"/>
-      <c r="O158" s="1" t="n"/>
+      <c r="O158" s="2" t="n">
+        <v>46244</v>
+      </c>
       <c r="P158" s="1" t="n"/>
       <c r="Q158" s="1" t="inlineStr"/>
       <c r="R158" s="1" t="inlineStr"/>
@@ -15971,7 +16003,7 @@
       </c>
       <c r="L190" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M190" s="1" t="inlineStr">
@@ -15979,7 +16011,9 @@
           <t>Beatriz Rangel</t>
         </is>
       </c>
-      <c r="N190" s="1" t="n"/>
+      <c r="N190" s="2" t="n">
+        <v>46203.40411403935</v>
+      </c>
       <c r="O190" s="1" t="n"/>
       <c r="P190" s="1" t="n"/>
       <c r="Q190" s="1" t="inlineStr"/>
@@ -21277,26 +21311,26 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>77913</v>
+        <v>81524</v>
       </c>
       <c r="B263" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C263" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Vencimento de Tarefas</t>
         </is>
       </c>
       <c r="D263" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E263" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t>Boa tarde!Por favor, alterar o vencimento das tarefas abaixo para o dia 30 a partir da competência 08/2026. O Pagamento do cliente é dentro do mês.Cliente 3693Folha Mensal /Pró-laboreRecibo de pagamentoRelação bancáriaObrigado</t>
         </is>
       </c>
       <c r="F263" s="1" t="n">
@@ -21305,42 +21339,35 @@
       <c r="G263" s="1" t="n"/>
       <c r="H263" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Gabriel Amaral</t>
         </is>
       </c>
       <c r="I263" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J263" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46231.51921663195</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>46097</v>
+        <v>46232</v>
       </c>
       <c r="L263" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M263" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
-        </is>
-      </c>
-      <c r="N263" s="2" t="n">
-        <v>46223.70421145833</v>
-      </c>
+          <t>David Bragança</t>
+        </is>
+      </c>
+      <c r="N263" s="1" t="n"/>
       <c r="O263" s="1" t="n"/>
       <c r="P263" s="1" t="n"/>
       <c r="Q263" s="1" t="inlineStr"/>
-      <c r="R263" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
-        </is>
-      </c>
+      <c r="R263" s="1" t="inlineStr"/>
       <c r="S263" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21351,39 +21378,35 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>79793</v>
+        <v>77913</v>
       </c>
       <c r="B264" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C264" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D264" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E264" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F264" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G264" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G264" s="1" t="n"/>
       <c r="H264" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I264" s="1" t="inlineStr">
@@ -21392,26 +21415,33 @@
         </is>
       </c>
       <c r="J264" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K264" s="2" t="n">
-        <v>46185</v>
+        <v>46097</v>
       </c>
       <c r="L264" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M264" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N264" s="1" t="n"/>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N264" s="2" t="n">
+        <v>46223.70421145833</v>
+      </c>
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
       <c r="Q264" s="1" t="inlineStr"/>
-      <c r="R264" s="1" t="inlineStr"/>
+      <c r="R264" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
+        </is>
+      </c>
       <c r="S264" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21422,34 +21452,34 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>79833</v>
+        <v>79793</v>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C265" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D265" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E265" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F265" s="1" t="n">
-        <v>6125</v>
+        <v>5655</v>
       </c>
       <c r="G265" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>VANESSA DUARTE RODRIGUES</t>
         </is>
       </c>
       <c r="H265" s="1" t="inlineStr">
@@ -21459,36 +21489,30 @@
       </c>
       <c r="I265" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J265" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K265" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L265" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M265" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N265" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N265" s="1" t="n"/>
       <c r="O265" s="1" t="n"/>
       <c r="P265" s="1" t="n"/>
       <c r="Q265" s="1" t="inlineStr"/>
-      <c r="R265" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R265" s="1" t="inlineStr"/>
       <c r="S265" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21499,7 +21523,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>79834</v>
+        <v>79833</v>
       </c>
       <c r="B266" s="1" t="inlineStr">
         <is>
@@ -21522,11 +21546,11 @@
         </is>
       </c>
       <c r="F266" s="1" t="n">
-        <v>6162</v>
+        <v>6125</v>
       </c>
       <c r="G266" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H266" s="1" t="inlineStr">
@@ -21540,14 +21564,14 @@
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K266" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="L266" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M266" s="1" t="inlineStr">
@@ -21555,11 +21579,17 @@
           <t>Tatiana Linardi</t>
         </is>
       </c>
-      <c r="N266" s="1" t="n"/>
+      <c r="N266" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
       <c r="Q266" s="1" t="inlineStr"/>
-      <c r="R266" s="1" t="inlineStr"/>
+      <c r="R266" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S266" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21570,7 +21600,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>79835</v>
+        <v>79834</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
@@ -21593,11 +21623,11 @@
         </is>
       </c>
       <c r="F267" s="1" t="n">
-        <v>6485</v>
+        <v>6162</v>
       </c>
       <c r="G267" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H267" s="1" t="inlineStr">
@@ -21611,7 +21641,7 @@
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K267" s="2" t="n">
         <v>46184</v>
@@ -21641,16 +21671,16 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>79854</v>
+        <v>79835</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C268" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D268" s="1" t="inlineStr">
@@ -21660,15 +21690,15 @@
       </c>
       <c r="E268" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F268" s="1" t="n">
-        <v>6302</v>
+        <v>6485</v>
       </c>
       <c r="G268" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H268" s="1" t="inlineStr">
@@ -21682,7 +21712,7 @@
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K268" s="2" t="n">
         <v>46184</v>
@@ -21712,7 +21742,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>79855</v>
+        <v>79854</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
@@ -21731,15 +21761,15 @@
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
-        <v>4765</v>
+        <v>6302</v>
       </c>
       <c r="G269" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H269" s="1" t="inlineStr">
@@ -21753,10 +21783,10 @@
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L269" s="1" t="inlineStr">
         <is>
@@ -21783,7 +21813,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>79856</v>
+        <v>79855</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
@@ -21802,15 +21832,15 @@
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
-        <v>4225</v>
+        <v>4765</v>
       </c>
       <c r="G270" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H270" s="1" t="inlineStr">
@@ -21824,10 +21854,10 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
@@ -21854,7 +21884,7 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>79859</v>
+        <v>79856</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
@@ -21873,15 +21903,15 @@
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
-        <v>6570</v>
+        <v>4225</v>
       </c>
       <c r="G271" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H271" s="1" t="inlineStr">
@@ -21895,10 +21925,10 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21907,7 +21937,7 @@
       </c>
       <c r="M271" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N271" s="1" t="n"/>
@@ -21925,7 +21955,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>79860</v>
+        <v>79859</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
@@ -21944,15 +21974,15 @@
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
-        <v>6581</v>
+        <v>6570</v>
       </c>
       <c r="G272" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H272" s="1" t="inlineStr">
@@ -21966,7 +21996,7 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K272" s="2" t="n">
         <v>46185</v>
@@ -21996,7 +22026,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>79861</v>
+        <v>79860</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22015,15 +22045,15 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
-        <v>6583</v>
+        <v>6581</v>
       </c>
       <c r="G273" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H273" s="1" t="inlineStr">
@@ -22037,7 +22067,7 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K273" s="2" t="n">
         <v>46185</v>
@@ -22067,7 +22097,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>79863</v>
+        <v>79861</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22086,15 +22116,15 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>6404</v>
+        <v>6583</v>
       </c>
       <c r="G274" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H274" s="1" t="inlineStr">
@@ -22108,7 +22138,7 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K274" s="2" t="n">
         <v>46185</v>
@@ -22138,7 +22168,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>79865</v>
+        <v>79863</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22157,15 +22187,15 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
-        <v>6278</v>
+        <v>6404</v>
       </c>
       <c r="G275" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H275" s="1" t="inlineStr">
@@ -22179,7 +22209,7 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K275" s="2" t="n">
         <v>46185</v>
@@ -22209,7 +22239,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>79866</v>
+        <v>79865</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22228,15 +22258,15 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
-        <v>6539</v>
+        <v>6278</v>
       </c>
       <c r="G276" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H276" s="1" t="inlineStr">
@@ -22250,7 +22280,7 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K276" s="2" t="n">
         <v>46185</v>
@@ -22280,16 +22310,16 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>79867</v>
+        <v>79866</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C277" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D277" s="1" t="inlineStr">
@@ -22299,15 +22329,15 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
-        <v>6704</v>
+        <v>6539</v>
       </c>
       <c r="G277" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H277" s="1" t="inlineStr">
@@ -22321,7 +22351,7 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K277" s="2" t="n">
         <v>46185</v>
@@ -22351,69 +22381,67 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>80515</v>
+        <v>79867</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G278" s="1" t="n"/>
+        <v>6704</v>
+      </c>
+      <c r="G278" s="1" t="inlineStr">
+        <is>
+          <t>TECNO COM INFORMATICA LTDA</t>
+        </is>
+      </c>
       <c r="H278" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I278" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>46226</v>
+        <v>46185</v>
       </c>
       <c r="L278" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M278" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N278" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N278" s="1" t="n"/>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="Q278" s="1" t="inlineStr"/>
-      <c r="R278" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R278" s="1" t="inlineStr"/>
       <c r="S278" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22424,7 +22452,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80697</v>
+        <v>80515</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
@@ -22433,7 +22461,7 @@
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
@@ -22443,7 +22471,7 @@
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
@@ -22461,10 +22489,10 @@
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46237</v>
+        <v>46226</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
@@ -22477,14 +22505,14 @@
         </is>
       </c>
       <c r="N279" s="2" t="n">
-        <v>46224.68237751158</v>
+        <v>46219.75157017361</v>
       </c>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
       <c r="R279" s="1" t="inlineStr">
         <is>
-          <t>Em atendimento</t>
+          <t xml:space="preserve">Enviado para registro </t>
         </is>
       </c>
       <c r="S279" s="1" t="inlineStr">
@@ -22497,7 +22525,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80714</v>
+        <v>80697</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
@@ -22506,7 +22534,7 @@
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22516,7 +22544,7 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22525,7 +22553,7 @@
       <c r="G280" s="1" t="n"/>
       <c r="H280" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I280" s="1" t="inlineStr">
@@ -22534,10 +22562,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22550,15 +22578,14 @@
         </is>
       </c>
       <c r="N280" s="2" t="n">
-        <v>46223.41822326389</v>
+        <v>46224.68237751158</v>
       </c>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
       <c r="R280" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+          <t>Em atendimento</t>
         </is>
       </c>
       <c r="S280" s="1" t="inlineStr">
@@ -22571,16 +22598,16 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>80919</v>
+        <v>80714</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22590,7 +22617,7 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22608,10 +22635,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22624,16 +22651,15 @@
         </is>
       </c>
       <c r="N281" s="2" t="n">
-        <v>46225.48500983796</v>
+        <v>46223.41822326389</v>
       </c>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="Q281" s="1" t="inlineStr"/>
       <c r="R281" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezadas(os), bom dia!
-Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
-Atenciosamente, </t>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
         </is>
       </c>
       <c r="S281" s="1" t="inlineStr">
@@ -22646,16 +22672,16 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>80935</v>
+        <v>80919</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
@@ -22665,7 +22691,7 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22683,10 +22709,10 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
@@ -22699,15 +22725,16 @@
         </is>
       </c>
       <c r="N282" s="2" t="n">
-        <v>46223.41869637732</v>
+        <v>46225.48500983796</v>
       </c>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
       <c r="R282" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+          <t xml:space="preserve">Prezadas(os), bom dia!
+Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
+Atenciosamente, </t>
         </is>
       </c>
       <c r="S282" s="1" t="inlineStr">
@@ -22720,7 +22747,7 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>80936</v>
+        <v>80935</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
@@ -22729,7 +22756,7 @@
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
@@ -22739,7 +22766,7 @@
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
@@ -22748,7 +22775,7 @@
       <c r="G283" s="1" t="n"/>
       <c r="H283" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I283" s="1" t="inlineStr">
@@ -22757,7 +22784,7 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K283" s="2" t="n">
         <v>46241</v>
@@ -22773,14 +22800,15 @@
         </is>
       </c>
       <c r="N283" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46223.41869637732</v>
       </c>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
       <c r="R283" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
         </is>
       </c>
       <c r="S283" s="1" t="inlineStr">
@@ -22793,7 +22821,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>80951</v>
+        <v>80936</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
@@ -22802,7 +22830,7 @@
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
@@ -22812,7 +22840,7 @@
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22830,7 +22858,7 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K284" s="2" t="n">
         <v>46241</v>
@@ -22846,14 +22874,14 @@
         </is>
       </c>
       <c r="N284" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
       <c r="R284" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S284" s="1" t="inlineStr">
@@ -22866,39 +22894,35 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>81004</v>
+        <v>80951</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>6869</v>
-      </c>
-      <c r="G285" s="1" t="inlineStr">
-        <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G285" s="1" t="n"/>
       <c r="H285" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I285" s="1" t="inlineStr">
@@ -22907,26 +22931,32 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>46218</v>
+        <v>46241</v>
       </c>
       <c r="L285" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M285" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
-      <c r="N285" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N285" s="2" t="n">
+        <v>46219.74920023148</v>
+      </c>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
-      <c r="R285" s="1" t="inlineStr"/>
+      <c r="R285" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviada ao cliente</t>
+        </is>
+      </c>
       <c r="S285" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22937,7 +22967,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>81005</v>
+        <v>81004</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
@@ -22960,16 +22990,16 @@
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6870</v>
+        <v>6869</v>
       </c>
       <c r="G286" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H286" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I286" s="1" t="inlineStr">
@@ -22978,7 +23008,7 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K286" s="2" t="n">
         <v>46218</v>
@@ -23008,68 +23038,67 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81019</v>
+        <v>81005</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C287" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D287" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E287" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G287" s="1" t="n"/>
+        <v>6870</v>
+      </c>
+      <c r="G287" s="1" t="inlineStr">
+        <is>
+          <t>AC HOME PET RAÇÕES LTDA</t>
+        </is>
+      </c>
       <c r="H287" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I287" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K287" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="L287" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M287" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N287" s="1" t="n"/>
       <c r="O287" s="1" t="n"/>
       <c r="P287" s="1" t="n"/>
       <c r="Q287" s="1" t="inlineStr"/>
-      <c r="R287" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
+      <c r="R287" s="1" t="inlineStr"/>
       <c r="S287" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23080,7 +23109,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>81052</v>
+        <v>81019</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
@@ -23099,7 +23128,7 @@
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
@@ -23117,10 +23146,10 @@
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
@@ -23129,7 +23158,7 @@
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
@@ -23138,7 +23167,8 @@
       <c r="Q288" s="1" t="inlineStr"/>
       <c r="R288" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
         </is>
       </c>
       <c r="S288" s="1" t="inlineStr">
@@ -23151,7 +23181,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81055</v>
+        <v>81052</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -23170,7 +23200,7 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
@@ -23188,14 +23218,14 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K289" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M289" s="1" t="inlineStr">
@@ -23203,15 +23233,13 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N289" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+      <c r="N289" s="1" t="n"/>
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
       <c r="Q289" s="1" t="inlineStr"/>
       <c r="R289" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S289" s="1" t="inlineStr">
@@ -23224,36 +23252,32 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>81091</v>
+        <v>81055</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C290" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D290" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>6907</v>
-      </c>
-      <c r="G290" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G290" s="1" t="n"/>
       <c r="H290" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23261,30 +23285,36 @@
       </c>
       <c r="I290" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>46223</v>
+        <v>46219</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
-        </is>
-      </c>
-      <c r="N290" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N290" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
-      <c r="R290" s="1" t="inlineStr"/>
+      <c r="R290" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
       <c r="S290" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23295,16 +23325,16 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81209</v>
+        <v>81091</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
@@ -23314,20 +23344,20 @@
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6094</v>
+        <v>6907</v>
       </c>
       <c r="G291" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H291" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I291" s="1" t="inlineStr">
@@ -23336,10 +23366,10 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
@@ -23366,16 +23396,16 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>81213</v>
+        <v>81209</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
@@ -23385,20 +23415,20 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Cliente não possuí acesso cadastrado</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6946</v>
+        <v>6094</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t>FFRA CONCRETOS LTDA</t>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
         </is>
       </c>
       <c r="H292" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I292" s="1" t="inlineStr">
@@ -23407,14 +23437,14 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46223.5798869213</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M292" s="1" t="inlineStr">
@@ -23422,17 +23452,11 @@
           <t>Denis Reis</t>
         </is>
       </c>
-      <c r="N292" s="2" t="n">
-        <v>46230.54938295139</v>
-      </c>
+      <c r="N292" s="1" t="n"/>
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
       <c r="Q292" s="1" t="inlineStr"/>
-      <c r="R292" s="1" t="inlineStr">
-        <is>
-          <t>Verificando os procedimentos para solicitação de cadastro.</t>
-        </is>
-      </c>
+      <c r="R292" s="1" t="inlineStr"/>
       <c r="S292" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23443,44 +23467,48 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>81215</v>
+        <v>81213</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C293" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D293" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>Cliente não possuí acesso cadastrado</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G293" s="1" t="n"/>
+        <v>6946</v>
+      </c>
+      <c r="G293" s="1" t="inlineStr">
+        <is>
+          <t>FFRA CONCRETOS LTDA</t>
+        </is>
+      </c>
       <c r="H293" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I293" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46223.60068402778</v>
+        <v>46223.5798869213</v>
       </c>
       <c r="K293" s="2" t="n">
         <v>46225</v>
@@ -23492,18 +23520,18 @@
       </c>
       <c r="M293" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N293" s="2" t="n">
-        <v>46225.56780570602</v>
+        <v>46230.54938295139</v>
       </c>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
       <c r="R293" s="1" t="inlineStr">
         <is>
-          <t>Cobramos novamente a contabilidade.</t>
+          <t>Verificando os procedimentos para solicitação de cadastro.</t>
         </is>
       </c>
       <c r="S293" s="1" t="inlineStr">
@@ -23516,7 +23544,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>81217</v>
+        <v>81215</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
@@ -23535,7 +23563,7 @@
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
@@ -23553,7 +23581,7 @@
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46223.60780787037</v>
+        <v>46223.60068402778</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>46225</v>
@@ -23569,14 +23597,14 @@
         </is>
       </c>
       <c r="N294" s="2" t="n">
-        <v>46225.56888491898</v>
+        <v>46225.56780570602</v>
       </c>
       <c r="O294" s="1" t="n"/>
       <c r="P294" s="1" t="n"/>
       <c r="Q294" s="1" t="inlineStr"/>
       <c r="R294" s="1" t="inlineStr">
         <is>
-          <t>Cobramos novamente.</t>
+          <t>Cobramos novamente a contabilidade.</t>
         </is>
       </c>
       <c r="S294" s="1" t="inlineStr">
@@ -23589,7 +23617,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>81218</v>
+        <v>81217</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
@@ -23608,7 +23636,7 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
@@ -23626,7 +23654,7 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46223.6082516551</v>
+        <v>46223.60780787037</v>
       </c>
       <c r="K295" s="2" t="n">
         <v>46225</v>
@@ -23642,7 +23670,7 @@
         </is>
       </c>
       <c r="N295" s="2" t="n">
-        <v>46225.57019641204</v>
+        <v>46225.56888491898</v>
       </c>
       <c r="O295" s="1" t="n"/>
       <c r="P295" s="1" t="n"/>
@@ -23662,26 +23690,26 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>81227</v>
+        <v>81218</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C296" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D296" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E296" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
@@ -23690,35 +23718,41 @@
       <c r="G296" s="1" t="n"/>
       <c r="H296" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I296" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46223.6082516551</v>
       </c>
       <c r="K296" s="2" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L296" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M296" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
-        </is>
-      </c>
-      <c r="N296" s="1" t="n"/>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N296" s="2" t="n">
+        <v>46225.57019641204</v>
+      </c>
       <c r="O296" s="1" t="n"/>
       <c r="P296" s="1" t="n"/>
       <c r="Q296" s="1" t="inlineStr"/>
-      <c r="R296" s="1" t="inlineStr"/>
+      <c r="R296" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos novamente.</t>
+        </is>
+      </c>
       <c r="S296" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23729,26 +23763,26 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>81228</v>
+        <v>81227</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
@@ -23757,74 +23791,65 @@
       <c r="G297" s="1" t="n"/>
       <c r="H297" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I297" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46223.70694884259</v>
+        <v>46223.69836307871</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N297" s="1" t="n"/>
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
       <c r="Q297" s="1" t="inlineStr"/>
-      <c r="R297" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Estou verificando o acesso  junto a prefeitura.</t>
-        </is>
-      </c>
+      <c r="R297" s="1" t="inlineStr"/>
       <c r="S297" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T297" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
+      <c r="T297" s="1" t="n"/>
       <c r="U297" s="1" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>81244</v>
+        <v>81228</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C298" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D298" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
+          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
@@ -23833,39 +23858,38 @@
       <c r="G298" s="1" t="n"/>
       <c r="H298" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I298" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46224.42615887732</v>
+        <v>46223.70694884259</v>
       </c>
       <c r="K298" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N298" s="2" t="n">
-        <v>46225.4986497338</v>
-      </c>
+          <t>Beatriz Ferreira</t>
+        </is>
+      </c>
+      <c r="N298" s="1" t="n"/>
       <c r="O298" s="1" t="n"/>
       <c r="P298" s="1" t="n"/>
       <c r="Q298" s="1" t="inlineStr"/>
       <c r="R298" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aguardando contato do contador. </t>
+          <t>Boa tarde!
+Estou verificando o acesso  junto a prefeitura.</t>
         </is>
       </c>
       <c r="S298" s="1" t="inlineStr">
@@ -23873,12 +23897,16 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T298" s="1" t="n"/>
+      <c r="T298" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
       <c r="U298" s="1" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>81245</v>
+        <v>81244</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
@@ -23897,7 +23925,7 @@
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
+          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
@@ -23915,7 +23943,7 @@
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46224.42947079861</v>
+        <v>46224.42615887732</v>
       </c>
       <c r="K299" s="2" t="n">
         <v>46226</v>
@@ -23931,14 +23959,14 @@
         </is>
       </c>
       <c r="N299" s="2" t="n">
-        <v>46225.4960193287</v>
+        <v>46225.4986497338</v>
       </c>
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
       <c r="Q299" s="1" t="inlineStr"/>
       <c r="R299" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobramos novamente. </t>
+          <t xml:space="preserve">Aguardando contato do contador. </t>
         </is>
       </c>
       <c r="S299" s="1" t="inlineStr">
@@ -23951,7 +23979,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>81247</v>
+        <v>81245</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
@@ -23970,7 +23998,7 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
@@ -23988,14 +24016,14 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46224.42947079861</v>
       </c>
       <c r="K300" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L300" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M300" s="1" t="inlineStr">
@@ -24003,13 +24031,15 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N300" s="1" t="n"/>
+      <c r="N300" s="2" t="n">
+        <v>46225.4960193287</v>
+      </c>
       <c r="O300" s="1" t="n"/>
       <c r="P300" s="1" t="n"/>
       <c r="Q300" s="1" t="inlineStr"/>
       <c r="R300" s="1" t="inlineStr">
         <is>
-          <t>Aguardando os dados do contador.</t>
+          <t xml:space="preserve">Cobramos novamente. </t>
         </is>
       </c>
       <c r="S300" s="1" t="inlineStr">
@@ -24022,7 +24052,7 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>81248</v>
+        <v>81247</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
@@ -24041,7 +24071,7 @@
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
@@ -24059,14 +24089,14 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46224.43289853009</v>
+        <v>46224.43143758102</v>
       </c>
       <c r="K301" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M301" s="1" t="inlineStr">
@@ -24074,15 +24104,13 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N301" s="2" t="n">
-        <v>46225.48954270833</v>
-      </c>
+      <c r="N301" s="1" t="n"/>
       <c r="O301" s="1" t="n"/>
       <c r="P301" s="1" t="n"/>
       <c r="Q301" s="1" t="inlineStr"/>
       <c r="R301" s="1" t="inlineStr">
         <is>
-          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+          <t>Aguardando os dados do contador.</t>
         </is>
       </c>
       <c r="S301" s="1" t="inlineStr">
@@ -24095,26 +24123,26 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>81250</v>
+        <v>81248</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C302" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D302" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
+          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
@@ -24123,35 +24151,41 @@
       <c r="G302" s="1" t="n"/>
       <c r="H302" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I302" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46224.44502184028</v>
+        <v>46224.43289853009</v>
       </c>
       <c r="K302" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L302" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M302" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
-        </is>
-      </c>
-      <c r="N302" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N302" s="2" t="n">
+        <v>46225.48954270833</v>
+      </c>
       <c r="O302" s="1" t="n"/>
       <c r="P302" s="1" t="n"/>
       <c r="Q302" s="1" t="inlineStr"/>
-      <c r="R302" s="1" t="inlineStr"/>
+      <c r="R302" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+        </is>
+      </c>
       <c r="S302" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24162,7 +24196,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>81251</v>
+        <v>81250</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
@@ -24181,7 +24215,7 @@
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
+          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
@@ -24199,7 +24233,7 @@
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46224.44796296296</v>
+        <v>46224.44502184028</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46226</v>
@@ -24229,26 +24263,26 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>81267</v>
+        <v>81251</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C304" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D304" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
+          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
@@ -24266,10 +24300,10 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46224.66958634259</v>
+        <v>46224.44796296296</v>
       </c>
       <c r="K304" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L304" s="1" t="inlineStr">
         <is>
@@ -24278,7 +24312,7 @@
       </c>
       <c r="M304" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Rafaella Massuia</t>
         </is>
       </c>
       <c r="N304" s="1" t="n"/>
@@ -24296,39 +24330,35 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>81270</v>
+        <v>81267</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C305" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D305" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
+          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
-        <v>5604</v>
-      </c>
-      <c r="G305" s="1" t="inlineStr">
-        <is>
-          <t>GRAFICA TABOAO LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G305" s="1" t="n"/>
       <c r="H305" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I305" s="1" t="inlineStr">
@@ -24337,32 +24367,26 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46224.69047569444</v>
+        <v>46224.66958634259</v>
       </c>
       <c r="K305" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="L305" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M305" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N305" s="1" t="n"/>
       <c r="O305" s="1" t="n"/>
       <c r="P305" s="1" t="n"/>
       <c r="Q305" s="1" t="inlineStr"/>
-      <c r="R305" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.
-Por gentileza, solicitar o AVCB e o IPTU (vigentes).
-Att,</t>
-        </is>
-      </c>
+      <c r="R305" s="1" t="inlineStr"/>
       <c r="S305" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24373,35 +24397,39 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>81274</v>
+        <v>81270</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C306" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D306" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
+          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G306" s="1" t="n"/>
+        <v>5604</v>
+      </c>
+      <c r="G306" s="1" t="inlineStr">
+        <is>
+          <t>GRAFICA TABOAO LTDA</t>
+        </is>
+      </c>
       <c r="H306" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I306" s="1" t="inlineStr">
@@ -24410,26 +24438,32 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46224.71483579861</v>
+        <v>46224.69047569444</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N306" s="1" t="n"/>
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="n"/>
       <c r="Q306" s="1" t="inlineStr"/>
-      <c r="R306" s="1" t="inlineStr"/>
+      <c r="R306" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.
+Por gentileza, solicitar o AVCB e o IPTU (vigentes).
+Att,</t>
+        </is>
+      </c>
       <c r="S306" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24440,39 +24474,35 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>81316</v>
+        <v>81274</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C307" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inclusão de Ata </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D307" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E307" s="1" t="inlineStr">
         <is>
-          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
+          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
-        <v>6674</v>
-      </c>
-      <c r="G307" s="1" t="inlineStr">
-        <is>
-          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G307" s="1" t="n"/>
       <c r="H307" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I307" s="1" t="inlineStr">
@@ -24481,39 +24511,29 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46225.61705821759</v>
+        <v>46224.71483579861</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>46231</v>
+        <v>46226</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M307" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N307" s="1" t="n"/>
       <c r="O307" s="1" t="n"/>
-      <c r="P307" s="2" t="n">
-        <v>46230.66303518519</v>
-      </c>
-      <c r="Q307" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R307" s="1" t="inlineStr">
-        <is>
-          <t>Enviar a planilha devidamente preenchida e completa.</t>
-        </is>
-      </c>
+      <c r="P307" s="1" t="n"/>
+      <c r="Q307" s="1" t="inlineStr"/>
+      <c r="R307" s="1" t="inlineStr"/>
       <c r="S307" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T307" s="1" t="n"/>
@@ -24521,7 +24541,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>81317</v>
+        <v>81316</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
@@ -24540,15 +24560,15 @@
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
+          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
-        <v>6673</v>
+        <v>6674</v>
       </c>
       <c r="G308" s="1" t="inlineStr">
         <is>
-          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
+          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
         </is>
       </c>
       <c r="H308" s="1" t="inlineStr">
@@ -24562,7 +24582,7 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46225.61752997685</v>
+        <v>46225.61705821759</v>
       </c>
       <c r="K308" s="2" t="n">
         <v>46231</v>
@@ -24580,7 +24600,7 @@
       <c r="N308" s="1" t="n"/>
       <c r="O308" s="1" t="n"/>
       <c r="P308" s="2" t="n">
-        <v>46230.66237318287</v>
+        <v>46230.66303518519</v>
       </c>
       <c r="Q308" s="1" t="inlineStr">
         <is>
@@ -24589,7 +24609,7 @@
       </c>
       <c r="R308" s="1" t="inlineStr">
         <is>
-          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
+          <t>Enviar a planilha devidamente preenchida e completa.</t>
         </is>
       </c>
       <c r="S308" s="1" t="inlineStr">
@@ -24602,34 +24622,34 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>81343</v>
+        <v>81317</v>
       </c>
       <c r="B309" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C309" s="1" t="inlineStr">
         <is>
-          <t>Protestos</t>
+          <t xml:space="preserve">Inclusão de Ata </t>
         </is>
       </c>
       <c r="D309" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E309" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
+          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
         </is>
       </c>
       <c r="F309" s="1" t="n">
-        <v>6538</v>
+        <v>6673</v>
       </c>
       <c r="G309" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
         </is>
       </c>
       <c r="H309" s="1" t="inlineStr">
@@ -24643,10 +24663,10 @@
         </is>
       </c>
       <c r="J309" s="2" t="n">
-        <v>46225.78787369213</v>
+        <v>46225.61752997685</v>
       </c>
       <c r="K309" s="2" t="n">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="L309" s="1" t="inlineStr">
         <is>
@@ -24655,13 +24675,13 @@
       </c>
       <c r="M309" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="N309" s="1" t="n"/>
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="2" t="n">
-        <v>46230.55531678241</v>
+        <v>46230.66237318287</v>
       </c>
       <c r="Q309" s="1" t="inlineStr">
         <is>
@@ -24670,7 +24690,7 @@
       </c>
       <c r="R309" s="1" t="inlineStr">
         <is>
-          <t>SEGUE BOLETO DAS CUSTAS SOLICITADAS.</t>
+          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
         </is>
       </c>
       <c r="S309" s="1" t="inlineStr">
@@ -24683,73 +24703,80 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>81348</v>
+        <v>81343</v>
       </c>
       <c r="B310" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C310" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Protestos</t>
         </is>
       </c>
       <c r="D310" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E310" s="1" t="inlineStr">
         <is>
-          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
+          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
         </is>
       </c>
       <c r="F310" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G310" s="1" t="n"/>
+        <v>6538</v>
+      </c>
+      <c r="G310" s="1" t="inlineStr">
+        <is>
+          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+        </is>
+      </c>
       <c r="H310" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I310" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J310" s="2" t="n">
-        <v>46226.4148858449</v>
+        <v>46225.78787369213</v>
       </c>
       <c r="K310" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="L310" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M310" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N310" s="2" t="n">
-        <v>46230.72068440972</v>
-      </c>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N310" s="1" t="n"/>
       <c r="O310" s="1" t="n"/>
-      <c r="P310" s="1" t="n"/>
-      <c r="Q310" s="1" t="inlineStr"/>
+      <c r="P310" s="2" t="n">
+        <v>46230.55531678241</v>
+      </c>
+      <c r="Q310" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="R310" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!
-Cobramos novamente.</t>
+          <t>SEGUE BOLETO DAS CUSTAS SOLICITADAS.</t>
         </is>
       </c>
       <c r="S310" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T310" s="1" t="n"/>
@@ -24757,67 +24784,70 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>81351</v>
+        <v>81348</v>
       </c>
       <c r="B311" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C311" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D311" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E311" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
         </is>
       </c>
       <c r="F311" s="1" t="n">
-        <v>3587</v>
-      </c>
-      <c r="G311" s="1" t="inlineStr">
-        <is>
-          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G311" s="1" t="n"/>
       <c r="H311" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I311" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J311" s="2" t="n">
-        <v>46226.44303796296</v>
+        <v>46226.4148858449</v>
       </c>
       <c r="K311" s="2" t="n">
-        <v>46230</v>
+        <v>46227</v>
       </c>
       <c r="L311" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M311" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
-        </is>
-      </c>
-      <c r="N311" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N311" s="2" t="n">
+        <v>46230.72068440972</v>
+      </c>
       <c r="O311" s="1" t="n"/>
       <c r="P311" s="1" t="n"/>
       <c r="Q311" s="1" t="inlineStr"/>
-      <c r="R311" s="1" t="inlineStr"/>
+      <c r="R311" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Cobramos novamente.</t>
+        </is>
+      </c>
       <c r="S311" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24828,7 +24858,7 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>81352</v>
+        <v>81351</v>
       </c>
       <c r="B312" s="1" t="inlineStr">
         <is>
@@ -24851,16 +24881,16 @@
         </is>
       </c>
       <c r="F312" s="1" t="n">
-        <v>3812</v>
+        <v>3587</v>
       </c>
       <c r="G312" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
+          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
         </is>
       </c>
       <c r="H312" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I312" s="1" t="inlineStr">
@@ -24869,14 +24899,14 @@
         </is>
       </c>
       <c r="J312" s="2" t="n">
-        <v>46226.4440716088</v>
+        <v>46226.44303796296</v>
       </c>
       <c r="K312" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L312" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M312" s="1" t="inlineStr">
@@ -24884,18 +24914,11 @@
           <t>Francisco Pimenta</t>
         </is>
       </c>
-      <c r="N312" s="2" t="n">
-        <v>46230.66455783565</v>
-      </c>
+      <c r="N312" s="1" t="n"/>
       <c r="O312" s="1" t="n"/>
       <c r="P312" s="1" t="n"/>
       <c r="Q312" s="1" t="inlineStr"/>
-      <c r="R312" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Estou verificando o acesso junto a prefeitura.</t>
-        </is>
-      </c>
+      <c r="R312" s="1" t="inlineStr"/>
       <c r="S312" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24906,7 +24929,7 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>81353</v>
+        <v>81352</v>
       </c>
       <c r="B313" s="1" t="inlineStr">
         <is>
@@ -24929,11 +24952,11 @@
         </is>
       </c>
       <c r="F313" s="1" t="n">
-        <v>3878</v>
+        <v>3812</v>
       </c>
       <c r="G313" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cucinare Pro Alimentação </t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
         </is>
       </c>
       <c r="H313" s="1" t="inlineStr">
@@ -24947,7 +24970,7 @@
         </is>
       </c>
       <c r="J313" s="2" t="n">
-        <v>46226.44431542824</v>
+        <v>46226.4440716088</v>
       </c>
       <c r="K313" s="2" t="n">
         <v>46230</v>
@@ -24963,7 +24986,7 @@
         </is>
       </c>
       <c r="N313" s="2" t="n">
-        <v>46230.66437326389</v>
+        <v>46230.66455783565</v>
       </c>
       <c r="O313" s="1" t="n"/>
       <c r="P313" s="1" t="n"/>
@@ -24984,7 +25007,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>81355</v>
+        <v>81353</v>
       </c>
       <c r="B314" s="1" t="inlineStr">
         <is>
@@ -25007,11 +25030,11 @@
         </is>
       </c>
       <c r="F314" s="1" t="n">
-        <v>4012</v>
+        <v>3878</v>
       </c>
       <c r="G314" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+          <t xml:space="preserve">Cucinare Pro Alimentação </t>
         </is>
       </c>
       <c r="H314" s="1" t="inlineStr">
@@ -25025,7 +25048,7 @@
         </is>
       </c>
       <c r="J314" s="2" t="n">
-        <v>46226.44472357639</v>
+        <v>46226.44431542824</v>
       </c>
       <c r="K314" s="2" t="n">
         <v>46230</v>
@@ -25041,89 +25064,96 @@
         </is>
       </c>
       <c r="N314" s="2" t="n">
-        <v>46230.66408684028</v>
+        <v>46230.66437326389</v>
       </c>
       <c r="O314" s="1" t="n"/>
       <c r="P314" s="1" t="n"/>
       <c r="Q314" s="1" t="inlineStr"/>
       <c r="R314" s="1" t="inlineStr">
         <is>
+          <t>Boa tarde!
+Estou verificando o acesso junto a prefeitura.</t>
+        </is>
+      </c>
+      <c r="S314" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T314" s="1" t="n"/>
+      <c r="U314" s="1" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="1" t="n">
+        <v>81355</v>
+      </c>
+      <c r="B315" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C315" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D315" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E315" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+        </is>
+      </c>
+      <c r="F315" s="1" t="n">
+        <v>4012</v>
+      </c>
+      <c r="G315" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+        </is>
+      </c>
+      <c r="H315" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
+      <c r="I315" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="n">
+        <v>46226.44472357639</v>
+      </c>
+      <c r="K315" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="L315" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M315" s="1" t="inlineStr">
+        <is>
+          <t>Francisco Pimenta</t>
+        </is>
+      </c>
+      <c r="N315" s="2" t="n">
+        <v>46230.66408684028</v>
+      </c>
+      <c r="O315" s="1" t="n"/>
+      <c r="P315" s="1" t="n"/>
+      <c r="Q315" s="1" t="inlineStr"/>
+      <c r="R315" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Boa tarde!
 Estou verificando o acesso junto a prefeitura.
 </t>
         </is>
       </c>
-      <c r="S314" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T314" s="1" t="n"/>
-      <c r="U314" s="1" t="inlineStr"/>
-    </row>
-    <row r="315">
-      <c r="A315" s="1" t="n">
-        <v>81362</v>
-      </c>
-      <c r="B315" s="1" t="inlineStr">
-        <is>
-          <t>Senha</t>
-        </is>
-      </c>
-      <c r="C315" s="1" t="inlineStr">
-        <is>
-          <t>Prefeitura</t>
-        </is>
-      </c>
-      <c r="D315" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="E315" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
-        </is>
-      </c>
-      <c r="F315" s="1" t="n">
-        <v>4804</v>
-      </c>
-      <c r="G315" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
-        </is>
-      </c>
-      <c r="H315" s="1" t="inlineStr">
-        <is>
-          <t>Talita Silva</t>
-        </is>
-      </c>
-      <c r="I315" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J315" s="2" t="n">
-        <v>46226.44931420139</v>
-      </c>
-      <c r="K315" s="2" t="n">
-        <v>46230</v>
-      </c>
-      <c r="L315" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M315" s="1" t="inlineStr">
-        <is>
-          <t>Francisco Pimenta</t>
-        </is>
-      </c>
-      <c r="N315" s="1" t="n"/>
-      <c r="O315" s="1" t="n"/>
-      <c r="P315" s="1" t="n"/>
-      <c r="Q315" s="1" t="inlineStr"/>
-      <c r="R315" s="1" t="inlineStr"/>
       <c r="S315" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25134,7 +25164,7 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="n">
-        <v>81363</v>
+        <v>81362</v>
       </c>
       <c r="B316" s="1" t="inlineStr">
         <is>
@@ -25157,11 +25187,11 @@
         </is>
       </c>
       <c r="F316" s="1" t="n">
-        <v>4841</v>
+        <v>4804</v>
       </c>
       <c r="G316" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
+          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
         </is>
       </c>
       <c r="H316" s="1" t="inlineStr">
@@ -25175,7 +25205,7 @@
         </is>
       </c>
       <c r="J316" s="2" t="n">
-        <v>46226.45019482639</v>
+        <v>46226.44931420139</v>
       </c>
       <c r="K316" s="2" t="n">
         <v>46230</v>
@@ -25205,7 +25235,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>81364</v>
+        <v>81363</v>
       </c>
       <c r="B317" s="1" t="inlineStr">
         <is>
@@ -25228,11 +25258,11 @@
         </is>
       </c>
       <c r="F317" s="1" t="n">
-        <v>4918</v>
+        <v>4841</v>
       </c>
       <c r="G317" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
+          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H317" s="1" t="inlineStr">
@@ -25246,7 +25276,7 @@
         </is>
       </c>
       <c r="J317" s="2" t="n">
-        <v>46226.45123028935</v>
+        <v>46226.45019482639</v>
       </c>
       <c r="K317" s="2" t="n">
         <v>46230</v>
@@ -25276,7 +25306,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>81365</v>
+        <v>81364</v>
       </c>
       <c r="B318" s="1" t="inlineStr">
         <is>
@@ -25299,11 +25329,11 @@
         </is>
       </c>
       <c r="F318" s="1" t="n">
-        <v>5017</v>
+        <v>4918</v>
       </c>
       <c r="G318" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
         </is>
       </c>
       <c r="H318" s="1" t="inlineStr">
@@ -25317,7 +25347,7 @@
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>46226.45200285879</v>
+        <v>46226.45123028935</v>
       </c>
       <c r="K318" s="2" t="n">
         <v>46230</v>
@@ -25347,7 +25377,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>81367</v>
+        <v>81365</v>
       </c>
       <c r="B319" s="1" t="inlineStr">
         <is>
@@ -25370,11 +25400,11 @@
         </is>
       </c>
       <c r="F319" s="1" t="n">
-        <v>5153</v>
+        <v>5017</v>
       </c>
       <c r="G319" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
         </is>
       </c>
       <c r="H319" s="1" t="inlineStr">
@@ -25388,7 +25418,7 @@
         </is>
       </c>
       <c r="J319" s="2" t="n">
-        <v>46226.45361840277</v>
+        <v>46226.45200285879</v>
       </c>
       <c r="K319" s="2" t="n">
         <v>46230</v>
@@ -25418,7 +25448,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>81368</v>
+        <v>81367</v>
       </c>
       <c r="B320" s="1" t="inlineStr">
         <is>
@@ -25441,11 +25471,11 @@
         </is>
       </c>
       <c r="F320" s="1" t="n">
-        <v>5154</v>
+        <v>5153</v>
       </c>
       <c r="G320" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
         </is>
       </c>
       <c r="H320" s="1" t="inlineStr">
@@ -25459,7 +25489,7 @@
         </is>
       </c>
       <c r="J320" s="2" t="n">
-        <v>46226.45395802084</v>
+        <v>46226.45361840277</v>
       </c>
       <c r="K320" s="2" t="n">
         <v>46230</v>
@@ -25489,7 +25519,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>81369</v>
+        <v>81368</v>
       </c>
       <c r="B321" s="1" t="inlineStr">
         <is>
@@ -25508,15 +25538,15 @@
       </c>
       <c r="E321" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F321" s="1" t="n">
-        <v>3049</v>
+        <v>5154</v>
       </c>
       <c r="G321" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
         </is>
       </c>
       <c r="H321" s="1" t="inlineStr">
@@ -25530,7 +25560,7 @@
         </is>
       </c>
       <c r="J321" s="2" t="n">
-        <v>46226.45434436342</v>
+        <v>46226.45395802084</v>
       </c>
       <c r="K321" s="2" t="n">
         <v>46230</v>
@@ -25542,7 +25572,7 @@
       </c>
       <c r="M321" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N321" s="1" t="n"/>
@@ -25560,7 +25590,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>81370</v>
+        <v>81369</v>
       </c>
       <c r="B322" s="1" t="inlineStr">
         <is>
@@ -25579,15 +25609,15 @@
       </c>
       <c r="E322" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
-        <v>5222</v>
+        <v>3049</v>
       </c>
       <c r="G322" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
         </is>
       </c>
       <c r="H322" s="1" t="inlineStr">
@@ -25601,7 +25631,7 @@
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>46226.45476809028</v>
+        <v>46226.45434436342</v>
       </c>
       <c r="K322" s="2" t="n">
         <v>46230</v>
@@ -25613,7 +25643,7 @@
       </c>
       <c r="M322" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N322" s="1" t="n"/>
@@ -25631,7 +25661,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>81371</v>
+        <v>81370</v>
       </c>
       <c r="B323" s="1" t="inlineStr">
         <is>
@@ -25654,11 +25684,11 @@
         </is>
       </c>
       <c r="F323" s="1" t="n">
-        <v>5224</v>
+        <v>5222</v>
       </c>
       <c r="G323" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
         </is>
       </c>
       <c r="H323" s="1" t="inlineStr">
@@ -25672,7 +25702,7 @@
         </is>
       </c>
       <c r="J323" s="2" t="n">
-        <v>46226.45489934028</v>
+        <v>46226.45476809028</v>
       </c>
       <c r="K323" s="2" t="n">
         <v>46230</v>
@@ -25702,7 +25732,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>81372</v>
+        <v>81371</v>
       </c>
       <c r="B324" s="1" t="inlineStr">
         <is>
@@ -25725,11 +25755,11 @@
         </is>
       </c>
       <c r="F324" s="1" t="n">
-        <v>5311</v>
+        <v>5224</v>
       </c>
       <c r="G324" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
         </is>
       </c>
       <c r="H324" s="1" t="inlineStr">
@@ -25743,7 +25773,7 @@
         </is>
       </c>
       <c r="J324" s="2" t="n">
-        <v>46226.45548961806</v>
+        <v>46226.45489934028</v>
       </c>
       <c r="K324" s="2" t="n">
         <v>46230</v>
@@ -25773,7 +25803,7 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>81375</v>
+        <v>81372</v>
       </c>
       <c r="B325" s="1" t="inlineStr">
         <is>
@@ -25796,16 +25826,16 @@
         </is>
       </c>
       <c r="F325" s="1" t="n">
-        <v>5584</v>
+        <v>5311</v>
       </c>
       <c r="G325" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
+          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
         </is>
       </c>
       <c r="H325" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I325" s="1" t="inlineStr">
@@ -25814,7 +25844,7 @@
         </is>
       </c>
       <c r="J325" s="2" t="n">
-        <v>46226.45693457176</v>
+        <v>46226.45548961806</v>
       </c>
       <c r="K325" s="2" t="n">
         <v>46230</v>
@@ -25844,7 +25874,7 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>81376</v>
+        <v>81375</v>
       </c>
       <c r="B326" s="1" t="inlineStr">
         <is>
@@ -25863,20 +25893,20 @@
       </c>
       <c r="E326" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F326" s="1" t="n">
-        <v>2745</v>
+        <v>5584</v>
       </c>
       <c r="G326" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H326" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I326" s="1" t="inlineStr">
@@ -25885,7 +25915,7 @@
         </is>
       </c>
       <c r="J326" s="2" t="n">
-        <v>46226.46478128473</v>
+        <v>46226.45693457176</v>
       </c>
       <c r="K326" s="2" t="n">
         <v>46230</v>
@@ -25897,7 +25927,7 @@
       </c>
       <c r="M326" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N326" s="1" t="n"/>
@@ -25915,7 +25945,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>81377</v>
+        <v>81376</v>
       </c>
       <c r="B327" s="1" t="inlineStr">
         <is>
@@ -25938,11 +25968,11 @@
         </is>
       </c>
       <c r="F327" s="1" t="n">
-        <v>3601</v>
+        <v>2745</v>
       </c>
       <c r="G327" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H327" s="1" t="inlineStr">
@@ -25956,7 +25986,7 @@
         </is>
       </c>
       <c r="J327" s="2" t="n">
-        <v>46226.4658295949</v>
+        <v>46226.46478128473</v>
       </c>
       <c r="K327" s="2" t="n">
         <v>46230</v>
@@ -25986,7 +26016,7 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>81379</v>
+        <v>81377</v>
       </c>
       <c r="B328" s="1" t="inlineStr">
         <is>
@@ -26005,20 +26035,20 @@
       </c>
       <c r="E328" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F328" s="1" t="n">
-        <v>4079</v>
+        <v>3601</v>
       </c>
       <c r="G328" s="1" t="inlineStr">
         <is>
-          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
         </is>
       </c>
       <c r="H328" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I328" s="1" t="inlineStr">
@@ -26027,7 +26057,7 @@
         </is>
       </c>
       <c r="J328" s="2" t="n">
-        <v>46226.47010887731</v>
+        <v>46226.4658295949</v>
       </c>
       <c r="K328" s="2" t="n">
         <v>46230</v>
@@ -26057,7 +26087,7 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>81380</v>
+        <v>81379</v>
       </c>
       <c r="B329" s="1" t="inlineStr">
         <is>
@@ -26080,16 +26110,16 @@
         </is>
       </c>
       <c r="F329" s="1" t="n">
-        <v>4339</v>
+        <v>4079</v>
       </c>
       <c r="G329" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
+          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
         </is>
       </c>
       <c r="H329" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I329" s="1" t="inlineStr">
@@ -26098,7 +26128,7 @@
         </is>
       </c>
       <c r="J329" s="2" t="n">
-        <v>46226.47113148148</v>
+        <v>46226.47010887731</v>
       </c>
       <c r="K329" s="2" t="n">
         <v>46230</v>
@@ -26128,7 +26158,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>81381</v>
+        <v>81380</v>
       </c>
       <c r="B330" s="1" t="inlineStr">
         <is>
@@ -26151,16 +26181,16 @@
         </is>
       </c>
       <c r="F330" s="1" t="n">
-        <v>4625</v>
+        <v>4339</v>
       </c>
       <c r="G330" s="1" t="inlineStr">
         <is>
-          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
         </is>
       </c>
       <c r="H330" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I330" s="1" t="inlineStr">
@@ -26169,7 +26199,7 @@
         </is>
       </c>
       <c r="J330" s="2" t="n">
-        <v>46226.47206631945</v>
+        <v>46226.47113148148</v>
       </c>
       <c r="K330" s="2" t="n">
         <v>46230</v>
@@ -26199,7 +26229,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>81382</v>
+        <v>81381</v>
       </c>
       <c r="B331" s="1" t="inlineStr">
         <is>
@@ -26222,11 +26252,11 @@
         </is>
       </c>
       <c r="F331" s="1" t="n">
-        <v>4842</v>
+        <v>4625</v>
       </c>
       <c r="G331" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 03)</t>
+          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H331" s="1" t="inlineStr">
@@ -26240,7 +26270,7 @@
         </is>
       </c>
       <c r="J331" s="2" t="n">
-        <v>46226.47387114583</v>
+        <v>46226.47206631945</v>
       </c>
       <c r="K331" s="2" t="n">
         <v>46230</v>
@@ -26270,7 +26300,7 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>81385</v>
+        <v>81382</v>
       </c>
       <c r="B332" s="1" t="inlineStr">
         <is>
@@ -26293,16 +26323,16 @@
         </is>
       </c>
       <c r="F332" s="1" t="n">
-        <v>5143</v>
+        <v>4842</v>
       </c>
       <c r="G332" s="1" t="inlineStr">
         <is>
-          <t>OLIMPIA ADMINISTRADORA DE SERVIÇOS LTDA</t>
+          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 03)</t>
         </is>
       </c>
       <c r="H332" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I332" s="1" t="inlineStr">
@@ -26311,14 +26341,14 @@
         </is>
       </c>
       <c r="J332" s="2" t="n">
-        <v>46226.48074552084</v>
+        <v>46226.47387114583</v>
       </c>
       <c r="K332" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L332" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M332" s="1" t="inlineStr">
@@ -26326,90 +26356,90 @@
           <t>Izabely Araujo</t>
         </is>
       </c>
-      <c r="N332" s="2" t="n">
-        <v>46230.64821527778</v>
-      </c>
+      <c r="N332" s="1" t="n"/>
       <c r="O332" s="1" t="n"/>
       <c r="P332" s="1" t="n"/>
       <c r="Q332" s="1" t="inlineStr"/>
-      <c r="R332" s="1" t="inlineStr">
+      <c r="R332" s="1" t="inlineStr"/>
+      <c r="S332" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T332" s="1" t="n"/>
+      <c r="U332" s="1" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="1" t="n">
+        <v>81385</v>
+      </c>
+      <c r="B333" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C333" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D333" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E333" s="1" t="inlineStr">
+        <is>
+          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+        </is>
+      </c>
+      <c r="F333" s="1" t="n">
+        <v>5143</v>
+      </c>
+      <c r="G333" s="1" t="inlineStr">
+        <is>
+          <t>OLIMPIA ADMINISTRADORA DE SERVIÇOS LTDA</t>
+        </is>
+      </c>
+      <c r="H333" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
+      <c r="I333" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="n">
+        <v>46226.48074552084</v>
+      </c>
+      <c r="K333" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="L333" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M333" s="1" t="inlineStr">
+        <is>
+          <t>Izabely Araujo</t>
+        </is>
+      </c>
+      <c r="N333" s="2" t="n">
+        <v>46230.64821527778</v>
+      </c>
+      <c r="O333" s="1" t="n"/>
+      <c r="P333" s="1" t="n"/>
+      <c r="Q333" s="1" t="inlineStr"/>
+      <c r="R333" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Prezados, boa tarde!
 Estamos providenciando o acesso. 
 Atenciosamente, </t>
         </is>
       </c>
-      <c r="S332" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T332" s="1" t="n"/>
-      <c r="U332" s="1" t="inlineStr"/>
-    </row>
-    <row r="333">
-      <c r="A333" s="1" t="n">
-        <v>81387</v>
-      </c>
-      <c r="B333" s="1" t="inlineStr">
-        <is>
-          <t>Senha</t>
-        </is>
-      </c>
-      <c r="C333" s="1" t="inlineStr">
-        <is>
-          <t>Prefeitura</t>
-        </is>
-      </c>
-      <c r="D333" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="E333" s="1" t="inlineStr">
-        <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
-        </is>
-      </c>
-      <c r="F333" s="1" t="n">
-        <v>5508</v>
-      </c>
-      <c r="G333" s="1" t="inlineStr">
-        <is>
-          <t>ALEXANDRA LIBRAZI GIUNGI BARRETO</t>
-        </is>
-      </c>
-      <c r="H333" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
-      <c r="I333" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J333" s="2" t="n">
-        <v>46226.4871065162</v>
-      </c>
-      <c r="K333" s="2" t="n">
-        <v>46230</v>
-      </c>
-      <c r="L333" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M333" s="1" t="inlineStr">
-        <is>
-          <t>Izabely Araujo</t>
-        </is>
-      </c>
-      <c r="N333" s="1" t="n"/>
-      <c r="O333" s="1" t="n"/>
-      <c r="P333" s="1" t="n"/>
-      <c r="Q333" s="1" t="inlineStr"/>
-      <c r="R333" s="1" t="inlineStr"/>
       <c r="S333" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -26420,7 +26450,7 @@
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
-        <v>81388</v>
+        <v>81387</v>
       </c>
       <c r="B334" s="1" t="inlineStr">
         <is>
@@ -26443,11 +26473,11 @@
         </is>
       </c>
       <c r="F334" s="1" t="n">
-        <v>5654</v>
+        <v>5508</v>
       </c>
       <c r="G334" s="1" t="inlineStr">
         <is>
-          <t>DUARTE E SILVA LTDA</t>
+          <t>ALEXANDRA LIBRAZI GIUNGI BARRETO</t>
         </is>
       </c>
       <c r="H334" s="1" t="inlineStr">
@@ -26461,7 +26491,7 @@
         </is>
       </c>
       <c r="J334" s="2" t="n">
-        <v>46226.4878119213</v>
+        <v>46226.4871065162</v>
       </c>
       <c r="K334" s="2" t="n">
         <v>46230</v>
@@ -26491,7 +26521,7 @@
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
-        <v>81390</v>
+        <v>81388</v>
       </c>
       <c r="B335" s="1" t="inlineStr">
         <is>
@@ -26514,16 +26544,16 @@
         </is>
       </c>
       <c r="F335" s="1" t="n">
-        <v>5876</v>
+        <v>5654</v>
       </c>
       <c r="G335" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 82)</t>
+          <t>DUARTE E SILVA LTDA</t>
         </is>
       </c>
       <c r="H335" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I335" s="1" t="inlineStr">
@@ -26532,7 +26562,7 @@
         </is>
       </c>
       <c r="J335" s="2" t="n">
-        <v>46226.48955505787</v>
+        <v>46226.4878119213</v>
       </c>
       <c r="K335" s="2" t="n">
         <v>46230</v>
@@ -26562,7 +26592,7 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>81391</v>
+        <v>81390</v>
       </c>
       <c r="B336" s="1" t="inlineStr">
         <is>
@@ -26585,11 +26615,11 @@
         </is>
       </c>
       <c r="F336" s="1" t="n">
-        <v>5877</v>
+        <v>5876</v>
       </c>
       <c r="G336" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 83)</t>
+          <t>Cucinare Pro Alimentacao (Filial 82)</t>
         </is>
       </c>
       <c r="H336" s="1" t="inlineStr">
@@ -26603,7 +26633,7 @@
         </is>
       </c>
       <c r="J336" s="2" t="n">
-        <v>46226.4918327199</v>
+        <v>46226.48955505787</v>
       </c>
       <c r="K336" s="2" t="n">
         <v>46230</v>
@@ -26633,7 +26663,7 @@
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
-        <v>81393</v>
+        <v>81391</v>
       </c>
       <c r="B337" s="1" t="inlineStr">
         <is>
@@ -26656,11 +26686,11 @@
         </is>
       </c>
       <c r="F337" s="1" t="n">
-        <v>5878</v>
+        <v>5877</v>
       </c>
       <c r="G337" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentacao (Filial 84)</t>
+          <t>Cucinare Pro Alimentacao (Filial 83)</t>
         </is>
       </c>
       <c r="H337" s="1" t="inlineStr">
@@ -26674,7 +26704,7 @@
         </is>
       </c>
       <c r="J337" s="2" t="n">
-        <v>46226.49427164352</v>
+        <v>46226.4918327199</v>
       </c>
       <c r="K337" s="2" t="n">
         <v>46230</v>
@@ -26704,7 +26734,7 @@
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
-        <v>81394</v>
+        <v>81393</v>
       </c>
       <c r="B338" s="1" t="inlineStr">
         <is>
@@ -26727,16 +26757,16 @@
         </is>
       </c>
       <c r="F338" s="1" t="n">
-        <v>5038</v>
+        <v>5878</v>
       </c>
       <c r="G338" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRAL DISTRIBUIDORA DE GESSO LTDA (FILIAL 01) </t>
+          <t>Cucinare Pro Alimentacao (Filial 84)</t>
         </is>
       </c>
       <c r="H338" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I338" s="1" t="inlineStr">
@@ -26745,7 +26775,7 @@
         </is>
       </c>
       <c r="J338" s="2" t="n">
-        <v>46226.49645659722</v>
+        <v>46226.49427164352</v>
       </c>
       <c r="K338" s="2" t="n">
         <v>46230</v>

</xml_diff>

<commit_message>
data: atualização base chamados 28-07-26 1406
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -2812,7 +2812,7 @@
       <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="2" t="n">
-        <v>46225.6206803588</v>
+        <v>46231.5843647338</v>
       </c>
       <c r="Q29" s="1" t="inlineStr">
         <is>
@@ -21378,70 +21378,59 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>77913</v>
+        <v>81526</v>
       </c>
       <c r="B264" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>MG Controle</t>
         </is>
       </c>
       <c r="C264" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Reabertura de tarefa</t>
         </is>
       </c>
       <c r="D264" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E264" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
+          <t xml:space="preserve">Boa tarde!Solicito a reabertura das tarefas referente a competencia 07/2026, da empresa 3219 IRMÃOS DALBEN LTDA. Devido alteração no quadro societário da empresa na competência em questão, serão alterados os valores na folha de pagamento e nos encargos previdenciários.Fico aguardando vosso retorno. Obrigado.  </t>
         </is>
       </c>
       <c r="F264" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G264" s="1" t="n"/>
-      <c r="H264" s="1" t="inlineStr">
-        <is>
-          <t>Bianca Ribeiro</t>
-        </is>
-      </c>
+      <c r="H264" s="1" t="n"/>
       <c r="I264" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J264" s="2" t="n">
-        <v>46092.7773144676</v>
+        <v>46231.5568997338</v>
       </c>
       <c r="K264" s="2" t="n">
-        <v>46097</v>
+        <v>46232</v>
       </c>
       <c r="L264" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M264" s="1" t="inlineStr">
         <is>
-          <t>Larissa Félix</t>
-        </is>
-      </c>
-      <c r="N264" s="2" t="n">
-        <v>46223.70421145833</v>
-      </c>
+          <t>Vitor Guedes</t>
+        </is>
+      </c>
+      <c r="N264" s="1" t="n"/>
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
       <c r="Q264" s="1" t="inlineStr"/>
-      <c r="R264" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prezados(as), boa tarde!
-Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
-        </is>
-      </c>
+      <c r="R264" s="1" t="n"/>
       <c r="S264" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21452,39 +21441,35 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>79793</v>
+        <v>77913</v>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C265" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D265" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E265" s="1" t="inlineStr">
         <is>
-          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
+          <t>Boa tarde, Por gentileza, preciso que inclua login e senha para o acesso a prefeitura da loja 6353 - ARMANDO E MARGARIDA RESTAURANTE E LANCHONETE LTDA (FILIAL 1).Aguardo um retorno,Obrigada!</t>
         </is>
       </c>
       <c r="F265" s="1" t="n">
-        <v>5655</v>
-      </c>
-      <c r="G265" s="1" t="inlineStr">
-        <is>
-          <t>VANESSA DUARTE RODRIGUES</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G265" s="1" t="n"/>
       <c r="H265" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I265" s="1" t="inlineStr">
@@ -21493,26 +21478,33 @@
         </is>
       </c>
       <c r="J265" s="2" t="n">
-        <v>46182.60128996528</v>
+        <v>46092.7773144676</v>
       </c>
       <c r="K265" s="2" t="n">
-        <v>46185</v>
+        <v>46097</v>
       </c>
       <c r="L265" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M265" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="N265" s="1" t="n"/>
+          <t>Larissa Félix</t>
+        </is>
+      </c>
+      <c r="N265" s="2" t="n">
+        <v>46223.70421145833</v>
+      </c>
       <c r="O265" s="1" t="n"/>
       <c r="P265" s="1" t="n"/>
       <c r="Q265" s="1" t="inlineStr"/>
-      <c r="R265" s="1" t="inlineStr"/>
+      <c r="R265" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Estamos verificando com a Prefeitura, tendo em vista que não recebemos os documentos por parte do cliente. </t>
+        </is>
+      </c>
       <c r="S265" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21523,34 +21515,34 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>79833</v>
+        <v>79793</v>
       </c>
       <c r="B266" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C266" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D266" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E266" s="1" t="inlineStr">
         <is>
-          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
+          <t>caros, boa tarde.cliente solicita:Certidão de inteiro TEOR junta comercial BA, e a CND Federal.apenas da empresa 5655 - Vanessa Duarte.</t>
         </is>
       </c>
       <c r="F266" s="1" t="n">
-        <v>6125</v>
+        <v>5655</v>
       </c>
       <c r="G266" s="1" t="inlineStr">
         <is>
-          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
+          <t>VANESSA DUARTE RODRIGUES</t>
         </is>
       </c>
       <c r="H266" s="1" t="inlineStr">
@@ -21560,36 +21552,30 @@
       </c>
       <c r="I266" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>46183.45917465278</v>
+        <v>46182.60128996528</v>
       </c>
       <c r="K266" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L266" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M266" s="1" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
-        </is>
-      </c>
-      <c r="N266" s="2" t="n">
-        <v>46219.71277496528</v>
-      </c>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N266" s="1" t="n"/>
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
       <c r="Q266" s="1" t="inlineStr"/>
-      <c r="R266" s="1" t="inlineStr">
-        <is>
-          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
-        </is>
-      </c>
+      <c r="R266" s="1" t="inlineStr"/>
       <c r="S266" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21600,7 +21586,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>79834</v>
+        <v>79833</v>
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
@@ -21623,11 +21609,11 @@
         </is>
       </c>
       <c r="F267" s="1" t="n">
-        <v>6162</v>
+        <v>6125</v>
       </c>
       <c r="G267" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
+          <t>CORA SERVIÇOS EMPRESARIAIS LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H267" s="1" t="inlineStr">
@@ -21641,14 +21627,14 @@
         </is>
       </c>
       <c r="J267" s="2" t="n">
-        <v>46183.45954846065</v>
+        <v>46183.45917465278</v>
       </c>
       <c r="K267" s="2" t="n">
         <v>46184</v>
       </c>
       <c r="L267" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M267" s="1" t="inlineStr">
@@ -21656,11 +21642,17 @@
           <t>Tatiana Linardi</t>
         </is>
       </c>
-      <c r="N267" s="1" t="n"/>
+      <c r="N267" s="2" t="n">
+        <v>46219.71277496528</v>
+      </c>
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
       <c r="Q267" s="1" t="inlineStr"/>
-      <c r="R267" s="1" t="inlineStr"/>
+      <c r="R267" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos o antigo contador, porem nao tivemos retorno</t>
+        </is>
+      </c>
       <c r="S267" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -21671,7 +21663,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>79835</v>
+        <v>79834</v>
       </c>
       <c r="B268" s="1" t="inlineStr">
         <is>
@@ -21694,11 +21686,11 @@
         </is>
       </c>
       <c r="F268" s="1" t="n">
-        <v>6485</v>
+        <v>6162</v>
       </c>
       <c r="G268" s="1" t="inlineStr">
         <is>
-          <t>SMA AGRONEGOCIOS LTDA</t>
+          <t xml:space="preserve">RENOVACAO EMPREENDIMENTOS HOTELEIROS LTDA </t>
         </is>
       </c>
       <c r="H268" s="1" t="inlineStr">
@@ -21712,7 +21704,7 @@
         </is>
       </c>
       <c r="J268" s="2" t="n">
-        <v>46183.45993642361</v>
+        <v>46183.45954846065</v>
       </c>
       <c r="K268" s="2" t="n">
         <v>46184</v>
@@ -21742,16 +21734,16 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>79854</v>
+        <v>79835</v>
       </c>
       <c r="B269" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C269" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D269" s="1" t="inlineStr">
@@ -21761,15 +21753,15 @@
       </c>
       <c r="E269" s="1" t="inlineStr">
         <is>
-          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
+          <t>Favor solicitar o balancete de implantação para a entrega do Sped 2025</t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
-        <v>6302</v>
+        <v>6485</v>
       </c>
       <c r="G269" s="1" t="inlineStr">
         <is>
-          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
+          <t>SMA AGRONEGOCIOS LTDA</t>
         </is>
       </c>
       <c r="H269" s="1" t="inlineStr">
@@ -21783,7 +21775,7 @@
         </is>
       </c>
       <c r="J269" s="2" t="n">
-        <v>46183.60582329861</v>
+        <v>46183.45993642361</v>
       </c>
       <c r="K269" s="2" t="n">
         <v>46184</v>
@@ -21813,7 +21805,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>79855</v>
+        <v>79854</v>
       </c>
       <c r="B270" s="1" t="inlineStr">
         <is>
@@ -21832,15 +21824,15 @@
       </c>
       <c r="E270" s="1" t="inlineStr">
         <is>
-          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>6302 - Coocerqui - Para enviar o Sped 2025 precisamos do Sped do periodo do ex contador ( Adriano ).</t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
-        <v>4765</v>
+        <v>6302</v>
       </c>
       <c r="G270" s="1" t="inlineStr">
         <is>
-          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
+          <t>COOPERATIVA DE CONSUMO POPULAR DE CERQUILHO (MATRIZ)</t>
         </is>
       </c>
       <c r="H270" s="1" t="inlineStr">
@@ -21854,10 +21846,10 @@
         </is>
       </c>
       <c r="J270" s="2" t="n">
-        <v>46183.60712457176</v>
+        <v>46183.60582329861</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L270" s="1" t="inlineStr">
         <is>
@@ -21884,7 +21876,7 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>79856</v>
+        <v>79855</v>
       </c>
       <c r="B271" s="1" t="inlineStr">
         <is>
@@ -21903,15 +21895,15 @@
       </c>
       <c r="E271" s="1" t="inlineStr">
         <is>
-          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
+          <t>Brasileirão - verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
-        <v>4225</v>
+        <v>4765</v>
       </c>
       <c r="G271" s="1" t="inlineStr">
         <is>
-          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
+          <t>BRASILEIRÃO ATACADO COMÉRCIO DE PRODUTOS ALIMENTICIOS SOCIEDADE ANÔNIMA</t>
         </is>
       </c>
       <c r="H271" s="1" t="inlineStr">
@@ -21925,10 +21917,10 @@
         </is>
       </c>
       <c r="J271" s="2" t="n">
-        <v>46183.60759024305</v>
+        <v>46183.60712457176</v>
       </c>
       <c r="K271" s="2" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="L271" s="1" t="inlineStr">
         <is>
@@ -21955,7 +21947,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>79859</v>
+        <v>79856</v>
       </c>
       <c r="B272" s="1" t="inlineStr">
         <is>
@@ -21974,15 +21966,15 @@
       </c>
       <c r="E272" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>verificar se o atual contador vai enviar o periodo inteiro de 2025, pois só temos 2 meses com a Mg.</t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
-        <v>6570</v>
+        <v>4225</v>
       </c>
       <c r="G272" s="1" t="inlineStr">
         <is>
-          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
+          <t>ORGANIZAÇÕES FARINHA PURA LTDA</t>
         </is>
       </c>
       <c r="H272" s="1" t="inlineStr">
@@ -21996,10 +21988,10 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>46183.61569366898</v>
+        <v>46183.60759024305</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="L272" s="1" t="inlineStr">
         <is>
@@ -22008,7 +22000,7 @@
       </c>
       <c r="M272" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Tatiana Linardi</t>
         </is>
       </c>
       <c r="N272" s="1" t="n"/>
@@ -22026,7 +22018,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>79860</v>
+        <v>79859</v>
       </c>
       <c r="B273" s="1" t="inlineStr">
         <is>
@@ -22045,15 +22037,15 @@
       </c>
       <c r="E273" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6570.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
-        <v>6581</v>
+        <v>6570</v>
       </c>
       <c r="G273" s="1" t="inlineStr">
         <is>
-          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
+          <t>DROGARIA MIX I LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H273" s="1" t="inlineStr">
@@ -22067,7 +22059,7 @@
         </is>
       </c>
       <c r="J273" s="2" t="n">
-        <v>46183.61707056713</v>
+        <v>46183.61569366898</v>
       </c>
       <c r="K273" s="2" t="n">
         <v>46185</v>
@@ -22097,7 +22089,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>79861</v>
+        <v>79860</v>
       </c>
       <c r="B274" s="1" t="inlineStr">
         <is>
@@ -22116,15 +22108,15 @@
       </c>
       <c r="E274" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6581.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>6583</v>
+        <v>6581</v>
       </c>
       <c r="G274" s="1" t="inlineStr">
         <is>
-          <t>DROGA MX LTDA (MATRIZ)</t>
+          <t>PARIS STORE PERFUMARIA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H274" s="1" t="inlineStr">
@@ -22138,7 +22130,7 @@
         </is>
       </c>
       <c r="J274" s="2" t="n">
-        <v>46183.61758677083</v>
+        <v>46183.61707056713</v>
       </c>
       <c r="K274" s="2" t="n">
         <v>46185</v>
@@ -22168,7 +22160,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>79863</v>
+        <v>79861</v>
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
@@ -22187,15 +22179,15 @@
       </c>
       <c r="E275" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/09/2025, da empresa 6583.A primeira solicitação foi feita por e-mail em 18/05.</t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
-        <v>6404</v>
+        <v>6583</v>
       </c>
       <c r="G275" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>DROGA MX LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H275" s="1" t="inlineStr">
@@ -22209,7 +22201,7 @@
         </is>
       </c>
       <c r="J275" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.61758677083</v>
       </c>
       <c r="K275" s="2" t="n">
         <v>46185</v>
@@ -22239,7 +22231,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>79865</v>
+        <v>79863</v>
       </c>
       <c r="B276" s="1" t="inlineStr">
         <is>
@@ -22258,15 +22250,15 @@
       </c>
       <c r="E276" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
-        <v>6278</v>
+        <v>6404</v>
       </c>
       <c r="G276" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H276" s="1" t="inlineStr">
@@ -22280,7 +22272,7 @@
         </is>
       </c>
       <c r="J276" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K276" s="2" t="n">
         <v>46185</v>
@@ -22310,7 +22302,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>79866</v>
+        <v>79865</v>
       </c>
       <c r="B277" s="1" t="inlineStr">
         <is>
@@ -22329,15 +22321,15 @@
       </c>
       <c r="E277" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
-        <v>6539</v>
+        <v>6278</v>
       </c>
       <c r="G277" s="1" t="inlineStr">
         <is>
-          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="H277" s="1" t="inlineStr">
@@ -22351,7 +22343,7 @@
         </is>
       </c>
       <c r="J277" s="2" t="n">
-        <v>46183.62343017361</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K277" s="2" t="n">
         <v>46185</v>
@@ -22381,16 +22373,16 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>79867</v>
+        <v>79866</v>
       </c>
       <c r="B278" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C278" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D278" s="1" t="inlineStr">
@@ -22400,15 +22392,15 @@
       </c>
       <c r="E278" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/10/2025, da empresa 6539.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
-        <v>6704</v>
+        <v>6539</v>
       </c>
       <c r="G278" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>TECHFEED ADITIVOS PARA NUTRICAO ANIMAL LTDA</t>
         </is>
       </c>
       <c r="H278" s="1" t="inlineStr">
@@ -22422,7 +22414,7 @@
         </is>
       </c>
       <c r="J278" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46183.62343017361</v>
       </c>
       <c r="K278" s="2" t="n">
         <v>46185</v>
@@ -22452,69 +22444,67 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>80515</v>
+        <v>79867</v>
       </c>
       <c r="B279" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C279" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D279" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E279" s="1" t="inlineStr">
         <is>
-          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G279" s="1" t="n"/>
+        <v>6704</v>
+      </c>
+      <c r="G279" s="1" t="inlineStr">
+        <is>
+          <t>TECNO COM INFORMATICA LTDA</t>
+        </is>
+      </c>
       <c r="H279" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I279" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J279" s="2" t="n">
-        <v>46196.7259258449</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K279" s="2" t="n">
-        <v>46226</v>
+        <v>46185</v>
       </c>
       <c r="L279" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M279" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N279" s="2" t="n">
-        <v>46219.75157017361</v>
-      </c>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N279" s="1" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="Q279" s="1" t="inlineStr"/>
-      <c r="R279" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enviado para registro </t>
-        </is>
-      </c>
+      <c r="R279" s="1" t="inlineStr"/>
       <c r="S279" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -22525,7 +22515,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>80697</v>
+        <v>80515</v>
       </c>
       <c r="B280" s="1" t="inlineStr">
         <is>
@@ -22534,7 +22524,7 @@
       </c>
       <c r="C280" s="1" t="inlineStr">
         <is>
-          <t>Eireli - Serviços</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D280" s="1" t="inlineStr">
@@ -22544,7 +22534,7 @@
       </c>
       <c r="E280" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
+          <t>Pedido de abertura de empresa prestadora de serviços que será um novo cliente, sem vínculo com qualquer um outro cliente MG Contécnica.No pedido de abertura contém:_ 3 sujestões de nome;_ CNAE´s já pré definidos;_ Objeto social (Considerar empresa já cliente DUO Cenografia como exemplo)_ Capital social já definido;_ e-mail da sócia para envio da minuta para conferência;_ Telefone e e-mail do Sr. Felipe Silveira, responsável pelas documentações;</t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
@@ -22562,10 +22552,10 @@
         </is>
       </c>
       <c r="J280" s="2" t="n">
-        <v>46205.39919077546</v>
+        <v>46196.7259258449</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>46237</v>
+        <v>46226</v>
       </c>
       <c r="L280" s="1" t="inlineStr">
         <is>
@@ -22578,14 +22568,14 @@
         </is>
       </c>
       <c r="N280" s="2" t="n">
-        <v>46224.68237751158</v>
+        <v>46219.75157017361</v>
       </c>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="Q280" s="1" t="inlineStr"/>
       <c r="R280" s="1" t="inlineStr">
         <is>
-          <t>Em atendimento</t>
+          <t xml:space="preserve">Enviado para registro </t>
         </is>
       </c>
       <c r="S280" s="1" t="inlineStr">
@@ -22598,7 +22588,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>80714</v>
+        <v>80697</v>
       </c>
       <c r="B281" s="1" t="inlineStr">
         <is>
@@ -22607,7 +22597,7 @@
       </c>
       <c r="C281" s="1" t="inlineStr">
         <is>
-          <t>Sociedade - Serviços</t>
+          <t>Eireli - Serviços</t>
         </is>
       </c>
       <c r="D281" s="1" t="inlineStr">
@@ -22617,7 +22607,7 @@
       </c>
       <c r="E281" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
+          <t>ABERTURA DE NOVA EMPRESA DO GRUPO 1803 - SERVISUL, EMPRESA COM  TRIBUTAÇÃO SIMPLES NACIONAL, TIPO DE ATIVIDADE: SERVIÇOS, FINALIDADE: OPERACIONAL E FORMA JURIDICA: LTDA. PROPOSTA NEGOCIADA COM O VALOR DE R$1.800,00. RAZÃO SOCIAL: MCESCON ASSESSORIA EMPRESARIAL LTDA. OBJETO SOCIAL: APOIO ADMINISTRATIVO/COBRANÇA. CAPITAL SOCIAL:10.000,00. DOCUMENTAÇÃO DISPONIBILIZADA: RG / CPF / CNH, IPTU E COMPROVANTE DE ENDEREÇO.</t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
@@ -22626,7 +22616,7 @@
       <c r="G281" s="1" t="n"/>
       <c r="H281" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I281" s="1" t="inlineStr">
@@ -22635,10 +22625,10 @@
         </is>
       </c>
       <c r="J281" s="2" t="n">
-        <v>46206.37795378472</v>
+        <v>46205.39919077546</v>
       </c>
       <c r="K281" s="2" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="L281" s="1" t="inlineStr">
         <is>
@@ -22651,15 +22641,14 @@
         </is>
       </c>
       <c r="N281" s="2" t="n">
-        <v>46223.41822326389</v>
+        <v>46224.68237751158</v>
       </c>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="Q281" s="1" t="inlineStr"/>
       <c r="R281" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
+          <t>Em atendimento</t>
         </is>
       </c>
       <c r="S281" s="1" t="inlineStr">
@@ -22672,16 +22661,16 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>80919</v>
+        <v>80714</v>
       </c>
       <c r="B282" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C282" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Sociedade - Serviços</t>
         </is>
       </c>
       <c r="D282" s="1" t="inlineStr">
@@ -22691,7 +22680,7 @@
       </c>
       <c r="E282" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
+          <t>ABERTURA DE FILIAL - RIO DE JANEIRO</t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
@@ -22709,10 +22698,10 @@
         </is>
       </c>
       <c r="J282" s="2" t="n">
-        <v>46211.63019085648</v>
+        <v>46206.37795378472</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="L282" s="1" t="inlineStr">
         <is>
@@ -22725,16 +22714,15 @@
         </is>
       </c>
       <c r="N282" s="2" t="n">
-        <v>46225.48500983796</v>
+        <v>46223.41822326389</v>
       </c>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="Q282" s="1" t="inlineStr"/>
       <c r="R282" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prezadas(os), bom dia!
-Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
-Atenciosamente, </t>
+          <t xml:space="preserve">PROCESSO ENCONTRA-SE EM ANDAMENTO. 
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL. </t>
         </is>
       </c>
       <c r="S282" s="1" t="inlineStr">
@@ -22747,16 +22735,16 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>80935</v>
+        <v>80919</v>
       </c>
       <c r="B283" s="1" t="inlineStr">
         <is>
-          <t>Abertura de Empresa</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C283" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Razão Social</t>
         </is>
       </c>
       <c r="D283" s="1" t="inlineStr">
@@ -22766,7 +22754,7 @@
       </c>
       <c r="E283" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
+          <t xml:space="preserve">ALTERAÇÃO CONTRATUAL DA RAZÃO SOCIAL, ATIVIDADE E ENDEREÇO DO CLIENTE 6651 - POLEN COMERCIO DE EMBALAGENS. PROPOSTA JÁ NEGOCIADA. </t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
@@ -22784,10 +22772,10 @@
         </is>
       </c>
       <c r="J283" s="2" t="n">
-        <v>46213.35976299769</v>
+        <v>46211.63019085648</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>46241</v>
+        <v>46239</v>
       </c>
       <c r="L283" s="1" t="inlineStr">
         <is>
@@ -22800,15 +22788,16 @@
         </is>
       </c>
       <c r="N283" s="2" t="n">
-        <v>46223.41869637732</v>
+        <v>46225.48500983796</v>
       </c>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="Q283" s="1" t="inlineStr"/>
       <c r="R283" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
-TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
+          <t xml:space="preserve">Prezadas(os), bom dia!
+Para ciência, informamos que essa alteração contratual já encontra-se em andamento. 
+Atenciosamente, </t>
         </is>
       </c>
       <c r="S283" s="1" t="inlineStr">
@@ -22821,7 +22810,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>80936</v>
+        <v>80935</v>
       </c>
       <c r="B284" s="1" t="inlineStr">
         <is>
@@ -22830,7 +22819,7 @@
       </c>
       <c r="C284" s="1" t="inlineStr">
         <is>
-          <t>Individual - Serviços</t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D284" s="1" t="inlineStr">
@@ -22840,7 +22829,7 @@
       </c>
       <c r="E284" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 2681 - PARANÁ GUARULHOSTRIBUTAÇÃO: LUCRO PRESUMIDOTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: H FARIAS NEGÓCIOS LTDA</t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
@@ -22849,7 +22838,7 @@
       <c r="G284" s="1" t="n"/>
       <c r="H284" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I284" s="1" t="inlineStr">
@@ -22858,7 +22847,7 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>46213.36620841435</v>
+        <v>46213.35976299769</v>
       </c>
       <c r="K284" s="2" t="n">
         <v>46241</v>
@@ -22874,14 +22863,15 @@
         </is>
       </c>
       <c r="N284" s="2" t="n">
-        <v>46220.45547311343</v>
+        <v>46223.41869637732</v>
       </c>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="Q284" s="1" t="inlineStr"/>
       <c r="R284" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviado ao cliente</t>
+          <t>PROCESSO ENCONTRA-SE EM ANDAMENTO.
+TRATATIVA REALIZADA COM O CLIENTE VIA E-MAIL.</t>
         </is>
       </c>
       <c r="S284" s="1" t="inlineStr">
@@ -22894,7 +22884,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>80951</v>
+        <v>80936</v>
       </c>
       <c r="B285" s="1" t="inlineStr">
         <is>
@@ -22903,7 +22893,7 @@
       </c>
       <c r="C285" s="1" t="inlineStr">
         <is>
-          <t>Individual - Comércio</t>
+          <t>Individual - Serviços</t>
         </is>
       </c>
       <c r="D285" s="1" t="inlineStr">
@@ -22913,7 +22903,7 @@
       </c>
       <c r="E285" s="1" t="inlineStr">
         <is>
-          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 5442 - EQUIPOOLSTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.100,00RAZÃO SOCIAL: VANLOG SERVICOS DE EMBALAGEM E GALPAO LOGISTICO LTDA</t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
@@ -22931,7 +22921,7 @@
         </is>
       </c>
       <c r="J285" s="2" t="n">
-        <v>46213.66707554398</v>
+        <v>46213.36620841435</v>
       </c>
       <c r="K285" s="2" t="n">
         <v>46241</v>
@@ -22947,14 +22937,14 @@
         </is>
       </c>
       <c r="N285" s="2" t="n">
-        <v>46219.74920023148</v>
+        <v>46220.45547311343</v>
       </c>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="Q285" s="1" t="inlineStr"/>
       <c r="R285" s="1" t="inlineStr">
         <is>
-          <t>Minuta enviada ao cliente</t>
+          <t>Minuta enviado ao cliente</t>
         </is>
       </c>
       <c r="S285" s="1" t="inlineStr">
@@ -22967,39 +22957,35 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>81004</v>
+        <v>80951</v>
       </c>
       <c r="B286" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Abertura de Empresa</t>
         </is>
       </c>
       <c r="C286" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Individual - Comércio</t>
         </is>
       </c>
       <c r="D286" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E286" s="1" t="inlineStr">
         <is>
-          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
+          <t>ABERTURA DE EMPRESA DO GRUPO: 3697 - BOSTON.TRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIOFINALIDADE: OPERACIONALFORMA JURIDICA: LTDARAZÃO SOCIAL: NOVA BOSTON GRILL RESTAURANTE LTDA</t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>6869</v>
-      </c>
-      <c r="G286" s="1" t="inlineStr">
-        <is>
-          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G286" s="1" t="n"/>
       <c r="H286" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I286" s="1" t="inlineStr">
@@ -23008,26 +22994,32 @@
         </is>
       </c>
       <c r="J286" s="2" t="n">
-        <v>46217.37983028935</v>
+        <v>46213.66707554398</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>46218</v>
+        <v>46241</v>
       </c>
       <c r="L286" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M286" s="1" t="inlineStr">
         <is>
-          <t>Lorrane Santos</t>
-        </is>
-      </c>
-      <c r="N286" s="1" t="n"/>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N286" s="2" t="n">
+        <v>46219.74920023148</v>
+      </c>
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
       <c r="Q286" s="1" t="inlineStr"/>
-      <c r="R286" s="1" t="inlineStr"/>
+      <c r="R286" s="1" t="inlineStr">
+        <is>
+          <t>Minuta enviada ao cliente</t>
+        </is>
+      </c>
       <c r="S286" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23038,7 +23030,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>81005</v>
+        <v>81004</v>
       </c>
       <c r="B287" s="1" t="inlineStr">
         <is>
@@ -23061,16 +23053,16 @@
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>6870</v>
+        <v>6869</v>
       </c>
       <c r="G287" s="1" t="inlineStr">
         <is>
-          <t>AC HOME PET RAÇÕES LTDA</t>
+          <t>PET HOME EXPRESS COMERCIO DE RACOES LTDA</t>
         </is>
       </c>
       <c r="H287" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I287" s="1" t="inlineStr">
@@ -23079,7 +23071,7 @@
         </is>
       </c>
       <c r="J287" s="2" t="n">
-        <v>46217.38025162037</v>
+        <v>46217.37983028935</v>
       </c>
       <c r="K287" s="2" t="n">
         <v>46218</v>
@@ -23109,68 +23101,67 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>81019</v>
+        <v>81005</v>
       </c>
       <c r="B288" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C288" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D288" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E288" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
+          <t>Bom dia! Referente AS LOJAS 6869 e 6870 do grupo PET HOME – ao fazer a entrega da SEDIF mostra que o CPF do responsável esta invalido, porem esta conforme o MG CONTROLE, pode nos ajudar com esse caso?</t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G288" s="1" t="n"/>
+        <v>6870</v>
+      </c>
+      <c r="G288" s="1" t="inlineStr">
+        <is>
+          <t>AC HOME PET RAÇÕES LTDA</t>
+        </is>
+      </c>
       <c r="H288" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I288" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J288" s="2" t="n">
-        <v>46217.43210269676</v>
+        <v>46217.38025162037</v>
       </c>
       <c r="K288" s="2" t="n">
         <v>46218</v>
       </c>
       <c r="L288" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M288" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Lorrane Santos</t>
         </is>
       </c>
       <c r="N288" s="1" t="n"/>
       <c r="O288" s="1" t="n"/>
       <c r="P288" s="1" t="n"/>
       <c r="Q288" s="1" t="inlineStr"/>
-      <c r="R288" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia 
-Segue recibos conforme solictiado </t>
-        </is>
-      </c>
+      <c r="R288" s="1" t="inlineStr"/>
       <c r="S288" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23181,7 +23172,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>81052</v>
+        <v>81019</v>
       </c>
       <c r="B289" s="1" t="inlineStr">
         <is>
@@ -23200,7 +23191,7 @@
       </c>
       <c r="E289" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t xml:space="preserve">Por gentileza, solicitar que enviem as folhas de pagamento SEM RATEIO. </t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
@@ -23218,10 +23209,10 @@
         </is>
       </c>
       <c r="J289" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46217.43210269676</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="L289" s="1" t="inlineStr">
         <is>
@@ -23230,7 +23221,7 @@
       </c>
       <c r="M289" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N289" s="1" t="n"/>
@@ -23239,7 +23230,8 @@
       <c r="Q289" s="1" t="inlineStr"/>
       <c r="R289" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t xml:space="preserve">Bom dia 
+Segue recibos conforme solictiado </t>
         </is>
       </c>
       <c r="S289" s="1" t="inlineStr">
@@ -23252,7 +23244,7 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>81055</v>
+        <v>81052</v>
       </c>
       <c r="B290" s="1" t="inlineStr">
         <is>
@@ -23271,7 +23263,7 @@
       </c>
       <c r="E290" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
@@ -23289,14 +23281,14 @@
         </is>
       </c>
       <c r="J290" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K290" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="L290" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M290" s="1" t="inlineStr">
@@ -23304,15 +23296,13 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N290" s="2" t="n">
-        <v>46219.50607847222</v>
-      </c>
+      <c r="N290" s="1" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="Q290" s="1" t="inlineStr"/>
       <c r="R290" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S290" s="1" t="inlineStr">
@@ -23325,36 +23315,32 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>81091</v>
+        <v>81055</v>
       </c>
       <c r="B291" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C291" s="1" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D291" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E291" s="1" t="inlineStr">
         <is>
-          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>6907</v>
-      </c>
-      <c r="G291" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G291" s="1" t="n"/>
       <c r="H291" s="1" t="inlineStr">
         <is>
           <t>Edney Xavier</t>
@@ -23362,30 +23348,36 @@
       </c>
       <c r="I291" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>46219.3374690162</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>46223</v>
+        <v>46219</v>
       </c>
       <c r="L291" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M291" s="1" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
-        </is>
-      </c>
-      <c r="N291" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N291" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
       <c r="Q291" s="1" t="inlineStr"/>
-      <c r="R291" s="1" t="inlineStr"/>
+      <c r="R291" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retorno dos dados do contador</t>
+        </is>
+      </c>
       <c r="S291" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23396,16 +23388,16 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>81209</v>
+        <v>81091</v>
       </c>
       <c r="B292" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C292" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Outra</t>
         </is>
       </c>
       <c r="D292" s="1" t="inlineStr">
@@ -23415,20 +23407,20 @@
       </c>
       <c r="E292" s="1" t="inlineStr">
         <is>
-          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
+          <t>Favor providenciar login e senha ou regularizar pois CPF não bate com o cadastrado no SEDIF.</t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>6094</v>
+        <v>6907</v>
       </c>
       <c r="G292" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
+          <t xml:space="preserve">JDM DISTRIBUIDORA DE PRODUTOS ALIMENTÍCIOS LTDA </t>
         </is>
       </c>
       <c r="H292" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I292" s="1" t="inlineStr">
@@ -23437,10 +23429,10 @@
         </is>
       </c>
       <c r="J292" s="2" t="n">
-        <v>46223.52088677084</v>
+        <v>46219.3374690162</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="L292" s="1" t="inlineStr">
         <is>
@@ -23467,16 +23459,16 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>81213</v>
+        <v>81209</v>
       </c>
       <c r="B293" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C293" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D293" s="1" t="inlineStr">
@@ -23486,20 +23478,20 @@
       </c>
       <c r="E293" s="1" t="inlineStr">
         <is>
-          <t>Cliente não possuí acesso cadastrado</t>
+          <t>Cliente cancelou NFS-e posterior a emissão da guia de ISS no mês de junho e emitiu notas fiscais em junho com competência em maio, informado ao GC do ocorrido, o qual solicitou que o cliente cancelasse as notas emitidas na competência errada e que já esta encerrada e emitisse corretamente na competência de junho, contudo esta prefeitura (Itapetininga) não é possível cancelar as guias geradas de forma remota sendo necessário protocolar pessoalmente no balcão do setor de protocolos.</t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>6946</v>
+        <v>6094</v>
       </c>
       <c r="G293" s="1" t="inlineStr">
         <is>
-          <t>FFRA CONCRETOS LTDA</t>
+          <t xml:space="preserve">CLINICA SAUDE &amp; VIDA LTDA </t>
         </is>
       </c>
       <c r="H293" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I293" s="1" t="inlineStr">
@@ -23508,14 +23500,14 @@
         </is>
       </c>
       <c r="J293" s="2" t="n">
-        <v>46223.5798869213</v>
+        <v>46223.52088677084</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="L293" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M293" s="1" t="inlineStr">
@@ -23523,17 +23515,11 @@
           <t>Denis Reis</t>
         </is>
       </c>
-      <c r="N293" s="2" t="n">
-        <v>46230.54938295139</v>
-      </c>
+      <c r="N293" s="1" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="Q293" s="1" t="inlineStr"/>
-      <c r="R293" s="1" t="inlineStr">
-        <is>
-          <t>Verificando os procedimentos para solicitação de cadastro.</t>
-        </is>
-      </c>
+      <c r="R293" s="1" t="inlineStr"/>
       <c r="S293" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23544,44 +23530,48 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>81215</v>
+        <v>81213</v>
       </c>
       <c r="B294" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C294" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D294" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E294" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>Cliente não possuí acesso cadastrado</t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G294" s="1" t="n"/>
+        <v>6946</v>
+      </c>
+      <c r="G294" s="1" t="inlineStr">
+        <is>
+          <t>FFRA CONCRETOS LTDA</t>
+        </is>
+      </c>
       <c r="H294" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I294" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J294" s="2" t="n">
-        <v>46223.60068402778</v>
+        <v>46223.5798869213</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>46225</v>
@@ -23593,18 +23583,18 @@
       </c>
       <c r="M294" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="N294" s="2" t="n">
-        <v>46225.56780570602</v>
+        <v>46230.54938295139</v>
       </c>
       <c r="O294" s="1" t="n"/>
       <c r="P294" s="1" t="n"/>
       <c r="Q294" s="1" t="inlineStr"/>
       <c r="R294" s="1" t="inlineStr">
         <is>
-          <t>Cobramos novamente a contabilidade.</t>
+          <t>Verificando os procedimentos para solicitação de cadastro.</t>
         </is>
       </c>
       <c r="S294" s="1" t="inlineStr">
@@ -23617,7 +23607,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>81217</v>
+        <v>81215</v>
       </c>
       <c r="B295" s="1" t="inlineStr">
         <is>
@@ -23636,7 +23626,7 @@
       </c>
       <c r="E295" s="1" t="inlineStr">
         <is>
-          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t xml:space="preserve">Boa tarde, por gentileza, precisamos dos demais documentos do Checklist em anexo. Itens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
@@ -23654,7 +23644,7 @@
         </is>
       </c>
       <c r="J295" s="2" t="n">
-        <v>46223.60780787037</v>
+        <v>46223.60068402778</v>
       </c>
       <c r="K295" s="2" t="n">
         <v>46225</v>
@@ -23670,14 +23660,14 @@
         </is>
       </c>
       <c r="N295" s="2" t="n">
-        <v>46225.56888491898</v>
+        <v>46225.56780570602</v>
       </c>
       <c r="O295" s="1" t="n"/>
       <c r="P295" s="1" t="n"/>
       <c r="Q295" s="1" t="inlineStr"/>
       <c r="R295" s="1" t="inlineStr">
         <is>
-          <t>Cobramos novamente.</t>
+          <t>Cobramos novamente a contabilidade.</t>
         </is>
       </c>
       <c r="S295" s="1" t="inlineStr">
@@ -23690,7 +23680,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>81218</v>
+        <v>81217</v>
       </c>
       <c r="B296" s="1" t="inlineStr">
         <is>
@@ -23709,7 +23699,7 @@
       </c>
       <c r="E296" s="1" t="inlineStr">
         <is>
-          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>6959 - WISPOT. Boa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
@@ -23727,7 +23717,7 @@
         </is>
       </c>
       <c r="J296" s="2" t="n">
-        <v>46223.6082516551</v>
+        <v>46223.60780787037</v>
       </c>
       <c r="K296" s="2" t="n">
         <v>46225</v>
@@ -23743,7 +23733,7 @@
         </is>
       </c>
       <c r="N296" s="2" t="n">
-        <v>46225.57019641204</v>
+        <v>46225.56888491898</v>
       </c>
       <c r="O296" s="1" t="n"/>
       <c r="P296" s="1" t="n"/>
@@ -23763,26 +23753,26 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>81227</v>
+        <v>81218</v>
       </c>
       <c r="B297" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C297" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D297" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E297" s="1" t="inlineStr">
         <is>
-          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
+          <t>6960 - PRO ADVANCEDBoa tarde, por gentileza, precisamos do documentos do Checklist em anexo.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
@@ -23791,35 +23781,41 @@
       <c r="G297" s="1" t="n"/>
       <c r="H297" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I297" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J297" s="2" t="n">
-        <v>46223.69836307871</v>
+        <v>46223.6082516551</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L297" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M297" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
-        </is>
-      </c>
-      <c r="N297" s="1" t="n"/>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N297" s="2" t="n">
+        <v>46225.57019641204</v>
+      </c>
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
       <c r="Q297" s="1" t="inlineStr"/>
-      <c r="R297" s="1" t="inlineStr"/>
+      <c r="R297" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos novamente.</t>
+        </is>
+      </c>
       <c r="S297" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -23830,26 +23826,26 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>81228</v>
+        <v>81227</v>
       </c>
       <c r="B298" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C298" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>RFB</t>
         </is>
       </c>
       <c r="D298" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E298" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
+          <t>Empresa 5988 - Maurício Toniati - Cliente que haviamos feito a apuração incorreta de pis e cofins - Foi feito parcelamento , mais depois da retificação dos impostos não teria imposto a apagar. Gerei um relatório da situação fiscal e não consta nenhuma informação referente à Malha Fiscal, apenas a indicação de Parcelamento Suspenso.Poderia verificar, por gentileza, se há algum procedimento adicional que precise ser realizado ou alguma outra consulta que devemos efetuar?</t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
@@ -23858,74 +23854,65 @@
       <c r="G298" s="1" t="n"/>
       <c r="H298" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I298" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J298" s="2" t="n">
-        <v>46223.70694884259</v>
+        <v>46223.69836307871</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>46226</v>
+        <v>46224</v>
       </c>
       <c r="L298" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M298" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Ferreira</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N298" s="1" t="n"/>
       <c r="O298" s="1" t="n"/>
       <c r="P298" s="1" t="n"/>
       <c r="Q298" s="1" t="inlineStr"/>
-      <c r="R298" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Estou verificando o acesso  junto a prefeitura.</t>
-        </is>
-      </c>
+      <c r="R298" s="1" t="inlineStr"/>
       <c r="S298" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T298" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
+      <c r="T298" s="1" t="n"/>
       <c r="U298" s="1" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>81244</v>
+        <v>81228</v>
       </c>
       <c r="B299" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C299" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D299" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E299" s="1" t="inlineStr">
         <is>
-          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
+          <t>Boa tarde, Poderiam por gentileza disponibilizar o login e senha da loja 6353.Obrigada!</t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
@@ -23934,39 +23921,38 @@
       <c r="G299" s="1" t="n"/>
       <c r="H299" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I299" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J299" s="2" t="n">
-        <v>46224.42615887732</v>
+        <v>46223.70694884259</v>
       </c>
       <c r="K299" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L299" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Solicitante</t>
         </is>
       </c>
       <c r="M299" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N299" s="2" t="n">
-        <v>46225.4986497338</v>
-      </c>
+          <t>Beatriz Ferreira</t>
+        </is>
+      </c>
+      <c r="N299" s="1" t="n"/>
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
       <c r="Q299" s="1" t="inlineStr"/>
       <c r="R299" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aguardando contato do contador. </t>
+          <t>Boa tarde!
+Estou verificando o acesso  junto a prefeitura.</t>
         </is>
       </c>
       <c r="S299" s="1" t="inlineStr">
@@ -23974,12 +23960,16 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T299" s="1" t="n"/>
+      <c r="T299" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
       <c r="U299" s="1" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>81245</v>
+        <v>81244</v>
       </c>
       <c r="B300" s="1" t="inlineStr">
         <is>
@@ -23998,7 +23988,7 @@
       </c>
       <c r="E300" s="1" t="inlineStr">
         <is>
-          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
+          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
@@ -24016,7 +24006,7 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>46224.42947079861</v>
+        <v>46224.42615887732</v>
       </c>
       <c r="K300" s="2" t="n">
         <v>46226</v>
@@ -24032,14 +24022,14 @@
         </is>
       </c>
       <c r="N300" s="2" t="n">
-        <v>46225.4960193287</v>
+        <v>46225.4986497338</v>
       </c>
       <c r="O300" s="1" t="n"/>
       <c r="P300" s="1" t="n"/>
       <c r="Q300" s="1" t="inlineStr"/>
       <c r="R300" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobramos novamente. </t>
+          <t xml:space="preserve">Aguardando contato do contador. </t>
         </is>
       </c>
       <c r="S300" s="1" t="inlineStr">
@@ -24052,7 +24042,7 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>81247</v>
+        <v>81245</v>
       </c>
       <c r="B301" s="1" t="inlineStr">
         <is>
@@ -24071,7 +24061,7 @@
       </c>
       <c r="E301" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6964 - SUPER DIJAN COMERCIAL LTDAPor gentileza, providenciar as documentações de implantação da empresa, anexo o checklist.</t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
@@ -24089,14 +24079,14 @@
         </is>
       </c>
       <c r="J301" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46224.42947079861</v>
       </c>
       <c r="K301" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L301" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M301" s="1" t="inlineStr">
@@ -24104,13 +24094,15 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N301" s="1" t="n"/>
+      <c r="N301" s="2" t="n">
+        <v>46225.4960193287</v>
+      </c>
       <c r="O301" s="1" t="n"/>
       <c r="P301" s="1" t="n"/>
       <c r="Q301" s="1" t="inlineStr"/>
       <c r="R301" s="1" t="inlineStr">
         <is>
-          <t>Aguardando os dados do contador.</t>
+          <t xml:space="preserve">Cobramos novamente. </t>
         </is>
       </c>
       <c r="S301" s="1" t="inlineStr">
@@ -24123,7 +24115,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>81248</v>
+        <v>81247</v>
       </c>
       <c r="B302" s="1" t="inlineStr">
         <is>
@@ -24142,7 +24134,7 @@
       </c>
       <c r="E302" s="1" t="inlineStr">
         <is>
-          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
@@ -24160,14 +24152,14 @@
         </is>
       </c>
       <c r="J302" s="2" t="n">
-        <v>46224.43289853009</v>
+        <v>46224.43143758102</v>
       </c>
       <c r="K302" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L302" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M302" s="1" t="inlineStr">
@@ -24175,15 +24167,13 @@
           <t>Gabriela Peres</t>
         </is>
       </c>
-      <c r="N302" s="2" t="n">
-        <v>46225.48954270833</v>
-      </c>
+      <c r="N302" s="1" t="n"/>
       <c r="O302" s="1" t="n"/>
       <c r="P302" s="1" t="n"/>
       <c r="Q302" s="1" t="inlineStr"/>
       <c r="R302" s="1" t="inlineStr">
         <is>
-          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+          <t>Aguardando os dados do contador.</t>
         </is>
       </c>
       <c r="S302" s="1" t="inlineStr">
@@ -24196,26 +24186,26 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>81250</v>
+        <v>81248</v>
       </c>
       <c r="B303" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Municipal</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C303" s="1" t="inlineStr">
         <is>
-          <t>Divida Ativa</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D303" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - GC</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E303" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
+          <t>6981 - LUIZ GOMES DA SILVA - O GOIANO - SUPERMERCADO AVENIDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
@@ -24224,35 +24214,41 @@
       <c r="G303" s="1" t="n"/>
       <c r="H303" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I303" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J303" s="2" t="n">
-        <v>46224.44502184028</v>
+        <v>46224.43289853009</v>
       </c>
       <c r="K303" s="2" t="n">
         <v>46226</v>
       </c>
       <c r="L303" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M303" s="1" t="inlineStr">
         <is>
-          <t>Rafaella Massuia</t>
-        </is>
-      </c>
-      <c r="N303" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N303" s="2" t="n">
+        <v>46225.48954270833</v>
+      </c>
       <c r="O303" s="1" t="n"/>
       <c r="P303" s="1" t="n"/>
       <c r="Q303" s="1" t="inlineStr"/>
-      <c r="R303" s="1" t="inlineStr"/>
+      <c r="R303" s="1" t="inlineStr">
+        <is>
+          <t>Cobramos a antiga contabilidade. O certificado digital está no DINAMO.</t>
+        </is>
+      </c>
       <c r="S303" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24263,7 +24259,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>81251</v>
+        <v>81250</v>
       </c>
       <c r="B304" s="1" t="inlineStr">
         <is>
@@ -24282,7 +24278,7 @@
       </c>
       <c r="E304" s="1" t="inlineStr">
         <is>
-          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
+          <t xml:space="preserve">3172 - A B ANDRADE SUPERMERCADO - parcelamento ex- cliente. - efetivar parcelamento em 5 parcelas.Foi enviado a simulação, enviar as guias para os e-mails : dp.supandrade@gmail.com e adm.smandrade@gmail.com </t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
@@ -24300,7 +24296,7 @@
         </is>
       </c>
       <c r="J304" s="2" t="n">
-        <v>46224.44796296296</v>
+        <v>46224.44502184028</v>
       </c>
       <c r="K304" s="2" t="n">
         <v>46226</v>
@@ -24330,26 +24326,26 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>81267</v>
+        <v>81251</v>
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Processo de Prefeitura</t>
+          <t>Parcelamento Municipal</t>
         </is>
       </c>
       <c r="C305" s="1" t="inlineStr">
         <is>
-          <t>Geral</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D305" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - GC</t>
         </is>
       </c>
       <c r="E305" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
+          <t>3146 - Andrade - simular parcelamento municipal Bom Dia, o depósito da empresa 3146 está no nome de pessoa fisíca, o cliente quer regularizar.</t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
@@ -24367,10 +24363,10 @@
         </is>
       </c>
       <c r="J305" s="2" t="n">
-        <v>46224.66958634259</v>
+        <v>46224.44796296296</v>
       </c>
       <c r="K305" s="2" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="L305" s="1" t="inlineStr">
         <is>
@@ -24379,7 +24375,7 @@
       </c>
       <c r="M305" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Rafaella Massuia</t>
         </is>
       </c>
       <c r="N305" s="1" t="n"/>
@@ -24397,39 +24393,35 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>81270</v>
+        <v>81267</v>
       </c>
       <c r="B306" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C306" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D306" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E306" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
+          <t>Boa tarde, poderia cancelar a nota na prefeitura do cliente 4422 - ALL Service , numero da nota 841</t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>5604</v>
-      </c>
-      <c r="G306" s="1" t="inlineStr">
-        <is>
-          <t>GRAFICA TABOAO LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G306" s="1" t="n"/>
       <c r="H306" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I306" s="1" t="inlineStr">
@@ -24438,32 +24430,26 @@
         </is>
       </c>
       <c r="J306" s="2" t="n">
-        <v>46224.69047569444</v>
+        <v>46224.66958634259</v>
       </c>
       <c r="K306" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="L306" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M306" s="1" t="inlineStr">
         <is>
-          <t>Beatriz Rangel</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N306" s="1" t="n"/>
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="n"/>
       <c r="Q306" s="1" t="inlineStr"/>
-      <c r="R306" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde.
-Por gentileza, solicitar o AVCB e o IPTU (vigentes).
-Att,</t>
-        </is>
-      </c>
+      <c r="R306" s="1" t="inlineStr"/>
       <c r="S306" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24474,35 +24460,39 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>81274</v>
+        <v>81270</v>
       </c>
       <c r="B307" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C307" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D307" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E307" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
+          <t xml:space="preserve">Boa tarde! A empresa Grafica Taboão recebeu um email informando que o CLI está próximo do vencimento, é solicitou a renovação. </t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G307" s="1" t="n"/>
+        <v>5604</v>
+      </c>
+      <c r="G307" s="1" t="inlineStr">
+        <is>
+          <t>GRAFICA TABOAO LTDA</t>
+        </is>
+      </c>
       <c r="H307" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I307" s="1" t="inlineStr">
@@ -24511,26 +24501,32 @@
         </is>
       </c>
       <c r="J307" s="2" t="n">
-        <v>46224.71483579861</v>
+        <v>46224.69047569444</v>
       </c>
       <c r="K307" s="2" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="L307" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M307" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Beatriz Rangel</t>
         </is>
       </c>
       <c r="N307" s="1" t="n"/>
       <c r="O307" s="1" t="n"/>
       <c r="P307" s="1" t="n"/>
       <c r="Q307" s="1" t="inlineStr"/>
-      <c r="R307" s="1" t="inlineStr"/>
+      <c r="R307" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.
+Por gentileza, solicitar o AVCB e o IPTU (vigentes).
+Att,</t>
+        </is>
+      </c>
       <c r="S307" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24541,39 +24537,35 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>81316</v>
+        <v>81274</v>
       </c>
       <c r="B308" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C308" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inclusão de Ata </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D308" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E308" s="1" t="inlineStr">
         <is>
-          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
+          <t>Boa tarde, poderia cadastra a senha no MG Controle da empresa 6955 - Vale Concreto Bombas</t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
-        <v>6674</v>
-      </c>
-      <c r="G308" s="1" t="inlineStr">
-        <is>
-          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G308" s="1" t="n"/>
       <c r="H308" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I308" s="1" t="inlineStr">
@@ -24582,39 +24574,29 @@
         </is>
       </c>
       <c r="J308" s="2" t="n">
-        <v>46225.61705821759</v>
+        <v>46224.71483579861</v>
       </c>
       <c r="K308" s="2" t="n">
-        <v>46231</v>
+        <v>46226</v>
       </c>
       <c r="L308" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M308" s="1" t="inlineStr">
         <is>
-          <t>Daniela Silva</t>
+          <t>Romario Silva</t>
         </is>
       </c>
       <c r="N308" s="1" t="n"/>
       <c r="O308" s="1" t="n"/>
-      <c r="P308" s="2" t="n">
-        <v>46230.66303518519</v>
-      </c>
-      <c r="Q308" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R308" s="1" t="inlineStr">
-        <is>
-          <t>Enviar a planilha devidamente preenchida e completa.</t>
-        </is>
-      </c>
+      <c r="P308" s="1" t="n"/>
+      <c r="Q308" s="1" t="inlineStr"/>
+      <c r="R308" s="1" t="inlineStr"/>
       <c r="S308" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T308" s="1" t="n"/>
@@ -24622,7 +24604,7 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>81317</v>
+        <v>81316</v>
       </c>
       <c r="B309" s="1" t="inlineStr">
         <is>
@@ -24641,15 +24623,15 @@
       </c>
       <c r="E309" s="1" t="inlineStr">
         <is>
-          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
+          <t>6674 – HORTIFRUTI CENTRALAlteração contratual incluindo o CPF dos sócios da Nippo com o Fernando“No Hortifruti vai receber os sócios da Nippo. Fazer essa alteração contratual. Vamos aguardar o cliente definir as participações societárias na empresa. Enviar relação de documentos.”</t>
         </is>
       </c>
       <c r="F309" s="1" t="n">
-        <v>6673</v>
+        <v>6674</v>
       </c>
       <c r="G309" s="1" t="inlineStr">
         <is>
-          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
+          <t>HORTIFRUTI CENTRAL DO COIMBRA LTDA</t>
         </is>
       </c>
       <c r="H309" s="1" t="inlineStr">
@@ -24663,7 +24645,7 @@
         </is>
       </c>
       <c r="J309" s="2" t="n">
-        <v>46225.61752997685</v>
+        <v>46225.61705821759</v>
       </c>
       <c r="K309" s="2" t="n">
         <v>46231</v>
@@ -24681,7 +24663,7 @@
       <c r="N309" s="1" t="n"/>
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="2" t="n">
-        <v>46230.66237318287</v>
+        <v>46230.66303518519</v>
       </c>
       <c r="Q309" s="1" t="inlineStr">
         <is>
@@ -24690,7 +24672,7 @@
       </c>
       <c r="R309" s="1" t="inlineStr">
         <is>
-          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
+          <t>Enviar a planilha devidamente preenchida e completa.</t>
         </is>
       </c>
       <c r="S309" s="1" t="inlineStr">
@@ -24703,34 +24685,34 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>81343</v>
+        <v>81317</v>
       </c>
       <c r="B310" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C310" s="1" t="inlineStr">
         <is>
-          <t>Protestos</t>
+          <t xml:space="preserve">Inclusão de Ata </t>
         </is>
       </c>
       <c r="D310" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E310" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
+          <t>6673 – CHER SOLUÇÕESAlteração contratual na empresa CHER tirando a Juliana“Necessário realizar a alteração contratual tirando a JULIANA do quadro societário e a sócia remanescente ficará com 100% das cotas da empresa. Enviar a relação de documentos necessários.”</t>
         </is>
       </c>
       <c r="F310" s="1" t="n">
-        <v>6538</v>
+        <v>6673</v>
       </c>
       <c r="G310" s="1" t="inlineStr">
         <is>
-          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+          <t>CHER SOLUÇÕES COMERCIAIS LTDA</t>
         </is>
       </c>
       <c r="H310" s="1" t="inlineStr">
@@ -24744,10 +24726,10 @@
         </is>
       </c>
       <c r="J310" s="2" t="n">
-        <v>46225.78787369213</v>
+        <v>46225.61752997685</v>
       </c>
       <c r="K310" s="2" t="n">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="L310" s="1" t="inlineStr">
         <is>
@@ -24756,13 +24738,13 @@
       </c>
       <c r="M310" s="1" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Daniela Silva</t>
         </is>
       </c>
       <c r="N310" s="1" t="n"/>
       <c r="O310" s="1" t="n"/>
       <c r="P310" s="2" t="n">
-        <v>46230.55531678241</v>
+        <v>46230.66237318287</v>
       </c>
       <c r="Q310" s="1" t="inlineStr">
         <is>
@@ -24771,7 +24753,7 @@
       </c>
       <c r="R310" s="1" t="inlineStr">
         <is>
-          <t>SEGUE BOLETO DAS CUSTAS SOLICITADAS.</t>
+          <t>Enviar a planilha devidamente preechida (com todas as informações).</t>
         </is>
       </c>
       <c r="S310" s="1" t="inlineStr">
@@ -24784,73 +24766,80 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>81348</v>
+        <v>81343</v>
       </c>
       <c r="B311" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C311" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Protestos</t>
         </is>
       </c>
       <c r="D311" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E311" s="1" t="inlineStr">
         <is>
-          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
+          <t>SALDAO CASA E LAR - CUSTAS DO CARTÓRIOPreciso do boleto atualizado das custas do cartório, 1º Cartório de Embu das Artes, pagamos o imposto direto pelo dívida ativa.Att.Vander</t>
         </is>
       </c>
       <c r="F311" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G311" s="1" t="n"/>
+        <v>6538</v>
+      </c>
+      <c r="G311" s="1" t="inlineStr">
+        <is>
+          <t>SALDAO CASA &amp; LAR MOVEIS E ELETRODOMESTICOS LTDA</t>
+        </is>
+      </c>
       <c r="H311" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I311" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J311" s="2" t="n">
-        <v>46226.4148858449</v>
+        <v>46225.78787369213</v>
       </c>
       <c r="K311" s="2" t="n">
         <v>46227</v>
       </c>
       <c r="L311" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M311" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N311" s="2" t="n">
-        <v>46230.72068440972</v>
-      </c>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N311" s="1" t="n"/>
       <c r="O311" s="1" t="n"/>
-      <c r="P311" s="1" t="n"/>
-      <c r="Q311" s="1" t="inlineStr"/>
+      <c r="P311" s="2" t="n">
+        <v>46230.55531678241</v>
+      </c>
+      <c r="Q311" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="R311" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!
-Cobramos novamente.</t>
+          <t>SEGUE BOLETO DAS CUSTAS SOLICITADAS.</t>
         </is>
       </c>
       <c r="S311" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T311" s="1" t="n"/>
@@ -24858,67 +24847,70 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>81351</v>
+        <v>81348</v>
       </c>
       <c r="B312" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C312" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D312" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E312" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>6949 - TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDAConforme e-mail já enviado anteriormente, aguardo o envio dos resumos das folhas de pagamento e a folha de 13º 2025.Anexo o checklist.</t>
         </is>
       </c>
       <c r="F312" s="1" t="n">
-        <v>3587</v>
-      </c>
-      <c r="G312" s="1" t="inlineStr">
-        <is>
-          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G312" s="1" t="n"/>
       <c r="H312" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I312" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J312" s="2" t="n">
-        <v>46226.44303796296</v>
+        <v>46226.4148858449</v>
       </c>
       <c r="K312" s="2" t="n">
-        <v>46230</v>
+        <v>46227</v>
       </c>
       <c r="L312" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M312" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
-        </is>
-      </c>
-      <c r="N312" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N312" s="2" t="n">
+        <v>46230.72068440972</v>
+      </c>
       <c r="O312" s="1" t="n"/>
       <c r="P312" s="1" t="n"/>
       <c r="Q312" s="1" t="inlineStr"/>
-      <c r="R312" s="1" t="inlineStr"/>
+      <c r="R312" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Cobramos novamente.</t>
+        </is>
+      </c>
       <c r="S312" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -24929,7 +24921,7 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>81352</v>
+        <v>81351</v>
       </c>
       <c r="B313" s="1" t="inlineStr">
         <is>
@@ -24952,16 +24944,16 @@
         </is>
       </c>
       <c r="F313" s="1" t="n">
-        <v>3812</v>
+        <v>3587</v>
       </c>
       <c r="G313" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
+          <t>MERCADINHO RIZARDI CAJAMAR LTDA</t>
         </is>
       </c>
       <c r="H313" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I313" s="1" t="inlineStr">
@@ -24970,14 +24962,14 @@
         </is>
       </c>
       <c r="J313" s="2" t="n">
-        <v>46226.4440716088</v>
+        <v>46226.44303796296</v>
       </c>
       <c r="K313" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L313" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M313" s="1" t="inlineStr">
@@ -24985,18 +24977,11 @@
           <t>Francisco Pimenta</t>
         </is>
       </c>
-      <c r="N313" s="2" t="n">
-        <v>46230.66455783565</v>
-      </c>
+      <c r="N313" s="1" t="n"/>
       <c r="O313" s="1" t="n"/>
       <c r="P313" s="1" t="n"/>
       <c r="Q313" s="1" t="inlineStr"/>
-      <c r="R313" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Estou verificando o acesso junto a prefeitura.</t>
-        </is>
-      </c>
+      <c r="R313" s="1" t="inlineStr"/>
       <c r="S313" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25007,7 +24992,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>81353</v>
+        <v>81352</v>
       </c>
       <c r="B314" s="1" t="inlineStr">
         <is>
@@ -25030,11 +25015,11 @@
         </is>
       </c>
       <c r="F314" s="1" t="n">
-        <v>3878</v>
+        <v>3812</v>
       </c>
       <c r="G314" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cucinare Pro Alimentação </t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 37)</t>
         </is>
       </c>
       <c r="H314" s="1" t="inlineStr">
@@ -25048,7 +25033,7 @@
         </is>
       </c>
       <c r="J314" s="2" t="n">
-        <v>46226.44431542824</v>
+        <v>46226.4440716088</v>
       </c>
       <c r="K314" s="2" t="n">
         <v>46230</v>
@@ -25064,7 +25049,7 @@
         </is>
       </c>
       <c r="N314" s="2" t="n">
-        <v>46230.66437326389</v>
+        <v>46230.66455783565</v>
       </c>
       <c r="O314" s="1" t="n"/>
       <c r="P314" s="1" t="n"/>
@@ -25085,7 +25070,7 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
-        <v>81355</v>
+        <v>81353</v>
       </c>
       <c r="B315" s="1" t="inlineStr">
         <is>
@@ -25108,11 +25093,11 @@
         </is>
       </c>
       <c r="F315" s="1" t="n">
-        <v>4012</v>
+        <v>3878</v>
       </c>
       <c r="G315" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+          <t xml:space="preserve">Cucinare Pro Alimentação </t>
         </is>
       </c>
       <c r="H315" s="1" t="inlineStr">
@@ -25126,7 +25111,7 @@
         </is>
       </c>
       <c r="J315" s="2" t="n">
-        <v>46226.44472357639</v>
+        <v>46226.44431542824</v>
       </c>
       <c r="K315" s="2" t="n">
         <v>46230</v>
@@ -25142,89 +25127,96 @@
         </is>
       </c>
       <c r="N315" s="2" t="n">
-        <v>46230.66408684028</v>
+        <v>46230.66437326389</v>
       </c>
       <c r="O315" s="1" t="n"/>
       <c r="P315" s="1" t="n"/>
       <c r="Q315" s="1" t="inlineStr"/>
       <c r="R315" s="1" t="inlineStr">
         <is>
+          <t>Boa tarde!
+Estou verificando o acesso junto a prefeitura.</t>
+        </is>
+      </c>
+      <c r="S315" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T315" s="1" t="n"/>
+      <c r="U315" s="1" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="1" t="n">
+        <v>81355</v>
+      </c>
+      <c r="B316" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C316" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D316" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E316" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+        </is>
+      </c>
+      <c r="F316" s="1" t="n">
+        <v>4012</v>
+      </c>
+      <c r="G316" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 50) </t>
+        </is>
+      </c>
+      <c r="H316" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
+      <c r="I316" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="n">
+        <v>46226.44472357639</v>
+      </c>
+      <c r="K316" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="L316" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M316" s="1" t="inlineStr">
+        <is>
+          <t>Francisco Pimenta</t>
+        </is>
+      </c>
+      <c r="N316" s="2" t="n">
+        <v>46230.66408684028</v>
+      </c>
+      <c r="O316" s="1" t="n"/>
+      <c r="P316" s="1" t="n"/>
+      <c r="Q316" s="1" t="inlineStr"/>
+      <c r="R316" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Boa tarde!
 Estou verificando o acesso junto a prefeitura.
 </t>
         </is>
       </c>
-      <c r="S315" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T315" s="1" t="n"/>
-      <c r="U315" s="1" t="inlineStr"/>
-    </row>
-    <row r="316">
-      <c r="A316" s="1" t="n">
-        <v>81362</v>
-      </c>
-      <c r="B316" s="1" t="inlineStr">
-        <is>
-          <t>Senha</t>
-        </is>
-      </c>
-      <c r="C316" s="1" t="inlineStr">
-        <is>
-          <t>Prefeitura</t>
-        </is>
-      </c>
-      <c r="D316" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="E316" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
-        </is>
-      </c>
-      <c r="F316" s="1" t="n">
-        <v>4804</v>
-      </c>
-      <c r="G316" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
-        </is>
-      </c>
-      <c r="H316" s="1" t="inlineStr">
-        <is>
-          <t>Talita Silva</t>
-        </is>
-      </c>
-      <c r="I316" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J316" s="2" t="n">
-        <v>46226.44931420139</v>
-      </c>
-      <c r="K316" s="2" t="n">
-        <v>46230</v>
-      </c>
-      <c r="L316" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M316" s="1" t="inlineStr">
-        <is>
-          <t>Francisco Pimenta</t>
-        </is>
-      </c>
-      <c r="N316" s="1" t="n"/>
-      <c r="O316" s="1" t="n"/>
-      <c r="P316" s="1" t="n"/>
-      <c r="Q316" s="1" t="inlineStr"/>
-      <c r="R316" s="1" t="inlineStr"/>
       <c r="S316" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25235,7 +25227,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>81363</v>
+        <v>81362</v>
       </c>
       <c r="B317" s="1" t="inlineStr">
         <is>
@@ -25258,11 +25250,11 @@
         </is>
       </c>
       <c r="F317" s="1" t="n">
-        <v>4841</v>
+        <v>4804</v>
       </c>
       <c r="G317" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
+          <t xml:space="preserve">FLV 7 RESTAURANTES LTDA (FILIAL 07) </t>
         </is>
       </c>
       <c r="H317" s="1" t="inlineStr">
@@ -25276,14 +25268,14 @@
         </is>
       </c>
       <c r="J317" s="2" t="n">
-        <v>46226.45019482639</v>
+        <v>46226.44931420139</v>
       </c>
       <c r="K317" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L317" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M317" s="1" t="inlineStr">
@@ -25291,11 +25283,18 @@
           <t>Francisco Pimenta</t>
         </is>
       </c>
-      <c r="N317" s="1" t="n"/>
+      <c r="N317" s="2" t="n">
+        <v>46231.55945818287</v>
+      </c>
       <c r="O317" s="1" t="n"/>
       <c r="P317" s="1" t="n"/>
       <c r="Q317" s="1" t="inlineStr"/>
-      <c r="R317" s="1" t="inlineStr"/>
+      <c r="R317" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Estou verificando o acesso junto a prefeitura.</t>
+        </is>
+      </c>
       <c r="S317" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -25306,7 +25305,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>81364</v>
+        <v>81363</v>
       </c>
       <c r="B318" s="1" t="inlineStr">
         <is>
@@ -25329,11 +25328,11 @@
         </is>
       </c>
       <c r="F318" s="1" t="n">
-        <v>4918</v>
+        <v>4841</v>
       </c>
       <c r="G318" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
+          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H318" s="1" t="inlineStr">
@@ -25347,7 +25346,7 @@
         </is>
       </c>
       <c r="J318" s="2" t="n">
-        <v>46226.45123028935</v>
+        <v>46226.45019482639</v>
       </c>
       <c r="K318" s="2" t="n">
         <v>46230</v>
@@ -25377,7 +25376,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>81365</v>
+        <v>81364</v>
       </c>
       <c r="B319" s="1" t="inlineStr">
         <is>
@@ -25400,11 +25399,11 @@
         </is>
       </c>
       <c r="F319" s="1" t="n">
-        <v>5017</v>
+        <v>4918</v>
       </c>
       <c r="G319" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 61)</t>
         </is>
       </c>
       <c r="H319" s="1" t="inlineStr">
@@ -25418,7 +25417,7 @@
         </is>
       </c>
       <c r="J319" s="2" t="n">
-        <v>46226.45200285879</v>
+        <v>46226.45123028935</v>
       </c>
       <c r="K319" s="2" t="n">
         <v>46230</v>
@@ -25448,7 +25447,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>81367</v>
+        <v>81365</v>
       </c>
       <c r="B320" s="1" t="inlineStr">
         <is>
@@ -25471,11 +25470,11 @@
         </is>
       </c>
       <c r="F320" s="1" t="n">
-        <v>5153</v>
+        <v>5017</v>
       </c>
       <c r="G320" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 24)</t>
         </is>
       </c>
       <c r="H320" s="1" t="inlineStr">
@@ -25489,7 +25488,7 @@
         </is>
       </c>
       <c r="J320" s="2" t="n">
-        <v>46226.45361840277</v>
+        <v>46226.45200285879</v>
       </c>
       <c r="K320" s="2" t="n">
         <v>46230</v>
@@ -25519,7 +25518,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>81368</v>
+        <v>81367</v>
       </c>
       <c r="B321" s="1" t="inlineStr">
         <is>
@@ -25542,11 +25541,11 @@
         </is>
       </c>
       <c r="F321" s="1" t="n">
-        <v>5154</v>
+        <v>5153</v>
       </c>
       <c r="G321" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
         </is>
       </c>
       <c r="H321" s="1" t="inlineStr">
@@ -25560,7 +25559,7 @@
         </is>
       </c>
       <c r="J321" s="2" t="n">
-        <v>46226.45395802084</v>
+        <v>46226.45361840277</v>
       </c>
       <c r="K321" s="2" t="n">
         <v>46230</v>
@@ -25590,7 +25589,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>81369</v>
+        <v>81368</v>
       </c>
       <c r="B322" s="1" t="inlineStr">
         <is>
@@ -25609,15 +25608,15 @@
       </c>
       <c r="E322" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
-        <v>3049</v>
+        <v>5154</v>
       </c>
       <c r="G322" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
         </is>
       </c>
       <c r="H322" s="1" t="inlineStr">
@@ -25631,7 +25630,7 @@
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>46226.45434436342</v>
+        <v>46226.45395802084</v>
       </c>
       <c r="K322" s="2" t="n">
         <v>46230</v>
@@ -25643,7 +25642,7 @@
       </c>
       <c r="M322" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N322" s="1" t="n"/>
@@ -25661,7 +25660,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>81370</v>
+        <v>81369</v>
       </c>
       <c r="B323" s="1" t="inlineStr">
         <is>
@@ -25680,15 +25679,15 @@
       </c>
       <c r="E323" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F323" s="1" t="n">
-        <v>5222</v>
+        <v>3049</v>
       </c>
       <c r="G323" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 04)</t>
         </is>
       </c>
       <c r="H323" s="1" t="inlineStr">
@@ -25702,7 +25701,7 @@
         </is>
       </c>
       <c r="J323" s="2" t="n">
-        <v>46226.45476809028</v>
+        <v>46226.45434436342</v>
       </c>
       <c r="K323" s="2" t="n">
         <v>46230</v>
@@ -25714,7 +25713,7 @@
       </c>
       <c r="M323" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Izabely Araujo</t>
         </is>
       </c>
       <c r="N323" s="1" t="n"/>
@@ -25732,7 +25731,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>81371</v>
+        <v>81370</v>
       </c>
       <c r="B324" s="1" t="inlineStr">
         <is>
@@ -25755,11 +25754,11 @@
         </is>
       </c>
       <c r="F324" s="1" t="n">
-        <v>5224</v>
+        <v>5222</v>
       </c>
       <c r="G324" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
         </is>
       </c>
       <c r="H324" s="1" t="inlineStr">
@@ -25773,7 +25772,7 @@
         </is>
       </c>
       <c r="J324" s="2" t="n">
-        <v>46226.45489934028</v>
+        <v>46226.45476809028</v>
       </c>
       <c r="K324" s="2" t="n">
         <v>46230</v>
@@ -25803,7 +25802,7 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>81372</v>
+        <v>81371</v>
       </c>
       <c r="B325" s="1" t="inlineStr">
         <is>
@@ -25826,11 +25825,11 @@
         </is>
       </c>
       <c r="F325" s="1" t="n">
-        <v>5311</v>
+        <v>5224</v>
       </c>
       <c r="G325" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 70)</t>
         </is>
       </c>
       <c r="H325" s="1" t="inlineStr">
@@ -25844,7 +25843,7 @@
         </is>
       </c>
       <c r="J325" s="2" t="n">
-        <v>46226.45548961806</v>
+        <v>46226.45489934028</v>
       </c>
       <c r="K325" s="2" t="n">
         <v>46230</v>
@@ -25874,7 +25873,7 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>81375</v>
+        <v>81372</v>
       </c>
       <c r="B326" s="1" t="inlineStr">
         <is>
@@ -25897,16 +25896,16 @@
         </is>
       </c>
       <c r="F326" s="1" t="n">
-        <v>5584</v>
+        <v>5311</v>
       </c>
       <c r="G326" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
+          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
         </is>
       </c>
       <c r="H326" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I326" s="1" t="inlineStr">
@@ -25915,7 +25914,7 @@
         </is>
       </c>
       <c r="J326" s="2" t="n">
-        <v>46226.45693457176</v>
+        <v>46226.45548961806</v>
       </c>
       <c r="K326" s="2" t="n">
         <v>46230</v>
@@ -25945,7 +25944,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>81376</v>
+        <v>81375</v>
       </c>
       <c r="B327" s="1" t="inlineStr">
         <is>
@@ -25964,20 +25963,20 @@
       </c>
       <c r="E327" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Por gentileza, incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F327" s="1" t="n">
-        <v>2745</v>
+        <v>5584</v>
       </c>
       <c r="G327" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H327" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I327" s="1" t="inlineStr">
@@ -25986,7 +25985,7 @@
         </is>
       </c>
       <c r="J327" s="2" t="n">
-        <v>46226.46478128473</v>
+        <v>46226.45693457176</v>
       </c>
       <c r="K327" s="2" t="n">
         <v>46230</v>
@@ -25998,7 +25997,7 @@
       </c>
       <c r="M327" s="1" t="inlineStr">
         <is>
-          <t>Izabely Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N327" s="1" t="n"/>
@@ -26016,7 +26015,7 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>81377</v>
+        <v>81376</v>
       </c>
       <c r="B328" s="1" t="inlineStr">
         <is>
@@ -26039,11 +26038,11 @@
         </is>
       </c>
       <c r="F328" s="1" t="n">
-        <v>3601</v>
+        <v>2745</v>
       </c>
       <c r="G328" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H328" s="1" t="inlineStr">
@@ -26057,7 +26056,7 @@
         </is>
       </c>
       <c r="J328" s="2" t="n">
-        <v>46226.4658295949</v>
+        <v>46226.46478128473</v>
       </c>
       <c r="K328" s="2" t="n">
         <v>46230</v>
@@ -26087,7 +26086,7 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>81379</v>
+        <v>81377</v>
       </c>
       <c r="B329" s="1" t="inlineStr">
         <is>
@@ -26106,20 +26105,20 @@
       </c>
       <c r="E329" s="1" t="inlineStr">
         <is>
-          <t>Olá bom dia, sem senha no intranet, por gentileza incluir senha da prefeitura na mg controle.</t>
+          <t>Olá bom dia, senha da intranet está como inválida, por gentileza incluir senha da prefeitura na mg controle.</t>
         </is>
       </c>
       <c r="F329" s="1" t="n">
-        <v>4079</v>
+        <v>3601</v>
       </c>
       <c r="G329" s="1" t="inlineStr">
         <is>
-          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 12)</t>
         </is>
       </c>
       <c r="H329" s="1" t="inlineStr">
         <is>
-          <t>Thifany Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I329" s="1" t="inlineStr">
@@ -26128,7 +26127,7 @@
         </is>
       </c>
       <c r="J329" s="2" t="n">
-        <v>46226.47010887731</v>
+        <v>46226.4658295949</v>
       </c>
       <c r="K329" s="2" t="n">
         <v>46230</v>
@@ -26158,7 +26157,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>81380</v>
+        <v>81379</v>
       </c>
       <c r="B330" s="1" t="inlineStr">
         <is>
@@ -26181,16 +26180,16 @@
         </is>
       </c>
       <c r="F330" s="1" t="n">
-        <v>4339</v>
+        <v>4079</v>
       </c>
       <c r="G330" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
+          <t>VIT FRUT DISTRIBUIDORA DE FRUTAS LTDA FILIAL 01.</t>
         </is>
       </c>
       <c r="H330" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Thifany Leite</t>
         </is>
       </c>
       <c r="I330" s="1" t="inlineStr">
@@ -26199,7 +26198,7 @@
         </is>
       </c>
       <c r="J330" s="2" t="n">
-        <v>46226.47113148148</v>
+        <v>46226.47010887731</v>
       </c>
       <c r="K330" s="2" t="n">
         <v>46230</v>
@@ -26229,7 +26228,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>81381</v>
+        <v>81380</v>
       </c>
       <c r="B331" s="1" t="inlineStr">
         <is>
@@ -26252,16 +26251,16 @@
         </is>
       </c>
       <c r="F331" s="1" t="n">
-        <v>4625</v>
+        <v>4339</v>
       </c>
       <c r="G331" s="1" t="inlineStr">
         <is>
-          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 60)</t>
         </is>
       </c>
       <c r="H331" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I331" s="1" t="inlineStr">
@@ -26270,7 +26269,7 @@
         </is>
       </c>
       <c r="J331" s="2" t="n">
-        <v>46226.47206631945</v>
+        <v>46226.47113148148</v>
       </c>
       <c r="K331" s="2" t="n">
         <v>46230</v>
@@ -26300,7 +26299,7 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>81382</v>
+        <v>81381</v>
       </c>
       <c r="B332" s="1" t="inlineStr">
         <is>
@@ -26323,11 +26322,11 @@
         </is>
       </c>
       <c r="F332" s="1" t="n">
-        <v>4842</v>
+        <v>4625</v>
       </c>
       <c r="G332" s="1" t="inlineStr">
         <is>
-          <t>MERCADINHO REILAR DE ITAQUA LTDA (FILIAL 03)</t>
+          <t>HORUS ATACADO COMÉRCIO DE ALIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H332" s="1" t="inlineStr">
@@ -26341,14 +26340,14 @@
         </is>
       </c>
       <c r="J332" s="2" t="n">
-        <v>46226.47387114583</v>
+        <v>46226.47206631945</v>
       </c>
       <c r="K332" s="2" t="n">
         <v>46230</v>
       </c>
       <c r="L332" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M332" s="1" t="inlineStr">
@@ -26356,11 +26355,18 @@
           <t>Izabely Araujo</t>
         </is>
       </c>
-      <c r="N332" s="1" t="n"/>
+      <c r="N332" s="2" t="n">
+        <v>46231.55605555556</v>
+      </c>
       <c r="O332" s="1" t="n"/>
       <c r="P332" s="1" t="n"/>
       <c r="Q332" s="1" t="inlineStr"/>
-      <c r="R332" s="1" t="inlineStr"/>
+      <c r="R332" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aguardamos o retorno da prefeitura de Paraty.
+</t>
+        </is>
+      </c>
       <c r="S332" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-03 18:14
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U382" headerRowCount="1">
-  <autoFilter ref="A1:U382"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U383" headerRowCount="1">
+  <autoFilter ref="A1:U383"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U382"/>
+  <dimension ref="A1:U383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="L27" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M27" s="1" t="inlineStr">
@@ -2725,8 +2725,14 @@
       <c r="O27" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="P27" s="1" t="n"/>
-      <c r="Q27" s="1" t="inlineStr"/>
+      <c r="P27" s="2" t="n">
+        <v>46237.75345100695</v>
+      </c>
+      <c r="Q27" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="R27" s="1" t="inlineStr">
         <is>
           <t>olperação realizando o atendimento</t>
@@ -2734,7 +2740,7 @@
       </c>
       <c r="S27" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T27" s="1" t="n"/>
@@ -2855,7 +2861,7 @@
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Nayara Oliveira</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -2871,7 +2877,7 @@
       </c>
       <c r="L29" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M29" s="1" t="inlineStr">
@@ -2883,8 +2889,14 @@
       <c r="O29" s="2" t="n">
         <v>46237</v>
       </c>
-      <c r="P29" s="1" t="n"/>
-      <c r="Q29" s="1" t="inlineStr"/>
+      <c r="P29" s="2" t="n">
+        <v>46237.7525496875</v>
+      </c>
+      <c r="Q29" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
       <c r="R29" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">isso não é pertinente ao depto fiscal </t>
@@ -2892,7 +2904,7 @@
       </c>
       <c r="S29" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T29" s="1" t="n"/>
@@ -20880,76 +20892,62 @@
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
-        <v>80165</v>
+        <v>81813</v>
       </c>
       <c r="B253" s="1" t="inlineStr">
         <is>
-          <t>MG Controle</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C253" s="1" t="inlineStr">
         <is>
-          <t>Erro de Baixa</t>
+          <t>Teste</t>
         </is>
       </c>
       <c r="D253" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Olá, Daniel, boa tarde.No dia 03/08 solicitei ao cliente Luciano um novo SPED ICMS da loja 3829, referente a outubro de 2025, pois o arquivo enviado na época apresentava erro nas NFC-es. No entanto, não tivemos retorno desde então.Preciso da sua ajuda com esse caso, pois recebemos uma notificação informando que a entrega precisa ser realizada com urgência. e estamos no período de fechamento fiscal o quanto antes é melhor.</t>
         </is>
       </c>
       <c r="F253" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G253" s="1" t="n"/>
-      <c r="H253" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
+      <c r="H253" s="1" t="n"/>
       <c r="I253" s="1" t="inlineStr">
         <is>
-          <t>CONTROLADORIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J253" s="2" t="n">
-        <v>46190.71175925926</v>
+        <v>46237.75563526621</v>
       </c>
       <c r="K253" s="2" t="n">
-        <v>46191</v>
+        <v>46239</v>
       </c>
       <c r="L253" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M253" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Vanessa Tavares</t>
         </is>
       </c>
       <c r="N253" s="1" t="n"/>
       <c r="O253" s="1" t="n"/>
-      <c r="P253" s="2" t="n">
-        <v>46190.7346272338</v>
-      </c>
-      <c r="Q253" s="1" t="inlineStr">
-        <is>
-          <t>Gabriel Amaral</t>
-        </is>
-      </c>
-      <c r="R253" s="1" t="inlineStr">
-        <is>
-          <t>Tarefas baixadas</t>
-        </is>
-      </c>
+      <c r="P253" s="1" t="n"/>
+      <c r="Q253" s="1" t="inlineStr"/>
+      <c r="R253" s="1" t="n"/>
       <c r="S253" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T253" s="1" t="n"/>
@@ -20957,7 +20955,7 @@
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
-        <v>80250</v>
+        <v>80165</v>
       </c>
       <c r="B254" s="1" t="inlineStr">
         <is>
@@ -20976,7 +20974,7 @@
       </c>
       <c r="E254" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F254" s="1" t="n">
@@ -20994,21 +20992,25 @@
         </is>
       </c>
       <c r="J254" s="2" t="n">
-        <v>46192.6584477662</v>
+        <v>46190.71175925926</v>
       </c>
       <c r="K254" s="2" t="n">
-        <v>46195</v>
+        <v>46191</v>
       </c>
       <c r="L254" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M254" s="1" t="n"/>
+      <c r="M254" s="1" t="inlineStr">
+        <is>
+          <t>Leticia Queiroz</t>
+        </is>
+      </c>
       <c r="N254" s="1" t="n"/>
       <c r="O254" s="1" t="n"/>
       <c r="P254" s="2" t="n">
-        <v>46192.70597966435</v>
+        <v>46190.7346272338</v>
       </c>
       <c r="Q254" s="1" t="inlineStr">
         <is>
@@ -21030,7 +21032,7 @@
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
-        <v>80709</v>
+        <v>80250</v>
       </c>
       <c r="B255" s="1" t="inlineStr">
         <is>
@@ -21049,7 +21051,7 @@
       </c>
       <c r="E255" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde!Por gentileza, baixar as consultas Dec das seguintes empresas;635765986911</t>
         </is>
       </c>
       <c r="F255" s="1" t="n">
@@ -21067,25 +21069,21 @@
         </is>
       </c>
       <c r="J255" s="2" t="n">
-        <v>46205.72485570602</v>
+        <v>46192.6584477662</v>
       </c>
       <c r="K255" s="2" t="n">
-        <v>46206</v>
+        <v>46195</v>
       </c>
       <c r="L255" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M255" s="1" t="inlineStr">
-        <is>
-          <t>Leticia Queiroz</t>
-        </is>
-      </c>
+      <c r="M255" s="1" t="n"/>
       <c r="N255" s="1" t="n"/>
       <c r="O255" s="1" t="n"/>
       <c r="P255" s="2" t="n">
-        <v>46205.73248877314</v>
+        <v>46192.70597966435</v>
       </c>
       <c r="Q255" s="1" t="inlineStr">
         <is>
@@ -21107,7 +21105,7 @@
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
-        <v>81083</v>
+        <v>80709</v>
       </c>
       <c r="B256" s="1" t="inlineStr">
         <is>
@@ -21126,7 +21124,7 @@
       </c>
       <c r="E256" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 1º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F256" s="1" t="n">
@@ -21144,10 +21142,10 @@
         </is>
       </c>
       <c r="J256" s="2" t="n">
-        <v>46218.68119872685</v>
+        <v>46205.72485570602</v>
       </c>
       <c r="K256" s="2" t="n">
-        <v>46219</v>
+        <v>46206</v>
       </c>
       <c r="L256" s="1" t="inlineStr">
         <is>
@@ -21162,7 +21160,7 @@
       <c r="N256" s="1" t="n"/>
       <c r="O256" s="1" t="n"/>
       <c r="P256" s="2" t="n">
-        <v>46218.7466727662</v>
+        <v>46205.73248877314</v>
       </c>
       <c r="Q256" s="1" t="inlineStr">
         <is>
@@ -21171,7 +21169,7 @@
       </c>
       <c r="R256" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
+          <t>Tarefas baixadas</t>
         </is>
       </c>
       <c r="S256" s="1" t="inlineStr">
@@ -21184,7 +21182,7 @@
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
-        <v>81735</v>
+        <v>81083</v>
       </c>
       <c r="B257" s="1" t="inlineStr">
         <is>
@@ -21203,7 +21201,7 @@
       </c>
       <c r="E257" s="1" t="inlineStr">
         <is>
-          <t>Bom dia, por gentileza, poderiam baixar as tarefas de DEC 1º quinzena das seguintes empresas: DEC ACESSO NEGADO 5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO6913 66.497.830/0001-84 ACESSO NEGADO6850 00.545.793/0001-24 ACESSO NEGADO</t>
+          <t>Boa tarde, por gentileza baixar a tarefa de DEC 2º quinzena das seguintes empresas:DEC ACESSO NEGADO - RODRIGO5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F257" s="1" t="n">
@@ -21221,10 +21219,10 @@
         </is>
       </c>
       <c r="J257" s="2" t="n">
-        <v>46237.38211200231</v>
+        <v>46218.68119872685</v>
       </c>
       <c r="K257" s="2" t="n">
-        <v>46238</v>
+        <v>46219</v>
       </c>
       <c r="L257" s="1" t="inlineStr">
         <is>
@@ -21239,7 +21237,7 @@
       <c r="N257" s="1" t="n"/>
       <c r="O257" s="1" t="n"/>
       <c r="P257" s="2" t="n">
-        <v>46237.40692600694</v>
+        <v>46218.7466727662</v>
       </c>
       <c r="Q257" s="1" t="inlineStr">
         <is>
@@ -21248,7 +21246,7 @@
       </c>
       <c r="R257" s="1" t="inlineStr">
         <is>
-          <t>Tarefas baixadas</t>
+          <t xml:space="preserve">Tarefas já se encontram baixadas </t>
         </is>
       </c>
       <c r="S257" s="1" t="inlineStr">
@@ -21261,7 +21259,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>81805</v>
+        <v>81735</v>
       </c>
       <c r="B258" s="1" t="inlineStr">
         <is>
@@ -21275,48 +21273,62 @@
       </c>
       <c r="D258" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E258" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Prezados,Solicito a reabertura da tarefa FOPAG IMPRESSÃO PDF da empresa 5835 - CAETE COMUNICAÇÃO VISUAL DESIGNER ref. 07/2026.Grata!</t>
+          <t>Bom dia, por gentileza, poderiam baixar as tarefas de DEC 1º quinzena das seguintes empresas: DEC ACESSO NEGADO 5043 17.081.544/0001-28 ACESSO NEGADO6548 23.707.689/0001-94 ACESSO NEGADO6486 28.604.255/0001-82 ACESSO NEGADO3545 29.621.654/0001-14 ACESSO NEGADO6707 41.963.494/0002-78 ACESSO NEGADO6118 43.462.720/0010-72 ACESSO NEGADO6619 04.596.502/0116-27 ACESSO NEGADO6082 59.041.787/0001-82 ACESSO NEGADO6913 66.497.830/0001-84 ACESSO NEGADO6850 00.545.793/0001-24 ACESSO NEGADO</t>
         </is>
       </c>
       <c r="F258" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G258" s="1" t="n"/>
-      <c r="H258" s="1" t="n"/>
+      <c r="H258" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I258" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
         </is>
       </c>
       <c r="J258" s="2" t="n">
-        <v>46237.72901894676</v>
+        <v>46237.38211200231</v>
       </c>
       <c r="K258" s="2" t="n">
         <v>46238</v>
       </c>
       <c r="L258" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M258" s="1" t="inlineStr">
         <is>
-          <t>Oliene Mariano</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N258" s="1" t="n"/>
       <c r="O258" s="1" t="n"/>
-      <c r="P258" s="1" t="n"/>
-      <c r="Q258" s="1" t="inlineStr"/>
-      <c r="R258" s="1" t="n"/>
+      <c r="P258" s="2" t="n">
+        <v>46237.40692600694</v>
+      </c>
+      <c r="Q258" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
+      <c r="R258" s="1" t="inlineStr">
+        <is>
+          <t>Tarefas baixadas</t>
+        </is>
+      </c>
       <c r="S258" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T258" s="1" t="n"/>
@@ -28496,7 +28508,7 @@
       </c>
       <c r="L352" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M352" s="1" t="inlineStr">
@@ -28506,8 +28518,14 @@
       </c>
       <c r="N352" s="1" t="n"/>
       <c r="O352" s="1" t="n"/>
-      <c r="P352" s="1" t="n"/>
-      <c r="Q352" s="1" t="inlineStr"/>
+      <c r="P352" s="2" t="n">
+        <v>46237.74492465278</v>
+      </c>
+      <c r="Q352" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
       <c r="R352" s="1" t="inlineStr">
         <is>
           <t>Bom dia!
@@ -28516,7 +28534,7 @@
       </c>
       <c r="S352" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T352" s="1" t="n"/>
@@ -30592,6 +30610,73 @@
       </c>
       <c r="T382" s="1" t="n"/>
       <c r="U382" s="1" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="1" t="n">
+        <v>81811</v>
+      </c>
+      <c r="B383" s="1" t="inlineStr">
+        <is>
+          <t>Abertura de Empresa</t>
+        </is>
+      </c>
+      <c r="C383" s="1" t="inlineStr">
+        <is>
+          <t>Sociedade - Serviços</t>
+        </is>
+      </c>
+      <c r="D383" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA MASTER</t>
+        </is>
+      </c>
+      <c r="E383" s="1" t="inlineStr">
+        <is>
+          <t>ABERTURA DE EMPRESA DO GRUPO 6963-PROMOTORAS GYNTRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: SERVIÇOSFINALIDADE: OPERACIONALFORMA JURIDICA: LTDAPROPOSTA JÁ NEOCIADA NO VALOR DE R$2.500,00A abertura desta empresa tem como objetivo substituir a empresa Promotoras GYN, que atualmente está enquadrada no regime de Lucro Presumido. A nova empresa será constituída e enquadrada no regime de Lucro Real.</t>
+        </is>
+      </c>
+      <c r="F383" s="1" t="n">
+        <v>6963</v>
+      </c>
+      <c r="G383" s="1" t="inlineStr">
+        <is>
+          <t>PROMOTORAS GYN LTDA</t>
+        </is>
+      </c>
+      <c r="H383" s="1" t="n"/>
+      <c r="I383" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J383" s="2" t="n">
+        <v>46237.74869586805</v>
+      </c>
+      <c r="K383" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="L383" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M383" s="1" t="inlineStr">
+        <is>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N383" s="1" t="n"/>
+      <c r="O383" s="1" t="n"/>
+      <c r="P383" s="1" t="n"/>
+      <c r="Q383" s="1" t="inlineStr"/>
+      <c r="R383" s="1" t="n"/>
+      <c r="S383" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T383" s="1" t="n"/>
+      <c r="U383" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-05 17:57
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U479" headerRowCount="1">
-  <autoFilter ref="A1:U479"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U481" headerRowCount="1">
+  <autoFilter ref="A1:U481"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U479"/>
+  <dimension ref="A1:U481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1342,7 +1342,11 @@
         <v>0</v>
       </c>
       <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>Vitoria Regina</t>
+        </is>
+      </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL HOLDING</t>
@@ -1356,7 +1360,7 @@
       </c>
       <c r="L11" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M11" s="1" t="inlineStr">
@@ -1365,17 +1369,23 @@
         </is>
       </c>
       <c r="N11" s="1" t="n"/>
-      <c r="O11" s="1" t="n"/>
+      <c r="O11" s="2" t="n">
+        <v>46241</v>
+      </c>
       <c r="P11" s="1" t="n"/>
       <c r="Q11" s="1" t="inlineStr"/>
-      <c r="R11" s="1" t="n"/>
+      <c r="R11" s="1" t="inlineStr"/>
       <c r="S11" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T11" s="1" t="n"/>
-      <c r="U11" s="1" t="inlineStr"/>
+      <c r="U11" s="1" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -2526,7 +2536,7 @@
       </c>
       <c r="N25" s="1" t="n"/>
       <c r="O25" s="2" t="n">
-        <v>46237</v>
+        <v>46241</v>
       </c>
       <c r="P25" s="1" t="n"/>
       <c r="Q25" s="1" t="inlineStr"/>
@@ -6912,7 +6922,7 @@
       </c>
       <c r="L78" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M78" s="1" t="inlineStr">
@@ -6924,12 +6934,22 @@
       <c r="O78" s="2" t="n">
         <v>46240</v>
       </c>
-      <c r="P78" s="1" t="n"/>
-      <c r="Q78" s="1" t="inlineStr"/>
-      <c r="R78" s="1" t="inlineStr"/>
+      <c r="P78" s="2" t="n">
+        <v>46239.7068994213</v>
+      </c>
+      <c r="Q78" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
+      <c r="R78" s="1" t="inlineStr">
+        <is>
+          <t>DFC,não é possivel pois não foi entregue, é um relatorio a parte.</t>
+        </is>
+      </c>
       <c r="S78" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T78" s="1" t="n"/>
@@ -9625,7 +9645,11 @@
           <t>G13 IMPORTACAO E EXPORTACAO LTDA</t>
         </is>
       </c>
-      <c r="H111" s="1" t="n"/>
+      <c r="H111" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="I111" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -9639,7 +9663,7 @@
       </c>
       <c r="L111" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M111" s="1" t="inlineStr">
@@ -9651,14 +9675,18 @@
       <c r="O111" s="1" t="n"/>
       <c r="P111" s="1" t="n"/>
       <c r="Q111" s="1" t="inlineStr"/>
-      <c r="R111" s="1" t="n"/>
+      <c r="R111" s="1" t="inlineStr"/>
       <c r="S111" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T111" s="1" t="n"/>
-      <c r="U111" s="1" t="inlineStr"/>
+      <c r="U111" s="1" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -12070,7 +12098,11 @@
           <t xml:space="preserve">PS3 INSTALACOES E MONTAGENS LTDA </t>
         </is>
       </c>
-      <c r="H140" s="1" t="n"/>
+      <c r="H140" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
       <c r="I140" s="1" t="inlineStr">
         <is>
           <t>CTB - CONTÁBIL INDUSTRIA</t>
@@ -12084,7 +12116,7 @@
       </c>
       <c r="L140" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M140" s="1" t="inlineStr">
@@ -12093,17 +12125,23 @@
         </is>
       </c>
       <c r="N140" s="1" t="n"/>
-      <c r="O140" s="1" t="n"/>
+      <c r="O140" s="2" t="n">
+        <v>46241</v>
+      </c>
       <c r="P140" s="1" t="n"/>
       <c r="Q140" s="1" t="inlineStr"/>
-      <c r="R140" s="1" t="n"/>
+      <c r="R140" s="1" t="inlineStr"/>
       <c r="S140" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T140" s="1" t="n"/>
-      <c r="U140" s="1" t="inlineStr"/>
+      <c r="U140" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -34940,7 +34978,7 @@
       </c>
       <c r="L442" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M442" s="1" t="inlineStr">
@@ -34948,11 +34986,17 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N442" s="1" t="n"/>
+      <c r="N442" s="2" t="n">
+        <v>46239.72105385417</v>
+      </c>
       <c r="O442" s="1" t="n"/>
       <c r="P442" s="1" t="n"/>
       <c r="Q442" s="1" t="inlineStr"/>
-      <c r="R442" s="1" t="inlineStr"/>
+      <c r="R442" s="1" t="inlineStr">
+        <is>
+          <t>Documentos enviados para assinaturas</t>
+        </is>
+      </c>
       <c r="S442" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -37035,67 +37079,59 @@
     </row>
     <row r="473">
       <c r="A473" s="1" t="n">
-        <v>81909</v>
+        <v>81912</v>
       </c>
       <c r="B473" s="1" t="inlineStr">
         <is>
-          <t>Levantamento de Débitos</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C473" s="1" t="inlineStr">
         <is>
-          <t>RFB</t>
+          <t xml:space="preserve">Novo </t>
         </is>
       </c>
       <c r="D473" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E473" s="1" t="inlineStr">
         <is>
-          <t>Boa tardePor gentileza realizar o levantamento de débitos para a loja 1619-Lourencini, pendente na situação fiscalObrigado e no aguardo</t>
+          <t>POR GENTILEZA PODE CADASTRAR O CLIENTE 1619 LOURENCINI E AS SUAS FILIAIS NO NOVO SISTEMA DA GISS ONLINE PARA QUE POSSAMOS REALIZAR A APURAÇÃO DOS TRIBUTOS.</t>
         </is>
       </c>
       <c r="F473" s="1" t="n">
-        <v>1619</v>
-      </c>
-      <c r="G473" s="1" t="inlineStr">
-        <is>
-          <t>LOURENCINI COMÉRCIO DE ALIMENTOS LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H473" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G473" s="1" t="n"/>
+      <c r="H473" s="1" t="n"/>
       <c r="I473" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J473" s="2" t="n">
-        <v>46239.49885309028</v>
+        <v>46239.54500825232</v>
       </c>
       <c r="K473" s="2" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="L473" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M473" s="1" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Diego Pereira</t>
         </is>
       </c>
       <c r="N473" s="1" t="n"/>
       <c r="O473" s="1" t="n"/>
       <c r="P473" s="1" t="n"/>
       <c r="Q473" s="1" t="inlineStr"/>
-      <c r="R473" s="1" t="inlineStr"/>
+      <c r="R473" s="1" t="n"/>
       <c r="S473" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -37106,62 +37142,80 @@
     </row>
     <row r="474">
       <c r="A474" s="1" t="n">
-        <v>81912</v>
+        <v>81920</v>
       </c>
       <c r="B474" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C474" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Novo </t>
+          <t>Simples Nacional</t>
         </is>
       </c>
       <c r="D474" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E474" s="1" t="inlineStr">
         <is>
-          <t>POR GENTILEZA PODE CADASTRAR O CLIENTE 1619 LOURENCINI E AS SUAS FILIAIS NO NOVO SISTEMA DA GISS ONLINE PARA QUE POSSAMOS REALIZAR A APURAÇÃO DOS TRIBUTOS.</t>
+          <t>Prezados, boa tarde!!Por gentileza, realizar simulação de parcelamentos de pendencia do SN da empresa 5650.</t>
         </is>
       </c>
       <c r="F474" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G474" s="1" t="n"/>
-      <c r="H474" s="1" t="n"/>
+        <v>5650</v>
+      </c>
+      <c r="G474" s="1" t="inlineStr">
+        <is>
+          <t>RICHETTI COMERCIO DE BEBIDAS E ALIMENTOS LTDA</t>
+        </is>
+      </c>
+      <c r="H474" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="I474" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J474" s="2" t="n">
-        <v>46239.54500825232</v>
+        <v>46239.6513278588</v>
       </c>
       <c r="K474" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="L474" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M474" s="1" t="inlineStr">
         <is>
-          <t>Diego Pereira</t>
+          <t>Rogerio Egidio</t>
         </is>
       </c>
       <c r="N474" s="1" t="n"/>
       <c r="O474" s="1" t="n"/>
-      <c r="P474" s="1" t="n"/>
-      <c r="Q474" s="1" t="inlineStr"/>
-      <c r="R474" s="1" t="n"/>
+      <c r="P474" s="2" t="n">
+        <v>46239.69918232639</v>
+      </c>
+      <c r="Q474" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="R474" s="1" t="inlineStr">
+        <is>
+          <t>Segue levantamento de débitos do cliente 5650 - RICHETTI e simulados juntamente à proposta para parcelamentos dos débitos federais.</t>
+        </is>
+      </c>
       <c r="S474" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T474" s="1" t="n"/>
@@ -37169,80 +37223,66 @@
     </row>
     <row r="475">
       <c r="A475" s="1" t="n">
-        <v>81920</v>
+        <v>81926</v>
       </c>
       <c r="B475" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento RFB</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C475" s="1" t="inlineStr">
         <is>
-          <t>Simples Nacional</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D475" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E475" s="1" t="inlineStr">
         <is>
-          <t>Prezados, boa tarde!!Por gentileza, realizar simulação de parcelamentos de pendencia do SN da empresa 5650.</t>
+          <t>Boa tarde, Prezados!Solicito por gentileza, da criação / vinculação de acesso à Prefeitura de Foz do Iguaçu - PR, para emissão da guia do ISS, conforme notas fiscais em anexo</t>
         </is>
       </c>
       <c r="F475" s="1" t="n">
-        <v>5650</v>
+        <v>6537</v>
       </c>
       <c r="G475" s="1" t="inlineStr">
         <is>
-          <t>RICHETTI COMERCIO DE BEBIDAS E ALIMENTOS LTDA</t>
-        </is>
-      </c>
-      <c r="H475" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+          <t xml:space="preserve">NAKABOX - COMERCIO DE PECAS E ACESSORIOS PARA VEICULOS E MOTOCICLETAS LTDA  </t>
+        </is>
+      </c>
+      <c r="H475" s="1" t="n"/>
       <c r="I475" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J475" s="2" t="n">
-        <v>46239.6513278588</v>
+        <v>46239.68096542824</v>
       </c>
       <c r="K475" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="L475" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M475" s="1" t="inlineStr">
         <is>
-          <t>Rogerio Egidio</t>
+          <t>Cristiana Grizostomo</t>
         </is>
       </c>
       <c r="N475" s="1" t="n"/>
       <c r="O475" s="1" t="n"/>
-      <c r="P475" s="2" t="n">
-        <v>46239.69918232639</v>
-      </c>
-      <c r="Q475" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="R475" s="1" t="inlineStr">
-        <is>
-          <t>Segue levantamento de débitos do cliente 5650 - RICHETTI e simulados juntamente à proposta para parcelamentos dos débitos federais.</t>
-        </is>
-      </c>
+      <c r="P475" s="1" t="n"/>
+      <c r="Q475" s="1" t="inlineStr"/>
+      <c r="R475" s="1" t="n"/>
       <c r="S475" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T475" s="1" t="n"/>
@@ -37250,7 +37290,7 @@
     </row>
     <row r="476">
       <c r="A476" s="1" t="n">
-        <v>81926</v>
+        <v>81927</v>
       </c>
       <c r="B476" s="1" t="inlineStr">
         <is>
@@ -37264,20 +37304,20 @@
       </c>
       <c r="D476" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E476" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Prezados!Solicito por gentileza, da criação / vinculação de acesso à Prefeitura de Foz do Iguaçu - PR, para emissão da guia do ISS, conforme notas fiscais em anexo</t>
+          <t>Boa tarde , tudo bem estou tentando escriturar notas no portal do giss online mas aparece um erro falando que tem uma nova atualização da plataforma ,e senha esta no mg controle não entra nessa nova plataforma</t>
         </is>
       </c>
       <c r="F476" s="1" t="n">
-        <v>6537</v>
+        <v>1071</v>
       </c>
       <c r="G476" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAKABOX - COMERCIO DE PECAS E ACESSORIOS PARA VEICULOS E MOTOCICLETAS LTDA  </t>
+          <t>SUPERMERCADO KIYOMOTO LTDA</t>
         </is>
       </c>
       <c r="H476" s="1" t="n"/>
@@ -37287,7 +37327,7 @@
         </is>
       </c>
       <c r="J476" s="2" t="n">
-        <v>46239.68096542824</v>
+        <v>46239.68396504629</v>
       </c>
       <c r="K476" s="2" t="n">
         <v>46241</v>
@@ -37299,7 +37339,7 @@
       </c>
       <c r="M476" s="1" t="inlineStr">
         <is>
-          <t>Cristiana Grizostomo</t>
+          <t>Bruna Souza</t>
         </is>
       </c>
       <c r="N476" s="1" t="n"/>
@@ -37317,7 +37357,7 @@
     </row>
     <row r="477">
       <c r="A477" s="1" t="n">
-        <v>81927</v>
+        <v>81928</v>
       </c>
       <c r="B477" s="1" t="inlineStr">
         <is>
@@ -37336,15 +37376,15 @@
       </c>
       <c r="E477" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde , tudo bem estou tentando escriturar notas no portal do giss online mas aparece um erro falando que tem uma nova atualização da plataforma ,e senha esta no mg controle não entra nessa nova plataforma</t>
+          <t>Boa tarde , tudo bem ?estou tentando escriturar notas no portal do giss online mas aparece um erro falando que tem uma nova atualização da plataforma ,e senha esta no mg controle não entra nessa nova plataforma</t>
         </is>
       </c>
       <c r="F477" s="1" t="n">
-        <v>1071</v>
+        <v>4685</v>
       </c>
       <c r="G477" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO KIYOMOTO LTDA</t>
+          <t xml:space="preserve">EMPÓRIO SOLERA LTDA </t>
         </is>
       </c>
       <c r="H477" s="1" t="n"/>
@@ -37354,7 +37394,7 @@
         </is>
       </c>
       <c r="J477" s="2" t="n">
-        <v>46239.68396504629</v>
+        <v>46239.69066068287</v>
       </c>
       <c r="K477" s="2" t="n">
         <v>46241</v>
@@ -37384,7 +37424,7 @@
     </row>
     <row r="478">
       <c r="A478" s="1" t="n">
-        <v>81928</v>
+        <v>81929</v>
       </c>
       <c r="B478" s="1" t="inlineStr">
         <is>
@@ -37398,22 +37438,18 @@
       </c>
       <c r="D478" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E478" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde , tudo bem ?estou tentando escriturar notas no portal do giss online mas aparece um erro falando que tem uma nova atualização da plataforma ,e senha esta no mg controle não entra nessa nova plataforma</t>
+          <t xml:space="preserve">Por gentileza, validar se a empresa 5920- filial , não possui Inscrição municipal. Pois ela toma diversos serviços e estou sem acesso para escritura-los. </t>
         </is>
       </c>
       <c r="F478" s="1" t="n">
-        <v>4685</v>
-      </c>
-      <c r="G478" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EMPÓRIO SOLERA LTDA </t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G478" s="1" t="n"/>
       <c r="H478" s="1" t="n"/>
       <c r="I478" s="1" t="inlineStr">
         <is>
@@ -37421,7 +37457,7 @@
         </is>
       </c>
       <c r="J478" s="2" t="n">
-        <v>46239.69066068287</v>
+        <v>46239.69870706018</v>
       </c>
       <c r="K478" s="2" t="n">
         <v>46241</v>
@@ -37433,7 +37469,7 @@
       </c>
       <c r="M478" s="1" t="inlineStr">
         <is>
-          <t>Bruna Souza</t>
+          <t>Thayna Melo</t>
         </is>
       </c>
       <c r="N478" s="1" t="n"/>
@@ -37451,32 +37487,36 @@
     </row>
     <row r="479">
       <c r="A479" s="1" t="n">
-        <v>81929</v>
+        <v>81932</v>
       </c>
       <c r="B479" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C479" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D479" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E479" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por gentileza, validar se a empresa 5920- filial , não possui Inscrição municipal. Pois ela toma diversos serviços e estou sem acesso para escritura-los. </t>
+          <t>ALTERAÇÃO CONTRATUAL DE QSA. EMPRESA: 6921-METALÚRGICA G3 LTDAGRUPO: G4 LINHA VIVAPROPOSTA JÁ NEGOCIADA.</t>
         </is>
       </c>
       <c r="F479" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G479" s="1" t="n"/>
+        <v>6921</v>
+      </c>
+      <c r="G479" s="1" t="inlineStr">
+        <is>
+          <t>METALURGICA G3 LTDA</t>
+        </is>
+      </c>
       <c r="H479" s="1" t="n"/>
       <c r="I479" s="1" t="inlineStr">
         <is>
@@ -37484,10 +37524,10 @@
         </is>
       </c>
       <c r="J479" s="2" t="n">
-        <v>46239.69870706018</v>
+        <v>46239.71162623842</v>
       </c>
       <c r="K479" s="2" t="n">
-        <v>46241</v>
+        <v>46267</v>
       </c>
       <c r="L479" s="1" t="inlineStr">
         <is>
@@ -37496,7 +37536,7 @@
       </c>
       <c r="M479" s="1" t="inlineStr">
         <is>
-          <t>Thayna Melo</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N479" s="1" t="n"/>
@@ -37511,6 +37551,136 @@
       </c>
       <c r="T479" s="1" t="n"/>
       <c r="U479" s="1" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" s="1" t="n">
+        <v>81933</v>
+      </c>
+      <c r="B480" s="1" t="inlineStr">
+        <is>
+          <t>Certidão</t>
+        </is>
+      </c>
+      <c r="C480" s="1" t="inlineStr">
+        <is>
+          <t>Outras</t>
+        </is>
+      </c>
+      <c r="D480" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E480" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, providenciar:6990 - RC MATERIAIS ELETRICOS E HIDRAULICOS (MATRIZ) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL6991 - RC MATERIAIS ELETRICOS E HIDRAULICOS (FILIAL 1) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="F480" s="1" t="n">
+        <v>6990</v>
+      </c>
+      <c r="G480" s="1" t="inlineStr">
+        <is>
+          <t>AMANCIO S ELETRICA, HIDRAULICA E CONSTRUCAO EM GERAL LTDA (MATRIZ)</t>
+        </is>
+      </c>
+      <c r="H480" s="1" t="n"/>
+      <c r="I480" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J480" s="2" t="n">
+        <v>46239.72520292824</v>
+      </c>
+      <c r="K480" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="L480" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M480" s="1" t="inlineStr">
+        <is>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N480" s="1" t="n"/>
+      <c r="O480" s="1" t="n"/>
+      <c r="P480" s="1" t="n"/>
+      <c r="Q480" s="1" t="inlineStr"/>
+      <c r="R480" s="1" t="n"/>
+      <c r="S480" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T480" s="1" t="n"/>
+      <c r="U480" s="1" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="1" t="n">
+        <v>81934</v>
+      </c>
+      <c r="B481" s="1" t="inlineStr">
+        <is>
+          <t>Processo de Prefeitura</t>
+        </is>
+      </c>
+      <c r="C481" s="1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="D481" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E481" s="1" t="inlineStr">
+        <is>
+          <t>POR GENTILEZA PODE EFETUAR O CADASTRO DA LOJA 4788 - R. LOURENCINI  LTDA NO NOVO PORTAL DA GISS ONLINE PARA LANÇAMENTOS E APURAÇÃO DAS NF DE SERVIÇO</t>
+        </is>
+      </c>
+      <c r="F481" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G481" s="1" t="n"/>
+      <c r="H481" s="1" t="n"/>
+      <c r="I481" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J481" s="2" t="n">
+        <v>46239.72563020833</v>
+      </c>
+      <c r="K481" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="L481" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M481" s="1" t="inlineStr">
+        <is>
+          <t>Diego Pereira</t>
+        </is>
+      </c>
+      <c r="N481" s="1" t="n"/>
+      <c r="O481" s="1" t="n"/>
+      <c r="P481" s="1" t="n"/>
+      <c r="Q481" s="1" t="inlineStr"/>
+      <c r="R481" s="1" t="n"/>
+      <c r="S481" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T481" s="1" t="n"/>
+      <c r="U481" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-12 16:27
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -1038,7 +1038,7 @@
       </c>
       <c r="N7" s="1" t="n"/>
       <c r="O7" s="2" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="P7" s="1" t="n"/>
       <c r="Q7" s="1" t="inlineStr"/>
@@ -13910,7 +13910,11 @@
           <t xml:space="preserve">ARARAS ONLINE COMERCIO DIGITAL LTDA </t>
         </is>
       </c>
-      <c r="H161" s="1" t="n"/>
+      <c r="H161" s="1" t="inlineStr">
+        <is>
+          <t>Priscila Volpe</t>
+        </is>
+      </c>
       <c r="I161" s="1" t="inlineStr">
         <is>
           <t>EF - INDUSTRIA</t>
@@ -13924,7 +13928,7 @@
       </c>
       <c r="L161" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M161" s="1" t="inlineStr">
@@ -13936,14 +13940,18 @@
       <c r="O161" s="1" t="n"/>
       <c r="P161" s="1" t="n"/>
       <c r="Q161" s="1" t="inlineStr"/>
-      <c r="R161" s="1" t="n"/>
+      <c r="R161" s="1" t="inlineStr"/>
       <c r="S161" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T161" s="1" t="n"/>
-      <c r="U161" s="1" t="inlineStr"/>
+      <c r="U161" s="1" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -38994,7 +39002,7 @@
       </c>
       <c r="L494" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M494" s="1" t="inlineStr">
@@ -39002,11 +39010,19 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N494" s="1" t="n"/>
+      <c r="N494" s="2" t="n">
+        <v>46246.66714818287</v>
+      </c>
       <c r="O494" s="1" t="n"/>
       <c r="P494" s="1" t="n"/>
       <c r="Q494" s="1" t="inlineStr"/>
-      <c r="R494" s="1" t="inlineStr"/>
+      <c r="R494" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Processo de abertura em andamento. 
+Atenciosamente, </t>
+        </is>
+      </c>
       <c r="S494" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -39217,7 +39233,7 @@
       </c>
       <c r="L497" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M497" s="1" t="inlineStr">
@@ -39225,11 +39241,19 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N497" s="1" t="n"/>
+      <c r="N497" s="2" t="n">
+        <v>46246.66900671296</v>
+      </c>
       <c r="O497" s="1" t="n"/>
       <c r="P497" s="1" t="n"/>
       <c r="Q497" s="1" t="inlineStr"/>
-      <c r="R497" s="1" t="inlineStr"/>
+      <c r="R497" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados(as), boa tarde!
+Alteração contratual em andamento. 
+Atenciosamente, </t>
+        </is>
+      </c>
       <c r="S497" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -43859,7 +43883,7 @@
       </c>
       <c r="L558" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M558" s="1" t="inlineStr">
@@ -43869,12 +43893,23 @@
       </c>
       <c r="N558" s="1" t="n"/>
       <c r="O558" s="1" t="n"/>
-      <c r="P558" s="1" t="n"/>
-      <c r="Q558" s="1" t="inlineStr"/>
-      <c r="R558" s="1" t="inlineStr"/>
+      <c r="P558" s="2" t="n">
+        <v>46246.66841165509</v>
+      </c>
+      <c r="Q558" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R558" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde!
+Não há débitos em aberto, seguem certidões. </t>
+        </is>
+      </c>
       <c r="S558" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T558" s="1" t="n"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-14 09:44
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U617" headerRowCount="1">
-  <autoFilter ref="A1:U617"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U619" headerRowCount="1">
+  <autoFilter ref="A1:U619"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U617"/>
+  <dimension ref="A1:U619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="L178" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M178" s="1" t="inlineStr">
@@ -15467,12 +15467,22 @@
       <c r="O178" s="2" t="n">
         <v>46248</v>
       </c>
-      <c r="P178" s="1" t="n"/>
-      <c r="Q178" s="1" t="inlineStr"/>
-      <c r="R178" s="1" t="inlineStr"/>
+      <c r="P178" s="2" t="n">
+        <v>46248.38525096065</v>
+      </c>
+      <c r="Q178" s="1" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
+      <c r="R178" s="1" t="inlineStr">
+        <is>
+          <t>Em anexo</t>
+        </is>
+      </c>
       <c r="S178" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T178" s="1" t="n"/>
@@ -44849,16 +44859,16 @@
     </row>
     <row r="572">
       <c r="A572" s="1" t="n">
-        <v>82257</v>
+        <v>82253</v>
       </c>
       <c r="B572" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Processo de Prefeitura</t>
         </is>
       </c>
       <c r="C572" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Geral</t>
         </is>
       </c>
       <c r="D572" s="1" t="inlineStr">
@@ -44868,7 +44878,7 @@
       </c>
       <c r="E572" s="1" t="inlineStr">
         <is>
-          <t>4546 - FB - Preciso do login da nova versão do GissOnline, pois a partir de 07/2026 toda movimentação tem que esta na nova versão.</t>
+          <t>Boa tarde, Poderiam verificar a prefeitura da loja 6954 pois não tem a opção de escriturar NFTS.Fico no aguardo.</t>
         </is>
       </c>
       <c r="F572" s="1" t="n">
@@ -44877,7 +44887,7 @@
       <c r="G572" s="1" t="n"/>
       <c r="H572" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I572" s="1" t="inlineStr">
@@ -44886,26 +44896,30 @@
         </is>
       </c>
       <c r="J572" s="2" t="n">
-        <v>46245.74198217592</v>
+        <v>46245.71506697917</v>
       </c>
       <c r="K572" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="L572" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M572" s="1" t="inlineStr">
         <is>
-          <t>Nathany Silva</t>
+          <t>Beatriz Ferreira</t>
         </is>
       </c>
       <c r="N572" s="1" t="n"/>
       <c r="O572" s="1" t="n"/>
       <c r="P572" s="1" t="n"/>
       <c r="Q572" s="1" t="inlineStr"/>
-      <c r="R572" s="1" t="inlineStr"/>
+      <c r="R572" s="1" t="inlineStr">
+        <is>
+          <t>Empresa não é optante pelo simples nacional, neste caso, deve ser feito o acesso com certificado digital.</t>
+        </is>
+      </c>
       <c r="S572" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -44916,11 +44930,11 @@
     </row>
     <row r="573">
       <c r="A573" s="1" t="n">
-        <v>82258</v>
+        <v>82257</v>
       </c>
       <c r="B573" s="1" t="inlineStr">
         <is>
-          <t>Levantamento de Débitos</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C573" s="1" t="inlineStr">
@@ -44930,25 +44944,21 @@
       </c>
       <c r="D573" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E573" s="1" t="inlineStr">
         <is>
-          <t>prezados, favor providenciar levantamento de débitos junto a prefeitura e providenciar simulado de parcelamento. empresas: 6963 e 6962.</t>
+          <t>4546 - FB - Preciso do login da nova versão do GissOnline, pois a partir de 07/2026 toda movimentação tem que esta na nova versão.</t>
         </is>
       </c>
       <c r="F573" s="1" t="n">
-        <v>6963</v>
-      </c>
-      <c r="G573" s="1" t="inlineStr">
-        <is>
-          <t>PROMOTORAS GYN LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G573" s="1" t="n"/>
       <c r="H573" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I573" s="1" t="inlineStr">
@@ -44957,10 +44967,10 @@
         </is>
       </c>
       <c r="J573" s="2" t="n">
-        <v>46245.76093032408</v>
+        <v>46245.74198217592</v>
       </c>
       <c r="K573" s="2" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="L573" s="1" t="inlineStr">
         <is>
@@ -44969,7 +44979,7 @@
       </c>
       <c r="M573" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Nathany Silva</t>
         </is>
       </c>
       <c r="N573" s="1" t="n"/>
@@ -44987,11 +44997,11 @@
     </row>
     <row r="574">
       <c r="A574" s="1" t="n">
-        <v>82264</v>
+        <v>82258</v>
       </c>
       <c r="B574" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Levantamento de Débitos</t>
         </is>
       </c>
       <c r="C574" s="1" t="inlineStr">
@@ -45001,25 +45011,25 @@
       </c>
       <c r="D574" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E574" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza enviar a guia atualizada da TFEdas duas empresas do grupo BOMBEIROS 6621 E 6622</t>
+          <t>prezados, favor providenciar levantamento de débitos junto a prefeitura e providenciar simulado de parcelamento. empresas: 6963 e 6962.</t>
         </is>
       </c>
       <c r="F574" s="1" t="n">
-        <v>6621</v>
+        <v>6963</v>
       </c>
       <c r="G574" s="1" t="inlineStr">
         <is>
-          <t>BOMBEIROS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANÇA LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="H574" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I574" s="1" t="inlineStr">
@@ -45028,40 +45038,29 @@
         </is>
       </c>
       <c r="J574" s="2" t="n">
-        <v>46246.3872690162</v>
+        <v>46245.76093032408</v>
       </c>
       <c r="K574" s="2" t="n">
-        <v>46248</v>
+        <v>46246</v>
       </c>
       <c r="L574" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M574" s="1" t="inlineStr">
         <is>
-          <t>Leticia Queiroz</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="N574" s="1" t="n"/>
       <c r="O574" s="1" t="n"/>
-      <c r="P574" s="2" t="n">
-        <v>46246.66841165509</v>
-      </c>
-      <c r="Q574" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
-      <c r="R574" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Boa tarde!
-Não há débitos em aberto, seguem certidões. </t>
-        </is>
-      </c>
+      <c r="P574" s="1" t="n"/>
+      <c r="Q574" s="1" t="inlineStr"/>
+      <c r="R574" s="1" t="inlineStr"/>
       <c r="S574" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T574" s="1" t="n"/>
@@ -45069,11 +45068,11 @@
     </row>
     <row r="575">
       <c r="A575" s="1" t="n">
-        <v>82288</v>
+        <v>82264</v>
       </c>
       <c r="B575" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C575" s="1" t="inlineStr">
@@ -45083,21 +45082,25 @@
       </c>
       <c r="D575" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E575" s="1" t="inlineStr">
         <is>
-          <t>Renovação de Alvará - 6939 - Unirellos - segue documentos para renovação.</t>
+          <t>Por gentileza enviar a guia atualizada da TFEdas duas empresas do grupo BOMBEIROS 6621 E 6622</t>
         </is>
       </c>
       <c r="F575" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G575" s="1" t="n"/>
+        <v>6621</v>
+      </c>
+      <c r="G575" s="1" t="inlineStr">
+        <is>
+          <t>BOMBEIROS.COM.BR COMERCIO DE EQUIPAMENTOS DE SEGURANÇA LTDA</t>
+        </is>
+      </c>
       <c r="H575" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I575" s="1" t="inlineStr">
@@ -45106,7 +45109,7 @@
         </is>
       </c>
       <c r="J575" s="2" t="n">
-        <v>46246.50698491898</v>
+        <v>46246.3872690162</v>
       </c>
       <c r="K575" s="2" t="n">
         <v>46248</v>
@@ -45118,96 +45121,107 @@
       </c>
       <c r="M575" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
+          <t>Leticia Queiroz</t>
         </is>
       </c>
       <c r="N575" s="1" t="n"/>
       <c r="O575" s="1" t="n"/>
       <c r="P575" s="2" t="n">
+        <v>46246.66841165509</v>
+      </c>
+      <c r="Q575" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R575" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde!
+Não há débitos em aberto, seguem certidões. </t>
+        </is>
+      </c>
+      <c r="S575" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T575" s="1" t="n"/>
+      <c r="U575" s="1" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="1" t="n">
+        <v>82288</v>
+      </c>
+      <c r="B576" s="1" t="inlineStr">
+        <is>
+          <t>Regularização</t>
+        </is>
+      </c>
+      <c r="C576" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D576" s="1" t="inlineStr">
+        <is>
+          <t>SANTOS - ADM</t>
+        </is>
+      </c>
+      <c r="E576" s="1" t="inlineStr">
+        <is>
+          <t>Renovação de Alvará - 6939 - Unirellos - segue documentos para renovação.</t>
+        </is>
+      </c>
+      <c r="F576" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G576" s="1" t="n"/>
+      <c r="H576" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
+      <c r="I576" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J576" s="2" t="n">
+        <v>46246.50698491898</v>
+      </c>
+      <c r="K576" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="L576" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M576" s="1" t="inlineStr">
+        <is>
+          <t>Lidia Tavares</t>
+        </is>
+      </c>
+      <c r="N576" s="1" t="n"/>
+      <c r="O576" s="1" t="n"/>
+      <c r="P576" s="2" t="n">
         <v>46247.73764479167</v>
       </c>
-      <c r="Q575" s="1" t="inlineStr">
+      <c r="Q576" s="1" t="inlineStr">
         <is>
           <t>Bianca Ribeiro</t>
         </is>
       </c>
-      <c r="R575" s="1" t="inlineStr">
+      <c r="R576" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Prezados(as), boa tarde!
 Conforme solicitado, segue anexo o ALVARÁ - UNIRELOS TRANSPORTES E LOGISTICA LTDA (Válido até 31/12/2026).
 Atenciosamente, </t>
         </is>
       </c>
-      <c r="S575" s="1" t="inlineStr">
+      <c r="S576" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="T575" s="1" t="n"/>
-      <c r="U575" s="1" t="inlineStr"/>
-    </row>
-    <row r="576">
-      <c r="A576" s="1" t="n">
-        <v>82296</v>
-      </c>
-      <c r="B576" s="1" t="inlineStr">
-        <is>
-          <t>Parcelamento Estadual</t>
-        </is>
-      </c>
-      <c r="C576" s="1" t="inlineStr">
-        <is>
-          <t>Divida Ativa</t>
-        </is>
-      </c>
-      <c r="D576" s="1" t="inlineStr">
-        <is>
-          <t>SANTOS - ADM</t>
-        </is>
-      </c>
-      <c r="E576" s="1" t="inlineStr">
-        <is>
-          <t>Cliente 5219 e 5551 solicitou parcelamento do ICMS , pode fazer a simulação</t>
-        </is>
-      </c>
-      <c r="F576" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G576" s="1" t="n"/>
-      <c r="H576" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="I576" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J576" s="2" t="n">
-        <v>46246.6211778588</v>
-      </c>
-      <c r="K576" s="2" t="n">
-        <v>46248</v>
-      </c>
-      <c r="L576" s="1" t="inlineStr">
-        <is>
-          <t>Esperando Atendimento</t>
-        </is>
-      </c>
-      <c r="M576" s="1" t="inlineStr">
-        <is>
-          <t>Lidia Tavares</t>
-        </is>
-      </c>
-      <c r="N576" s="1" t="n"/>
-      <c r="O576" s="1" t="n"/>
-      <c r="P576" s="1" t="n"/>
-      <c r="Q576" s="1" t="inlineStr"/>
-      <c r="R576" s="1" t="inlineStr"/>
-      <c r="S576" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="T576" s="1" t="n"/>
@@ -45215,63 +45229,63 @@
     </row>
     <row r="577">
       <c r="A577" s="1" t="n">
-        <v>82298</v>
+        <v>82296</v>
       </c>
       <c r="B577" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Parcelamento Estadual</t>
         </is>
       </c>
       <c r="C577" s="1" t="inlineStr">
         <is>
-          <t>Outras Cláusulas</t>
+          <t>Divida Ativa</t>
         </is>
       </c>
       <c r="D577" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E577" s="1" t="inlineStr">
         <is>
-          <t>Cliente solicitou declaração do Contador informando qual foi a ultima alteração contratual da empresa antes do óbito da Sra. Maria da Conceição, bem como a composição societária vigente à época, indicando quem eram os sócios,Com  esclarecimentos e documentação correspondente às referidas alterações. E motivo</t>
+          <t>Cliente 5219 e 5551 solicitou parcelamento do ICMS , pode fazer a simulação</t>
         </is>
       </c>
       <c r="F577" s="1" t="n">
-        <v>2620</v>
-      </c>
-      <c r="G577" s="1" t="inlineStr">
-        <is>
-          <t>ANTOCON GALVANOPLASTIA LTDA</t>
-        </is>
-      </c>
-      <c r="H577" s="1" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G577" s="1" t="n"/>
+      <c r="H577" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="I577" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J577" s="2" t="n">
-        <v>46246.6301065625</v>
+        <v>46246.6211778588</v>
       </c>
       <c r="K577" s="2" t="n">
-        <v>46267</v>
+        <v>46248</v>
       </c>
       <c r="L577" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M577" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N577" s="1" t="n"/>
       <c r="O577" s="1" t="n"/>
       <c r="P577" s="1" t="n"/>
       <c r="Q577" s="1" t="inlineStr"/>
-      <c r="R577" s="1" t="n"/>
+      <c r="R577" s="1" t="inlineStr"/>
       <c r="S577" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -45282,67 +45296,63 @@
     </row>
     <row r="578">
       <c r="A578" s="1" t="n">
-        <v>82304</v>
+        <v>82298</v>
       </c>
       <c r="B578" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento RFB</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C578" s="1" t="inlineStr">
         <is>
-          <t>Simplificado</t>
+          <t>Outras Cláusulas</t>
         </is>
       </c>
       <c r="D578" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E578" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Cliente solicitou a simulação dos parcelamentos em atraso, poderiam me enviar por gentileza?Aguardo, obrigada!</t>
+          <t>Cliente solicitou declaração do Contador informando qual foi a ultima alteração contratual da empresa antes do óbito da Sra. Maria da Conceição, bem como a composição societária vigente à época, indicando quem eram os sócios,Com  esclarecimentos e documentação correspondente às referidas alterações. E motivo</t>
         </is>
       </c>
       <c r="F578" s="1" t="n">
-        <v>4414</v>
+        <v>2620</v>
       </c>
       <c r="G578" s="1" t="inlineStr">
         <is>
-          <t>HN LEONE ADMINISTRAÇÃO DE BENS LTDA</t>
-        </is>
-      </c>
-      <c r="H578" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+          <t>ANTOCON GALVANOPLASTIA LTDA</t>
+        </is>
+      </c>
+      <c r="H578" s="1" t="n"/>
       <c r="I578" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J578" s="2" t="n">
-        <v>46246.7503934838</v>
+        <v>46246.6301065625</v>
       </c>
       <c r="K578" s="2" t="n">
-        <v>46248</v>
+        <v>46267</v>
       </c>
       <c r="L578" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M578" s="1" t="inlineStr">
         <is>
-          <t>Isabelli Afonso</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N578" s="1" t="n"/>
       <c r="O578" s="1" t="n"/>
       <c r="P578" s="1" t="n"/>
       <c r="Q578" s="1" t="inlineStr"/>
-      <c r="R578" s="1" t="inlineStr"/>
+      <c r="R578" s="1" t="n"/>
       <c r="S578" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -45353,48 +45363,48 @@
     </row>
     <row r="579">
       <c r="A579" s="1" t="n">
-        <v>82310</v>
+        <v>82304</v>
       </c>
       <c r="B579" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C579" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Simplificado</t>
         </is>
       </c>
       <c r="D579" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E579" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
+          <t>Boa tarde!Cliente solicitou a simulação dos parcelamentos em atraso, poderiam me enviar por gentileza?Aguardo, obrigada!</t>
         </is>
       </c>
       <c r="F579" s="1" t="n">
-        <v>6974</v>
+        <v>4414</v>
       </c>
       <c r="G579" s="1" t="inlineStr">
         <is>
-          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
+          <t>HN LEONE ADMINISTRAÇÃO DE BENS LTDA</t>
         </is>
       </c>
       <c r="H579" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I579" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J579" s="2" t="n">
-        <v>46247.3783179051</v>
+        <v>46246.7503934838</v>
       </c>
       <c r="K579" s="2" t="n">
         <v>46248</v>
@@ -45406,7 +45416,7 @@
       </c>
       <c r="M579" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Isabelli Afonso</t>
         </is>
       </c>
       <c r="N579" s="1" t="n"/>
@@ -45424,51 +45434,51 @@
     </row>
     <row r="580">
       <c r="A580" s="1" t="n">
-        <v>82314</v>
+        <v>82310</v>
       </c>
       <c r="B580" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C580" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D580" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E580" s="1" t="inlineStr">
         <is>
-          <t>Não possui login/senha de acesso à prefeitura.</t>
+          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
         </is>
       </c>
       <c r="F580" s="1" t="n">
-        <v>5016</v>
+        <v>6974</v>
       </c>
       <c r="G580" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 23)</t>
+          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
         </is>
       </c>
       <c r="H580" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I580" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J580" s="2" t="n">
-        <v>46247.41629224537</v>
+        <v>46247.3783179051</v>
       </c>
       <c r="K580" s="2" t="n">
-        <v>46251</v>
+        <v>46248</v>
       </c>
       <c r="L580" s="1" t="inlineStr">
         <is>
@@ -45477,7 +45487,7 @@
       </c>
       <c r="M580" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
       <c r="N580" s="1" t="n"/>
@@ -45495,63 +45505,67 @@
     </row>
     <row r="581">
       <c r="A581" s="1" t="n">
-        <v>82315</v>
+        <v>82314</v>
       </c>
       <c r="B581" s="1" t="inlineStr">
         <is>
-          <t>Notificação</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C581" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D581" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E581" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia, poderiam verificar a possibilidade de abrir um processo de revisão sobre um perdcomp feito 2025, recebemos despacho decisório sobre a não homologação da mesma! porem ao revisar não encontramos problema algum na perdcomp, foi paga em duplicidade porem em periodos diferentes, houve alteração em um código  e invés de pagar somente a diferença foi pago a darf com multa e juros por inteiro. então foi feito perdcomp da primeira darf. e ainda sobraria valor a compensar +/- 1.400,00. </t>
+          <t>Não possui login/senha de acesso à prefeitura.</t>
         </is>
       </c>
       <c r="F581" s="1" t="n">
-        <v>46</v>
+        <v>5016</v>
       </c>
       <c r="G581" s="1" t="inlineStr">
         <is>
-          <t>ASSOC RETIRO DE RECUP DA SAUDE DE ITAPECERICA DA SERRA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H581" s="1" t="n"/>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 23)</t>
+        </is>
+      </c>
+      <c r="H581" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I581" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J581" s="2" t="n">
-        <v>46247.42548993055</v>
+        <v>46247.41629224537</v>
       </c>
       <c r="K581" s="2" t="n">
-        <v>46254</v>
+        <v>46251</v>
       </c>
       <c r="L581" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M581" s="1" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N581" s="1" t="n"/>
       <c r="O581" s="1" t="n"/>
       <c r="P581" s="1" t="n"/>
       <c r="Q581" s="1" t="inlineStr"/>
-      <c r="R581" s="1" t="n"/>
+      <c r="R581" s="1" t="inlineStr"/>
       <c r="S581" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -45562,67 +45576,63 @@
     </row>
     <row r="582">
       <c r="A582" s="1" t="n">
-        <v>82316</v>
+        <v>82315</v>
       </c>
       <c r="B582" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Notificação</t>
         </is>
       </c>
       <c r="C582" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D582" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="E582" s="1" t="inlineStr">
         <is>
-          <t>Não possui login/senha de acesso à prefeitura.</t>
+          <t xml:space="preserve">Bom dia, poderiam verificar a possibilidade de abrir um processo de revisão sobre um perdcomp feito 2025, recebemos despacho decisório sobre a não homologação da mesma! porem ao revisar não encontramos problema algum na perdcomp, foi paga em duplicidade porem em periodos diferentes, houve alteração em um código  e invés de pagar somente a diferença foi pago a darf com multa e juros por inteiro. então foi feito perdcomp da primeira darf. e ainda sobraria valor a compensar +/- 1.400,00. </t>
         </is>
       </c>
       <c r="F582" s="1" t="n">
-        <v>5083</v>
+        <v>46</v>
       </c>
       <c r="G582" s="1" t="inlineStr">
         <is>
-          <t>PAULO S. DA SILVA</t>
-        </is>
-      </c>
-      <c r="H582" s="1" t="inlineStr">
-        <is>
-          <t>Edson Silva</t>
-        </is>
-      </c>
+          <t>ASSOC RETIRO DE RECUP DA SAUDE DE ITAPECERICA DA SERRA (MATRIZ)</t>
+        </is>
+      </c>
+      <c r="H582" s="1" t="n"/>
       <c r="I582" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J582" s="2" t="n">
-        <v>46247.42681547454</v>
+        <v>46247.42548993055</v>
       </c>
       <c r="K582" s="2" t="n">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="L582" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M582" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="N582" s="1" t="n"/>
       <c r="O582" s="1" t="n"/>
       <c r="P582" s="1" t="n"/>
       <c r="Q582" s="1" t="inlineStr"/>
-      <c r="R582" s="1" t="inlineStr"/>
+      <c r="R582" s="1" t="n"/>
       <c r="S582" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -45633,7 +45643,7 @@
     </row>
     <row r="583">
       <c r="A583" s="1" t="n">
-        <v>82317</v>
+        <v>82316</v>
       </c>
       <c r="B583" s="1" t="inlineStr">
         <is>
@@ -45656,16 +45666,16 @@
         </is>
       </c>
       <c r="F583" s="1" t="n">
-        <v>5149</v>
+        <v>5083</v>
       </c>
       <c r="G583" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 28)</t>
+          <t>PAULO S. DA SILVA</t>
         </is>
       </c>
       <c r="H583" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I583" s="1" t="inlineStr">
@@ -45674,7 +45684,7 @@
         </is>
       </c>
       <c r="J583" s="2" t="n">
-        <v>46247.42827943287</v>
+        <v>46247.42681547454</v>
       </c>
       <c r="K583" s="2" t="n">
         <v>46251</v>
@@ -45704,7 +45714,7 @@
     </row>
     <row r="584">
       <c r="A584" s="1" t="n">
-        <v>82318</v>
+        <v>82317</v>
       </c>
       <c r="B584" s="1" t="inlineStr">
         <is>
@@ -45723,15 +45733,15 @@
       </c>
       <c r="E584" s="1" t="inlineStr">
         <is>
-          <t>Login/senha disponibilizado na MGC está incorreto.</t>
+          <t>Não possui login/senha de acesso à prefeitura.</t>
         </is>
       </c>
       <c r="F584" s="1" t="n">
-        <v>5154</v>
+        <v>5149</v>
       </c>
       <c r="G584" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 28)</t>
         </is>
       </c>
       <c r="H584" s="1" t="inlineStr">
@@ -45745,7 +45755,7 @@
         </is>
       </c>
       <c r="J584" s="2" t="n">
-        <v>46247.43042322917</v>
+        <v>46247.42827943287</v>
       </c>
       <c r="K584" s="2" t="n">
         <v>46251</v>
@@ -45775,7 +45785,7 @@
     </row>
     <row r="585">
       <c r="A585" s="1" t="n">
-        <v>82320</v>
+        <v>82318</v>
       </c>
       <c r="B585" s="1" t="inlineStr">
         <is>
@@ -45794,15 +45804,15 @@
       </c>
       <c r="E585" s="1" t="inlineStr">
         <is>
-          <t>Não possui login/senha de acesso à prefeitura.</t>
+          <t>Login/senha disponibilizado na MGC está incorreto.</t>
         </is>
       </c>
       <c r="F585" s="1" t="n">
-        <v>5222</v>
+        <v>5154</v>
       </c>
       <c r="G585" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 67)</t>
         </is>
       </c>
       <c r="H585" s="1" t="inlineStr">
@@ -45816,7 +45826,7 @@
         </is>
       </c>
       <c r="J585" s="2" t="n">
-        <v>46247.43315929398</v>
+        <v>46247.43042322917</v>
       </c>
       <c r="K585" s="2" t="n">
         <v>46251</v>
@@ -45846,7 +45856,7 @@
     </row>
     <row r="586">
       <c r="A586" s="1" t="n">
-        <v>82323</v>
+        <v>82320</v>
       </c>
       <c r="B586" s="1" t="inlineStr">
         <is>
@@ -45869,11 +45879,11 @@
         </is>
       </c>
       <c r="F586" s="1" t="n">
-        <v>5311</v>
+        <v>5222</v>
       </c>
       <c r="G586" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 68)</t>
         </is>
       </c>
       <c r="H586" s="1" t="inlineStr">
@@ -45887,7 +45897,7 @@
         </is>
       </c>
       <c r="J586" s="2" t="n">
-        <v>46247.43662021991</v>
+        <v>46247.43315929398</v>
       </c>
       <c r="K586" s="2" t="n">
         <v>46251</v>
@@ -45917,7 +45927,7 @@
     </row>
     <row r="587">
       <c r="A587" s="1" t="n">
-        <v>82326</v>
+        <v>82323</v>
       </c>
       <c r="B587" s="1" t="inlineStr">
         <is>
@@ -45940,16 +45950,16 @@
         </is>
       </c>
       <c r="F587" s="1" t="n">
-        <v>5583</v>
+        <v>5311</v>
       </c>
       <c r="G587" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 01)</t>
+          <t>FLV 7 RESTAURANTE LTDA (FILIAL 30)</t>
         </is>
       </c>
       <c r="H587" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I587" s="1" t="inlineStr">
@@ -45958,7 +45968,7 @@
         </is>
       </c>
       <c r="J587" s="2" t="n">
-        <v>46247.43739552084</v>
+        <v>46247.43662021991</v>
       </c>
       <c r="K587" s="2" t="n">
         <v>46251</v>
@@ -45988,7 +45998,7 @@
     </row>
     <row r="588">
       <c r="A588" s="1" t="n">
-        <v>82328</v>
+        <v>82326</v>
       </c>
       <c r="B588" s="1" t="inlineStr">
         <is>
@@ -46011,11 +46021,11 @@
         </is>
       </c>
       <c r="F588" s="1" t="n">
-        <v>5584</v>
+        <v>5583</v>
       </c>
       <c r="G588" s="1" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H588" s="1" t="inlineStr">
@@ -46029,7 +46039,7 @@
         </is>
       </c>
       <c r="J588" s="2" t="n">
-        <v>46247.43814440972</v>
+        <v>46247.43739552084</v>
       </c>
       <c r="K588" s="2" t="n">
         <v>46251</v>
@@ -46059,7 +46069,7 @@
     </row>
     <row r="589">
       <c r="A589" s="1" t="n">
-        <v>82330</v>
+        <v>82328</v>
       </c>
       <c r="B589" s="1" t="inlineStr">
         <is>
@@ -46082,11 +46092,11 @@
         </is>
       </c>
       <c r="F589" s="1" t="n">
-        <v>5622</v>
+        <v>5584</v>
       </c>
       <c r="G589" s="1" t="inlineStr">
         <is>
-          <t>GHOST KITCHENS ALIMENTOS LTDA (FILIAL)</t>
+          <t>DISTRIBUIDORA FERRAZ GUERRA LTDA (FILIAL 02)</t>
         </is>
       </c>
       <c r="H589" s="1" t="inlineStr">
@@ -46100,7 +46110,7 @@
         </is>
       </c>
       <c r="J589" s="2" t="n">
-        <v>46247.43952728009</v>
+        <v>46247.43814440972</v>
       </c>
       <c r="K589" s="2" t="n">
         <v>46251</v>
@@ -46130,7 +46140,7 @@
     </row>
     <row r="590">
       <c r="A590" s="1" t="n">
-        <v>82336</v>
+        <v>82330</v>
       </c>
       <c r="B590" s="1" t="inlineStr">
         <is>
@@ -46149,15 +46159,15 @@
       </c>
       <c r="E590" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1065 - MARTINICA COMERCIAL LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Não possui login/senha de acesso à prefeitura.</t>
         </is>
       </c>
       <c r="F590" s="1" t="n">
-        <v>1065</v>
+        <v>5622</v>
       </c>
       <c r="G590" s="1" t="inlineStr">
         <is>
-          <t>MARTINICA COMERCIAL LTDA</t>
+          <t>GHOST KITCHENS ALIMENTOS LTDA (FILIAL)</t>
         </is>
       </c>
       <c r="H590" s="1" t="inlineStr">
@@ -46171,7 +46181,7 @@
         </is>
       </c>
       <c r="J590" s="2" t="n">
-        <v>46247.47948295139</v>
+        <v>46247.43952728009</v>
       </c>
       <c r="K590" s="2" t="n">
         <v>46251</v>
@@ -46201,7 +46211,7 @@
     </row>
     <row r="591">
       <c r="A591" s="1" t="n">
-        <v>82337</v>
+        <v>82336</v>
       </c>
       <c r="B591" s="1" t="inlineStr">
         <is>
@@ -46215,45 +46225,53 @@
       </c>
       <c r="D591" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E591" s="1" t="inlineStr">
         <is>
-          <t>Bom diaCriar a senha da prefeitura Nova Gissonline, para o cliente 5276 ESS IND E COM, prefeitura de Hortolândia. no aguardo</t>
+          <t>Bom dia,A empresa 1065 - MARTINICA COMERCIAL LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F591" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G591" s="1" t="n"/>
-      <c r="H591" s="1" t="n"/>
+        <v>1065</v>
+      </c>
+      <c r="G591" s="1" t="inlineStr">
+        <is>
+          <t>MARTINICA COMERCIAL LTDA</t>
+        </is>
+      </c>
+      <c r="H591" s="1" t="inlineStr">
+        <is>
+          <t>Edson Silva</t>
+        </is>
+      </c>
       <c r="I591" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J591" s="2" t="n">
-        <v>46247.48493194445</v>
+        <v>46247.47948295139</v>
       </c>
       <c r="K591" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L591" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M591" s="1" t="inlineStr">
         <is>
-          <t>Suede Gomes</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N591" s="1" t="n"/>
       <c r="O591" s="1" t="n"/>
       <c r="P591" s="1" t="n"/>
       <c r="Q591" s="1" t="inlineStr"/>
-      <c r="R591" s="1" t="n"/>
+      <c r="R591" s="1" t="inlineStr"/>
       <c r="S591" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -46264,7 +46282,7 @@
     </row>
     <row r="592">
       <c r="A592" s="1" t="n">
-        <v>82338</v>
+        <v>82337</v>
       </c>
       <c r="B592" s="1" t="inlineStr">
         <is>
@@ -46278,53 +46296,45 @@
       </c>
       <c r="D592" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E592" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1475 - SUPERMERCADO CAMILÓPOLIS LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom diaCriar a senha da prefeitura Nova Gissonline, para o cliente 5276 ESS IND E COM, prefeitura de Hortolândia. no aguardo</t>
         </is>
       </c>
       <c r="F592" s="1" t="n">
-        <v>1475</v>
-      </c>
-      <c r="G592" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO CAMILÓPOLIS LTDA</t>
-        </is>
-      </c>
-      <c r="H592" s="1" t="inlineStr">
-        <is>
-          <t>Talita Silva</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G592" s="1" t="n"/>
+      <c r="H592" s="1" t="n"/>
       <c r="I592" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J592" s="2" t="n">
-        <v>46247.49555084491</v>
+        <v>46247.48493194445</v>
       </c>
       <c r="K592" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L592" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M592" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Suede Gomes</t>
         </is>
       </c>
       <c r="N592" s="1" t="n"/>
       <c r="O592" s="1" t="n"/>
       <c r="P592" s="1" t="n"/>
       <c r="Q592" s="1" t="inlineStr"/>
-      <c r="R592" s="1" t="inlineStr"/>
+      <c r="R592" s="1" t="n"/>
       <c r="S592" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -46335,7 +46345,7 @@
     </row>
     <row r="593">
       <c r="A593" s="1" t="n">
-        <v>82339</v>
+        <v>82338</v>
       </c>
       <c r="B593" s="1" t="inlineStr">
         <is>
@@ -46354,15 +46364,15 @@
       </c>
       <c r="E593" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1718 - SUPERMERCADO MATRIZ LTDA  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom dia,A empresa 1475 - SUPERMERCADO CAMILÓPOLIS LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F593" s="1" t="n">
-        <v>1718</v>
+        <v>1475</v>
       </c>
       <c r="G593" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERMERCADO MATRIZ LTDA </t>
+          <t>SUPERMERCADO CAMILÓPOLIS LTDA</t>
         </is>
       </c>
       <c r="H593" s="1" t="inlineStr">
@@ -46376,7 +46386,7 @@
         </is>
       </c>
       <c r="J593" s="2" t="n">
-        <v>46247.49647716435</v>
+        <v>46247.49555084491</v>
       </c>
       <c r="K593" s="2" t="n">
         <v>46251</v>
@@ -46406,7 +46416,7 @@
     </row>
     <row r="594">
       <c r="A594" s="1" t="n">
-        <v>82340</v>
+        <v>82339</v>
       </c>
       <c r="B594" s="1" t="inlineStr">
         <is>
@@ -46425,32 +46435,36 @@
       </c>
       <c r="E594" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1871 - COMÉRCIO DE HORTI FRUTTI LEONILDA LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 1718 - SUPERMERCADO MATRIZ LTDA  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F594" s="1" t="n">
-        <v>1871</v>
+        <v>1718</v>
       </c>
       <c r="G594" s="1" t="inlineStr">
         <is>
-          <t>COMÉRCIO DE HORTI FRUTTI LEONILDA LTDA</t>
-        </is>
-      </c>
-      <c r="H594" s="1" t="n"/>
+          <t xml:space="preserve">SUPERMERCADO MATRIZ LTDA </t>
+        </is>
+      </c>
+      <c r="H594" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I594" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J594" s="2" t="n">
-        <v>46247.49783040509</v>
+        <v>46247.49647716435</v>
       </c>
       <c r="K594" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L594" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M594" s="1" t="inlineStr">
@@ -46462,7 +46476,7 @@
       <c r="O594" s="1" t="n"/>
       <c r="P594" s="1" t="n"/>
       <c r="Q594" s="1" t="inlineStr"/>
-      <c r="R594" s="1" t="n"/>
+      <c r="R594" s="1" t="inlineStr"/>
       <c r="S594" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -46473,7 +46487,7 @@
     </row>
     <row r="595">
       <c r="A595" s="1" t="n">
-        <v>82341</v>
+        <v>82340</v>
       </c>
       <c r="B595" s="1" t="inlineStr">
         <is>
@@ -46492,36 +46506,32 @@
       </c>
       <c r="E595" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1927 - ABS DISTRIBUIDORA LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 1871 - COMÉRCIO DE HORTI FRUTTI LEONILDA LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F595" s="1" t="n">
-        <v>1927</v>
+        <v>1871</v>
       </c>
       <c r="G595" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABS DISTRIBUIDORA LTDA </t>
-        </is>
-      </c>
-      <c r="H595" s="1" t="inlineStr">
-        <is>
-          <t>Edson Silva</t>
-        </is>
-      </c>
+          <t>COMÉRCIO DE HORTI FRUTTI LEONILDA LTDA</t>
+        </is>
+      </c>
+      <c r="H595" s="1" t="n"/>
       <c r="I595" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J595" s="2" t="n">
-        <v>46247.49867638889</v>
+        <v>46247.49783040509</v>
       </c>
       <c r="K595" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L595" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M595" s="1" t="inlineStr">
@@ -46533,7 +46543,7 @@
       <c r="O595" s="1" t="n"/>
       <c r="P595" s="1" t="n"/>
       <c r="Q595" s="1" t="inlineStr"/>
-      <c r="R595" s="1" t="inlineStr"/>
+      <c r="R595" s="1" t="n"/>
       <c r="S595" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -46544,7 +46554,7 @@
     </row>
     <row r="596">
       <c r="A596" s="1" t="n">
-        <v>82342</v>
+        <v>82341</v>
       </c>
       <c r="B596" s="1" t="inlineStr">
         <is>
@@ -46563,20 +46573,20 @@
       </c>
       <c r="E596" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ola, boa tardepoderia me ajudar a solucionar o problema desta loja.para encerrar a competência é solicitado "utilize nova versão" no GISSONLINE, poderiam escriturar  na nova prefeitura/novo site do GISSONLINE? </t>
+          <t>Bom dia,A empresa 1927 - ABS DISTRIBUIDORA LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F596" s="1" t="n">
-        <v>3565</v>
+        <v>1927</v>
       </c>
       <c r="G596" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (F9)</t>
+          <t xml:space="preserve">ABS DISTRIBUIDORA LTDA </t>
         </is>
       </c>
       <c r="H596" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I596" s="1" t="inlineStr">
@@ -46585,10 +46595,10 @@
         </is>
       </c>
       <c r="J596" s="2" t="n">
-        <v>46247.49874748843</v>
+        <v>46247.49867638889</v>
       </c>
       <c r="K596" s="2" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="L596" s="1" t="inlineStr">
         <is>
@@ -46597,7 +46607,7 @@
       </c>
       <c r="M596" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N596" s="1" t="n"/>
@@ -46615,7 +46625,7 @@
     </row>
     <row r="597">
       <c r="A597" s="1" t="n">
-        <v>82343</v>
+        <v>82342</v>
       </c>
       <c r="B597" s="1" t="inlineStr">
         <is>
@@ -46634,20 +46644,20 @@
       </c>
       <c r="E597" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 2284 - EMPORIUM SAN GENNARO DO ABC EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t xml:space="preserve">Ola, boa tardepoderia me ajudar a solucionar o problema desta loja.para encerrar a competência é solicitado "utilize nova versão" no GISSONLINE, poderiam escriturar  na nova prefeitura/novo site do GISSONLINE? </t>
         </is>
       </c>
       <c r="F597" s="1" t="n">
-        <v>2284</v>
+        <v>3565</v>
       </c>
       <c r="G597" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIUM SAN GENNARO DO ABC EIRELI </t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (F9)</t>
         </is>
       </c>
       <c r="H597" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I597" s="1" t="inlineStr">
@@ -46656,10 +46666,10 @@
         </is>
       </c>
       <c r="J597" s="2" t="n">
-        <v>46247.49937804398</v>
+        <v>46247.49874748843</v>
       </c>
       <c r="K597" s="2" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="L597" s="1" t="inlineStr">
         <is>
@@ -46668,7 +46678,7 @@
       </c>
       <c r="M597" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N597" s="1" t="n"/>
@@ -46686,7 +46696,7 @@
     </row>
     <row r="598">
       <c r="A598" s="1" t="n">
-        <v>82344</v>
+        <v>82343</v>
       </c>
       <c r="B598" s="1" t="inlineStr">
         <is>
@@ -46705,15 +46715,15 @@
       </c>
       <c r="E598" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 2684 - MIKAIL APOIO ADMINISTRATIVO LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 2284 - EMPORIUM SAN GENNARO DO ABC EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F598" s="1" t="n">
-        <v>2684</v>
+        <v>2284</v>
       </c>
       <c r="G598" s="1" t="inlineStr">
         <is>
-          <t>MIKAIL APOIO ADMINISTRATIVO LTDA</t>
+          <t xml:space="preserve">EMPORIUM SAN GENNARO DO ABC EIRELI </t>
         </is>
       </c>
       <c r="H598" s="1" t="inlineStr">
@@ -46727,7 +46737,7 @@
         </is>
       </c>
       <c r="J598" s="2" t="n">
-        <v>46247.49982866898</v>
+        <v>46247.49937804398</v>
       </c>
       <c r="K598" s="2" t="n">
         <v>46251</v>
@@ -46757,7 +46767,7 @@
     </row>
     <row r="599">
       <c r="A599" s="1" t="n">
-        <v>82345</v>
+        <v>82344</v>
       </c>
       <c r="B599" s="1" t="inlineStr">
         <is>
@@ -46776,20 +46786,20 @@
       </c>
       <c r="E599" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 3937 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 2684 - MIKAIL APOIO ADMINISTRATIVO LTDA está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F599" s="1" t="n">
-        <v>3937</v>
+        <v>2684</v>
       </c>
       <c r="G599" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)</t>
+          <t>MIKAIL APOIO ADMINISTRATIVO LTDA</t>
         </is>
       </c>
       <c r="H599" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I599" s="1" t="inlineStr">
@@ -46798,7 +46808,7 @@
         </is>
       </c>
       <c r="J599" s="2" t="n">
-        <v>46247.50216585648</v>
+        <v>46247.49982866898</v>
       </c>
       <c r="K599" s="2" t="n">
         <v>46251</v>
@@ -46828,7 +46838,7 @@
     </row>
     <row r="600">
       <c r="A600" s="1" t="n">
-        <v>82347</v>
+        <v>82345</v>
       </c>
       <c r="B600" s="1" t="inlineStr">
         <is>
@@ -46847,15 +46857,15 @@
       </c>
       <c r="E600" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4011 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 3937 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F600" s="1" t="n">
-        <v>4011</v>
+        <v>3937</v>
       </c>
       <c r="G600" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)</t>
         </is>
       </c>
       <c r="H600" s="1" t="inlineStr">
@@ -46869,7 +46879,7 @@
         </is>
       </c>
       <c r="J600" s="2" t="n">
-        <v>46247.50307665509</v>
+        <v>46247.50216585648</v>
       </c>
       <c r="K600" s="2" t="n">
         <v>46251</v>
@@ -46899,7 +46909,7 @@
     </row>
     <row r="601">
       <c r="A601" s="1" t="n">
-        <v>82348</v>
+        <v>82347</v>
       </c>
       <c r="B601" s="1" t="inlineStr">
         <is>
@@ -46918,15 +46928,15 @@
       </c>
       <c r="E601" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4013 - Cucinare Pro Alimentaçao Ltda (FL 51)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4011 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F601" s="1" t="n">
-        <v>4013</v>
+        <v>4011</v>
       </c>
       <c r="G601" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49)</t>
         </is>
       </c>
       <c r="H601" s="1" t="inlineStr">
@@ -46940,7 +46950,7 @@
         </is>
       </c>
       <c r="J601" s="2" t="n">
-        <v>46247.50329737268</v>
+        <v>46247.50307665509</v>
       </c>
       <c r="K601" s="2" t="n">
         <v>46251</v>
@@ -46970,7 +46980,7 @@
     </row>
     <row r="602">
       <c r="A602" s="1" t="n">
-        <v>82350</v>
+        <v>82348</v>
       </c>
       <c r="B602" s="1" t="inlineStr">
         <is>
@@ -46989,32 +46999,36 @@
       </c>
       <c r="E602" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4572 - YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4013 - Cucinare Pro Alimentaçao Ltda (FL 51)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F602" s="1" t="n">
-        <v>4572</v>
+        <v>4013</v>
       </c>
       <c r="G602" s="1" t="inlineStr">
         <is>
-          <t>YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI</t>
-        </is>
-      </c>
-      <c r="H602" s="1" t="n"/>
+          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
+        </is>
+      </c>
+      <c r="H602" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I602" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J602" s="2" t="n">
-        <v>46247.51033761574</v>
+        <v>46247.50329737268</v>
       </c>
       <c r="K602" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L602" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M602" s="1" t="inlineStr">
@@ -47026,7 +47040,7 @@
       <c r="O602" s="1" t="n"/>
       <c r="P602" s="1" t="n"/>
       <c r="Q602" s="1" t="inlineStr"/>
-      <c r="R602" s="1" t="n"/>
+      <c r="R602" s="1" t="inlineStr"/>
       <c r="S602" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -47037,7 +47051,7 @@
     </row>
     <row r="603">
       <c r="A603" s="1" t="n">
-        <v>82351</v>
+        <v>82350</v>
       </c>
       <c r="B603" s="1" t="inlineStr">
         <is>
@@ -47056,36 +47070,32 @@
       </c>
       <c r="E603" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4892 - FLV 7 RESTAURANTES LTDA (FILIAL 14)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4572 - YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F603" s="1" t="n">
-        <v>4892</v>
+        <v>4572</v>
       </c>
       <c r="G603" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 14)</t>
-        </is>
-      </c>
-      <c r="H603" s="1" t="inlineStr">
-        <is>
-          <t>Talita Silva</t>
-        </is>
-      </c>
+          <t>YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI</t>
+        </is>
+      </c>
+      <c r="H603" s="1" t="n"/>
       <c r="I603" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J603" s="2" t="n">
-        <v>46247.51152873843</v>
+        <v>46247.51033761574</v>
       </c>
       <c r="K603" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L603" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M603" s="1" t="inlineStr">
@@ -47097,7 +47107,7 @@
       <c r="O603" s="1" t="n"/>
       <c r="P603" s="1" t="n"/>
       <c r="Q603" s="1" t="inlineStr"/>
-      <c r="R603" s="1" t="inlineStr"/>
+      <c r="R603" s="1" t="n"/>
       <c r="S603" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -47108,7 +47118,7 @@
     </row>
     <row r="604">
       <c r="A604" s="1" t="n">
-        <v>82352</v>
+        <v>82351</v>
       </c>
       <c r="B604" s="1" t="inlineStr">
         <is>
@@ -47127,15 +47137,15 @@
       </c>
       <c r="E604" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5152 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4892 - FLV 7 RESTAURANTES LTDA (FILIAL 14)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F604" s="1" t="n">
-        <v>5152</v>
+        <v>4892</v>
       </c>
       <c r="G604" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 14)</t>
         </is>
       </c>
       <c r="H604" s="1" t="inlineStr">
@@ -47149,7 +47159,7 @@
         </is>
       </c>
       <c r="J604" s="2" t="n">
-        <v>46247.512321875</v>
+        <v>46247.51152873843</v>
       </c>
       <c r="K604" s="2" t="n">
         <v>46251</v>
@@ -47179,7 +47189,7 @@
     </row>
     <row r="605">
       <c r="A605" s="1" t="n">
-        <v>82353</v>
+        <v>82352</v>
       </c>
       <c r="B605" s="1" t="inlineStr">
         <is>
@@ -47198,15 +47208,15 @@
       </c>
       <c r="E605" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5270 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5152 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F605" s="1" t="n">
-        <v>5270</v>
+        <v>5152</v>
       </c>
       <c r="G605" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)</t>
         </is>
       </c>
       <c r="H605" s="1" t="inlineStr">
@@ -47220,7 +47230,7 @@
         </is>
       </c>
       <c r="J605" s="2" t="n">
-        <v>46247.51311061343</v>
+        <v>46247.512321875</v>
       </c>
       <c r="K605" s="2" t="n">
         <v>46251</v>
@@ -47250,7 +47260,7 @@
     </row>
     <row r="606">
       <c r="A606" s="1" t="n">
-        <v>82354</v>
+        <v>82353</v>
       </c>
       <c r="B606" s="1" t="inlineStr">
         <is>
@@ -47269,15 +47279,15 @@
       </c>
       <c r="E606" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5271 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5270 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F606" s="1" t="n">
-        <v>5271</v>
+        <v>5270</v>
       </c>
       <c r="G606" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)</t>
         </is>
       </c>
       <c r="H606" s="1" t="inlineStr">
@@ -47291,7 +47301,7 @@
         </is>
       </c>
       <c r="J606" s="2" t="n">
-        <v>46247.51352311343</v>
+        <v>46247.51311061343</v>
       </c>
       <c r="K606" s="2" t="n">
         <v>46251</v>
@@ -47321,7 +47331,7 @@
     </row>
     <row r="607">
       <c r="A607" s="1" t="n">
-        <v>82355</v>
+        <v>82354</v>
       </c>
       <c r="B607" s="1" t="inlineStr">
         <is>
@@ -47340,15 +47350,15 @@
       </c>
       <c r="E607" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5272 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5271 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F607" s="1" t="n">
-        <v>5272</v>
+        <v>5271</v>
       </c>
       <c r="G607" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)</t>
         </is>
       </c>
       <c r="H607" s="1" t="inlineStr">
@@ -47362,7 +47372,7 @@
         </is>
       </c>
       <c r="J607" s="2" t="n">
-        <v>46247.51430975695</v>
+        <v>46247.51352311343</v>
       </c>
       <c r="K607" s="2" t="n">
         <v>46251</v>
@@ -47392,7 +47402,7 @@
     </row>
     <row r="608">
       <c r="A608" s="1" t="n">
-        <v>82357</v>
+        <v>82355</v>
       </c>
       <c r="B608" s="1" t="inlineStr">
         <is>
@@ -47411,15 +47421,15 @@
       </c>
       <c r="E608" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5367 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom dia,A empresa 5272 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F608" s="1" t="n">
-        <v>5367</v>
+        <v>5272</v>
       </c>
       <c r="G608" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)</t>
         </is>
       </c>
       <c r="H608" s="1" t="inlineStr">
@@ -47433,7 +47443,7 @@
         </is>
       </c>
       <c r="J608" s="2" t="n">
-        <v>46247.51567353009</v>
+        <v>46247.51430975695</v>
       </c>
       <c r="K608" s="2" t="n">
         <v>46251</v>
@@ -47463,7 +47473,7 @@
     </row>
     <row r="609">
       <c r="A609" s="1" t="n">
-        <v>82358</v>
+        <v>82357</v>
       </c>
       <c r="B609" s="1" t="inlineStr">
         <is>
@@ -47482,15 +47492,15 @@
       </c>
       <c r="E609" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5368 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5367 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F609" s="1" t="n">
-        <v>5368</v>
+        <v>5367</v>
       </c>
       <c r="G609" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)</t>
         </is>
       </c>
       <c r="H609" s="1" t="inlineStr">
@@ -47504,7 +47514,7 @@
         </is>
       </c>
       <c r="J609" s="2" t="n">
-        <v>46247.51638197916</v>
+        <v>46247.51567353009</v>
       </c>
       <c r="K609" s="2" t="n">
         <v>46251</v>
@@ -47534,59 +47544,67 @@
     </row>
     <row r="610">
       <c r="A610" s="1" t="n">
-        <v>82359</v>
+        <v>82358</v>
       </c>
       <c r="B610" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Contabilista</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C610" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vincular </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D610" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E610" s="1" t="inlineStr">
         <is>
-          <t>A empresa 6521, não estou conseguindo entregar a DESTDA. A empresa está com saida da MG 30/09, porém já está dando este erro.CPF do socio está correto.</t>
+          <t>Bom dia,A empresa 5368 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F610" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G610" s="1" t="n"/>
-      <c r="H610" s="1" t="n"/>
+        <v>5368</v>
+      </c>
+      <c r="G610" s="1" t="inlineStr">
+        <is>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76)</t>
+        </is>
+      </c>
+      <c r="H610" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I610" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J610" s="2" t="n">
-        <v>46247.52414039352</v>
+        <v>46247.51638197916</v>
       </c>
       <c r="K610" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L610" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M610" s="1" t="inlineStr">
         <is>
-          <t>Caroline Nascimento</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N610" s="1" t="n"/>
       <c r="O610" s="1" t="n"/>
       <c r="P610" s="1" t="n"/>
       <c r="Q610" s="1" t="inlineStr"/>
-      <c r="R610" s="1" t="n"/>
+      <c r="R610" s="1" t="inlineStr"/>
       <c r="S610" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -47597,67 +47615,59 @@
     </row>
     <row r="611">
       <c r="A611" s="1" t="n">
-        <v>82362</v>
+        <v>82359</v>
       </c>
       <c r="B611" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração de Contabilista</t>
         </is>
       </c>
       <c r="C611" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Vincular </t>
         </is>
       </c>
       <c r="D611" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E611" s="1" t="inlineStr">
         <is>
-          <t>Não possui login/senha de acesso à prefeitura.</t>
+          <t>A empresa 6521, não estou conseguindo entregar a DESTDA. A empresa está com saida da MG 30/09, porém já está dando este erro.CPF do socio está correto.</t>
         </is>
       </c>
       <c r="F611" s="1" t="n">
-        <v>5150</v>
-      </c>
-      <c r="G611" s="1" t="inlineStr">
-        <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 63)</t>
-        </is>
-      </c>
-      <c r="H611" s="1" t="inlineStr">
-        <is>
-          <t>Talita Silva</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G611" s="1" t="n"/>
+      <c r="H611" s="1" t="n"/>
       <c r="I611" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J611" s="2" t="n">
-        <v>46247.52804065972</v>
+        <v>46247.52414039352</v>
       </c>
       <c r="K611" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L611" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M611" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Caroline Nascimento</t>
         </is>
       </c>
       <c r="N611" s="1" t="n"/>
       <c r="O611" s="1" t="n"/>
       <c r="P611" s="1" t="n"/>
       <c r="Q611" s="1" t="inlineStr"/>
-      <c r="R611" s="1" t="inlineStr"/>
+      <c r="R611" s="1" t="n"/>
       <c r="S611" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -47668,7 +47678,7 @@
     </row>
     <row r="612">
       <c r="A612" s="1" t="n">
-        <v>82363</v>
+        <v>82362</v>
       </c>
       <c r="B612" s="1" t="inlineStr">
         <is>
@@ -47691,11 +47701,11 @@
         </is>
       </c>
       <c r="F612" s="1" t="n">
-        <v>5153</v>
+        <v>5150</v>
       </c>
       <c r="G612" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 63)</t>
         </is>
       </c>
       <c r="H612" s="1" t="inlineStr">
@@ -47709,7 +47719,7 @@
         </is>
       </c>
       <c r="J612" s="2" t="n">
-        <v>46247.53012986111</v>
+        <v>46247.52804065972</v>
       </c>
       <c r="K612" s="2" t="n">
         <v>46251</v>
@@ -47739,7 +47749,7 @@
     </row>
     <row r="613">
       <c r="A613" s="1" t="n">
-        <v>82364</v>
+        <v>82363</v>
       </c>
       <c r="B613" s="1" t="inlineStr">
         <is>
@@ -47758,40 +47768,48 @@
       </c>
       <c r="E613" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, precisamos da senha da prefeitura da empresa 5713 - S&amp;S supermercados. Solicitada há vários meses por e-mail.Fico no aguardo. Obrigada!</t>
+          <t>Não possui login/senha de acesso à prefeitura.</t>
         </is>
       </c>
       <c r="F613" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G613" s="1" t="n"/>
-      <c r="H613" s="1" t="n"/>
+        <v>5153</v>
+      </c>
+      <c r="G613" s="1" t="inlineStr">
+        <is>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (66)</t>
+        </is>
+      </c>
+      <c r="H613" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I613" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J613" s="2" t="n">
-        <v>46247.55619429398</v>
+        <v>46247.53012986111</v>
       </c>
       <c r="K613" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L613" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M613" s="1" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N613" s="1" t="n"/>
       <c r="O613" s="1" t="n"/>
       <c r="P613" s="1" t="n"/>
       <c r="Q613" s="1" t="inlineStr"/>
-      <c r="R613" s="1" t="n"/>
+      <c r="R613" s="1" t="inlineStr"/>
       <c r="S613" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -47802,67 +47820,59 @@
     </row>
     <row r="614">
       <c r="A614" s="1" t="n">
-        <v>82366</v>
+        <v>82364</v>
       </c>
       <c r="B614" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C614" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Novo </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D614" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E614" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Favor cadastrar o cliente da imagem em anexo sob Código 9076 no MG Controle e vincular ao grupo da empresa 6076-Film Facil.Obrigado.</t>
+          <t>Boa tarde!Por gentileza, precisamos da senha da prefeitura da empresa 5713 - S&amp;S supermercados. Solicitada há vários meses por e-mail.Fico no aguardo. Obrigada!</t>
         </is>
       </c>
       <c r="F614" s="1" t="n">
-        <v>6976</v>
-      </c>
-      <c r="G614" s="1" t="inlineStr">
-        <is>
-          <t>FILM FACIL LTDA</t>
-        </is>
-      </c>
-      <c r="H614" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G614" s="1" t="n"/>
+      <c r="H614" s="1" t="n"/>
       <c r="I614" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J614" s="2" t="n">
-        <v>46247.57558356482</v>
+        <v>46247.55619429398</v>
       </c>
       <c r="K614" s="2" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="L614" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M614" s="1" t="inlineStr">
         <is>
-          <t>Leandro Matos</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="N614" s="1" t="n"/>
       <c r="O614" s="1" t="n"/>
       <c r="P614" s="1" t="n"/>
       <c r="Q614" s="1" t="inlineStr"/>
-      <c r="R614" s="1" t="inlineStr"/>
+      <c r="R614" s="1" t="n"/>
       <c r="S614" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -48075,6 +48085,136 @@
       </c>
       <c r="T617" s="1" t="n"/>
       <c r="U617" s="1" t="inlineStr"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="1" t="n">
+        <v>82412</v>
+      </c>
+      <c r="B618" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C618" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D618" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E618" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia!Por gentileza, Solicito a senha da prefeitura referente a empresa: 6802 - TOME AGROVETERINARIA LTDA. Que não consta no MGC e foi solicitado desde o mês 05/2026.Ficamos no aguardo!!</t>
+        </is>
+      </c>
+      <c r="F618" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G618" s="1" t="n"/>
+      <c r="H618" s="1" t="n"/>
+      <c r="I618" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J618" s="2" t="n">
+        <v>46248.39979934028</v>
+      </c>
+      <c r="K618" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="L618" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M618" s="1" t="inlineStr">
+        <is>
+          <t>Cristina Leite</t>
+        </is>
+      </c>
+      <c r="N618" s="1" t="n"/>
+      <c r="O618" s="1" t="n"/>
+      <c r="P618" s="1" t="n"/>
+      <c r="Q618" s="1" t="inlineStr"/>
+      <c r="R618" s="1" t="n"/>
+      <c r="S618" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T618" s="1" t="n"/>
+      <c r="U618" s="1" t="inlineStr"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="1" t="n">
+        <v>82413</v>
+      </c>
+      <c r="B619" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C619" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D619" s="1" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="E619" s="1" t="inlineStr">
+        <is>
+          <t>Login/senha disponibilizado na MGC está incorreto.</t>
+        </is>
+      </c>
+      <c r="F619" s="1" t="n">
+        <v>5408</v>
+      </c>
+      <c r="G619" s="1" t="inlineStr">
+        <is>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 78)</t>
+        </is>
+      </c>
+      <c r="H619" s="1" t="n"/>
+      <c r="I619" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J619" s="2" t="n">
+        <v>46248.4003153588</v>
+      </c>
+      <c r="K619" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="L619" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M619" s="1" t="inlineStr">
+        <is>
+          <t>Daisa Araujo</t>
+        </is>
+      </c>
+      <c r="N619" s="1" t="n"/>
+      <c r="O619" s="1" t="n"/>
+      <c r="P619" s="1" t="n"/>
+      <c r="Q619" s="1" t="inlineStr"/>
+      <c r="R619" s="1" t="n"/>
+      <c r="S619" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T619" s="1" t="n"/>
+      <c r="U619" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 14:55
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U666" headerRowCount="1">
-  <autoFilter ref="A1:U666"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U667" headerRowCount="1">
+  <autoFilter ref="A1:U667"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U666"/>
+  <dimension ref="A1:U667"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5271,7 +5271,11 @@
           <t>FUNCHAL INDUSTRIA E COMERCIO DE PAPEIS LTDA</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n"/>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>Idna Sousa</t>
+        </is>
+      </c>
       <c r="I58" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -5285,7 +5289,7 @@
       </c>
       <c r="L58" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M58" s="1" t="inlineStr">
@@ -5297,14 +5301,18 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="n"/>
       <c r="Q58" s="1" t="inlineStr"/>
-      <c r="R58" s="1" t="n"/>
+      <c r="R58" s="1" t="inlineStr"/>
       <c r="S58" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T58" s="1" t="n"/>
-      <c r="U58" s="1" t="inlineStr"/>
+      <c r="U58" s="1" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -5338,7 +5346,11 @@
           <t>FUNCHAL INDUSTRIA E COMERCIO DE PAPEIS LTDA</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n"/>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>Idna Sousa</t>
+        </is>
+      </c>
       <c r="I59" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -5352,7 +5364,7 @@
       </c>
       <c r="L59" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M59" s="1" t="inlineStr">
@@ -5364,14 +5376,18 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="n"/>
       <c r="Q59" s="1" t="inlineStr"/>
-      <c r="R59" s="1" t="n"/>
+      <c r="R59" s="1" t="inlineStr"/>
       <c r="S59" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T59" s="1" t="n"/>
-      <c r="U59" s="1" t="inlineStr"/>
+      <c r="U59" s="1" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -48955,7 +48971,7 @@
     </row>
     <row r="631">
       <c r="A631" s="1" t="n">
-        <v>82338</v>
+        <v>82337</v>
       </c>
       <c r="B631" s="1" t="inlineStr">
         <is>
@@ -48969,25 +48985,21 @@
       </c>
       <c r="D631" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E631" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1475 - SUPERMERCADO CAMILÓPOLIS LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom diaCriar a senha da prefeitura Nova Gissonline, para o cliente 5276 ESS IND E COM, prefeitura de Hortolândia. no aguardo</t>
         </is>
       </c>
       <c r="F631" s="1" t="n">
-        <v>1475</v>
-      </c>
-      <c r="G631" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO CAMILÓPOLIS LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G631" s="1" t="n"/>
       <c r="H631" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I631" s="1" t="inlineStr">
@@ -48996,26 +49008,32 @@
         </is>
       </c>
       <c r="J631" s="2" t="n">
-        <v>46247.49555084491</v>
+        <v>46247.48493194445</v>
       </c>
       <c r="K631" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L631" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido</t>
         </is>
       </c>
       <c r="M631" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Suede Gomes</t>
         </is>
       </c>
       <c r="N631" s="1" t="n"/>
       <c r="O631" s="1" t="n"/>
       <c r="P631" s="1" t="n"/>
       <c r="Q631" s="1" t="inlineStr"/>
-      <c r="R631" s="1" t="inlineStr"/>
+      <c r="R631" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde.
+Senha cadastrada no MGC.
+Atenciosamente,</t>
+        </is>
+      </c>
       <c r="S631" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -49026,7 +49044,7 @@
     </row>
     <row r="632">
       <c r="A632" s="1" t="n">
-        <v>82339</v>
+        <v>82338</v>
       </c>
       <c r="B632" s="1" t="inlineStr">
         <is>
@@ -49045,15 +49063,15 @@
       </c>
       <c r="E632" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 1718 - SUPERMERCADO MATRIZ LTDA  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom dia,A empresa 1475 - SUPERMERCADO CAMILÓPOLIS LTDA está solicitando a atualização para uma nova versão no sistema GissOnline. Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F632" s="1" t="n">
-        <v>1718</v>
+        <v>1475</v>
       </c>
       <c r="G632" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERMERCADO MATRIZ LTDA </t>
+          <t>SUPERMERCADO CAMILÓPOLIS LTDA</t>
         </is>
       </c>
       <c r="H632" s="1" t="inlineStr">
@@ -49067,7 +49085,7 @@
         </is>
       </c>
       <c r="J632" s="2" t="n">
-        <v>46247.49647716435</v>
+        <v>46247.49555084491</v>
       </c>
       <c r="K632" s="2" t="n">
         <v>46251</v>
@@ -49097,7 +49115,7 @@
     </row>
     <row r="633">
       <c r="A633" s="1" t="n">
-        <v>82342</v>
+        <v>82339</v>
       </c>
       <c r="B633" s="1" t="inlineStr">
         <is>
@@ -49116,15 +49134,15 @@
       </c>
       <c r="E633" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ola, boa tardepoderia me ajudar a solucionar o problema desta loja.para encerrar a competência é solicitado "utilize nova versão" no GISSONLINE, poderiam escriturar  na nova prefeitura/novo site do GISSONLINE? </t>
+          <t>Bom dia,A empresa 1718 - SUPERMERCADO MATRIZ LTDA  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F633" s="1" t="n">
-        <v>3565</v>
+        <v>1718</v>
       </c>
       <c r="G633" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (F9)</t>
+          <t xml:space="preserve">SUPERMERCADO MATRIZ LTDA </t>
         </is>
       </c>
       <c r="H633" s="1" t="inlineStr">
@@ -49138,10 +49156,10 @@
         </is>
       </c>
       <c r="J633" s="2" t="n">
-        <v>46247.49874748843</v>
+        <v>46247.49647716435</v>
       </c>
       <c r="K633" s="2" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="L633" s="1" t="inlineStr">
         <is>
@@ -49150,7 +49168,7 @@
       </c>
       <c r="M633" s="1" t="inlineStr">
         <is>
-          <t>Francisco Pimenta</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N633" s="1" t="n"/>
@@ -49168,7 +49186,7 @@
     </row>
     <row r="634">
       <c r="A634" s="1" t="n">
-        <v>82345</v>
+        <v>82342</v>
       </c>
       <c r="B634" s="1" t="inlineStr">
         <is>
@@ -49187,15 +49205,15 @@
       </c>
       <c r="E634" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 3937 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t xml:space="preserve">Ola, boa tardepoderia me ajudar a solucionar o problema desta loja.para encerrar a competência é solicitado "utilize nova versão" no GISSONLINE, poderiam escriturar  na nova prefeitura/novo site do GISSONLINE? </t>
         </is>
       </c>
       <c r="F634" s="1" t="n">
-        <v>3937</v>
+        <v>3565</v>
       </c>
       <c r="G634" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (F9)</t>
         </is>
       </c>
       <c r="H634" s="1" t="inlineStr">
@@ -49209,10 +49227,10 @@
         </is>
       </c>
       <c r="J634" s="2" t="n">
-        <v>46247.50216585648</v>
+        <v>46247.49874748843</v>
       </c>
       <c r="K634" s="2" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="L634" s="1" t="inlineStr">
         <is>
@@ -49221,7 +49239,7 @@
       </c>
       <c r="M634" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Francisco Pimenta</t>
         </is>
       </c>
       <c r="N634" s="1" t="n"/>
@@ -49239,7 +49257,7 @@
     </row>
     <row r="635">
       <c r="A635" s="1" t="n">
-        <v>82347</v>
+        <v>82345</v>
       </c>
       <c r="B635" s="1" t="inlineStr">
         <is>
@@ -49258,15 +49276,15 @@
       </c>
       <c r="E635" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4011 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 3937 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F635" s="1" t="n">
-        <v>4011</v>
+        <v>3937</v>
       </c>
       <c r="G635" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 47)</t>
         </is>
       </c>
       <c r="H635" s="1" t="inlineStr">
@@ -49280,7 +49298,7 @@
         </is>
       </c>
       <c r="J635" s="2" t="n">
-        <v>46247.50307665509</v>
+        <v>46247.50216585648</v>
       </c>
       <c r="K635" s="2" t="n">
         <v>46251</v>
@@ -49310,7 +49328,7 @@
     </row>
     <row r="636">
       <c r="A636" s="1" t="n">
-        <v>82348</v>
+        <v>82347</v>
       </c>
       <c r="B636" s="1" t="inlineStr">
         <is>
@@ -49329,15 +49347,15 @@
       </c>
       <c r="E636" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4013 - Cucinare Pro Alimentaçao Ltda (FL 51)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4011 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F636" s="1" t="n">
-        <v>4013</v>
+        <v>4011</v>
       </c>
       <c r="G636" s="1" t="inlineStr">
         <is>
-          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 49)</t>
         </is>
       </c>
       <c r="H636" s="1" t="inlineStr">
@@ -49351,7 +49369,7 @@
         </is>
       </c>
       <c r="J636" s="2" t="n">
-        <v>46247.50329737268</v>
+        <v>46247.50307665509</v>
       </c>
       <c r="K636" s="2" t="n">
         <v>46251</v>
@@ -49381,7 +49399,7 @@
     </row>
     <row r="637">
       <c r="A637" s="1" t="n">
-        <v>82350</v>
+        <v>82348</v>
       </c>
       <c r="B637" s="1" t="inlineStr">
         <is>
@@ -49400,15 +49418,15 @@
       </c>
       <c r="E637" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4572 - YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4013 - Cucinare Pro Alimentaçao Ltda (FL 51)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F637" s="1" t="n">
-        <v>4572</v>
+        <v>4013</v>
       </c>
       <c r="G637" s="1" t="inlineStr">
         <is>
-          <t>YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI</t>
+          <t>Cucinare Pro Alimentaçao Ltda (FL 51)</t>
         </is>
       </c>
       <c r="H637" s="1" t="inlineStr">
@@ -49422,7 +49440,7 @@
         </is>
       </c>
       <c r="J637" s="2" t="n">
-        <v>46247.51033761574</v>
+        <v>46247.50329737268</v>
       </c>
       <c r="K637" s="2" t="n">
         <v>46251</v>
@@ -49452,7 +49470,7 @@
     </row>
     <row r="638">
       <c r="A638" s="1" t="n">
-        <v>82351</v>
+        <v>82350</v>
       </c>
       <c r="B638" s="1" t="inlineStr">
         <is>
@@ -49471,15 +49489,15 @@
       </c>
       <c r="E638" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 4892 - FLV 7 RESTAURANTES LTDA (FILIAL 14)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4572 - YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F638" s="1" t="n">
-        <v>4892</v>
+        <v>4572</v>
       </c>
       <c r="G638" s="1" t="inlineStr">
         <is>
-          <t>FLV 7 RESTAURANTES LTDA (FILIAL 14)</t>
+          <t>YUKO COMÉRCIO DE ALIMENTOS E SERVIÇOS EIRELI</t>
         </is>
       </c>
       <c r="H638" s="1" t="inlineStr">
@@ -49493,7 +49511,7 @@
         </is>
       </c>
       <c r="J638" s="2" t="n">
-        <v>46247.51152873843</v>
+        <v>46247.51033761574</v>
       </c>
       <c r="K638" s="2" t="n">
         <v>46251</v>
@@ -49523,7 +49541,7 @@
     </row>
     <row r="639">
       <c r="A639" s="1" t="n">
-        <v>82352</v>
+        <v>82351</v>
       </c>
       <c r="B639" s="1" t="inlineStr">
         <is>
@@ -49542,15 +49560,15 @@
       </c>
       <c r="E639" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5152 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 4892 - FLV 7 RESTAURANTES LTDA (FILIAL 14)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F639" s="1" t="n">
-        <v>5152</v>
+        <v>4892</v>
       </c>
       <c r="G639" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)</t>
+          <t>FLV 7 RESTAURANTES LTDA (FILIAL 14)</t>
         </is>
       </c>
       <c r="H639" s="1" t="inlineStr">
@@ -49564,7 +49582,7 @@
         </is>
       </c>
       <c r="J639" s="2" t="n">
-        <v>46247.512321875</v>
+        <v>46247.51152873843</v>
       </c>
       <c r="K639" s="2" t="n">
         <v>46251</v>
@@ -49594,7 +49612,7 @@
     </row>
     <row r="640">
       <c r="A640" s="1" t="n">
-        <v>82353</v>
+        <v>82352</v>
       </c>
       <c r="B640" s="1" t="inlineStr">
         <is>
@@ -49613,15 +49631,15 @@
       </c>
       <c r="E640" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5270 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5152 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F640" s="1" t="n">
-        <v>5270</v>
+        <v>5152</v>
       </c>
       <c r="G640" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 65)</t>
         </is>
       </c>
       <c r="H640" s="1" t="inlineStr">
@@ -49635,7 +49653,7 @@
         </is>
       </c>
       <c r="J640" s="2" t="n">
-        <v>46247.51311061343</v>
+        <v>46247.512321875</v>
       </c>
       <c r="K640" s="2" t="n">
         <v>46251</v>
@@ -49665,7 +49683,7 @@
     </row>
     <row r="641">
       <c r="A641" s="1" t="n">
-        <v>82354</v>
+        <v>82353</v>
       </c>
       <c r="B641" s="1" t="inlineStr">
         <is>
@@ -49684,15 +49702,15 @@
       </c>
       <c r="E641" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5271 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5270 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F641" s="1" t="n">
-        <v>5271</v>
+        <v>5270</v>
       </c>
       <c r="G641" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 74)</t>
         </is>
       </c>
       <c r="H641" s="1" t="inlineStr">
@@ -49706,7 +49724,7 @@
         </is>
       </c>
       <c r="J641" s="2" t="n">
-        <v>46247.51352311343</v>
+        <v>46247.51311061343</v>
       </c>
       <c r="K641" s="2" t="n">
         <v>46251</v>
@@ -49736,7 +49754,7 @@
     </row>
     <row r="642">
       <c r="A642" s="1" t="n">
-        <v>82355</v>
+        <v>82354</v>
       </c>
       <c r="B642" s="1" t="inlineStr">
         <is>
@@ -49755,15 +49773,15 @@
       </c>
       <c r="E642" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5272 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5271 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F642" s="1" t="n">
-        <v>5272</v>
+        <v>5271</v>
       </c>
       <c r="G642" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 72)</t>
         </is>
       </c>
       <c r="H642" s="1" t="inlineStr">
@@ -49777,7 +49795,7 @@
         </is>
       </c>
       <c r="J642" s="2" t="n">
-        <v>46247.51430975695</v>
+        <v>46247.51352311343</v>
       </c>
       <c r="K642" s="2" t="n">
         <v>46251</v>
@@ -49807,7 +49825,7 @@
     </row>
     <row r="643">
       <c r="A643" s="1" t="n">
-        <v>82357</v>
+        <v>82355</v>
       </c>
       <c r="B643" s="1" t="inlineStr">
         <is>
@@ -49826,15 +49844,15 @@
       </c>
       <c r="E643" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5367 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
+          <t>Bom dia,A empresa 5272 - CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F643" s="1" t="n">
-        <v>5367</v>
+        <v>5272</v>
       </c>
       <c r="G643" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)</t>
+          <t>CUCINARE PRO ALIMENTAÇÃO LTDA (FILIAL 73)</t>
         </is>
       </c>
       <c r="H643" s="1" t="inlineStr">
@@ -49848,7 +49866,7 @@
         </is>
       </c>
       <c r="J643" s="2" t="n">
-        <v>46247.51567353009</v>
+        <v>46247.51430975695</v>
       </c>
       <c r="K643" s="2" t="n">
         <v>46251</v>
@@ -49878,7 +49896,7 @@
     </row>
     <row r="644">
       <c r="A644" s="1" t="n">
-        <v>82358</v>
+        <v>82357</v>
       </c>
       <c r="B644" s="1" t="inlineStr">
         <is>
@@ -49897,15 +49915,15 @@
       </c>
       <c r="E644" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,A empresa 5368 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
+          <t>Bom dia,A empresa 5367 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)  está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno.</t>
         </is>
       </c>
       <c r="F644" s="1" t="n">
-        <v>5368</v>
+        <v>5367</v>
       </c>
       <c r="G644" s="1" t="inlineStr">
         <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76)</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 75)</t>
         </is>
       </c>
       <c r="H644" s="1" t="inlineStr">
@@ -49919,7 +49937,7 @@
         </is>
       </c>
       <c r="J644" s="2" t="n">
-        <v>46247.51638197916</v>
+        <v>46247.51567353009</v>
       </c>
       <c r="K644" s="2" t="n">
         <v>46251</v>
@@ -49949,35 +49967,39 @@
     </row>
     <row r="645">
       <c r="A645" s="1" t="n">
-        <v>82359</v>
+        <v>82358</v>
       </c>
       <c r="B645" s="1" t="inlineStr">
         <is>
-          <t>Alteração de Contabilista</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C645" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vincular </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D645" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E645" s="1" t="inlineStr">
         <is>
-          <t>A empresa 6521, não estou conseguindo entregar a DESTDA. A empresa está com saida da MG 30/09, porém já está dando este erro.CPF do socio está correto.</t>
+          <t>Bom dia,A empresa 5368 - CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76) está solicitando a atualização para uma nova versão no sistema GissOnline.Agradeço desde já pela atenção e fico no aguardo do retorno</t>
         </is>
       </c>
       <c r="F645" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G645" s="1" t="n"/>
+        <v>5368</v>
+      </c>
+      <c r="G645" s="1" t="inlineStr">
+        <is>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 76)</t>
+        </is>
+      </c>
       <c r="H645" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I645" s="1" t="inlineStr">
@@ -49986,7 +50008,7 @@
         </is>
       </c>
       <c r="J645" s="2" t="n">
-        <v>46247.52414039352</v>
+        <v>46247.51638197916</v>
       </c>
       <c r="K645" s="2" t="n">
         <v>46251</v>
@@ -49998,7 +50020,7 @@
       </c>
       <c r="M645" s="1" t="inlineStr">
         <is>
-          <t>Caroline Nascimento</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N645" s="1" t="n"/>
@@ -50016,39 +50038,35 @@
     </row>
     <row r="646">
       <c r="A646" s="1" t="n">
-        <v>82362</v>
+        <v>82359</v>
       </c>
       <c r="B646" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Alteração de Contabilista</t>
         </is>
       </c>
       <c r="C646" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t xml:space="preserve">Vincular </t>
         </is>
       </c>
       <c r="D646" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E646" s="1" t="inlineStr">
         <is>
-          <t>Não possui login/senha de acesso à prefeitura.</t>
+          <t>A empresa 6521, não estou conseguindo entregar a DESTDA. A empresa está com saida da MG 30/09, porém já está dando este erro.CPF do socio está correto.</t>
         </is>
       </c>
       <c r="F646" s="1" t="n">
-        <v>5150</v>
-      </c>
-      <c r="G646" s="1" t="inlineStr">
-        <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 63)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G646" s="1" t="n"/>
       <c r="H646" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I646" s="1" t="inlineStr">
@@ -50057,7 +50075,7 @@
         </is>
       </c>
       <c r="J646" s="2" t="n">
-        <v>46247.52804065972</v>
+        <v>46247.52414039352</v>
       </c>
       <c r="K646" s="2" t="n">
         <v>46251</v>
@@ -50069,7 +50087,7 @@
       </c>
       <c r="M646" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Caroline Nascimento</t>
         </is>
       </c>
       <c r="N646" s="1" t="n"/>
@@ -50087,7 +50105,7 @@
     </row>
     <row r="647">
       <c r="A647" s="1" t="n">
-        <v>82364</v>
+        <v>82362</v>
       </c>
       <c r="B647" s="1" t="inlineStr">
         <is>
@@ -50106,13 +50124,17 @@
       </c>
       <c r="E647" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por gentileza, precisamos da senha da prefeitura da empresa 5713 - S&amp;S supermercados. Solicitada há vários meses por e-mail.Fico no aguardo. Obrigada!</t>
+          <t>Não possui login/senha de acesso à prefeitura.</t>
         </is>
       </c>
       <c r="F647" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G647" s="1" t="n"/>
+        <v>5150</v>
+      </c>
+      <c r="G647" s="1" t="inlineStr">
+        <is>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 63)</t>
+        </is>
+      </c>
       <c r="H647" s="1" t="inlineStr">
         <is>
           <t>Talita Silva</t>
@@ -50124,7 +50146,7 @@
         </is>
       </c>
       <c r="J647" s="2" t="n">
-        <v>46247.55619429398</v>
+        <v>46247.52804065972</v>
       </c>
       <c r="K647" s="2" t="n">
         <v>46251</v>
@@ -50136,7 +50158,7 @@
       </c>
       <c r="M647" s="1" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N647" s="1" t="n"/>
@@ -50154,39 +50176,35 @@
     </row>
     <row r="648">
       <c r="A648" s="1" t="n">
-        <v>82368</v>
+        <v>82364</v>
       </c>
       <c r="B648" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião de Sócios</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C648" s="1" t="inlineStr">
         <is>
-          <t>Reeleição de Diretoria</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D648" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E648" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por gentileza, poderia encaminhar a ATA DE ASSEMBLEIA DE ELEIÇÃO / ESTATUTO SOCIAL.</t>
+          <t>Boa tarde!Por gentileza, precisamos da senha da prefeitura da empresa 5713 - S&amp;S supermercados. Solicitada há vários meses por e-mail.Fico no aguardo. Obrigada!</t>
         </is>
       </c>
       <c r="F648" s="1" t="n">
-        <v>2576</v>
-      </c>
-      <c r="G648" s="1" t="inlineStr">
-        <is>
-          <t>P.E Latina Maquinas para Rotulagem Ltda.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G648" s="1" t="n"/>
       <c r="H648" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I648" s="1" t="inlineStr">
@@ -50195,7 +50213,7 @@
         </is>
       </c>
       <c r="J648" s="2" t="n">
-        <v>46247.5870821412</v>
+        <v>46247.55619429398</v>
       </c>
       <c r="K648" s="2" t="n">
         <v>46251</v>
@@ -50207,7 +50225,7 @@
       </c>
       <c r="M648" s="1" t="inlineStr">
         <is>
-          <t>Ana Santana</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="N648" s="1" t="n"/>
@@ -50225,16 +50243,16 @@
     </row>
     <row r="649">
       <c r="A649" s="1" t="n">
-        <v>82395</v>
+        <v>82368</v>
       </c>
       <c r="B649" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento RFB</t>
+          <t>Ata de Reunião de Sócios</t>
         </is>
       </c>
       <c r="C649" s="1" t="inlineStr">
         <is>
-          <t>Simplificado</t>
+          <t>Reeleição de Diretoria</t>
         </is>
       </c>
       <c r="D649" s="1" t="inlineStr">
@@ -50244,20 +50262,20 @@
       </c>
       <c r="E649" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde prezados!!Por gentileza, realizar simulação de parcelamento de débitos na RFB. </t>
+          <t>Boa tarde! Por gentileza, poderia encaminhar a ATA DE ASSEMBLEIA DE ELEIÇÃO / ESTATUTO SOCIAL.</t>
         </is>
       </c>
       <c r="F649" s="1" t="n">
-        <v>6984</v>
+        <v>2576</v>
       </c>
       <c r="G649" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
+          <t>P.E Latina Maquinas para Rotulagem Ltda.</t>
         </is>
       </c>
       <c r="H649" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I649" s="1" t="inlineStr">
@@ -50266,7 +50284,7 @@
         </is>
       </c>
       <c r="J649" s="2" t="n">
-        <v>46247.70127098379</v>
+        <v>46247.5870821412</v>
       </c>
       <c r="K649" s="2" t="n">
         <v>46251</v>
@@ -50278,7 +50296,7 @@
       </c>
       <c r="M649" s="1" t="inlineStr">
         <is>
-          <t>Yasmin Peixoto</t>
+          <t>Ana Santana</t>
         </is>
       </c>
       <c r="N649" s="1" t="n"/>
@@ -50296,39 +50314,39 @@
     </row>
     <row r="650">
       <c r="A650" s="1" t="n">
-        <v>82411</v>
+        <v>82395</v>
       </c>
       <c r="B650" s="1" t="inlineStr">
         <is>
-          <t>Parcelamento Estadual</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C650" s="1" t="inlineStr">
         <is>
-          <t>ICMS</t>
+          <t>Simplificado</t>
         </is>
       </c>
       <c r="D650" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E650" s="1" t="inlineStr">
         <is>
-          <t>Prezados, bom dia!Por favor o cliente está me informando que as guias do parcelamento está sendo enviado para o e-mail do Sr. Vagner, porém a Adriana informou que precisa receber no e-mail: vjalmeida@uol.com.br para que ela consiga programar os pagamentos dos parcelamentos. Podem corrigir e enviar novamente a guia dos parcelamentos que vencem no dia 31/08/2026?</t>
+          <t xml:space="preserve">Boa tarde prezados!!Por gentileza, realizar simulação de parcelamento de débitos na RFB. </t>
         </is>
       </c>
       <c r="F650" s="1" t="n">
-        <v>4319</v>
+        <v>6984</v>
       </c>
       <c r="G650" s="1" t="inlineStr">
         <is>
-          <t>SUPERMERCADO SANTA MARIA LTDA</t>
+          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
         </is>
       </c>
       <c r="H650" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I650" s="1" t="inlineStr">
@@ -50337,39 +50355,29 @@
         </is>
       </c>
       <c r="J650" s="2" t="n">
-        <v>46248.37009363426</v>
+        <v>46247.70127098379</v>
       </c>
       <c r="K650" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L650" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M650" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Yasmin Peixoto</t>
         </is>
       </c>
       <c r="N650" s="1" t="n"/>
       <c r="O650" s="1" t="n"/>
-      <c r="P650" s="2" t="n">
-        <v>46248.46031493055</v>
-      </c>
-      <c r="Q650" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R650" s="1" t="inlineStr">
-        <is>
-          <t>Já está sendo enviado para este e-mail, inclusive com você em cópia, anexo o ultimo e-mail enviado.</t>
-        </is>
-      </c>
+      <c r="P650" s="1" t="n"/>
+      <c r="Q650" s="1" t="inlineStr"/>
+      <c r="R650" s="1" t="inlineStr"/>
       <c r="S650" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T650" s="1" t="n"/>
@@ -50377,35 +50385,39 @@
     </row>
     <row r="651">
       <c r="A651" s="1" t="n">
-        <v>82412</v>
+        <v>82411</v>
       </c>
       <c r="B651" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Parcelamento Estadual</t>
         </is>
       </c>
       <c r="C651" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>ICMS</t>
         </is>
       </c>
       <c r="D651" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E651" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Por gentileza, Solicito a senha da prefeitura referente a empresa: 6802 - TOME AGROVETERINARIA LTDA. Que não consta no MGC e foi solicitado desde o mês 05/2026.Ficamos no aguardo!!</t>
+          <t>Prezados, bom dia!Por favor o cliente está me informando que as guias do parcelamento está sendo enviado para o e-mail do Sr. Vagner, porém a Adriana informou que precisa receber no e-mail: vjalmeida@uol.com.br para que ela consiga programar os pagamentos dos parcelamentos. Podem corrigir e enviar novamente a guia dos parcelamentos que vencem no dia 31/08/2026?</t>
         </is>
       </c>
       <c r="F651" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G651" s="1" t="n"/>
+        <v>4319</v>
+      </c>
+      <c r="G651" s="1" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO SANTA MARIA LTDA</t>
+        </is>
+      </c>
       <c r="H651" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I651" s="1" t="inlineStr">
@@ -50414,29 +50426,39 @@
         </is>
       </c>
       <c r="J651" s="2" t="n">
-        <v>46248.39979934028</v>
+        <v>46248.37009363426</v>
       </c>
       <c r="K651" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L651" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M651" s="1" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Rodrigo Rego</t>
         </is>
       </c>
       <c r="N651" s="1" t="n"/>
       <c r="O651" s="1" t="n"/>
-      <c r="P651" s="1" t="n"/>
-      <c r="Q651" s="1" t="inlineStr"/>
-      <c r="R651" s="1" t="inlineStr"/>
+      <c r="P651" s="2" t="n">
+        <v>46248.46031493055</v>
+      </c>
+      <c r="Q651" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="R651" s="1" t="inlineStr">
+        <is>
+          <t>Já está sendo enviado para este e-mail, inclusive com você em cópia, anexo o ultimo e-mail enviado.</t>
+        </is>
+      </c>
       <c r="S651" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T651" s="1" t="n"/>
@@ -50444,7 +50466,7 @@
     </row>
     <row r="652">
       <c r="A652" s="1" t="n">
-        <v>82413</v>
+        <v>82412</v>
       </c>
       <c r="B652" s="1" t="inlineStr">
         <is>
@@ -50463,20 +50485,16 @@
       </c>
       <c r="E652" s="1" t="inlineStr">
         <is>
-          <t>Login/senha disponibilizado na MGC está incorreto.</t>
+          <t>Bom dia!Por gentileza, Solicito a senha da prefeitura referente a empresa: 6802 - TOME AGROVETERINARIA LTDA. Que não consta no MGC e foi solicitado desde o mês 05/2026.Ficamos no aguardo!!</t>
         </is>
       </c>
       <c r="F652" s="1" t="n">
-        <v>5408</v>
-      </c>
-      <c r="G652" s="1" t="inlineStr">
-        <is>
-          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 78)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G652" s="1" t="n"/>
       <c r="H652" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I652" s="1" t="inlineStr">
@@ -50485,7 +50503,7 @@
         </is>
       </c>
       <c r="J652" s="2" t="n">
-        <v>46248.4003153588</v>
+        <v>46248.39979934028</v>
       </c>
       <c r="K652" s="2" t="n">
         <v>46251</v>
@@ -50497,7 +50515,7 @@
       </c>
       <c r="M652" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="N652" s="1" t="n"/>
@@ -50515,39 +50533,39 @@
     </row>
     <row r="653">
       <c r="A653" s="1" t="n">
-        <v>82421</v>
+        <v>82413</v>
       </c>
       <c r="B653" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C653" s="1" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D653" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E653" s="1" t="inlineStr">
         <is>
-          <t>EMISSÃO DO CLI CONFORME SOLICITAÇÃO VIA E-MAIL</t>
+          <t>Login/senha disponibilizado na MGC está incorreto.</t>
         </is>
       </c>
       <c r="F653" s="1" t="n">
-        <v>4717</v>
+        <v>5408</v>
       </c>
       <c r="G653" s="1" t="inlineStr">
         <is>
-          <t>J K CAFETERIA E CONVENIÊNCIAS LTDA</t>
+          <t>CUCINARE PRO ALIMENTACAO LTDA (FILIAL 78)</t>
         </is>
       </c>
       <c r="H653" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Talita Silva</t>
         </is>
       </c>
       <c r="I653" s="1" t="inlineStr">
@@ -50556,7 +50574,7 @@
         </is>
       </c>
       <c r="J653" s="2" t="n">
-        <v>46248.45310289352</v>
+        <v>46248.4003153588</v>
       </c>
       <c r="K653" s="2" t="n">
         <v>46251</v>
@@ -50568,7 +50586,7 @@
       </c>
       <c r="M653" s="1" t="inlineStr">
         <is>
-          <t>Fernando Sensulini</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N653" s="1" t="n"/>
@@ -50586,7 +50604,7 @@
     </row>
     <row r="654">
       <c r="A654" s="1" t="n">
-        <v>82422</v>
+        <v>82421</v>
       </c>
       <c r="B654" s="1" t="inlineStr">
         <is>
@@ -50605,15 +50623,15 @@
       </c>
       <c r="E654" s="1" t="inlineStr">
         <is>
-          <t>EMISSÃO DO CLI CONFORME SOLITADO VIA E-MAIL</t>
+          <t>EMISSÃO DO CLI CONFORME SOLICITAÇÃO VIA E-MAIL</t>
         </is>
       </c>
       <c r="F654" s="1" t="n">
-        <v>5145</v>
+        <v>4717</v>
       </c>
       <c r="G654" s="1" t="inlineStr">
         <is>
-          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA</t>
+          <t>J K CAFETERIA E CONVENIÊNCIAS LTDA</t>
         </is>
       </c>
       <c r="H654" s="1" t="inlineStr">
@@ -50627,7 +50645,7 @@
         </is>
       </c>
       <c r="J654" s="2" t="n">
-        <v>46248.45380443287</v>
+        <v>46248.45310289352</v>
       </c>
       <c r="K654" s="2" t="n">
         <v>46251</v>
@@ -50657,7 +50675,7 @@
     </row>
     <row r="655">
       <c r="A655" s="1" t="n">
-        <v>82423</v>
+        <v>82422</v>
       </c>
       <c r="B655" s="1" t="inlineStr">
         <is>
@@ -50680,11 +50698,11 @@
         </is>
       </c>
       <c r="F655" s="1" t="n">
-        <v>5686</v>
+        <v>5145</v>
       </c>
       <c r="G655" s="1" t="inlineStr">
         <is>
-          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA (FILIAL 01)</t>
+          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA</t>
         </is>
       </c>
       <c r="H655" s="1" t="inlineStr">
@@ -50698,7 +50716,7 @@
         </is>
       </c>
       <c r="J655" s="2" t="n">
-        <v>46248.45420443287</v>
+        <v>46248.45380443287</v>
       </c>
       <c r="K655" s="2" t="n">
         <v>46251</v>
@@ -50728,7 +50746,7 @@
     </row>
     <row r="656">
       <c r="A656" s="1" t="n">
-        <v>82424</v>
+        <v>82423</v>
       </c>
       <c r="B656" s="1" t="inlineStr">
         <is>
@@ -50751,11 +50769,11 @@
         </is>
       </c>
       <c r="F656" s="1" t="n">
-        <v>5765</v>
+        <v>5686</v>
       </c>
       <c r="G656" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">4R Alimentos e Conveniencias LTDA </t>
+          <t>JK BURITI CAFETERIA E CONVENIENCIAS LTDA (FILIAL 01)</t>
         </is>
       </c>
       <c r="H656" s="1" t="inlineStr">
@@ -50769,7 +50787,7 @@
         </is>
       </c>
       <c r="J656" s="2" t="n">
-        <v>46248.4545744213</v>
+        <v>46248.45420443287</v>
       </c>
       <c r="K656" s="2" t="n">
         <v>46251</v>
@@ -50799,39 +50817,39 @@
     </row>
     <row r="657">
       <c r="A657" s="1" t="n">
-        <v>82426</v>
+        <v>82424</v>
       </c>
       <c r="B657" s="1" t="inlineStr">
         <is>
-          <t>Notificação</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C657" s="1" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Outro</t>
         </is>
       </c>
       <c r="D657" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E657" s="1" t="inlineStr">
         <is>
-          <t>Bom dia.Nosso cliente Grupo Paraná Guarulhos recebeu uma carta de Execução Fiscal. Segundo o histórico se referia a um débito da empresa que agora está sendo cobrado no CPF do sócio.Preciso de apoio para identificar o ocorrido e como regularizar.obrigado</t>
+          <t>EMISSÃO DO CLI CONFORME SOLITADO VIA E-MAIL</t>
         </is>
       </c>
       <c r="F657" s="1" t="n">
-        <v>2681</v>
+        <v>5765</v>
       </c>
       <c r="G657" s="1" t="inlineStr">
         <is>
-          <t>COMÉRCIO DE ALIMENTOS ALVES E FARIAS LTDA</t>
+          <t xml:space="preserve">4R Alimentos e Conveniencias LTDA </t>
         </is>
       </c>
       <c r="H657" s="1" t="inlineStr">
         <is>
-          <t>Ellen Leite</t>
+          <t>Bianca Ribeiro</t>
         </is>
       </c>
       <c r="I657" s="1" t="inlineStr">
@@ -50840,7 +50858,7 @@
         </is>
       </c>
       <c r="J657" s="2" t="n">
-        <v>46248.46228961806</v>
+        <v>46248.4545744213</v>
       </c>
       <c r="K657" s="2" t="n">
         <v>46251</v>
@@ -50852,7 +50870,7 @@
       </c>
       <c r="M657" s="1" t="inlineStr">
         <is>
-          <t>Daniel Oliveira</t>
+          <t>Fernando Sensulini</t>
         </is>
       </c>
       <c r="N657" s="1" t="n"/>
@@ -50870,35 +50888,39 @@
     </row>
     <row r="658">
       <c r="A658" s="1" t="n">
-        <v>82428</v>
+        <v>82426</v>
       </c>
       <c r="B658" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Notificação</t>
         </is>
       </c>
       <c r="C658" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D658" s="1" t="inlineStr">
         <is>
-          <t>SANTOS - ADM</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="E658" s="1" t="inlineStr">
         <is>
-          <t>Teria alguma previsão da inscrição municipal da empresa  6994 - Unirelos Logistica , pois cliente precisa emitir nota e está me cobrando</t>
+          <t>Bom dia.Nosso cliente Grupo Paraná Guarulhos recebeu uma carta de Execução Fiscal. Segundo o histórico se referia a um débito da empresa que agora está sendo cobrado no CPF do sócio.Preciso de apoio para identificar o ocorrido e como regularizar.obrigado</t>
         </is>
       </c>
       <c r="F658" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G658" s="1" t="n"/>
+        <v>2681</v>
+      </c>
+      <c r="G658" s="1" t="inlineStr">
+        <is>
+          <t>COMÉRCIO DE ALIMENTOS ALVES E FARIAS LTDA</t>
+        </is>
+      </c>
       <c r="H658" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I658" s="1" t="inlineStr">
@@ -50907,39 +50929,29 @@
         </is>
       </c>
       <c r="J658" s="2" t="n">
-        <v>46248.46819579861</v>
+        <v>46248.46228961806</v>
       </c>
       <c r="K658" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L658" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M658" s="1" t="inlineStr">
         <is>
-          <t>Lidia Tavares</t>
+          <t>Daniel Oliveira</t>
         </is>
       </c>
       <c r="N658" s="1" t="n"/>
       <c r="O658" s="1" t="n"/>
-      <c r="P658" s="2" t="n">
-        <v>46248.48863896991</v>
-      </c>
-      <c r="Q658" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R658" s="1" t="inlineStr">
-        <is>
-          <t>Possui cadastro e o cliente foi informado desde 28/07 (e-mail anexo). Acesso a nota fiscal é com certificado digital.</t>
-        </is>
-      </c>
+      <c r="P658" s="1" t="n"/>
+      <c r="Q658" s="1" t="inlineStr"/>
+      <c r="R658" s="1" t="inlineStr"/>
       <c r="S658" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T658" s="1" t="n"/>
@@ -50947,39 +50959,35 @@
     </row>
     <row r="659">
       <c r="A659" s="1" t="n">
-        <v>82429</v>
+        <v>82428</v>
       </c>
       <c r="B659" s="1" t="inlineStr">
         <is>
-          <t>Cadastro de Cliente</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C659" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alteração </t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D659" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>SANTOS - ADM</t>
         </is>
       </c>
       <c r="E659" s="1" t="inlineStr">
         <is>
-          <t>Conforme e-mail enviado em 14/08, o grupo Promotora GYN (6962 / 6963) será no Lucro presumido</t>
+          <t>Teria alguma previsão da inscrição municipal da empresa  6994 - Unirelos Logistica , pois cliente precisa emitir nota e está me cobrando</t>
         </is>
       </c>
       <c r="F659" s="1" t="n">
-        <v>6962</v>
-      </c>
-      <c r="G659" s="1" t="inlineStr">
-        <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G659" s="1" t="n"/>
       <c r="H659" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I659" s="1" t="inlineStr">
@@ -50988,29 +50996,39 @@
         </is>
       </c>
       <c r="J659" s="2" t="n">
-        <v>46248.46862962963</v>
+        <v>46248.46819579861</v>
       </c>
       <c r="K659" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L659" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M659" s="1" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Lidia Tavares</t>
         </is>
       </c>
       <c r="N659" s="1" t="n"/>
       <c r="O659" s="1" t="n"/>
-      <c r="P659" s="1" t="n"/>
-      <c r="Q659" s="1" t="inlineStr"/>
-      <c r="R659" s="1" t="inlineStr"/>
+      <c r="P659" s="2" t="n">
+        <v>46248.48863896991</v>
+      </c>
+      <c r="Q659" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="R659" s="1" t="inlineStr">
+        <is>
+          <t>Possui cadastro e o cliente foi informado desde 28/07 (e-mail anexo). Acesso a nota fiscal é com certificado digital.</t>
+        </is>
+      </c>
       <c r="S659" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T659" s="1" t="n"/>
@@ -51018,44 +51036,48 @@
     </row>
     <row r="660">
       <c r="A660" s="1" t="n">
-        <v>82430</v>
+        <v>82429</v>
       </c>
       <c r="B660" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Cadastro de Cliente</t>
         </is>
       </c>
       <c r="C660" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t xml:space="preserve">Alteração </t>
         </is>
       </c>
       <c r="D660" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E660" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia!Segue checklist atualizado da empresa 7007 - SANTOS&amp;DIAN Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>Conforme e-mail enviado em 14/08, o grupo Promotora GYN (6962 / 6963) será no Lucro presumido</t>
         </is>
       </c>
       <c r="F660" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G660" s="1" t="n"/>
+        <v>6962</v>
+      </c>
+      <c r="G660" s="1" t="inlineStr">
+        <is>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+        </is>
+      </c>
       <c r="H660" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I660" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J660" s="2" t="n">
-        <v>46248.47311612269</v>
+        <v>46248.46862962963</v>
       </c>
       <c r="K660" s="2" t="n">
         <v>46251</v>
@@ -51067,7 +51089,7 @@
       </c>
       <c r="M660" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="N660" s="1" t="n"/>
@@ -51085,48 +51107,44 @@
     </row>
     <row r="661">
       <c r="A661" s="1" t="n">
-        <v>82440</v>
+        <v>82430</v>
       </c>
       <c r="B661" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C661" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D661" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E661" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde,Não estou conseguindo acessar o portal da prefeitura com os dados salvos em Senhas/Registros dos clientes. Poderiam me ajudar, por favor.Grato!</t>
+          <t xml:space="preserve">Bom dia!Segue checklist atualizado da empresa 7007 - SANTOS&amp;DIAN Itens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F661" s="1" t="n">
-        <v>2825</v>
-      </c>
-      <c r="G661" s="1" t="inlineStr">
-        <is>
-          <t>J MATERIAIS DE CONSTRUÇÃO LTDA</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G661" s="1" t="n"/>
       <c r="H661" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I661" s="1" t="inlineStr">
         <is>
-          <t>PARALEGAL</t>
+          <t>PL - AUDITORIA</t>
         </is>
       </c>
       <c r="J661" s="2" t="n">
-        <v>46248.52663244213</v>
+        <v>46248.47311612269</v>
       </c>
       <c r="K661" s="2" t="n">
         <v>46251</v>
@@ -51138,7 +51156,7 @@
       </c>
       <c r="M661" s="1" t="inlineStr">
         <is>
-          <t>Edimar Santos</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N661" s="1" t="n"/>
@@ -51156,63 +51174,67 @@
     </row>
     <row r="662">
       <c r="A662" s="1" t="n">
-        <v>82452</v>
+        <v>82440</v>
       </c>
       <c r="B662" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C662" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D662" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E662" s="1" t="inlineStr">
         <is>
-          <t>Alteração contratual do QSA da empresa 2620-ANTOCON GALVANOPLASTIA LTDA.Grupo: AntoconDevido o falecimento da sócia Sra MARIA DA CONCEIÇÃO FONSECA SIQUEIRA, faz-se necessária substituição do QSA para LILIAN APARECIDA SIQUEIRA NEGOCIADO COM O CLIENTE O VALOR 1.800,OO</t>
+          <t>Boa tarde,Não estou conseguindo acessar o portal da prefeitura com os dados salvos em Senhas/Registros dos clientes. Poderiam me ajudar, por favor.Grato!</t>
         </is>
       </c>
       <c r="F662" s="1" t="n">
-        <v>2620</v>
+        <v>2825</v>
       </c>
       <c r="G662" s="1" t="inlineStr">
         <is>
-          <t>ANTOCON GALVANOPLASTIA LTDA</t>
-        </is>
-      </c>
-      <c r="H662" s="1" t="n"/>
+          <t>J MATERIAIS DE CONSTRUÇÃO LTDA</t>
+        </is>
+      </c>
+      <c r="H662" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
       <c r="I662" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J662" s="2" t="n">
-        <v>46248.60492549768</v>
+        <v>46248.52663244213</v>
       </c>
       <c r="K662" s="2" t="n">
-        <v>46276</v>
+        <v>46251</v>
       </c>
       <c r="L662" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M662" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
+          <t>Edimar Santos</t>
         </is>
       </c>
       <c r="N662" s="1" t="n"/>
       <c r="O662" s="1" t="n"/>
       <c r="P662" s="1" t="n"/>
       <c r="Q662" s="1" t="inlineStr"/>
-      <c r="R662" s="1" t="n"/>
+      <c r="R662" s="1" t="inlineStr"/>
       <c r="S662" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -51223,32 +51245,36 @@
     </row>
     <row r="663">
       <c r="A663" s="1" t="n">
-        <v>82466</v>
+        <v>82452</v>
       </c>
       <c r="B663" s="1" t="inlineStr">
         <is>
-          <t>Regularização de Débitos</t>
+          <t>Alteração Contratual</t>
         </is>
       </c>
       <c r="C663" s="1" t="inlineStr">
         <is>
-          <t>PGFN</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D663" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA MASTER</t>
         </is>
       </c>
       <c r="E663" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, o ex-cliente 6477 - Hplast esta questionando um debito dentro do REGULARIZE, porem não estamos conseguindo localizar esse debito, e ao que parece, pertence ao período de trabalho da MG, poderiam verificar do que se retrata essas pendências por favor, estou anexando a única referenciaria que temos</t>
+          <t>Alteração contratual do QSA da empresa 2620-ANTOCON GALVANOPLASTIA LTDA.Grupo: AntoconDevido o falecimento da sócia Sra MARIA DA CONCEIÇÃO FONSECA SIQUEIRA, faz-se necessária substituição do QSA para LILIAN APARECIDA SIQUEIRA NEGOCIADO COM O CLIENTE O VALOR 1.800,OO</t>
         </is>
       </c>
       <c r="F663" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G663" s="1" t="n"/>
+        <v>2620</v>
+      </c>
+      <c r="G663" s="1" t="inlineStr">
+        <is>
+          <t>ANTOCON GALVANOPLASTIA LTDA</t>
+        </is>
+      </c>
       <c r="H663" s="1" t="n"/>
       <c r="I663" s="1" t="inlineStr">
         <is>
@@ -51256,10 +51282,10 @@
         </is>
       </c>
       <c r="J663" s="2" t="n">
-        <v>46248.66333116898</v>
+        <v>46248.60492549768</v>
       </c>
       <c r="K663" s="2" t="n">
-        <v>46251</v>
+        <v>46276</v>
       </c>
       <c r="L663" s="1" t="inlineStr">
         <is>
@@ -51268,7 +51294,7 @@
       </c>
       <c r="M663" s="1" t="inlineStr">
         <is>
-          <t>Gustavo Tonan</t>
+          <t>Raisa Sousa</t>
         </is>
       </c>
       <c r="N663" s="1" t="n"/>
@@ -51286,67 +51312,59 @@
     </row>
     <row r="664">
       <c r="A664" s="1" t="n">
-        <v>82491</v>
+        <v>82466</v>
       </c>
       <c r="B664" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Regularização de Débitos</t>
         </is>
       </c>
       <c r="C664" s="1" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>PGFN</t>
         </is>
       </c>
       <c r="D664" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="E664" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, Ellen.Conforme conversado, por gentileza realizar a alteração do período de apuração de 31/03/2026 para 31/07/2026.</t>
+          <t>Boa tarde, o ex-cliente 6477 - Hplast esta questionando um debito dentro do REGULARIZE, porem não estamos conseguindo localizar esse debito, e ao que parece, pertence ao período de trabalho da MG, poderiam verificar do que se retrata essas pendências por favor, estou anexando a única referenciaria que temos</t>
         </is>
       </c>
       <c r="F664" s="1" t="n">
-        <v>861</v>
-      </c>
-      <c r="G664" s="1" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO CASTELO DA SERRA LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H664" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G664" s="1" t="n"/>
+      <c r="H664" s="1" t="n"/>
       <c r="I664" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J664" s="2" t="n">
-        <v>46248.7069753125</v>
+        <v>46248.66333116898</v>
       </c>
       <c r="K664" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="L664" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M664" s="1" t="inlineStr">
         <is>
-          <t>Karina Fonseca</t>
+          <t>Gustavo Tonan</t>
         </is>
       </c>
       <c r="N664" s="1" t="n"/>
       <c r="O664" s="1" t="n"/>
       <c r="P664" s="1" t="n"/>
       <c r="Q664" s="1" t="inlineStr"/>
-      <c r="R664" s="1" t="inlineStr"/>
+      <c r="R664" s="1" t="n"/>
       <c r="S664" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -51357,39 +51375,39 @@
     </row>
     <row r="665">
       <c r="A665" s="1" t="n">
-        <v>82498</v>
+        <v>82491</v>
       </c>
       <c r="B665" s="1" t="inlineStr">
         <is>
-          <t>Senha</t>
+          <t>Regularização</t>
         </is>
       </c>
       <c r="C665" s="1" t="inlineStr">
         <is>
-          <t>Prefeitura</t>
+          <t>Outro</t>
         </is>
       </c>
       <c r="D665" s="1" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E665" s="1" t="inlineStr">
         <is>
-          <t>Login/senha disponibilizado na MGC está incorreto</t>
+          <t>Boa tarde, Ellen.Conforme conversado, por gentileza realizar a alteração do período de apuração de 31/03/2026 para 31/07/2026.</t>
         </is>
       </c>
       <c r="F665" s="1" t="n">
-        <v>1082</v>
+        <v>861</v>
       </c>
       <c r="G665" s="1" t="inlineStr">
         <is>
-          <t>Supermercado Fenícia Ltda - Filial</t>
+          <t>SUPERMERCADO CASTELO DA SERRA LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H665" s="1" t="inlineStr">
         <is>
-          <t>Talita Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I665" s="1" t="inlineStr">
@@ -51398,10 +51416,10 @@
         </is>
       </c>
       <c r="J665" s="2" t="n">
-        <v>46251.39316516204</v>
+        <v>46248.7069753125</v>
       </c>
       <c r="K665" s="2" t="n">
-        <v>46254</v>
+        <v>46251</v>
       </c>
       <c r="L665" s="1" t="inlineStr">
         <is>
@@ -51410,7 +51428,7 @@
       </c>
       <c r="M665" s="1" t="inlineStr">
         <is>
-          <t>Daisa Araujo</t>
+          <t>Karina Fonseca</t>
         </is>
       </c>
       <c r="N665" s="1" t="n"/>
@@ -51428,7 +51446,7 @@
     </row>
     <row r="666">
       <c r="A666" s="1" t="n">
-        <v>82525</v>
+        <v>82498</v>
       </c>
       <c r="B666" s="1" t="inlineStr">
         <is>
@@ -51442,45 +51460,53 @@
       </c>
       <c r="D666" s="1" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E666" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde, poderia criar a senha do cliente 6936 - N&amp;S GLOBAL - da prefeitura e salva no MG Controle </t>
+          <t>Login/senha disponibilizado na MGC está incorreto</t>
         </is>
       </c>
       <c r="F666" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G666" s="1" t="n"/>
-      <c r="H666" s="1" t="n"/>
+        <v>1082</v>
+      </c>
+      <c r="G666" s="1" t="inlineStr">
+        <is>
+          <t>Supermercado Fenícia Ltda - Filial</t>
+        </is>
+      </c>
+      <c r="H666" s="1" t="inlineStr">
+        <is>
+          <t>Talita Silva</t>
+        </is>
+      </c>
       <c r="I666" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J666" s="2" t="n">
-        <v>46251.58507395833</v>
+        <v>46251.39316516204</v>
       </c>
       <c r="K666" s="2" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="L666" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M666" s="1" t="inlineStr">
         <is>
-          <t>Romario Silva</t>
+          <t>Daisa Araujo</t>
         </is>
       </c>
       <c r="N666" s="1" t="n"/>
       <c r="O666" s="1" t="n"/>
       <c r="P666" s="1" t="n"/>
       <c r="Q666" s="1" t="inlineStr"/>
-      <c r="R666" s="1" t="n"/>
+      <c r="R666" s="1" t="inlineStr"/>
       <c r="S666" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -51488,6 +51514,69 @@
       </c>
       <c r="T666" s="1" t="n"/>
       <c r="U666" s="1" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="1" t="n">
+        <v>82525</v>
+      </c>
+      <c r="B667" s="1" t="inlineStr">
+        <is>
+          <t>Senha</t>
+        </is>
+      </c>
+      <c r="C667" s="1" t="inlineStr">
+        <is>
+          <t>Prefeitura</t>
+        </is>
+      </c>
+      <c r="D667" s="1" t="inlineStr">
+        <is>
+          <t>EF - INDUSTRIA</t>
+        </is>
+      </c>
+      <c r="E667" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde, poderia criar a senha do cliente 6936 - N&amp;S GLOBAL - da prefeitura e salva no MG Controle </t>
+        </is>
+      </c>
+      <c r="F667" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G667" s="1" t="n"/>
+      <c r="H667" s="1" t="n"/>
+      <c r="I667" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J667" s="2" t="n">
+        <v>46251.58507395833</v>
+      </c>
+      <c r="K667" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="L667" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M667" s="1" t="inlineStr">
+        <is>
+          <t>Romario Silva</t>
+        </is>
+      </c>
+      <c r="N667" s="1" t="n"/>
+      <c r="O667" s="1" t="n"/>
+      <c r="P667" s="1" t="n"/>
+      <c r="Q667" s="1" t="inlineStr"/>
+      <c r="R667" s="1" t="n"/>
+      <c r="S667" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T667" s="1" t="n"/>
+      <c r="U667" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 15:04
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -2357,7 +2357,7 @@
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="H57" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Idna Sousa</t>
         </is>
       </c>
       <c r="I57" s="1" t="inlineStr">
@@ -9096,7 +9096,11 @@
           <t xml:space="preserve">SMART BREAK COMERCIO LANCHES S.A. (FILIAL 01) </t>
         </is>
       </c>
-      <c r="H103" s="1" t="n"/>
+      <c r="H103" s="1" t="inlineStr">
+        <is>
+          <t>Thaiza Oliveira</t>
+        </is>
+      </c>
       <c r="I103" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -9110,7 +9114,7 @@
       </c>
       <c r="L103" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M103" s="1" t="inlineStr">
@@ -9122,14 +9126,18 @@
       <c r="O103" s="1" t="n"/>
       <c r="P103" s="1" t="n"/>
       <c r="Q103" s="1" t="inlineStr"/>
-      <c r="R103" s="1" t="n"/>
+      <c r="R103" s="1" t="inlineStr"/>
       <c r="S103" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
       <c r="T103" s="1" t="n"/>
-      <c r="U103" s="1" t="inlineStr"/>
+      <c r="U103" s="1" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -13737,7 +13745,11 @@
           <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
         </is>
       </c>
-      <c r="H158" s="1" t="n"/>
+      <c r="H158" s="1" t="inlineStr">
+        <is>
+          <t>Juan Rodrigues</t>
+        </is>
+      </c>
       <c r="I158" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -13751,7 +13763,7 @@
       </c>
       <c r="L158" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M158" s="1" t="inlineStr">
@@ -13761,12 +13773,22 @@
       </c>
       <c r="N158" s="1" t="n"/>
       <c r="O158" s="1" t="n"/>
-      <c r="P158" s="1" t="n"/>
-      <c r="Q158" s="1" t="inlineStr"/>
-      <c r="R158" s="1" t="n"/>
+      <c r="P158" s="2" t="n">
+        <v>46251.62104864584</v>
+      </c>
+      <c r="Q158" s="1" t="inlineStr">
+        <is>
+          <t>Juan Rodrigues</t>
+        </is>
+      </c>
+      <c r="R158" s="1" t="inlineStr">
+        <is>
+          <t>Chamado criado ao departamento errado.</t>
+        </is>
+      </c>
       <c r="S158" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T158" s="1" t="n"/>
@@ -13871,7 +13893,11 @@
           <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
         </is>
       </c>
-      <c r="H160" s="1" t="n"/>
+      <c r="H160" s="1" t="inlineStr">
+        <is>
+          <t>Juan Rodrigues</t>
+        </is>
+      </c>
       <c r="I160" s="1" t="inlineStr">
         <is>
           <t>EF - VAREJO</t>
@@ -13885,7 +13911,7 @@
       </c>
       <c r="L160" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M160" s="1" t="inlineStr">
@@ -13895,12 +13921,22 @@
       </c>
       <c r="N160" s="1" t="n"/>
       <c r="O160" s="1" t="n"/>
-      <c r="P160" s="1" t="n"/>
-      <c r="Q160" s="1" t="inlineStr"/>
-      <c r="R160" s="1" t="n"/>
+      <c r="P160" s="2" t="n">
+        <v>46251.62092025463</v>
+      </c>
+      <c r="Q160" s="1" t="inlineStr">
+        <is>
+          <t>Juan Rodrigues</t>
+        </is>
+      </c>
+      <c r="R160" s="1" t="inlineStr">
+        <is>
+          <t>Chamado criado ao departamento errado.</t>
+        </is>
+      </c>
       <c r="S160" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T160" s="1" t="n"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-21 16:56
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U698" headerRowCount="1">
-  <autoFilter ref="A1:U698"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U699" headerRowCount="1">
+  <autoFilter ref="A1:U699"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U698"/>
+  <dimension ref="A1:U699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -41320,7 +41320,11 @@
         <v>0</v>
       </c>
       <c r="G528" s="1" t="n"/>
-      <c r="H528" s="1" t="n"/>
+      <c r="H528" s="1" t="inlineStr">
+        <is>
+          <t>Gabriel Amaral</t>
+        </is>
+      </c>
       <c r="I528" s="1" t="inlineStr">
         <is>
           <t>CONTROLADORIA</t>
@@ -41334,7 +41338,7 @@
       </c>
       <c r="L528" s="1" t="inlineStr">
         <is>
-          <t>Sem Responsavel Atribuido</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M528" s="1" t="inlineStr">
@@ -41346,7 +41350,7 @@
       <c r="O528" s="1" t="n"/>
       <c r="P528" s="1" t="n"/>
       <c r="Q528" s="1" t="inlineStr"/>
-      <c r="R528" s="1" t="n"/>
+      <c r="R528" s="1" t="inlineStr"/>
       <c r="S528" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -51536,7 +51540,7 @@
     </row>
     <row r="664">
       <c r="A664" s="1" t="n">
-        <v>81738</v>
+        <v>82821</v>
       </c>
       <c r="B664" s="1" t="inlineStr">
         <is>
@@ -51545,7 +51549,7 @@
       </c>
       <c r="C664" s="1" t="inlineStr">
         <is>
-          <t>Razão Social</t>
+          <t>Outras Cláusulas</t>
         </is>
       </c>
       <c r="D664" s="1" t="inlineStr">
@@ -51555,36 +51559,32 @@
       </c>
       <c r="E664" s="1" t="inlineStr">
         <is>
-          <t>ALTERAR A RAZÃO SOCIAL DA EMPRESA 6838-GR MIX GRUPO: GR MIXTRIBUTAÇÃO: LUCRO REALTIPO: COMÉRCIO, SERVIÇO E INDUSTRIAFINALIDADE: OPERACIONALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00Opção 1 da razão social: RG MIX CONCRETOS LTDA</t>
+          <t>Alteração contratual do CNAE da empresa: 6767-ALCANTARA LOGÍSTICA E TRANSPORTE LTDAGrupo: TW ALCANTARAProposta já negociada no valor de: R$ 2.500,00Incluir CNAE - 4712-1/00 COMO PRINCIPAL e o atual como secundário</t>
         </is>
       </c>
       <c r="F664" s="1" t="n">
-        <v>6838</v>
+        <v>6767</v>
       </c>
       <c r="G664" s="1" t="inlineStr">
         <is>
-          <t>GR MIX CONCRETOS LTDA</t>
-        </is>
-      </c>
-      <c r="H664" s="1" t="inlineStr">
-        <is>
-          <t>Edson Silva</t>
-        </is>
-      </c>
+          <t>ALCANTARA LOGÍSTICA E TRANSPORTE LTDA</t>
+        </is>
+      </c>
+      <c r="H664" s="1" t="n"/>
       <c r="I664" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J664" s="2" t="n">
-        <v>46237.43106087963</v>
+        <v>46255.68806971065</v>
       </c>
       <c r="K664" s="2" t="n">
-        <v>46265</v>
+        <v>46283</v>
       </c>
       <c r="L664" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M664" s="1" t="inlineStr">
@@ -51592,104 +51592,93 @@
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N664" s="2" t="n">
-        <v>46245.69663642361</v>
-      </c>
+      <c r="N664" s="1" t="n"/>
       <c r="O664" s="1" t="n"/>
       <c r="P664" s="1" t="n"/>
       <c r="Q664" s="1" t="inlineStr"/>
-      <c r="R664" s="1" t="inlineStr">
+      <c r="R664" s="1" t="n"/>
+      <c r="S664" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T664" s="1" t="n"/>
+      <c r="U664" s="1" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" s="1" t="n">
+        <v>81738</v>
+      </c>
+      <c r="B665" s="1" t="inlineStr">
+        <is>
+          <t>Alteração Contratual</t>
+        </is>
+      </c>
+      <c r="C665" s="1" t="inlineStr">
+        <is>
+          <t>Razão Social</t>
+        </is>
+      </c>
+      <c r="D665" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA MASTER</t>
+        </is>
+      </c>
+      <c r="E665" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAR A RAZÃO SOCIAL DA EMPRESA 6838-GR MIX GRUPO: GR MIXTRIBUTAÇÃO: LUCRO REALTIPO: COMÉRCIO, SERVIÇO E INDUSTRIAFINALIDADE: OPERACIONALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00Opção 1 da razão social: RG MIX CONCRETOS LTDA</t>
+        </is>
+      </c>
+      <c r="F665" s="1" t="n">
+        <v>6838</v>
+      </c>
+      <c r="G665" s="1" t="inlineStr">
+        <is>
+          <t>GR MIX CONCRETOS LTDA</t>
+        </is>
+      </c>
+      <c r="H665" s="1" t="inlineStr">
+        <is>
+          <t>Edson Silva</t>
+        </is>
+      </c>
+      <c r="I665" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J665" s="2" t="n">
+        <v>46237.43106087963</v>
+      </c>
+      <c r="K665" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="L665" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M665" s="1" t="inlineStr">
+        <is>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N665" s="2" t="n">
+        <v>46245.69663642361</v>
+      </c>
+      <c r="O665" s="1" t="n"/>
+      <c r="P665" s="1" t="n"/>
+      <c r="Q665" s="1" t="inlineStr"/>
+      <c r="R665" s="1" t="inlineStr">
         <is>
           <t>Boa tarde.
 Minuta enviada para o cliente
 Atenciosamente</t>
         </is>
       </c>
-      <c r="S664" s="1" t="inlineStr">
+      <c r="S665" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T664" s="1" t="n"/>
-      <c r="U664" s="1" t="inlineStr"/>
-    </row>
-    <row r="665">
-      <c r="A665" s="1" t="n">
-        <v>81426</v>
-      </c>
-      <c r="B665" s="1" t="inlineStr">
-        <is>
-          <t>Parcelamento RFB</t>
-        </is>
-      </c>
-      <c r="C665" s="1" t="inlineStr">
-        <is>
-          <t>Ordinário</t>
-        </is>
-      </c>
-      <c r="D665" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E665" s="1" t="inlineStr">
-        <is>
-          <t>ACERT - SIMULAÇÃO DE PARCELAMENTOCliente solicita simulação de parcelamento FEDERAL</t>
-        </is>
-      </c>
-      <c r="F665" s="1" t="n">
-        <v>6559</v>
-      </c>
-      <c r="G665" s="1" t="inlineStr">
-        <is>
-          <t>ACERTONLINE ASSESSORIA EMPRESARIAL LTDA</t>
-        </is>
-      </c>
-      <c r="H665" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
-      <c r="I665" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J665" s="2" t="n">
-        <v>46226.7238943287</v>
-      </c>
-      <c r="K665" s="2" t="n">
-        <v>46230</v>
-      </c>
-      <c r="L665" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M665" s="1" t="inlineStr">
-        <is>
-          <t>Vander Silva</t>
-        </is>
-      </c>
-      <c r="N665" s="1" t="n"/>
-      <c r="O665" s="1" t="n"/>
-      <c r="P665" s="2" t="n">
-        <v>46230.73675598379</v>
-      </c>
-      <c r="Q665" s="1" t="inlineStr">
-        <is>
-          <t>Karina Dantas</t>
-        </is>
-      </c>
-      <c r="R665" s="1" t="inlineStr">
-        <is>
-          <t>Boa tarde!
-Segue em anexo simulado e proposta.</t>
-        </is>
-      </c>
-      <c r="S665" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
         </is>
       </c>
       <c r="T665" s="1" t="n"/>
@@ -51697,16 +51686,16 @@
     </row>
     <row r="666">
       <c r="A666" s="1" t="n">
-        <v>82737</v>
+        <v>81426</v>
       </c>
       <c r="B666" s="1" t="inlineStr">
         <is>
-          <t>Regularização</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C666" s="1" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Ordinário</t>
         </is>
       </c>
       <c r="D666" s="1" t="inlineStr">
@@ -51716,20 +51705,20 @@
       </c>
       <c r="E666" s="1" t="inlineStr">
         <is>
-          <t>Prezados, cliente solicita alteração o contato de e-mail no cartão do CNPJ.e-mail atualizado - nanasupermercado@gmail.com</t>
+          <t>ACERT - SIMULAÇÃO DE PARCELAMENTOCliente solicita simulação de parcelamento FEDERAL</t>
         </is>
       </c>
       <c r="F666" s="1" t="n">
-        <v>6974</v>
+        <v>6559</v>
       </c>
       <c r="G666" s="1" t="inlineStr">
         <is>
-          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
+          <t>ACERTONLINE ASSESSORIA EMPRESARIAL LTDA</t>
         </is>
       </c>
       <c r="H666" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I666" s="1" t="inlineStr">
@@ -51738,10 +51727,10 @@
         </is>
       </c>
       <c r="J666" s="2" t="n">
-        <v>46254.60349059028</v>
+        <v>46226.7238943287</v>
       </c>
       <c r="K666" s="2" t="n">
-        <v>46258</v>
+        <v>46230</v>
       </c>
       <c r="L666" s="1" t="inlineStr">
         <is>
@@ -51750,107 +51739,108 @@
       </c>
       <c r="M666" s="1" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="N666" s="1" t="n"/>
       <c r="O666" s="1" t="n"/>
       <c r="P666" s="2" t="n">
+        <v>46230.73675598379</v>
+      </c>
+      <c r="Q666" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="R666" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!
+Segue em anexo simulado e proposta.</t>
+        </is>
+      </c>
+      <c r="S666" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T666" s="1" t="n"/>
+      <c r="U666" s="1" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="1" t="n">
+        <v>82737</v>
+      </c>
+      <c r="B667" s="1" t="inlineStr">
+        <is>
+          <t>Regularização</t>
+        </is>
+      </c>
+      <c r="C667" s="1" t="inlineStr">
+        <is>
+          <t>Outro</t>
+        </is>
+      </c>
+      <c r="D667" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E667" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, cliente solicita alteração o contato de e-mail no cartão do CNPJ.e-mail atualizado - nanasupermercado@gmail.com</t>
+        </is>
+      </c>
+      <c r="F667" s="1" t="n">
+        <v>6974</v>
+      </c>
+      <c r="G667" s="1" t="inlineStr">
+        <is>
+          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
+        </is>
+      </c>
+      <c r="H667" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
+      <c r="I667" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J667" s="2" t="n">
+        <v>46254.60349059028</v>
+      </c>
+      <c r="K667" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="L667" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M667" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N667" s="1" t="n"/>
+      <c r="O667" s="1" t="n"/>
+      <c r="P667" s="2" t="n">
         <v>46255.55876797454</v>
       </c>
-      <c r="Q666" s="1" t="inlineStr">
+      <c r="Q667" s="1" t="inlineStr">
         <is>
           <t>Bianca Ribeiro</t>
         </is>
       </c>
-      <c r="R666" s="1" t="inlineStr">
+      <c r="R667" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Prezados(as), boa tarde!
 Alteração realizada, conforme solicitado. 
 Atenciosamente, </t>
         </is>
       </c>
-      <c r="S666" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T666" s="1" t="n"/>
-      <c r="U666" s="1" t="inlineStr"/>
-    </row>
-    <row r="667">
-      <c r="A667" s="1" t="n">
-        <v>81987</v>
-      </c>
-      <c r="B667" s="1" t="inlineStr">
-        <is>
-          <t>Alteração Contratual</t>
-        </is>
-      </c>
-      <c r="C667" s="1" t="inlineStr">
-        <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="D667" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E667" s="1" t="inlineStr">
-        <is>
-          <t>6977 - PROTECTION SHIELD - MUDANÇAS NO CONTRATO SOCIALO Cliente precisa mudar o CNAI e incluir um sócio, poderia nos informar qual o honorário e quais documento você precisa?Desejo do cliente é fazer a transferência dos funcionário que estão hoje na 6976, para 6977, para isto é necessário haver a equiparação de atividades para não ter problemas Sindicais, então será necessita mudanças no CNAE, e para haver formação de grupo econômico a sócia deseja ter 1% de participação na 6977, hoje ela  da sociedade apenas como tutora do socio de menor, e como administradora.  Mais informações com o REYNALDO.Att.Vander</t>
-        </is>
-      </c>
-      <c r="F667" s="1" t="n">
-        <v>6977</v>
-      </c>
-      <c r="G667" s="1" t="inlineStr">
-        <is>
-          <t>PROTECTION SHIELD LTDA</t>
-        </is>
-      </c>
-      <c r="H667" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="I667" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J667" s="2" t="n">
-        <v>46240.55237392361</v>
-      </c>
-      <c r="K667" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="L667" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M667" s="1" t="inlineStr">
-        <is>
-          <t>Vander Silva</t>
-        </is>
-      </c>
-      <c r="N667" s="1" t="n"/>
-      <c r="O667" s="1" t="n"/>
-      <c r="P667" s="2" t="n">
-        <v>46251.68881709491</v>
-      </c>
-      <c r="Q667" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R667" s="1" t="inlineStr">
-        <is>
-          <t>Favor, informar o que vai ser alterado de fato.</t>
-        </is>
-      </c>
       <c r="S667" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -51861,240 +51851,240 @@
     </row>
     <row r="668">
       <c r="A668" s="1" t="n">
+        <v>81987</v>
+      </c>
+      <c r="B668" s="1" t="inlineStr">
+        <is>
+          <t>Alteração Contratual</t>
+        </is>
+      </c>
+      <c r="C668" s="1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="D668" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E668" s="1" t="inlineStr">
+        <is>
+          <t>6977 - PROTECTION SHIELD - MUDANÇAS NO CONTRATO SOCIALO Cliente precisa mudar o CNAI e incluir um sócio, poderia nos informar qual o honorário e quais documento você precisa?Desejo do cliente é fazer a transferência dos funcionário que estão hoje na 6976, para 6977, para isto é necessário haver a equiparação de atividades para não ter problemas Sindicais, então será necessita mudanças no CNAE, e para haver formação de grupo econômico a sócia deseja ter 1% de participação na 6977, hoje ela  da sociedade apenas como tutora do socio de menor, e como administradora.  Mais informações com o REYNALDO.Att.Vander</t>
+        </is>
+      </c>
+      <c r="F668" s="1" t="n">
+        <v>6977</v>
+      </c>
+      <c r="G668" s="1" t="inlineStr">
+        <is>
+          <t>PROTECTION SHIELD LTDA</t>
+        </is>
+      </c>
+      <c r="H668" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="I668" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J668" s="2" t="n">
+        <v>46240.55237392361</v>
+      </c>
+      <c r="K668" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="L668" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M668" s="1" t="inlineStr">
+        <is>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N668" s="1" t="n"/>
+      <c r="O668" s="1" t="n"/>
+      <c r="P668" s="2" t="n">
+        <v>46251.68881709491</v>
+      </c>
+      <c r="Q668" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="R668" s="1" t="inlineStr">
+        <is>
+          <t>Favor, informar o que vai ser alterado de fato.</t>
+        </is>
+      </c>
+      <c r="S668" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T668" s="1" t="n"/>
+      <c r="U668" s="1" t="inlineStr"/>
+    </row>
+    <row r="669">
+      <c r="A669" s="1" t="n">
         <v>81753</v>
       </c>
-      <c r="B668" s="1" t="inlineStr">
+      <c r="B669" s="1" t="inlineStr">
         <is>
           <t>Abertura de Empresa</t>
         </is>
       </c>
-      <c r="C668" s="1" t="inlineStr">
+      <c r="C669" s="1" t="inlineStr">
         <is>
           <t>Sociedade - Comércio</t>
         </is>
       </c>
-      <c r="D668" s="1" t="inlineStr">
+      <c r="D669" s="1" t="inlineStr">
         <is>
           <t>GERENCIA MASTER</t>
         </is>
       </c>
-      <c r="E668" s="1" t="inlineStr">
+      <c r="E669" s="1" t="inlineStr">
         <is>
           <t>ABERTURA DE EMPRESA - 6981-LUIZ GOMES DA SILVA - O GOIANOGRUPO: SUPERMERCADO AVENIDATRIBUTAÇÃO: SIMPLES NACIONALTIPO DE ATIVIDADE: COMÉRCIO FINALIDADE: HOLDING/ESTRATÉGIAFORMA JURIDICA: LTDAPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00EMPRESA DE ESTRATÉGIA, APÓS CONSTITUIDA MIGRAR OS FUNCIONARIOS. APÓS TERMINO DA MIGRAÇÃO ALTERAR ATIVIDADE E QUADRO SOCIETÁRIO.</t>
         </is>
       </c>
-      <c r="F668" s="1" t="n">
+      <c r="F669" s="1" t="n">
         <v>6981</v>
       </c>
-      <c r="G668" s="1" t="inlineStr">
+      <c r="G669" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
         </is>
       </c>
-      <c r="H668" s="1" t="inlineStr">
+      <c r="H669" s="1" t="inlineStr">
         <is>
           <t>Bianca Ribeiro</t>
         </is>
       </c>
-      <c r="I668" s="1" t="inlineStr">
+      <c r="I669" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J668" s="2" t="n">
+      <c r="J669" s="2" t="n">
         <v>46237.51070853009</v>
       </c>
-      <c r="K668" s="2" t="n">
+      <c r="K669" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="L668" s="1" t="inlineStr">
+      <c r="L669" s="1" t="inlineStr">
         <is>
           <t>Em Atendimento</t>
         </is>
       </c>
-      <c r="M668" s="1" t="inlineStr">
+      <c r="M669" s="1" t="inlineStr">
         <is>
           <t>Raisa Sousa</t>
         </is>
       </c>
-      <c r="N668" s="2" t="n">
+      <c r="N669" s="2" t="n">
         <v>46246.66714818287</v>
       </c>
-      <c r="O668" s="1" t="n"/>
-      <c r="P668" s="1" t="n"/>
-      <c r="Q668" s="1" t="inlineStr"/>
-      <c r="R668" s="1" t="inlineStr">
+      <c r="O669" s="1" t="n"/>
+      <c r="P669" s="1" t="n"/>
+      <c r="Q669" s="1" t="inlineStr"/>
+      <c r="R669" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Prezados(as), boa tarde!
 Processo de abertura em andamento. 
 Atenciosamente, </t>
         </is>
       </c>
-      <c r="S668" s="1" t="inlineStr">
+      <c r="S669" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="T668" s="1" t="n"/>
-      <c r="U668" s="1" t="inlineStr"/>
-    </row>
-    <row r="669">
-      <c r="A669" s="1" t="n">
+      <c r="T669" s="1" t="n"/>
+      <c r="U669" s="1" t="inlineStr"/>
+    </row>
+    <row r="670">
+      <c r="A670" s="1" t="n">
         <v>82173</v>
       </c>
-      <c r="B669" s="1" t="inlineStr">
+      <c r="B670" s="1" t="inlineStr">
         <is>
           <t>Certidão</t>
         </is>
       </c>
-      <c r="C669" s="1" t="inlineStr">
+      <c r="C670" s="1" t="inlineStr">
         <is>
           <t>Municipal</t>
         </is>
       </c>
-      <c r="D669" s="1" t="inlineStr">
+      <c r="D670" s="1" t="inlineStr">
         <is>
           <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E669" s="1" t="inlineStr">
+      <c r="E670" s="1" t="inlineStr">
         <is>
           <t>Boa tarde!!Por gentileza, gerar CND MUNICIPAL da empresa 6984.</t>
         </is>
       </c>
-      <c r="F669" s="1" t="n">
+      <c r="F670" s="1" t="n">
         <v>6984</v>
       </c>
-      <c r="G669" s="1" t="inlineStr">
+      <c r="G670" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
         </is>
       </c>
-      <c r="H669" s="1" t="inlineStr">
+      <c r="H670" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="I669" s="1" t="inlineStr">
+      <c r="I670" s="1" t="inlineStr">
         <is>
           <t>PARALEGAL</t>
         </is>
       </c>
-      <c r="J669" s="2" t="n">
+      <c r="J670" s="2" t="n">
         <v>46244.63940714121</v>
       </c>
-      <c r="K669" s="2" t="n">
+      <c r="K670" s="2" t="n">
         <v>46245</v>
       </c>
-      <c r="L669" s="1" t="inlineStr">
+      <c r="L670" s="1" t="inlineStr">
         <is>
           <t>Entregue Ao Solicitante</t>
         </is>
       </c>
-      <c r="M669" s="1" t="inlineStr">
+      <c r="M670" s="1" t="inlineStr">
         <is>
           <t>Yasmin Peixoto</t>
         </is>
       </c>
-      <c r="N669" s="2" t="n">
+      <c r="N670" s="2" t="n">
         <v>46245.46407800926</v>
       </c>
-      <c r="O669" s="1" t="n"/>
-      <c r="P669" s="2" t="n">
+      <c r="O670" s="1" t="n"/>
+      <c r="P670" s="2" t="n">
         <v>46246.37610829861</v>
       </c>
-      <c r="Q669" s="1" t="inlineStr">
+      <c r="Q670" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R669" s="1" t="inlineStr">
+      <c r="R670" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bom dia!
 Para emissão de CND Municipal em Itapecerica há um custo, o cliente está ciente? </t>
         </is>
       </c>
-      <c r="S669" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T669" s="1" t="n"/>
-      <c r="U669" s="1" t="inlineStr"/>
-    </row>
-    <row r="670">
-      <c r="A670" s="1" t="n">
-        <v>82395</v>
-      </c>
-      <c r="B670" s="1" t="inlineStr">
-        <is>
-          <t>Parcelamento RFB</t>
-        </is>
-      </c>
-      <c r="C670" s="1" t="inlineStr">
-        <is>
-          <t>Simplificado</t>
-        </is>
-      </c>
-      <c r="D670" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E670" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Boa tarde prezados!!Por gentileza, realizar simulação de parcelamento de débitos na RFB. </t>
-        </is>
-      </c>
-      <c r="F670" s="1" t="n">
-        <v>6984</v>
-      </c>
-      <c r="G670" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
-        </is>
-      </c>
-      <c r="H670" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="I670" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J670" s="2" t="n">
-        <v>46247.70127098379</v>
-      </c>
-      <c r="K670" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="L670" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M670" s="1" t="inlineStr">
-        <is>
-          <t>Yasmin Peixoto</t>
-        </is>
-      </c>
-      <c r="N670" s="1" t="n"/>
-      <c r="O670" s="1" t="n"/>
-      <c r="P670" s="2" t="n">
-        <v>46252.57205790509</v>
-      </c>
-      <c r="Q670" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="R670" s="1" t="inlineStr">
-        <is>
-          <t>Segue simulado e proposta para parcelamento dos débitos federais em aberto do cliente 6984 - SUPERMERCADOS BANDEIRA.</t>
-        </is>
-      </c>
       <c r="S670" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -52105,16 +52095,16 @@
     </row>
     <row r="671">
       <c r="A671" s="1" t="n">
-        <v>82174</v>
+        <v>82395</v>
       </c>
       <c r="B671" s="1" t="inlineStr">
         <is>
-          <t>Certidão</t>
+          <t>Parcelamento RFB</t>
         </is>
       </c>
       <c r="C671" s="1" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Simplificado</t>
         </is>
       </c>
       <c r="D671" s="1" t="inlineStr">
@@ -52124,20 +52114,20 @@
       </c>
       <c r="E671" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!!Por gentileza, gerar CND MUNICIPAL da empresa 6985.</t>
+          <t xml:space="preserve">Boa tarde prezados!!Por gentileza, realizar simulação de parcelamento de débitos na RFB. </t>
         </is>
       </c>
       <c r="F671" s="1" t="n">
-        <v>6985</v>
+        <v>6984</v>
       </c>
       <c r="G671" s="1" t="inlineStr">
         <is>
-          <t>T F MIRANDA MERCADO LTDA</t>
+          <t xml:space="preserve"> SUPERMERCADOS BANDEIRA LTDA.</t>
         </is>
       </c>
       <c r="H671" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I671" s="1" t="inlineStr">
@@ -52146,10 +52136,10 @@
         </is>
       </c>
       <c r="J671" s="2" t="n">
-        <v>46244.64014872685</v>
+        <v>46247.70127098379</v>
       </c>
       <c r="K671" s="2" t="n">
-        <v>46245</v>
+        <v>46251</v>
       </c>
       <c r="L671" s="1" t="inlineStr">
         <is>
@@ -52161,105 +52151,105 @@
           <t>Yasmin Peixoto</t>
         </is>
       </c>
-      <c r="N671" s="2" t="n">
-        <v>46245.46419699074</v>
-      </c>
+      <c r="N671" s="1" t="n"/>
       <c r="O671" s="1" t="n"/>
       <c r="P671" s="2" t="n">
+        <v>46252.57205790509</v>
+      </c>
+      <c r="Q671" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
+      <c r="R671" s="1" t="inlineStr">
+        <is>
+          <t>Segue simulado e proposta para parcelamento dos débitos federais em aberto do cliente 6984 - SUPERMERCADOS BANDEIRA.</t>
+        </is>
+      </c>
+      <c r="S671" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T671" s="1" t="n"/>
+      <c r="U671" s="1" t="inlineStr"/>
+    </row>
+    <row r="672">
+      <c r="A672" s="1" t="n">
+        <v>82174</v>
+      </c>
+      <c r="B672" s="1" t="inlineStr">
+        <is>
+          <t>Certidão</t>
+        </is>
+      </c>
+      <c r="C672" s="1" t="inlineStr">
+        <is>
+          <t>Municipal</t>
+        </is>
+      </c>
+      <c r="D672" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E672" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde!!Por gentileza, gerar CND MUNICIPAL da empresa 6985.</t>
+        </is>
+      </c>
+      <c r="F672" s="1" t="n">
+        <v>6985</v>
+      </c>
+      <c r="G672" s="1" t="inlineStr">
+        <is>
+          <t>T F MIRANDA MERCADO LTDA</t>
+        </is>
+      </c>
+      <c r="H672" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="I672" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J672" s="2" t="n">
+        <v>46244.64014872685</v>
+      </c>
+      <c r="K672" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="L672" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M672" s="1" t="inlineStr">
+        <is>
+          <t>Yasmin Peixoto</t>
+        </is>
+      </c>
+      <c r="N672" s="2" t="n">
+        <v>46245.46419699074</v>
+      </c>
+      <c r="O672" s="1" t="n"/>
+      <c r="P672" s="2" t="n">
         <v>46246.37627866898</v>
       </c>
-      <c r="Q671" s="1" t="inlineStr">
+      <c r="Q672" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R671" s="1" t="inlineStr">
+      <c r="R672" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bom dia!
 Para emissão de CND Municipal em Itapecerica há um custo, o cliente está ciente? </t>
         </is>
       </c>
-      <c r="S671" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="T671" s="1" t="n"/>
-      <c r="U671" s="1" t="inlineStr"/>
-    </row>
-    <row r="672">
-      <c r="A672" s="1" t="n">
-        <v>81933</v>
-      </c>
-      <c r="B672" s="1" t="inlineStr">
-        <is>
-          <t>Certidão</t>
-        </is>
-      </c>
-      <c r="C672" s="1" t="inlineStr">
-        <is>
-          <t>Outras</t>
-        </is>
-      </c>
-      <c r="D672" s="1" t="inlineStr">
-        <is>
-          <t>GC - ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="E672" s="1" t="inlineStr">
-        <is>
-          <t>Por gentileza, providenciar:6990 - RC MATERIAIS ELETRICOS E HIDRAULICOS (MATRIZ) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL6991 - RC MATERIAIS ELETRICOS E HIDRAULICOS (FILIAL 1) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL</t>
-        </is>
-      </c>
-      <c r="F672" s="1" t="n">
-        <v>6990</v>
-      </c>
-      <c r="G672" s="1" t="inlineStr">
-        <is>
-          <t>AMANCIO S ELETRICA, HIDRAULICA E CONSTRUCAO EM GERAL LTDA (MATRIZ)</t>
-        </is>
-      </c>
-      <c r="H672" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="I672" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J672" s="2" t="n">
-        <v>46239.72520292824</v>
-      </c>
-      <c r="K672" s="2" t="n">
-        <v>46241</v>
-      </c>
-      <c r="L672" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M672" s="1" t="inlineStr">
-        <is>
-          <t>Bruno Contieri</t>
-        </is>
-      </c>
-      <c r="N672" s="1" t="n"/>
-      <c r="O672" s="1" t="n"/>
-      <c r="P672" s="2" t="n">
-        <v>46241.65195802083</v>
-      </c>
-      <c r="Q672" s="1" t="inlineStr">
-        <is>
-          <t>Ellen Leite</t>
-        </is>
-      </c>
-      <c r="R672" s="1" t="inlineStr">
-        <is>
-          <t>Abrir um chamado por empresa, por gentileza.</t>
-        </is>
-      </c>
       <c r="S672" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -52270,39 +52260,39 @@
     </row>
     <row r="673">
       <c r="A673" s="1" t="n">
-        <v>81932</v>
+        <v>81933</v>
       </c>
       <c r="B673" s="1" t="inlineStr">
         <is>
-          <t>Alteração Contratual</t>
+          <t>Certidão</t>
         </is>
       </c>
       <c r="C673" s="1" t="inlineStr">
         <is>
-          <t>Sócios</t>
+          <t>Outras</t>
         </is>
       </c>
       <c r="D673" s="1" t="inlineStr">
         <is>
-          <t>GERENCIA MASTER</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E673" s="1" t="inlineStr">
         <is>
-          <t>ALTERAÇÃO CONTRATUAL DE QSA. EMPRESA: 6921-METALÚRGICA G3 LTDAGRUPO: G4 LINHA VIVAPROPOSTA JÁ NEGOCIADA.</t>
+          <t>Por gentileza, providenciar:6990 - RC MATERIAIS ELETRICOS E HIDRAULICOS (MATRIZ) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL6991 - RC MATERIAIS ELETRICOS E HIDRAULICOS (FILIAL 1) - CERTIDÃO ESTADUAL FEDERAL, ESTADUAL E MUNICIPAL</t>
         </is>
       </c>
       <c r="F673" s="1" t="n">
-        <v>6921</v>
+        <v>6990</v>
       </c>
       <c r="G673" s="1" t="inlineStr">
         <is>
-          <t>METALURGICA G3 LTDA</t>
+          <t>AMANCIO S ELETRICA, HIDRAULICA E CONSTRUCAO EM GERAL LTDA (MATRIZ)</t>
         </is>
       </c>
       <c r="H673" s="1" t="inlineStr">
         <is>
-          <t>Edson Silva</t>
+          <t>Ellen Leite</t>
         </is>
       </c>
       <c r="I673" s="1" t="inlineStr">
@@ -52311,37 +52301,39 @@
         </is>
       </c>
       <c r="J673" s="2" t="n">
-        <v>46239.71162623842</v>
+        <v>46239.72520292824</v>
       </c>
       <c r="K673" s="2" t="n">
-        <v>46267</v>
+        <v>46241</v>
       </c>
       <c r="L673" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M673" s="1" t="inlineStr">
         <is>
-          <t>Raisa Sousa</t>
-        </is>
-      </c>
-      <c r="N673" s="2" t="n">
-        <v>46247.44207098379</v>
-      </c>
+          <t>Bruno Contieri</t>
+        </is>
+      </c>
+      <c r="N673" s="1" t="n"/>
       <c r="O673" s="1" t="n"/>
-      <c r="P673" s="1" t="n"/>
-      <c r="Q673" s="1" t="inlineStr"/>
+      <c r="P673" s="2" t="n">
+        <v>46241.65195802083</v>
+      </c>
+      <c r="Q673" s="1" t="inlineStr">
+        <is>
+          <t>Ellen Leite</t>
+        </is>
+      </c>
       <c r="R673" s="1" t="inlineStr">
         <is>
-          <t>Bom dia,
-Minuta em andamento.
-Atenciosamente</t>
+          <t>Abrir um chamado por empresa, por gentileza.</t>
         </is>
       </c>
       <c r="S673" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T673" s="1" t="n"/>
@@ -52349,7 +52341,7 @@
     </row>
     <row r="674">
       <c r="A674" s="1" t="n">
-        <v>81780</v>
+        <v>81932</v>
       </c>
       <c r="B674" s="1" t="inlineStr">
         <is>
@@ -52358,7 +52350,7 @@
       </c>
       <c r="C674" s="1" t="inlineStr">
         <is>
-          <t>Objeto Social</t>
+          <t>Sócios</t>
         </is>
       </c>
       <c r="D674" s="1" t="inlineStr">
@@ -52368,20 +52360,20 @@
       </c>
       <c r="E674" s="1" t="inlineStr">
         <is>
-          <t>ALTERAÇÃO CONTRATUAL DA EMPRESA: 6993-GOMES SERVIÇOS - LTDAGRUPO: CRISTO REIALTERAÇÃO DE QSA E OBJETO SOCIALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00MESMA ATIVIDADE E SÓCIOS DO SUP. AVENIDA, APÓS ALTERAÇÃO MIGRAR FUNCIONÁRIOS PARA NOVA EMPRESA ALTERAR QSA E OBJETO SOCIAL.</t>
+          <t>ALTERAÇÃO CONTRATUAL DE QSA. EMPRESA: 6921-METALÚRGICA G3 LTDAGRUPO: G4 LINHA VIVAPROPOSTA JÁ NEGOCIADA.</t>
         </is>
       </c>
       <c r="F674" s="1" t="n">
-        <v>6993</v>
+        <v>6921</v>
       </c>
       <c r="G674" s="1" t="inlineStr">
         <is>
-          <t>GOMES SERVIÇOS - LTDA</t>
+          <t>METALURGICA G3 LTDA</t>
         </is>
       </c>
       <c r="H674" s="1" t="inlineStr">
         <is>
-          <t>Bianca Ribeiro</t>
+          <t>Edson Silva</t>
         </is>
       </c>
       <c r="I674" s="1" t="inlineStr">
@@ -52390,10 +52382,10 @@
         </is>
       </c>
       <c r="J674" s="2" t="n">
-        <v>46237.62372283565</v>
+        <v>46239.71162623842</v>
       </c>
       <c r="K674" s="2" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="L674" s="1" t="inlineStr">
         <is>
@@ -52406,85 +52398,97 @@
         </is>
       </c>
       <c r="N674" s="2" t="n">
-        <v>46246.66900671296</v>
+        <v>46247.44207098379</v>
       </c>
       <c r="O674" s="1" t="n"/>
       <c r="P674" s="1" t="n"/>
       <c r="Q674" s="1" t="inlineStr"/>
       <c r="R674" s="1" t="inlineStr">
         <is>
+          <t>Bom dia,
+Minuta em andamento.
+Atenciosamente</t>
+        </is>
+      </c>
+      <c r="S674" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T674" s="1" t="n"/>
+      <c r="U674" s="1" t="inlineStr"/>
+    </row>
+    <row r="675">
+      <c r="A675" s="1" t="n">
+        <v>81780</v>
+      </c>
+      <c r="B675" s="1" t="inlineStr">
+        <is>
+          <t>Alteração Contratual</t>
+        </is>
+      </c>
+      <c r="C675" s="1" t="inlineStr">
+        <is>
+          <t>Objeto Social</t>
+        </is>
+      </c>
+      <c r="D675" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA MASTER</t>
+        </is>
+      </c>
+      <c r="E675" s="1" t="inlineStr">
+        <is>
+          <t>ALTERAÇÃO CONTRATUAL DA EMPRESA: 6993-GOMES SERVIÇOS - LTDAGRUPO: CRISTO REIALTERAÇÃO DE QSA E OBJETO SOCIALPROPOSTA JÁ NEGOCIADA NO VALOR DE R$2.500,00MESMA ATIVIDADE E SÓCIOS DO SUP. AVENIDA, APÓS ALTERAÇÃO MIGRAR FUNCIONÁRIOS PARA NOVA EMPRESA ALTERAR QSA E OBJETO SOCIAL.</t>
+        </is>
+      </c>
+      <c r="F675" s="1" t="n">
+        <v>6993</v>
+      </c>
+      <c r="G675" s="1" t="inlineStr">
+        <is>
+          <t>GOMES SERVIÇOS - LTDA</t>
+        </is>
+      </c>
+      <c r="H675" s="1" t="inlineStr">
+        <is>
+          <t>Bianca Ribeiro</t>
+        </is>
+      </c>
+      <c r="I675" s="1" t="inlineStr">
+        <is>
+          <t>PARALEGAL</t>
+        </is>
+      </c>
+      <c r="J675" s="2" t="n">
+        <v>46237.62372283565</v>
+      </c>
+      <c r="K675" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="L675" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M675" s="1" t="inlineStr">
+        <is>
+          <t>Raisa Sousa</t>
+        </is>
+      </c>
+      <c r="N675" s="2" t="n">
+        <v>46246.66900671296</v>
+      </c>
+      <c r="O675" s="1" t="n"/>
+      <c r="P675" s="1" t="n"/>
+      <c r="Q675" s="1" t="inlineStr"/>
+      <c r="R675" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Prezados(as), boa tarde!
 Alteração contratual em andamento. 
 Atenciosamente, </t>
         </is>
       </c>
-      <c r="S674" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T674" s="1" t="n"/>
-      <c r="U674" s="1" t="inlineStr"/>
-    </row>
-    <row r="675">
-      <c r="A675" s="1" t="n">
-        <v>82773</v>
-      </c>
-      <c r="B675" s="1" t="inlineStr">
-        <is>
-          <t>Senha</t>
-        </is>
-      </c>
-      <c r="C675" s="1" t="inlineStr">
-        <is>
-          <t>Prefeitura</t>
-        </is>
-      </c>
-      <c r="D675" s="1" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="E675" s="1" t="inlineStr">
-        <is>
-          <t>Bom dia,Por gentileza, esse cliente é novo na MG e não temos dados cadastrados em Senhas/ Registros no cadastro na intranetmg.Quando possível poderiam nos ajudar a respeito.Grato.Edimar Santos.</t>
-        </is>
-      </c>
-      <c r="F675" s="1" t="n">
-        <v>6998</v>
-      </c>
-      <c r="G675" s="1" t="inlineStr">
-        <is>
-          <t>NOVA BOSTON GRILL RESTAURANTE LTDA</t>
-        </is>
-      </c>
-      <c r="H675" s="1" t="n"/>
-      <c r="I675" s="1" t="inlineStr">
-        <is>
-          <t>PARALEGAL</t>
-        </is>
-      </c>
-      <c r="J675" s="2" t="n">
-        <v>46255.40404629629</v>
-      </c>
-      <c r="K675" s="2" t="n">
-        <v>46265</v>
-      </c>
-      <c r="L675" s="1" t="inlineStr">
-        <is>
-          <t>Sem Responsavel Atribuido</t>
-        </is>
-      </c>
-      <c r="M675" s="1" t="inlineStr">
-        <is>
-          <t>Edimar Santos</t>
-        </is>
-      </c>
-      <c r="N675" s="1" t="n"/>
-      <c r="O675" s="1" t="n"/>
-      <c r="P675" s="1" t="n"/>
-      <c r="Q675" s="1" t="inlineStr"/>
-      <c r="R675" s="1" t="n"/>
       <c r="S675" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52495,71 +52499,63 @@
     </row>
     <row r="676">
       <c r="A676" s="1" t="n">
-        <v>82755</v>
+        <v>82773</v>
       </c>
       <c r="B676" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Senha</t>
         </is>
       </c>
       <c r="C676" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Prefeitura</t>
         </is>
       </c>
       <c r="D676" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="E676" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
+          <t>Bom dia,Por gentileza, esse cliente é novo na MG e não temos dados cadastrados em Senhas/ Registros no cadastro na intranetmg.Quando possível poderiam nos ajudar a respeito.Grato.Edimar Santos.</t>
         </is>
       </c>
       <c r="F676" s="1" t="n">
-        <v>7005</v>
+        <v>6998</v>
       </c>
       <c r="G676" s="1" t="inlineStr">
         <is>
-          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
-        </is>
-      </c>
-      <c r="H676" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
+          <t>NOVA BOSTON GRILL RESTAURANTE LTDA</t>
+        </is>
+      </c>
+      <c r="H676" s="1" t="n"/>
       <c r="I676" s="1" t="inlineStr">
         <is>
-          <t>PL - AUDITORIA</t>
+          <t>PARALEGAL</t>
         </is>
       </c>
       <c r="J676" s="2" t="n">
-        <v>46254.65957604167</v>
+        <v>46255.40404629629</v>
       </c>
       <c r="K676" s="2" t="n">
-        <v>46255</v>
+        <v>46265</v>
       </c>
       <c r="L676" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Sem Responsavel Atribuido</t>
         </is>
       </c>
       <c r="M676" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
+          <t>Edimar Santos</t>
         </is>
       </c>
       <c r="N676" s="1" t="n"/>
       <c r="O676" s="1" t="n"/>
       <c r="P676" s="1" t="n"/>
       <c r="Q676" s="1" t="inlineStr"/>
-      <c r="R676" s="1" t="inlineStr">
-        <is>
-          <t>cobramos novamente o retorno dos documentos</t>
-        </is>
-      </c>
+      <c r="R676" s="1" t="n"/>
       <c r="S676" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52570,7 +52566,7 @@
     </row>
     <row r="677">
       <c r="A677" s="1" t="n">
-        <v>82756</v>
+        <v>82755</v>
       </c>
       <c r="B677" s="1" t="inlineStr">
         <is>
@@ -52593,11 +52589,11 @@
         </is>
       </c>
       <c r="F677" s="1" t="n">
-        <v>7006</v>
+        <v>7005</v>
       </c>
       <c r="G677" s="1" t="inlineStr">
         <is>
-          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+          <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H677" s="1" t="inlineStr">
@@ -52611,7 +52607,7 @@
         </is>
       </c>
       <c r="J677" s="2" t="n">
-        <v>46254.65986380787</v>
+        <v>46254.65957604167</v>
       </c>
       <c r="K677" s="2" t="n">
         <v>46255</v>
@@ -52632,7 +52628,7 @@
       <c r="Q677" s="1" t="inlineStr"/>
       <c r="R677" s="1" t="inlineStr">
         <is>
-          <t>cobramos novamente os documentos</t>
+          <t>cobramos novamente o retorno dos documentos</t>
         </is>
       </c>
       <c r="S677" s="1" t="inlineStr">
@@ -52645,7 +52641,7 @@
     </row>
     <row r="678">
       <c r="A678" s="1" t="n">
-        <v>82754</v>
+        <v>82756</v>
       </c>
       <c r="B678" s="1" t="inlineStr">
         <is>
@@ -52668,11 +52664,11 @@
         </is>
       </c>
       <c r="F678" s="1" t="n">
-        <v>6995</v>
+        <v>7006</v>
       </c>
       <c r="G678" s="1" t="inlineStr">
         <is>
-          <t>TRIZGA COMÉRCIO DE ACESSÓRIOS LTDA</t>
+          <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
         </is>
       </c>
       <c r="H678" s="1" t="inlineStr">
@@ -52686,14 +52682,14 @@
         </is>
       </c>
       <c r="J678" s="2" t="n">
-        <v>46254.6592349537</v>
+        <v>46254.65986380787</v>
       </c>
       <c r="K678" s="2" t="n">
         <v>46255</v>
       </c>
       <c r="L678" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M678" s="1" t="inlineStr">
@@ -52705,7 +52701,11 @@
       <c r="O678" s="1" t="n"/>
       <c r="P678" s="1" t="n"/>
       <c r="Q678" s="1" t="inlineStr"/>
-      <c r="R678" s="1" t="inlineStr"/>
+      <c r="R678" s="1" t="inlineStr">
+        <is>
+          <t>cobramos novamente os documentos</t>
+        </is>
+      </c>
       <c r="S678" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -52716,7 +52716,7 @@
     </row>
     <row r="679">
       <c r="A679" s="1" t="n">
-        <v>82752</v>
+        <v>82754</v>
       </c>
       <c r="B679" s="1" t="inlineStr">
         <is>
@@ -52739,11 +52739,11 @@
         </is>
       </c>
       <c r="F679" s="1" t="n">
-        <v>6992</v>
+        <v>6995</v>
       </c>
       <c r="G679" s="1" t="inlineStr">
         <is>
-          <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
+          <t>TRIZGA COMÉRCIO DE ACESSÓRIOS LTDA</t>
         </is>
       </c>
       <c r="H679" s="1" t="inlineStr">
@@ -52757,7 +52757,7 @@
         </is>
       </c>
       <c r="J679" s="2" t="n">
-        <v>46254.65860883102</v>
+        <v>46254.6592349537</v>
       </c>
       <c r="K679" s="2" t="n">
         <v>46255</v>
@@ -52787,7 +52787,7 @@
     </row>
     <row r="680">
       <c r="A680" s="1" t="n">
-        <v>82753</v>
+        <v>82752</v>
       </c>
       <c r="B680" s="1" t="inlineStr">
         <is>
@@ -52810,11 +52810,11 @@
         </is>
       </c>
       <c r="F680" s="1" t="n">
-        <v>6993</v>
+        <v>6992</v>
       </c>
       <c r="G680" s="1" t="inlineStr">
         <is>
-          <t>GOMES SERVIÇOS - LTDA</t>
+          <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
         </is>
       </c>
       <c r="H680" s="1" t="inlineStr">
@@ -52828,7 +52828,7 @@
         </is>
       </c>
       <c r="J680" s="2" t="n">
-        <v>46254.65888769676</v>
+        <v>46254.65860883102</v>
       </c>
       <c r="K680" s="2" t="n">
         <v>46255</v>
@@ -52858,39 +52858,39 @@
     </row>
     <row r="681">
       <c r="A681" s="1" t="n">
-        <v>82053</v>
+        <v>82753</v>
       </c>
       <c r="B681" s="1" t="inlineStr">
         <is>
-          <t>Ata de Reunião</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C681" s="1" t="inlineStr">
         <is>
-          <t>Inclusão de Ata</t>
+          <t>Implantação DP</t>
         </is>
       </c>
       <c r="D681" s="1" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="E681" s="1" t="inlineStr">
         <is>
-          <t>6913	CL Comércio	MAED	Verificar pendência5254	RCL	MAED	Enviar guias para pagamento</t>
+          <t>Boa tarde, por gentileza, providenciar documentos para implantação.</t>
         </is>
       </c>
       <c r="F681" s="1" t="n">
-        <v>6913</v>
+        <v>6993</v>
       </c>
       <c r="G681" s="1" t="inlineStr">
         <is>
-          <t>CL COMERCIO VAREJISTA E ROTISSERIE LTDA</t>
+          <t>GOMES SERVIÇOS - LTDA</t>
         </is>
       </c>
       <c r="H681" s="1" t="inlineStr">
         <is>
-          <t>Ronaldo Dias</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I681" s="1" t="inlineStr">
@@ -52899,39 +52899,29 @@
         </is>
       </c>
       <c r="J681" s="2" t="n">
-        <v>46241.45808179398</v>
+        <v>46254.65888769676</v>
       </c>
       <c r="K681" s="2" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="L681" s="1" t="inlineStr">
         <is>
-          <t>Entregue Ao Solicitante</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M681" s="1" t="inlineStr">
         <is>
-          <t>Rodrigo Rego</t>
+          <t>Santos Karina</t>
         </is>
       </c>
       <c r="N681" s="1" t="n"/>
       <c r="O681" s="1" t="n"/>
-      <c r="P681" s="2" t="n">
-        <v>46241.7067102662</v>
-      </c>
-      <c r="Q681" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R681" s="1" t="inlineStr">
-        <is>
-          <t>Deve ser aberto um chamado por solicitação / cliente.</t>
-        </is>
-      </c>
+      <c r="P681" s="1" t="n"/>
+      <c r="Q681" s="1" t="inlineStr"/>
+      <c r="R681" s="1" t="inlineStr"/>
       <c r="S681" s="1" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="T681" s="1" t="n"/>
@@ -52939,39 +52929,39 @@
     </row>
     <row r="682">
       <c r="A682" s="1" t="n">
-        <v>82310</v>
+        <v>82053</v>
       </c>
       <c r="B682" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Ata de Reunião</t>
         </is>
       </c>
       <c r="C682" s="1" t="inlineStr">
         <is>
-          <t>Implantação Contábil</t>
+          <t>Inclusão de Ata</t>
         </is>
       </c>
       <c r="D682" s="1" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="E682" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
+          <t>6913	CL Comércio	MAED	Verificar pendência5254	RCL	MAED	Enviar guias para pagamento</t>
         </is>
       </c>
       <c r="F682" s="1" t="n">
-        <v>6974</v>
+        <v>6913</v>
       </c>
       <c r="G682" s="1" t="inlineStr">
         <is>
-          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
+          <t>CL COMERCIO VAREJISTA E ROTISSERIE LTDA</t>
         </is>
       </c>
       <c r="H682" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I682" s="1" t="inlineStr">
@@ -52980,35 +52970,39 @@
         </is>
       </c>
       <c r="J682" s="2" t="n">
-        <v>46247.3783179051</v>
+        <v>46241.45808179398</v>
       </c>
       <c r="K682" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="L682" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Entregue Ao Solicitante</t>
         </is>
       </c>
       <c r="M682" s="1" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
-        </is>
-      </c>
-      <c r="N682" s="2" t="n">
-        <v>46253.39089305556</v>
-      </c>
+          <t>Rodrigo Rego</t>
+        </is>
+      </c>
+      <c r="N682" s="1" t="n"/>
       <c r="O682" s="1" t="n"/>
-      <c r="P682" s="1" t="n"/>
-      <c r="Q682" s="1" t="inlineStr"/>
+      <c r="P682" s="2" t="n">
+        <v>46241.7067102662</v>
+      </c>
+      <c r="Q682" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
       <c r="R682" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t>Deve ser aberto um chamado por solicitação / cliente.</t>
         </is>
       </c>
       <c r="S682" s="1" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="T682" s="1" t="n"/>
@@ -53016,7 +53010,7 @@
     </row>
     <row r="683">
       <c r="A683" s="1" t="n">
-        <v>79867</v>
+        <v>82310</v>
       </c>
       <c r="B683" s="1" t="inlineStr">
         <is>
@@ -53035,20 +53029,20 @@
       </c>
       <c r="E683" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
+          <t>Bom dia!Por favor, solicitar ao antigo contador o balanço de abertura.</t>
         </is>
       </c>
       <c r="F683" s="1" t="n">
-        <v>6704</v>
+        <v>6974</v>
       </c>
       <c r="G683" s="1" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>FRANCINALDO FERREIRA DE ANDRADE LTDA</t>
         </is>
       </c>
       <c r="H683" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I683" s="1" t="inlineStr">
@@ -53057,10 +53051,10 @@
         </is>
       </c>
       <c r="J683" s="2" t="n">
-        <v>46183.62582114583</v>
+        <v>46247.3783179051</v>
       </c>
       <c r="K683" s="2" t="n">
-        <v>46185</v>
+        <v>46248</v>
       </c>
       <c r="L683" s="1" t="inlineStr">
         <is>
@@ -53073,15 +53067,14 @@
         </is>
       </c>
       <c r="N683" s="2" t="n">
-        <v>46237.4174340625</v>
+        <v>46253.39089305556</v>
       </c>
       <c r="O683" s="1" t="n"/>
       <c r="P683" s="1" t="n"/>
       <c r="Q683" s="1" t="inlineStr"/>
       <c r="R683" s="1" t="inlineStr">
         <is>
-          <t>Bom dia!
-Cobramos a antiga contabilidade.</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S683" s="1" t="inlineStr">
@@ -53094,16 +53087,16 @@
     </row>
     <row r="684">
       <c r="A684" s="1" t="n">
-        <v>79863</v>
+        <v>79867</v>
       </c>
       <c r="B684" s="1" t="inlineStr">
         <is>
-          <t>Arquivo</t>
+          <t>Auditoria</t>
         </is>
       </c>
       <c r="C684" s="1" t="inlineStr">
         <is>
-          <t>Solicitação de Documentos</t>
+          <t>Implantação Contábil</t>
         </is>
       </c>
       <c r="D684" s="1" t="inlineStr">
@@ -53113,20 +53106,20 @@
       </c>
       <c r="E684" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde!Por favor, solicitar ao antigo contador balanço abertura.</t>
         </is>
       </c>
       <c r="F684" s="1" t="n">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="G684" s="1" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="H684" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I684" s="1" t="inlineStr">
@@ -53135,14 +53128,14 @@
         </is>
       </c>
       <c r="J684" s="2" t="n">
-        <v>46183.6188202199</v>
+        <v>46183.62582114583</v>
       </c>
       <c r="K684" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L684" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M684" s="1" t="inlineStr">
@@ -53150,11 +53143,18 @@
           <t>Fernanda Araujo</t>
         </is>
       </c>
-      <c r="N684" s="1" t="n"/>
+      <c r="N684" s="2" t="n">
+        <v>46237.4174340625</v>
+      </c>
       <c r="O684" s="1" t="n"/>
       <c r="P684" s="1" t="n"/>
       <c r="Q684" s="1" t="inlineStr"/>
-      <c r="R684" s="1" t="inlineStr"/>
+      <c r="R684" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia!
+Cobramos a antiga contabilidade.</t>
+        </is>
+      </c>
       <c r="S684" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -53165,7 +53165,7 @@
     </row>
     <row r="685">
       <c r="A685" s="1" t="n">
-        <v>79865</v>
+        <v>79863</v>
       </c>
       <c r="B685" s="1" t="inlineStr">
         <is>
@@ -53184,15 +53184,15 @@
       </c>
       <c r="E685" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 31/08/2025, da empresa 6404.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F685" s="1" t="n">
-        <v>6278</v>
+        <v>6404</v>
       </c>
       <c r="G685" s="1" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="H685" s="1" t="inlineStr">
@@ -53206,7 +53206,7 @@
         </is>
       </c>
       <c r="J685" s="2" t="n">
-        <v>46183.62243564815</v>
+        <v>46183.6188202199</v>
       </c>
       <c r="K685" s="2" t="n">
         <v>46185</v>
@@ -53236,35 +53236,39 @@
     </row>
     <row r="686">
       <c r="A686" s="1" t="n">
-        <v>81422</v>
+        <v>79865</v>
       </c>
       <c r="B686" s="1" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Arquivo</t>
         </is>
       </c>
       <c r="C686" s="1" t="inlineStr">
         <is>
-          <t>Implantação DP</t>
+          <t>Solicitação de Documentos</t>
         </is>
       </c>
       <c r="D686" s="1" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="E686" s="1" t="inlineStr">
         <is>
-          <t>6990 - AMANCIO S ELETRICA (MATRIZ) - por gentileza providencias os documentos do Checklist.</t>
+          <t>Boa tarde! Por favor, preciso que seja solicitado ao antigo contador a ECD , de 01/01/2025 a 30/06/2025, da empresa 6278.A primeira solicitação foi feita por e-mail em 05/06.</t>
         </is>
       </c>
       <c r="F686" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G686" s="1" t="n"/>
+        <v>6278</v>
+      </c>
+      <c r="G686" s="1" t="inlineStr">
+        <is>
+          <t>EMPORIO DOS FRIOS LTDA</t>
+        </is>
+      </c>
       <c r="H686" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I686" s="1" t="inlineStr">
@@ -53273,118 +53277,104 @@
         </is>
       </c>
       <c r="J686" s="2" t="n">
-        <v>46226.70303271991</v>
+        <v>46183.62243564815</v>
       </c>
       <c r="K686" s="2" t="n">
-        <v>46230</v>
+        <v>46185</v>
       </c>
       <c r="L686" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M686" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N686" s="2" t="n">
-        <v>46230.39939193287</v>
-      </c>
+          <t>Fernanda Araujo</t>
+        </is>
+      </c>
+      <c r="N686" s="1" t="n"/>
       <c r="O686" s="1" t="n"/>
       <c r="P686" s="1" t="n"/>
       <c r="Q686" s="1" t="inlineStr"/>
-      <c r="R686" s="1" t="inlineStr">
+      <c r="R686" s="1" t="inlineStr"/>
+      <c r="S686" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T686" s="1" t="n"/>
+      <c r="U686" s="1" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" s="1" t="n">
+        <v>81422</v>
+      </c>
+      <c r="B687" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C687" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D687" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E687" s="1" t="inlineStr">
+        <is>
+          <t>6990 - AMANCIO S ELETRICA (MATRIZ) - por gentileza providencias os documentos do Checklist.</t>
+        </is>
+      </c>
+      <c r="F687" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G687" s="1" t="n"/>
+      <c r="H687" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="I687" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J687" s="2" t="n">
+        <v>46226.70303271991</v>
+      </c>
+      <c r="K687" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="L687" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M687" s="1" t="inlineStr">
+        <is>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N687" s="2" t="n">
+        <v>46230.39939193287</v>
+      </c>
+      <c r="O687" s="1" t="n"/>
+      <c r="P687" s="1" t="n"/>
+      <c r="Q687" s="1" t="inlineStr"/>
+      <c r="R687" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bom dia!
 Estou aguardando o contato do contador.
 </t>
         </is>
       </c>
-      <c r="S686" s="1" t="inlineStr">
+      <c r="S687" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
-        </is>
-      </c>
-      <c r="T686" s="1" t="n"/>
-      <c r="U686" s="1" t="inlineStr"/>
-    </row>
-    <row r="687">
-      <c r="A687" s="1" t="n">
-        <v>81901</v>
-      </c>
-      <c r="B687" s="1" t="inlineStr">
-        <is>
-          <t>Arquivo</t>
-        </is>
-      </c>
-      <c r="C687" s="1" t="inlineStr">
-        <is>
-          <t>Solicitação de Documentos</t>
-        </is>
-      </c>
-      <c r="D687" s="1" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="E687" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bom dia.Não localizei na pasta os contratos digitalizados.Poderiam, por gentileza, disponibilizar o arquivo da última alteração contratual das empresas 2459 – HERAEL e 2458 – SUPAMA?Obrigada. </t>
-        </is>
-      </c>
-      <c r="F687" s="1" t="n">
-        <v>2459</v>
-      </c>
-      <c r="G687" s="1" t="inlineStr">
-        <is>
-          <t>Herael Participações Ltda.</t>
-        </is>
-      </c>
-      <c r="H687" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="I687" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J687" s="2" t="n">
-        <v>46239.4584244213</v>
-      </c>
-      <c r="K687" s="2" t="n">
-        <v>46240</v>
-      </c>
-      <c r="L687" s="1" t="inlineStr">
-        <is>
-          <t>Entregue Ao Solicitante</t>
-        </is>
-      </c>
-      <c r="M687" s="1" t="inlineStr">
-        <is>
-          <t>Karine Gusmão</t>
-        </is>
-      </c>
-      <c r="N687" s="1" t="n"/>
-      <c r="O687" s="1" t="n"/>
-      <c r="P687" s="2" t="n">
-        <v>46240.66209961806</v>
-      </c>
-      <c r="Q687" s="1" t="inlineStr">
-        <is>
-          <t>Ronaldo Dias</t>
-        </is>
-      </c>
-      <c r="R687" s="1" t="inlineStr">
-        <is>
-          <t>Segue o que temos em arquivo.</t>
-        </is>
-      </c>
-      <c r="S687" s="1" t="inlineStr">
-        <is>
-          <t>SIM</t>
         </is>
       </c>
       <c r="T687" s="1" t="n"/>
@@ -53392,7 +53382,7 @@
     </row>
     <row r="688">
       <c r="A688" s="1" t="n">
-        <v>81714</v>
+        <v>81901</v>
       </c>
       <c r="B688" s="1" t="inlineStr">
         <is>
@@ -53411,20 +53401,20 @@
       </c>
       <c r="E688" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boa tarde.O cliente 2107 JMM solicitou o envio do Contrato Social da empresa, não localizei na pasta dos contratos digitalizados. Poderia verificar, por favor? Obrigada. </t>
+          <t xml:space="preserve">Bom dia.Não localizei na pasta os contratos digitalizados.Poderiam, por gentileza, disponibilizar o arquivo da última alteração contratual das empresas 2459 – HERAEL e 2458 – SUPAMA?Obrigada. </t>
         </is>
       </c>
       <c r="F688" s="1" t="n">
-        <v>2107</v>
+        <v>2459</v>
       </c>
       <c r="G688" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">JMM CARRASCOSA SOLUÇÕES EMPRESARIAIS LTDA </t>
+          <t>Herael Participações Ltda.</t>
         </is>
       </c>
       <c r="H688" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Ronaldo Dias</t>
         </is>
       </c>
       <c r="I688" s="1" t="inlineStr">
@@ -53433,10 +53423,10 @@
         </is>
       </c>
       <c r="J688" s="2" t="n">
-        <v>46234.61626284722</v>
+        <v>46239.4584244213</v>
       </c>
       <c r="K688" s="2" t="n">
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="L688" s="1" t="inlineStr">
         <is>
@@ -53451,95 +53441,103 @@
       <c r="N688" s="1" t="n"/>
       <c r="O688" s="1" t="n"/>
       <c r="P688" s="2" t="n">
+        <v>46240.66209961806</v>
+      </c>
+      <c r="Q688" s="1" t="inlineStr">
+        <is>
+          <t>Ronaldo Dias</t>
+        </is>
+      </c>
+      <c r="R688" s="1" t="inlineStr">
+        <is>
+          <t>Segue o que temos em arquivo.</t>
+        </is>
+      </c>
+      <c r="S688" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T688" s="1" t="n"/>
+      <c r="U688" s="1" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" s="1" t="n">
+        <v>81714</v>
+      </c>
+      <c r="B689" s="1" t="inlineStr">
+        <is>
+          <t>Arquivo</t>
+        </is>
+      </c>
+      <c r="C689" s="1" t="inlineStr">
+        <is>
+          <t>Solicitação de Documentos</t>
+        </is>
+      </c>
+      <c r="D689" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E689" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde.O cliente 2107 JMM solicitou o envio do Contrato Social da empresa, não localizei na pasta dos contratos digitalizados. Poderia verificar, por favor? Obrigada. </t>
+        </is>
+      </c>
+      <c r="F689" s="1" t="n">
+        <v>2107</v>
+      </c>
+      <c r="G689" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JMM CARRASCOSA SOLUÇÕES EMPRESARIAIS LTDA </t>
+        </is>
+      </c>
+      <c r="H689" s="1" t="inlineStr">
+        <is>
+          <t>Karina Dantas</t>
+        </is>
+      </c>
+      <c r="I689" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J689" s="2" t="n">
+        <v>46234.61626284722</v>
+      </c>
+      <c r="K689" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="L689" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M689" s="1" t="inlineStr">
+        <is>
+          <t>Karine Gusmão</t>
+        </is>
+      </c>
+      <c r="N689" s="1" t="n"/>
+      <c r="O689" s="1" t="n"/>
+      <c r="P689" s="2" t="n">
         <v>46237.4136784375</v>
       </c>
-      <c r="Q688" s="1" t="inlineStr">
+      <c r="Q689" s="1" t="inlineStr">
         <is>
           <t>Karina Dantas</t>
         </is>
       </c>
-      <c r="R688" s="1" t="inlineStr">
+      <c r="R689" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bom dia!
 Não temos o contrato social da JMM. </t>
         </is>
       </c>
-      <c r="S688" s="1" t="inlineStr">
+      <c r="S689" s="1" t="inlineStr">
         <is>
           <t>SIM</t>
-        </is>
-      </c>
-      <c r="T688" s="1" t="n"/>
-      <c r="U688" s="1" t="inlineStr"/>
-    </row>
-    <row r="689">
-      <c r="A689" s="1" t="n">
-        <v>82699</v>
-      </c>
-      <c r="B689" s="1" t="inlineStr">
-        <is>
-          <t>Auditoria</t>
-        </is>
-      </c>
-      <c r="C689" s="1" t="inlineStr">
-        <is>
-          <t>Implantação DP</t>
-        </is>
-      </c>
-      <c r="D689" s="1" t="inlineStr">
-        <is>
-          <t>DP - DEPTO. PESSOAL</t>
-        </is>
-      </c>
-      <c r="E689" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Boa tarde, por gentileza, solicitar documentos para implantação da empresa 6872 - F. MARQUESItens dispensáveis, por gentileza, sinalizar. </t>
-        </is>
-      </c>
-      <c r="F689" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G689" s="1" t="n"/>
-      <c r="H689" s="1" t="inlineStr">
-        <is>
-          <t>Edney Xavier</t>
-        </is>
-      </c>
-      <c r="I689" s="1" t="inlineStr">
-        <is>
-          <t>PL - AUDITORIA</t>
-        </is>
-      </c>
-      <c r="J689" s="2" t="n">
-        <v>46253.70661435185</v>
-      </c>
-      <c r="K689" s="2" t="n">
-        <v>46255</v>
-      </c>
-      <c r="L689" s="1" t="inlineStr">
-        <is>
-          <t>Em Atendimento</t>
-        </is>
-      </c>
-      <c r="M689" s="1" t="inlineStr">
-        <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N689" s="2" t="n">
-        <v>46255.4431121875</v>
-      </c>
-      <c r="O689" s="1" t="n"/>
-      <c r="P689" s="1" t="n"/>
-      <c r="Q689" s="1" t="inlineStr"/>
-      <c r="R689" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cobramos novamente os documentos </t>
-        </is>
-      </c>
-      <c r="S689" s="1" t="inlineStr">
-        <is>
-          <t>NÃO</t>
         </is>
       </c>
       <c r="T689" s="1" t="n"/>
@@ -53547,7 +53545,7 @@
     </row>
     <row r="690">
       <c r="A690" s="1" t="n">
-        <v>82700</v>
+        <v>82699</v>
       </c>
       <c r="B690" s="1" t="inlineStr">
         <is>
@@ -53566,7 +53564,7 @@
       </c>
       <c r="E690" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 7036 - VIASUPRIItens dispensáveis, por gentileza, sinalizar.</t>
+          <t xml:space="preserve">Boa tarde, por gentileza, solicitar documentos para implantação da empresa 6872 - F. MARQUESItens dispensáveis, por gentileza, sinalizar. </t>
         </is>
       </c>
       <c r="F690" s="1" t="n">
@@ -53584,7 +53582,7 @@
         </is>
       </c>
       <c r="J690" s="2" t="n">
-        <v>46253.71050454861</v>
+        <v>46253.70661435185</v>
       </c>
       <c r="K690" s="2" t="n">
         <v>46255</v>
@@ -53600,14 +53598,14 @@
         </is>
       </c>
       <c r="N690" s="2" t="n">
-        <v>46255.46871099537</v>
+        <v>46255.4431121875</v>
       </c>
       <c r="O690" s="1" t="n"/>
       <c r="P690" s="1" t="n"/>
       <c r="Q690" s="1" t="inlineStr"/>
       <c r="R690" s="1" t="inlineStr">
         <is>
-          <t>Cobramos os documentos das duas empresas</t>
+          <t xml:space="preserve">Cobramos novamente os documentos </t>
         </is>
       </c>
       <c r="S690" s="1" t="inlineStr">
@@ -53620,7 +53618,7 @@
     </row>
     <row r="691">
       <c r="A691" s="1" t="n">
-        <v>82701</v>
+        <v>82700</v>
       </c>
       <c r="B691" s="1" t="inlineStr">
         <is>
@@ -53639,7 +53637,7 @@
       </c>
       <c r="E691" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providencias documentos de implantação da empresa: 7037 - EXPANDItens dispensáveis, por gentileza, sinalizar.</t>
+          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 7036 - VIASUPRIItens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F691" s="1" t="n">
@@ -53657,7 +53655,7 @@
         </is>
       </c>
       <c r="J691" s="2" t="n">
-        <v>46253.71124814815</v>
+        <v>46253.71050454861</v>
       </c>
       <c r="K691" s="2" t="n">
         <v>46255</v>
@@ -53673,14 +53671,14 @@
         </is>
       </c>
       <c r="N691" s="2" t="n">
-        <v>46255.46909065972</v>
+        <v>46255.46871099537</v>
       </c>
       <c r="O691" s="1" t="n"/>
       <c r="P691" s="1" t="n"/>
       <c r="Q691" s="1" t="inlineStr"/>
       <c r="R691" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CObramos os documentos </t>
+          <t>Cobramos os documentos das duas empresas</t>
         </is>
       </c>
       <c r="S691" s="1" t="inlineStr">
@@ -53693,7 +53691,7 @@
     </row>
     <row r="692">
       <c r="A692" s="1" t="n">
-        <v>82704</v>
+        <v>82701</v>
       </c>
       <c r="B692" s="1" t="inlineStr">
         <is>
@@ -53712,7 +53710,7 @@
       </c>
       <c r="E692" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar os documentos de implantação para a empresa: 6812 - DANIEL DE JESUSItens dispensáveis, por gentileza, sinalizar.</t>
+          <t>Boa tarde, por gentileza, providencias documentos de implantação da empresa: 7037 - EXPANDItens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F692" s="1" t="n">
@@ -53730,14 +53728,14 @@
         </is>
       </c>
       <c r="J692" s="2" t="n">
-        <v>46253.71813614584</v>
+        <v>46253.71124814815</v>
       </c>
       <c r="K692" s="2" t="n">
         <v>46255</v>
       </c>
       <c r="L692" s="1" t="inlineStr">
         <is>
-          <t>Esperando Atendimento</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M692" s="1" t="inlineStr">
@@ -53745,11 +53743,17 @@
           <t>Santos Karina</t>
         </is>
       </c>
-      <c r="N692" s="1" t="n"/>
+      <c r="N692" s="2" t="n">
+        <v>46255.46909065972</v>
+      </c>
       <c r="O692" s="1" t="n"/>
       <c r="P692" s="1" t="n"/>
       <c r="Q692" s="1" t="inlineStr"/>
-      <c r="R692" s="1" t="inlineStr"/>
+      <c r="R692" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CObramos os documentos </t>
+        </is>
+      </c>
       <c r="S692" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -53760,7 +53764,7 @@
     </row>
     <row r="693">
       <c r="A693" s="1" t="n">
-        <v>82706</v>
+        <v>82704</v>
       </c>
       <c r="B693" s="1" t="inlineStr">
         <is>
@@ -53779,7 +53783,7 @@
       </c>
       <c r="E693" s="1" t="inlineStr">
         <is>
-          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 6978 - HEPA FILTROS.Itens dispensáveis, por gentileza, sinalizar.</t>
+          <t>Boa tarde, por gentileza, providenciar os documentos de implantação para a empresa: 6812 - DANIEL DE JESUSItens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F693" s="1" t="n">
@@ -53797,14 +53801,14 @@
         </is>
       </c>
       <c r="J693" s="2" t="n">
-        <v>46253.72086076389</v>
+        <v>46253.71813614584</v>
       </c>
       <c r="K693" s="2" t="n">
         <v>46255</v>
       </c>
       <c r="L693" s="1" t="inlineStr">
         <is>
-          <t>Devolvido para Responsável</t>
+          <t>Esperando Atendimento</t>
         </is>
       </c>
       <c r="M693" s="1" t="inlineStr">
@@ -53816,11 +53820,7 @@
       <c r="O693" s="1" t="n"/>
       <c r="P693" s="1" t="n"/>
       <c r="Q693" s="1" t="inlineStr"/>
-      <c r="R693" s="1" t="inlineStr">
-        <is>
-          <t>cobramos os documentos.</t>
-        </is>
-      </c>
+      <c r="R693" s="1" t="inlineStr"/>
       <c r="S693" s="1" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -53831,7 +53831,7 @@
     </row>
     <row r="694">
       <c r="A694" s="1" t="n">
-        <v>81244</v>
+        <v>82706</v>
       </c>
       <c r="B694" s="1" t="inlineStr">
         <is>
@@ -53850,7 +53850,7 @@
       </c>
       <c r="E694" s="1" t="inlineStr">
         <is>
-          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
+          <t>Boa tarde, por gentileza, providenciar documentos de implantação da empresa: 6978 - HEPA FILTROS.Itens dispensáveis, por gentileza, sinalizar.</t>
         </is>
       </c>
       <c r="F694" s="1" t="n">
@@ -53859,7 +53859,7 @@
       <c r="G694" s="1" t="n"/>
       <c r="H694" s="1" t="inlineStr">
         <is>
-          <t>Karina Dantas</t>
+          <t>Edney Xavier</t>
         </is>
       </c>
       <c r="I694" s="1" t="inlineStr">
@@ -53868,30 +53868,28 @@
         </is>
       </c>
       <c r="J694" s="2" t="n">
-        <v>46224.42615887732</v>
+        <v>46253.72086076389</v>
       </c>
       <c r="K694" s="2" t="n">
-        <v>46226</v>
+        <v>46255</v>
       </c>
       <c r="L694" s="1" t="inlineStr">
         <is>
-          <t>Em Atendimento</t>
+          <t>Devolvido para Responsável</t>
         </is>
       </c>
       <c r="M694" s="1" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
-      <c r="N694" s="2" t="n">
-        <v>46225.4986497338</v>
-      </c>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N694" s="1" t="n"/>
       <c r="O694" s="1" t="n"/>
       <c r="P694" s="1" t="n"/>
       <c r="Q694" s="1" t="inlineStr"/>
       <c r="R694" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aguardando contato do contador. </t>
+          <t>cobramos os documentos.</t>
         </is>
       </c>
       <c r="S694" s="1" t="inlineStr">
@@ -53904,7 +53902,7 @@
     </row>
     <row r="695">
       <c r="A695" s="1" t="n">
-        <v>81247</v>
+        <v>81244</v>
       </c>
       <c r="B695" s="1" t="inlineStr">
         <is>
@@ -53923,7 +53921,7 @@
       </c>
       <c r="E695" s="1" t="inlineStr">
         <is>
-          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
+          <t>6966 - HELBRAZ COMERCIO DE PAPELARIA LTDA6967 - JL DISTRIBUIDORA DE PAPELARIA LTDAPor gentileza, providenciar as documentações de implantação das empresas, anexo o checklist.</t>
         </is>
       </c>
       <c r="F695" s="1" t="n">
@@ -53941,7 +53939,7 @@
         </is>
       </c>
       <c r="J695" s="2" t="n">
-        <v>46224.43143758102</v>
+        <v>46224.42615887732</v>
       </c>
       <c r="K695" s="2" t="n">
         <v>46226</v>
@@ -53957,14 +53955,14 @@
         </is>
       </c>
       <c r="N695" s="2" t="n">
-        <v>46225.49170355324</v>
+        <v>46225.4986497338</v>
       </c>
       <c r="O695" s="1" t="n"/>
       <c r="P695" s="1" t="n"/>
       <c r="Q695" s="1" t="inlineStr"/>
       <c r="R695" s="1" t="inlineStr">
         <is>
-          <t>Aguardando os dados do contador.</t>
+          <t xml:space="preserve">Aguardando contato do contador. </t>
         </is>
       </c>
       <c r="S695" s="1" t="inlineStr">
@@ -53977,7 +53975,7 @@
     </row>
     <row r="696">
       <c r="A696" s="1" t="n">
-        <v>81052</v>
+        <v>81247</v>
       </c>
       <c r="B696" s="1" t="inlineStr">
         <is>
@@ -53996,7 +53994,7 @@
       </c>
       <c r="E696" s="1" t="inlineStr">
         <is>
-          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
+          <t>6976 - FILM FACIL LTDA6977 - PROTECTION SHIELD LTDAPor gentileza providenciar as documentações de implantação, anexo o checklist.</t>
         </is>
       </c>
       <c r="F696" s="1" t="n">
@@ -54005,7 +54003,7 @@
       <c r="G696" s="1" t="n"/>
       <c r="H696" s="1" t="inlineStr">
         <is>
-          <t>Edney Xavier</t>
+          <t>Karina Dantas</t>
         </is>
       </c>
       <c r="I696" s="1" t="inlineStr">
@@ -54014,10 +54012,10 @@
         </is>
       </c>
       <c r="J696" s="2" t="n">
-        <v>46218.38736744213</v>
+        <v>46224.43143758102</v>
       </c>
       <c r="K696" s="2" t="n">
-        <v>46219</v>
+        <v>46226</v>
       </c>
       <c r="L696" s="1" t="inlineStr">
         <is>
@@ -54030,14 +54028,14 @@
         </is>
       </c>
       <c r="N696" s="2" t="n">
-        <v>46219.50471747686</v>
+        <v>46225.49170355324</v>
       </c>
       <c r="O696" s="1" t="n"/>
       <c r="P696" s="1" t="n"/>
       <c r="Q696" s="1" t="inlineStr"/>
       <c r="R696" s="1" t="inlineStr">
         <is>
-          <t>cobramos os documentos do antigo contador.</t>
+          <t>Aguardando os dados do contador.</t>
         </is>
       </c>
       <c r="S696" s="1" t="inlineStr">
@@ -54050,7 +54048,7 @@
     </row>
     <row r="697">
       <c r="A697" s="1" t="n">
-        <v>81055</v>
+        <v>81052</v>
       </c>
       <c r="B697" s="1" t="inlineStr">
         <is>
@@ -54069,7 +54067,7 @@
       </c>
       <c r="E697" s="1" t="inlineStr">
         <is>
-          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
+          <t>Por gentileza, providenciar os documentos pendentes no checklist anexo com urgência, já estamos no dia 15/07 e não recebemos nenhuma documentação, o atendimento ao cliente está prejudicado.</t>
         </is>
       </c>
       <c r="F697" s="1" t="n">
@@ -54087,7 +54085,7 @@
         </is>
       </c>
       <c r="J697" s="2" t="n">
-        <v>46218.40379614583</v>
+        <v>46218.38736744213</v>
       </c>
       <c r="K697" s="2" t="n">
         <v>46219</v>
@@ -54103,14 +54101,14 @@
         </is>
       </c>
       <c r="N697" s="2" t="n">
-        <v>46219.50607847222</v>
+        <v>46219.50471747686</v>
       </c>
       <c r="O697" s="1" t="n"/>
       <c r="P697" s="1" t="n"/>
       <c r="Q697" s="1" t="inlineStr"/>
       <c r="R697" s="1" t="inlineStr">
         <is>
-          <t>Aguardando retorno dos dados do contador</t>
+          <t>cobramos os documentos do antigo contador.</t>
         </is>
       </c>
       <c r="S697" s="1" t="inlineStr">
@@ -54123,7 +54121,7 @@
     </row>
     <row r="698">
       <c r="A698" s="1" t="n">
-        <v>82430</v>
+        <v>81055</v>
       </c>
       <c r="B698" s="1" t="inlineStr">
         <is>
@@ -54142,7 +54140,7 @@
       </c>
       <c r="E698" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bom dia!Segue checklist atualizado da empresa 7007 - SANTOS&amp;DIAN Itens dispensáveis, por gentileza, sinalizar. </t>
+          <t>6984 - SUPERMERCADOS BANDEIRA LTDA6985 - T F MIRANDA MERCADO LTDAPor gentileza, providenciar as documentações de implantação com urgência, cliente com grande quantidade de funcionários.</t>
         </is>
       </c>
       <c r="F698" s="1" t="n">
@@ -54160,28 +54158,30 @@
         </is>
       </c>
       <c r="J698" s="2" t="n">
-        <v>46248.47311612269</v>
+        <v>46218.40379614583</v>
       </c>
       <c r="K698" s="2" t="n">
-        <v>46251</v>
+        <v>46219</v>
       </c>
       <c r="L698" s="1" t="inlineStr">
         <is>
-          <t>Devolvido</t>
+          <t>Em Atendimento</t>
         </is>
       </c>
       <c r="M698" s="1" t="inlineStr">
         <is>
-          <t>Santos Karina</t>
-        </is>
-      </c>
-      <c r="N698" s="1" t="n"/>
+          <t>Gabriela Peres</t>
+        </is>
+      </c>
+      <c r="N698" s="2" t="n">
+        <v>46219.50607847222</v>
+      </c>
       <c r="O698" s="1" t="n"/>
       <c r="P698" s="1" t="n"/>
       <c r="Q698" s="1" t="inlineStr"/>
       <c r="R698" s="1" t="inlineStr">
         <is>
-          <t>cobramos novamente o antigo contador</t>
+          <t>Aguardando retorno dos dados do contador</t>
         </is>
       </c>
       <c r="S698" s="1" t="inlineStr">
@@ -54191,6 +54191,77 @@
       </c>
       <c r="T698" s="1" t="n"/>
       <c r="U698" s="1" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="1" t="n">
+        <v>82430</v>
+      </c>
+      <c r="B699" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="C699" s="1" t="inlineStr">
+        <is>
+          <t>Implantação DP</t>
+        </is>
+      </c>
+      <c r="D699" s="1" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="E699" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bom dia!Segue checklist atualizado da empresa 7007 - SANTOS&amp;DIAN Itens dispensáveis, por gentileza, sinalizar. </t>
+        </is>
+      </c>
+      <c r="F699" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G699" s="1" t="n"/>
+      <c r="H699" s="1" t="inlineStr">
+        <is>
+          <t>Edney Xavier</t>
+        </is>
+      </c>
+      <c r="I699" s="1" t="inlineStr">
+        <is>
+          <t>PL - AUDITORIA</t>
+        </is>
+      </c>
+      <c r="J699" s="2" t="n">
+        <v>46248.47311612269</v>
+      </c>
+      <c r="K699" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="L699" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido</t>
+        </is>
+      </c>
+      <c r="M699" s="1" t="inlineStr">
+        <is>
+          <t>Santos Karina</t>
+        </is>
+      </c>
+      <c r="N699" s="1" t="n"/>
+      <c r="O699" s="1" t="n"/>
+      <c r="P699" s="1" t="n"/>
+      <c r="Q699" s="1" t="inlineStr"/>
+      <c r="R699" s="1" t="inlineStr">
+        <is>
+          <t>cobramos novamente o antigo contador</t>
+        </is>
+      </c>
+      <c r="S699" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T699" s="1" t="n"/>
+      <c r="U699" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-09-11 12:00
</commit_message>
<xml_diff>
--- a/data/base.xlsx
+++ b/data/base.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U794" headerRowCount="1">
-  <autoFilter ref="A1:U794"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela2" displayName="Tabela2" ref="A1:U818" headerRowCount="1">
+  <autoFilter ref="A1:U818"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Categoria"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U794"/>
+  <dimension ref="A1:U818"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60940,6 +60940,1901 @@
       <c r="T794" s="1" t="n"/>
       <c r="U794" s="1" t="inlineStr"/>
     </row>
+    <row r="795">
+      <c r="A795" s="1" t="n">
+        <v>82881</v>
+      </c>
+      <c r="B795" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C795" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D795" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E795" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados, bom dia.Estou formalizando, via chamado, a solicitação de revisão do cadastro de produtos da empresa.Em anexo, encaminho o e-mail com a tratativa referente ao assunto. </t>
+        </is>
+      </c>
+      <c r="F795" s="1" t="n">
+        <v>6336</v>
+      </c>
+      <c r="G795" s="1" t="inlineStr">
+        <is>
+          <t>BEL LINE COMERCIO DE COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="H795" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I795" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J795" s="2" t="n">
+        <v>46258.42822939815</v>
+      </c>
+      <c r="K795" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="L795" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M795" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N795" s="1" t="n"/>
+      <c r="O795" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P795" s="2" t="n">
+        <v>46265.43684837963</v>
+      </c>
+      <c r="Q795" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R795" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia 
+Cadastro analisado e enviado por email</t>
+        </is>
+      </c>
+      <c r="S795" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T795" s="1" t="n"/>
+      <c r="U795" s="1" t="inlineStr"/>
+    </row>
+    <row r="796">
+      <c r="A796" s="1" t="n">
+        <v>81757</v>
+      </c>
+      <c r="B796" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C796" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D796" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E796" s="1" t="inlineStr">
+        <is>
+          <t>6945 - BRASIL DISTRIBUIDORA DE PEÇAS - CADASTRO DE INTENS, PARA INCLUSÃO DE INFORMAÇÕES TRIBUTÁRIAS.Por favor dar início na inclusão das informações tributarias no cadastro de itens do clienteAtt.Vander</t>
+        </is>
+      </c>
+      <c r="F796" s="1" t="n">
+        <v>6945</v>
+      </c>
+      <c r="G796" s="1" t="inlineStr">
+        <is>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+        </is>
+      </c>
+      <c r="H796" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I796" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J796" s="2" t="n">
+        <v>46237.52224869213</v>
+      </c>
+      <c r="K796" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="L796" s="1" t="inlineStr">
+        <is>
+          <t>Devolvido</t>
+        </is>
+      </c>
+      <c r="M796" s="1" t="inlineStr">
+        <is>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N796" s="1" t="n"/>
+      <c r="O796" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="P796" s="1" t="n"/>
+      <c r="Q796" s="1" t="inlineStr"/>
+      <c r="R796" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por favor , enviar a planilha de cadastro no layout padrão para analise 
+Enviar a planilha no layout correto e abrir novo chamado anexando email </t>
+        </is>
+      </c>
+      <c r="S796" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T796" s="1" t="n"/>
+      <c r="U796" s="1" t="inlineStr"/>
+    </row>
+    <row r="797">
+      <c r="A797" s="1" t="n">
+        <v>82777</v>
+      </c>
+      <c r="B797" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C797" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D797" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC</t>
+        </is>
+      </c>
+      <c r="E797" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, bom dia!Enviei um e-mail sobre a solicitação da Jéssica sobre o cliente JEM TRUCK.Por favor verificar e validar se chegam a mesma conclusão antes de envio ao cliente.</t>
+        </is>
+      </c>
+      <c r="F797" s="1" t="n">
+        <v>6979</v>
+      </c>
+      <c r="G797" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JEM TRUCK TRANSPORTE DE CARGAS E TERRAPLANAGEM LTDA </t>
+        </is>
+      </c>
+      <c r="H797" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I797" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J797" s="2" t="n">
+        <v>46255.4226837963</v>
+      </c>
+      <c r="K797" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="L797" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M797" s="1" t="inlineStr">
+        <is>
+          <t>Maicon Costa</t>
+        </is>
+      </c>
+      <c r="N797" s="1" t="n"/>
+      <c r="O797" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="P797" s="2" t="n">
+        <v>46262.63475393518</v>
+      </c>
+      <c r="Q797" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R797" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boa tarde 
+Informação já respondida por email
+Assuntos sobre duvidas tributarias, não deve ser aberto chamado </t>
+        </is>
+      </c>
+      <c r="S797" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T797" s="1" t="n"/>
+      <c r="U797" s="1" t="inlineStr"/>
+    </row>
+    <row r="798">
+      <c r="A798" s="1" t="n">
+        <v>82815</v>
+      </c>
+      <c r="B798" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C798" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D798" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E798" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F798" s="1" t="n">
+        <v>5789</v>
+      </c>
+      <c r="G798" s="1" t="inlineStr">
+        <is>
+          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
+        </is>
+      </c>
+      <c r="H798" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I798" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J798" s="2" t="n">
+        <v>46255.67638510417</v>
+      </c>
+      <c r="K798" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L798" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M798" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N798" s="2" t="n">
+        <v>46262.65963637731</v>
+      </c>
+      <c r="O798" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P798" s="2" t="n">
+        <v>46266.5932252662</v>
+      </c>
+      <c r="Q798" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R798" s="1" t="inlineStr">
+        <is>
+          <t>Em fila para atendimento</t>
+        </is>
+      </c>
+      <c r="S798" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T798" s="1" t="n"/>
+      <c r="U798" s="1" t="inlineStr"/>
+    </row>
+    <row r="799">
+      <c r="A799" s="1" t="n">
+        <v>82817</v>
+      </c>
+      <c r="B799" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C799" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D799" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E799" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F799" s="1" t="n">
+        <v>3808</v>
+      </c>
+      <c r="G799" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mercearia Doce Bom Ltda. </t>
+        </is>
+      </c>
+      <c r="H799" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I799" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J799" s="2" t="n">
+        <v>46255.6791724537</v>
+      </c>
+      <c r="K799" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L799" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M799" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N799" s="1" t="n"/>
+      <c r="O799" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P799" s="2" t="n">
+        <v>46262.65880697917</v>
+      </c>
+      <c r="Q799" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R799" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde
+Cadastro analisado e devolvido por email em 24/08</t>
+        </is>
+      </c>
+      <c r="S799" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T799" s="1" t="n"/>
+      <c r="U799" s="1" t="inlineStr"/>
+    </row>
+    <row r="800">
+      <c r="A800" s="1" t="n">
+        <v>82818</v>
+      </c>
+      <c r="B800" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C800" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D800" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E800" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F800" s="1" t="n">
+        <v>4222</v>
+      </c>
+      <c r="G800" s="1" t="inlineStr">
+        <is>
+          <t>STOCK FRANGO DISTRIBUIDORA DE GÊNEROS ALIMENTÍCIOS E TRANSPORTE LTDA</t>
+        </is>
+      </c>
+      <c r="H800" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I800" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J800" s="2" t="n">
+        <v>46255.67973850694</v>
+      </c>
+      <c r="K800" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L800" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M800" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N800" s="1" t="n"/>
+      <c r="O800" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P800" s="2" t="n">
+        <v>46262.65957361111</v>
+      </c>
+      <c r="Q800" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R800" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde 
+Cadastro analisado e enviado por email em 24/08</t>
+        </is>
+      </c>
+      <c r="S800" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T800" s="1" t="n"/>
+      <c r="U800" s="1" t="inlineStr"/>
+    </row>
+    <row r="801">
+      <c r="A801" s="1" t="n">
+        <v>82819</v>
+      </c>
+      <c r="B801" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C801" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D801" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E801" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F801" s="1" t="n">
+        <v>6529</v>
+      </c>
+      <c r="G801" s="1" t="inlineStr">
+        <is>
+          <t>VALLEMAR MERCADO LTDA</t>
+        </is>
+      </c>
+      <c r="H801" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I801" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J801" s="2" t="n">
+        <v>46255.68034375</v>
+      </c>
+      <c r="K801" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="L801" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M801" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N801" s="1" t="n"/>
+      <c r="O801" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P801" s="2" t="n">
+        <v>46262.66115917824</v>
+      </c>
+      <c r="Q801" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R801" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde 
+Cadastro analisado e devolvido por email em 24/08</t>
+        </is>
+      </c>
+      <c r="S801" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T801" s="1" t="n"/>
+      <c r="U801" s="1" t="inlineStr"/>
+    </row>
+    <row r="802">
+      <c r="A802" s="1" t="n">
+        <v>82901</v>
+      </c>
+      <c r="B802" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C802" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D802" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E802" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F802" s="1" t="n">
+        <v>4604</v>
+      </c>
+      <c r="G802" s="1" t="inlineStr">
+        <is>
+          <t>H P T COMERCIO E INDUSTRIA DE MÓVEIS LTDA</t>
+        </is>
+      </c>
+      <c r="H802" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I802" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J802" s="2" t="n">
+        <v>46258.64696304398</v>
+      </c>
+      <c r="K802" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="L802" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M802" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N802" s="2" t="n">
+        <v>46265.43650153935</v>
+      </c>
+      <c r="O802" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P802" s="2" t="n">
+        <v>46266.6452650463</v>
+      </c>
+      <c r="Q802" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R802" s="1" t="inlineStr">
+        <is>
+          <t>Na fila para atendimento</t>
+        </is>
+      </c>
+      <c r="S802" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T802" s="1" t="n"/>
+      <c r="U802" s="1" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" s="1" t="n">
+        <v>82924</v>
+      </c>
+      <c r="B803" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C803" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D803" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E803" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F803" s="1" t="n">
+        <v>5739</v>
+      </c>
+      <c r="G803" s="1" t="inlineStr">
+        <is>
+          <t>GOLD REAL MOVEIS LTDA</t>
+        </is>
+      </c>
+      <c r="H803" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I803" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J803" s="2" t="n">
+        <v>46258.73919143518</v>
+      </c>
+      <c r="K803" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="L803" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M803" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N803" s="2" t="n">
+        <v>46265.44787318287</v>
+      </c>
+      <c r="O803" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="P803" s="2" t="n">
+        <v>46266.64227896991</v>
+      </c>
+      <c r="Q803" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R803" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Em fila de atendimento </t>
+        </is>
+      </c>
+      <c r="S803" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T803" s="1" t="n"/>
+      <c r="U803" s="1" t="inlineStr"/>
+    </row>
+    <row r="804">
+      <c r="A804" s="1" t="n">
+        <v>82951</v>
+      </c>
+      <c r="B804" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C804" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D804" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E804" s="1" t="inlineStr">
+        <is>
+          <t>Bom dia, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F804" s="1" t="n">
+        <v>3959</v>
+      </c>
+      <c r="G804" s="1" t="inlineStr">
+        <is>
+          <t>ALDEBARAN DISTRIBUIDORA E COMÉRCIO DE MATERIAL MÉDICO E HOSPITALAR LTDA</t>
+        </is>
+      </c>
+      <c r="H804" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I804" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J804" s="2" t="n">
+        <v>46259.43735</v>
+      </c>
+      <c r="K804" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="L804" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M804" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N804" s="2" t="n">
+        <v>46265.45876041667</v>
+      </c>
+      <c r="O804" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="P804" s="1" t="n"/>
+      <c r="Q804" s="1" t="inlineStr"/>
+      <c r="R804" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Em fila de atendimento </t>
+        </is>
+      </c>
+      <c r="S804" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T804" s="1" t="n"/>
+      <c r="U804" s="1" t="inlineStr"/>
+    </row>
+    <row r="805">
+      <c r="A805" s="1" t="n">
+        <v>83005</v>
+      </c>
+      <c r="B805" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C805" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D805" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E805" s="1" t="inlineStr">
+        <is>
+          <t>Boa tarde, segue em anexo cadastro de produtos da empresa para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F805" s="1" t="n">
+        <v>6523</v>
+      </c>
+      <c r="G805" s="1" t="inlineStr">
+        <is>
+          <t>PARADA DOS PAES LTDA</t>
+        </is>
+      </c>
+      <c r="H805" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I805" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J805" s="2" t="n">
+        <v>46259.70646643519</v>
+      </c>
+      <c r="K805" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="L805" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M805" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N805" s="2" t="n">
+        <v>46265.51365540509</v>
+      </c>
+      <c r="O805" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="P805" s="2" t="n">
+        <v>46268.69805833334</v>
+      </c>
+      <c r="Q805" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R805" s="1" t="inlineStr">
+        <is>
+          <t>Em fila de atendimento</t>
+        </is>
+      </c>
+      <c r="S805" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T805" s="1" t="n"/>
+      <c r="U805" s="1" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" s="1" t="n">
+        <v>82502</v>
+      </c>
+      <c r="B806" s="1" t="inlineStr">
+        <is>
+          <t>Ata de Reunião</t>
+        </is>
+      </c>
+      <c r="C806" s="1" t="inlineStr">
+        <is>
+          <t>Inclusão de Ata</t>
+        </is>
+      </c>
+      <c r="D806" s="1" t="inlineStr">
+        <is>
+          <t>GC - ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E806" s="1" t="inlineStr">
+        <is>
+          <t>6070	MEGACAR	Cliente informou que já enviou o cadastro de produto, por favor verificar se já foi revisado e devolvido para o cliente. Como esta o andamento?</t>
+        </is>
+      </c>
+      <c r="F806" s="1" t="n">
+        <v>6070</v>
+      </c>
+      <c r="G806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEGACAR DISTRIBUIDORA AUTOMOTIVA LTDA </t>
+        </is>
+      </c>
+      <c r="H806" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I806" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J806" s="2" t="n">
+        <v>46251.42708194444</v>
+      </c>
+      <c r="K806" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="L806" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M806" s="1" t="inlineStr">
+        <is>
+          <t>Leticia Queiroz</t>
+        </is>
+      </c>
+      <c r="N806" s="1" t="n"/>
+      <c r="O806" s="1" t="n"/>
+      <c r="P806" s="2" t="n">
+        <v>46261.54547850695</v>
+      </c>
+      <c r="Q806" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R806" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Em 2026, não recebemos nenhuma solicitação referente a esse cliente 
+Por favor, solicitar o cadastro de produtos atualizado, enviar por email para @integracaocadastroechat e abrir novo chamado </t>
+        </is>
+      </c>
+      <c r="S806" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T806" s="1" t="n"/>
+      <c r="U806" s="1" t="inlineStr"/>
+    </row>
+    <row r="807">
+      <c r="A807" s="1" t="n">
+        <v>83231</v>
+      </c>
+      <c r="B807" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C807" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D807" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E807" s="1" t="inlineStr">
+        <is>
+          <t>Por gentileza, realizar a analise do cadastro dos produtos anexo.</t>
+        </is>
+      </c>
+      <c r="F807" s="1" t="n">
+        <v>4469</v>
+      </c>
+      <c r="G807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REI DOS GRÃOS LTDA </t>
+        </is>
+      </c>
+      <c r="H807" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I807" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J807" s="2" t="n">
+        <v>46262.59248885416</v>
+      </c>
+      <c r="K807" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="L807" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M807" s="1" t="inlineStr">
+        <is>
+          <t>Rogerio Egidio</t>
+        </is>
+      </c>
+      <c r="N807" s="2" t="n">
+        <v>46265.59963434028</v>
+      </c>
+      <c r="O807" s="1" t="n"/>
+      <c r="P807" s="2" t="n">
+        <v>46269.6534278125</v>
+      </c>
+      <c r="Q807" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R807" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Em fila de atendimento
+Por favor sempre anexar o email no chamado </t>
+        </is>
+      </c>
+      <c r="S807" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T807" s="1" t="n"/>
+      <c r="U807" s="1" t="inlineStr"/>
+    </row>
+    <row r="808">
+      <c r="A808" s="1" t="n">
+        <v>83139</v>
+      </c>
+      <c r="B808" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C808" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D808" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E808" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, boa tarde! Segue anexo e-mail enviado com a planilha de cadastro de produtos da empresa.</t>
+        </is>
+      </c>
+      <c r="F808" s="1" t="n">
+        <v>6049</v>
+      </c>
+      <c r="G808" s="1" t="inlineStr">
+        <is>
+          <t>ESTACAO DO PEIXE RESTAURANTE LTDA</t>
+        </is>
+      </c>
+      <c r="H808" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I808" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J808" s="2" t="n">
+        <v>46261.59434112268</v>
+      </c>
+      <c r="K808" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="L808" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M808" s="1" t="inlineStr">
+        <is>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N808" s="2" t="n">
+        <v>46265.60815690972</v>
+      </c>
+      <c r="O808" s="1" t="n"/>
+      <c r="P808" s="1" t="n"/>
+      <c r="Q808" s="1" t="inlineStr"/>
+      <c r="R808" s="1" t="inlineStr">
+        <is>
+          <t>Em fila de atendimento</t>
+        </is>
+      </c>
+      <c r="S808" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T808" s="1" t="n"/>
+      <c r="U808" s="1" t="inlineStr"/>
+    </row>
+    <row r="809">
+      <c r="A809" s="1" t="n">
+        <v>83262</v>
+      </c>
+      <c r="B809" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C809" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D809" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E809" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados, bom dia! Segue e-mail enviado com a planilha de cadastro de produtos. </t>
+        </is>
+      </c>
+      <c r="F809" s="1" t="n">
+        <v>6540</v>
+      </c>
+      <c r="G809" s="1" t="inlineStr">
+        <is>
+          <t>MERCADINHO BAMBINA LTDA</t>
+        </is>
+      </c>
+      <c r="H809" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I809" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J809" s="2" t="n">
+        <v>46265.4616653125</v>
+      </c>
+      <c r="K809" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L809" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M809" s="1" t="inlineStr">
+        <is>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N809" s="2" t="n">
+        <v>46265.62414548611</v>
+      </c>
+      <c r="O809" s="1" t="n"/>
+      <c r="P809" s="1" t="n"/>
+      <c r="Q809" s="1" t="inlineStr"/>
+      <c r="R809" s="1" t="inlineStr">
+        <is>
+          <t>Em fila de atendimento</t>
+        </is>
+      </c>
+      <c r="S809" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T809" s="1" t="n"/>
+      <c r="U809" s="1" t="inlineStr"/>
+    </row>
+    <row r="810">
+      <c r="A810" s="1" t="n">
+        <v>83367</v>
+      </c>
+      <c r="B810" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C810" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D810" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E810" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, boa tarde!Segue em anexo cadastro de produtos da empresa 5789 – ACE FRUIT para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F810" s="1" t="n">
+        <v>5789</v>
+      </c>
+      <c r="G810" s="1" t="inlineStr">
+        <is>
+          <t>ACE FRUIT COMERCIO DE ALIMENTOS LTDA (Filial 2)</t>
+        </is>
+      </c>
+      <c r="H810" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I810" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J810" s="2" t="n">
+        <v>46266.64626565972</v>
+      </c>
+      <c r="K810" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L810" s="1" t="inlineStr">
+        <is>
+          <t>Em Atendimento</t>
+        </is>
+      </c>
+      <c r="M810" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N810" s="2" t="n">
+        <v>46269.66462141203</v>
+      </c>
+      <c r="O810" s="1" t="n"/>
+      <c r="P810" s="1" t="n"/>
+      <c r="Q810" s="1" t="inlineStr"/>
+      <c r="R810" s="1" t="inlineStr">
+        <is>
+          <t>Em fila para atendimento</t>
+        </is>
+      </c>
+      <c r="S810" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T810" s="1" t="n"/>
+      <c r="U810" s="1" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" s="1" t="n">
+        <v>83429</v>
+      </c>
+      <c r="B811" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C811" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D811" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E811" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados, boa tarde!Segue novamente planilha de IBS/CBS da empresa 3965 - TUTTI DELI, ela já foi enviada anteriormente o número do chamado antigo é 82784, porém ela foi retornada mesmo estando completa. Na planilha consta NCM, Descrição e EAN. </t>
+        </is>
+      </c>
+      <c r="F811" s="1" t="n">
+        <v>3965</v>
+      </c>
+      <c r="G811" s="1" t="inlineStr">
+        <is>
+          <t>TUTTI QUITUTE PRODUTOS ALIMENTICIOS LTDA</t>
+        </is>
+      </c>
+      <c r="H811" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I811" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J811" s="2" t="n">
+        <v>46266.75154699074</v>
+      </c>
+      <c r="K811" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="L811" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M811" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N811" s="1" t="n"/>
+      <c r="O811" s="1" t="n"/>
+      <c r="P811" s="1" t="n"/>
+      <c r="Q811" s="1" t="inlineStr"/>
+      <c r="R811" s="1" t="inlineStr"/>
+      <c r="S811" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T811" s="1" t="n"/>
+      <c r="U811" s="1" t="inlineStr"/>
+    </row>
+    <row r="812">
+      <c r="A812" s="1" t="n">
+        <v>83313</v>
+      </c>
+      <c r="B812" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C812" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D812" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E812" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prezados, bom dia.Segue e-mail enviado com a planilha de cadastro de produtos. Conforme falado com o gerente de contas Bruno, fica de acordo realizar a validação do cadastro de acordo com as informações enviadas ao cliente. Caso validação não seja realizada por completo iremos comunicar ao cliente. </t>
+        </is>
+      </c>
+      <c r="F812" s="1" t="n">
+        <v>6644</v>
+      </c>
+      <c r="G812" s="1" t="inlineStr">
+        <is>
+          <t>MAPA DISTRIBUIDORA DE ALIMENTOS IMPORTACAO E EXPORTACAO LTDA</t>
+        </is>
+      </c>
+      <c r="H812" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I812" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J812" s="2" t="n">
+        <v>46266.41307797454</v>
+      </c>
+      <c r="K812" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="L812" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M812" s="1" t="inlineStr">
+        <is>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N812" s="1" t="n"/>
+      <c r="O812" s="1" t="n"/>
+      <c r="P812" s="1" t="n"/>
+      <c r="Q812" s="1" t="inlineStr"/>
+      <c r="R812" s="1" t="inlineStr"/>
+      <c r="S812" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T812" s="1" t="n"/>
+      <c r="U812" s="1" t="inlineStr"/>
+    </row>
+    <row r="813">
+      <c r="A813" s="1" t="n">
+        <v>83541</v>
+      </c>
+      <c r="B813" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C813" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D813" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E813" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F813" s="1" t="n">
+        <v>4411</v>
+      </c>
+      <c r="G813" s="1" t="inlineStr">
+        <is>
+          <t>JPS MATERIAIS DE CONSTRUÇÃO E DECORAÇÕES LTDA</t>
+        </is>
+      </c>
+      <c r="H813" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I813" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J813" s="2" t="n">
+        <v>46268.43361015046</v>
+      </c>
+      <c r="K813" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L813" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M813" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N813" s="1" t="n"/>
+      <c r="O813" s="1" t="n"/>
+      <c r="P813" s="2" t="n">
+        <v>46273.43621866898</v>
+      </c>
+      <c r="Q813" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R813" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro analisado e enviado por email em 04/09</t>
+        </is>
+      </c>
+      <c r="S813" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T813" s="1" t="n"/>
+      <c r="U813" s="1" t="inlineStr"/>
+    </row>
+    <row r="814">
+      <c r="A814" s="1" t="n">
+        <v>83542</v>
+      </c>
+      <c r="B814" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C814" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D814" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E814" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, bom dia!Segue em anexo cadastro de produtos da empresa 4411 – JPS MATERIAIS para validação do CBS/IBS.</t>
+        </is>
+      </c>
+      <c r="F814" s="1" t="n">
+        <v>6412</v>
+      </c>
+      <c r="G814" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SPJ MATERIAIS DE CONSTRUCAO LTDA </t>
+        </is>
+      </c>
+      <c r="H814" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I814" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J814" s="2" t="n">
+        <v>46268.43411693287</v>
+      </c>
+      <c r="K814" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L814" s="1" t="inlineStr">
+        <is>
+          <t>Entregue Ao Solicitante</t>
+        </is>
+      </c>
+      <c r="M814" s="1" t="inlineStr">
+        <is>
+          <t>Lohany Martins</t>
+        </is>
+      </c>
+      <c r="N814" s="1" t="n"/>
+      <c r="O814" s="1" t="n"/>
+      <c r="P814" s="2" t="n">
+        <v>46273.43373032408</v>
+      </c>
+      <c r="Q814" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="R814" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro analisado e enviado por email em 04/03</t>
+        </is>
+      </c>
+      <c r="S814" s="1" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="T814" s="1" t="n"/>
+      <c r="U814" s="1" t="inlineStr"/>
+    </row>
+    <row r="815">
+      <c r="A815" s="1" t="n">
+        <v>83562</v>
+      </c>
+      <c r="B815" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C815" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D815" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E815" s="1" t="inlineStr">
+        <is>
+          <t>6947 - F. MARQUES DE SA LTDA - PLANILHA DE INTENS Em anexo email enviado com a planilha.</t>
+        </is>
+      </c>
+      <c r="F815" s="1" t="n">
+        <v>6947</v>
+      </c>
+      <c r="G815" s="1" t="inlineStr">
+        <is>
+          <t>F. MARQUES DE SA LTDA</t>
+        </is>
+      </c>
+      <c r="H815" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I815" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J815" s="2" t="n">
+        <v>46268.52269753473</v>
+      </c>
+      <c r="K815" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L815" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M815" s="1" t="inlineStr">
+        <is>
+          <t>Vander Silva</t>
+        </is>
+      </c>
+      <c r="N815" s="1" t="n"/>
+      <c r="O815" s="1" t="n"/>
+      <c r="P815" s="1" t="n"/>
+      <c r="Q815" s="1" t="inlineStr"/>
+      <c r="R815" s="1" t="inlineStr"/>
+      <c r="S815" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T815" s="1" t="n"/>
+      <c r="U815" s="1" t="inlineStr"/>
+    </row>
+    <row r="816">
+      <c r="A816" s="1" t="n">
+        <v>83432</v>
+      </c>
+      <c r="B816" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C816" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D816" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E816" s="1" t="inlineStr">
+        <is>
+          <t>Revisão de cadastro de produtos da Ki-Preco</t>
+        </is>
+      </c>
+      <c r="F816" s="1" t="n">
+        <v>6442</v>
+      </c>
+      <c r="G816" s="1" t="inlineStr">
+        <is>
+          <t>KI PRECO SERVICOS ADMINISTRATIVOS LTDA</t>
+        </is>
+      </c>
+      <c r="H816" s="1" t="inlineStr">
+        <is>
+          <t>Fernanda Bertunes</t>
+        </is>
+      </c>
+      <c r="I816" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J816" s="2" t="n">
+        <v>46266.81141119213</v>
+      </c>
+      <c r="K816" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="L816" s="1" t="inlineStr">
+        <is>
+          <t>Esperando Atendimento</t>
+        </is>
+      </c>
+      <c r="M816" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N816" s="1" t="n"/>
+      <c r="O816" s="1" t="n"/>
+      <c r="P816" s="1" t="n"/>
+      <c r="Q816" s="1" t="inlineStr"/>
+      <c r="R816" s="1" t="inlineStr"/>
+      <c r="S816" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T816" s="1" t="n"/>
+      <c r="U816" s="1" t="inlineStr"/>
+    </row>
+    <row r="817">
+      <c r="A817" s="1" t="n">
+        <v>83644</v>
+      </c>
+      <c r="B817" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C817" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D817" s="1" t="inlineStr">
+        <is>
+          <t>GERENCIA DE CONTAS</t>
+        </is>
+      </c>
+      <c r="E817" s="1" t="inlineStr">
+        <is>
+          <t>Prezadas, conforme solicitado pelo Nilton, segue:Abrir um chamado para esta empresa fazer a análise do cadastro de produtos dividido em 3 partes:1º - primeira parte analisar os produtos que estão com a exclusão a partir de primeiro de outubro fusão do ICMS – ST (que acho que não deve ter nenhum)2º - segunda parte fazer a classificação da alíquota teste do IBS e CBS3º - Classificação total das alíquotas atuais de ICMS PIS e COFINScadastro enviado no e-mail.</t>
+        </is>
+      </c>
+      <c r="F817" s="1" t="n">
+        <v>1603</v>
+      </c>
+      <c r="G817" s="1" t="inlineStr">
+        <is>
+          <t>MERCADINHO KI PREÇO BAIXO LTDA</t>
+        </is>
+      </c>
+      <c r="H817" s="1" t="n"/>
+      <c r="I817" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J817" s="2" t="n">
+        <v>46273.47367033565</v>
+      </c>
+      <c r="K817" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="L817" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M817" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="N817" s="1" t="n"/>
+      <c r="O817" s="1" t="n"/>
+      <c r="P817" s="1" t="n"/>
+      <c r="Q817" s="1" t="inlineStr"/>
+      <c r="R817" s="1" t="n"/>
+      <c r="S817" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T817" s="1" t="n"/>
+      <c r="U817" s="1" t="inlineStr"/>
+    </row>
+    <row r="818">
+      <c r="A818" s="1" t="n">
+        <v>83654</v>
+      </c>
+      <c r="B818" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de Produtos</t>
+        </is>
+      </c>
+      <c r="C818" s="1" t="inlineStr">
+        <is>
+          <t>Cadastro de produtos</t>
+        </is>
+      </c>
+      <c r="D818" s="1" t="inlineStr">
+        <is>
+          <t>RJ - GC ADMINISTRATIVO</t>
+        </is>
+      </c>
+      <c r="E818" s="1" t="inlineStr">
+        <is>
+          <t>Prezados, segue em anexo e-mail com planilha de cadastro de produtos da empresa.</t>
+        </is>
+      </c>
+      <c r="F818" s="1" t="n">
+        <v>5714</v>
+      </c>
+      <c r="G818" s="1" t="inlineStr">
+        <is>
+          <t>DIBRAMASUL MADEIRAS LTDA</t>
+        </is>
+      </c>
+      <c r="H818" s="1" t="n"/>
+      <c r="I818" s="1" t="inlineStr">
+        <is>
+          <t>CADASTRO DE PRODUTOS</t>
+        </is>
+      </c>
+      <c r="J818" s="2" t="n">
+        <v>46273.54331446759</v>
+      </c>
+      <c r="K818" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="L818" s="1" t="inlineStr">
+        <is>
+          <t>Sem Responsavel Atribuido</t>
+        </is>
+      </c>
+      <c r="M818" s="1" t="inlineStr">
+        <is>
+          <t>Amanda Mesquita</t>
+        </is>
+      </c>
+      <c r="N818" s="1" t="n"/>
+      <c r="O818" s="1" t="n"/>
+      <c r="P818" s="1" t="n"/>
+      <c r="Q818" s="1" t="inlineStr"/>
+      <c r="R818" s="1" t="n"/>
+      <c r="S818" s="1" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="T818" s="1" t="n"/>
+      <c r="U818" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>